<commit_message>
Auto update stocks_data.xlsx [2026-03-02 05:06:54]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH119"/>
+  <dimension ref="A1:AI119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="15"/>
@@ -551,6 +551,7 @@
     <col width="15" customWidth="1" min="32" max="32"/>
     <col width="15" customWidth="1" min="33" max="33"/>
     <col width="15" customWidth="1" min="34" max="34"/>
+    <col width="15" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -724,6 +725,11 @@
           <t>2026/02/26</t>
         </is>
       </c>
+      <c r="AI1" s="13" t="inlineStr">
+        <is>
+          <t>2026/03/02</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -896,6 +902,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="AI2" s="14" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1000,6 +1011,9 @@
       <c r="AH3" s="13" t="n">
         <v>69.66</v>
       </c>
+      <c r="AI3" s="13" t="n">
+        <v>69.75</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1103,6 +1117,9 @@
       </c>
       <c r="AH4" s="13" t="n">
         <v>4147.93</v>
+      </c>
+      <c r="AI4" s="13" t="n">
+        <v>4169.02</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1140,6 +1157,7 @@
       <c r="AF5" s="13" t="n"/>
       <c r="AG5" s="13" t="n"/>
       <c r="AH5" s="13" t="n"/>
+      <c r="AI5" s="13" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1224,6 +1242,7 @@
       <c r="AF6" s="13" t="n"/>
       <c r="AG6" s="13" t="n"/>
       <c r="AH6" s="13" t="n"/>
+      <c r="AI6" s="13" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1327,6 +1346,9 @@
       </c>
       <c r="AH7" s="13" t="n">
         <v>51.5</v>
+      </c>
+      <c r="AI7" s="13" t="n">
+        <v>51.3</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -1384,6 +1406,9 @@
       <c r="AH8" s="13" t="n">
         <v>5970.65</v>
       </c>
+      <c r="AI8" s="13" t="n">
+        <v>5969.32</v>
+      </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -1468,6 +1493,7 @@
       <c r="AF9" s="13" t="n"/>
       <c r="AG9" s="13" t="n"/>
       <c r="AH9" s="13" t="n"/>
+      <c r="AI9" s="13" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -1571,6 +1597,9 @@
       </c>
       <c r="AH10" s="13" t="n">
         <v>54.67</v>
+      </c>
+      <c r="AI10" s="13" t="n">
+        <v>53.78</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -1628,6 +1657,9 @@
       <c r="AH11" s="13" t="n">
         <v>4731.98</v>
       </c>
+      <c r="AI11" s="13" t="n">
+        <v>4717.74</v>
+      </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -1712,6 +1744,7 @@
       <c r="AF12" s="13" t="n"/>
       <c r="AG12" s="13" t="n"/>
       <c r="AH12" s="13" t="n"/>
+      <c r="AI12" s="13" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -1815,6 +1848,9 @@
       </c>
       <c r="AH13" s="13" t="n">
         <v>61.68</v>
+      </c>
+      <c r="AI13" s="13" t="n">
+        <v>61.85</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -1872,6 +1908,9 @@
       <c r="AH14" s="13" t="n">
         <v>8575.25</v>
       </c>
+      <c r="AI14" s="13" t="n">
+        <v>8629.24</v>
+      </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -1956,6 +1995,7 @@
       <c r="AF15" s="13" t="n"/>
       <c r="AG15" s="13" t="n"/>
       <c r="AH15" s="13" t="n"/>
+      <c r="AI15" s="13" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -2059,6 +2099,9 @@
       </c>
       <c r="AH16" s="13" t="n">
         <v>29.81</v>
+      </c>
+      <c r="AI16" s="13" t="n">
+        <v>28.59</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -2116,6 +2159,9 @@
       <c r="AH17" s="13" t="n">
         <v>2748.51</v>
       </c>
+      <c r="AI17" s="13" t="n">
+        <v>2687.84</v>
+      </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="3" t="n">
@@ -2200,6 +2246,7 @@
       <c r="AF18" s="13" t="n"/>
       <c r="AG18" s="13" t="n"/>
       <c r="AH18" s="13" t="n"/>
+      <c r="AI18" s="13" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -2303,6 +2350,9 @@
       </c>
       <c r="AH19" s="13" t="n">
         <v>95.75</v>
+      </c>
+      <c r="AI19" s="13" t="n">
+        <v>95.22</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -2360,6 +2410,9 @@
       <c r="AH20" s="13" t="n">
         <v>6946.13</v>
       </c>
+      <c r="AI20" s="13" t="n">
+        <v>6878.88</v>
+      </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -2444,6 +2497,7 @@
       <c r="AF21" s="13" t="n"/>
       <c r="AG21" s="13" t="n"/>
       <c r="AH21" s="13" t="n"/>
+      <c r="AI21" s="13" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -2545,6 +2599,9 @@
       </c>
       <c r="AH22" s="13" t="n">
         <v>60.13</v>
+      </c>
+      <c r="AI22" s="13" t="n">
+        <v>58.02</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1">
@@ -2602,6 +2659,9 @@
       <c r="AH23" s="13" t="n">
         <v>82443.33</v>
       </c>
+      <c r="AI23" s="13" t="n">
+        <v>80311.49000000001</v>
+      </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="3" t="n">
@@ -2686,6 +2746,7 @@
       <c r="AF24" s="13" t="n"/>
       <c r="AG24" s="13" t="n"/>
       <c r="AH24" s="13" t="n"/>
+      <c r="AI24" s="13" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -2789,6 +2850,9 @@
       </c>
       <c r="AH25" s="13" t="n">
         <v>81.65000000000001</v>
+      </c>
+      <c r="AI25" s="13" t="n">
+        <v>87.75</v>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="1">
@@ -2846,6 +2910,9 @@
       <c r="AH26" s="13" t="n">
         <v>25175.94</v>
       </c>
+      <c r="AI26" s="13" t="n">
+        <v>25284.26</v>
+      </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -2930,6 +2997,7 @@
       <c r="AF27" s="13" t="n"/>
       <c r="AG27" s="13" t="n"/>
       <c r="AH27" s="13" t="n"/>
+      <c r="AI27" s="13" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -3033,6 +3101,9 @@
       </c>
       <c r="AH28" s="13" t="n">
         <v>77.40000000000001</v>
+      </c>
+      <c r="AI28" s="13" t="n">
+        <v>79.7</v>
       </c>
     </row>
     <row r="29" ht="14.25" customHeight="1">
@@ -3090,6 +3161,9 @@
       <c r="AH29" s="13" t="n">
         <v>58662.72</v>
       </c>
+      <c r="AI29" s="13" t="n">
+        <v>57880.6</v>
+      </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="3" t="n">
@@ -3174,6 +3248,7 @@
       <c r="AF30" s="13" t="n"/>
       <c r="AG30" s="13" t="n"/>
       <c r="AH30" s="13" t="n"/>
+      <c r="AI30" s="13" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -3277,6 +3352,9 @@
       </c>
       <c r="AH31" s="13" t="n">
         <v>51.42</v>
+      </c>
+      <c r="AI31" s="13" t="n">
+        <v>50.94</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -3334,6 +3412,9 @@
       <c r="AH32" s="13" t="n">
         <v>5765.52</v>
       </c>
+      <c r="AI32" s="13" t="n">
+        <v>5871.71</v>
+      </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
       <c r="A33" s="3" t="n">
@@ -3418,6 +3499,7 @@
       <c r="AF33" s="13" t="n"/>
       <c r="AG33" s="13" t="n"/>
       <c r="AH33" s="13" t="n"/>
+      <c r="AI33" s="13" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -3521,6 +3603,9 @@
       </c>
       <c r="AH34" s="13" t="n">
         <v>2.27</v>
+      </c>
+      <c r="AI34" s="13" t="n">
+        <v>1.95</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -3578,6 +3663,9 @@
       <c r="AH35" s="13" t="n">
         <v>34383.02</v>
       </c>
+      <c r="AI35" s="13" t="n">
+        <v>34543.15</v>
+      </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="3" t="n">
@@ -3662,6 +3750,7 @@
       <c r="AF36" s="13" t="n"/>
       <c r="AG36" s="13" t="n"/>
       <c r="AH36" s="13" t="n"/>
+      <c r="AI36" s="13" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -3765,6 +3854,9 @@
       </c>
       <c r="AH37" s="13" t="n">
         <v>32.22</v>
+      </c>
+      <c r="AI37" s="13" t="n">
+        <v>31.2</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -3822,6 +3914,9 @@
       <c r="AH38" s="13" t="n">
         <v>3502.92</v>
       </c>
+      <c r="AI38" s="13" t="n">
+        <v>3448.58</v>
+      </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
       <c r="A39" s="3" t="n">
@@ -3906,6 +4001,7 @@
       <c r="AF39" s="13" t="n"/>
       <c r="AG39" s="13" t="n"/>
       <c r="AH39" s="13" t="n"/>
+      <c r="AI39" s="13" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -4009,6 +4105,9 @@
       </c>
       <c r="AH40" s="13" t="n">
         <v>55.73</v>
+      </c>
+      <c r="AI40" s="13" t="n">
+        <v>55.38</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -4066,6 +4165,9 @@
       <c r="AH41" s="13" t="n">
         <v>3347.54</v>
       </c>
+      <c r="AI41" s="13" t="n">
+        <v>3302.8</v>
+      </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
       <c r="A42" s="3" t="n">
@@ -4150,6 +4252,7 @@
       <c r="AF42" s="13" t="n"/>
       <c r="AG42" s="13" t="n"/>
       <c r="AH42" s="13" t="n"/>
+      <c r="AI42" s="13" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -4253,6 +4356,9 @@
       </c>
       <c r="AH43" s="13" t="n">
         <v>18.91</v>
+      </c>
+      <c r="AI43" s="13" t="n">
+        <v>18.26</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -4310,6 +4416,9 @@
       <c r="AH44" s="13" t="n">
         <v>7037.7</v>
       </c>
+      <c r="AI44" s="13" t="n">
+        <v>6923.32</v>
+      </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
       <c r="A45" s="3" t="n">
@@ -4394,6 +4503,7 @@
       <c r="AF45" s="13" t="n"/>
       <c r="AG45" s="13" t="n"/>
       <c r="AH45" s="13" t="n"/>
+      <c r="AI45" s="13" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -4497,6 +4607,9 @@
       </c>
       <c r="AH46" s="13" t="n">
         <v>23.97</v>
+      </c>
+      <c r="AI46" s="13" t="n">
+        <v>22.62</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -4554,6 +4667,9 @@
       <c r="AH47" s="13" t="n">
         <v>8262.309999999999</v>
       </c>
+      <c r="AI47" s="13" t="n">
+        <v>8069.33</v>
+      </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
       <c r="A48" s="3" t="n">
@@ -4638,6 +4754,7 @@
       <c r="AF48" s="13" t="n"/>
       <c r="AG48" s="13" t="n"/>
       <c r="AH48" s="13" t="n"/>
+      <c r="AI48" s="13" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -4741,6 +4858,9 @@
       </c>
       <c r="AH49" s="13" t="n">
         <v>8.82</v>
+      </c>
+      <c r="AI49" s="13" t="n">
+        <v>7.65</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -4798,6 +4918,9 @@
       <c r="AH50" s="13" t="n">
         <v>12530.04</v>
       </c>
+      <c r="AI50" s="13" t="n">
+        <v>12172.05</v>
+      </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
       <c r="A51" s="3" t="n">
@@ -4882,6 +5005,7 @@
       <c r="AF51" s="13" t="n"/>
       <c r="AG51" s="13" t="n"/>
       <c r="AH51" s="13" t="n"/>
+      <c r="AI51" s="13" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -4985,6 +5109,9 @@
       </c>
       <c r="AH52" s="13" t="n">
         <v>30.71</v>
+      </c>
+      <c r="AI52" s="13" t="n">
+        <v>28.63</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -5042,6 +5169,9 @@
       <c r="AH53" s="13" t="n">
         <v>12997.41</v>
       </c>
+      <c r="AI53" s="13" t="n">
+        <v>12727.06</v>
+      </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
       <c r="A54" s="3" t="n">
@@ -5126,6 +5256,7 @@
       <c r="AF54" s="13" t="n"/>
       <c r="AG54" s="13" t="n"/>
       <c r="AH54" s="13" t="n"/>
+      <c r="AI54" s="13" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -5229,6 +5360,9 @@
       </c>
       <c r="AH55" s="13" t="n">
         <v>19.46</v>
+      </c>
+      <c r="AI55" s="13" t="n">
+        <v>17.75</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -5286,6 +5420,9 @@
       <c r="AH56" s="13" t="n">
         <v>8453.26</v>
       </c>
+      <c r="AI56" s="13" t="n">
+        <v>8277.93</v>
+      </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
       <c r="A57" s="3" t="n">
@@ -5370,6 +5507,7 @@
       <c r="AF57" s="13" t="n"/>
       <c r="AG57" s="13" t="n"/>
       <c r="AH57" s="13" t="n"/>
+      <c r="AI57" s="13" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -5473,6 +5611,9 @@
       </c>
       <c r="AH58" s="13" t="n">
         <v>26.3</v>
+      </c>
+      <c r="AI58" s="13" t="n">
+        <v>25.95</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -5530,6 +5671,9 @@
       <c r="AH59" s="13" t="n">
         <v>14835.13</v>
       </c>
+      <c r="AI59" s="13" t="n">
+        <v>14772.64</v>
+      </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
       <c r="A60" s="3" t="n">
@@ -5614,6 +5758,7 @@
       <c r="AF60" s="13" t="n"/>
       <c r="AG60" s="13" t="n"/>
       <c r="AH60" s="13" t="n"/>
+      <c r="AI60" s="13" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -5717,6 +5862,9 @@
       </c>
       <c r="AH61" s="13" t="n">
         <v>30.84</v>
+      </c>
+      <c r="AI61" s="13" t="n">
+        <v>29.92</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -5774,6 +5922,9 @@
       <c r="AH62" s="13" t="n">
         <v>15377.58</v>
       </c>
+      <c r="AI62" s="13" t="n">
+        <v>14774.52</v>
+      </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
       <c r="A63" s="3" t="n">
@@ -5858,6 +6009,7 @@
       <c r="AF63" s="13" t="n"/>
       <c r="AG63" s="13" t="n"/>
       <c r="AH63" s="13" t="n"/>
+      <c r="AI63" s="13" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -5961,6 +6113,9 @@
       </c>
       <c r="AH64" s="13" t="n">
         <v>16.7</v>
+      </c>
+      <c r="AI64" s="13" t="n">
+        <v>15.93</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -6018,6 +6173,9 @@
       <c r="AH65" s="13" t="n">
         <v>8421.98</v>
       </c>
+      <c r="AI65" s="13" t="n">
+        <v>8178.68</v>
+      </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
       <c r="A66" s="3" t="n">
@@ -6102,6 +6260,7 @@
       <c r="AF66" s="13" t="n"/>
       <c r="AG66" s="13" t="n"/>
       <c r="AH66" s="13" t="n"/>
+      <c r="AI66" s="13" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -6205,6 +6364,9 @@
       </c>
       <c r="AH67" s="13" t="n">
         <v>10.75</v>
+      </c>
+      <c r="AI67" s="13" t="n">
+        <v>10.03</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -6262,6 +6424,9 @@
       <c r="AH68" s="13" t="n">
         <v>9582.959999999999</v>
       </c>
+      <c r="AI68" s="13" t="n">
+        <v>9474.83</v>
+      </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
       <c r="A69" s="3" t="n">
@@ -6346,6 +6511,7 @@
       <c r="AF69" s="13" t="n"/>
       <c r="AG69" s="13" t="n"/>
       <c r="AH69" s="13" t="n"/>
+      <c r="AI69" s="13" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -6449,6 +6615,9 @@
       </c>
       <c r="AH70" s="13" t="n">
         <v>20.15</v>
+      </c>
+      <c r="AI70" s="13" t="n">
+        <v>19.81</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -6506,6 +6675,9 @@
       <c r="AH71" s="13" t="n">
         <v>2731.91</v>
       </c>
+      <c r="AI71" s="13" t="n">
+        <v>2650.05</v>
+      </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
       <c r="A72" s="3" t="n">
@@ -6590,6 +6762,7 @@
       <c r="AF72" s="13" t="n"/>
       <c r="AG72" s="13" t="n"/>
       <c r="AH72" s="13" t="n"/>
+      <c r="AI72" s="13" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -6693,6 +6866,9 @@
       </c>
       <c r="AH73" s="13" t="n">
         <v>39.39</v>
+      </c>
+      <c r="AI73" s="13" t="n">
+        <v>37.64</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -6750,6 +6926,9 @@
       <c r="AH74" s="13" t="n">
         <v>5167.11</v>
       </c>
+      <c r="AI74" s="13" t="n">
+        <v>5030.11</v>
+      </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
       <c r="A75" s="3" t="n">
@@ -6834,6 +7013,7 @@
       <c r="AF75" s="13" t="n"/>
       <c r="AG75" s="13" t="n"/>
       <c r="AH75" s="13" t="n"/>
+      <c r="AI75" s="13" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -6937,6 +7117,9 @@
       </c>
       <c r="AH76" s="13" t="n">
         <v>22.99</v>
+      </c>
+      <c r="AI76" s="13" t="n">
+        <v>21.57</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -6994,6 +7177,9 @@
       <c r="AH77" s="13" t="n">
         <v>8813.01</v>
       </c>
+      <c r="AI77" s="13" t="n">
+        <v>8648.879999999999</v>
+      </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
       <c r="A78" s="3" t="n">
@@ -7078,6 +7264,7 @@
       <c r="AF78" s="13" t="n"/>
       <c r="AG78" s="13" t="n"/>
       <c r="AH78" s="13" t="n"/>
+      <c r="AI78" s="13" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -7181,6 +7368,9 @@
       </c>
       <c r="AH79" s="13" t="n">
         <v>17.66</v>
+      </c>
+      <c r="AI79" s="13" t="n">
+        <v>17.02</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -7238,6 +7428,9 @@
       <c r="AH80" s="13" t="n">
         <v>1462.19</v>
       </c>
+      <c r="AI80" s="13" t="n">
+        <v>1419.21</v>
+      </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
       <c r="A81" s="3" t="n">
@@ -7322,6 +7515,7 @@
       <c r="AF81" s="13" t="n"/>
       <c r="AG81" s="13" t="n"/>
       <c r="AH81" s="13" t="n"/>
+      <c r="AI81" s="13" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -7425,6 +7619,9 @@
       </c>
       <c r="AH82" s="13" t="n">
         <v>16.34</v>
+      </c>
+      <c r="AI82" s="13" t="n">
+        <v>15.29</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -7482,6 +7679,9 @@
       <c r="AH83" s="13" t="n">
         <v>16497.29</v>
       </c>
+      <c r="AI83" s="13" t="n">
+        <v>16255.31</v>
+      </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
       <c r="A84" s="3" t="n">
@@ -7566,6 +7766,7 @@
       <c r="AF84" s="13" t="n"/>
       <c r="AG84" s="13" t="n"/>
       <c r="AH84" s="13" t="n"/>
+      <c r="AI84" s="13" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -7669,6 +7870,9 @@
       </c>
       <c r="AH85" s="13" t="n">
         <v>55.06</v>
+      </c>
+      <c r="AI85" s="13" t="n">
+        <v>54.2</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -7726,6 +7930,9 @@
       <c r="AH86" s="13" t="n">
         <v>3055.67</v>
       </c>
+      <c r="AI86" s="13" t="n">
+        <v>3049.19</v>
+      </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
       <c r="A87" s="3" t="n">
@@ -7810,6 +8017,7 @@
       <c r="AF87" s="13" t="n"/>
       <c r="AG87" s="13" t="n"/>
       <c r="AH87" s="13" t="n"/>
+      <c r="AI87" s="13" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -7913,6 +8121,9 @@
       </c>
       <c r="AH88" s="13" t="n">
         <v>58.66</v>
+      </c>
+      <c r="AI88" s="13" t="n">
+        <v>57.59</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -7970,6 +8181,9 @@
       <c r="AH89" s="13" t="n">
         <v>3325.49</v>
       </c>
+      <c r="AI89" s="13" t="n">
+        <v>3379.4</v>
+      </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
       <c r="A90" s="3" t="n">
@@ -8054,6 +8268,7 @@
       <c r="AF90" s="13" t="n"/>
       <c r="AG90" s="13" t="n"/>
       <c r="AH90" s="13" t="n"/>
+      <c r="AI90" s="13" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -8157,6 +8372,9 @@
       </c>
       <c r="AH91" s="13" t="n">
         <v>51.62</v>
+      </c>
+      <c r="AI91" s="13" t="n">
+        <v>49.56</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -8214,6 +8432,9 @@
       <c r="AH92" s="13" t="n">
         <v>3096.89</v>
       </c>
+      <c r="AI92" s="13" t="n">
+        <v>3088.37</v>
+      </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
       <c r="A93" s="3" t="n">
@@ -8298,6 +8519,7 @@
       <c r="AF93" s="13" t="n"/>
       <c r="AG93" s="13" t="n"/>
       <c r="AH93" s="13" t="n"/>
+      <c r="AI93" s="13" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -8401,6 +8623,9 @@
       </c>
       <c r="AH94" s="13" t="n">
         <v>40.96</v>
+      </c>
+      <c r="AI94" s="13" t="n">
+        <v>38.18</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -8458,6 +8683,9 @@
       <c r="AH95" s="13" t="n">
         <v>1879.37</v>
       </c>
+      <c r="AI95" s="13" t="n">
+        <v>1879.37</v>
+      </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
       <c r="A96" s="3" t="n">
@@ -8542,6 +8770,7 @@
       <c r="AF96" s="13" t="n"/>
       <c r="AG96" s="13" t="n"/>
       <c r="AH96" s="13" t="n"/>
+      <c r="AI96" s="13" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -8645,6 +8874,9 @@
       </c>
       <c r="AH97" s="13" t="n">
         <v>27.08</v>
+      </c>
+      <c r="AI97" s="13" t="n">
+        <v>26.84</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -8702,6 +8934,9 @@
       <c r="AH98" s="13" t="n">
         <v>10184.4</v>
       </c>
+      <c r="AI98" s="13" t="n">
+        <v>10362.77</v>
+      </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
       <c r="A99" s="3" t="n">
@@ -8786,6 +9021,7 @@
       <c r="AF99" s="13" t="n"/>
       <c r="AG99" s="13" t="n"/>
       <c r="AH99" s="13" t="n"/>
+      <c r="AI99" s="13" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -8889,6 +9125,9 @@
       </c>
       <c r="AH100" s="13" t="n">
         <v>87.61</v>
+      </c>
+      <c r="AI100" s="13" t="n">
+        <v>87.66</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -8946,6 +9185,9 @@
       <c r="AH101" s="13" t="n">
         <v>10690.49</v>
       </c>
+      <c r="AI101" s="13" t="n">
+        <v>10430.16</v>
+      </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
       <c r="A102" s="3" t="n">
@@ -9030,6 +9272,7 @@
       <c r="AF102" s="13" t="n"/>
       <c r="AG102" s="13" t="n"/>
       <c r="AH102" s="13" t="n"/>
+      <c r="AI102" s="13" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -9133,6 +9376,9 @@
       </c>
       <c r="AH103" s="13" t="n">
         <v>59.91</v>
+      </c>
+      <c r="AI103" s="13" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -9190,6 +9436,9 @@
       <c r="AH104" s="13" t="n">
         <v>15852.73</v>
       </c>
+      <c r="AI104" s="13" t="n">
+        <v>16098.45</v>
+      </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
       <c r="A105" s="3" t="n">
@@ -9274,6 +9523,7 @@
       <c r="AF105" s="13" t="n"/>
       <c r="AG105" s="13" t="n"/>
       <c r="AH105" s="13" t="n"/>
+      <c r="AI105" s="13" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -9377,6 +9627,9 @@
       </c>
       <c r="AH106" s="13" t="n">
         <v>7.81</v>
+      </c>
+      <c r="AI106" s="13" t="n">
+        <v>8.539999999999999</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -9434,6 +9687,9 @@
       <c r="AH107" s="13" t="n">
         <v>2199.65</v>
       </c>
+      <c r="AI107" s="13" t="n">
+        <v>2220.51</v>
+      </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
       <c r="A108" s="3" t="n">
@@ -9518,6 +9774,7 @@
       <c r="AF108" s="13" t="n"/>
       <c r="AG108" s="13" t="n"/>
       <c r="AH108" s="13" t="n"/>
+      <c r="AI108" s="13" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -9621,6 +9878,9 @@
       </c>
       <c r="AH109" s="13" t="n">
         <v>25.03</v>
+      </c>
+      <c r="AI109" s="13" t="n">
+        <v>24.93</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -9678,6 +9938,9 @@
       <c r="AH110" s="13" t="n">
         <v>819.92</v>
       </c>
+      <c r="AI110" s="13" t="n">
+        <v>809.76</v>
+      </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
       <c r="A111" s="3" t="n">
@@ -9762,6 +10025,7 @@
       <c r="AF111" s="13" t="n"/>
       <c r="AG111" s="13" t="n"/>
       <c r="AH111" s="13" t="n"/>
+      <c r="AI111" s="13" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -9865,6 +10129,9 @@
       </c>
       <c r="AH112" s="13" t="n">
         <v>33.73</v>
+      </c>
+      <c r="AI112" s="13" t="n">
+        <v>33.79</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -9922,6 +10189,9 @@
       <c r="AH113" s="13" t="n">
         <v>3760.14</v>
       </c>
+      <c r="AI113" s="13" t="n">
+        <v>3868.67</v>
+      </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
       <c r="A114" s="3" t="n">
@@ -10006,6 +10276,7 @@
       <c r="AF114" s="13" t="n"/>
       <c r="AG114" s="13" t="n"/>
       <c r="AH114" s="13" t="n"/>
+      <c r="AI114" s="13" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -10109,6 +10380,9 @@
       </c>
       <c r="AH115" s="13" t="n">
         <v>22.57</v>
+      </c>
+      <c r="AI115" s="13" t="n">
+        <v>23.26</v>
       </c>
     </row>
     <row r="116">
@@ -10151,6 +10425,9 @@
       <c r="AH116" s="13" t="n">
         <v>4172.56</v>
       </c>
+      <c r="AI116" s="13" t="n">
+        <v>4210.94</v>
+      </c>
     </row>
     <row r="117">
       <c r="P117" s="13" t="n">
@@ -10190,6 +10467,7 @@
       <c r="AF117" s="13" t="n"/>
       <c r="AG117" s="13" t="n"/>
       <c r="AH117" s="13" t="n"/>
+      <c r="AI117" s="13" t="n"/>
     </row>
     <row r="118">
       <c r="P118" s="13" t="n">
@@ -10249,6 +10527,9 @@
       <c r="AH118" s="13" t="n">
         <v>29.02</v>
       </c>
+      <c r="AI118" s="13" t="n">
+        <v>29.02</v>
+      </c>
     </row>
     <row r="119">
       <c r="Y119" s="13" t="n">
@@ -10280,6 +10561,9 @@
       </c>
       <c r="AH119" s="13" t="n">
         <v>3083.4</v>
+      </c>
+      <c r="AI119" s="13" t="n">
+        <v>3078.01</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-03-05 05:04:24]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI119"/>
+  <dimension ref="A1:AJ119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="15"/>
@@ -552,6 +552,7 @@
     <col width="15" customWidth="1" min="33" max="33"/>
     <col width="15" customWidth="1" min="34" max="34"/>
     <col width="15" customWidth="1" min="35" max="35"/>
+    <col width="15" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -730,6 +731,11 @@
           <t>2026/03/02</t>
         </is>
       </c>
+      <c r="AJ1" s="13" t="inlineStr">
+        <is>
+          <t>2026/03/05</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -907,6 +913,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="AJ2" s="14" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1014,6 +1025,9 @@
       <c r="AI3" s="13" t="n">
         <v>69.75</v>
       </c>
+      <c r="AJ3" s="13" t="n">
+        <v>68.06</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1120,6 +1134,9 @@
       </c>
       <c r="AI4" s="13" t="n">
         <v>4169.02</v>
+      </c>
+      <c r="AJ4" s="13" t="n">
+        <v>4116.77</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1158,6 +1175,7 @@
       <c r="AG5" s="13" t="n"/>
       <c r="AH5" s="13" t="n"/>
       <c r="AI5" s="13" t="n"/>
+      <c r="AJ5" s="13" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1243,6 +1261,7 @@
       <c r="AG6" s="13" t="n"/>
       <c r="AH6" s="13" t="n"/>
       <c r="AI6" s="13" t="n"/>
+      <c r="AJ6" s="13" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1349,6 +1368,9 @@
       </c>
       <c r="AI7" s="13" t="n">
         <v>51.3</v>
+      </c>
+      <c r="AJ7" s="13" t="n">
+        <v>50.81</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -1409,6 +1431,9 @@
       <c r="AI8" s="13" t="n">
         <v>5969.32</v>
       </c>
+      <c r="AJ8" s="13" t="n">
+        <v>5863.71</v>
+      </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -1494,6 +1519,7 @@
       <c r="AG9" s="13" t="n"/>
       <c r="AH9" s="13" t="n"/>
       <c r="AI9" s="13" t="n"/>
+      <c r="AJ9" s="13" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -1600,6 +1626,9 @@
       </c>
       <c r="AI10" s="13" t="n">
         <v>53.78</v>
+      </c>
+      <c r="AJ10" s="13" t="n">
+        <v>53.68</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -1660,6 +1689,9 @@
       <c r="AI11" s="13" t="n">
         <v>4717.74</v>
       </c>
+      <c r="AJ11" s="13" t="n">
+        <v>4662.92</v>
+      </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -1745,6 +1777,7 @@
       <c r="AG12" s="13" t="n"/>
       <c r="AH12" s="13" t="n"/>
       <c r="AI12" s="13" t="n"/>
+      <c r="AJ12" s="13" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -1851,6 +1884,9 @@
       </c>
       <c r="AI13" s="13" t="n">
         <v>61.85</v>
+      </c>
+      <c r="AJ13" s="13" t="n">
+        <v>60.8</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -1911,6 +1947,9 @@
       <c r="AI14" s="13" t="n">
         <v>8629.24</v>
       </c>
+      <c r="AJ14" s="13" t="n">
+        <v>8346.25</v>
+      </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -1996,6 +2035,7 @@
       <c r="AG15" s="13" t="n"/>
       <c r="AH15" s="13" t="n"/>
       <c r="AI15" s="13" t="n"/>
+      <c r="AJ15" s="13" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -2102,6 +2142,9 @@
       </c>
       <c r="AI16" s="13" t="n">
         <v>28.59</v>
+      </c>
+      <c r="AJ16" s="13" t="n">
+        <v>26.65</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -2162,6 +2205,9 @@
       <c r="AI17" s="13" t="n">
         <v>2687.84</v>
       </c>
+      <c r="AJ17" s="13" t="n">
+        <v>2629.32</v>
+      </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="3" t="n">
@@ -2247,6 +2293,7 @@
       <c r="AG18" s="13" t="n"/>
       <c r="AH18" s="13" t="n"/>
       <c r="AI18" s="13" t="n"/>
+      <c r="AJ18" s="13" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -2353,6 +2400,9 @@
       </c>
       <c r="AI19" s="13" t="n">
         <v>95.22</v>
+      </c>
+      <c r="AJ19" s="13" t="n">
+        <v>95.16</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -2413,6 +2463,9 @@
       <c r="AI20" s="13" t="n">
         <v>6878.88</v>
       </c>
+      <c r="AJ20" s="13" t="n">
+        <v>6869.5</v>
+      </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -2498,6 +2551,7 @@
       <c r="AG21" s="13" t="n"/>
       <c r="AH21" s="13" t="n"/>
       <c r="AI21" s="13" t="n"/>
+      <c r="AJ21" s="13" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -2602,6 +2656,9 @@
       </c>
       <c r="AI22" s="13" t="n">
         <v>58.02</v>
+      </c>
+      <c r="AJ22" s="13" t="n">
+        <v>54.48</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1">
@@ -2662,6 +2719,9 @@
       <c r="AI23" s="13" t="n">
         <v>80311.49000000001</v>
       </c>
+      <c r="AJ23" s="13" t="n">
+        <v>79463.50999999999</v>
+      </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="3" t="n">
@@ -2747,6 +2807,7 @@
       <c r="AG24" s="13" t="n"/>
       <c r="AH24" s="13" t="n"/>
       <c r="AI24" s="13" t="n"/>
+      <c r="AJ24" s="13" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -2853,6 +2914,9 @@
       </c>
       <c r="AI25" s="13" t="n">
         <v>87.75</v>
+      </c>
+      <c r="AJ25" s="13" t="n">
+        <v>77.13</v>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="1">
@@ -2913,6 +2977,9 @@
       <c r="AI26" s="13" t="n">
         <v>25284.26</v>
       </c>
+      <c r="AJ26" s="13" t="n">
+        <v>24205.36</v>
+      </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -2998,6 +3065,7 @@
       <c r="AG27" s="13" t="n"/>
       <c r="AH27" s="13" t="n"/>
       <c r="AI27" s="13" t="n"/>
+      <c r="AJ27" s="13" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -3104,6 +3172,9 @@
       </c>
       <c r="AI28" s="13" t="n">
         <v>79.7</v>
+      </c>
+      <c r="AJ28" s="13" t="n">
+        <v>75.56</v>
       </c>
     </row>
     <row r="29" ht="14.25" customHeight="1">
@@ -3164,6 +3235,9 @@
       <c r="AI29" s="13" t="n">
         <v>57880.6</v>
       </c>
+      <c r="AJ29" s="13" t="n">
+        <v>55673.59</v>
+      </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="3" t="n">
@@ -3249,6 +3323,7 @@
       <c r="AG30" s="13" t="n"/>
       <c r="AH30" s="13" t="n"/>
       <c r="AI30" s="13" t="n"/>
+      <c r="AJ30" s="13" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -3355,6 +3430,9 @@
       </c>
       <c r="AI31" s="13" t="n">
         <v>50.94</v>
+      </c>
+      <c r="AJ31" s="13" t="n">
+        <v>51.62</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -3415,6 +3493,9 @@
       <c r="AI32" s="13" t="n">
         <v>5871.71</v>
       </c>
+      <c r="AJ32" s="13" t="n">
+        <v>5842.72</v>
+      </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
       <c r="A33" s="3" t="n">
@@ -3500,6 +3581,7 @@
       <c r="AG33" s="13" t="n"/>
       <c r="AH33" s="13" t="n"/>
       <c r="AI33" s="13" t="n"/>
+      <c r="AJ33" s="13" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -3606,6 +3688,9 @@
       </c>
       <c r="AI34" s="13" t="n">
         <v>1.95</v>
+      </c>
+      <c r="AJ34" s="13" t="n">
+        <v>2.26</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -3666,6 +3751,9 @@
       <c r="AI35" s="13" t="n">
         <v>34543.15</v>
       </c>
+      <c r="AJ35" s="13" t="n">
+        <v>33320.04</v>
+      </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="3" t="n">
@@ -3751,6 +3839,7 @@
       <c r="AG36" s="13" t="n"/>
       <c r="AH36" s="13" t="n"/>
       <c r="AI36" s="13" t="n"/>
+      <c r="AJ36" s="13" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -3857,6 +3946,9 @@
       </c>
       <c r="AI37" s="13" t="n">
         <v>31.2</v>
+      </c>
+      <c r="AJ37" s="13" t="n">
+        <v>28.91</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -3917,6 +4009,9 @@
       <c r="AI38" s="13" t="n">
         <v>3448.58</v>
       </c>
+      <c r="AJ38" s="13" t="n">
+        <v>3402.4</v>
+      </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
       <c r="A39" s="3" t="n">
@@ -4002,6 +4097,7 @@
       <c r="AG39" s="13" t="n"/>
       <c r="AH39" s="13" t="n"/>
       <c r="AI39" s="13" t="n"/>
+      <c r="AJ39" s="13" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -4108,6 +4204,9 @@
       </c>
       <c r="AI40" s="13" t="n">
         <v>55.38</v>
+      </c>
+      <c r="AJ40" s="13" t="n">
+        <v>48.3</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -4168,6 +4267,9 @@
       <c r="AI41" s="13" t="n">
         <v>3302.8</v>
       </c>
+      <c r="AJ41" s="13" t="n">
+        <v>3247.03</v>
+      </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
       <c r="A42" s="3" t="n">
@@ -4253,6 +4355,7 @@
       <c r="AG42" s="13" t="n"/>
       <c r="AH42" s="13" t="n"/>
       <c r="AI42" s="13" t="n"/>
+      <c r="AJ42" s="13" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -4359,6 +4462,9 @@
       </c>
       <c r="AI43" s="13" t="n">
         <v>18.26</v>
+      </c>
+      <c r="AJ43" s="13" t="n">
+        <v>13.71</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -4419,6 +4525,9 @@
       <c r="AI44" s="13" t="n">
         <v>6923.32</v>
       </c>
+      <c r="AJ44" s="13" t="n">
+        <v>6700.07</v>
+      </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
       <c r="A45" s="3" t="n">
@@ -4504,6 +4613,7 @@
       <c r="AG45" s="13" t="n"/>
       <c r="AH45" s="13" t="n"/>
       <c r="AI45" s="13" t="n"/>
+      <c r="AJ45" s="13" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -4610,6 +4720,9 @@
       </c>
       <c r="AI46" s="13" t="n">
         <v>22.62</v>
+      </c>
+      <c r="AJ46" s="13" t="n">
+        <v>18.43</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -4670,6 +4783,9 @@
       <c r="AI47" s="13" t="n">
         <v>8069.33</v>
       </c>
+      <c r="AJ47" s="13" t="n">
+        <v>7898.82</v>
+      </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
       <c r="A48" s="3" t="n">
@@ -4755,6 +4871,7 @@
       <c r="AG48" s="13" t="n"/>
       <c r="AH48" s="13" t="n"/>
       <c r="AI48" s="13" t="n"/>
+      <c r="AJ48" s="13" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -4861,6 +4978,9 @@
       </c>
       <c r="AI49" s="13" t="n">
         <v>7.65</v>
+      </c>
+      <c r="AJ49" s="13" t="n">
+        <v>6.29</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -4921,6 +5041,9 @@
       <c r="AI50" s="13" t="n">
         <v>12172.05</v>
       </c>
+      <c r="AJ50" s="13" t="n">
+        <v>12045.88</v>
+      </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
       <c r="A51" s="3" t="n">
@@ -5006,6 +5129,7 @@
       <c r="AG51" s="13" t="n"/>
       <c r="AH51" s="13" t="n"/>
       <c r="AI51" s="13" t="n"/>
+      <c r="AJ51" s="13" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -5112,6 +5236,9 @@
       </c>
       <c r="AI52" s="13" t="n">
         <v>28.63</v>
+      </c>
+      <c r="AJ52" s="13" t="n">
+        <v>22.52</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -5172,6 +5299,9 @@
       <c r="AI53" s="13" t="n">
         <v>12727.06</v>
       </c>
+      <c r="AJ53" s="13" t="n">
+        <v>12404.95</v>
+      </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
       <c r="A54" s="3" t="n">
@@ -5257,6 +5387,7 @@
       <c r="AG54" s="13" t="n"/>
       <c r="AH54" s="13" t="n"/>
       <c r="AI54" s="13" t="n"/>
+      <c r="AJ54" s="13" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -5363,6 +5494,9 @@
       </c>
       <c r="AI55" s="13" t="n">
         <v>17.75</v>
+      </c>
+      <c r="AJ55" s="13" t="n">
+        <v>15.49</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -5423,6 +5557,9 @@
       <c r="AI56" s="13" t="n">
         <v>8277.93</v>
       </c>
+      <c r="AJ56" s="13" t="n">
+        <v>8034.34</v>
+      </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
       <c r="A57" s="3" t="n">
@@ -5508,6 +5645,7 @@
       <c r="AG57" s="13" t="n"/>
       <c r="AH57" s="13" t="n"/>
       <c r="AI57" s="13" t="n"/>
+      <c r="AJ57" s="13" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -5614,6 +5752,9 @@
       </c>
       <c r="AI58" s="13" t="n">
         <v>25.95</v>
+      </c>
+      <c r="AJ58" s="13" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -5674,6 +5815,9 @@
       <c r="AI59" s="13" t="n">
         <v>14772.64</v>
       </c>
+      <c r="AJ59" s="13" t="n">
+        <v>14562.36</v>
+      </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
       <c r="A60" s="3" t="n">
@@ -5759,6 +5903,7 @@
       <c r="AG60" s="13" t="n"/>
       <c r="AH60" s="13" t="n"/>
       <c r="AI60" s="13" t="n"/>
+      <c r="AJ60" s="13" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -5865,6 +6010,9 @@
       </c>
       <c r="AI61" s="13" t="n">
         <v>29.92</v>
+      </c>
+      <c r="AJ61" s="13" t="n">
+        <v>27.88</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -5925,6 +6073,9 @@
       <c r="AI62" s="13" t="n">
         <v>14774.52</v>
       </c>
+      <c r="AJ62" s="13" t="n">
+        <v>14190.38</v>
+      </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
       <c r="A63" s="3" t="n">
@@ -6010,6 +6161,7 @@
       <c r="AG63" s="13" t="n"/>
       <c r="AH63" s="13" t="n"/>
       <c r="AI63" s="13" t="n"/>
+      <c r="AJ63" s="13" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -6116,6 +6268,9 @@
       </c>
       <c r="AI64" s="13" t="n">
         <v>15.93</v>
+      </c>
+      <c r="AJ64" s="13" t="n">
+        <v>14.79</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -6176,6 +6331,9 @@
       <c r="AI65" s="13" t="n">
         <v>8178.68</v>
       </c>
+      <c r="AJ65" s="13" t="n">
+        <v>8010.64</v>
+      </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
       <c r="A66" s="3" t="n">
@@ -6261,6 +6419,7 @@
       <c r="AG66" s="13" t="n"/>
       <c r="AH66" s="13" t="n"/>
       <c r="AI66" s="13" t="n"/>
+      <c r="AJ66" s="13" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -6367,6 +6526,9 @@
       </c>
       <c r="AI67" s="13" t="n">
         <v>10.03</v>
+      </c>
+      <c r="AJ67" s="13" t="n">
+        <v>8.09</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -6427,6 +6589,9 @@
       <c r="AI68" s="13" t="n">
         <v>9474.83</v>
       </c>
+      <c r="AJ68" s="13" t="n">
+        <v>9309.690000000001</v>
+      </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
       <c r="A69" s="3" t="n">
@@ -6512,6 +6677,7 @@
       <c r="AG69" s="13" t="n"/>
       <c r="AH69" s="13" t="n"/>
       <c r="AI69" s="13" t="n"/>
+      <c r="AJ69" s="13" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -6618,6 +6784,9 @@
       </c>
       <c r="AI70" s="13" t="n">
         <v>19.81</v>
+      </c>
+      <c r="AJ70" s="13" t="n">
+        <v>18.05</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -6678,6 +6847,9 @@
       <c r="AI71" s="13" t="n">
         <v>2650.05</v>
       </c>
+      <c r="AJ71" s="13" t="n">
+        <v>2550.85</v>
+      </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
       <c r="A72" s="3" t="n">
@@ -6763,6 +6935,7 @@
       <c r="AG72" s="13" t="n"/>
       <c r="AH72" s="13" t="n"/>
       <c r="AI72" s="13" t="n"/>
+      <c r="AJ72" s="13" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -6869,6 +7042,9 @@
       </c>
       <c r="AI73" s="13" t="n">
         <v>37.64</v>
+      </c>
+      <c r="AJ73" s="13" t="n">
+        <v>33.52</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -6929,6 +7105,9 @@
       <c r="AI74" s="13" t="n">
         <v>5030.11</v>
       </c>
+      <c r="AJ74" s="13" t="n">
+        <v>4829.9</v>
+      </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
       <c r="A75" s="3" t="n">
@@ -7014,6 +7193,7 @@
       <c r="AG75" s="13" t="n"/>
       <c r="AH75" s="13" t="n"/>
       <c r="AI75" s="13" t="n"/>
+      <c r="AJ75" s="13" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -7120,6 +7300,9 @@
       </c>
       <c r="AI76" s="13" t="n">
         <v>21.57</v>
+      </c>
+      <c r="AJ76" s="13" t="n">
+        <v>16.71</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -7180,6 +7363,9 @@
       <c r="AI77" s="13" t="n">
         <v>8648.879999999999</v>
       </c>
+      <c r="AJ77" s="13" t="n">
+        <v>8441.200000000001</v>
+      </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
       <c r="A78" s="3" t="n">
@@ -7265,6 +7451,7 @@
       <c r="AG78" s="13" t="n"/>
       <c r="AH78" s="13" t="n"/>
       <c r="AI78" s="13" t="n"/>
+      <c r="AJ78" s="13" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -7371,6 +7558,9 @@
       </c>
       <c r="AI79" s="13" t="n">
         <v>17.02</v>
+      </c>
+      <c r="AJ79" s="13" t="n">
+        <v>16.61</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -7431,6 +7621,9 @@
       <c r="AI80" s="13" t="n">
         <v>1419.21</v>
       </c>
+      <c r="AJ80" s="13" t="n">
+        <v>1381.85</v>
+      </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
       <c r="A81" s="3" t="n">
@@ -7516,6 +7709,7 @@
       <c r="AG81" s="13" t="n"/>
       <c r="AH81" s="13" t="n"/>
       <c r="AI81" s="13" t="n"/>
+      <c r="AJ81" s="13" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -7622,6 +7816,9 @@
       </c>
       <c r="AI82" s="13" t="n">
         <v>15.29</v>
+      </c>
+      <c r="AJ82" s="13" t="n">
+        <v>13.63</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -7682,6 +7879,9 @@
       <c r="AI83" s="13" t="n">
         <v>16255.31</v>
       </c>
+      <c r="AJ83" s="13" t="n">
+        <v>15636.49</v>
+      </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
       <c r="A84" s="3" t="n">
@@ -7767,6 +7967,7 @@
       <c r="AG84" s="13" t="n"/>
       <c r="AH84" s="13" t="n"/>
       <c r="AI84" s="13" t="n"/>
+      <c r="AJ84" s="13" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -7873,6 +8074,9 @@
       </c>
       <c r="AI85" s="13" t="n">
         <v>54.2</v>
+      </c>
+      <c r="AJ85" s="13" t="n">
+        <v>54.27</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -7933,6 +8137,9 @@
       <c r="AI86" s="13" t="n">
         <v>3049.19</v>
       </c>
+      <c r="AJ86" s="13" t="n">
+        <v>3009.48</v>
+      </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
       <c r="A87" s="3" t="n">
@@ -8018,6 +8225,7 @@
       <c r="AG87" s="13" t="n"/>
       <c r="AH87" s="13" t="n"/>
       <c r="AI87" s="13" t="n"/>
+      <c r="AJ87" s="13" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -8124,6 +8332,9 @@
       </c>
       <c r="AI88" s="13" t="n">
         <v>57.59</v>
+      </c>
+      <c r="AJ88" s="13" t="n">
+        <v>58.66</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -8184,6 +8395,9 @@
       <c r="AI89" s="13" t="n">
         <v>3379.4</v>
       </c>
+      <c r="AJ89" s="13" t="n">
+        <v>3329.77</v>
+      </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
       <c r="A90" s="3" t="n">
@@ -8269,6 +8483,7 @@
       <c r="AG90" s="13" t="n"/>
       <c r="AH90" s="13" t="n"/>
       <c r="AI90" s="13" t="n"/>
+      <c r="AJ90" s="13" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -8375,6 +8590,9 @@
       </c>
       <c r="AI91" s="13" t="n">
         <v>49.56</v>
+      </c>
+      <c r="AJ91" s="13" t="n">
+        <v>48.41</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -8435,6 +8653,9 @@
       <c r="AI92" s="13" t="n">
         <v>3088.37</v>
       </c>
+      <c r="AJ92" s="13" t="n">
+        <v>2936.97</v>
+      </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
       <c r="A93" s="3" t="n">
@@ -8520,6 +8741,7 @@
       <c r="AG93" s="13" t="n"/>
       <c r="AH93" s="13" t="n"/>
       <c r="AI93" s="13" t="n"/>
+      <c r="AJ93" s="13" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -8626,6 +8848,9 @@
       </c>
       <c r="AI94" s="13" t="n">
         <v>38.18</v>
+      </c>
+      <c r="AJ94" s="13" t="n">
+        <v>29.98</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -8686,6 +8911,9 @@
       <c r="AI95" s="13" t="n">
         <v>1879.37</v>
       </c>
+      <c r="AJ95" s="13" t="n">
+        <v>1821.26</v>
+      </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
       <c r="A96" s="3" t="n">
@@ -8771,6 +8999,7 @@
       <c r="AG96" s="13" t="n"/>
       <c r="AH96" s="13" t="n"/>
       <c r="AI96" s="13" t="n"/>
+      <c r="AJ96" s="13" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -8877,6 +9106,9 @@
       </c>
       <c r="AI97" s="13" t="n">
         <v>26.84</v>
+      </c>
+      <c r="AJ97" s="13" t="n">
+        <v>25.51</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -8937,6 +9169,9 @@
       <c r="AI98" s="13" t="n">
         <v>10362.77</v>
       </c>
+      <c r="AJ98" s="13" t="n">
+        <v>9895.74</v>
+      </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
       <c r="A99" s="3" t="n">
@@ -9022,6 +9257,7 @@
       <c r="AG99" s="13" t="n"/>
       <c r="AH99" s="13" t="n"/>
       <c r="AI99" s="13" t="n"/>
+      <c r="AJ99" s="13" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -9128,6 +9364,9 @@
       </c>
       <c r="AI100" s="13" t="n">
         <v>87.66</v>
+      </c>
+      <c r="AJ100" s="13" t="n">
+        <v>84.81</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -9188,6 +9427,9 @@
       <c r="AI101" s="13" t="n">
         <v>10430.16</v>
       </c>
+      <c r="AJ101" s="13" t="n">
+        <v>10056.13</v>
+      </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
       <c r="A102" s="3" t="n">
@@ -9273,6 +9515,7 @@
       <c r="AG102" s="13" t="n"/>
       <c r="AH102" s="13" t="n"/>
       <c r="AI102" s="13" t="n"/>
+      <c r="AJ102" s="13" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -9379,6 +9622,9 @@
       </c>
       <c r="AI103" s="13" t="n">
         <v>60</v>
+      </c>
+      <c r="AJ103" s="13" t="n">
+        <v>59.67</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -9439,6 +9685,9 @@
       <c r="AI104" s="13" t="n">
         <v>16098.45</v>
       </c>
+      <c r="AJ104" s="13" t="n">
+        <v>15354.25</v>
+      </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
       <c r="A105" s="3" t="n">
@@ -9524,6 +9773,7 @@
       <c r="AG105" s="13" t="n"/>
       <c r="AH105" s="13" t="n"/>
       <c r="AI105" s="13" t="n"/>
+      <c r="AJ105" s="13" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -9630,6 +9880,9 @@
       </c>
       <c r="AI106" s="13" t="n">
         <v>8.539999999999999</v>
+      </c>
+      <c r="AJ106" s="13" t="n">
+        <v>8.529999999999999</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -9690,6 +9943,9 @@
       <c r="AI107" s="13" t="n">
         <v>2220.51</v>
       </c>
+      <c r="AJ107" s="13" t="n">
+        <v>2193.94</v>
+      </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
       <c r="A108" s="3" t="n">
@@ -9775,6 +10031,7 @@
       <c r="AG108" s="13" t="n"/>
       <c r="AH108" s="13" t="n"/>
       <c r="AI108" s="13" t="n"/>
+      <c r="AJ108" s="13" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -9881,6 +10138,9 @@
       </c>
       <c r="AI109" s="13" t="n">
         <v>24.93</v>
+      </c>
+      <c r="AJ109" s="13" t="n">
+        <v>24.31</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -9941,6 +10201,9 @@
       <c r="AI110" s="13" t="n">
         <v>809.76</v>
       </c>
+      <c r="AJ110" s="13" t="n">
+        <v>787.05</v>
+      </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
       <c r="A111" s="3" t="n">
@@ -10026,6 +10289,7 @@
       <c r="AG111" s="13" t="n"/>
       <c r="AH111" s="13" t="n"/>
       <c r="AI111" s="13" t="n"/>
+      <c r="AJ111" s="13" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -10132,6 +10396,9 @@
       </c>
       <c r="AI112" s="13" t="n">
         <v>33.79</v>
+      </c>
+      <c r="AJ112" s="13" t="n">
+        <v>33.7</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -10192,6 +10459,9 @@
       <c r="AI113" s="13" t="n">
         <v>3868.67</v>
       </c>
+      <c r="AJ113" s="13" t="n">
+        <v>3746.7</v>
+      </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
       <c r="A114" s="3" t="n">
@@ -10277,6 +10547,7 @@
       <c r="AG114" s="13" t="n"/>
       <c r="AH114" s="13" t="n"/>
       <c r="AI114" s="13" t="n"/>
+      <c r="AJ114" s="13" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -10383,6 +10654,9 @@
       </c>
       <c r="AI115" s="13" t="n">
         <v>23.26</v>
+      </c>
+      <c r="AJ115" s="13" t="n">
+        <v>21.95</v>
       </c>
     </row>
     <row r="116">
@@ -10428,6 +10702,9 @@
       <c r="AI116" s="13" t="n">
         <v>4210.94</v>
       </c>
+      <c r="AJ116" s="13" t="n">
+        <v>4141.59</v>
+      </c>
     </row>
     <row r="117">
       <c r="P117" s="13" t="n">
@@ -10468,6 +10745,7 @@
       <c r="AG117" s="13" t="n"/>
       <c r="AH117" s="13" t="n"/>
       <c r="AI117" s="13" t="n"/>
+      <c r="AJ117" s="13" t="n"/>
     </row>
     <row r="118">
       <c r="P118" s="13" t="n">
@@ -10530,6 +10808,9 @@
       <c r="AI118" s="13" t="n">
         <v>29.02</v>
       </c>
+      <c r="AJ118" s="13" t="n">
+        <v>29.02</v>
+      </c>
     </row>
     <row r="119">
       <c r="Y119" s="13" t="n">
@@ -10564,6 +10845,9 @@
       </c>
       <c r="AI119" s="13" t="n">
         <v>3078.01</v>
+      </c>
+      <c r="AJ119" s="13" t="n">
+        <v>2900.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-03-09 05:11:05]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ119"/>
+  <dimension ref="A1:AK119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="15"/>
@@ -553,6 +553,7 @@
     <col width="15" customWidth="1" min="34" max="34"/>
     <col width="15" customWidth="1" min="35" max="35"/>
     <col width="15" customWidth="1" min="36" max="36"/>
+    <col width="15" customWidth="1" min="37" max="37"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -736,6 +737,11 @@
           <t>2026/03/05</t>
         </is>
       </c>
+      <c r="AK1" s="13" t="inlineStr">
+        <is>
+          <t>2026/03/09</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -918,6 +924,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="AK2" s="14" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1028,6 +1039,9 @@
       <c r="AJ3" s="13" t="n">
         <v>68.06</v>
       </c>
+      <c r="AK3" s="13" t="n">
+        <v>69.54000000000001</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1137,6 +1151,9 @@
       </c>
       <c r="AJ4" s="13" t="n">
         <v>4116.77</v>
+      </c>
+      <c r="AK4" s="13" t="n">
+        <v>4087.48</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1176,6 +1193,7 @@
       <c r="AH5" s="13" t="n"/>
       <c r="AI5" s="13" t="n"/>
       <c r="AJ5" s="13" t="n"/>
+      <c r="AK5" s="13" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1262,6 +1280,7 @@
       <c r="AH6" s="13" t="n"/>
       <c r="AI6" s="13" t="n"/>
       <c r="AJ6" s="13" t="n"/>
+      <c r="AK6" s="13" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1371,6 +1390,9 @@
       </c>
       <c r="AJ7" s="13" t="n">
         <v>50.81</v>
+      </c>
+      <c r="AK7" s="13" t="n">
+        <v>51.1</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -1434,6 +1456,9 @@
       <c r="AJ8" s="13" t="n">
         <v>5863.71</v>
       </c>
+      <c r="AK8" s="13" t="n">
+        <v>5770.26</v>
+      </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -1520,6 +1545,7 @@
       <c r="AH9" s="13" t="n"/>
       <c r="AI9" s="13" t="n"/>
       <c r="AJ9" s="13" t="n"/>
+      <c r="AK9" s="13" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -1629,6 +1655,9 @@
       </c>
       <c r="AJ10" s="13" t="n">
         <v>53.68</v>
+      </c>
+      <c r="AK10" s="13" t="n">
+        <v>54.64</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -1692,6 +1721,9 @@
       <c r="AJ11" s="13" t="n">
         <v>4662.92</v>
       </c>
+      <c r="AK11" s="13" t="n">
+        <v>4595.27</v>
+      </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -1778,6 +1810,7 @@
       <c r="AH12" s="13" t="n"/>
       <c r="AI12" s="13" t="n"/>
       <c r="AJ12" s="13" t="n"/>
+      <c r="AK12" s="13" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -1887,6 +1920,9 @@
       </c>
       <c r="AJ13" s="13" t="n">
         <v>60.8</v>
+      </c>
+      <c r="AK13" s="13" t="n">
+        <v>61.08</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -1950,6 +1986,9 @@
       <c r="AJ14" s="13" t="n">
         <v>8346.25</v>
       </c>
+      <c r="AK14" s="13" t="n">
+        <v>8214.530000000001</v>
+      </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -2036,6 +2075,7 @@
       <c r="AH15" s="13" t="n"/>
       <c r="AI15" s="13" t="n"/>
       <c r="AJ15" s="13" t="n"/>
+      <c r="AK15" s="13" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -2145,6 +2185,9 @@
       </c>
       <c r="AJ16" s="13" t="n">
         <v>26.65</v>
+      </c>
+      <c r="AK16" s="13" t="n">
+        <v>27.44</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -2208,6 +2251,9 @@
       <c r="AJ17" s="13" t="n">
         <v>2629.32</v>
       </c>
+      <c r="AK17" s="13" t="n">
+        <v>2606.23</v>
+      </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="3" t="n">
@@ -2294,6 +2340,7 @@
       <c r="AH18" s="13" t="n"/>
       <c r="AI18" s="13" t="n"/>
       <c r="AJ18" s="13" t="n"/>
+      <c r="AK18" s="13" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -2403,6 +2450,9 @@
       </c>
       <c r="AJ19" s="13" t="n">
         <v>95.16</v>
+      </c>
+      <c r="AK19" s="13" t="n">
+        <v>94.33</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -2466,6 +2516,9 @@
       <c r="AJ20" s="13" t="n">
         <v>6869.5</v>
       </c>
+      <c r="AK20" s="13" t="n">
+        <v>6740.02</v>
+      </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -2552,6 +2605,7 @@
       <c r="AH21" s="13" t="n"/>
       <c r="AI21" s="13" t="n"/>
       <c r="AJ21" s="13" t="n"/>
+      <c r="AK21" s="13" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -2659,6 +2713,9 @@
       </c>
       <c r="AJ22" s="13" t="n">
         <v>54.48</v>
+      </c>
+      <c r="AK22" s="13" t="n">
+        <v>54.34</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1">
@@ -2722,6 +2779,9 @@
       <c r="AJ23" s="13" t="n">
         <v>79463.50999999999</v>
       </c>
+      <c r="AK23" s="13" t="n">
+        <v>76741.48</v>
+      </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="3" t="n">
@@ -2808,6 +2868,7 @@
       <c r="AH24" s="13" t="n"/>
       <c r="AI24" s="13" t="n"/>
       <c r="AJ24" s="13" t="n"/>
+      <c r="AK24" s="13" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -2916,6 +2977,9 @@
         <v>87.75</v>
       </c>
       <c r="AJ25" s="13" t="n">
+        <v>77.13</v>
+      </c>
+      <c r="AK25" s="13" t="n">
         <v>77.13</v>
       </c>
     </row>
@@ -2980,6 +3044,9 @@
       <c r="AJ26" s="13" t="n">
         <v>24205.36</v>
       </c>
+      <c r="AK26" s="13" t="n">
+        <v>23591.03</v>
+      </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -3066,6 +3133,7 @@
       <c r="AH27" s="13" t="n"/>
       <c r="AI27" s="13" t="n"/>
       <c r="AJ27" s="13" t="n"/>
+      <c r="AK27" s="13" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -3175,6 +3243,9 @@
       </c>
       <c r="AJ28" s="13" t="n">
         <v>75.56</v>
+      </c>
+      <c r="AK28" s="13" t="n">
+        <v>73.62</v>
       </c>
     </row>
     <row r="29" ht="14.25" customHeight="1">
@@ -3238,6 +3309,9 @@
       <c r="AJ29" s="13" t="n">
         <v>55673.59</v>
       </c>
+      <c r="AK29" s="13" t="n">
+        <v>51961.41</v>
+      </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="3" t="n">
@@ -3324,6 +3398,7 @@
       <c r="AH30" s="13" t="n"/>
       <c r="AI30" s="13" t="n"/>
       <c r="AJ30" s="13" t="n"/>
+      <c r="AK30" s="13" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -3433,6 +3508,9 @@
       </c>
       <c r="AJ31" s="13" t="n">
         <v>51.62</v>
+      </c>
+      <c r="AK31" s="13" t="n">
+        <v>51.74</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -3496,6 +3574,9 @@
       <c r="AJ32" s="13" t="n">
         <v>5842.72</v>
       </c>
+      <c r="AK32" s="13" t="n">
+        <v>5897.58</v>
+      </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
       <c r="A33" s="3" t="n">
@@ -3582,6 +3663,7 @@
       <c r="AH33" s="13" t="n"/>
       <c r="AI33" s="13" t="n"/>
       <c r="AJ33" s="13" t="n"/>
+      <c r="AK33" s="13" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -3691,6 +3773,9 @@
       </c>
       <c r="AJ34" s="13" t="n">
         <v>2.26</v>
+      </c>
+      <c r="AK34" s="13" t="n">
+        <v>2.37</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -3754,6 +3839,9 @@
       <c r="AJ35" s="13" t="n">
         <v>33320.04</v>
       </c>
+      <c r="AK35" s="13" t="n">
+        <v>33497.5</v>
+      </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="3" t="n">
@@ -3840,6 +3928,7 @@
       <c r="AH36" s="13" t="n"/>
       <c r="AI36" s="13" t="n"/>
       <c r="AJ36" s="13" t="n"/>
+      <c r="AK36" s="13" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -3949,6 +4038,9 @@
       </c>
       <c r="AJ37" s="13" t="n">
         <v>28.91</v>
+      </c>
+      <c r="AK37" s="13" t="n">
+        <v>29.76</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -4012,6 +4104,9 @@
       <c r="AJ38" s="13" t="n">
         <v>3402.4</v>
       </c>
+      <c r="AK38" s="13" t="n">
+        <v>3303.71</v>
+      </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
       <c r="A39" s="3" t="n">
@@ -4098,6 +4193,7 @@
       <c r="AH39" s="13" t="n"/>
       <c r="AI39" s="13" t="n"/>
       <c r="AJ39" s="13" t="n"/>
+      <c r="AK39" s="13" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -4207,6 +4303,9 @@
       </c>
       <c r="AJ40" s="13" t="n">
         <v>48.3</v>
+      </c>
+      <c r="AK40" s="13" t="n">
+        <v>50.05</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -4270,6 +4369,9 @@
       <c r="AJ41" s="13" t="n">
         <v>3247.03</v>
       </c>
+      <c r="AK41" s="13" t="n">
+        <v>3164.02</v>
+      </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
       <c r="A42" s="3" t="n">
@@ -4356,6 +4458,7 @@
       <c r="AH42" s="13" t="n"/>
       <c r="AI42" s="13" t="n"/>
       <c r="AJ42" s="13" t="n"/>
+      <c r="AK42" s="13" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -4465,6 +4568,9 @@
       </c>
       <c r="AJ43" s="13" t="n">
         <v>13.71</v>
+      </c>
+      <c r="AK43" s="13" t="n">
+        <v>15.2</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -4528,6 +4634,9 @@
       <c r="AJ44" s="13" t="n">
         <v>6700.07</v>
       </c>
+      <c r="AK44" s="13" t="n">
+        <v>6686.41</v>
+      </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
       <c r="A45" s="3" t="n">
@@ -4614,6 +4723,7 @@
       <c r="AH45" s="13" t="n"/>
       <c r="AI45" s="13" t="n"/>
       <c r="AJ45" s="13" t="n"/>
+      <c r="AK45" s="13" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -4723,6 +4833,9 @@
       </c>
       <c r="AJ46" s="13" t="n">
         <v>18.43</v>
+      </c>
+      <c r="AK46" s="13" t="n">
+        <v>21.11</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -4786,6 +4899,9 @@
       <c r="AJ47" s="13" t="n">
         <v>7898.82</v>
       </c>
+      <c r="AK47" s="13" t="n">
+        <v>7956.86</v>
+      </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
       <c r="A48" s="3" t="n">
@@ -4872,6 +4988,7 @@
       <c r="AH48" s="13" t="n"/>
       <c r="AI48" s="13" t="n"/>
       <c r="AJ48" s="13" t="n"/>
+      <c r="AK48" s="13" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -4981,6 +5098,9 @@
       </c>
       <c r="AJ49" s="13" t="n">
         <v>6.29</v>
+      </c>
+      <c r="AK49" s="13" t="n">
+        <v>6.65</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -5044,6 +5164,9 @@
       <c r="AJ50" s="13" t="n">
         <v>12045.88</v>
       </c>
+      <c r="AK50" s="13" t="n">
+        <v>12073.76</v>
+      </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
       <c r="A51" s="3" t="n">
@@ -5130,6 +5253,7 @@
       <c r="AH51" s="13" t="n"/>
       <c r="AI51" s="13" t="n"/>
       <c r="AJ51" s="13" t="n"/>
+      <c r="AK51" s="13" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -5239,6 +5363,9 @@
       </c>
       <c r="AJ52" s="13" t="n">
         <v>22.52</v>
+      </c>
+      <c r="AK52" s="13" t="n">
+        <v>24.57</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -5302,6 +5429,9 @@
       <c r="AJ53" s="13" t="n">
         <v>12404.95</v>
       </c>
+      <c r="AK53" s="13" t="n">
+        <v>12404.95</v>
+      </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
       <c r="A54" s="3" t="n">
@@ -5388,6 +5518,7 @@
       <c r="AH54" s="13" t="n"/>
       <c r="AI54" s="13" t="n"/>
       <c r="AJ54" s="13" t="n"/>
+      <c r="AK54" s="13" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -5497,6 +5628,9 @@
       </c>
       <c r="AJ55" s="13" t="n">
         <v>15.49</v>
+      </c>
+      <c r="AK55" s="13" t="n">
+        <v>15.91</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -5560,6 +5694,9 @@
       <c r="AJ56" s="13" t="n">
         <v>8034.34</v>
       </c>
+      <c r="AK56" s="13" t="n">
+        <v>8062.54</v>
+      </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
       <c r="A57" s="3" t="n">
@@ -5646,6 +5783,7 @@
       <c r="AH57" s="13" t="n"/>
       <c r="AI57" s="13" t="n"/>
       <c r="AJ57" s="13" t="n"/>
+      <c r="AK57" s="13" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -5755,6 +5893,9 @@
       </c>
       <c r="AJ58" s="13" t="n">
         <v>24</v>
+      </c>
+      <c r="AK58" s="13" t="n">
+        <v>25.04</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -5818,6 +5959,9 @@
       <c r="AJ59" s="13" t="n">
         <v>14562.36</v>
       </c>
+      <c r="AK59" s="13" t="n">
+        <v>14896.72</v>
+      </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
       <c r="A60" s="3" t="n">
@@ -5904,6 +6048,7 @@
       <c r="AH60" s="13" t="n"/>
       <c r="AI60" s="13" t="n"/>
       <c r="AJ60" s="13" t="n"/>
+      <c r="AK60" s="13" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -6013,6 +6158,9 @@
       </c>
       <c r="AJ61" s="13" t="n">
         <v>27.88</v>
+      </c>
+      <c r="AK61" s="13" t="n">
+        <v>29.33</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -6076,6 +6224,9 @@
       <c r="AJ62" s="13" t="n">
         <v>14190.38</v>
       </c>
+      <c r="AK62" s="13" t="n">
+        <v>14020.75</v>
+      </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
       <c r="A63" s="3" t="n">
@@ -6162,6 +6313,7 @@
       <c r="AH63" s="13" t="n"/>
       <c r="AI63" s="13" t="n"/>
       <c r="AJ63" s="13" t="n"/>
+      <c r="AK63" s="13" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -6271,6 +6423,9 @@
       </c>
       <c r="AJ64" s="13" t="n">
         <v>14.79</v>
+      </c>
+      <c r="AK64" s="13" t="n">
+        <v>15.52</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -6334,6 +6489,9 @@
       <c r="AJ65" s="13" t="n">
         <v>8010.64</v>
       </c>
+      <c r="AK65" s="13" t="n">
+        <v>7890.88</v>
+      </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
       <c r="A66" s="3" t="n">
@@ -6420,6 +6578,7 @@
       <c r="AH66" s="13" t="n"/>
       <c r="AI66" s="13" t="n"/>
       <c r="AJ66" s="13" t="n"/>
+      <c r="AK66" s="13" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -6529,6 +6688,9 @@
       </c>
       <c r="AJ67" s="13" t="n">
         <v>8.09</v>
+      </c>
+      <c r="AK67" s="13" t="n">
+        <v>8.93</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -6592,6 +6754,9 @@
       <c r="AJ68" s="13" t="n">
         <v>9309.690000000001</v>
       </c>
+      <c r="AK68" s="13" t="n">
+        <v>9369.9</v>
+      </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
       <c r="A69" s="3" t="n">
@@ -6678,6 +6843,7 @@
       <c r="AH69" s="13" t="n"/>
       <c r="AI69" s="13" t="n"/>
       <c r="AJ69" s="13" t="n"/>
+      <c r="AK69" s="13" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -6787,6 +6953,9 @@
       </c>
       <c r="AJ70" s="13" t="n">
         <v>18.05</v>
+      </c>
+      <c r="AK70" s="13" t="n">
+        <v>19.75</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -6850,6 +7019,9 @@
       <c r="AJ71" s="13" t="n">
         <v>2550.85</v>
       </c>
+      <c r="AK71" s="13" t="n">
+        <v>2546.26</v>
+      </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
       <c r="A72" s="3" t="n">
@@ -6936,6 +7108,7 @@
       <c r="AH72" s="13" t="n"/>
       <c r="AI72" s="13" t="n"/>
       <c r="AJ72" s="13" t="n"/>
+      <c r="AK72" s="13" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -7045,6 +7218,9 @@
       </c>
       <c r="AJ73" s="13" t="n">
         <v>33.52</v>
+      </c>
+      <c r="AK73" s="13" t="n">
+        <v>36.53</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -7108,6 +7284,9 @@
       <c r="AJ74" s="13" t="n">
         <v>4829.9</v>
       </c>
+      <c r="AK74" s="13" t="n">
+        <v>4832.36</v>
+      </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
       <c r="A75" s="3" t="n">
@@ -7194,6 +7373,7 @@
       <c r="AH75" s="13" t="n"/>
       <c r="AI75" s="13" t="n"/>
       <c r="AJ75" s="13" t="n"/>
+      <c r="AK75" s="13" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -7303,6 +7483,9 @@
       </c>
       <c r="AJ76" s="13" t="n">
         <v>16.71</v>
+      </c>
+      <c r="AK76" s="13" t="n">
+        <v>19.62</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -7366,6 +7549,9 @@
       <c r="AJ77" s="13" t="n">
         <v>8441.200000000001</v>
       </c>
+      <c r="AK77" s="13" t="n">
+        <v>8499.879999999999</v>
+      </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
       <c r="A78" s="3" t="n">
@@ -7452,6 +7638,7 @@
       <c r="AH78" s="13" t="n"/>
       <c r="AI78" s="13" t="n"/>
       <c r="AJ78" s="13" t="n"/>
+      <c r="AK78" s="13" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -7561,6 +7748,9 @@
       </c>
       <c r="AJ79" s="13" t="n">
         <v>16.61</v>
+      </c>
+      <c r="AK79" s="13" t="n">
+        <v>16.8</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -7624,6 +7814,9 @@
       <c r="AJ80" s="13" t="n">
         <v>1381.85</v>
       </c>
+      <c r="AK80" s="13" t="n">
+        <v>1398.81</v>
+      </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
       <c r="A81" s="3" t="n">
@@ -7710,6 +7903,7 @@
       <c r="AH81" s="13" t="n"/>
       <c r="AI81" s="13" t="n"/>
       <c r="AJ81" s="13" t="n"/>
+      <c r="AK81" s="13" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -7819,6 +8013,9 @@
       </c>
       <c r="AJ82" s="13" t="n">
         <v>13.63</v>
+      </c>
+      <c r="AK82" s="13" t="n">
+        <v>13.91</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -7882,6 +8079,9 @@
       <c r="AJ83" s="13" t="n">
         <v>15636.49</v>
       </c>
+      <c r="AK83" s="13" t="n">
+        <v>15852.88</v>
+      </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
       <c r="A84" s="3" t="n">
@@ -7968,6 +8168,7 @@
       <c r="AH84" s="13" t="n"/>
       <c r="AI84" s="13" t="n"/>
       <c r="AJ84" s="13" t="n"/>
+      <c r="AK84" s="13" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -8077,6 +8278,9 @@
       </c>
       <c r="AJ85" s="13" t="n">
         <v>54.27</v>
+      </c>
+      <c r="AK85" s="13" t="n">
+        <v>54.64</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -8140,6 +8344,9 @@
       <c r="AJ86" s="13" t="n">
         <v>3009.48</v>
       </c>
+      <c r="AK86" s="13" t="n">
+        <v>3029.24</v>
+      </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
       <c r="A87" s="3" t="n">
@@ -8226,6 +8433,7 @@
       <c r="AH87" s="13" t="n"/>
       <c r="AI87" s="13" t="n"/>
       <c r="AJ87" s="13" t="n"/>
+      <c r="AK87" s="13" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -8335,6 +8543,9 @@
       </c>
       <c r="AJ88" s="13" t="n">
         <v>58.66</v>
+      </c>
+      <c r="AK88" s="13" t="n">
+        <v>58.69</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -8398,6 +8609,9 @@
       <c r="AJ89" s="13" t="n">
         <v>3329.77</v>
       </c>
+      <c r="AK89" s="13" t="n">
+        <v>3396.3</v>
+      </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
       <c r="A90" s="3" t="n">
@@ -8484,6 +8698,7 @@
       <c r="AH90" s="13" t="n"/>
       <c r="AI90" s="13" t="n"/>
       <c r="AJ90" s="13" t="n"/>
+      <c r="AK90" s="13" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -8593,6 +8808,9 @@
       </c>
       <c r="AJ91" s="13" t="n">
         <v>48.41</v>
+      </c>
+      <c r="AK91" s="13" t="n">
+        <v>48.73</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -8656,6 +8874,9 @@
       <c r="AJ92" s="13" t="n">
         <v>2936.97</v>
       </c>
+      <c r="AK92" s="13" t="n">
+        <v>2927.73</v>
+      </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
       <c r="A93" s="3" t="n">
@@ -8742,6 +8963,7 @@
       <c r="AH93" s="13" t="n"/>
       <c r="AI93" s="13" t="n"/>
       <c r="AJ93" s="13" t="n"/>
+      <c r="AK93" s="13" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -8851,6 +9073,9 @@
       </c>
       <c r="AJ94" s="13" t="n">
         <v>29.98</v>
+      </c>
+      <c r="AK94" s="13" t="n">
+        <v>33.77</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -8914,6 +9139,9 @@
       <c r="AJ95" s="13" t="n">
         <v>1821.26</v>
       </c>
+      <c r="AK95" s="13" t="n">
+        <v>1794.2</v>
+      </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
       <c r="A96" s="3" t="n">
@@ -9000,6 +9228,7 @@
       <c r="AH96" s="13" t="n"/>
       <c r="AI96" s="13" t="n"/>
       <c r="AJ96" s="13" t="n"/>
+      <c r="AK96" s="13" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -9109,6 +9338,9 @@
       </c>
       <c r="AJ97" s="13" t="n">
         <v>25.51</v>
+      </c>
+      <c r="AK97" s="13" t="n">
+        <v>26.49</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -9172,6 +9404,9 @@
       <c r="AJ98" s="13" t="n">
         <v>9895.74</v>
       </c>
+      <c r="AK98" s="13" t="n">
+        <v>9934.41</v>
+      </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
       <c r="A99" s="3" t="n">
@@ -9258,6 +9493,7 @@
       <c r="AH99" s="13" t="n"/>
       <c r="AI99" s="13" t="n"/>
       <c r="AJ99" s="13" t="n"/>
+      <c r="AK99" s="13" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -9367,6 +9603,9 @@
       </c>
       <c r="AJ100" s="13" t="n">
         <v>84.81</v>
+      </c>
+      <c r="AK100" s="13" t="n">
+        <v>85.68000000000001</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -9430,6 +9669,9 @@
       <c r="AJ101" s="13" t="n">
         <v>10056.13</v>
       </c>
+      <c r="AK101" s="13" t="n">
+        <v>9627.27</v>
+      </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
       <c r="A102" s="3" t="n">
@@ -9516,6 +9758,7 @@
       <c r="AH102" s="13" t="n"/>
       <c r="AI102" s="13" t="n"/>
       <c r="AJ102" s="13" t="n"/>
+      <c r="AK102" s="13" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -9625,6 +9868,9 @@
       </c>
       <c r="AJ103" s="13" t="n">
         <v>59.67</v>
+      </c>
+      <c r="AK103" s="13" t="n">
+        <v>59.83</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -9688,6 +9934,9 @@
       <c r="AJ104" s="13" t="n">
         <v>15354.25</v>
       </c>
+      <c r="AK104" s="13" t="n">
+        <v>15202</v>
+      </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
       <c r="A105" s="3" t="n">
@@ -9774,6 +10023,7 @@
       <c r="AH105" s="13" t="n"/>
       <c r="AI105" s="13" t="n"/>
       <c r="AJ105" s="13" t="n"/>
+      <c r="AK105" s="13" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -9883,6 +10133,9 @@
       </c>
       <c r="AJ106" s="13" t="n">
         <v>8.529999999999999</v>
+      </c>
+      <c r="AK106" s="13" t="n">
+        <v>9.81</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -9946,6 +10199,9 @@
       <c r="AJ107" s="13" t="n">
         <v>2193.94</v>
       </c>
+      <c r="AK107" s="13" t="n">
+        <v>2274.7</v>
+      </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
       <c r="A108" s="3" t="n">
@@ -10032,6 +10288,7 @@
       <c r="AH108" s="13" t="n"/>
       <c r="AI108" s="13" t="n"/>
       <c r="AJ108" s="13" t="n"/>
+      <c r="AK108" s="13" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -10141,6 +10398,9 @@
       </c>
       <c r="AJ109" s="13" t="n">
         <v>24.31</v>
+      </c>
+      <c r="AK109" s="13" t="n">
+        <v>24.52</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -10204,6 +10464,9 @@
       <c r="AJ110" s="13" t="n">
         <v>787.05</v>
       </c>
+      <c r="AK110" s="13" t="n">
+        <v>781.02</v>
+      </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
       <c r="A111" s="3" t="n">
@@ -10290,6 +10553,7 @@
       <c r="AH111" s="13" t="n"/>
       <c r="AI111" s="13" t="n"/>
       <c r="AJ111" s="13" t="n"/>
+      <c r="AK111" s="13" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -10399,6 +10663,9 @@
       </c>
       <c r="AJ112" s="13" t="n">
         <v>33.7</v>
+      </c>
+      <c r="AK112" s="13" t="n">
+        <v>33.41</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -10462,6 +10729,9 @@
       <c r="AJ113" s="13" t="n">
         <v>3746.7</v>
       </c>
+      <c r="AK113" s="13" t="n">
+        <v>3658.46</v>
+      </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
       <c r="A114" s="3" t="n">
@@ -10548,6 +10818,7 @@
       <c r="AH114" s="13" t="n"/>
       <c r="AI114" s="13" t="n"/>
       <c r="AJ114" s="13" t="n"/>
+      <c r="AK114" s="13" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -10657,6 +10928,9 @@
       </c>
       <c r="AJ115" s="13" t="n">
         <v>21.95</v>
+      </c>
+      <c r="AK115" s="13" t="n">
+        <v>23.28</v>
       </c>
     </row>
     <row r="116">
@@ -10705,6 +10979,9 @@
       <c r="AJ116" s="13" t="n">
         <v>4141.59</v>
       </c>
+      <c r="AK116" s="13" t="n">
+        <v>4165.85</v>
+      </c>
     </row>
     <row r="117">
       <c r="P117" s="13" t="n">
@@ -10746,6 +11023,7 @@
       <c r="AH117" s="13" t="n"/>
       <c r="AI117" s="13" t="n"/>
       <c r="AJ117" s="13" t="n"/>
+      <c r="AK117" s="13" t="n"/>
     </row>
     <row r="118">
       <c r="P118" s="13" t="n">
@@ -10811,6 +11089,9 @@
       <c r="AJ118" s="13" t="n">
         <v>29.02</v>
       </c>
+      <c r="AK118" s="13" t="n">
+        <v>29.02</v>
+      </c>
     </row>
     <row r="119">
       <c r="Y119" s="13" t="n">
@@ -10848,6 +11129,9 @@
       </c>
       <c r="AJ119" s="13" t="n">
         <v>2900.3</v>
+      </c>
+      <c r="AK119" s="13" t="n">
+        <v>2879.13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-03-16 05:31:00]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK119"/>
+  <dimension ref="A1:AL119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="15"/>
@@ -554,6 +554,7 @@
     <col width="15" customWidth="1" min="35" max="35"/>
     <col width="15" customWidth="1" min="36" max="36"/>
     <col width="15" customWidth="1" min="37" max="37"/>
+    <col width="15" customWidth="1" min="38" max="38"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -742,6 +743,11 @@
           <t>2026/03/09</t>
         </is>
       </c>
+      <c r="AL1" s="13" t="inlineStr">
+        <is>
+          <t>2026/03/16</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -929,6 +935,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="AL2" s="14" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1042,6 +1053,9 @@
       <c r="AK3" s="13" t="n">
         <v>69.54000000000001</v>
       </c>
+      <c r="AL3" s="13" t="n">
+        <v>69.7</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1154,6 +1168,9 @@
       </c>
       <c r="AK4" s="13" t="n">
         <v>4087.48</v>
+      </c>
+      <c r="AL4" s="13" t="n">
+        <v>4079.72</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1194,6 +1211,7 @@
       <c r="AI5" s="13" t="n"/>
       <c r="AJ5" s="13" t="n"/>
       <c r="AK5" s="13" t="n"/>
+      <c r="AL5" s="13" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1281,6 +1299,7 @@
       <c r="AI6" s="13" t="n"/>
       <c r="AJ6" s="13" t="n"/>
       <c r="AK6" s="13" t="n"/>
+      <c r="AL6" s="13" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1393,6 +1412,9 @@
       </c>
       <c r="AK7" s="13" t="n">
         <v>51.1</v>
+      </c>
+      <c r="AL7" s="13" t="n">
+        <v>50.89</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -1459,6 +1481,9 @@
       <c r="AK8" s="13" t="n">
         <v>5770.26</v>
       </c>
+      <c r="AL8" s="13" t="n">
+        <v>5820.14</v>
+      </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -1546,6 +1571,7 @@
       <c r="AI9" s="13" t="n"/>
       <c r="AJ9" s="13" t="n"/>
       <c r="AK9" s="13" t="n"/>
+      <c r="AL9" s="13" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -1658,6 +1684,9 @@
       </c>
       <c r="AK10" s="13" t="n">
         <v>54.64</v>
+      </c>
+      <c r="AL10" s="13" t="n">
+        <v>54.66</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -1724,6 +1753,9 @@
       <c r="AK11" s="13" t="n">
         <v>4595.27</v>
       </c>
+      <c r="AL11" s="13" t="n">
+        <v>4658.8</v>
+      </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -1811,6 +1843,7 @@
       <c r="AI12" s="13" t="n"/>
       <c r="AJ12" s="13" t="n"/>
       <c r="AK12" s="13" t="n"/>
+      <c r="AL12" s="13" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -1923,6 +1956,9 @@
       </c>
       <c r="AK13" s="13" t="n">
         <v>61.08</v>
+      </c>
+      <c r="AL13" s="13" t="n">
+        <v>60.76</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -1989,6 +2025,9 @@
       <c r="AK14" s="13" t="n">
         <v>8214.530000000001</v>
       </c>
+      <c r="AL14" s="13" t="n">
+        <v>8174.9</v>
+      </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -2076,6 +2115,7 @@
       <c r="AI15" s="13" t="n"/>
       <c r="AJ15" s="13" t="n"/>
       <c r="AK15" s="13" t="n"/>
+      <c r="AL15" s="13" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -2188,6 +2228,9 @@
       </c>
       <c r="AK16" s="13" t="n">
         <v>27.44</v>
+      </c>
+      <c r="AL16" s="13" t="n">
+        <v>27.71</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -2254,6 +2297,9 @@
       <c r="AK17" s="13" t="n">
         <v>2606.23</v>
       </c>
+      <c r="AL17" s="13" t="n">
+        <v>2652.96</v>
+      </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="3" t="n">
@@ -2341,6 +2387,7 @@
       <c r="AI18" s="13" t="n"/>
       <c r="AJ18" s="13" t="n"/>
       <c r="AK18" s="13" t="n"/>
+      <c r="AL18" s="13" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -2453,6 +2500,9 @@
       </c>
       <c r="AK19" s="13" t="n">
         <v>94.33</v>
+      </c>
+      <c r="AL19" s="13" t="n">
+        <v>93.73999999999999</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -2519,6 +2569,9 @@
       <c r="AK20" s="13" t="n">
         <v>6740.02</v>
       </c>
+      <c r="AL20" s="13" t="n">
+        <v>6632.19</v>
+      </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -2606,6 +2659,7 @@
       <c r="AI21" s="13" t="n"/>
       <c r="AJ21" s="13" t="n"/>
       <c r="AK21" s="13" t="n"/>
+      <c r="AL21" s="13" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -2716,6 +2770,9 @@
       </c>
       <c r="AK22" s="13" t="n">
         <v>54.34</v>
+      </c>
+      <c r="AL22" s="13" t="n">
+        <v>52.51</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1">
@@ -2782,6 +2839,9 @@
       <c r="AK23" s="13" t="n">
         <v>76741.48</v>
       </c>
+      <c r="AL23" s="13" t="n">
+        <v>74278.63</v>
+      </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="3" t="n">
@@ -2869,6 +2929,7 @@
       <c r="AI24" s="13" t="n"/>
       <c r="AJ24" s="13" t="n"/>
       <c r="AK24" s="13" t="n"/>
+      <c r="AL24" s="13" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -2981,6 +3042,9 @@
       </c>
       <c r="AK25" s="13" t="n">
         <v>77.13</v>
+      </c>
+      <c r="AL25" s="13" t="n">
+        <v>78.75</v>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="1">
@@ -3047,6 +3111,9 @@
       <c r="AK26" s="13" t="n">
         <v>23591.03</v>
       </c>
+      <c r="AL26" s="13" t="n">
+        <v>23447.29</v>
+      </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -3134,6 +3201,7 @@
       <c r="AI27" s="13" t="n"/>
       <c r="AJ27" s="13" t="n"/>
       <c r="AK27" s="13" t="n"/>
+      <c r="AL27" s="13" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -3246,6 +3314,9 @@
       </c>
       <c r="AK28" s="13" t="n">
         <v>73.62</v>
+      </c>
+      <c r="AL28" s="13" t="n">
+        <v>71.06</v>
       </c>
     </row>
     <row r="29" ht="14.25" customHeight="1">
@@ -3312,6 +3383,9 @@
       <c r="AK29" s="13" t="n">
         <v>51961.41</v>
       </c>
+      <c r="AL29" s="13" t="n">
+        <v>53436.04</v>
+      </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="3" t="n">
@@ -3399,6 +3473,7 @@
       <c r="AI30" s="13" t="n"/>
       <c r="AJ30" s="13" t="n"/>
       <c r="AK30" s="13" t="n"/>
+      <c r="AL30" s="13" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -3511,6 +3586,9 @@
       </c>
       <c r="AK31" s="13" t="n">
         <v>51.74</v>
+      </c>
+      <c r="AL31" s="13" t="n">
+        <v>51.96</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -3577,6 +3655,9 @@
       <c r="AK32" s="13" t="n">
         <v>5897.58</v>
       </c>
+      <c r="AL32" s="13" t="n">
+        <v>5909.4</v>
+      </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
       <c r="A33" s="3" t="n">
@@ -3664,6 +3745,7 @@
       <c r="AI33" s="13" t="n"/>
       <c r="AJ33" s="13" t="n"/>
       <c r="AK33" s="13" t="n"/>
+      <c r="AL33" s="13" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -3776,6 +3858,9 @@
       </c>
       <c r="AK34" s="13" t="n">
         <v>2.37</v>
+      </c>
+      <c r="AL34" s="13" t="n">
+        <v>2.86</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -3842,6 +3927,9 @@
       <c r="AK35" s="13" t="n">
         <v>33497.5</v>
       </c>
+      <c r="AL35" s="13" t="n">
+        <v>33463.01</v>
+      </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="3" t="n">
@@ -3929,6 +4017,7 @@
       <c r="AI36" s="13" t="n"/>
       <c r="AJ36" s="13" t="n"/>
       <c r="AK36" s="13" t="n"/>
+      <c r="AL36" s="13" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -4041,6 +4130,9 @@
       </c>
       <c r="AK37" s="13" t="n">
         <v>29.76</v>
+      </c>
+      <c r="AL37" s="13" t="n">
+        <v>28.36</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -4107,6 +4199,9 @@
       <c r="AK38" s="13" t="n">
         <v>3303.71</v>
       </c>
+      <c r="AL38" s="13" t="n">
+        <v>3501.16</v>
+      </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
       <c r="A39" s="3" t="n">
@@ -4194,6 +4289,7 @@
       <c r="AI39" s="13" t="n"/>
       <c r="AJ39" s="13" t="n"/>
       <c r="AK39" s="13" t="n"/>
+      <c r="AL39" s="13" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -4306,6 +4402,9 @@
       </c>
       <c r="AK40" s="13" t="n">
         <v>50.05</v>
+      </c>
+      <c r="AL40" s="13" t="n">
+        <v>48.92</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -4372,6 +4471,9 @@
       <c r="AK41" s="13" t="n">
         <v>3164.02</v>
       </c>
+      <c r="AL41" s="13" t="n">
+        <v>3338.53</v>
+      </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
       <c r="A42" s="3" t="n">
@@ -4459,6 +4561,7 @@
       <c r="AI42" s="13" t="n"/>
       <c r="AJ42" s="13" t="n"/>
       <c r="AK42" s="13" t="n"/>
+      <c r="AL42" s="13" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -4571,6 +4674,9 @@
       </c>
       <c r="AK43" s="13" t="n">
         <v>15.2</v>
+      </c>
+      <c r="AL43" s="13" t="n">
+        <v>14.71</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -4637,6 +4743,9 @@
       <c r="AK44" s="13" t="n">
         <v>6686.41</v>
       </c>
+      <c r="AL44" s="13" t="n">
+        <v>6735.52</v>
+      </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
       <c r="A45" s="3" t="n">
@@ -4724,6 +4833,7 @@
       <c r="AI45" s="13" t="n"/>
       <c r="AJ45" s="13" t="n"/>
       <c r="AK45" s="13" t="n"/>
+      <c r="AL45" s="13" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -4836,6 +4946,9 @@
       </c>
       <c r="AK46" s="13" t="n">
         <v>21.11</v>
+      </c>
+      <c r="AL46" s="13" t="n">
+        <v>20.46</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -4902,6 +5015,9 @@
       <c r="AK47" s="13" t="n">
         <v>7956.86</v>
       </c>
+      <c r="AL47" s="13" t="n">
+        <v>7990.9</v>
+      </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
       <c r="A48" s="3" t="n">
@@ -4989,6 +5105,7 @@
       <c r="AI48" s="13" t="n"/>
       <c r="AJ48" s="13" t="n"/>
       <c r="AK48" s="13" t="n"/>
+      <c r="AL48" s="13" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -5101,6 +5218,9 @@
       </c>
       <c r="AK49" s="13" t="n">
         <v>6.65</v>
+      </c>
+      <c r="AL49" s="13" t="n">
+        <v>7.07</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -5167,6 +5287,9 @@
       <c r="AK50" s="13" t="n">
         <v>12073.76</v>
       </c>
+      <c r="AL50" s="13" t="n">
+        <v>12141.96</v>
+      </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
       <c r="A51" s="3" t="n">
@@ -5254,6 +5377,7 @@
       <c r="AI51" s="13" t="n"/>
       <c r="AJ51" s="13" t="n"/>
       <c r="AK51" s="13" t="n"/>
+      <c r="AL51" s="13" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -5366,6 +5490,9 @@
       </c>
       <c r="AK52" s="13" t="n">
         <v>24.57</v>
+      </c>
+      <c r="AL52" s="13" t="n">
+        <v>24.96</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -5432,6 +5559,9 @@
       <c r="AK53" s="13" t="n">
         <v>12404.95</v>
       </c>
+      <c r="AL53" s="13" t="n">
+        <v>12546.64</v>
+      </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
       <c r="A54" s="3" t="n">
@@ -5519,6 +5649,7 @@
       <c r="AI54" s="13" t="n"/>
       <c r="AJ54" s="13" t="n"/>
       <c r="AK54" s="13" t="n"/>
+      <c r="AL54" s="13" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -5631,6 +5762,9 @@
       </c>
       <c r="AK55" s="13" t="n">
         <v>15.91</v>
+      </c>
+      <c r="AL55" s="13" t="n">
+        <v>16.25</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -5697,6 +5831,9 @@
       <c r="AK56" s="13" t="n">
         <v>8062.54</v>
       </c>
+      <c r="AL56" s="13" t="n">
+        <v>8271.620000000001</v>
+      </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
       <c r="A57" s="3" t="n">
@@ -5784,6 +5921,7 @@
       <c r="AI57" s="13" t="n"/>
       <c r="AJ57" s="13" t="n"/>
       <c r="AK57" s="13" t="n"/>
+      <c r="AL57" s="13" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -5896,6 +6034,9 @@
       </c>
       <c r="AK58" s="13" t="n">
         <v>25.04</v>
+      </c>
+      <c r="AL58" s="13" t="n">
+        <v>26.05</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -5962,6 +6103,9 @@
       <c r="AK59" s="13" t="n">
         <v>14896.72</v>
       </c>
+      <c r="AL59" s="13" t="n">
+        <v>15194.78</v>
+      </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
       <c r="A60" s="3" t="n">
@@ -6049,6 +6193,7 @@
       <c r="AI60" s="13" t="n"/>
       <c r="AJ60" s="13" t="n"/>
       <c r="AK60" s="13" t="n"/>
+      <c r="AL60" s="13" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -6161,6 +6306,9 @@
       </c>
       <c r="AK61" s="13" t="n">
         <v>29.33</v>
+      </c>
+      <c r="AL61" s="13" t="n">
+        <v>30.63</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -6227,6 +6375,9 @@
       <c r="AK62" s="13" t="n">
         <v>14020.75</v>
       </c>
+      <c r="AL62" s="13" t="n">
+        <v>14315.47</v>
+      </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
       <c r="A63" s="3" t="n">
@@ -6314,6 +6465,7 @@
       <c r="AI63" s="13" t="n"/>
       <c r="AJ63" s="13" t="n"/>
       <c r="AK63" s="13" t="n"/>
+      <c r="AL63" s="13" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -6426,6 +6578,9 @@
       </c>
       <c r="AK64" s="13" t="n">
         <v>15.52</v>
+      </c>
+      <c r="AL64" s="13" t="n">
+        <v>16.12</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -6492,6 +6647,9 @@
       <c r="AK65" s="13" t="n">
         <v>7890.88</v>
       </c>
+      <c r="AL65" s="13" t="n">
+        <v>8112.48</v>
+      </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
       <c r="A66" s="3" t="n">
@@ -6579,6 +6737,7 @@
       <c r="AI66" s="13" t="n"/>
       <c r="AJ66" s="13" t="n"/>
       <c r="AK66" s="13" t="n"/>
+      <c r="AL66" s="13" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -6691,6 +6850,9 @@
       </c>
       <c r="AK67" s="13" t="n">
         <v>8.93</v>
+      </c>
+      <c r="AL67" s="13" t="n">
+        <v>8.710000000000001</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -6757,6 +6919,9 @@
       <c r="AK68" s="13" t="n">
         <v>9369.9</v>
       </c>
+      <c r="AL68" s="13" t="n">
+        <v>9439.43</v>
+      </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
       <c r="A69" s="3" t="n">
@@ -6844,6 +7009,7 @@
       <c r="AI69" s="13" t="n"/>
       <c r="AJ69" s="13" t="n"/>
       <c r="AK69" s="13" t="n"/>
+      <c r="AL69" s="13" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -6956,6 +7122,9 @@
       </c>
       <c r="AK70" s="13" t="n">
         <v>19.75</v>
+      </c>
+      <c r="AL70" s="13" t="n">
+        <v>20.99</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -7022,6 +7191,9 @@
       <c r="AK71" s="13" t="n">
         <v>2546.26</v>
       </c>
+      <c r="AL71" s="13" t="n">
+        <v>2677.12</v>
+      </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
       <c r="A72" s="3" t="n">
@@ -7109,6 +7281,7 @@
       <c r="AI72" s="13" t="n"/>
       <c r="AJ72" s="13" t="n"/>
       <c r="AK72" s="13" t="n"/>
+      <c r="AL72" s="13" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -7221,6 +7394,9 @@
       </c>
       <c r="AK73" s="13" t="n">
         <v>36.53</v>
+      </c>
+      <c r="AL73" s="13" t="n">
+        <v>37.95</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -7287,6 +7463,9 @@
       <c r="AK74" s="13" t="n">
         <v>4832.36</v>
       </c>
+      <c r="AL74" s="13" t="n">
+        <v>5101.03</v>
+      </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
       <c r="A75" s="3" t="n">
@@ -7374,6 +7553,7 @@
       <c r="AI75" s="13" t="n"/>
       <c r="AJ75" s="13" t="n"/>
       <c r="AK75" s="13" t="n"/>
+      <c r="AL75" s="13" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -7486,6 +7666,9 @@
       </c>
       <c r="AK76" s="13" t="n">
         <v>19.62</v>
+      </c>
+      <c r="AL76" s="13" t="n">
+        <v>19.38</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -7552,6 +7735,9 @@
       <c r="AK77" s="13" t="n">
         <v>8499.879999999999</v>
       </c>
+      <c r="AL77" s="13" t="n">
+        <v>8597.75</v>
+      </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
       <c r="A78" s="3" t="n">
@@ -7639,6 +7825,7 @@
       <c r="AI78" s="13" t="n"/>
       <c r="AJ78" s="13" t="n"/>
       <c r="AK78" s="13" t="n"/>
+      <c r="AL78" s="13" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -7751,6 +7938,9 @@
       </c>
       <c r="AK79" s="13" t="n">
         <v>16.8</v>
+      </c>
+      <c r="AL79" s="13" t="n">
+        <v>16.54</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -7817,6 +8007,9 @@
       <c r="AK80" s="13" t="n">
         <v>1398.81</v>
       </c>
+      <c r="AL80" s="13" t="n">
+        <v>1369.48</v>
+      </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
       <c r="A81" s="3" t="n">
@@ -7904,6 +8097,7 @@
       <c r="AI81" s="13" t="n"/>
       <c r="AJ81" s="13" t="n"/>
       <c r="AK81" s="13" t="n"/>
+      <c r="AL81" s="13" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -8016,6 +8210,9 @@
       </c>
       <c r="AK82" s="13" t="n">
         <v>13.91</v>
+      </c>
+      <c r="AL82" s="13" t="n">
+        <v>13.99</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -8082,6 +8279,9 @@
       <c r="AK83" s="13" t="n">
         <v>15852.88</v>
       </c>
+      <c r="AL83" s="13" t="n">
+        <v>15895.36</v>
+      </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
       <c r="A84" s="3" t="n">
@@ -8169,6 +8369,7 @@
       <c r="AI84" s="13" t="n"/>
       <c r="AJ84" s="13" t="n"/>
       <c r="AK84" s="13" t="n"/>
+      <c r="AL84" s="13" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -8281,6 +8482,9 @@
       </c>
       <c r="AK85" s="13" t="n">
         <v>54.64</v>
+      </c>
+      <c r="AL85" s="13" t="n">
+        <v>54.95</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -8347,6 +8551,9 @@
       <c r="AK86" s="13" t="n">
         <v>3029.24</v>
       </c>
+      <c r="AL86" s="13" t="n">
+        <v>3138.15</v>
+      </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
       <c r="A87" s="3" t="n">
@@ -8434,6 +8641,7 @@
       <c r="AI87" s="13" t="n"/>
       <c r="AJ87" s="13" t="n"/>
       <c r="AK87" s="13" t="n"/>
+      <c r="AL87" s="13" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -8546,6 +8754,9 @@
       </c>
       <c r="AK88" s="13" t="n">
         <v>58.69</v>
+      </c>
+      <c r="AL88" s="13" t="n">
+        <v>58.73</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -8612,6 +8823,9 @@
       <c r="AK89" s="13" t="n">
         <v>3396.3</v>
       </c>
+      <c r="AL89" s="13" t="n">
+        <v>3385.64</v>
+      </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
       <c r="A90" s="3" t="n">
@@ -8699,6 +8913,7 @@
       <c r="AI90" s="13" t="n"/>
       <c r="AJ90" s="13" t="n"/>
       <c r="AK90" s="13" t="n"/>
+      <c r="AL90" s="13" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -8811,6 +9026,9 @@
       </c>
       <c r="AK91" s="13" t="n">
         <v>48.73</v>
+      </c>
+      <c r="AL91" s="13" t="n">
+        <v>49.27</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -8877,6 +9095,9 @@
       <c r="AK92" s="13" t="n">
         <v>2927.73</v>
       </c>
+      <c r="AL92" s="13" t="n">
+        <v>3098.06</v>
+      </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
       <c r="A93" s="3" t="n">
@@ -8964,6 +9185,7 @@
       <c r="AI93" s="13" t="n"/>
       <c r="AJ93" s="13" t="n"/>
       <c r="AK93" s="13" t="n"/>
+      <c r="AL93" s="13" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -9076,6 +9298,9 @@
       </c>
       <c r="AK94" s="13" t="n">
         <v>33.77</v>
+      </c>
+      <c r="AL94" s="13" t="n">
+        <v>32.67</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -9142,6 +9367,9 @@
       <c r="AK95" s="13" t="n">
         <v>1794.2</v>
       </c>
+      <c r="AL95" s="13" t="n">
+        <v>1820.53</v>
+      </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
       <c r="A96" s="3" t="n">
@@ -9229,6 +9457,7 @@
       <c r="AI96" s="13" t="n"/>
       <c r="AJ96" s="13" t="n"/>
       <c r="AK96" s="13" t="n"/>
+      <c r="AL96" s="13" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -9341,6 +9570,9 @@
       </c>
       <c r="AK97" s="13" t="n">
         <v>26.49</v>
+      </c>
+      <c r="AL97" s="13" t="n">
+        <v>26.62</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -9407,6 +9639,9 @@
       <c r="AK98" s="13" t="n">
         <v>9934.41</v>
       </c>
+      <c r="AL98" s="13" t="n">
+        <v>9850.629999999999</v>
+      </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
       <c r="A99" s="3" t="n">
@@ -9494,6 +9729,7 @@
       <c r="AI99" s="13" t="n"/>
       <c r="AJ99" s="13" t="n"/>
       <c r="AK99" s="13" t="n"/>
+      <c r="AL99" s="13" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -9606,6 +9842,9 @@
       </c>
       <c r="AK100" s="13" t="n">
         <v>85.68000000000001</v>
+      </c>
+      <c r="AL100" s="13" t="n">
+        <v>84.42</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -9672,6 +9911,9 @@
       <c r="AK101" s="13" t="n">
         <v>9627.27</v>
       </c>
+      <c r="AL101" s="13" t="n">
+        <v>9921.99</v>
+      </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
       <c r="A102" s="3" t="n">
@@ -9759,6 +10001,7 @@
       <c r="AI102" s="13" t="n"/>
       <c r="AJ102" s="13" t="n"/>
       <c r="AK102" s="13" t="n"/>
+      <c r="AL102" s="13" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -9871,6 +10114,9 @@
       </c>
       <c r="AK103" s="13" t="n">
         <v>59.83</v>
+      </c>
+      <c r="AL103" s="13" t="n">
+        <v>58.19</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -9937,6 +10183,9 @@
       <c r="AK104" s="13" t="n">
         <v>15202</v>
       </c>
+      <c r="AL104" s="13" t="n">
+        <v>14420.86</v>
+      </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
       <c r="A105" s="3" t="n">
@@ -10024,6 +10273,7 @@
       <c r="AI105" s="13" t="n"/>
       <c r="AJ105" s="13" t="n"/>
       <c r="AK105" s="13" t="n"/>
+      <c r="AL105" s="13" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -10136,6 +10386,9 @@
       </c>
       <c r="AK106" s="13" t="n">
         <v>9.81</v>
+      </c>
+      <c r="AL106" s="13" t="n">
+        <v>10.47</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -10202,6 +10455,9 @@
       <c r="AK107" s="13" t="n">
         <v>2274.7</v>
       </c>
+      <c r="AL107" s="13" t="n">
+        <v>2334.73</v>
+      </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
       <c r="A108" s="3" t="n">
@@ -10289,6 +10545,7 @@
       <c r="AI108" s="13" t="n"/>
       <c r="AJ108" s="13" t="n"/>
       <c r="AK108" s="13" t="n"/>
+      <c r="AL108" s="13" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -10401,6 +10658,9 @@
       </c>
       <c r="AK109" s="13" t="n">
         <v>24.52</v>
+      </c>
+      <c r="AL109" s="13" t="n">
+        <v>24.26</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -10467,6 +10727,9 @@
       <c r="AK110" s="13" t="n">
         <v>781.02</v>
       </c>
+      <c r="AL110" s="13" t="n">
+        <v>776.53</v>
+      </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
       <c r="A111" s="3" t="n">
@@ -10554,6 +10817,7 @@
       <c r="AI111" s="13" t="n"/>
       <c r="AJ111" s="13" t="n"/>
       <c r="AK111" s="13" t="n"/>
+      <c r="AL111" s="13" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -10666,6 +10930,9 @@
       </c>
       <c r="AK112" s="13" t="n">
         <v>33.41</v>
+      </c>
+      <c r="AL112" s="13" t="n">
+        <v>32.77</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -10732,6 +10999,9 @@
       <c r="AK113" s="13" t="n">
         <v>3658.46</v>
       </c>
+      <c r="AL113" s="13" t="n">
+        <v>3424.51</v>
+      </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
       <c r="A114" s="3" t="n">
@@ -10819,6 +11089,7 @@
       <c r="AI114" s="13" t="n"/>
       <c r="AJ114" s="13" t="n"/>
       <c r="AK114" s="13" t="n"/>
+      <c r="AL114" s="13" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -10931,6 +11202,9 @@
       </c>
       <c r="AK115" s="13" t="n">
         <v>23.28</v>
+      </c>
+      <c r="AL115" s="13" t="n">
+        <v>24.31</v>
       </c>
     </row>
     <row r="116">
@@ -10981,6 +11255,9 @@
       </c>
       <c r="AK116" s="13" t="n">
         <v>4165.85</v>
+      </c>
+      <c r="AL116" s="13" t="n">
+        <v>4279.29</v>
       </c>
     </row>
     <row r="117">
@@ -11024,6 +11301,7 @@
       <c r="AI117" s="13" t="n"/>
       <c r="AJ117" s="13" t="n"/>
       <c r="AK117" s="13" t="n"/>
+      <c r="AL117" s="13" t="n"/>
     </row>
     <row r="118">
       <c r="P118" s="13" t="n">
@@ -11092,6 +11370,9 @@
       <c r="AK118" s="13" t="n">
         <v>29.02</v>
       </c>
+      <c r="AL118" s="13" t="n">
+        <v>29.02</v>
+      </c>
     </row>
     <row r="119">
       <c r="Y119" s="13" t="n">
@@ -11132,6 +11413,9 @@
       </c>
       <c r="AK119" s="13" t="n">
         <v>2879.13</v>
+      </c>
+      <c r="AL119" s="13" t="n">
+        <v>2925.77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-03-19 05:13:29]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL119"/>
+  <dimension ref="A1:AM119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="15"/>
@@ -555,6 +555,7 @@
     <col width="15" customWidth="1" min="36" max="36"/>
     <col width="15" customWidth="1" min="37" max="37"/>
     <col width="15" customWidth="1" min="38" max="38"/>
+    <col width="15" customWidth="1" min="39" max="39"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -748,6 +749,11 @@
           <t>2026/03/16</t>
         </is>
       </c>
+      <c r="AM1" s="13" t="inlineStr">
+        <is>
+          <t>2026/03/19</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -940,6 +946,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="AM2" s="14" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1056,6 +1067,9 @@
       <c r="AL3" s="13" t="n">
         <v>69.7</v>
       </c>
+      <c r="AM3" s="13" t="n">
+        <v>69.39</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1171,6 +1185,9 @@
       </c>
       <c r="AL4" s="13" t="n">
         <v>4079.72</v>
+      </c>
+      <c r="AM4" s="13" t="n">
+        <v>4016.66</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1212,6 +1229,7 @@
       <c r="AJ5" s="13" t="n"/>
       <c r="AK5" s="13" t="n"/>
       <c r="AL5" s="13" t="n"/>
+      <c r="AM5" s="13" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1300,6 +1318,7 @@
       <c r="AJ6" s="13" t="n"/>
       <c r="AK6" s="13" t="n"/>
       <c r="AL6" s="13" t="n"/>
+      <c r="AM6" s="13" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1415,6 +1434,9 @@
       </c>
       <c r="AL7" s="13" t="n">
         <v>50.89</v>
+      </c>
+      <c r="AM7" s="13" t="n">
+        <v>50.68</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -1484,6 +1506,9 @@
       <c r="AL8" s="13" t="n">
         <v>5820.14</v>
       </c>
+      <c r="AM8" s="13" t="n">
+        <v>5712.76</v>
+      </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -1572,6 +1597,7 @@
       <c r="AJ9" s="13" t="n"/>
       <c r="AK9" s="13" t="n"/>
       <c r="AL9" s="13" t="n"/>
+      <c r="AM9" s="13" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -1687,6 +1713,9 @@
       </c>
       <c r="AL10" s="13" t="n">
         <v>54.66</v>
+      </c>
+      <c r="AM10" s="13" t="n">
+        <v>54.48</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -1756,6 +1785,9 @@
       <c r="AL11" s="13" t="n">
         <v>4658.8</v>
       </c>
+      <c r="AM11" s="13" t="n">
+        <v>4601.63</v>
+      </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -1844,6 +1876,7 @@
       <c r="AJ12" s="13" t="n"/>
       <c r="AK12" s="13" t="n"/>
       <c r="AL12" s="13" t="n"/>
+      <c r="AM12" s="13" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -1959,6 +1992,9 @@
       </c>
       <c r="AL13" s="13" t="n">
         <v>60.76</v>
+      </c>
+      <c r="AM13" s="13" t="n">
+        <v>60.44</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -2028,6 +2064,9 @@
       <c r="AL14" s="13" t="n">
         <v>8174.9</v>
       </c>
+      <c r="AM14" s="13" t="n">
+        <v>7910.55</v>
+      </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -2116,6 +2155,7 @@
       <c r="AJ15" s="13" t="n"/>
       <c r="AK15" s="13" t="n"/>
       <c r="AL15" s="13" t="n"/>
+      <c r="AM15" s="13" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -2231,6 +2271,9 @@
       </c>
       <c r="AL16" s="13" t="n">
         <v>27.71</v>
+      </c>
+      <c r="AM16" s="13" t="n">
+        <v>28.38</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -2300,6 +2343,9 @@
       <c r="AL17" s="13" t="n">
         <v>2652.96</v>
       </c>
+      <c r="AM17" s="13" t="n">
+        <v>2652.96</v>
+      </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="3" t="n">
@@ -2388,6 +2434,7 @@
       <c r="AJ18" s="13" t="n"/>
       <c r="AK18" s="13" t="n"/>
       <c r="AL18" s="13" t="n"/>
+      <c r="AM18" s="13" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -2503,6 +2550,9 @@
       </c>
       <c r="AL19" s="13" t="n">
         <v>93.73999999999999</v>
+      </c>
+      <c r="AM19" s="13" t="n">
+        <v>93.65000000000001</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -2572,6 +2622,9 @@
       <c r="AL20" s="13" t="n">
         <v>6632.19</v>
       </c>
+      <c r="AM20" s="13" t="n">
+        <v>6624.7</v>
+      </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -2660,6 +2713,7 @@
       <c r="AJ21" s="13" t="n"/>
       <c r="AK21" s="13" t="n"/>
       <c r="AL21" s="13" t="n"/>
+      <c r="AM21" s="13" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -2773,6 +2827,9 @@
       </c>
       <c r="AL22" s="13" t="n">
         <v>52.51</v>
+      </c>
+      <c r="AM22" s="13" t="n">
+        <v>51.98</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1">
@@ -2842,6 +2899,9 @@
       <c r="AL23" s="13" t="n">
         <v>74278.63</v>
       </c>
+      <c r="AM23" s="13" t="n">
+        <v>75070.34</v>
+      </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="3" t="n">
@@ -2930,6 +2990,7 @@
       <c r="AJ24" s="13" t="n"/>
       <c r="AK24" s="13" t="n"/>
       <c r="AL24" s="13" t="n"/>
+      <c r="AM24" s="13" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -3045,6 +3106,9 @@
       </c>
       <c r="AL25" s="13" t="n">
         <v>78.75</v>
+      </c>
+      <c r="AM25" s="13" t="n">
+        <v>79.94</v>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="1">
@@ -3114,6 +3178,9 @@
       <c r="AL26" s="13" t="n">
         <v>23447.29</v>
       </c>
+      <c r="AM26" s="13" t="n">
+        <v>23502.25</v>
+      </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -3202,6 +3269,7 @@
       <c r="AJ27" s="13" t="n"/>
       <c r="AK27" s="13" t="n"/>
       <c r="AL27" s="13" t="n"/>
+      <c r="AM27" s="13" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -3317,6 +3385,9 @@
       </c>
       <c r="AL28" s="13" t="n">
         <v>71.06</v>
+      </c>
+      <c r="AM28" s="13" t="n">
+        <v>70.94</v>
       </c>
     </row>
     <row r="29" ht="14.25" customHeight="1">
@@ -3386,6 +3457,9 @@
       <c r="AL29" s="13" t="n">
         <v>53436.04</v>
       </c>
+      <c r="AM29" s="13" t="n">
+        <v>53512.29</v>
+      </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="3" t="n">
@@ -3474,6 +3548,7 @@
       <c r="AJ30" s="13" t="n"/>
       <c r="AK30" s="13" t="n"/>
       <c r="AL30" s="13" t="n"/>
+      <c r="AM30" s="13" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -3589,6 +3664,9 @@
       </c>
       <c r="AL31" s="13" t="n">
         <v>51.96</v>
+      </c>
+      <c r="AM31" s="13" t="n">
+        <v>51.6</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -3658,6 +3736,9 @@
       <c r="AL32" s="13" t="n">
         <v>5909.4</v>
       </c>
+      <c r="AM32" s="13" t="n">
+        <v>5814.73</v>
+      </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
       <c r="A33" s="3" t="n">
@@ -3746,6 +3827,7 @@
       <c r="AJ33" s="13" t="n"/>
       <c r="AK33" s="13" t="n"/>
       <c r="AL33" s="13" t="n"/>
+      <c r="AM33" s="13" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -3861,6 +3943,9 @@
       </c>
       <c r="AL34" s="13" t="n">
         <v>2.86</v>
+      </c>
+      <c r="AM34" s="13" t="n">
+        <v>2.65</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -3930,6 +4015,9 @@
       <c r="AL35" s="13" t="n">
         <v>33463.01</v>
       </c>
+      <c r="AM35" s="13" t="n">
+        <v>33053.45</v>
+      </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="3" t="n">
@@ -4018,6 +4106,7 @@
       <c r="AJ36" s="13" t="n"/>
       <c r="AK36" s="13" t="n"/>
       <c r="AL36" s="13" t="n"/>
+      <c r="AM36" s="13" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -4133,6 +4222,9 @@
       </c>
       <c r="AL37" s="13" t="n">
         <v>28.36</v>
+      </c>
+      <c r="AM37" s="13" t="n">
+        <v>28.88</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -4202,6 +4294,9 @@
       <c r="AL38" s="13" t="n">
         <v>3501.16</v>
       </c>
+      <c r="AM38" s="13" t="n">
+        <v>3515.6</v>
+      </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
       <c r="A39" s="3" t="n">
@@ -4290,6 +4385,7 @@
       <c r="AJ39" s="13" t="n"/>
       <c r="AK39" s="13" t="n"/>
       <c r="AL39" s="13" t="n"/>
+      <c r="AM39" s="13" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -4405,6 +4501,9 @@
       </c>
       <c r="AL40" s="13" t="n">
         <v>48.92</v>
+      </c>
+      <c r="AM40" s="13" t="n">
+        <v>49.26</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -4474,6 +4573,9 @@
       <c r="AL41" s="13" t="n">
         <v>3338.53</v>
       </c>
+      <c r="AM41" s="13" t="n">
+        <v>3331.96</v>
+      </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
       <c r="A42" s="3" t="n">
@@ -4562,6 +4664,7 @@
       <c r="AJ42" s="13" t="n"/>
       <c r="AK42" s="13" t="n"/>
       <c r="AL42" s="13" t="n"/>
+      <c r="AM42" s="13" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -4677,6 +4780,9 @@
       </c>
       <c r="AL43" s="13" t="n">
         <v>14.71</v>
+      </c>
+      <c r="AM43" s="13" t="n">
+        <v>14.62</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -4746,6 +4852,9 @@
       <c r="AL44" s="13" t="n">
         <v>6735.52</v>
       </c>
+      <c r="AM44" s="13" t="n">
+        <v>6627.03</v>
+      </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
       <c r="A45" s="3" t="n">
@@ -4834,6 +4943,7 @@
       <c r="AJ45" s="13" t="n"/>
       <c r="AK45" s="13" t="n"/>
       <c r="AL45" s="13" t="n"/>
+      <c r="AM45" s="13" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -4949,6 +5059,9 @@
       </c>
       <c r="AL46" s="13" t="n">
         <v>20.46</v>
+      </c>
+      <c r="AM46" s="13" t="n">
+        <v>21.07</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -5018,6 +5131,9 @@
       <c r="AL47" s="13" t="n">
         <v>7990.9</v>
       </c>
+      <c r="AM47" s="13" t="n">
+        <v>7932.57</v>
+      </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
       <c r="A48" s="3" t="n">
@@ -5106,6 +5222,7 @@
       <c r="AJ48" s="13" t="n"/>
       <c r="AK48" s="13" t="n"/>
       <c r="AL48" s="13" t="n"/>
+      <c r="AM48" s="13" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -5221,6 +5338,9 @@
       </c>
       <c r="AL49" s="13" t="n">
         <v>7.07</v>
+      </c>
+      <c r="AM49" s="13" t="n">
+        <v>7.46</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -5290,6 +5410,9 @@
       <c r="AL50" s="13" t="n">
         <v>12141.96</v>
       </c>
+      <c r="AM50" s="13" t="n">
+        <v>12043.31</v>
+      </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
       <c r="A51" s="3" t="n">
@@ -5378,6 +5501,7 @@
       <c r="AJ51" s="13" t="n"/>
       <c r="AK51" s="13" t="n"/>
       <c r="AL51" s="13" t="n"/>
+      <c r="AM51" s="13" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -5493,6 +5617,9 @@
       </c>
       <c r="AL52" s="13" t="n">
         <v>24.96</v>
+      </c>
+      <c r="AM52" s="13" t="n">
+        <v>23.31</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -5562,6 +5689,9 @@
       <c r="AL53" s="13" t="n">
         <v>12546.64</v>
       </c>
+      <c r="AM53" s="13" t="n">
+        <v>12135.2</v>
+      </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
       <c r="A54" s="3" t="n">
@@ -5650,6 +5780,7 @@
       <c r="AJ54" s="13" t="n"/>
       <c r="AK54" s="13" t="n"/>
       <c r="AL54" s="13" t="n"/>
+      <c r="AM54" s="13" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -5765,6 +5896,9 @@
       </c>
       <c r="AL55" s="13" t="n">
         <v>16.25</v>
+      </c>
+      <c r="AM55" s="13" t="n">
+        <v>17.72</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -5834,6 +5968,9 @@
       <c r="AL56" s="13" t="n">
         <v>8271.620000000001</v>
       </c>
+      <c r="AM56" s="13" t="n">
+        <v>8073.5</v>
+      </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
       <c r="A57" s="3" t="n">
@@ -5922,6 +6059,7 @@
       <c r="AJ57" s="13" t="n"/>
       <c r="AK57" s="13" t="n"/>
       <c r="AL57" s="13" t="n"/>
+      <c r="AM57" s="13" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -6037,6 +6175,9 @@
       </c>
       <c r="AL58" s="13" t="n">
         <v>26.05</v>
+      </c>
+      <c r="AM58" s="13" t="n">
+        <v>26.59</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -6106,6 +6247,9 @@
       <c r="AL59" s="13" t="n">
         <v>15194.78</v>
       </c>
+      <c r="AM59" s="13" t="n">
+        <v>14862.37</v>
+      </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
       <c r="A60" s="3" t="n">
@@ -6194,6 +6338,7 @@
       <c r="AJ60" s="13" t="n"/>
       <c r="AK60" s="13" t="n"/>
       <c r="AL60" s="13" t="n"/>
+      <c r="AM60" s="13" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -6309,6 +6454,9 @@
       </c>
       <c r="AL61" s="13" t="n">
         <v>30.63</v>
+      </c>
+      <c r="AM61" s="13" t="n">
+        <v>38.89</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -6378,6 +6526,9 @@
       <c r="AL62" s="13" t="n">
         <v>14315.47</v>
       </c>
+      <c r="AM62" s="13" t="n">
+        <v>14265.28</v>
+      </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
       <c r="A63" s="3" t="n">
@@ -6466,6 +6617,7 @@
       <c r="AJ63" s="13" t="n"/>
       <c r="AK63" s="13" t="n"/>
       <c r="AL63" s="13" t="n"/>
+      <c r="AM63" s="13" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -6581,6 +6733,9 @@
       </c>
       <c r="AL64" s="13" t="n">
         <v>16.12</v>
+      </c>
+      <c r="AM64" s="13" t="n">
+        <v>16.3</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -6650,6 +6805,9 @@
       <c r="AL65" s="13" t="n">
         <v>8112.48</v>
       </c>
+      <c r="AM65" s="13" t="n">
+        <v>8055.17</v>
+      </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
       <c r="A66" s="3" t="n">
@@ -6738,6 +6896,7 @@
       <c r="AJ66" s="13" t="n"/>
       <c r="AK66" s="13" t="n"/>
       <c r="AL66" s="13" t="n"/>
+      <c r="AM66" s="13" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -6853,6 +7012,9 @@
       </c>
       <c r="AL67" s="13" t="n">
         <v>8.710000000000001</v>
+      </c>
+      <c r="AM67" s="13" t="n">
+        <v>9.039999999999999</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -6922,6 +7084,9 @@
       <c r="AL68" s="13" t="n">
         <v>9439.43</v>
       </c>
+      <c r="AM68" s="13" t="n">
+        <v>9392.139999999999</v>
+      </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
       <c r="A69" s="3" t="n">
@@ -7010,6 +7175,7 @@
       <c r="AJ69" s="13" t="n"/>
       <c r="AK69" s="13" t="n"/>
       <c r="AL69" s="13" t="n"/>
+      <c r="AM69" s="13" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -7125,6 +7291,9 @@
       </c>
       <c r="AL70" s="13" t="n">
         <v>20.99</v>
+      </c>
+      <c r="AM70" s="13" t="n">
+        <v>21.58</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -7194,6 +7363,9 @@
       <c r="AL71" s="13" t="n">
         <v>2677.12</v>
       </c>
+      <c r="AM71" s="13" t="n">
+        <v>2634.48</v>
+      </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
       <c r="A72" s="3" t="n">
@@ -7282,6 +7454,7 @@
       <c r="AJ72" s="13" t="n"/>
       <c r="AK72" s="13" t="n"/>
       <c r="AL72" s="13" t="n"/>
+      <c r="AM72" s="13" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -7397,6 +7570,9 @@
       </c>
       <c r="AL73" s="13" t="n">
         <v>37.95</v>
+      </c>
+      <c r="AM73" s="13" t="n">
+        <v>38.07</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -7466,6 +7642,9 @@
       <c r="AL74" s="13" t="n">
         <v>5101.03</v>
       </c>
+      <c r="AM74" s="13" t="n">
+        <v>5027.69</v>
+      </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
       <c r="A75" s="3" t="n">
@@ -7554,6 +7733,7 @@
       <c r="AJ75" s="13" t="n"/>
       <c r="AK75" s="13" t="n"/>
       <c r="AL75" s="13" t="n"/>
+      <c r="AM75" s="13" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -7669,6 +7849,9 @@
       </c>
       <c r="AL76" s="13" t="n">
         <v>19.38</v>
+      </c>
+      <c r="AM76" s="13" t="n">
+        <v>19.93</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -7738,6 +7921,9 @@
       <c r="AL77" s="13" t="n">
         <v>8597.75</v>
       </c>
+      <c r="AM77" s="13" t="n">
+        <v>8553.15</v>
+      </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
       <c r="A78" s="3" t="n">
@@ -7826,6 +8012,7 @@
       <c r="AJ78" s="13" t="n"/>
       <c r="AK78" s="13" t="n"/>
       <c r="AL78" s="13" t="n"/>
+      <c r="AM78" s="13" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -7941,6 +8128,9 @@
       </c>
       <c r="AL79" s="13" t="n">
         <v>16.54</v>
+      </c>
+      <c r="AM79" s="13" t="n">
+        <v>16.84</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -8010,6 +8200,9 @@
       <c r="AL80" s="13" t="n">
         <v>1369.48</v>
       </c>
+      <c r="AM80" s="13" t="n">
+        <v>1392.69</v>
+      </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
       <c r="A81" s="3" t="n">
@@ -8098,6 +8291,7 @@
       <c r="AJ81" s="13" t="n"/>
       <c r="AK81" s="13" t="n"/>
       <c r="AL81" s="13" t="n"/>
+      <c r="AM81" s="13" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -8213,6 +8407,9 @@
       </c>
       <c r="AL82" s="13" t="n">
         <v>13.99</v>
+      </c>
+      <c r="AM82" s="13" t="n">
+        <v>14.71</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -8282,6 +8479,9 @@
       <c r="AL83" s="13" t="n">
         <v>15895.36</v>
       </c>
+      <c r="AM83" s="13" t="n">
+        <v>16153.6</v>
+      </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
       <c r="A84" s="3" t="n">
@@ -8370,6 +8570,7 @@
       <c r="AJ84" s="13" t="n"/>
       <c r="AK84" s="13" t="n"/>
       <c r="AL84" s="13" t="n"/>
+      <c r="AM84" s="13" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -8485,6 +8686,9 @@
       </c>
       <c r="AL85" s="13" t="n">
         <v>54.95</v>
+      </c>
+      <c r="AM85" s="13" t="n">
+        <v>53.41</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -8554,6 +8758,9 @@
       <c r="AL86" s="13" t="n">
         <v>3138.15</v>
       </c>
+      <c r="AM86" s="13" t="n">
+        <v>3002.99</v>
+      </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
       <c r="A87" s="3" t="n">
@@ -8642,6 +8849,7 @@
       <c r="AJ87" s="13" t="n"/>
       <c r="AK87" s="13" t="n"/>
       <c r="AL87" s="13" t="n"/>
+      <c r="AM87" s="13" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -8757,6 +8965,9 @@
       </c>
       <c r="AL88" s="13" t="n">
         <v>58.73</v>
+      </c>
+      <c r="AM88" s="13" t="n">
+        <v>58.59</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -8826,6 +9037,9 @@
       <c r="AL89" s="13" t="n">
         <v>3385.64</v>
       </c>
+      <c r="AM89" s="13" t="n">
+        <v>3336.89</v>
+      </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
       <c r="A90" s="3" t="n">
@@ -8914,6 +9128,7 @@
       <c r="AJ90" s="13" t="n"/>
       <c r="AK90" s="13" t="n"/>
       <c r="AL90" s="13" t="n"/>
+      <c r="AM90" s="13" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -9029,6 +9244,9 @@
       </c>
       <c r="AL91" s="13" t="n">
         <v>49.27</v>
+      </c>
+      <c r="AM91" s="13" t="n">
+        <v>48.59</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -9098,6 +9316,9 @@
       <c r="AL92" s="13" t="n">
         <v>3098.06</v>
       </c>
+      <c r="AM92" s="13" t="n">
+        <v>2949.03</v>
+      </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
       <c r="A93" s="3" t="n">
@@ -9186,6 +9407,7 @@
       <c r="AJ93" s="13" t="n"/>
       <c r="AK93" s="13" t="n"/>
       <c r="AL93" s="13" t="n"/>
+      <c r="AM93" s="13" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -9301,6 +9523,9 @@
       </c>
       <c r="AL94" s="13" t="n">
         <v>32.67</v>
+      </c>
+      <c r="AM94" s="13" t="n">
+        <v>35.28</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -9370,6 +9595,9 @@
       <c r="AL95" s="13" t="n">
         <v>1820.53</v>
       </c>
+      <c r="AM95" s="13" t="n">
+        <v>1849.22</v>
+      </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
       <c r="A96" s="3" t="n">
@@ -9458,6 +9686,7 @@
       <c r="AJ96" s="13" t="n"/>
       <c r="AK96" s="13" t="n"/>
       <c r="AL96" s="13" t="n"/>
+      <c r="AM96" s="13" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -9573,6 +9802,9 @@
       </c>
       <c r="AL97" s="13" t="n">
         <v>26.62</v>
+      </c>
+      <c r="AM97" s="13" t="n">
+        <v>26.52</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -9642,6 +9874,9 @@
       <c r="AL98" s="13" t="n">
         <v>9850.629999999999</v>
       </c>
+      <c r="AM98" s="13" t="n">
+        <v>9960.77</v>
+      </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
       <c r="A99" s="3" t="n">
@@ -9730,6 +9965,7 @@
       <c r="AJ99" s="13" t="n"/>
       <c r="AK99" s="13" t="n"/>
       <c r="AL99" s="13" t="n"/>
+      <c r="AM99" s="13" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -9845,6 +10081,9 @@
       </c>
       <c r="AL100" s="13" t="n">
         <v>84.42</v>
+      </c>
+      <c r="AM100" s="13" t="n">
+        <v>85.04000000000001</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -9914,6 +10153,9 @@
       <c r="AL101" s="13" t="n">
         <v>9921.99</v>
       </c>
+      <c r="AM101" s="13" t="n">
+        <v>9688.93</v>
+      </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
       <c r="A102" s="3" t="n">
@@ -10002,6 +10244,7 @@
       <c r="AJ102" s="13" t="n"/>
       <c r="AK102" s="13" t="n"/>
       <c r="AL102" s="13" t="n"/>
+      <c r="AM102" s="13" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -10117,6 +10360,9 @@
       </c>
       <c r="AL103" s="13" t="n">
         <v>58.19</v>
+      </c>
+      <c r="AM103" s="13" t="n">
+        <v>58.04</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -10186,6 +10432,9 @@
       <c r="AL104" s="13" t="n">
         <v>14420.86</v>
       </c>
+      <c r="AM104" s="13" t="n">
+        <v>13964.57</v>
+      </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
       <c r="A105" s="3" t="n">
@@ -10274,6 +10523,7 @@
       <c r="AJ105" s="13" t="n"/>
       <c r="AK105" s="13" t="n"/>
       <c r="AL105" s="13" t="n"/>
+      <c r="AM105" s="13" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -10389,6 +10639,9 @@
       </c>
       <c r="AL106" s="13" t="n">
         <v>10.47</v>
+      </c>
+      <c r="AM106" s="13" t="n">
+        <v>10.07</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -10458,6 +10711,9 @@
       <c r="AL107" s="13" t="n">
         <v>2334.73</v>
       </c>
+      <c r="AM107" s="13" t="n">
+        <v>2249.02</v>
+      </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
       <c r="A108" s="3" t="n">
@@ -10546,6 +10802,7 @@
       <c r="AJ108" s="13" t="n"/>
       <c r="AK108" s="13" t="n"/>
       <c r="AL108" s="13" t="n"/>
+      <c r="AM108" s="13" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -10661,6 +10918,9 @@
       </c>
       <c r="AL109" s="13" t="n">
         <v>24.26</v>
+      </c>
+      <c r="AM109" s="13" t="n">
+        <v>24.35</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -10730,6 +10990,9 @@
       <c r="AL110" s="13" t="n">
         <v>776.53</v>
       </c>
+      <c r="AM110" s="13" t="n">
+        <v>773.0700000000001</v>
+      </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
       <c r="A111" s="3" t="n">
@@ -10818,6 +11081,7 @@
       <c r="AJ111" s="13" t="n"/>
       <c r="AK111" s="13" t="n"/>
       <c r="AL111" s="13" t="n"/>
+      <c r="AM111" s="13" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -10933,6 +11197,9 @@
       </c>
       <c r="AL112" s="13" t="n">
         <v>32.77</v>
+      </c>
+      <c r="AM112" s="13" t="n">
+        <v>32.03</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -11002,6 +11269,9 @@
       <c r="AL113" s="13" t="n">
         <v>3424.51</v>
       </c>
+      <c r="AM113" s="13" t="n">
+        <v>3181.59</v>
+      </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
       <c r="A114" s="3" t="n">
@@ -11090,6 +11360,7 @@
       <c r="AJ114" s="13" t="n"/>
       <c r="AK114" s="13" t="n"/>
       <c r="AL114" s="13" t="n"/>
+      <c r="AM114" s="13" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -11205,6 +11476,9 @@
       </c>
       <c r="AL115" s="13" t="n">
         <v>24.31</v>
+      </c>
+      <c r="AM115" s="13" t="n">
+        <v>23.32</v>
       </c>
     </row>
     <row r="116">
@@ -11258,6 +11532,9 @@
       </c>
       <c r="AL116" s="13" t="n">
         <v>4279.29</v>
+      </c>
+      <c r="AM116" s="13" t="n">
+        <v>4151.11</v>
       </c>
     </row>
     <row r="117">
@@ -11302,6 +11579,7 @@
       <c r="AJ117" s="13" t="n"/>
       <c r="AK117" s="13" t="n"/>
       <c r="AL117" s="13" t="n"/>
+      <c r="AM117" s="13" t="n"/>
     </row>
     <row r="118">
       <c r="P118" s="13" t="n">
@@ -11373,6 +11651,9 @@
       <c r="AL118" s="13" t="n">
         <v>29.02</v>
       </c>
+      <c r="AM118" s="13" t="n">
+        <v>29.02</v>
+      </c>
     </row>
     <row r="119">
       <c r="Y119" s="13" t="n">
@@ -11416,6 +11697,9 @@
       </c>
       <c r="AL119" s="13" t="n">
         <v>2925.77</v>
+      </c>
+      <c r="AM119" s="13" t="n">
+        <v>2854.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-03-23 05:22:42]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM119"/>
+  <dimension ref="A1:AN119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="15"/>
@@ -556,6 +556,7 @@
     <col width="15" customWidth="1" min="37" max="37"/>
     <col width="15" customWidth="1" min="38" max="38"/>
     <col width="15" customWidth="1" min="39" max="39"/>
+    <col width="15" customWidth="1" min="40" max="40"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -754,6 +755,11 @@
           <t>2026/03/19</t>
         </is>
       </c>
+      <c r="AN1" s="13" t="inlineStr">
+        <is>
+          <t>2026/03/23</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -951,6 +957,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="AN2" s="14" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1070,6 +1081,9 @@
       <c r="AM3" s="13" t="n">
         <v>69.39</v>
       </c>
+      <c r="AN3" s="13" t="n">
+        <v>68.06999999999999</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1188,6 +1202,9 @@
       </c>
       <c r="AM4" s="13" t="n">
         <v>4016.66</v>
+      </c>
+      <c r="AN4" s="13" t="n">
+        <v>3849.59</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1230,6 +1247,7 @@
       <c r="AK5" s="13" t="n"/>
       <c r="AL5" s="13" t="n"/>
       <c r="AM5" s="13" t="n"/>
+      <c r="AN5" s="13" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1319,6 +1337,7 @@
       <c r="AK6" s="13" t="n"/>
       <c r="AL6" s="13" t="n"/>
       <c r="AM6" s="13" t="n"/>
+      <c r="AN6" s="13" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1437,6 +1456,9 @@
       </c>
       <c r="AM7" s="13" t="n">
         <v>50.68</v>
+      </c>
+      <c r="AN7" s="13" t="n">
+        <v>49.95</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -1509,6 +1531,9 @@
       <c r="AM8" s="13" t="n">
         <v>5712.76</v>
       </c>
+      <c r="AN8" s="13" t="n">
+        <v>5515.26</v>
+      </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -1598,6 +1623,7 @@
       <c r="AK9" s="13" t="n"/>
       <c r="AL9" s="13" t="n"/>
       <c r="AM9" s="13" t="n"/>
+      <c r="AN9" s="13" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -1716,6 +1742,9 @@
       </c>
       <c r="AM10" s="13" t="n">
         <v>54.48</v>
+      </c>
+      <c r="AN10" s="13" t="n">
+        <v>52.83</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -1788,6 +1817,9 @@
       <c r="AM11" s="13" t="n">
         <v>4601.63</v>
       </c>
+      <c r="AN11" s="13" t="n">
+        <v>4452.87</v>
+      </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -1877,6 +1909,7 @@
       <c r="AK12" s="13" t="n"/>
       <c r="AL12" s="13" t="n"/>
       <c r="AM12" s="13" t="n"/>
+      <c r="AN12" s="13" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -1995,6 +2028,9 @@
       </c>
       <c r="AM13" s="13" t="n">
         <v>60.44</v>
+      </c>
+      <c r="AN13" s="13" t="n">
+        <v>59.81</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -2067,6 +2103,9 @@
       <c r="AM14" s="13" t="n">
         <v>7910.55</v>
       </c>
+      <c r="AN14" s="13" t="n">
+        <v>7524.97</v>
+      </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -2156,6 +2195,7 @@
       <c r="AK15" s="13" t="n"/>
       <c r="AL15" s="13" t="n"/>
       <c r="AM15" s="13" t="n"/>
+      <c r="AN15" s="13" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -2274,6 +2314,9 @@
       </c>
       <c r="AM16" s="13" t="n">
         <v>28.38</v>
+      </c>
+      <c r="AN16" s="13" t="n">
+        <v>27.09</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -2346,6 +2389,9 @@
       <c r="AM17" s="13" t="n">
         <v>2652.96</v>
       </c>
+      <c r="AN17" s="13" t="n">
+        <v>2652.96</v>
+      </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="3" t="n">
@@ -2435,6 +2481,7 @@
       <c r="AK18" s="13" t="n"/>
       <c r="AL18" s="13" t="n"/>
       <c r="AM18" s="13" t="n"/>
+      <c r="AN18" s="13" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -2553,6 +2600,9 @@
       </c>
       <c r="AM19" s="13" t="n">
         <v>93.65000000000001</v>
+      </c>
+      <c r="AN19" s="13" t="n">
+        <v>92.77</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -2625,6 +2675,9 @@
       <c r="AM20" s="13" t="n">
         <v>6624.7</v>
       </c>
+      <c r="AN20" s="13" t="n">
+        <v>6506.48</v>
+      </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -2714,6 +2767,7 @@
       <c r="AK21" s="13" t="n"/>
       <c r="AL21" s="13" t="n"/>
       <c r="AM21" s="13" t="n"/>
+      <c r="AN21" s="13" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -2830,6 +2884,9 @@
       </c>
       <c r="AM22" s="13" t="n">
         <v>51.98</v>
+      </c>
+      <c r="AN22" s="13" t="n">
+        <v>49.47</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1">
@@ -2902,6 +2959,9 @@
       <c r="AM23" s="13" t="n">
         <v>75070.34</v>
       </c>
+      <c r="AN23" s="13" t="n">
+        <v>72759.96000000001</v>
+      </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="3" t="n">
@@ -2991,6 +3051,7 @@
       <c r="AK24" s="13" t="n"/>
       <c r="AL24" s="13" t="n"/>
       <c r="AM24" s="13" t="n"/>
+      <c r="AN24" s="13" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -3109,6 +3170,9 @@
       </c>
       <c r="AM25" s="13" t="n">
         <v>79.94</v>
+      </c>
+      <c r="AN25" s="13" t="n">
+        <v>75.02</v>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="1">
@@ -3181,6 +3245,9 @@
       <c r="AM26" s="13" t="n">
         <v>23502.25</v>
       </c>
+      <c r="AN26" s="13" t="n">
+        <v>22380.19</v>
+      </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -3270,6 +3337,7 @@
       <c r="AK27" s="13" t="n"/>
       <c r="AL27" s="13" t="n"/>
       <c r="AM27" s="13" t="n"/>
+      <c r="AN27" s="13" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -3388,6 +3456,9 @@
       </c>
       <c r="AM28" s="13" t="n">
         <v>70.94</v>
+      </c>
+      <c r="AN28" s="13" t="n">
+        <v>70.17</v>
       </c>
     </row>
     <row r="29" ht="14.25" customHeight="1">
@@ -3460,6 +3531,9 @@
       <c r="AM29" s="13" t="n">
         <v>53512.29</v>
       </c>
+      <c r="AN29" s="13" t="n">
+        <v>51589.75</v>
+      </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="3" t="n">
@@ -3549,6 +3623,7 @@
       <c r="AK30" s="13" t="n"/>
       <c r="AL30" s="13" t="n"/>
       <c r="AM30" s="13" t="n"/>
+      <c r="AN30" s="13" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -3667,6 +3742,9 @@
       </c>
       <c r="AM31" s="13" t="n">
         <v>51.6</v>
+      </c>
+      <c r="AN31" s="13" t="n">
+        <v>51.92</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -3739,6 +3817,9 @@
       <c r="AM32" s="13" t="n">
         <v>5814.73</v>
       </c>
+      <c r="AN32" s="13" t="n">
+        <v>5677.17</v>
+      </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
       <c r="A33" s="3" t="n">
@@ -3828,6 +3909,7 @@
       <c r="AK33" s="13" t="n"/>
       <c r="AL33" s="13" t="n"/>
       <c r="AM33" s="13" t="n"/>
+      <c r="AN33" s="13" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -3946,6 +4028,9 @@
       </c>
       <c r="AM34" s="13" t="n">
         <v>2.65</v>
+      </c>
+      <c r="AN34" s="13" t="n">
+        <v>2.79</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -4018,6 +4103,9 @@
       <c r="AM35" s="13" t="n">
         <v>33053.45</v>
       </c>
+      <c r="AN35" s="13" t="n">
+        <v>31921.84</v>
+      </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="3" t="n">
@@ -4107,6 +4195,7 @@
       <c r="AK36" s="13" t="n"/>
       <c r="AL36" s="13" t="n"/>
       <c r="AM36" s="13" t="n"/>
+      <c r="AN36" s="13" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -4225,6 +4314,9 @@
       </c>
       <c r="AM37" s="13" t="n">
         <v>28.88</v>
+      </c>
+      <c r="AN37" s="13" t="n">
+        <v>29.22</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -4297,6 +4389,9 @@
       <c r="AM38" s="13" t="n">
         <v>3515.6</v>
       </c>
+      <c r="AN38" s="13" t="n">
+        <v>3467.53</v>
+      </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
       <c r="A39" s="3" t="n">
@@ -4386,6 +4481,7 @@
       <c r="AK39" s="13" t="n"/>
       <c r="AL39" s="13" t="n"/>
       <c r="AM39" s="13" t="n"/>
+      <c r="AN39" s="13" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -4504,6 +4600,9 @@
       </c>
       <c r="AM40" s="13" t="n">
         <v>49.26</v>
+      </c>
+      <c r="AN40" s="13" t="n">
+        <v>49.3</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -4576,6 +4675,9 @@
       <c r="AM41" s="13" t="n">
         <v>3331.96</v>
       </c>
+      <c r="AN41" s="13" t="n">
+        <v>3274.84</v>
+      </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
       <c r="A42" s="3" t="n">
@@ -4665,6 +4767,7 @@
       <c r="AK42" s="13" t="n"/>
       <c r="AL42" s="13" t="n"/>
       <c r="AM42" s="13" t="n"/>
+      <c r="AN42" s="13" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -4783,6 +4886,9 @@
       </c>
       <c r="AM43" s="13" t="n">
         <v>14.62</v>
+      </c>
+      <c r="AN43" s="13" t="n">
+        <v>12.29</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -4855,6 +4961,9 @@
       <c r="AM44" s="13" t="n">
         <v>6627.03</v>
       </c>
+      <c r="AN44" s="13" t="n">
+        <v>6251.37</v>
+      </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
       <c r="A45" s="3" t="n">
@@ -4944,6 +5053,7 @@
       <c r="AK45" s="13" t="n"/>
       <c r="AL45" s="13" t="n"/>
       <c r="AM45" s="13" t="n"/>
+      <c r="AN45" s="13" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -5062,6 +5172,9 @@
       </c>
       <c r="AM46" s="13" t="n">
         <v>21.07</v>
+      </c>
+      <c r="AN46" s="13" t="n">
+        <v>18.98</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -5134,6 +5247,9 @@
       <c r="AM47" s="13" t="n">
         <v>7932.57</v>
       </c>
+      <c r="AN47" s="13" t="n">
+        <v>7601.72</v>
+      </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
       <c r="A48" s="3" t="n">
@@ -5223,6 +5339,7 @@
       <c r="AK48" s="13" t="n"/>
       <c r="AL48" s="13" t="n"/>
       <c r="AM48" s="13" t="n"/>
+      <c r="AN48" s="13" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -5341,6 +5458,9 @@
       </c>
       <c r="AM49" s="13" t="n">
         <v>7.46</v>
+      </c>
+      <c r="AN49" s="13" t="n">
+        <v>6.5</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -5413,6 +5533,9 @@
       <c r="AM50" s="13" t="n">
         <v>12043.31</v>
       </c>
+      <c r="AN50" s="13" t="n">
+        <v>11587.45</v>
+      </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
       <c r="A51" s="3" t="n">
@@ -5502,6 +5625,7 @@
       <c r="AK51" s="13" t="n"/>
       <c r="AL51" s="13" t="n"/>
       <c r="AM51" s="13" t="n"/>
+      <c r="AN51" s="13" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -5620,6 +5744,9 @@
       </c>
       <c r="AM52" s="13" t="n">
         <v>23.31</v>
+      </c>
+      <c r="AN52" s="13" t="n">
+        <v>19.18</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -5692,6 +5819,9 @@
       <c r="AM53" s="13" t="n">
         <v>12135.2</v>
       </c>
+      <c r="AN53" s="13" t="n">
+        <v>12135.2</v>
+      </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
       <c r="A54" s="3" t="n">
@@ -5781,6 +5911,7 @@
       <c r="AK54" s="13" t="n"/>
       <c r="AL54" s="13" t="n"/>
       <c r="AM54" s="13" t="n"/>
+      <c r="AN54" s="13" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -5899,6 +6030,9 @@
       </c>
       <c r="AM55" s="13" t="n">
         <v>17.72</v>
+      </c>
+      <c r="AN55" s="13" t="n">
+        <v>16.57</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -5971,6 +6105,9 @@
       <c r="AM56" s="13" t="n">
         <v>8073.5</v>
       </c>
+      <c r="AN56" s="13" t="n">
+        <v>7755.34</v>
+      </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
       <c r="A57" s="3" t="n">
@@ -6060,6 +6197,7 @@
       <c r="AK57" s="13" t="n"/>
       <c r="AL57" s="13" t="n"/>
       <c r="AM57" s="13" t="n"/>
+      <c r="AN57" s="13" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -6178,6 +6316,9 @@
       </c>
       <c r="AM58" s="13" t="n">
         <v>26.59</v>
+      </c>
+      <c r="AN58" s="13" t="n">
+        <v>25.54</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -6250,6 +6391,9 @@
       <c r="AM59" s="13" t="n">
         <v>14862.37</v>
       </c>
+      <c r="AN59" s="13" t="n">
+        <v>14251.93</v>
+      </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
       <c r="A60" s="3" t="n">
@@ -6339,6 +6483,7 @@
       <c r="AK60" s="13" t="n"/>
       <c r="AL60" s="13" t="n"/>
       <c r="AM60" s="13" t="n"/>
+      <c r="AN60" s="13" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -6457,6 +6602,9 @@
       </c>
       <c r="AM61" s="13" t="n">
         <v>38.89</v>
+      </c>
+      <c r="AN61" s="13" t="n">
+        <v>38.53</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -6529,6 +6677,9 @@
       <c r="AM62" s="13" t="n">
         <v>14265.28</v>
       </c>
+      <c r="AN62" s="13" t="n">
+        <v>13455.99</v>
+      </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
       <c r="A63" s="3" t="n">
@@ -6618,6 +6769,7 @@
       <c r="AK63" s="13" t="n"/>
       <c r="AL63" s="13" t="n"/>
       <c r="AM63" s="13" t="n"/>
+      <c r="AN63" s="13" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -6736,6 +6888,9 @@
       </c>
       <c r="AM64" s="13" t="n">
         <v>16.3</v>
+      </c>
+      <c r="AN64" s="13" t="n">
+        <v>15.55</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -6808,6 +6963,9 @@
       <c r="AM65" s="13" t="n">
         <v>8055.17</v>
       </c>
+      <c r="AN65" s="13" t="n">
+        <v>7574.13</v>
+      </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
       <c r="A66" s="3" t="n">
@@ -6897,6 +7055,7 @@
       <c r="AK66" s="13" t="n"/>
       <c r="AL66" s="13" t="n"/>
       <c r="AM66" s="13" t="n"/>
+      <c r="AN66" s="13" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -7015,6 +7174,9 @@
       </c>
       <c r="AM67" s="13" t="n">
         <v>9.039999999999999</v>
+      </c>
+      <c r="AN67" s="13" t="n">
+        <v>8.470000000000001</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -7087,6 +7249,9 @@
       <c r="AM68" s="13" t="n">
         <v>9392.139999999999</v>
       </c>
+      <c r="AN68" s="13" t="n">
+        <v>9330.690000000001</v>
+      </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
       <c r="A69" s="3" t="n">
@@ -7176,6 +7341,7 @@
       <c r="AK69" s="13" t="n"/>
       <c r="AL69" s="13" t="n"/>
       <c r="AM69" s="13" t="n"/>
+      <c r="AN69" s="13" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -7294,6 +7460,9 @@
       </c>
       <c r="AM70" s="13" t="n">
         <v>21.58</v>
+      </c>
+      <c r="AN70" s="13" t="n">
+        <v>22.6</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -7366,6 +7535,9 @@
       <c r="AM71" s="13" t="n">
         <v>2634.48</v>
       </c>
+      <c r="AN71" s="13" t="n">
+        <v>2456.89</v>
+      </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
       <c r="A72" s="3" t="n">
@@ -7455,6 +7627,7 @@
       <c r="AK72" s="13" t="n"/>
       <c r="AL72" s="13" t="n"/>
       <c r="AM72" s="13" t="n"/>
+      <c r="AN72" s="13" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -7573,6 +7746,9 @@
       </c>
       <c r="AM73" s="13" t="n">
         <v>38.07</v>
+      </c>
+      <c r="AN73" s="13" t="n">
+        <v>38.63</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -7645,6 +7821,9 @@
       <c r="AM74" s="13" t="n">
         <v>5027.69</v>
       </c>
+      <c r="AN74" s="13" t="n">
+        <v>4720.24</v>
+      </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
       <c r="A75" s="3" t="n">
@@ -7734,6 +7913,7 @@
       <c r="AK75" s="13" t="n"/>
       <c r="AL75" s="13" t="n"/>
       <c r="AM75" s="13" t="n"/>
+      <c r="AN75" s="13" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -7852,6 +8032,9 @@
       </c>
       <c r="AM76" s="13" t="n">
         <v>19.93</v>
+      </c>
+      <c r="AN76" s="13" t="n">
+        <v>17.54</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -7924,6 +8107,9 @@
       <c r="AM77" s="13" t="n">
         <v>8553.15</v>
       </c>
+      <c r="AN77" s="13" t="n">
+        <v>8134.94</v>
+      </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
       <c r="A78" s="3" t="n">
@@ -8013,6 +8199,7 @@
       <c r="AK78" s="13" t="n"/>
       <c r="AL78" s="13" t="n"/>
       <c r="AM78" s="13" t="n"/>
+      <c r="AN78" s="13" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -8131,6 +8318,9 @@
       </c>
       <c r="AM79" s="13" t="n">
         <v>16.84</v>
+      </c>
+      <c r="AN79" s="13" t="n">
+        <v>16.2</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -8203,6 +8393,9 @@
       <c r="AM80" s="13" t="n">
         <v>1392.69</v>
       </c>
+      <c r="AN80" s="13" t="n">
+        <v>1342.27</v>
+      </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
       <c r="A81" s="3" t="n">
@@ -8292,6 +8485,7 @@
       <c r="AK81" s="13" t="n"/>
       <c r="AL81" s="13" t="n"/>
       <c r="AM81" s="13" t="n"/>
+      <c r="AN81" s="13" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -8410,6 +8604,9 @@
       </c>
       <c r="AM82" s="13" t="n">
         <v>14.71</v>
+      </c>
+      <c r="AN82" s="13" t="n">
+        <v>13.82</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -8482,6 +8679,9 @@
       <c r="AM83" s="13" t="n">
         <v>16153.6</v>
       </c>
+      <c r="AN83" s="13" t="n">
+        <v>15818.37</v>
+      </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
       <c r="A84" s="3" t="n">
@@ -8571,6 +8771,7 @@
       <c r="AK84" s="13" t="n"/>
       <c r="AL84" s="13" t="n"/>
       <c r="AM84" s="13" t="n"/>
+      <c r="AN84" s="13" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -8689,6 +8890,9 @@
       </c>
       <c r="AM85" s="13" t="n">
         <v>53.41</v>
+      </c>
+      <c r="AN85" s="13" t="n">
+        <v>53.84</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -8761,6 +8965,9 @@
       <c r="AM86" s="13" t="n">
         <v>3002.99</v>
       </c>
+      <c r="AN86" s="13" t="n">
+        <v>3057.04</v>
+      </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
       <c r="A87" s="3" t="n">
@@ -8850,6 +9057,7 @@
       <c r="AK87" s="13" t="n"/>
       <c r="AL87" s="13" t="n"/>
       <c r="AM87" s="13" t="n"/>
+      <c r="AN87" s="13" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -8968,6 +9176,9 @@
       </c>
       <c r="AM88" s="13" t="n">
         <v>58.59</v>
+      </c>
+      <c r="AN88" s="13" t="n">
+        <v>58.66</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -9040,6 +9251,9 @@
       <c r="AM89" s="13" t="n">
         <v>3336.89</v>
       </c>
+      <c r="AN89" s="13" t="n">
+        <v>3362.05</v>
+      </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
       <c r="A90" s="3" t="n">
@@ -9129,6 +9343,7 @@
       <c r="AK90" s="13" t="n"/>
       <c r="AL90" s="13" t="n"/>
       <c r="AM90" s="13" t="n"/>
+      <c r="AN90" s="13" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -9246,6 +9461,9 @@
         <v>49.27</v>
       </c>
       <c r="AM91" s="13" t="n">
+        <v>48.59</v>
+      </c>
+      <c r="AN91" s="13" t="n">
         <v>48.59</v>
       </c>
     </row>
@@ -9319,6 +9537,9 @@
       <c r="AM92" s="13" t="n">
         <v>2949.03</v>
       </c>
+      <c r="AN92" s="13" t="n">
+        <v>3040.55</v>
+      </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
       <c r="A93" s="3" t="n">
@@ -9408,6 +9629,7 @@
       <c r="AK93" s="13" t="n"/>
       <c r="AL93" s="13" t="n"/>
       <c r="AM93" s="13" t="n"/>
+      <c r="AN93" s="13" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -9526,6 +9748,9 @@
       </c>
       <c r="AM94" s="13" t="n">
         <v>35.28</v>
+      </c>
+      <c r="AN94" s="13" t="n">
+        <v>32.69</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -9598,6 +9823,9 @@
       <c r="AM95" s="13" t="n">
         <v>1849.22</v>
       </c>
+      <c r="AN95" s="13" t="n">
+        <v>1727.4</v>
+      </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
       <c r="A96" s="3" t="n">
@@ -9687,6 +9915,7 @@
       <c r="AK96" s="13" t="n"/>
       <c r="AL96" s="13" t="n"/>
       <c r="AM96" s="13" t="n"/>
+      <c r="AN96" s="13" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -9805,6 +10034,9 @@
       </c>
       <c r="AM97" s="13" t="n">
         <v>26.52</v>
+      </c>
+      <c r="AN97" s="13" t="n">
+        <v>24.8</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -9877,6 +10109,9 @@
       <c r="AM98" s="13" t="n">
         <v>9960.77</v>
       </c>
+      <c r="AN98" s="13" t="n">
+        <v>9357.370000000001</v>
+      </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
       <c r="A99" s="3" t="n">
@@ -9966,6 +10201,7 @@
       <c r="AK99" s="13" t="n"/>
       <c r="AL99" s="13" t="n"/>
       <c r="AM99" s="13" t="n"/>
+      <c r="AN99" s="13" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -10084,6 +10320,9 @@
       </c>
       <c r="AM100" s="13" t="n">
         <v>85.04000000000001</v>
+      </c>
+      <c r="AN100" s="13" t="n">
+        <v>83.02</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -10156,6 +10395,9 @@
       <c r="AM101" s="13" t="n">
         <v>9688.93</v>
       </c>
+      <c r="AN101" s="13" t="n">
+        <v>9638.440000000001</v>
+      </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
       <c r="A102" s="3" t="n">
@@ -10245,6 +10487,7 @@
       <c r="AK102" s="13" t="n"/>
       <c r="AL102" s="13" t="n"/>
       <c r="AM102" s="13" t="n"/>
+      <c r="AN102" s="13" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -10363,6 +10606,9 @@
       </c>
       <c r="AM103" s="13" t="n">
         <v>58.04</v>
+      </c>
+      <c r="AN103" s="13" t="n">
+        <v>57.08</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -10435,6 +10681,9 @@
       <c r="AM104" s="13" t="n">
         <v>13964.57</v>
       </c>
+      <c r="AN104" s="13" t="n">
+        <v>13040.03</v>
+      </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
       <c r="A105" s="3" t="n">
@@ -10524,6 +10773,7 @@
       <c r="AK105" s="13" t="n"/>
       <c r="AL105" s="13" t="n"/>
       <c r="AM105" s="13" t="n"/>
+      <c r="AN105" s="13" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -10642,6 +10892,9 @@
       </c>
       <c r="AM106" s="13" t="n">
         <v>10.07</v>
+      </c>
+      <c r="AN106" s="13" t="n">
+        <v>9.4</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -10714,6 +10967,9 @@
       <c r="AM107" s="13" t="n">
         <v>2249.02</v>
       </c>
+      <c r="AN107" s="13" t="n">
+        <v>2098.11</v>
+      </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
       <c r="A108" s="3" t="n">
@@ -10803,6 +11059,7 @@
       <c r="AK108" s="13" t="n"/>
       <c r="AL108" s="13" t="n"/>
       <c r="AM108" s="13" t="n"/>
+      <c r="AN108" s="13" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -10921,6 +11178,9 @@
       </c>
       <c r="AM109" s="13" t="n">
         <v>24.35</v>
+      </c>
+      <c r="AN109" s="13" t="n">
+        <v>23.73</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -10993,6 +11253,9 @@
       <c r="AM110" s="13" t="n">
         <v>773.0700000000001</v>
       </c>
+      <c r="AN110" s="13" t="n">
+        <v>735.89</v>
+      </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
       <c r="A111" s="3" t="n">
@@ -11082,6 +11345,7 @@
       <c r="AK111" s="13" t="n"/>
       <c r="AL111" s="13" t="n"/>
       <c r="AM111" s="13" t="n"/>
+      <c r="AN111" s="13" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -11200,6 +11464,9 @@
       </c>
       <c r="AM112" s="13" t="n">
         <v>32.03</v>
+      </c>
+      <c r="AN112" s="13" t="n">
+        <v>31.03</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -11272,6 +11539,9 @@
       <c r="AM113" s="13" t="n">
         <v>3181.59</v>
       </c>
+      <c r="AN113" s="13" t="n">
+        <v>2996.71</v>
+      </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
       <c r="A114" s="3" t="n">
@@ -11361,6 +11631,7 @@
       <c r="AK114" s="13" t="n"/>
       <c r="AL114" s="13" t="n"/>
       <c r="AM114" s="13" t="n"/>
+      <c r="AN114" s="13" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -11479,6 +11750,9 @@
       </c>
       <c r="AM115" s="13" t="n">
         <v>23.32</v>
+      </c>
+      <c r="AN115" s="13" t="n">
+        <v>21.89</v>
       </c>
     </row>
     <row r="116">
@@ -11535,6 +11809,9 @@
       </c>
       <c r="AM116" s="13" t="n">
         <v>4151.11</v>
+      </c>
+      <c r="AN116" s="13" t="n">
+        <v>3952.96</v>
       </c>
     </row>
     <row r="117">
@@ -11580,6 +11857,7 @@
       <c r="AK117" s="13" t="n"/>
       <c r="AL117" s="13" t="n"/>
       <c r="AM117" s="13" t="n"/>
+      <c r="AN117" s="13" t="n"/>
     </row>
     <row r="118">
       <c r="P118" s="13" t="n">
@@ -11654,6 +11932,9 @@
       <c r="AM118" s="13" t="n">
         <v>29.02</v>
       </c>
+      <c r="AN118" s="13" t="n">
+        <v>29.02</v>
+      </c>
     </row>
     <row r="119">
       <c r="Y119" s="13" t="n">
@@ -11699,6 +11980,9 @@
         <v>2925.77</v>
       </c>
       <c r="AM119" s="13" t="n">
+        <v>2854.7</v>
+      </c>
+      <c r="AN119" s="13" t="n">
         <v>2854.7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-03-26 05:24:48]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN119"/>
+  <dimension ref="A1:AO119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="15"/>
@@ -557,6 +557,7 @@
     <col width="15" customWidth="1" min="38" max="38"/>
     <col width="15" customWidth="1" min="39" max="39"/>
     <col width="15" customWidth="1" min="40" max="40"/>
+    <col width="15" customWidth="1" min="41" max="41"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -760,6 +761,11 @@
           <t>2026/03/23</t>
         </is>
       </c>
+      <c r="AO1" s="13" t="inlineStr">
+        <is>
+          <t>2026/03/26</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -962,6 +968,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="AO2" s="14" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1084,6 +1095,9 @@
       <c r="AN3" s="13" t="n">
         <v>68.06999999999999</v>
       </c>
+      <c r="AO3" s="13" t="n">
+        <v>67.52</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1205,6 +1219,9 @@
       </c>
       <c r="AN4" s="13" t="n">
         <v>3849.59</v>
+      </c>
+      <c r="AO4" s="13" t="n">
+        <v>3895.73</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1248,6 +1265,7 @@
       <c r="AL5" s="13" t="n"/>
       <c r="AM5" s="13" t="n"/>
       <c r="AN5" s="13" t="n"/>
+      <c r="AO5" s="13" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1338,6 +1356,7 @@
       <c r="AL6" s="13" t="n"/>
       <c r="AM6" s="13" t="n"/>
       <c r="AN6" s="13" t="n"/>
+      <c r="AO6" s="13" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1459,6 +1478,9 @@
       </c>
       <c r="AN7" s="13" t="n">
         <v>49.95</v>
+      </c>
+      <c r="AO7" s="13" t="n">
+        <v>49.3</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -1534,6 +1556,9 @@
       <c r="AN8" s="13" t="n">
         <v>5515.26</v>
       </c>
+      <c r="AO8" s="13" t="n">
+        <v>5560.52</v>
+      </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -1624,6 +1649,7 @@
       <c r="AL9" s="13" t="n"/>
       <c r="AM9" s="13" t="n"/>
       <c r="AN9" s="13" t="n"/>
+      <c r="AO9" s="13" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -1745,6 +1771,9 @@
       </c>
       <c r="AN10" s="13" t="n">
         <v>52.83</v>
+      </c>
+      <c r="AO10" s="13" t="n">
+        <v>51.86</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -1820,6 +1849,9 @@
       <c r="AN11" s="13" t="n">
         <v>4452.87</v>
       </c>
+      <c r="AO11" s="13" t="n">
+        <v>4486.37</v>
+      </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -1910,6 +1942,7 @@
       <c r="AL12" s="13" t="n"/>
       <c r="AM12" s="13" t="n"/>
       <c r="AN12" s="13" t="n"/>
+      <c r="AO12" s="13" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2031,6 +2064,9 @@
       </c>
       <c r="AN13" s="13" t="n">
         <v>59.81</v>
+      </c>
+      <c r="AO13" s="13" t="n">
+        <v>59.98</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -2106,6 +2142,9 @@
       <c r="AN14" s="13" t="n">
         <v>7524.97</v>
       </c>
+      <c r="AO14" s="13" t="n">
+        <v>7638.14</v>
+      </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -2196,6 +2235,7 @@
       <c r="AL15" s="13" t="n"/>
       <c r="AM15" s="13" t="n"/>
       <c r="AN15" s="13" t="n"/>
+      <c r="AO15" s="13" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -2317,6 +2357,9 @@
       </c>
       <c r="AN16" s="13" t="n">
         <v>27.09</v>
+      </c>
+      <c r="AO16" s="13" t="n">
+        <v>26.02</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -2392,6 +2435,9 @@
       <c r="AN17" s="13" t="n">
         <v>2652.96</v>
       </c>
+      <c r="AO17" s="13" t="n">
+        <v>2548.76</v>
+      </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="3" t="n">
@@ -2482,6 +2528,7 @@
       <c r="AL18" s="13" t="n"/>
       <c r="AM18" s="13" t="n"/>
       <c r="AN18" s="13" t="n"/>
+      <c r="AO18" s="13" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -2603,6 +2650,9 @@
       </c>
       <c r="AN19" s="13" t="n">
         <v>92.77</v>
+      </c>
+      <c r="AO19" s="13" t="n">
+        <v>93.40000000000001</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -2678,6 +2728,9 @@
       <c r="AN20" s="13" t="n">
         <v>6506.48</v>
       </c>
+      <c r="AO20" s="13" t="n">
+        <v>6591.9</v>
+      </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -2768,6 +2821,7 @@
       <c r="AL21" s="13" t="n"/>
       <c r="AM21" s="13" t="n"/>
       <c r="AN21" s="13" t="n"/>
+      <c r="AO21" s="13" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -2887,6 +2941,9 @@
       </c>
       <c r="AN22" s="13" t="n">
         <v>49.47</v>
+      </c>
+      <c r="AO22" s="13" t="n">
+        <v>50.78</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1">
@@ -2962,6 +3019,9 @@
       <c r="AN23" s="13" t="n">
         <v>72759.96000000001</v>
       </c>
+      <c r="AO23" s="13" t="n">
+        <v>75273.45</v>
+      </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="3" t="n">
@@ -3052,6 +3112,7 @@
       <c r="AL24" s="13" t="n"/>
       <c r="AM24" s="13" t="n"/>
       <c r="AN24" s="13" t="n"/>
+      <c r="AO24" s="13" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -3173,6 +3234,9 @@
       </c>
       <c r="AN25" s="13" t="n">
         <v>75.02</v>
+      </c>
+      <c r="AO25" s="13" t="n">
+        <v>74.3</v>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="1">
@@ -3248,6 +3312,9 @@
       <c r="AN26" s="13" t="n">
         <v>22380.19</v>
       </c>
+      <c r="AO26" s="13" t="n">
+        <v>22957.08</v>
+      </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -3338,6 +3405,7 @@
       <c r="AL27" s="13" t="n"/>
       <c r="AM27" s="13" t="n"/>
       <c r="AN27" s="13" t="n"/>
+      <c r="AO27" s="13" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -3459,6 +3527,9 @@
       </c>
       <c r="AN28" s="13" t="n">
         <v>70.17</v>
+      </c>
+      <c r="AO28" s="13" t="n">
+        <v>67.98</v>
       </c>
     </row>
     <row r="29" ht="14.25" customHeight="1">
@@ -3534,6 +3605,9 @@
       <c r="AN29" s="13" t="n">
         <v>51589.75</v>
       </c>
+      <c r="AO29" s="13" t="n">
+        <v>53297.88</v>
+      </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="3" t="n">
@@ -3624,6 +3698,7 @@
       <c r="AL30" s="13" t="n"/>
       <c r="AM30" s="13" t="n"/>
       <c r="AN30" s="13" t="n"/>
+      <c r="AO30" s="13" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -3745,6 +3820,9 @@
       </c>
       <c r="AN31" s="13" t="n">
         <v>51.92</v>
+      </c>
+      <c r="AO31" s="13" t="n">
+        <v>52.08</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -3820,6 +3898,9 @@
       <c r="AN32" s="13" t="n">
         <v>5677.17</v>
       </c>
+      <c r="AO32" s="13" t="n">
+        <v>5729.98</v>
+      </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
       <c r="A33" s="3" t="n">
@@ -3910,6 +3991,7 @@
       <c r="AL33" s="13" t="n"/>
       <c r="AM33" s="13" t="n"/>
       <c r="AN33" s="13" t="n"/>
+      <c r="AO33" s="13" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -4031,6 +4113,9 @@
       </c>
       <c r="AN34" s="13" t="n">
         <v>2.79</v>
+      </c>
+      <c r="AO34" s="13" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -4106,6 +4191,9 @@
       <c r="AN35" s="13" t="n">
         <v>31921.84</v>
       </c>
+      <c r="AO35" s="13" t="n">
+        <v>32531.19</v>
+      </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="3" t="n">
@@ -4196,6 +4284,7 @@
       <c r="AL36" s="13" t="n"/>
       <c r="AM36" s="13" t="n"/>
       <c r="AN36" s="13" t="n"/>
+      <c r="AO36" s="13" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -4317,6 +4406,9 @@
       </c>
       <c r="AN37" s="13" t="n">
         <v>29.22</v>
+      </c>
+      <c r="AO37" s="13" t="n">
+        <v>28.7</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -4392,6 +4484,9 @@
       <c r="AN38" s="13" t="n">
         <v>3467.53</v>
       </c>
+      <c r="AO38" s="13" t="n">
+        <v>3466.96</v>
+      </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
       <c r="A39" s="3" t="n">
@@ -4482,6 +4577,7 @@
       <c r="AL39" s="13" t="n"/>
       <c r="AM39" s="13" t="n"/>
       <c r="AN39" s="13" t="n"/>
+      <c r="AO39" s="13" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -4603,6 +4699,9 @@
       </c>
       <c r="AN40" s="13" t="n">
         <v>49.3</v>
+      </c>
+      <c r="AO40" s="13" t="n">
+        <v>48.55</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -4678,6 +4777,9 @@
       <c r="AN41" s="13" t="n">
         <v>3274.84</v>
       </c>
+      <c r="AO41" s="13" t="n">
+        <v>3280.05</v>
+      </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
       <c r="A42" s="3" t="n">
@@ -4768,6 +4870,7 @@
       <c r="AL42" s="13" t="n"/>
       <c r="AM42" s="13" t="n"/>
       <c r="AN42" s="13" t="n"/>
+      <c r="AO42" s="13" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -4889,6 +4992,9 @@
       </c>
       <c r="AN43" s="13" t="n">
         <v>12.29</v>
+      </c>
+      <c r="AO43" s="13" t="n">
+        <v>7.67</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -4964,6 +5070,9 @@
       <c r="AN44" s="13" t="n">
         <v>6251.37</v>
       </c>
+      <c r="AO44" s="13" t="n">
+        <v>6343.57</v>
+      </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
       <c r="A45" s="3" t="n">
@@ -5054,6 +5163,7 @@
       <c r="AL45" s="13" t="n"/>
       <c r="AM45" s="13" t="n"/>
       <c r="AN45" s="13" t="n"/>
+      <c r="AO45" s="13" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -5175,6 +5285,9 @@
       </c>
       <c r="AN46" s="13" t="n">
         <v>18.98</v>
+      </c>
+      <c r="AO46" s="13" t="n">
+        <v>14.67</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -5250,6 +5363,9 @@
       <c r="AN47" s="13" t="n">
         <v>7601.72</v>
       </c>
+      <c r="AO47" s="13" t="n">
+        <v>7656.31</v>
+      </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
       <c r="A48" s="3" t="n">
@@ -5340,6 +5456,7 @@
       <c r="AL48" s="13" t="n"/>
       <c r="AM48" s="13" t="n"/>
       <c r="AN48" s="13" t="n"/>
+      <c r="AO48" s="13" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -5461,6 +5578,9 @@
       </c>
       <c r="AN49" s="13" t="n">
         <v>6.5</v>
+      </c>
+      <c r="AO49" s="13" t="n">
+        <v>5.85</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -5536,6 +5656,9 @@
       <c r="AN50" s="13" t="n">
         <v>11587.45</v>
       </c>
+      <c r="AO50" s="13" t="n">
+        <v>11587.45</v>
+      </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
       <c r="A51" s="3" t="n">
@@ -5626,6 +5749,7 @@
       <c r="AL51" s="13" t="n"/>
       <c r="AM51" s="13" t="n"/>
       <c r="AN51" s="13" t="n"/>
+      <c r="AO51" s="13" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -5747,6 +5871,9 @@
       </c>
       <c r="AN52" s="13" t="n">
         <v>19.18</v>
+      </c>
+      <c r="AO52" s="13" t="n">
+        <v>17.73</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -5822,6 +5949,9 @@
       <c r="AN53" s="13" t="n">
         <v>12135.2</v>
       </c>
+      <c r="AO53" s="13" t="n">
+        <v>12546.64</v>
+      </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
       <c r="A54" s="3" t="n">
@@ -5912,6 +6042,7 @@
       <c r="AL54" s="13" t="n"/>
       <c r="AM54" s="13" t="n"/>
       <c r="AN54" s="13" t="n"/>
+      <c r="AO54" s="13" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -6033,6 +6164,9 @@
       </c>
       <c r="AN55" s="13" t="n">
         <v>16.57</v>
+      </c>
+      <c r="AO55" s="13" t="n">
+        <v>15.43</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -6108,6 +6242,9 @@
       <c r="AN56" s="13" t="n">
         <v>7755.34</v>
       </c>
+      <c r="AO56" s="13" t="n">
+        <v>7734.45</v>
+      </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
       <c r="A57" s="3" t="n">
@@ -6198,6 +6335,7 @@
       <c r="AL57" s="13" t="n"/>
       <c r="AM57" s="13" t="n"/>
       <c r="AN57" s="13" t="n"/>
+      <c r="AO57" s="13" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -6319,6 +6457,9 @@
       </c>
       <c r="AN58" s="13" t="n">
         <v>25.54</v>
+      </c>
+      <c r="AO58" s="13" t="n">
+        <v>23.53</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -6394,6 +6535,9 @@
       <c r="AN59" s="13" t="n">
         <v>14251.93</v>
       </c>
+      <c r="AO59" s="13" t="n">
+        <v>14269.55</v>
+      </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
       <c r="A60" s="3" t="n">
@@ -6484,6 +6628,7 @@
       <c r="AL60" s="13" t="n"/>
       <c r="AM60" s="13" t="n"/>
       <c r="AN60" s="13" t="n"/>
+      <c r="AO60" s="13" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -6605,6 +6750,9 @@
       </c>
       <c r="AN61" s="13" t="n">
         <v>38.53</v>
+      </c>
+      <c r="AO61" s="13" t="n">
+        <v>37.27</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -6680,6 +6828,9 @@
       <c r="AN62" s="13" t="n">
         <v>13455.99</v>
       </c>
+      <c r="AO62" s="13" t="n">
+        <v>13810.33</v>
+      </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
       <c r="A63" s="3" t="n">
@@ -6770,6 +6921,7 @@
       <c r="AL63" s="13" t="n"/>
       <c r="AM63" s="13" t="n"/>
       <c r="AN63" s="13" t="n"/>
+      <c r="AO63" s="13" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -6891,6 +7043,9 @@
       </c>
       <c r="AN64" s="13" t="n">
         <v>15.55</v>
+      </c>
+      <c r="AO64" s="13" t="n">
+        <v>16.41</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -6966,6 +7121,9 @@
       <c r="AN65" s="13" t="n">
         <v>7574.13</v>
       </c>
+      <c r="AO65" s="13" t="n">
+        <v>7739.92</v>
+      </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
       <c r="A66" s="3" t="n">
@@ -7056,6 +7214,7 @@
       <c r="AL66" s="13" t="n"/>
       <c r="AM66" s="13" t="n"/>
       <c r="AN66" s="13" t="n"/>
+      <c r="AO66" s="13" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -7177,6 +7336,9 @@
       </c>
       <c r="AN67" s="13" t="n">
         <v>8.470000000000001</v>
+      </c>
+      <c r="AO67" s="13" t="n">
+        <v>7.28</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -7252,6 +7414,9 @@
       <c r="AN68" s="13" t="n">
         <v>9330.690000000001</v>
       </c>
+      <c r="AO68" s="13" t="n">
+        <v>9330.690000000001</v>
+      </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
       <c r="A69" s="3" t="n">
@@ -7342,6 +7507,7 @@
       <c r="AL69" s="13" t="n"/>
       <c r="AM69" s="13" t="n"/>
       <c r="AN69" s="13" t="n"/>
+      <c r="AO69" s="13" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -7463,6 +7629,9 @@
       </c>
       <c r="AN70" s="13" t="n">
         <v>22.6</v>
+      </c>
+      <c r="AO70" s="13" t="n">
+        <v>22.77</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -7538,6 +7707,9 @@
       <c r="AN71" s="13" t="n">
         <v>2456.89</v>
       </c>
+      <c r="AO71" s="13" t="n">
+        <v>2491.46</v>
+      </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
       <c r="A72" s="3" t="n">
@@ -7628,6 +7800,7 @@
       <c r="AL72" s="13" t="n"/>
       <c r="AM72" s="13" t="n"/>
       <c r="AN72" s="13" t="n"/>
+      <c r="AO72" s="13" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -7749,6 +7922,9 @@
       </c>
       <c r="AN73" s="13" t="n">
         <v>38.63</v>
+      </c>
+      <c r="AO73" s="13" t="n">
+        <v>39.25</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -7824,6 +8000,9 @@
       <c r="AN74" s="13" t="n">
         <v>4720.24</v>
       </c>
+      <c r="AO74" s="13" t="n">
+        <v>4800.87</v>
+      </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
       <c r="A75" s="3" t="n">
@@ -7914,6 +8093,7 @@
       <c r="AL75" s="13" t="n"/>
       <c r="AM75" s="13" t="n"/>
       <c r="AN75" s="13" t="n"/>
+      <c r="AO75" s="13" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -8035,6 +8215,9 @@
       </c>
       <c r="AN76" s="13" t="n">
         <v>17.54</v>
+      </c>
+      <c r="AO76" s="13" t="n">
+        <v>13.3</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -8110,6 +8293,9 @@
       <c r="AN77" s="13" t="n">
         <v>8134.94</v>
       </c>
+      <c r="AO77" s="13" t="n">
+        <v>8220.4</v>
+      </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
       <c r="A78" s="3" t="n">
@@ -8200,6 +8386,7 @@
       <c r="AL78" s="13" t="n"/>
       <c r="AM78" s="13" t="n"/>
       <c r="AN78" s="13" t="n"/>
+      <c r="AO78" s="13" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -8321,6 +8508,9 @@
       </c>
       <c r="AN79" s="13" t="n">
         <v>16.2</v>
+      </c>
+      <c r="AO79" s="13" t="n">
+        <v>15.84</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -8396,6 +8586,9 @@
       <c r="AN80" s="13" t="n">
         <v>1342.27</v>
       </c>
+      <c r="AO80" s="13" t="n">
+        <v>1314.77</v>
+      </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
       <c r="A81" s="3" t="n">
@@ -8486,6 +8679,7 @@
       <c r="AL81" s="13" t="n"/>
       <c r="AM81" s="13" t="n"/>
       <c r="AN81" s="13" t="n"/>
+      <c r="AO81" s="13" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -8607,6 +8801,9 @@
       </c>
       <c r="AN82" s="13" t="n">
         <v>13.82</v>
+      </c>
+      <c r="AO82" s="13" t="n">
+        <v>13.22</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -8682,6 +8879,9 @@
       <c r="AN83" s="13" t="n">
         <v>15818.37</v>
       </c>
+      <c r="AO83" s="13" t="n">
+        <v>15561.64</v>
+      </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
       <c r="A84" s="3" t="n">
@@ -8772,6 +8972,7 @@
       <c r="AL84" s="13" t="n"/>
       <c r="AM84" s="13" t="n"/>
       <c r="AN84" s="13" t="n"/>
+      <c r="AO84" s="13" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -8893,6 +9094,9 @@
       </c>
       <c r="AN85" s="13" t="n">
         <v>53.84</v>
+      </c>
+      <c r="AO85" s="13" t="n">
+        <v>53.89</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -8968,6 +9172,9 @@
       <c r="AN86" s="13" t="n">
         <v>3057.04</v>
       </c>
+      <c r="AO86" s="13" t="n">
+        <v>3063</v>
+      </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
       <c r="A87" s="3" t="n">
@@ -9058,6 +9265,7 @@
       <c r="AL87" s="13" t="n"/>
       <c r="AM87" s="13" t="n"/>
       <c r="AN87" s="13" t="n"/>
+      <c r="AO87" s="13" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -9179,6 +9387,9 @@
       </c>
       <c r="AN88" s="13" t="n">
         <v>58.66</v>
+      </c>
+      <c r="AO88" s="13" t="n">
+        <v>58.37</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -9254,6 +9465,9 @@
       <c r="AN89" s="13" t="n">
         <v>3362.05</v>
       </c>
+      <c r="AO89" s="13" t="n">
+        <v>3327.93</v>
+      </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
       <c r="A90" s="3" t="n">
@@ -9344,6 +9558,7 @@
       <c r="AL90" s="13" t="n"/>
       <c r="AM90" s="13" t="n"/>
       <c r="AN90" s="13" t="n"/>
+      <c r="AO90" s="13" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -9465,6 +9680,9 @@
       </c>
       <c r="AN91" s="13" t="n">
         <v>48.59</v>
+      </c>
+      <c r="AO91" s="13" t="n">
+        <v>48.48</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -9540,6 +9758,9 @@
       <c r="AN92" s="13" t="n">
         <v>3040.55</v>
       </c>
+      <c r="AO92" s="13" t="n">
+        <v>2949.03</v>
+      </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
       <c r="A93" s="3" t="n">
@@ -9630,6 +9851,7 @@
       <c r="AL93" s="13" t="n"/>
       <c r="AM93" s="13" t="n"/>
       <c r="AN93" s="13" t="n"/>
+      <c r="AO93" s="13" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -9751,6 +9973,9 @@
       </c>
       <c r="AN94" s="13" t="n">
         <v>32.69</v>
+      </c>
+      <c r="AO94" s="13" t="n">
+        <v>23.82</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -9826,6 +10051,9 @@
       <c r="AN95" s="13" t="n">
         <v>1727.4</v>
       </c>
+      <c r="AO95" s="13" t="n">
+        <v>1760.24</v>
+      </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
       <c r="A96" s="3" t="n">
@@ -9916,6 +10144,7 @@
       <c r="AL96" s="13" t="n"/>
       <c r="AM96" s="13" t="n"/>
       <c r="AN96" s="13" t="n"/>
+      <c r="AO96" s="13" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -10037,6 +10266,9 @@
       </c>
       <c r="AN97" s="13" t="n">
         <v>24.8</v>
+      </c>
+      <c r="AO97" s="13" t="n">
+        <v>24.26</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -10112,6 +10344,9 @@
       <c r="AN98" s="13" t="n">
         <v>9357.370000000001</v>
       </c>
+      <c r="AO98" s="13" t="n">
+        <v>9414.73</v>
+      </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
       <c r="A99" s="3" t="n">
@@ -10202,6 +10437,7 @@
       <c r="AL99" s="13" t="n"/>
       <c r="AM99" s="13" t="n"/>
       <c r="AN99" s="13" t="n"/>
+      <c r="AO99" s="13" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -10323,6 +10559,9 @@
       </c>
       <c r="AN100" s="13" t="n">
         <v>83.02</v>
+      </c>
+      <c r="AO100" s="13" t="n">
+        <v>82.66</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -10398,6 +10637,9 @@
       <c r="AN101" s="13" t="n">
         <v>9638.440000000001</v>
       </c>
+      <c r="AO101" s="13" t="n">
+        <v>9137.360000000001</v>
+      </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
       <c r="A102" s="3" t="n">
@@ -10488,6 +10730,7 @@
       <c r="AL102" s="13" t="n"/>
       <c r="AM102" s="13" t="n"/>
       <c r="AN102" s="13" t="n"/>
+      <c r="AO102" s="13" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -10609,6 +10852,9 @@
       </c>
       <c r="AN103" s="13" t="n">
         <v>57.08</v>
+      </c>
+      <c r="AO103" s="13" t="n">
+        <v>57.06</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -10684,6 +10930,9 @@
       <c r="AN104" s="13" t="n">
         <v>13040.03</v>
       </c>
+      <c r="AO104" s="13" t="n">
+        <v>13101.33</v>
+      </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
       <c r="A105" s="3" t="n">
@@ -10774,6 +11023,7 @@
       <c r="AL105" s="13" t="n"/>
       <c r="AM105" s="13" t="n"/>
       <c r="AN105" s="13" t="n"/>
+      <c r="AO105" s="13" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -10895,6 +11145,9 @@
       </c>
       <c r="AN106" s="13" t="n">
         <v>9.4</v>
+      </c>
+      <c r="AO106" s="13" t="n">
+        <v>7.63</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -10970,6 +11223,9 @@
       <c r="AN107" s="13" t="n">
         <v>2098.11</v>
       </c>
+      <c r="AO107" s="13" t="n">
+        <v>2275.37</v>
+      </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
       <c r="A108" s="3" t="n">
@@ -11060,6 +11316,7 @@
       <c r="AL108" s="13" t="n"/>
       <c r="AM108" s="13" t="n"/>
       <c r="AN108" s="13" t="n"/>
+      <c r="AO108" s="13" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -11181,6 +11438,9 @@
       </c>
       <c r="AN109" s="13" t="n">
         <v>23.73</v>
+      </c>
+      <c r="AO109" s="13" t="n">
+        <v>23.54</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -11256,6 +11516,9 @@
       <c r="AN110" s="13" t="n">
         <v>735.89</v>
       </c>
+      <c r="AO110" s="13" t="n">
+        <v>728.17</v>
+      </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
       <c r="A111" s="3" t="n">
@@ -11346,6 +11609,7 @@
       <c r="AL111" s="13" t="n"/>
       <c r="AM111" s="13" t="n"/>
       <c r="AN111" s="13" t="n"/>
+      <c r="AO111" s="13" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -11467,6 +11731,9 @@
       </c>
       <c r="AN112" s="13" t="n">
         <v>31.03</v>
+      </c>
+      <c r="AO112" s="13" t="n">
+        <v>30.5</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -11542,6 +11809,9 @@
       <c r="AN113" s="13" t="n">
         <v>2996.71</v>
       </c>
+      <c r="AO113" s="13" t="n">
+        <v>3082.03</v>
+      </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
       <c r="A114" s="3" t="n">
@@ -11632,6 +11902,7 @@
       <c r="AL114" s="13" t="n"/>
       <c r="AM114" s="13" t="n"/>
       <c r="AN114" s="13" t="n"/>
+      <c r="AO114" s="13" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -11753,6 +12024,9 @@
       </c>
       <c r="AN115" s="13" t="n">
         <v>21.89</v>
+      </c>
+      <c r="AO115" s="13" t="n">
+        <v>22.31</v>
       </c>
     </row>
     <row r="116">
@@ -11812,6 +12086,9 @@
       </c>
       <c r="AN116" s="13" t="n">
         <v>3952.96</v>
+      </c>
+      <c r="AO116" s="13" t="n">
+        <v>4045.82</v>
       </c>
     </row>
     <row r="117">
@@ -11858,6 +12135,7 @@
       <c r="AL117" s="13" t="n"/>
       <c r="AM117" s="13" t="n"/>
       <c r="AN117" s="13" t="n"/>
+      <c r="AO117" s="13" t="n"/>
     </row>
     <row r="118">
       <c r="P118" s="13" t="n">
@@ -11935,6 +12213,9 @@
       <c r="AN118" s="13" t="n">
         <v>29.02</v>
       </c>
+      <c r="AO118" s="13" t="n">
+        <v>29.02</v>
+      </c>
     </row>
     <row r="119">
       <c r="Y119" s="13" t="n">
@@ -11984,6 +12265,9 @@
       </c>
       <c r="AN119" s="13" t="n">
         <v>2854.7</v>
+      </c>
+      <c r="AO119" s="13" t="n">
+        <v>2727.34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-04-02 05:22:25]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO119"/>
+  <dimension ref="A1:AP119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="15"/>
@@ -558,6 +558,7 @@
     <col width="15" customWidth="1" min="39" max="39"/>
     <col width="15" customWidth="1" min="40" max="40"/>
     <col width="15" customWidth="1" min="41" max="41"/>
+    <col width="15" customWidth="1" min="42" max="42"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -766,6 +767,11 @@
           <t>2026/03/26</t>
         </is>
       </c>
+      <c r="AP1" s="13" t="inlineStr">
+        <is>
+          <t>2026/04/02</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -973,6 +979,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="AP2" s="14" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1098,6 +1109,9 @@
       <c r="AO3" s="13" t="n">
         <v>67.52</v>
       </c>
+      <c r="AP3" s="13" t="n">
+        <v>63.22</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1222,6 +1236,9 @@
       </c>
       <c r="AO4" s="13" t="n">
         <v>3895.73</v>
+      </c>
+      <c r="AP4" s="13" t="n">
+        <v>3914.46</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1266,6 +1283,7 @@
       <c r="AM5" s="13" t="n"/>
       <c r="AN5" s="13" t="n"/>
       <c r="AO5" s="13" t="n"/>
+      <c r="AP5" s="13" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1357,6 +1375,7 @@
       <c r="AM6" s="13" t="n"/>
       <c r="AN6" s="13" t="n"/>
       <c r="AO6" s="13" t="n"/>
+      <c r="AP6" s="13" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1481,6 +1500,9 @@
       </c>
       <c r="AO7" s="13" t="n">
         <v>49.3</v>
+      </c>
+      <c r="AP7" s="13" t="n">
+        <v>59.52</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -1559,6 +1581,9 @@
       <c r="AO8" s="13" t="n">
         <v>5560.52</v>
       </c>
+      <c r="AP8" s="13" t="n">
+        <v>5544.27</v>
+      </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -1650,6 +1675,7 @@
       <c r="AM9" s="13" t="n"/>
       <c r="AN9" s="13" t="n"/>
       <c r="AO9" s="13" t="n"/>
+      <c r="AP9" s="13" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -1774,6 +1800,9 @@
       </c>
       <c r="AO10" s="13" t="n">
         <v>51.86</v>
+      </c>
+      <c r="AP10" s="13" t="n">
+        <v>49.63</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -1852,6 +1881,9 @@
       <c r="AO11" s="13" t="n">
         <v>4486.37</v>
       </c>
+      <c r="AP11" s="13" t="n">
+        <v>4473.71</v>
+      </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -1943,6 +1975,7 @@
       <c r="AM12" s="13" t="n"/>
       <c r="AN12" s="13" t="n"/>
       <c r="AO12" s="13" t="n"/>
+      <c r="AP12" s="13" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2067,6 +2100,9 @@
       </c>
       <c r="AO13" s="13" t="n">
         <v>59.98</v>
+      </c>
+      <c r="AP13" s="13" t="n">
+        <v>62.42</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -2145,6 +2181,9 @@
       <c r="AO14" s="13" t="n">
         <v>7638.14</v>
       </c>
+      <c r="AP14" s="13" t="n">
+        <v>7607.01</v>
+      </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -2236,6 +2275,7 @@
       <c r="AM15" s="13" t="n"/>
       <c r="AN15" s="13" t="n"/>
       <c r="AO15" s="13" t="n"/>
+      <c r="AP15" s="13" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -2360,6 +2400,9 @@
       </c>
       <c r="AO16" s="13" t="n">
         <v>26.02</v>
+      </c>
+      <c r="AP16" s="13" t="n">
+        <v>31.71</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -2438,6 +2481,9 @@
       <c r="AO17" s="13" t="n">
         <v>2548.76</v>
       </c>
+      <c r="AP17" s="13" t="n">
+        <v>2652.96</v>
+      </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="3" t="n">
@@ -2529,6 +2575,7 @@
       <c r="AM18" s="13" t="n"/>
       <c r="AN18" s="13" t="n"/>
       <c r="AO18" s="13" t="n"/>
+      <c r="AP18" s="13" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -2653,6 +2700,9 @@
       </c>
       <c r="AO19" s="13" t="n">
         <v>93.40000000000001</v>
+      </c>
+      <c r="AP19" s="13" t="n">
+        <v>88.5</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -2731,6 +2781,9 @@
       <c r="AO20" s="13" t="n">
         <v>6591.9</v>
       </c>
+      <c r="AP20" s="13" t="n">
+        <v>6575.32</v>
+      </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -2822,6 +2875,7 @@
       <c r="AM21" s="13" t="n"/>
       <c r="AN21" s="13" t="n"/>
       <c r="AO21" s="13" t="n"/>
+      <c r="AP21" s="13" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -2944,6 +2998,9 @@
       </c>
       <c r="AO22" s="13" t="n">
         <v>50.78</v>
+      </c>
+      <c r="AP22" s="13" t="n">
+        <v>34.86</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1">
@@ -3022,6 +3079,9 @@
       <c r="AO23" s="13" t="n">
         <v>75273.45</v>
       </c>
+      <c r="AP23" s="13" t="n">
+        <v>71645.14</v>
+      </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="3" t="n">
@@ -3113,6 +3173,7 @@
       <c r="AM24" s="13" t="n"/>
       <c r="AN24" s="13" t="n"/>
       <c r="AO24" s="13" t="n"/>
+      <c r="AP24" s="13" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -3237,6 +3298,9 @@
       </c>
       <c r="AO25" s="13" t="n">
         <v>74.3</v>
+      </c>
+      <c r="AP25" s="13" t="n">
+        <v>35.16</v>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="1">
@@ -3315,6 +3379,9 @@
       <c r="AO26" s="13" t="n">
         <v>22957.08</v>
       </c>
+      <c r="AP26" s="13" t="n">
+        <v>23298.89</v>
+      </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -3406,6 +3473,7 @@
       <c r="AM27" s="13" t="n"/>
       <c r="AN27" s="13" t="n"/>
       <c r="AO27" s="13" t="n"/>
+      <c r="AP27" s="13" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -3530,6 +3598,9 @@
       </c>
       <c r="AO28" s="13" t="n">
         <v>67.98</v>
+      </c>
+      <c r="AP28" s="13" t="n">
+        <v>77.45</v>
       </c>
     </row>
     <row r="29" ht="14.25" customHeight="1">
@@ -3608,6 +3679,9 @@
       <c r="AO29" s="13" t="n">
         <v>53297.88</v>
       </c>
+      <c r="AP29" s="13" t="n">
+        <v>52421.04</v>
+      </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="3" t="n">
@@ -3699,6 +3773,7 @@
       <c r="AM30" s="13" t="n"/>
       <c r="AN30" s="13" t="n"/>
       <c r="AO30" s="13" t="n"/>
+      <c r="AP30" s="13" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -3823,6 +3898,9 @@
       </c>
       <c r="AO31" s="13" t="n">
         <v>52.08</v>
+      </c>
+      <c r="AP31" s="13" t="n">
+        <v>53.79</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -3901,6 +3979,9 @@
       <c r="AO32" s="13" t="n">
         <v>5729.98</v>
       </c>
+      <c r="AP32" s="13" t="n">
+        <v>5735.1</v>
+      </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
       <c r="A33" s="3" t="n">
@@ -3992,6 +4073,7 @@
       <c r="AM33" s="13" t="n"/>
       <c r="AN33" s="13" t="n"/>
       <c r="AO33" s="13" t="n"/>
+      <c r="AP33" s="13" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -4116,6 +4198,9 @@
       </c>
       <c r="AO34" s="13" t="n">
         <v>2</v>
+      </c>
+      <c r="AP34" s="13" t="n">
+        <v>1.4</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -4194,6 +4279,9 @@
       <c r="AO35" s="13" t="n">
         <v>32531.19</v>
       </c>
+      <c r="AP35" s="13" t="n">
+        <v>32685.33</v>
+      </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="3" t="n">
@@ -4285,6 +4373,7 @@
       <c r="AM36" s="13" t="n"/>
       <c r="AN36" s="13" t="n"/>
       <c r="AO36" s="13" t="n"/>
+      <c r="AP36" s="13" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -4409,6 +4498,9 @@
       </c>
       <c r="AO37" s="13" t="n">
         <v>28.7</v>
+      </c>
+      <c r="AP37" s="13" t="n">
+        <v>42.45</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -4487,6 +4579,9 @@
       <c r="AO38" s="13" t="n">
         <v>3466.96</v>
       </c>
+      <c r="AP38" s="13" t="n">
+        <v>3333.11</v>
+      </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
       <c r="A39" s="3" t="n">
@@ -4578,6 +4673,7 @@
       <c r="AM39" s="13" t="n"/>
       <c r="AN39" s="13" t="n"/>
       <c r="AO39" s="13" t="n"/>
+      <c r="AP39" s="13" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -4702,6 +4798,9 @@
       </c>
       <c r="AO40" s="13" t="n">
         <v>48.55</v>
+      </c>
+      <c r="AP40" s="13" t="n">
+        <v>44.02</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -4780,6 +4879,9 @@
       <c r="AO41" s="13" t="n">
         <v>3280.05</v>
       </c>
+      <c r="AP41" s="13" t="n">
+        <v>3169.1</v>
+      </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
       <c r="A42" s="3" t="n">
@@ -4871,6 +4973,7 @@
       <c r="AM42" s="13" t="n"/>
       <c r="AN42" s="13" t="n"/>
       <c r="AO42" s="13" t="n"/>
+      <c r="AP42" s="13" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -4995,6 +5098,9 @@
       </c>
       <c r="AO43" s="13" t="n">
         <v>7.67</v>
+      </c>
+      <c r="AP43" s="13" t="n">
+        <v>6.67</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -5073,6 +5179,9 @@
       <c r="AO44" s="13" t="n">
         <v>6343.57</v>
       </c>
+      <c r="AP44" s="13" t="n">
+        <v>6731.69</v>
+      </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
       <c r="A45" s="3" t="n">
@@ -5164,6 +5273,7 @@
       <c r="AM45" s="13" t="n"/>
       <c r="AN45" s="13" t="n"/>
       <c r="AO45" s="13" t="n"/>
+      <c r="AP45" s="13" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -5288,6 +5398,9 @@
       </c>
       <c r="AO46" s="13" t="n">
         <v>14.67</v>
+      </c>
+      <c r="AP46" s="13" t="n">
+        <v>10.81</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -5366,6 +5479,9 @@
       <c r="AO47" s="13" t="n">
         <v>7656.31</v>
       </c>
+      <c r="AP47" s="13" t="n">
+        <v>8118.86</v>
+      </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
       <c r="A48" s="3" t="n">
@@ -5457,6 +5573,7 @@
       <c r="AM48" s="13" t="n"/>
       <c r="AN48" s="13" t="n"/>
       <c r="AO48" s="13" t="n"/>
+      <c r="AP48" s="13" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -5581,6 +5698,9 @@
       </c>
       <c r="AO49" s="13" t="n">
         <v>5.85</v>
+      </c>
+      <c r="AP49" s="13" t="n">
+        <v>2.75</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -5659,6 +5779,9 @@
       <c r="AO50" s="13" t="n">
         <v>11587.45</v>
       </c>
+      <c r="AP50" s="13" t="n">
+        <v>11753.41</v>
+      </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
       <c r="A51" s="3" t="n">
@@ -5750,6 +5873,7 @@
       <c r="AM51" s="13" t="n"/>
       <c r="AN51" s="13" t="n"/>
       <c r="AO51" s="13" t="n"/>
+      <c r="AP51" s="13" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -5874,6 +5998,9 @@
       </c>
       <c r="AO52" s="13" t="n">
         <v>17.73</v>
+      </c>
+      <c r="AP52" s="13" t="n">
+        <v>13.25</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -5952,6 +6079,9 @@
       <c r="AO53" s="13" t="n">
         <v>12546.64</v>
       </c>
+      <c r="AP53" s="13" t="n">
+        <v>11706.81</v>
+      </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
       <c r="A54" s="3" t="n">
@@ -6043,6 +6173,7 @@
       <c r="AM54" s="13" t="n"/>
       <c r="AN54" s="13" t="n"/>
       <c r="AO54" s="13" t="n"/>
+      <c r="AP54" s="13" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -6167,6 +6298,9 @@
       </c>
       <c r="AO55" s="13" t="n">
         <v>15.43</v>
+      </c>
+      <c r="AP55" s="13" t="n">
+        <v>11.82</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -6245,6 +6379,9 @@
       <c r="AO56" s="13" t="n">
         <v>7734.45</v>
       </c>
+      <c r="AP56" s="13" t="n">
+        <v>7923.55</v>
+      </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
       <c r="A57" s="3" t="n">
@@ -6336,6 +6473,7 @@
       <c r="AM57" s="13" t="n"/>
       <c r="AN57" s="13" t="n"/>
       <c r="AO57" s="13" t="n"/>
+      <c r="AP57" s="13" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -6460,6 +6598,9 @@
       </c>
       <c r="AO58" s="13" t="n">
         <v>23.53</v>
+      </c>
+      <c r="AP58" s="13" t="n">
+        <v>16.3</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -6538,6 +6679,9 @@
       <c r="AO59" s="13" t="n">
         <v>14269.55</v>
       </c>
+      <c r="AP59" s="13" t="n">
+        <v>14545.96</v>
+      </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
       <c r="A60" s="3" t="n">
@@ -6629,6 +6773,7 @@
       <c r="AM60" s="13" t="n"/>
       <c r="AN60" s="13" t="n"/>
       <c r="AO60" s="13" t="n"/>
+      <c r="AP60" s="13" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -6753,6 +6898,9 @@
       </c>
       <c r="AO61" s="13" t="n">
         <v>37.27</v>
+      </c>
+      <c r="AP61" s="13" t="n">
+        <v>64.28</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -6831,6 +6979,9 @@
       <c r="AO62" s="13" t="n">
         <v>13810.33</v>
       </c>
+      <c r="AP62" s="13" t="n">
+        <v>15418.65</v>
+      </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
       <c r="A63" s="3" t="n">
@@ -6922,6 +7073,7 @@
       <c r="AM63" s="13" t="n"/>
       <c r="AN63" s="13" t="n"/>
       <c r="AO63" s="13" t="n"/>
+      <c r="AP63" s="13" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -7046,6 +7198,9 @@
       </c>
       <c r="AO64" s="13" t="n">
         <v>16.41</v>
+      </c>
+      <c r="AP64" s="13" t="n">
+        <v>4.38</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -7124,6 +7279,9 @@
       <c r="AO65" s="13" t="n">
         <v>7739.92</v>
       </c>
+      <c r="AP65" s="13" t="n">
+        <v>7693.9</v>
+      </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
       <c r="A66" s="3" t="n">
@@ -7215,6 +7373,7 @@
       <c r="AM66" s="13" t="n"/>
       <c r="AN66" s="13" t="n"/>
       <c r="AO66" s="13" t="n"/>
+      <c r="AP66" s="13" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -7339,6 +7498,9 @@
       </c>
       <c r="AO67" s="13" t="n">
         <v>7.28</v>
+      </c>
+      <c r="AP67" s="13" t="n">
+        <v>5.38</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -7417,6 +7579,9 @@
       <c r="AO68" s="13" t="n">
         <v>9330.690000000001</v>
       </c>
+      <c r="AP68" s="13" t="n">
+        <v>9360.23</v>
+      </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
       <c r="A69" s="3" t="n">
@@ -7508,6 +7673,7 @@
       <c r="AM69" s="13" t="n"/>
       <c r="AN69" s="13" t="n"/>
       <c r="AO69" s="13" t="n"/>
+      <c r="AP69" s="13" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -7632,6 +7798,9 @@
       </c>
       <c r="AO70" s="13" t="n">
         <v>22.77</v>
+      </c>
+      <c r="AP70" s="13" t="n">
+        <v>19.18</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -7710,6 +7879,9 @@
       <c r="AO71" s="13" t="n">
         <v>2491.46</v>
       </c>
+      <c r="AP71" s="13" t="n">
+        <v>2392.95</v>
+      </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
       <c r="A72" s="3" t="n">
@@ -7801,6 +7973,7 @@
       <c r="AM72" s="13" t="n"/>
       <c r="AN72" s="13" t="n"/>
       <c r="AO72" s="13" t="n"/>
+      <c r="AP72" s="13" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -7925,6 +8098,9 @@
       </c>
       <c r="AO73" s="13" t="n">
         <v>39.25</v>
+      </c>
+      <c r="AP73" s="13" t="n">
+        <v>24.59</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -8003,6 +8179,9 @@
       <c r="AO74" s="13" t="n">
         <v>4800.87</v>
       </c>
+      <c r="AP74" s="13" t="n">
+        <v>4629.22</v>
+      </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
       <c r="A75" s="3" t="n">
@@ -8094,6 +8273,7 @@
       <c r="AM75" s="13" t="n"/>
       <c r="AN75" s="13" t="n"/>
       <c r="AO75" s="13" t="n"/>
+      <c r="AP75" s="13" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -8218,6 +8398,9 @@
       </c>
       <c r="AO76" s="13" t="n">
         <v>13.3</v>
+      </c>
+      <c r="AP76" s="13" t="n">
+        <v>14.54</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -8296,6 +8479,9 @@
       <c r="AO77" s="13" t="n">
         <v>8220.4</v>
       </c>
+      <c r="AP77" s="13" t="n">
+        <v>8829</v>
+      </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
       <c r="A78" s="3" t="n">
@@ -8387,6 +8573,7 @@
       <c r="AM78" s="13" t="n"/>
       <c r="AN78" s="13" t="n"/>
       <c r="AO78" s="13" t="n"/>
+      <c r="AP78" s="13" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -8511,6 +8698,9 @@
       </c>
       <c r="AO79" s="13" t="n">
         <v>15.84</v>
+      </c>
+      <c r="AP79" s="13" t="n">
+        <v>8.109999999999999</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -8589,6 +8779,9 @@
       <c r="AO80" s="13" t="n">
         <v>1314.77</v>
       </c>
+      <c r="AP80" s="13" t="n">
+        <v>1259.93</v>
+      </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
       <c r="A81" s="3" t="n">
@@ -8680,6 +8873,7 @@
       <c r="AM81" s="13" t="n"/>
       <c r="AN81" s="13" t="n"/>
       <c r="AO81" s="13" t="n"/>
+      <c r="AP81" s="13" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -8804,6 +8998,9 @@
       </c>
       <c r="AO82" s="13" t="n">
         <v>13.22</v>
+      </c>
+      <c r="AP82" s="13" t="n">
+        <v>9.9</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -8882,6 +9079,9 @@
       <c r="AO83" s="13" t="n">
         <v>15561.64</v>
       </c>
+      <c r="AP83" s="13" t="n">
+        <v>15785.77</v>
+      </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
       <c r="A84" s="3" t="n">
@@ -8973,6 +9173,7 @@
       <c r="AM84" s="13" t="n"/>
       <c r="AN84" s="13" t="n"/>
       <c r="AO84" s="13" t="n"/>
+      <c r="AP84" s="13" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -9097,6 +9298,9 @@
       </c>
       <c r="AO85" s="13" t="n">
         <v>53.89</v>
+      </c>
+      <c r="AP85" s="13" t="n">
+        <v>60.58</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -9175,6 +9379,9 @@
       <c r="AO86" s="13" t="n">
         <v>3063</v>
       </c>
+      <c r="AP86" s="13" t="n">
+        <v>2890.71</v>
+      </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
       <c r="A87" s="3" t="n">
@@ -9266,6 +9473,7 @@
       <c r="AM87" s="13" t="n"/>
       <c r="AN87" s="13" t="n"/>
       <c r="AO87" s="13" t="n"/>
+      <c r="AP87" s="13" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -9390,6 +9598,9 @@
       </c>
       <c r="AO88" s="13" t="n">
         <v>58.37</v>
+      </c>
+      <c r="AP88" s="13" t="n">
+        <v>72.98</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -9468,6 +9679,9 @@
       <c r="AO89" s="13" t="n">
         <v>3327.93</v>
       </c>
+      <c r="AP89" s="13" t="n">
+        <v>3179.23</v>
+      </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
       <c r="A90" s="3" t="n">
@@ -9559,6 +9773,7 @@
       <c r="AM90" s="13" t="n"/>
       <c r="AN90" s="13" t="n"/>
       <c r="AO90" s="13" t="n"/>
+      <c r="AP90" s="13" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -9683,6 +9898,9 @@
       </c>
       <c r="AO91" s="13" t="n">
         <v>48.48</v>
+      </c>
+      <c r="AP91" s="13" t="n">
+        <v>52.94</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -9761,6 +9979,9 @@
       <c r="AO92" s="13" t="n">
         <v>2949.03</v>
       </c>
+      <c r="AP92" s="13" t="n">
+        <v>2973.51</v>
+      </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
       <c r="A93" s="3" t="n">
@@ -9852,6 +10073,7 @@
       <c r="AM93" s="13" t="n"/>
       <c r="AN93" s="13" t="n"/>
       <c r="AO93" s="13" t="n"/>
+      <c r="AP93" s="13" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -9976,6 +10198,9 @@
       </c>
       <c r="AO94" s="13" t="n">
         <v>23.82</v>
+      </c>
+      <c r="AP94" s="13" t="n">
+        <v>39.52</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -10054,6 +10279,9 @@
       <c r="AO95" s="13" t="n">
         <v>1760.24</v>
       </c>
+      <c r="AP95" s="13" t="n">
+        <v>1965.5</v>
+      </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
       <c r="A96" s="3" t="n">
@@ -10145,6 +10373,7 @@
       <c r="AM96" s="13" t="n"/>
       <c r="AN96" s="13" t="n"/>
       <c r="AO96" s="13" t="n"/>
+      <c r="AP96" s="13" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -10269,6 +10498,9 @@
       </c>
       <c r="AO97" s="13" t="n">
         <v>24.26</v>
+      </c>
+      <c r="AP97" s="13" t="n">
+        <v>24.48</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -10347,6 +10579,9 @@
       <c r="AO98" s="13" t="n">
         <v>9414.73</v>
       </c>
+      <c r="AP98" s="13" t="n">
+        <v>9357.370000000001</v>
+      </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
       <c r="A99" s="3" t="n">
@@ -10438,6 +10673,7 @@
       <c r="AM99" s="13" t="n"/>
       <c r="AN99" s="13" t="n"/>
       <c r="AO99" s="13" t="n"/>
+      <c r="AP99" s="13" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -10562,6 +10798,9 @@
       </c>
       <c r="AO100" s="13" t="n">
         <v>82.66</v>
+      </c>
+      <c r="AP100" s="13" t="n">
+        <v>80.22</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -10640,6 +10879,9 @@
       <c r="AO101" s="13" t="n">
         <v>9137.360000000001</v>
       </c>
+      <c r="AP101" s="13" t="n">
+        <v>9163.370000000001</v>
+      </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
       <c r="A102" s="3" t="n">
@@ -10731,6 +10973,7 @@
       <c r="AM102" s="13" t="n"/>
       <c r="AN102" s="13" t="n"/>
       <c r="AO102" s="13" t="n"/>
+      <c r="AP102" s="13" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -10855,6 +11098,9 @@
       </c>
       <c r="AO103" s="13" t="n">
         <v>57.06</v>
+      </c>
+      <c r="AP103" s="13" t="n">
+        <v>71.38</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -10933,6 +11179,9 @@
       <c r="AO104" s="13" t="n">
         <v>13101.33</v>
       </c>
+      <c r="AP104" s="13" t="n">
+        <v>13164.66</v>
+      </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
       <c r="A105" s="3" t="n">
@@ -11024,6 +11273,7 @@
       <c r="AM105" s="13" t="n"/>
       <c r="AN105" s="13" t="n"/>
       <c r="AO105" s="13" t="n"/>
+      <c r="AP105" s="13" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -11148,6 +11398,9 @@
       </c>
       <c r="AO106" s="13" t="n">
         <v>7.63</v>
+      </c>
+      <c r="AP106" s="13" t="n">
+        <v>11.33</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -11226,6 +11479,9 @@
       <c r="AO107" s="13" t="n">
         <v>2275.37</v>
       </c>
+      <c r="AP107" s="13" t="n">
+        <v>2136.48</v>
+      </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
       <c r="A108" s="3" t="n">
@@ -11317,6 +11573,7 @@
       <c r="AM108" s="13" t="n"/>
       <c r="AN108" s="13" t="n"/>
       <c r="AO108" s="13" t="n"/>
+      <c r="AP108" s="13" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -11441,6 +11698,9 @@
       </c>
       <c r="AO109" s="13" t="n">
         <v>23.54</v>
+      </c>
+      <c r="AP109" s="13" t="n">
+        <v>8.66</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -11519,6 +11779,9 @@
       <c r="AO110" s="13" t="n">
         <v>728.17</v>
       </c>
+      <c r="AP110" s="13" t="n">
+        <v>721.49</v>
+      </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
       <c r="A111" s="3" t="n">
@@ -11610,6 +11873,7 @@
       <c r="AM111" s="13" t="n"/>
       <c r="AN111" s="13" t="n"/>
       <c r="AO111" s="13" t="n"/>
+      <c r="AP111" s="13" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -11734,6 +11998,9 @@
       </c>
       <c r="AO112" s="13" t="n">
         <v>30.5</v>
+      </c>
+      <c r="AP112" s="13" t="n">
+        <v>77.28</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -11812,6 +12079,9 @@
       <c r="AO113" s="13" t="n">
         <v>3082.03</v>
       </c>
+      <c r="AP113" s="13" t="n">
+        <v>3260.62</v>
+      </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
       <c r="A114" s="3" t="n">
@@ -11903,6 +12173,7 @@
       <c r="AM114" s="13" t="n"/>
       <c r="AN114" s="13" t="n"/>
       <c r="AO114" s="13" t="n"/>
+      <c r="AP114" s="13" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -12027,6 +12298,9 @@
       </c>
       <c r="AO115" s="13" t="n">
         <v>22.31</v>
+      </c>
+      <c r="AP115" s="13" t="n">
+        <v>26.48</v>
       </c>
     </row>
     <row r="116">
@@ -12089,6 +12363,9 @@
       </c>
       <c r="AO116" s="13" t="n">
         <v>4045.82</v>
+      </c>
+      <c r="AP116" s="13" t="n">
+        <v>3975.24</v>
       </c>
     </row>
     <row r="117">
@@ -12136,6 +12413,7 @@
       <c r="AM117" s="13" t="n"/>
       <c r="AN117" s="13" t="n"/>
       <c r="AO117" s="13" t="n"/>
+      <c r="AP117" s="13" t="n"/>
     </row>
     <row r="118">
       <c r="P118" s="13" t="n">
@@ -12216,6 +12494,9 @@
       <c r="AO118" s="13" t="n">
         <v>29.02</v>
       </c>
+      <c r="AP118" s="13" t="n">
+        <v>29.02</v>
+      </c>
     </row>
     <row r="119">
       <c r="Y119" s="13" t="n">
@@ -12268,6 +12549,9 @@
       </c>
       <c r="AO119" s="13" t="n">
         <v>2727.34</v>
+      </c>
+      <c r="AP119" s="13" t="n">
+        <v>2648.44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-04-09 05:30:28]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP119"/>
+  <dimension ref="A1:AQ119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="15"/>
@@ -559,6 +559,7 @@
     <col width="15" customWidth="1" min="40" max="40"/>
     <col width="15" customWidth="1" min="41" max="41"/>
     <col width="15" customWidth="1" min="42" max="42"/>
+    <col width="15" customWidth="1" min="43" max="43"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -772,6 +773,11 @@
           <t>2026/04/02</t>
         </is>
       </c>
+      <c r="AQ1" s="13" t="inlineStr">
+        <is>
+          <t>2026/04/09</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -984,6 +990,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="AQ2" s="14" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1112,6 +1123,9 @@
       <c r="AP3" s="13" t="n">
         <v>63.22</v>
       </c>
+      <c r="AQ3" s="13" t="n">
+        <v>66.48</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1239,6 +1253,9 @@
       </c>
       <c r="AP4" s="13" t="n">
         <v>3914.46</v>
+      </c>
+      <c r="AQ4" s="13" t="n">
+        <v>3961.76</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1284,6 +1301,7 @@
       <c r="AN5" s="13" t="n"/>
       <c r="AO5" s="13" t="n"/>
       <c r="AP5" s="13" t="n"/>
+      <c r="AQ5" s="13" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1376,6 +1394,7 @@
       <c r="AN6" s="13" t="n"/>
       <c r="AO6" s="13" t="n"/>
       <c r="AP6" s="13" t="n"/>
+      <c r="AQ6" s="13" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1503,6 +1522,9 @@
       </c>
       <c r="AP7" s="13" t="n">
         <v>59.52</v>
+      </c>
+      <c r="AQ7" s="13" t="n">
+        <v>63.48</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -1584,6 +1606,9 @@
       <c r="AP8" s="13" t="n">
         <v>5544.27</v>
       </c>
+      <c r="AQ8" s="13" t="n">
+        <v>5694.55</v>
+      </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -1676,6 +1701,7 @@
       <c r="AN9" s="13" t="n"/>
       <c r="AO9" s="13" t="n"/>
       <c r="AP9" s="13" t="n"/>
+      <c r="AQ9" s="13" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -1803,6 +1829,9 @@
       </c>
       <c r="AP10" s="13" t="n">
         <v>49.63</v>
+      </c>
+      <c r="AQ10" s="13" t="n">
+        <v>52.86</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -1884,6 +1913,9 @@
       <c r="AP11" s="13" t="n">
         <v>4473.71</v>
       </c>
+      <c r="AQ11" s="13" t="n">
+        <v>4564.1</v>
+      </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -1976,6 +2008,7 @@
       <c r="AN12" s="13" t="n"/>
       <c r="AO12" s="13" t="n"/>
       <c r="AP12" s="13" t="n"/>
+      <c r="AQ12" s="13" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2103,6 +2136,9 @@
       </c>
       <c r="AP13" s="13" t="n">
         <v>62.42</v>
+      </c>
+      <c r="AQ13" s="13" t="n">
+        <v>65.58</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -2184,6 +2220,9 @@
       <c r="AP14" s="13" t="n">
         <v>7607.01</v>
       </c>
+      <c r="AQ14" s="13" t="n">
+        <v>7889.48</v>
+      </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -2276,6 +2315,7 @@
       <c r="AN15" s="13" t="n"/>
       <c r="AO15" s="13" t="n"/>
       <c r="AP15" s="13" t="n"/>
+      <c r="AQ15" s="13" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -2403,6 +2443,9 @@
       </c>
       <c r="AP16" s="13" t="n">
         <v>31.71</v>
+      </c>
+      <c r="AQ16" s="13" t="n">
+        <v>34.95</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -2484,6 +2527,9 @@
       <c r="AP17" s="13" t="n">
         <v>2652.96</v>
       </c>
+      <c r="AQ17" s="13" t="n">
+        <v>2603.88</v>
+      </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="3" t="n">
@@ -2576,6 +2622,7 @@
       <c r="AN18" s="13" t="n"/>
       <c r="AO18" s="13" t="n"/>
       <c r="AP18" s="13" t="n"/>
+      <c r="AQ18" s="13" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -2703,6 +2750,9 @@
       </c>
       <c r="AP19" s="13" t="n">
         <v>88.5</v>
+      </c>
+      <c r="AQ19" s="13" t="n">
+        <v>93.62</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -2784,6 +2834,9 @@
       <c r="AP20" s="13" t="n">
         <v>6575.32</v>
       </c>
+      <c r="AQ20" s="13" t="n">
+        <v>6782.81</v>
+      </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -2876,6 +2929,7 @@
       <c r="AN21" s="13" t="n"/>
       <c r="AO21" s="13" t="n"/>
       <c r="AP21" s="13" t="n"/>
+      <c r="AQ21" s="13" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -3001,6 +3055,9 @@
       </c>
       <c r="AP22" s="13" t="n">
         <v>34.86</v>
+      </c>
+      <c r="AQ22" s="13" t="n">
+        <v>45.14</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1">
@@ -3082,6 +3139,9 @@
       <c r="AP23" s="13" t="n">
         <v>71645.14</v>
       </c>
+      <c r="AQ23" s="13" t="n">
+        <v>76868</v>
+      </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="3" t="n">
@@ -3174,6 +3234,7 @@
       <c r="AN24" s="13" t="n"/>
       <c r="AO24" s="13" t="n"/>
       <c r="AP24" s="13" t="n"/>
+      <c r="AQ24" s="13" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -3301,6 +3362,9 @@
       </c>
       <c r="AP25" s="13" t="n">
         <v>35.16</v>
+      </c>
+      <c r="AQ25" s="13" t="n">
+        <v>39.88</v>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="1">
@@ -3382,6 +3446,9 @@
       <c r="AP26" s="13" t="n">
         <v>23298.89</v>
       </c>
+      <c r="AQ26" s="13" t="n">
+        <v>24080.63</v>
+      </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -3474,6 +3541,7 @@
       <c r="AN27" s="13" t="n"/>
       <c r="AO27" s="13" t="n"/>
       <c r="AP27" s="13" t="n"/>
+      <c r="AQ27" s="13" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -3601,6 +3669,9 @@
       </c>
       <c r="AP28" s="13" t="n">
         <v>77.45</v>
+      </c>
+      <c r="AQ28" s="13" t="n">
+        <v>77.64</v>
       </c>
     </row>
     <row r="29" ht="14.25" customHeight="1">
@@ -3682,6 +3753,9 @@
       <c r="AP29" s="13" t="n">
         <v>52421.04</v>
       </c>
+      <c r="AQ29" s="13" t="n">
+        <v>55960.86</v>
+      </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="3" t="n">
@@ -3774,6 +3848,7 @@
       <c r="AN30" s="13" t="n"/>
       <c r="AO30" s="13" t="n"/>
       <c r="AP30" s="13" t="n"/>
+      <c r="AQ30" s="13" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -3901,6 +3976,9 @@
       </c>
       <c r="AP31" s="13" t="n">
         <v>53.79</v>
+      </c>
+      <c r="AQ31" s="13" t="n">
+        <v>52.98</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -3982,6 +4060,9 @@
       <c r="AP32" s="13" t="n">
         <v>5735.1</v>
       </c>
+      <c r="AQ32" s="13" t="n">
+        <v>5681.52</v>
+      </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
       <c r="A33" s="3" t="n">
@@ -4074,6 +4155,7 @@
       <c r="AN33" s="13" t="n"/>
       <c r="AO33" s="13" t="n"/>
       <c r="AP33" s="13" t="n"/>
+      <c r="AQ33" s="13" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -4201,6 +4283,9 @@
       </c>
       <c r="AP34" s="13" t="n">
         <v>1.4</v>
+      </c>
+      <c r="AQ34" s="13" t="n">
+        <v>1.57</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -4282,6 +4367,9 @@
       <c r="AP35" s="13" t="n">
         <v>32685.33</v>
       </c>
+      <c r="AQ35" s="13" t="n">
+        <v>33457.58</v>
+      </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="3" t="n">
@@ -4374,6 +4462,7 @@
       <c r="AN36" s="13" t="n"/>
       <c r="AO36" s="13" t="n"/>
       <c r="AP36" s="13" t="n"/>
+      <c r="AQ36" s="13" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -4501,6 +4590,9 @@
       </c>
       <c r="AP37" s="13" t="n">
         <v>42.45</v>
+      </c>
+      <c r="AQ37" s="13" t="n">
+        <v>48.05</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -4582,6 +4674,9 @@
       <c r="AP38" s="13" t="n">
         <v>3333.11</v>
       </c>
+      <c r="AQ38" s="13" t="n">
+        <v>3508.72</v>
+      </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
       <c r="A39" s="3" t="n">
@@ -4674,6 +4769,7 @@
       <c r="AN39" s="13" t="n"/>
       <c r="AO39" s="13" t="n"/>
       <c r="AP39" s="13" t="n"/>
+      <c r="AQ39" s="13" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -4801,6 +4897,9 @@
       </c>
       <c r="AP40" s="13" t="n">
         <v>44.02</v>
+      </c>
+      <c r="AQ40" s="13" t="n">
+        <v>49.39</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -4882,6 +4981,9 @@
       <c r="AP41" s="13" t="n">
         <v>3169.1</v>
       </c>
+      <c r="AQ41" s="13" t="n">
+        <v>3323.04</v>
+      </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
       <c r="A42" s="3" t="n">
@@ -4974,6 +5076,7 @@
       <c r="AN42" s="13" t="n"/>
       <c r="AO42" s="13" t="n"/>
       <c r="AP42" s="13" t="n"/>
+      <c r="AQ42" s="13" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -5101,6 +5204,9 @@
       </c>
       <c r="AP43" s="13" t="n">
         <v>6.67</v>
+      </c>
+      <c r="AQ43" s="13" t="n">
+        <v>9.82</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -5182,6 +5288,9 @@
       <c r="AP44" s="13" t="n">
         <v>6731.69</v>
       </c>
+      <c r="AQ44" s="13" t="n">
+        <v>6679.05</v>
+      </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
       <c r="A45" s="3" t="n">
@@ -5274,6 +5383,7 @@
       <c r="AN45" s="13" t="n"/>
       <c r="AO45" s="13" t="n"/>
       <c r="AP45" s="13" t="n"/>
+      <c r="AQ45" s="13" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -5401,6 +5511,9 @@
       </c>
       <c r="AP46" s="13" t="n">
         <v>10.81</v>
+      </c>
+      <c r="AQ46" s="13" t="n">
+        <v>13.88</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -5482,6 +5595,9 @@
       <c r="AP47" s="13" t="n">
         <v>8118.86</v>
       </c>
+      <c r="AQ47" s="13" t="n">
+        <v>8093.93</v>
+      </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
       <c r="A48" s="3" t="n">
@@ -5574,6 +5690,7 @@
       <c r="AN48" s="13" t="n"/>
       <c r="AO48" s="13" t="n"/>
       <c r="AP48" s="13" t="n"/>
+      <c r="AQ48" s="13" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -5701,6 +5818,9 @@
       </c>
       <c r="AP49" s="13" t="n">
         <v>2.75</v>
+      </c>
+      <c r="AQ49" s="13" t="n">
+        <v>3.81</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -5782,6 +5902,9 @@
       <c r="AP50" s="13" t="n">
         <v>11753.41</v>
       </c>
+      <c r="AQ50" s="13" t="n">
+        <v>11690.71</v>
+      </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
       <c r="A51" s="3" t="n">
@@ -5874,6 +5997,7 @@
       <c r="AN51" s="13" t="n"/>
       <c r="AO51" s="13" t="n"/>
       <c r="AP51" s="13" t="n"/>
+      <c r="AQ51" s="13" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -6001,6 +6125,9 @@
       </c>
       <c r="AP52" s="13" t="n">
         <v>13.25</v>
+      </c>
+      <c r="AQ52" s="13" t="n">
+        <v>17.15</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -6082,6 +6209,9 @@
       <c r="AP53" s="13" t="n">
         <v>11706.81</v>
       </c>
+      <c r="AQ53" s="13" t="n">
+        <v>11720.09</v>
+      </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
       <c r="A54" s="3" t="n">
@@ -6174,6 +6304,7 @@
       <c r="AN54" s="13" t="n"/>
       <c r="AO54" s="13" t="n"/>
       <c r="AP54" s="13" t="n"/>
+      <c r="AQ54" s="13" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -6301,6 +6432,9 @@
       </c>
       <c r="AP55" s="13" t="n">
         <v>11.82</v>
+      </c>
+      <c r="AQ55" s="13" t="n">
+        <v>13.06</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -6382,6 +6516,9 @@
       <c r="AP56" s="13" t="n">
         <v>7923.55</v>
       </c>
+      <c r="AQ56" s="13" t="n">
+        <v>7730.15</v>
+      </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
       <c r="A57" s="3" t="n">
@@ -6474,6 +6611,7 @@
       <c r="AN57" s="13" t="n"/>
       <c r="AO57" s="13" t="n"/>
       <c r="AP57" s="13" t="n"/>
+      <c r="AQ57" s="13" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -6601,6 +6739,9 @@
       </c>
       <c r="AP58" s="13" t="n">
         <v>16.3</v>
+      </c>
+      <c r="AQ58" s="13" t="n">
+        <v>17.76</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -6682,6 +6823,9 @@
       <c r="AP59" s="13" t="n">
         <v>14545.96</v>
       </c>
+      <c r="AQ59" s="13" t="n">
+        <v>14355.15</v>
+      </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
       <c r="A60" s="3" t="n">
@@ -6774,6 +6918,7 @@
       <c r="AN60" s="13" t="n"/>
       <c r="AO60" s="13" t="n"/>
       <c r="AP60" s="13" t="n"/>
+      <c r="AQ60" s="13" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -6901,6 +7046,9 @@
       </c>
       <c r="AP61" s="13" t="n">
         <v>64.28</v>
+      </c>
+      <c r="AQ61" s="13" t="n">
+        <v>67.66</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -6982,6 +7130,9 @@
       <c r="AP62" s="13" t="n">
         <v>15418.65</v>
       </c>
+      <c r="AQ62" s="13" t="n">
+        <v>15372.38</v>
+      </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
       <c r="A63" s="3" t="n">
@@ -7074,6 +7225,7 @@
       <c r="AN63" s="13" t="n"/>
       <c r="AO63" s="13" t="n"/>
       <c r="AP63" s="13" t="n"/>
+      <c r="AQ63" s="13" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -7201,6 +7353,9 @@
       </c>
       <c r="AP64" s="13" t="n">
         <v>4.38</v>
+      </c>
+      <c r="AQ64" s="13" t="n">
+        <v>7.79</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -7282,6 +7437,9 @@
       <c r="AP65" s="13" t="n">
         <v>7693.9</v>
       </c>
+      <c r="AQ65" s="13" t="n">
+        <v>7497.88</v>
+      </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
       <c r="A66" s="3" t="n">
@@ -7374,6 +7532,7 @@
       <c r="AN66" s="13" t="n"/>
       <c r="AO66" s="13" t="n"/>
       <c r="AP66" s="13" t="n"/>
+      <c r="AQ66" s="13" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -7501,6 +7660,9 @@
       </c>
       <c r="AP67" s="13" t="n">
         <v>5.38</v>
+      </c>
+      <c r="AQ67" s="13" t="n">
+        <v>6.73</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -7582,6 +7744,9 @@
       <c r="AP68" s="13" t="n">
         <v>9360.23</v>
       </c>
+      <c r="AQ68" s="13" t="n">
+        <v>9168.190000000001</v>
+      </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
       <c r="A69" s="3" t="n">
@@ -7674,6 +7839,7 @@
       <c r="AN69" s="13" t="n"/>
       <c r="AO69" s="13" t="n"/>
       <c r="AP69" s="13" t="n"/>
+      <c r="AQ69" s="13" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -7801,6 +7967,9 @@
       </c>
       <c r="AP70" s="13" t="n">
         <v>19.18</v>
+      </c>
+      <c r="AQ70" s="13" t="n">
+        <v>23.03</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -7882,6 +8051,9 @@
       <c r="AP71" s="13" t="n">
         <v>2392.95</v>
       </c>
+      <c r="AQ71" s="13" t="n">
+        <v>2509.36</v>
+      </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
       <c r="A72" s="3" t="n">
@@ -7974,6 +8146,7 @@
       <c r="AN72" s="13" t="n"/>
       <c r="AO72" s="13" t="n"/>
       <c r="AP72" s="13" t="n"/>
+      <c r="AQ72" s="13" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -8101,6 +8274,9 @@
       </c>
       <c r="AP73" s="13" t="n">
         <v>24.59</v>
+      </c>
+      <c r="AQ73" s="13" t="n">
+        <v>33.47</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -8182,6 +8358,9 @@
       <c r="AP74" s="13" t="n">
         <v>4629.22</v>
       </c>
+      <c r="AQ74" s="13" t="n">
+        <v>4853.32</v>
+      </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
       <c r="A75" s="3" t="n">
@@ -8274,6 +8453,7 @@
       <c r="AN75" s="13" t="n"/>
       <c r="AO75" s="13" t="n"/>
       <c r="AP75" s="13" t="n"/>
+      <c r="AQ75" s="13" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -8401,6 +8581,9 @@
       </c>
       <c r="AP76" s="13" t="n">
         <v>14.54</v>
+      </c>
+      <c r="AQ76" s="13" t="n">
+        <v>19.37</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -8482,6 +8665,9 @@
       <c r="AP77" s="13" t="n">
         <v>8829</v>
       </c>
+      <c r="AQ77" s="13" t="n">
+        <v>8720.290000000001</v>
+      </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
       <c r="A78" s="3" t="n">
@@ -8574,6 +8760,7 @@
       <c r="AN78" s="13" t="n"/>
       <c r="AO78" s="13" t="n"/>
       <c r="AP78" s="13" t="n"/>
+      <c r="AQ78" s="13" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -8701,6 +8888,9 @@
       </c>
       <c r="AP79" s="13" t="n">
         <v>8.109999999999999</v>
+      </c>
+      <c r="AQ79" s="13" t="n">
+        <v>11.46</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -8782,6 +8972,9 @@
       <c r="AP80" s="13" t="n">
         <v>1259.93</v>
       </c>
+      <c r="AQ80" s="13" t="n">
+        <v>1254.89</v>
+      </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
       <c r="A81" s="3" t="n">
@@ -8874,6 +9067,7 @@
       <c r="AN81" s="13" t="n"/>
       <c r="AO81" s="13" t="n"/>
       <c r="AP81" s="13" t="n"/>
+      <c r="AQ81" s="13" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -9001,6 +9195,9 @@
       </c>
       <c r="AP82" s="13" t="n">
         <v>9.9</v>
+      </c>
+      <c r="AQ82" s="13" t="n">
+        <v>10.93</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -9082,6 +9279,9 @@
       <c r="AP83" s="13" t="n">
         <v>15785.77</v>
       </c>
+      <c r="AQ83" s="13" t="n">
+        <v>15715.7</v>
+      </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
       <c r="A84" s="3" t="n">
@@ -9174,6 +9374,7 @@
       <c r="AN84" s="13" t="n"/>
       <c r="AO84" s="13" t="n"/>
       <c r="AP84" s="13" t="n"/>
+      <c r="AQ84" s="13" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -9301,6 +9502,9 @@
       </c>
       <c r="AP85" s="13" t="n">
         <v>60.58</v>
+      </c>
+      <c r="AQ85" s="13" t="n">
+        <v>60.25</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -9382,6 +9586,9 @@
       <c r="AP86" s="13" t="n">
         <v>2890.71</v>
       </c>
+      <c r="AQ86" s="13" t="n">
+        <v>2906.96</v>
+      </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
       <c r="A87" s="3" t="n">
@@ -9474,6 +9681,7 @@
       <c r="AN87" s="13" t="n"/>
       <c r="AO87" s="13" t="n"/>
       <c r="AP87" s="13" t="n"/>
+      <c r="AQ87" s="13" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -9601,6 +9809,9 @@
       </c>
       <c r="AP88" s="13" t="n">
         <v>72.98</v>
+      </c>
+      <c r="AQ88" s="13" t="n">
+        <v>72.81</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -9682,6 +9893,9 @@
       <c r="AP89" s="13" t="n">
         <v>3179.23</v>
       </c>
+      <c r="AQ89" s="13" t="n">
+        <v>3064.47</v>
+      </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
       <c r="A90" s="3" t="n">
@@ -9774,6 +9988,7 @@
       <c r="AN90" s="13" t="n"/>
       <c r="AO90" s="13" t="n"/>
       <c r="AP90" s="13" t="n"/>
+      <c r="AQ90" s="13" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -9901,6 +10116,9 @@
       </c>
       <c r="AP91" s="13" t="n">
         <v>52.94</v>
+      </c>
+      <c r="AQ91" s="13" t="n">
+        <v>52.12</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -9982,6 +10200,9 @@
       <c r="AP92" s="13" t="n">
         <v>2973.51</v>
       </c>
+      <c r="AQ92" s="13" t="n">
+        <v>3015.84</v>
+      </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
       <c r="A93" s="3" t="n">
@@ -10074,6 +10295,7 @@
       <c r="AN93" s="13" t="n"/>
       <c r="AO93" s="13" t="n"/>
       <c r="AP93" s="13" t="n"/>
+      <c r="AQ93" s="13" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -10201,6 +10423,9 @@
       </c>
       <c r="AP94" s="13" t="n">
         <v>39.52</v>
+      </c>
+      <c r="AQ94" s="13" t="n">
+        <v>47.69</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -10282,6 +10507,9 @@
       <c r="AP95" s="13" t="n">
         <v>1965.5</v>
       </c>
+      <c r="AQ95" s="13" t="n">
+        <v>1828.38</v>
+      </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
       <c r="A96" s="3" t="n">
@@ -10374,6 +10602,7 @@
       <c r="AN96" s="13" t="n"/>
       <c r="AO96" s="13" t="n"/>
       <c r="AP96" s="13" t="n"/>
+      <c r="AQ96" s="13" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -10501,6 +10730,9 @@
       </c>
       <c r="AP97" s="13" t="n">
         <v>24.48</v>
+      </c>
+      <c r="AQ97" s="13" t="n">
+        <v>26.23</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -10582,6 +10814,9 @@
       <c r="AP98" s="13" t="n">
         <v>9357.370000000001</v>
       </c>
+      <c r="AQ98" s="13" t="n">
+        <v>9711.76</v>
+      </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
       <c r="A99" s="3" t="n">
@@ -10674,6 +10909,7 @@
       <c r="AN99" s="13" t="n"/>
       <c r="AO99" s="13" t="n"/>
       <c r="AP99" s="13" t="n"/>
+      <c r="AQ99" s="13" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -10801,6 +11037,9 @@
       </c>
       <c r="AP100" s="13" t="n">
         <v>80.22</v>
+      </c>
+      <c r="AQ100" s="13" t="n">
+        <v>85.66</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -10882,6 +11121,9 @@
       <c r="AP101" s="13" t="n">
         <v>9163.370000000001</v>
       </c>
+      <c r="AQ101" s="13" t="n">
+        <v>9633.639999999999</v>
+      </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
       <c r="A102" s="3" t="n">
@@ -10974,6 +11216,7 @@
       <c r="AN102" s="13" t="n"/>
       <c r="AO102" s="13" t="n"/>
       <c r="AP102" s="13" t="n"/>
+      <c r="AQ102" s="13" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -11101,6 +11344,9 @@
       </c>
       <c r="AP103" s="13" t="n">
         <v>71.38</v>
+      </c>
+      <c r="AQ103" s="13" t="n">
+        <v>72.7</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -11182,6 +11428,9 @@
       <c r="AP104" s="13" t="n">
         <v>13164.66</v>
       </c>
+      <c r="AQ104" s="13" t="n">
+        <v>13517.75</v>
+      </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
       <c r="A105" s="3" t="n">
@@ -11274,6 +11523,7 @@
       <c r="AN105" s="13" t="n"/>
       <c r="AO105" s="13" t="n"/>
       <c r="AP105" s="13" t="n"/>
+      <c r="AQ105" s="13" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -11401,6 +11651,9 @@
       </c>
       <c r="AP106" s="13" t="n">
         <v>11.33</v>
+      </c>
+      <c r="AQ106" s="13" t="n">
+        <v>13.83</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -11482,6 +11735,9 @@
       <c r="AP107" s="13" t="n">
         <v>2136.48</v>
       </c>
+      <c r="AQ107" s="13" t="n">
+        <v>2134.75</v>
+      </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
       <c r="A108" s="3" t="n">
@@ -11574,6 +11830,7 @@
       <c r="AN108" s="13" t="n"/>
       <c r="AO108" s="13" t="n"/>
       <c r="AP108" s="13" t="n"/>
+      <c r="AQ108" s="13" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -11701,6 +11958,9 @@
       </c>
       <c r="AP109" s="13" t="n">
         <v>8.66</v>
+      </c>
+      <c r="AQ109" s="13" t="n">
+        <v>11.62</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -11782,6 +12042,9 @@
       <c r="AP110" s="13" t="n">
         <v>721.49</v>
       </c>
+      <c r="AQ110" s="13" t="n">
+        <v>725.62</v>
+      </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
       <c r="A111" s="3" t="n">
@@ -11874,6 +12137,7 @@
       <c r="AN111" s="13" t="n"/>
       <c r="AO111" s="13" t="n"/>
       <c r="AP111" s="13" t="n"/>
+      <c r="AQ111" s="13" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -12001,6 +12265,9 @@
       </c>
       <c r="AP112" s="13" t="n">
         <v>77.28</v>
+      </c>
+      <c r="AQ112" s="13" t="n">
+        <v>80.81999999999999</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -12082,6 +12349,9 @@
       <c r="AP113" s="13" t="n">
         <v>3260.62</v>
       </c>
+      <c r="AQ113" s="13" t="n">
+        <v>3387.4</v>
+      </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
       <c r="A114" s="3" t="n">
@@ -12174,6 +12444,7 @@
       <c r="AN114" s="13" t="n"/>
       <c r="AO114" s="13" t="n"/>
       <c r="AP114" s="13" t="n"/>
+      <c r="AQ114" s="13" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -12301,6 +12572,9 @@
       </c>
       <c r="AP115" s="13" t="n">
         <v>26.48</v>
+      </c>
+      <c r="AQ115" s="13" t="n">
+        <v>32.43</v>
       </c>
     </row>
     <row r="116">
@@ -12366,6 +12640,9 @@
       </c>
       <c r="AP116" s="13" t="n">
         <v>3975.24</v>
+      </c>
+      <c r="AQ116" s="13" t="n">
+        <v>4025.45</v>
       </c>
     </row>
     <row r="117">
@@ -12414,6 +12691,7 @@
       <c r="AN117" s="13" t="n"/>
       <c r="AO117" s="13" t="n"/>
       <c r="AP117" s="13" t="n"/>
+      <c r="AQ117" s="13" t="n"/>
     </row>
     <row r="118">
       <c r="P118" s="13" t="n">
@@ -12497,6 +12775,9 @@
       <c r="AP118" s="13" t="n">
         <v>29.02</v>
       </c>
+      <c r="AQ118" s="13" t="n">
+        <v>29.02</v>
+      </c>
     </row>
     <row r="119">
       <c r="Y119" s="13" t="n">
@@ -12552,6 +12833,9 @@
       </c>
       <c r="AP119" s="13" t="n">
         <v>2648.44</v>
+      </c>
+      <c r="AQ119" s="13" t="n">
+        <v>2662.11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-04-20 06:03:23]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ119"/>
+  <dimension ref="A1:AR119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="15"/>
@@ -560,6 +560,7 @@
     <col width="15" customWidth="1" min="41" max="41"/>
     <col width="15" customWidth="1" min="42" max="42"/>
     <col width="15" customWidth="1" min="43" max="43"/>
+    <col width="15" customWidth="1" min="44" max="44"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -778,6 +779,11 @@
           <t>2026/04/09</t>
         </is>
       </c>
+      <c r="AR1" s="13" t="inlineStr">
+        <is>
+          <t>2026/04/20</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -995,6 +1001,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="AR2" s="14" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1126,6 +1137,9 @@
       <c r="AQ3" s="13" t="n">
         <v>66.48</v>
       </c>
+      <c r="AR3" s="13" t="n">
+        <v>69.16</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1256,6 +1270,9 @@
       </c>
       <c r="AQ4" s="13" t="n">
         <v>3961.76</v>
+      </c>
+      <c r="AR4" s="13" t="n">
+        <v>4072.26</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1302,6 +1319,7 @@
       <c r="AO5" s="13" t="n"/>
       <c r="AP5" s="13" t="n"/>
       <c r="AQ5" s="13" t="n"/>
+      <c r="AR5" s="13" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1395,6 +1413,7 @@
       <c r="AO6" s="13" t="n"/>
       <c r="AP6" s="13" t="n"/>
       <c r="AQ6" s="13" t="n"/>
+      <c r="AR6" s="13" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1525,6 +1544,9 @@
       </c>
       <c r="AQ7" s="13" t="n">
         <v>63.48</v>
+      </c>
+      <c r="AR7" s="13" t="n">
+        <v>66.72</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -1609,6 +1631,9 @@
       <c r="AQ8" s="13" t="n">
         <v>5694.55</v>
       </c>
+      <c r="AR8" s="13" t="n">
+        <v>5941.99</v>
+      </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -1702,6 +1727,7 @@
       <c r="AO9" s="13" t="n"/>
       <c r="AP9" s="13" t="n"/>
       <c r="AQ9" s="13" t="n"/>
+      <c r="AR9" s="13" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -1832,6 +1858,9 @@
       </c>
       <c r="AQ10" s="13" t="n">
         <v>52.86</v>
+      </c>
+      <c r="AR10" s="13" t="n">
+        <v>56.55</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -1916,6 +1945,9 @@
       <c r="AQ11" s="13" t="n">
         <v>4564.1</v>
       </c>
+      <c r="AR11" s="13" t="n">
+        <v>4747.66</v>
+      </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -2009,6 +2041,7 @@
       <c r="AO12" s="13" t="n"/>
       <c r="AP12" s="13" t="n"/>
       <c r="AQ12" s="13" t="n"/>
+      <c r="AR12" s="13" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2139,6 +2172,9 @@
       </c>
       <c r="AQ13" s="13" t="n">
         <v>65.58</v>
+      </c>
+      <c r="AR13" s="13" t="n">
+        <v>66.94</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -2223,6 +2259,9 @@
       <c r="AQ14" s="13" t="n">
         <v>7889.48</v>
       </c>
+      <c r="AR14" s="13" t="n">
+        <v>8273.200000000001</v>
+      </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -2316,6 +2355,7 @@
       <c r="AO15" s="13" t="n"/>
       <c r="AP15" s="13" t="n"/>
       <c r="AQ15" s="13" t="n"/>
+      <c r="AR15" s="13" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -2446,6 +2486,9 @@
       </c>
       <c r="AQ16" s="13" t="n">
         <v>34.95</v>
+      </c>
+      <c r="AR16" s="13" t="n">
+        <v>38.41</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -2530,6 +2573,9 @@
       <c r="AQ17" s="13" t="n">
         <v>2603.88</v>
       </c>
+      <c r="AR17" s="13" t="n">
+        <v>2686.56</v>
+      </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="3" t="n">
@@ -2623,6 +2669,7 @@
       <c r="AO18" s="13" t="n"/>
       <c r="AP18" s="13" t="n"/>
       <c r="AQ18" s="13" t="n"/>
+      <c r="AR18" s="13" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -2753,6 +2800,9 @@
       </c>
       <c r="AQ19" s="13" t="n">
         <v>93.62</v>
+      </c>
+      <c r="AR19" s="13" t="n">
+        <v>97.03</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -2837,6 +2887,9 @@
       <c r="AQ20" s="13" t="n">
         <v>6782.81</v>
       </c>
+      <c r="AR20" s="13" t="n">
+        <v>7126.06</v>
+      </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -2930,6 +2983,7 @@
       <c r="AO21" s="13" t="n"/>
       <c r="AP21" s="13" t="n"/>
       <c r="AQ21" s="13" t="n"/>
+      <c r="AR21" s="13" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -3058,6 +3112,9 @@
       </c>
       <c r="AQ22" s="13" t="n">
         <v>45.14</v>
+      </c>
+      <c r="AR22" s="13" t="n">
+        <v>47.12</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1">
@@ -3142,6 +3199,9 @@
       <c r="AQ23" s="13" t="n">
         <v>76868</v>
       </c>
+      <c r="AR23" s="13" t="n">
+        <v>78785.81</v>
+      </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="3" t="n">
@@ -3235,6 +3295,7 @@
       <c r="AO24" s="13" t="n"/>
       <c r="AP24" s="13" t="n"/>
       <c r="AQ24" s="13" t="n"/>
+      <c r="AR24" s="13" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -3365,6 +3426,9 @@
       </c>
       <c r="AQ25" s="13" t="n">
         <v>39.88</v>
+      </c>
+      <c r="AR25" s="13" t="n">
+        <v>51.61</v>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="1">
@@ -3449,6 +3513,9 @@
       <c r="AQ26" s="13" t="n">
         <v>24080.63</v>
       </c>
+      <c r="AR26" s="13" t="n">
+        <v>24702.24</v>
+      </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -3542,6 +3609,7 @@
       <c r="AO27" s="13" t="n"/>
       <c r="AP27" s="13" t="n"/>
       <c r="AQ27" s="13" t="n"/>
+      <c r="AR27" s="13" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -3672,6 +3740,9 @@
       </c>
       <c r="AQ28" s="13" t="n">
         <v>77.64</v>
+      </c>
+      <c r="AR28" s="13" t="n">
+        <v>87.84999999999999</v>
       </c>
     </row>
     <row r="29" ht="14.25" customHeight="1">
@@ -3756,6 +3827,9 @@
       <c r="AQ29" s="13" t="n">
         <v>55960.86</v>
       </c>
+      <c r="AR29" s="13" t="n">
+        <v>58843.53</v>
+      </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="3" t="n">
@@ -3849,6 +3923,7 @@
       <c r="AO30" s="13" t="n"/>
       <c r="AP30" s="13" t="n"/>
       <c r="AQ30" s="13" t="n"/>
+      <c r="AR30" s="13" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -3979,6 +4054,9 @@
       </c>
       <c r="AQ31" s="13" t="n">
         <v>52.98</v>
+      </c>
+      <c r="AR31" s="13" t="n">
+        <v>53.21</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -4063,6 +4141,9 @@
       <c r="AQ32" s="13" t="n">
         <v>5681.52</v>
       </c>
+      <c r="AR32" s="13" t="n">
+        <v>5699.93</v>
+      </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
       <c r="A33" s="3" t="n">
@@ -4156,6 +4237,7 @@
       <c r="AO33" s="13" t="n"/>
       <c r="AP33" s="13" t="n"/>
       <c r="AQ33" s="13" t="n"/>
+      <c r="AR33" s="13" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -4286,6 +4368,9 @@
       </c>
       <c r="AQ34" s="13" t="n">
         <v>1.57</v>
+      </c>
+      <c r="AR34" s="13" t="n">
+        <v>3.25</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -4370,6 +4455,9 @@
       <c r="AQ35" s="13" t="n">
         <v>33457.58</v>
       </c>
+      <c r="AR35" s="13" t="n">
+        <v>33972.49</v>
+      </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="3" t="n">
@@ -4463,6 +4551,7 @@
       <c r="AO36" s="13" t="n"/>
       <c r="AP36" s="13" t="n"/>
       <c r="AQ36" s="13" t="n"/>
+      <c r="AR36" s="13" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -4593,6 +4682,9 @@
       </c>
       <c r="AQ37" s="13" t="n">
         <v>48.05</v>
+      </c>
+      <c r="AR37" s="13" t="n">
+        <v>54.14</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -4677,6 +4769,9 @@
       <c r="AQ38" s="13" t="n">
         <v>3508.72</v>
       </c>
+      <c r="AR38" s="13" t="n">
+        <v>3921.47</v>
+      </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
       <c r="A39" s="3" t="n">
@@ -4770,6 +4865,7 @@
       <c r="AO39" s="13" t="n"/>
       <c r="AP39" s="13" t="n"/>
       <c r="AQ39" s="13" t="n"/>
+      <c r="AR39" s="13" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -4900,6 +4996,9 @@
       </c>
       <c r="AQ40" s="13" t="n">
         <v>49.39</v>
+      </c>
+      <c r="AR40" s="13" t="n">
+        <v>55.36</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -4984,6 +5083,9 @@
       <c r="AQ41" s="13" t="n">
         <v>3323.04</v>
       </c>
+      <c r="AR41" s="13" t="n">
+        <v>3666.26</v>
+      </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
       <c r="A42" s="3" t="n">
@@ -5077,6 +5179,7 @@
       <c r="AO42" s="13" t="n"/>
       <c r="AP42" s="13" t="n"/>
       <c r="AQ42" s="13" t="n"/>
+      <c r="AR42" s="13" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -5207,6 +5310,9 @@
       </c>
       <c r="AQ43" s="13" t="n">
         <v>9.82</v>
+      </c>
+      <c r="AR43" s="13" t="n">
+        <v>7.02</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -5291,6 +5397,9 @@
       <c r="AQ44" s="13" t="n">
         <v>6679.05</v>
       </c>
+      <c r="AR44" s="13" t="n">
+        <v>6653.77</v>
+      </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
       <c r="A45" s="3" t="n">
@@ -5384,6 +5493,7 @@
       <c r="AO45" s="13" t="n"/>
       <c r="AP45" s="13" t="n"/>
       <c r="AQ45" s="13" t="n"/>
+      <c r="AR45" s="13" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -5514,6 +5624,9 @@
       </c>
       <c r="AQ46" s="13" t="n">
         <v>13.88</v>
+      </c>
+      <c r="AR46" s="13" t="n">
+        <v>11.81</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -5598,6 +5711,9 @@
       <c r="AQ47" s="13" t="n">
         <v>8093.93</v>
       </c>
+      <c r="AR47" s="13" t="n">
+        <v>7928.24</v>
+      </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
       <c r="A48" s="3" t="n">
@@ -5691,6 +5807,7 @@
       <c r="AO48" s="13" t="n"/>
       <c r="AP48" s="13" t="n"/>
       <c r="AQ48" s="13" t="n"/>
+      <c r="AR48" s="13" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -5821,6 +5938,9 @@
       </c>
       <c r="AQ49" s="13" t="n">
         <v>3.81</v>
+      </c>
+      <c r="AR49" s="13" t="n">
+        <v>3.68</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -5905,6 +6025,9 @@
       <c r="AQ50" s="13" t="n">
         <v>11690.71</v>
       </c>
+      <c r="AR50" s="13" t="n">
+        <v>11720.61</v>
+      </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
       <c r="A51" s="3" t="n">
@@ -5998,6 +6121,7 @@
       <c r="AO51" s="13" t="n"/>
       <c r="AP51" s="13" t="n"/>
       <c r="AQ51" s="13" t="n"/>
+      <c r="AR51" s="13" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -6128,6 +6252,9 @@
       </c>
       <c r="AQ52" s="13" t="n">
         <v>17.15</v>
+      </c>
+      <c r="AR52" s="13" t="n">
+        <v>19.66</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -6212,6 +6339,9 @@
       <c r="AQ53" s="13" t="n">
         <v>11720.09</v>
       </c>
+      <c r="AR53" s="13" t="n">
+        <v>12119.41</v>
+      </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
       <c r="A54" s="3" t="n">
@@ -6305,6 +6435,7 @@
       <c r="AO54" s="13" t="n"/>
       <c r="AP54" s="13" t="n"/>
       <c r="AQ54" s="13" t="n"/>
+      <c r="AR54" s="13" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -6435,6 +6566,9 @@
       </c>
       <c r="AQ55" s="13" t="n">
         <v>13.06</v>
+      </c>
+      <c r="AR55" s="13" t="n">
+        <v>11.54</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -6519,6 +6653,9 @@
       <c r="AQ56" s="13" t="n">
         <v>7730.15</v>
       </c>
+      <c r="AR56" s="13" t="n">
+        <v>7674.01</v>
+      </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
       <c r="A57" s="3" t="n">
@@ -6612,6 +6749,7 @@
       <c r="AO57" s="13" t="n"/>
       <c r="AP57" s="13" t="n"/>
       <c r="AQ57" s="13" t="n"/>
+      <c r="AR57" s="13" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -6742,6 +6880,9 @@
       </c>
       <c r="AQ58" s="13" t="n">
         <v>17.76</v>
+      </c>
+      <c r="AR58" s="13" t="n">
+        <v>16.02</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -6826,6 +6967,9 @@
       <c r="AQ59" s="13" t="n">
         <v>14355.15</v>
       </c>
+      <c r="AR59" s="13" t="n">
+        <v>14280.65</v>
+      </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
       <c r="A60" s="3" t="n">
@@ -6919,6 +7063,7 @@
       <c r="AO60" s="13" t="n"/>
       <c r="AP60" s="13" t="n"/>
       <c r="AQ60" s="13" t="n"/>
+      <c r="AR60" s="13" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -7049,6 +7194,9 @@
       </c>
       <c r="AQ61" s="13" t="n">
         <v>67.66</v>
+      </c>
+      <c r="AR61" s="13" t="n">
+        <v>68.16</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -7133,6 +7281,9 @@
       <c r="AQ62" s="13" t="n">
         <v>15372.38</v>
       </c>
+      <c r="AR62" s="13" t="n">
+        <v>15713.35</v>
+      </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
       <c r="A63" s="3" t="n">
@@ -7226,6 +7377,7 @@
       <c r="AO63" s="13" t="n"/>
       <c r="AP63" s="13" t="n"/>
       <c r="AQ63" s="13" t="n"/>
+      <c r="AR63" s="13" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -7356,6 +7508,9 @@
       </c>
       <c r="AQ64" s="13" t="n">
         <v>7.79</v>
+      </c>
+      <c r="AR64" s="13" t="n">
+        <v>9.91</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -7440,6 +7595,9 @@
       <c r="AQ65" s="13" t="n">
         <v>7497.88</v>
       </c>
+      <c r="AR65" s="13" t="n">
+        <v>8126.29</v>
+      </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
       <c r="A66" s="3" t="n">
@@ -7533,6 +7691,7 @@
       <c r="AO66" s="13" t="n"/>
       <c r="AP66" s="13" t="n"/>
       <c r="AQ66" s="13" t="n"/>
+      <c r="AR66" s="13" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -7663,6 +7822,9 @@
       </c>
       <c r="AQ67" s="13" t="n">
         <v>6.73</v>
+      </c>
+      <c r="AR67" s="13" t="n">
+        <v>4.81</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -7747,6 +7909,9 @@
       <c r="AQ68" s="13" t="n">
         <v>9168.190000000001</v>
       </c>
+      <c r="AR68" s="13" t="n">
+        <v>9085.629999999999</v>
+      </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
       <c r="A69" s="3" t="n">
@@ -7840,6 +8005,7 @@
       <c r="AO69" s="13" t="n"/>
       <c r="AP69" s="13" t="n"/>
       <c r="AQ69" s="13" t="n"/>
+      <c r="AR69" s="13" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -7970,6 +8136,9 @@
       </c>
       <c r="AQ70" s="13" t="n">
         <v>23.03</v>
+      </c>
+      <c r="AR70" s="13" t="n">
+        <v>24.59</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -8054,6 +8223,9 @@
       <c r="AQ71" s="13" t="n">
         <v>2509.36</v>
       </c>
+      <c r="AR71" s="13" t="n">
+        <v>2621.46</v>
+      </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
       <c r="A72" s="3" t="n">
@@ -8147,6 +8319,7 @@
       <c r="AO72" s="13" t="n"/>
       <c r="AP72" s="13" t="n"/>
       <c r="AQ72" s="13" t="n"/>
+      <c r="AR72" s="13" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -8277,6 +8450,9 @@
       </c>
       <c r="AQ73" s="13" t="n">
         <v>33.47</v>
+      </c>
+      <c r="AR73" s="13" t="n">
+        <v>38.59</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -8361,6 +8537,9 @@
       <c r="AQ74" s="13" t="n">
         <v>4853.32</v>
       </c>
+      <c r="AR74" s="13" t="n">
+        <v>5058.73</v>
+      </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
       <c r="A75" s="3" t="n">
@@ -8454,6 +8633,7 @@
       <c r="AO75" s="13" t="n"/>
       <c r="AP75" s="13" t="n"/>
       <c r="AQ75" s="13" t="n"/>
+      <c r="AR75" s="13" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -8584,6 +8764,9 @@
       </c>
       <c r="AQ76" s="13" t="n">
         <v>19.37</v>
+      </c>
+      <c r="AR76" s="13" t="n">
+        <v>17.63</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -8668,6 +8851,9 @@
       <c r="AQ77" s="13" t="n">
         <v>8720.290000000001</v>
       </c>
+      <c r="AR77" s="13" t="n">
+        <v>8634.299999999999</v>
+      </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
       <c r="A78" s="3" t="n">
@@ -8761,6 +8947,7 @@
       <c r="AO78" s="13" t="n"/>
       <c r="AP78" s="13" t="n"/>
       <c r="AQ78" s="13" t="n"/>
+      <c r="AR78" s="13" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -8891,6 +9078,9 @@
       </c>
       <c r="AQ79" s="13" t="n">
         <v>11.46</v>
+      </c>
+      <c r="AR79" s="13" t="n">
+        <v>9.57</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -8975,6 +9165,9 @@
       <c r="AQ80" s="13" t="n">
         <v>1254.89</v>
       </c>
+      <c r="AR80" s="13" t="n">
+        <v>1285.52</v>
+      </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
       <c r="A81" s="3" t="n">
@@ -9068,6 +9261,7 @@
       <c r="AO81" s="13" t="n"/>
       <c r="AP81" s="13" t="n"/>
       <c r="AQ81" s="13" t="n"/>
+      <c r="AR81" s="13" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -9198,6 +9392,9 @@
       </c>
       <c r="AQ82" s="13" t="n">
         <v>10.93</v>
+      </c>
+      <c r="AR82" s="13" t="n">
+        <v>10.43</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -9282,6 +9479,9 @@
       <c r="AQ83" s="13" t="n">
         <v>15715.7</v>
       </c>
+      <c r="AR83" s="13" t="n">
+        <v>15524.12</v>
+      </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
       <c r="A84" s="3" t="n">
@@ -9375,6 +9575,7 @@
       <c r="AO84" s="13" t="n"/>
       <c r="AP84" s="13" t="n"/>
       <c r="AQ84" s="13" t="n"/>
+      <c r="AR84" s="13" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -9505,6 +9706,9 @@
       </c>
       <c r="AQ85" s="13" t="n">
         <v>60.25</v>
+      </c>
+      <c r="AR85" s="13" t="n">
+        <v>67.44</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -9589,6 +9793,9 @@
       <c r="AQ86" s="13" t="n">
         <v>2906.96</v>
       </c>
+      <c r="AR86" s="13" t="n">
+        <v>3148.13</v>
+      </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
       <c r="A87" s="3" t="n">
@@ -9682,6 +9889,7 @@
       <c r="AO87" s="13" t="n"/>
       <c r="AP87" s="13" t="n"/>
       <c r="AQ87" s="13" t="n"/>
+      <c r="AR87" s="13" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -9812,6 +10020,9 @@
       </c>
       <c r="AQ88" s="13" t="n">
         <v>72.81</v>
+      </c>
+      <c r="AR88" s="13" t="n">
+        <v>73.45</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -9896,6 +10107,9 @@
       <c r="AQ89" s="13" t="n">
         <v>3064.47</v>
       </c>
+      <c r="AR89" s="13" t="n">
+        <v>3223.51</v>
+      </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
       <c r="A90" s="3" t="n">
@@ -9989,6 +10203,7 @@
       <c r="AO90" s="13" t="n"/>
       <c r="AP90" s="13" t="n"/>
       <c r="AQ90" s="13" t="n"/>
+      <c r="AR90" s="13" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -10119,6 +10334,9 @@
       </c>
       <c r="AQ91" s="13" t="n">
         <v>52.12</v>
+      </c>
+      <c r="AR91" s="13" t="n">
+        <v>59.8</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -10203,6 +10421,9 @@
       <c r="AQ92" s="13" t="n">
         <v>3015.84</v>
       </c>
+      <c r="AR92" s="13" t="n">
+        <v>3260.45</v>
+      </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
       <c r="A93" s="3" t="n">
@@ -10296,6 +10517,7 @@
       <c r="AO93" s="13" t="n"/>
       <c r="AP93" s="13" t="n"/>
       <c r="AQ93" s="13" t="n"/>
+      <c r="AR93" s="13" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -10426,6 +10648,9 @@
       </c>
       <c r="AQ94" s="13" t="n">
         <v>47.69</v>
+      </c>
+      <c r="AR94" s="13" t="n">
+        <v>46.76</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -10510,6 +10735,9 @@
       <c r="AQ95" s="13" t="n">
         <v>1828.38</v>
       </c>
+      <c r="AR95" s="13" t="n">
+        <v>1929.07</v>
+      </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
       <c r="A96" s="3" t="n">
@@ -10603,6 +10831,7 @@
       <c r="AO96" s="13" t="n"/>
       <c r="AP96" s="13" t="n"/>
       <c r="AQ96" s="13" t="n"/>
+      <c r="AR96" s="13" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -10733,6 +10962,9 @@
       </c>
       <c r="AQ97" s="13" t="n">
         <v>26.23</v>
+      </c>
+      <c r="AR97" s="13" t="n">
+        <v>24.32</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -10817,6 +11049,9 @@
       <c r="AQ98" s="13" t="n">
         <v>9711.76</v>
       </c>
+      <c r="AR98" s="13" t="n">
+        <v>9738.120000000001</v>
+      </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
       <c r="A99" s="3" t="n">
@@ -10910,6 +11145,7 @@
       <c r="AO99" s="13" t="n"/>
       <c r="AP99" s="13" t="n"/>
       <c r="AQ99" s="13" t="n"/>
+      <c r="AR99" s="13" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -11040,6 +11276,9 @@
       </c>
       <c r="AQ100" s="13" t="n">
         <v>85.66</v>
+      </c>
+      <c r="AR100" s="13" t="n">
+        <v>87.91</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -11124,6 +11363,9 @@
       <c r="AQ101" s="13" t="n">
         <v>9633.639999999999</v>
       </c>
+      <c r="AR101" s="13" t="n">
+        <v>10378.55</v>
+      </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
       <c r="A102" s="3" t="n">
@@ -11217,6 +11459,7 @@
       <c r="AO102" s="13" t="n"/>
       <c r="AP102" s="13" t="n"/>
       <c r="AQ102" s="13" t="n"/>
+      <c r="AR102" s="13" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -11347,6 +11590,9 @@
       </c>
       <c r="AQ103" s="13" t="n">
         <v>72.7</v>
+      </c>
+      <c r="AR103" s="13" t="n">
+        <v>77.14</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -11431,6 +11677,9 @@
       <c r="AQ104" s="13" t="n">
         <v>13517.75</v>
       </c>
+      <c r="AR104" s="13" t="n">
+        <v>14539.63</v>
+      </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
       <c r="A105" s="3" t="n">
@@ -11524,6 +11773,7 @@
       <c r="AO105" s="13" t="n"/>
       <c r="AP105" s="13" t="n"/>
       <c r="AQ105" s="13" t="n"/>
+      <c r="AR105" s="13" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -11654,6 +11904,9 @@
       </c>
       <c r="AQ106" s="13" t="n">
         <v>13.83</v>
+      </c>
+      <c r="AR106" s="13" t="n">
+        <v>15.11</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -11738,6 +11991,9 @@
       <c r="AQ107" s="13" t="n">
         <v>2134.75</v>
       </c>
+      <c r="AR107" s="13" t="n">
+        <v>2181.31</v>
+      </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
       <c r="A108" s="3" t="n">
@@ -11831,6 +12087,7 @@
       <c r="AO108" s="13" t="n"/>
       <c r="AP108" s="13" t="n"/>
       <c r="AQ108" s="13" t="n"/>
+      <c r="AR108" s="13" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -11961,6 +12218,9 @@
       </c>
       <c r="AQ109" s="13" t="n">
         <v>11.62</v>
+      </c>
+      <c r="AR109" s="13" t="n">
+        <v>13.48</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -12045,6 +12305,9 @@
       <c r="AQ110" s="13" t="n">
         <v>725.62</v>
       </c>
+      <c r="AR110" s="13" t="n">
+        <v>754.5700000000001</v>
+      </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
       <c r="A111" s="3" t="n">
@@ -12138,6 +12401,7 @@
       <c r="AO111" s="13" t="n"/>
       <c r="AP111" s="13" t="n"/>
       <c r="AQ111" s="13" t="n"/>
+      <c r="AR111" s="13" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -12268,6 +12532,9 @@
       </c>
       <c r="AQ112" s="13" t="n">
         <v>80.81999999999999</v>
+      </c>
+      <c r="AR112" s="13" t="n">
+        <v>81.18000000000001</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -12352,6 +12619,9 @@
       <c r="AQ113" s="13" t="n">
         <v>3387.4</v>
       </c>
+      <c r="AR113" s="13" t="n">
+        <v>3499.39</v>
+      </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
       <c r="A114" s="3" t="n">
@@ -12445,6 +12715,7 @@
       <c r="AO114" s="13" t="n"/>
       <c r="AP114" s="13" t="n"/>
       <c r="AQ114" s="13" t="n"/>
+      <c r="AR114" s="13" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -12575,6 +12846,9 @@
       </c>
       <c r="AQ115" s="13" t="n">
         <v>32.43</v>
+      </c>
+      <c r="AR115" s="13" t="n">
+        <v>28.92</v>
       </c>
     </row>
     <row r="116">
@@ -12643,6 +12917,9 @@
       </c>
       <c r="AQ116" s="13" t="n">
         <v>4025.45</v>
+      </c>
+      <c r="AR116" s="13" t="n">
+        <v>4054.16</v>
       </c>
     </row>
     <row r="117">
@@ -12692,6 +12969,7 @@
       <c r="AO117" s="13" t="n"/>
       <c r="AP117" s="13" t="n"/>
       <c r="AQ117" s="13" t="n"/>
+      <c r="AR117" s="13" t="n"/>
     </row>
     <row r="118">
       <c r="P118" s="13" t="n">
@@ -12778,6 +13056,9 @@
       <c r="AQ118" s="13" t="n">
         <v>29.02</v>
       </c>
+      <c r="AR118" s="13" t="n">
+        <v>29.02</v>
+      </c>
     </row>
     <row r="119">
       <c r="Y119" s="13" t="n">
@@ -12836,6 +13117,9 @@
       </c>
       <c r="AQ119" s="13" t="n">
         <v>2662.11</v>
+      </c>
+      <c r="AR119" s="13" t="n">
+        <v>2780.43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-04-23 05:52:35]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR119"/>
+  <dimension ref="A1:AS119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="15"/>
@@ -561,6 +561,7 @@
     <col width="15" customWidth="1" min="42" max="42"/>
     <col width="15" customWidth="1" min="43" max="43"/>
     <col width="15" customWidth="1" min="44" max="44"/>
+    <col width="15" customWidth="1" min="45" max="45"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -784,6 +785,11 @@
           <t>2026/04/20</t>
         </is>
       </c>
+      <c r="AS1" s="13" t="inlineStr">
+        <is>
+          <t>2026/04/23</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1006,6 +1012,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="AS2" s="14" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1140,6 +1151,9 @@
       <c r="AR3" s="13" t="n">
         <v>69.16</v>
       </c>
+      <c r="AS3" s="13" t="n">
+        <v>70.06</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1273,6 +1287,9 @@
       </c>
       <c r="AR4" s="13" t="n">
         <v>4072.26</v>
+      </c>
+      <c r="AS4" s="13" t="n">
+        <v>4094.07</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1320,6 +1337,7 @@
       <c r="AP5" s="13" t="n"/>
       <c r="AQ5" s="13" t="n"/>
       <c r="AR5" s="13" t="n"/>
+      <c r="AS5" s="13" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1414,6 +1432,7 @@
       <c r="AP6" s="13" t="n"/>
       <c r="AQ6" s="13" t="n"/>
       <c r="AR6" s="13" t="n"/>
+      <c r="AS6" s="13" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1547,6 +1566,9 @@
       </c>
       <c r="AR7" s="13" t="n">
         <v>66.72</v>
+      </c>
+      <c r="AS7" s="13" t="n">
+        <v>68.37</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -1634,6 +1656,9 @@
       <c r="AR8" s="13" t="n">
         <v>5941.99</v>
       </c>
+      <c r="AS8" s="13" t="n">
+        <v>5985.8</v>
+      </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -1728,6 +1753,7 @@
       <c r="AP9" s="13" t="n"/>
       <c r="AQ9" s="13" t="n"/>
       <c r="AR9" s="13" t="n"/>
+      <c r="AS9" s="13" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -1861,6 +1887,9 @@
       </c>
       <c r="AR10" s="13" t="n">
         <v>56.55</v>
+      </c>
+      <c r="AS10" s="13" t="n">
+        <v>59.81</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -1948,6 +1977,9 @@
       <c r="AR11" s="13" t="n">
         <v>4747.66</v>
       </c>
+      <c r="AS11" s="13" t="n">
+        <v>4797.1</v>
+      </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -2042,6 +2074,7 @@
       <c r="AP12" s="13" t="n"/>
       <c r="AQ12" s="13" t="n"/>
       <c r="AR12" s="13" t="n"/>
+      <c r="AS12" s="13" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2175,6 +2208,9 @@
       </c>
       <c r="AR13" s="13" t="n">
         <v>66.94</v>
+      </c>
+      <c r="AS13" s="13" t="n">
+        <v>67.94</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -2262,6 +2298,9 @@
       <c r="AR14" s="13" t="n">
         <v>8273.200000000001</v>
       </c>
+      <c r="AS14" s="13" t="n">
+        <v>8311.73</v>
+      </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -2356,6 +2395,7 @@
       <c r="AP15" s="13" t="n"/>
       <c r="AQ15" s="13" t="n"/>
       <c r="AR15" s="13" t="n"/>
+      <c r="AS15" s="13" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -2489,6 +2529,9 @@
       </c>
       <c r="AR16" s="13" t="n">
         <v>38.41</v>
+      </c>
+      <c r="AS16" s="13" t="n">
+        <v>40.6</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -2576,6 +2619,9 @@
       <c r="AR17" s="13" t="n">
         <v>2686.56</v>
       </c>
+      <c r="AS17" s="13" t="n">
+        <v>2603.99</v>
+      </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="3" t="n">
@@ -2670,6 +2716,7 @@
       <c r="AP18" s="13" t="n"/>
       <c r="AQ18" s="13" t="n"/>
       <c r="AR18" s="13" t="n"/>
+      <c r="AS18" s="13" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -2803,6 +2850,9 @@
       </c>
       <c r="AR19" s="13" t="n">
         <v>97.03</v>
+      </c>
+      <c r="AS19" s="13" t="n">
+        <v>96.84</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -2890,6 +2940,9 @@
       <c r="AR20" s="13" t="n">
         <v>7126.06</v>
       </c>
+      <c r="AS20" s="13" t="n">
+        <v>7137.9</v>
+      </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -2984,6 +3037,7 @@
       <c r="AP21" s="13" t="n"/>
       <c r="AQ21" s="13" t="n"/>
       <c r="AR21" s="13" t="n"/>
+      <c r="AS21" s="13" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -3115,6 +3169,9 @@
       </c>
       <c r="AR22" s="13" t="n">
         <v>47.12</v>
+      </c>
+      <c r="AS22" s="13" t="n">
+        <v>46.82</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1">
@@ -3202,6 +3259,9 @@
       <c r="AR23" s="13" t="n">
         <v>78785.81</v>
       </c>
+      <c r="AS23" s="13" t="n">
+        <v>77880.09</v>
+      </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="3" t="n">
@@ -3296,6 +3356,7 @@
       <c r="AP24" s="13" t="n"/>
       <c r="AQ24" s="13" t="n"/>
       <c r="AR24" s="13" t="n"/>
+      <c r="AS24" s="13" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -3429,6 +3490,9 @@
       </c>
       <c r="AR25" s="13" t="n">
         <v>51.61</v>
+      </c>
+      <c r="AS25" s="13" t="n">
+        <v>77</v>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="1">
@@ -3516,6 +3580,7 @@
       <c r="AR26" s="13" t="n">
         <v>24702.24</v>
       </c>
+      <c r="AS26" s="13" t="inlineStr"/>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -3610,6 +3675,7 @@
       <c r="AP27" s="13" t="n"/>
       <c r="AQ27" s="13" t="n"/>
       <c r="AR27" s="13" t="n"/>
+      <c r="AS27" s="13" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -3743,6 +3809,9 @@
       </c>
       <c r="AR28" s="13" t="n">
         <v>87.84999999999999</v>
+      </c>
+      <c r="AS28" s="13" t="n">
+        <v>87.67</v>
       </c>
     </row>
     <row r="29" ht="14.25" customHeight="1">
@@ -3830,6 +3899,9 @@
       <c r="AR29" s="13" t="n">
         <v>58843.53</v>
       </c>
+      <c r="AS29" s="13" t="n">
+        <v>59114.07</v>
+      </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="3" t="n">
@@ -3924,6 +3996,7 @@
       <c r="AP30" s="13" t="n"/>
       <c r="AQ30" s="13" t="n"/>
       <c r="AR30" s="13" t="n"/>
+      <c r="AS30" s="13" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -4057,6 +4130,9 @@
       </c>
       <c r="AR31" s="13" t="n">
         <v>53.21</v>
+      </c>
+      <c r="AS31" s="13" t="n">
+        <v>52.9</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -4144,6 +4220,9 @@
       <c r="AR32" s="13" t="n">
         <v>5699.93</v>
       </c>
+      <c r="AS32" s="13" t="n">
+        <v>5783.37</v>
+      </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
       <c r="A33" s="3" t="n">
@@ -4238,6 +4317,7 @@
       <c r="AP33" s="13" t="n"/>
       <c r="AQ33" s="13" t="n"/>
       <c r="AR33" s="13" t="n"/>
+      <c r="AS33" s="13" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -4371,6 +4451,9 @@
       </c>
       <c r="AR34" s="13" t="n">
         <v>3.25</v>
+      </c>
+      <c r="AS34" s="13" t="n">
+        <v>3.83</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -4458,6 +4541,9 @@
       <c r="AR35" s="13" t="n">
         <v>33972.49</v>
       </c>
+      <c r="AS35" s="13" t="n">
+        <v>33566.19</v>
+      </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="3" t="n">
@@ -4552,6 +4638,7 @@
       <c r="AP36" s="13" t="n"/>
       <c r="AQ36" s="13" t="n"/>
       <c r="AR36" s="13" t="n"/>
+      <c r="AS36" s="13" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -4685,6 +4772,9 @@
       </c>
       <c r="AR37" s="13" t="n">
         <v>54.14</v>
+      </c>
+      <c r="AS37" s="13" t="n">
+        <v>57.78</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -4772,6 +4862,9 @@
       <c r="AR38" s="13" t="n">
         <v>3921.47</v>
       </c>
+      <c r="AS38" s="13" t="n">
+        <v>4006.23</v>
+      </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
       <c r="A39" s="3" t="n">
@@ -4866,6 +4959,7 @@
       <c r="AP39" s="13" t="n"/>
       <c r="AQ39" s="13" t="n"/>
       <c r="AR39" s="13" t="n"/>
+      <c r="AS39" s="13" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -4999,6 +5093,9 @@
       </c>
       <c r="AR40" s="13" t="n">
         <v>55.36</v>
+      </c>
+      <c r="AS40" s="13" t="n">
+        <v>59.44</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -5086,6 +5183,9 @@
       <c r="AR41" s="13" t="n">
         <v>3666.26</v>
       </c>
+      <c r="AS41" s="13" t="n">
+        <v>3739.56</v>
+      </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
       <c r="A42" s="3" t="n">
@@ -5180,6 +5280,7 @@
       <c r="AP42" s="13" t="n"/>
       <c r="AQ42" s="13" t="n"/>
       <c r="AR42" s="13" t="n"/>
+      <c r="AS42" s="13" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -5313,6 +5414,9 @@
       </c>
       <c r="AR43" s="13" t="n">
         <v>7.02</v>
+      </c>
+      <c r="AS43" s="13" t="n">
+        <v>8.449999999999999</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -5400,6 +5504,9 @@
       <c r="AR44" s="13" t="n">
         <v>6653.77</v>
       </c>
+      <c r="AS44" s="13" t="n">
+        <v>6662.32</v>
+      </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
       <c r="A45" s="3" t="n">
@@ -5494,6 +5601,7 @@
       <c r="AP45" s="13" t="n"/>
       <c r="AQ45" s="13" t="n"/>
       <c r="AR45" s="13" t="n"/>
+      <c r="AS45" s="13" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -5627,6 +5735,9 @@
       </c>
       <c r="AR46" s="13" t="n">
         <v>11.81</v>
+      </c>
+      <c r="AS46" s="13" t="n">
+        <v>12.35</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -5714,6 +5825,9 @@
       <c r="AR47" s="13" t="n">
         <v>7928.24</v>
       </c>
+      <c r="AS47" s="13" t="n">
+        <v>7931.04</v>
+      </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
       <c r="A48" s="3" t="n">
@@ -5808,6 +5922,7 @@
       <c r="AP48" s="13" t="n"/>
       <c r="AQ48" s="13" t="n"/>
       <c r="AR48" s="13" t="n"/>
+      <c r="AS48" s="13" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -5941,6 +6056,9 @@
       </c>
       <c r="AR49" s="13" t="n">
         <v>3.68</v>
+      </c>
+      <c r="AS49" s="13" t="n">
+        <v>6.81</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -6028,6 +6146,9 @@
       <c r="AR50" s="13" t="n">
         <v>11720.61</v>
       </c>
+      <c r="AS50" s="13" t="n">
+        <v>11652.13</v>
+      </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
       <c r="A51" s="3" t="n">
@@ -6122,6 +6243,7 @@
       <c r="AP51" s="13" t="n"/>
       <c r="AQ51" s="13" t="n"/>
       <c r="AR51" s="13" t="n"/>
+      <c r="AS51" s="13" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -6255,6 +6377,9 @@
       </c>
       <c r="AR52" s="13" t="n">
         <v>19.66</v>
+      </c>
+      <c r="AS52" s="13" t="n">
+        <v>22.38</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -6342,6 +6467,9 @@
       <c r="AR53" s="13" t="n">
         <v>12119.41</v>
       </c>
+      <c r="AS53" s="13" t="n">
+        <v>12200.71</v>
+      </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
       <c r="A54" s="3" t="n">
@@ -6436,6 +6564,7 @@
       <c r="AP54" s="13" t="n"/>
       <c r="AQ54" s="13" t="n"/>
       <c r="AR54" s="13" t="n"/>
+      <c r="AS54" s="13" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -6569,6 +6698,9 @@
       </c>
       <c r="AR55" s="13" t="n">
         <v>11.54</v>
+      </c>
+      <c r="AS55" s="13" t="n">
+        <v>11.38</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -6656,6 +6788,9 @@
       <c r="AR56" s="13" t="n">
         <v>7674.01</v>
       </c>
+      <c r="AS56" s="13" t="n">
+        <v>7784.09</v>
+      </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
       <c r="A57" s="3" t="n">
@@ -6750,6 +6885,7 @@
       <c r="AP57" s="13" t="n"/>
       <c r="AQ57" s="13" t="n"/>
       <c r="AR57" s="13" t="n"/>
+      <c r="AS57" s="13" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -6883,6 +7019,9 @@
       </c>
       <c r="AR58" s="13" t="n">
         <v>16.02</v>
+      </c>
+      <c r="AS58" s="13" t="n">
+        <v>18.02</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -6970,6 +7109,9 @@
       <c r="AR59" s="13" t="n">
         <v>14280.65</v>
       </c>
+      <c r="AS59" s="13" t="n">
+        <v>14208.87</v>
+      </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
       <c r="A60" s="3" t="n">
@@ -7064,6 +7206,7 @@
       <c r="AP60" s="13" t="n"/>
       <c r="AQ60" s="13" t="n"/>
       <c r="AR60" s="13" t="n"/>
+      <c r="AS60" s="13" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -7197,6 +7340,9 @@
       </c>
       <c r="AR61" s="13" t="n">
         <v>68.16</v>
+      </c>
+      <c r="AS61" s="13" t="n">
+        <v>66.11</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -7284,6 +7430,9 @@
       <c r="AR62" s="13" t="n">
         <v>15713.35</v>
       </c>
+      <c r="AS62" s="13" t="n">
+        <v>15569.82</v>
+      </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
       <c r="A63" s="3" t="n">
@@ -7378,6 +7527,7 @@
       <c r="AP63" s="13" t="n"/>
       <c r="AQ63" s="13" t="n"/>
       <c r="AR63" s="13" t="n"/>
+      <c r="AS63" s="13" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -7511,6 +7661,9 @@
       </c>
       <c r="AR64" s="13" t="n">
         <v>9.91</v>
+      </c>
+      <c r="AS64" s="13" t="n">
+        <v>7.65</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -7598,6 +7751,9 @@
       <c r="AR65" s="13" t="n">
         <v>8126.29</v>
       </c>
+      <c r="AS65" s="13" t="n">
+        <v>7776.03</v>
+      </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
       <c r="A66" s="3" t="n">
@@ -7692,6 +7848,7 @@
       <c r="AP66" s="13" t="n"/>
       <c r="AQ66" s="13" t="n"/>
       <c r="AR66" s="13" t="n"/>
+      <c r="AS66" s="13" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -7825,6 +7982,9 @@
       </c>
       <c r="AR67" s="13" t="n">
         <v>4.81</v>
+      </c>
+      <c r="AS67" s="13" t="n">
+        <v>4.29</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -7912,6 +8072,9 @@
       <c r="AR68" s="13" t="n">
         <v>9085.629999999999</v>
       </c>
+      <c r="AS68" s="13" t="n">
+        <v>9022.049999999999</v>
+      </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
       <c r="A69" s="3" t="n">
@@ -8006,6 +8169,7 @@
       <c r="AP69" s="13" t="n"/>
       <c r="AQ69" s="13" t="n"/>
       <c r="AR69" s="13" t="n"/>
+      <c r="AS69" s="13" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -8139,6 +8303,9 @@
       </c>
       <c r="AR70" s="13" t="n">
         <v>24.59</v>
+      </c>
+      <c r="AS70" s="13" t="n">
+        <v>23.49</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -8226,6 +8393,9 @@
       <c r="AR71" s="13" t="n">
         <v>2621.46</v>
       </c>
+      <c r="AS71" s="13" t="n">
+        <v>2511.45</v>
+      </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
       <c r="A72" s="3" t="n">
@@ -8320,6 +8490,7 @@
       <c r="AP72" s="13" t="n"/>
       <c r="AQ72" s="13" t="n"/>
       <c r="AR72" s="13" t="n"/>
+      <c r="AS72" s="13" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -8453,6 +8624,9 @@
       </c>
       <c r="AR73" s="13" t="n">
         <v>38.59</v>
+      </c>
+      <c r="AS73" s="13" t="n">
+        <v>34.62</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -8540,6 +8714,9 @@
       <c r="AR74" s="13" t="n">
         <v>5058.73</v>
       </c>
+      <c r="AS74" s="13" t="n">
+        <v>4862.12</v>
+      </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
       <c r="A75" s="3" t="n">
@@ -8634,6 +8811,7 @@
       <c r="AP75" s="13" t="n"/>
       <c r="AQ75" s="13" t="n"/>
       <c r="AR75" s="13" t="n"/>
+      <c r="AS75" s="13" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -8767,6 +8945,9 @@
       </c>
       <c r="AR76" s="13" t="n">
         <v>17.63</v>
+      </c>
+      <c r="AS76" s="13" t="n">
+        <v>17.66</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -8854,6 +9035,9 @@
       <c r="AR77" s="13" t="n">
         <v>8634.299999999999</v>
       </c>
+      <c r="AS77" s="13" t="n">
+        <v>8606.049999999999</v>
+      </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
       <c r="A78" s="3" t="n">
@@ -8948,6 +9132,7 @@
       <c r="AP78" s="13" t="n"/>
       <c r="AQ78" s="13" t="n"/>
       <c r="AR78" s="13" t="n"/>
+      <c r="AS78" s="13" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -9081,6 +9266,9 @@
       </c>
       <c r="AR79" s="13" t="n">
         <v>9.57</v>
+      </c>
+      <c r="AS79" s="13" t="n">
+        <v>9.98</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -9168,6 +9356,9 @@
       <c r="AR80" s="13" t="n">
         <v>1285.52</v>
       </c>
+      <c r="AS80" s="13" t="n">
+        <v>1283.89</v>
+      </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
       <c r="A81" s="3" t="n">
@@ -9262,6 +9453,7 @@
       <c r="AP81" s="13" t="n"/>
       <c r="AQ81" s="13" t="n"/>
       <c r="AR81" s="13" t="n"/>
+      <c r="AS81" s="13" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -9395,6 +9587,9 @@
       </c>
       <c r="AR82" s="13" t="n">
         <v>10.43</v>
+      </c>
+      <c r="AS82" s="13" t="n">
+        <v>10.59</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -9482,6 +9677,9 @@
       <c r="AR83" s="13" t="n">
         <v>15524.12</v>
       </c>
+      <c r="AS83" s="13" t="n">
+        <v>15515.64</v>
+      </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
       <c r="A84" s="3" t="n">
@@ -9576,6 +9774,7 @@
       <c r="AP84" s="13" t="n"/>
       <c r="AQ84" s="13" t="n"/>
       <c r="AR84" s="13" t="n"/>
+      <c r="AS84" s="13" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -9709,6 +9908,9 @@
       </c>
       <c r="AR85" s="13" t="n">
         <v>67.44</v>
+      </c>
+      <c r="AS85" s="13" t="n">
+        <v>70.63</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -9796,6 +9998,9 @@
       <c r="AR86" s="13" t="n">
         <v>3148.13</v>
       </c>
+      <c r="AS86" s="13" t="n">
+        <v>3155.78</v>
+      </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
       <c r="A87" s="3" t="n">
@@ -9890,6 +10095,7 @@
       <c r="AP87" s="13" t="n"/>
       <c r="AQ87" s="13" t="n"/>
       <c r="AR87" s="13" t="n"/>
+      <c r="AS87" s="13" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -10023,6 +10229,9 @@
       </c>
       <c r="AR88" s="13" t="n">
         <v>73.45</v>
+      </c>
+      <c r="AS88" s="13" t="n">
+        <v>74.06</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -10110,6 +10319,9 @@
       <c r="AR89" s="13" t="n">
         <v>3223.51</v>
       </c>
+      <c r="AS89" s="13" t="n">
+        <v>3218.21</v>
+      </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
       <c r="A90" s="3" t="n">
@@ -10204,6 +10416,7 @@
       <c r="AP90" s="13" t="n"/>
       <c r="AQ90" s="13" t="n"/>
       <c r="AR90" s="13" t="n"/>
+      <c r="AS90" s="13" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -10337,6 +10550,9 @@
       </c>
       <c r="AR91" s="13" t="n">
         <v>59.8</v>
+      </c>
+      <c r="AS91" s="13" t="n">
+        <v>60.49</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -10424,6 +10640,9 @@
       <c r="AR92" s="13" t="n">
         <v>3260.45</v>
       </c>
+      <c r="AS92" s="13" t="n">
+        <v>3260.88</v>
+      </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
       <c r="A93" s="3" t="n">
@@ -10518,6 +10737,7 @@
       <c r="AP93" s="13" t="n"/>
       <c r="AQ93" s="13" t="n"/>
       <c r="AR93" s="13" t="n"/>
+      <c r="AS93" s="13" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -10650,6 +10870,9 @@
         <v>47.69</v>
       </c>
       <c r="AR94" s="13" t="n">
+        <v>46.76</v>
+      </c>
+      <c r="AS94" s="13" t="n">
         <v>46.76</v>
       </c>
     </row>
@@ -10738,6 +10961,9 @@
       <c r="AR95" s="13" t="n">
         <v>1929.07</v>
       </c>
+      <c r="AS95" s="13" t="n">
+        <v>1889.03</v>
+      </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
       <c r="A96" s="3" t="n">
@@ -10832,6 +11058,7 @@
       <c r="AP96" s="13" t="n"/>
       <c r="AQ96" s="13" t="n"/>
       <c r="AR96" s="13" t="n"/>
+      <c r="AS96" s="13" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -10965,6 +11192,9 @@
       </c>
       <c r="AR97" s="13" t="n">
         <v>24.32</v>
+      </c>
+      <c r="AS97" s="13" t="n">
+        <v>25.27</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -11052,6 +11282,9 @@
       <c r="AR98" s="13" t="n">
         <v>9738.120000000001</v>
       </c>
+      <c r="AS98" s="13" t="n">
+        <v>9774.690000000001</v>
+      </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
       <c r="A99" s="3" t="n">
@@ -11146,6 +11379,7 @@
       <c r="AP99" s="13" t="n"/>
       <c r="AQ99" s="13" t="n"/>
       <c r="AR99" s="13" t="n"/>
+      <c r="AS99" s="13" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -11279,6 +11513,9 @@
       </c>
       <c r="AR100" s="13" t="n">
         <v>87.91</v>
+      </c>
+      <c r="AS100" s="13" t="n">
+        <v>90.58</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -11366,6 +11603,9 @@
       <c r="AR101" s="13" t="n">
         <v>10378.55</v>
       </c>
+      <c r="AS101" s="13" t="n">
+        <v>10434.95</v>
+      </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
       <c r="A102" s="3" t="n">
@@ -11460,6 +11700,7 @@
       <c r="AP102" s="13" t="n"/>
       <c r="AQ102" s="13" t="n"/>
       <c r="AR102" s="13" t="n"/>
+      <c r="AS102" s="13" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -11593,6 +11834,9 @@
       </c>
       <c r="AR103" s="13" t="n">
         <v>77.14</v>
+      </c>
+      <c r="AS103" s="13" t="n">
+        <v>80.34</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -11680,6 +11924,9 @@
       <c r="AR104" s="13" t="n">
         <v>14539.63</v>
       </c>
+      <c r="AS104" s="13" t="n">
+        <v>14577.16</v>
+      </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
       <c r="A105" s="3" t="n">
@@ -11774,6 +12021,7 @@
       <c r="AP105" s="13" t="n"/>
       <c r="AQ105" s="13" t="n"/>
       <c r="AR105" s="13" t="n"/>
+      <c r="AS105" s="13" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -11907,6 +12155,9 @@
       </c>
       <c r="AR106" s="13" t="n">
         <v>15.11</v>
+      </c>
+      <c r="AS106" s="13" t="n">
+        <v>22.43</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -11994,6 +12245,9 @@
       <c r="AR107" s="13" t="n">
         <v>2181.31</v>
       </c>
+      <c r="AS107" s="13" t="n">
+        <v>2153.1</v>
+      </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
       <c r="A108" s="3" t="n">
@@ -12088,6 +12342,7 @@
       <c r="AP108" s="13" t="n"/>
       <c r="AQ108" s="13" t="n"/>
       <c r="AR108" s="13" t="n"/>
+      <c r="AS108" s="13" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -12221,6 +12476,9 @@
       </c>
       <c r="AR109" s="13" t="n">
         <v>13.48</v>
+      </c>
+      <c r="AS109" s="13" t="n">
+        <v>12.59</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -12308,6 +12566,9 @@
       <c r="AR110" s="13" t="n">
         <v>754.5700000000001</v>
       </c>
+      <c r="AS110" s="13" t="n">
+        <v>749.27</v>
+      </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
       <c r="A111" s="3" t="n">
@@ -12402,6 +12663,7 @@
       <c r="AP111" s="13" t="n"/>
       <c r="AQ111" s="13" t="n"/>
       <c r="AR111" s="13" t="n"/>
+      <c r="AS111" s="13" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -12535,6 +12797,9 @@
       </c>
       <c r="AR112" s="13" t="n">
         <v>81.18000000000001</v>
+      </c>
+      <c r="AS112" s="13" t="n">
+        <v>79.61</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -12622,6 +12887,9 @@
       <c r="AR113" s="13" t="n">
         <v>3499.39</v>
       </c>
+      <c r="AS113" s="13" t="n">
+        <v>3393.05</v>
+      </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
       <c r="A114" s="3" t="n">
@@ -12716,6 +12984,7 @@
       <c r="AP114" s="13" t="n"/>
       <c r="AQ114" s="13" t="n"/>
       <c r="AR114" s="13" t="n"/>
+      <c r="AS114" s="13" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -12849,6 +13118,9 @@
       </c>
       <c r="AR115" s="13" t="n">
         <v>28.92</v>
+      </c>
+      <c r="AS115" s="13" t="n">
+        <v>30.88</v>
       </c>
     </row>
     <row r="116">
@@ -12920,6 +13192,9 @@
       </c>
       <c r="AR116" s="13" t="n">
         <v>4054.16</v>
+      </c>
+      <c r="AS116" s="13" t="n">
+        <v>4070.85</v>
       </c>
     </row>
     <row r="117">
@@ -12970,6 +13245,7 @@
       <c r="AP117" s="13" t="n"/>
       <c r="AQ117" s="13" t="n"/>
       <c r="AR117" s="13" t="n"/>
+      <c r="AS117" s="13" t="n"/>
     </row>
     <row r="118">
       <c r="P118" s="13" t="n">
@@ -13059,6 +13335,9 @@
       <c r="AR118" s="13" t="n">
         <v>29.02</v>
       </c>
+      <c r="AS118" s="13" t="n">
+        <v>29.02</v>
+      </c>
     </row>
     <row r="119">
       <c r="Y119" s="13" t="n">
@@ -13120,6 +13399,9 @@
       </c>
       <c r="AR119" s="13" t="n">
         <v>2780.43</v>
+      </c>
+      <c r="AS119" s="13" t="n">
+        <v>2792.96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-04-27 06:17:28]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS119"/>
+  <dimension ref="A1:AT119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="15"/>
@@ -562,6 +562,7 @@
     <col width="15" customWidth="1" min="43" max="43"/>
     <col width="15" customWidth="1" min="44" max="44"/>
     <col width="15" customWidth="1" min="45" max="45"/>
+    <col width="15" customWidth="1" min="46" max="46"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -790,6 +791,11 @@
           <t>2026/04/23</t>
         </is>
       </c>
+      <c r="AT1" s="13" t="inlineStr">
+        <is>
+          <t>2026/04/27</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1017,6 +1023,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="AT2" s="14" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1154,6 +1165,9 @@
       <c r="AS3" s="13" t="n">
         <v>70.06</v>
       </c>
+      <c r="AT3" s="13" t="n">
+        <v>69.06</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1290,6 +1304,9 @@
       </c>
       <c r="AS4" s="13" t="n">
         <v>4094.07</v>
+      </c>
+      <c r="AT4" s="13" t="n">
+        <v>4083.03</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1338,6 +1355,7 @@
       <c r="AQ5" s="13" t="n"/>
       <c r="AR5" s="13" t="n"/>
       <c r="AS5" s="13" t="n"/>
+      <c r="AT5" s="13" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1433,6 +1451,7 @@
       <c r="AQ6" s="13" t="n"/>
       <c r="AR6" s="13" t="n"/>
       <c r="AS6" s="13" t="n"/>
+      <c r="AT6" s="13" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1569,6 +1588,9 @@
       </c>
       <c r="AS7" s="13" t="n">
         <v>68.37</v>
+      </c>
+      <c r="AT7" s="13" t="n">
+        <v>67.44</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -1659,6 +1681,9 @@
       <c r="AS8" s="13" t="n">
         <v>5985.8</v>
       </c>
+      <c r="AT8" s="13" t="n">
+        <v>5960.28</v>
+      </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -1754,6 +1779,7 @@
       <c r="AQ9" s="13" t="n"/>
       <c r="AR9" s="13" t="n"/>
       <c r="AS9" s="13" t="n"/>
+      <c r="AT9" s="13" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -1890,6 +1916,9 @@
       </c>
       <c r="AS10" s="13" t="n">
         <v>59.81</v>
+      </c>
+      <c r="AT10" s="13" t="n">
+        <v>59.07</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -1980,6 +2009,9 @@
       <c r="AS11" s="13" t="n">
         <v>4797.1</v>
       </c>
+      <c r="AT11" s="13" t="n">
+        <v>4765.91</v>
+      </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -2075,6 +2107,7 @@
       <c r="AQ12" s="13" t="n"/>
       <c r="AR12" s="13" t="n"/>
       <c r="AS12" s="13" t="n"/>
+      <c r="AT12" s="13" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2211,6 +2244,9 @@
       </c>
       <c r="AS13" s="13" t="n">
         <v>67.94</v>
+      </c>
+      <c r="AT13" s="13" t="n">
+        <v>66.51000000000001</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -2301,6 +2337,9 @@
       <c r="AS14" s="13" t="n">
         <v>8311.73</v>
       </c>
+      <c r="AT14" s="13" t="n">
+        <v>8296.5</v>
+      </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -2396,6 +2435,7 @@
       <c r="AQ15" s="13" t="n"/>
       <c r="AR15" s="13" t="n"/>
       <c r="AS15" s="13" t="n"/>
+      <c r="AT15" s="13" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -2532,6 +2572,9 @@
       </c>
       <c r="AS16" s="13" t="n">
         <v>40.6</v>
+      </c>
+      <c r="AT16" s="13" t="n">
+        <v>39.94</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -2622,6 +2665,9 @@
       <c r="AS17" s="13" t="n">
         <v>2603.99</v>
       </c>
+      <c r="AT17" s="13" t="n">
+        <v>2630.77</v>
+      </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="3" t="n">
@@ -2717,6 +2763,7 @@
       <c r="AQ18" s="13" t="n"/>
       <c r="AR18" s="13" t="n"/>
       <c r="AS18" s="13" t="n"/>
+      <c r="AT18" s="13" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -2853,6 +2900,9 @@
       </c>
       <c r="AS19" s="13" t="n">
         <v>96.84</v>
+      </c>
+      <c r="AT19" s="13" t="n">
+        <v>97.05</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -2943,6 +2993,9 @@
       <c r="AS20" s="13" t="n">
         <v>7137.9</v>
       </c>
+      <c r="AT20" s="13" t="n">
+        <v>7165.08</v>
+      </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -3038,6 +3091,7 @@
       <c r="AQ21" s="13" t="n"/>
       <c r="AR21" s="13" t="n"/>
       <c r="AS21" s="13" t="n"/>
+      <c r="AT21" s="13" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -3172,6 +3226,9 @@
       </c>
       <c r="AS22" s="13" t="n">
         <v>46.82</v>
+      </c>
+      <c r="AT22" s="13" t="n">
+        <v>43.07</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1">
@@ -3262,6 +3319,9 @@
       <c r="AS23" s="13" t="n">
         <v>77880.09</v>
       </c>
+      <c r="AT23" s="13" t="n">
+        <v>77099.42999999999</v>
+      </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="3" t="n">
@@ -3357,6 +3417,7 @@
       <c r="AQ24" s="13" t="n"/>
       <c r="AR24" s="13" t="n"/>
       <c r="AS24" s="13" t="n"/>
+      <c r="AT24" s="13" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -3493,6 +3554,9 @@
       </c>
       <c r="AS25" s="13" t="n">
         <v>77</v>
+      </c>
+      <c r="AT25" s="13" t="n">
+        <v>50.17</v>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="1">
@@ -3581,6 +3645,9 @@
         <v>24702.24</v>
       </c>
       <c r="AS26" s="13" t="inlineStr"/>
+      <c r="AT26" s="13" t="n">
+        <v>24128.98</v>
+      </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -3676,6 +3743,7 @@
       <c r="AQ27" s="13" t="n"/>
       <c r="AR27" s="13" t="n"/>
       <c r="AS27" s="13" t="n"/>
+      <c r="AT27" s="13" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -3812,6 +3880,9 @@
       </c>
       <c r="AS28" s="13" t="n">
         <v>87.67</v>
+      </c>
+      <c r="AT28" s="13" t="n">
+        <v>87.04000000000001</v>
       </c>
     </row>
     <row r="29" ht="14.25" customHeight="1">
@@ -3902,6 +3973,9 @@
       <c r="AS29" s="13" t="n">
         <v>59114.07</v>
       </c>
+      <c r="AT29" s="13" t="n">
+        <v>60469.86</v>
+      </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="3" t="n">
@@ -3997,6 +4071,7 @@
       <c r="AQ30" s="13" t="n"/>
       <c r="AR30" s="13" t="n"/>
       <c r="AS30" s="13" t="n"/>
+      <c r="AT30" s="13" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -4133,6 +4208,9 @@
       </c>
       <c r="AS31" s="13" t="n">
         <v>52.9</v>
+      </c>
+      <c r="AT31" s="13" t="n">
+        <v>53.32</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -4223,6 +4301,9 @@
       <c r="AS32" s="13" t="n">
         <v>5783.37</v>
       </c>
+      <c r="AT32" s="13" t="n">
+        <v>5766.97</v>
+      </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
       <c r="A33" s="3" t="n">
@@ -4318,6 +4399,7 @@
       <c r="AQ33" s="13" t="n"/>
       <c r="AR33" s="13" t="n"/>
       <c r="AS33" s="13" t="n"/>
+      <c r="AT33" s="13" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -4454,6 +4536,9 @@
       </c>
       <c r="AS34" s="13" t="n">
         <v>3.83</v>
+      </c>
+      <c r="AT34" s="13" t="n">
+        <v>4.77</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -4544,6 +4629,9 @@
       <c r="AS35" s="13" t="n">
         <v>33566.19</v>
       </c>
+      <c r="AT35" s="13" t="n">
+        <v>34421.37</v>
+      </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="3" t="n">
@@ -4639,6 +4727,7 @@
       <c r="AQ36" s="13" t="n"/>
       <c r="AR36" s="13" t="n"/>
       <c r="AS36" s="13" t="n"/>
+      <c r="AT36" s="13" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -4775,6 +4864,9 @@
       </c>
       <c r="AS37" s="13" t="n">
         <v>57.78</v>
+      </c>
+      <c r="AT37" s="13" t="n">
+        <v>54.58</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -4865,6 +4957,9 @@
       <c r="AS38" s="13" t="n">
         <v>4006.23</v>
       </c>
+      <c r="AT38" s="13" t="n">
+        <v>3880.56</v>
+      </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
       <c r="A39" s="3" t="n">
@@ -4960,6 +5055,7 @@
       <c r="AQ39" s="13" t="n"/>
       <c r="AR39" s="13" t="n"/>
       <c r="AS39" s="13" t="n"/>
+      <c r="AT39" s="13" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -5096,6 +5192,9 @@
       </c>
       <c r="AS40" s="13" t="n">
         <v>59.44</v>
+      </c>
+      <c r="AT40" s="13" t="n">
+        <v>56.5</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -5186,6 +5285,9 @@
       <c r="AS41" s="13" t="n">
         <v>3739.56</v>
       </c>
+      <c r="AT41" s="13" t="n">
+        <v>3646.36</v>
+      </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
       <c r="A42" s="3" t="n">
@@ -5281,6 +5383,7 @@
       <c r="AQ42" s="13" t="n"/>
       <c r="AR42" s="13" t="n"/>
       <c r="AS42" s="13" t="n"/>
+      <c r="AT42" s="13" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -5417,6 +5520,9 @@
       </c>
       <c r="AS43" s="13" t="n">
         <v>8.449999999999999</v>
+      </c>
+      <c r="AT43" s="13" t="n">
+        <v>9.56</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -5507,6 +5613,9 @@
       <c r="AS44" s="13" t="n">
         <v>6662.32</v>
       </c>
+      <c r="AT44" s="13" t="n">
+        <v>6626.55</v>
+      </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
       <c r="A45" s="3" t="n">
@@ -5602,6 +5711,7 @@
       <c r="AQ45" s="13" t="n"/>
       <c r="AR45" s="13" t="n"/>
       <c r="AS45" s="13" t="n"/>
+      <c r="AT45" s="13" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -5738,6 +5848,9 @@
       </c>
       <c r="AS46" s="13" t="n">
         <v>12.35</v>
+      </c>
+      <c r="AT46" s="13" t="n">
+        <v>12.46</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -5828,6 +5941,9 @@
       <c r="AS47" s="13" t="n">
         <v>7931.04</v>
       </c>
+      <c r="AT47" s="13" t="n">
+        <v>7877.83</v>
+      </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
       <c r="A48" s="3" t="n">
@@ -5923,6 +6039,7 @@
       <c r="AQ48" s="13" t="n"/>
       <c r="AR48" s="13" t="n"/>
       <c r="AS48" s="13" t="n"/>
+      <c r="AT48" s="13" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -6059,6 +6176,9 @@
       </c>
       <c r="AS49" s="13" t="n">
         <v>6.81</v>
+      </c>
+      <c r="AT49" s="13" t="n">
+        <v>7.42</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -6149,6 +6269,9 @@
       <c r="AS50" s="13" t="n">
         <v>11652.13</v>
       </c>
+      <c r="AT50" s="13" t="n">
+        <v>11568.45</v>
+      </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
       <c r="A51" s="3" t="n">
@@ -6244,6 +6367,7 @@
       <c r="AQ51" s="13" t="n"/>
       <c r="AR51" s="13" t="n"/>
       <c r="AS51" s="13" t="n"/>
+      <c r="AT51" s="13" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -6380,6 +6504,9 @@
       </c>
       <c r="AS52" s="13" t="n">
         <v>22.38</v>
+      </c>
+      <c r="AT52" s="13" t="n">
+        <v>21.97</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -6470,6 +6597,9 @@
       <c r="AS53" s="13" t="n">
         <v>12200.71</v>
       </c>
+      <c r="AT53" s="13" t="n">
+        <v>12206.39</v>
+      </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
       <c r="A54" s="3" t="n">
@@ -6565,6 +6695,7 @@
       <c r="AQ54" s="13" t="n"/>
       <c r="AR54" s="13" t="n"/>
       <c r="AS54" s="13" t="n"/>
+      <c r="AT54" s="13" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -6701,6 +6832,9 @@
       </c>
       <c r="AS55" s="13" t="n">
         <v>11.38</v>
+      </c>
+      <c r="AT55" s="13" t="n">
+        <v>14.98</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -6791,6 +6925,9 @@
       <c r="AS56" s="13" t="n">
         <v>7784.09</v>
       </c>
+      <c r="AT56" s="13" t="n">
+        <v>7640.52</v>
+      </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
       <c r="A57" s="3" t="n">
@@ -6886,6 +7023,7 @@
       <c r="AQ57" s="13" t="n"/>
       <c r="AR57" s="13" t="n"/>
       <c r="AS57" s="13" t="n"/>
+      <c r="AT57" s="13" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -7022,6 +7160,9 @@
       </c>
       <c r="AS58" s="13" t="n">
         <v>18.02</v>
+      </c>
+      <c r="AT58" s="13" t="n">
+        <v>19.03</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -7112,6 +7253,9 @@
       <c r="AS59" s="13" t="n">
         <v>14208.87</v>
       </c>
+      <c r="AT59" s="13" t="n">
+        <v>14049.18</v>
+      </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
       <c r="A60" s="3" t="n">
@@ -7207,6 +7351,7 @@
       <c r="AQ60" s="13" t="n"/>
       <c r="AR60" s="13" t="n"/>
       <c r="AS60" s="13" t="n"/>
+      <c r="AT60" s="13" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -7343,6 +7488,9 @@
       </c>
       <c r="AS61" s="13" t="n">
         <v>66.11</v>
+      </c>
+      <c r="AT61" s="13" t="n">
+        <v>64.86</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -7433,6 +7581,9 @@
       <c r="AS62" s="13" t="n">
         <v>15569.82</v>
       </c>
+      <c r="AT62" s="13" t="n">
+        <v>15569.82</v>
+      </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
       <c r="A63" s="3" t="n">
@@ -7528,6 +7679,7 @@
       <c r="AQ63" s="13" t="n"/>
       <c r="AR63" s="13" t="n"/>
       <c r="AS63" s="13" t="n"/>
+      <c r="AT63" s="13" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -7664,6 +7816,9 @@
       </c>
       <c r="AS64" s="13" t="n">
         <v>7.65</v>
+      </c>
+      <c r="AT64" s="13" t="n">
+        <v>5.95</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -7754,6 +7909,9 @@
       <c r="AS65" s="13" t="n">
         <v>7776.03</v>
       </c>
+      <c r="AT65" s="13" t="n">
+        <v>7776.03</v>
+      </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
       <c r="A66" s="3" t="n">
@@ -7849,6 +8007,7 @@
       <c r="AQ66" s="13" t="n"/>
       <c r="AR66" s="13" t="n"/>
       <c r="AS66" s="13" t="n"/>
+      <c r="AT66" s="13" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -7985,6 +8144,9 @@
       </c>
       <c r="AS67" s="13" t="n">
         <v>4.29</v>
+      </c>
+      <c r="AT67" s="13" t="n">
+        <v>4.31</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -8075,6 +8237,9 @@
       <c r="AS68" s="13" t="n">
         <v>9022.049999999999</v>
       </c>
+      <c r="AT68" s="13" t="n">
+        <v>8970.6</v>
+      </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
       <c r="A69" s="3" t="n">
@@ -8170,6 +8335,7 @@
       <c r="AQ69" s="13" t="n"/>
       <c r="AR69" s="13" t="n"/>
       <c r="AS69" s="13" t="n"/>
+      <c r="AT69" s="13" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -8306,6 +8472,9 @@
       </c>
       <c r="AS70" s="13" t="n">
         <v>23.49</v>
+      </c>
+      <c r="AT70" s="13" t="n">
+        <v>22.27</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -8396,6 +8565,9 @@
       <c r="AS71" s="13" t="n">
         <v>2511.45</v>
       </c>
+      <c r="AT71" s="13" t="n">
+        <v>2498.12</v>
+      </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
       <c r="A72" s="3" t="n">
@@ -8491,6 +8663,7 @@
       <c r="AQ72" s="13" t="n"/>
       <c r="AR72" s="13" t="n"/>
       <c r="AS72" s="13" t="n"/>
+      <c r="AT72" s="13" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -8627,6 +8800,9 @@
       </c>
       <c r="AS73" s="13" t="n">
         <v>34.62</v>
+      </c>
+      <c r="AT73" s="13" t="n">
+        <v>32.66</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -8717,6 +8893,9 @@
       <c r="AS74" s="13" t="n">
         <v>4862.12</v>
       </c>
+      <c r="AT74" s="13" t="n">
+        <v>4932.77</v>
+      </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
       <c r="A75" s="3" t="n">
@@ -8812,6 +8991,7 @@
       <c r="AQ75" s="13" t="n"/>
       <c r="AR75" s="13" t="n"/>
       <c r="AS75" s="13" t="n"/>
+      <c r="AT75" s="13" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -8948,6 +9128,9 @@
       </c>
       <c r="AS76" s="13" t="n">
         <v>17.66</v>
+      </c>
+      <c r="AT76" s="13" t="n">
+        <v>16.33</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -9038,6 +9221,9 @@
       <c r="AS77" s="13" t="n">
         <v>8606.049999999999</v>
       </c>
+      <c r="AT77" s="13" t="n">
+        <v>8545.09</v>
+      </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
       <c r="A78" s="3" t="n">
@@ -9133,6 +9319,7 @@
       <c r="AQ78" s="13" t="n"/>
       <c r="AR78" s="13" t="n"/>
       <c r="AS78" s="13" t="n"/>
+      <c r="AT78" s="13" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -9269,6 +9456,9 @@
       </c>
       <c r="AS79" s="13" t="n">
         <v>9.98</v>
+      </c>
+      <c r="AT79" s="13" t="n">
+        <v>9.630000000000001</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -9359,6 +9549,9 @@
       <c r="AS80" s="13" t="n">
         <v>1283.89</v>
       </c>
+      <c r="AT80" s="13" t="n">
+        <v>1275.33</v>
+      </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
       <c r="A81" s="3" t="n">
@@ -9454,6 +9647,7 @@
       <c r="AQ81" s="13" t="n"/>
       <c r="AR81" s="13" t="n"/>
       <c r="AS81" s="13" t="n"/>
+      <c r="AT81" s="13" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -9590,6 +9784,9 @@
       </c>
       <c r="AS82" s="13" t="n">
         <v>10.59</v>
+      </c>
+      <c r="AT82" s="13" t="n">
+        <v>13.22</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -9680,6 +9877,9 @@
       <c r="AS83" s="13" t="n">
         <v>15515.64</v>
       </c>
+      <c r="AT83" s="13" t="n">
+        <v>15803.31</v>
+      </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
       <c r="A84" s="3" t="n">
@@ -9775,6 +9975,7 @@
       <c r="AQ84" s="13" t="n"/>
       <c r="AR84" s="13" t="n"/>
       <c r="AS84" s="13" t="n"/>
+      <c r="AT84" s="13" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -9911,6 +10112,9 @@
       </c>
       <c r="AS85" s="13" t="n">
         <v>70.63</v>
+      </c>
+      <c r="AT85" s="13" t="n">
+        <v>69.94</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -10001,6 +10205,9 @@
       <c r="AS86" s="13" t="n">
         <v>3155.78</v>
       </c>
+      <c r="AT86" s="13" t="n">
+        <v>3168.41</v>
+      </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
       <c r="A87" s="3" t="n">
@@ -10096,6 +10303,7 @@
       <c r="AQ87" s="13" t="n"/>
       <c r="AR87" s="13" t="n"/>
       <c r="AS87" s="13" t="n"/>
+      <c r="AT87" s="13" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -10232,6 +10440,9 @@
       </c>
       <c r="AS88" s="13" t="n">
         <v>74.06</v>
+      </c>
+      <c r="AT88" s="13" t="n">
+        <v>73.77</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -10322,6 +10533,9 @@
       <c r="AS89" s="13" t="n">
         <v>3218.21</v>
       </c>
+      <c r="AT89" s="13" t="n">
+        <v>3164.38</v>
+      </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
       <c r="A90" s="3" t="n">
@@ -10417,6 +10631,7 @@
       <c r="AQ90" s="13" t="n"/>
       <c r="AR90" s="13" t="n"/>
       <c r="AS90" s="13" t="n"/>
+      <c r="AT90" s="13" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -10553,6 +10768,9 @@
       </c>
       <c r="AS91" s="13" t="n">
         <v>60.49</v>
+      </c>
+      <c r="AT91" s="13" t="n">
+        <v>59.31</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -10643,6 +10861,9 @@
       <c r="AS92" s="13" t="n">
         <v>3260.88</v>
       </c>
+      <c r="AT92" s="13" t="n">
+        <v>3357.7</v>
+      </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
       <c r="A93" s="3" t="n">
@@ -10738,6 +10959,7 @@
       <c r="AQ93" s="13" t="n"/>
       <c r="AR93" s="13" t="n"/>
       <c r="AS93" s="13" t="n"/>
+      <c r="AT93" s="13" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -10874,6 +11096,9 @@
       </c>
       <c r="AS94" s="13" t="n">
         <v>46.76</v>
+      </c>
+      <c r="AT94" s="13" t="n">
+        <v>42.7</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -10964,6 +11189,9 @@
       <c r="AS95" s="13" t="n">
         <v>1889.03</v>
       </c>
+      <c r="AT95" s="13" t="n">
+        <v>1881.97</v>
+      </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
       <c r="A96" s="3" t="n">
@@ -11059,6 +11287,7 @@
       <c r="AQ96" s="13" t="n"/>
       <c r="AR96" s="13" t="n"/>
       <c r="AS96" s="13" t="n"/>
+      <c r="AT96" s="13" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -11195,6 +11424,9 @@
       </c>
       <c r="AS97" s="13" t="n">
         <v>25.27</v>
+      </c>
+      <c r="AT97" s="13" t="n">
+        <v>26.24</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -11285,6 +11517,9 @@
       <c r="AS98" s="13" t="n">
         <v>9774.690000000001</v>
       </c>
+      <c r="AT98" s="13" t="n">
+        <v>9774.690000000001</v>
+      </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
       <c r="A99" s="3" t="n">
@@ -11380,6 +11615,7 @@
       <c r="AQ99" s="13" t="n"/>
       <c r="AR99" s="13" t="n"/>
       <c r="AS99" s="13" t="n"/>
+      <c r="AT99" s="13" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -11516,6 +11752,9 @@
       </c>
       <c r="AS100" s="13" t="n">
         <v>90.58</v>
+      </c>
+      <c r="AT100" s="13" t="n">
+        <v>91.48999999999999</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -11606,6 +11845,9 @@
       <c r="AS101" s="13" t="n">
         <v>10434.95</v>
       </c>
+      <c r="AT101" s="13" t="n">
+        <v>11044.82</v>
+      </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
       <c r="A102" s="3" t="n">
@@ -11701,6 +11943,7 @@
       <c r="AQ102" s="13" t="n"/>
       <c r="AR102" s="13" t="n"/>
       <c r="AS102" s="13" t="n"/>
+      <c r="AT102" s="13" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -11837,6 +12080,9 @@
       </c>
       <c r="AS103" s="13" t="n">
         <v>80.34</v>
+      </c>
+      <c r="AT103" s="13" t="n">
+        <v>77.61</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -11927,6 +12173,9 @@
       <c r="AS104" s="13" t="n">
         <v>14577.16</v>
       </c>
+      <c r="AT104" s="13" t="n">
+        <v>14214.98</v>
+      </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
       <c r="A105" s="3" t="n">
@@ -12022,6 +12271,7 @@
       <c r="AQ105" s="13" t="n"/>
       <c r="AR105" s="13" t="n"/>
       <c r="AS105" s="13" t="n"/>
+      <c r="AT105" s="13" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -12158,6 +12408,9 @@
       </c>
       <c r="AS106" s="13" t="n">
         <v>22.43</v>
+      </c>
+      <c r="AT106" s="13" t="n">
+        <v>21.85</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -12248,6 +12501,9 @@
       <c r="AS107" s="13" t="n">
         <v>2153.1</v>
       </c>
+      <c r="AT107" s="13" t="n">
+        <v>2096.41</v>
+      </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
       <c r="A108" s="3" t="n">
@@ -12343,6 +12599,7 @@
       <c r="AQ108" s="13" t="n"/>
       <c r="AR108" s="13" t="n"/>
       <c r="AS108" s="13" t="n"/>
+      <c r="AT108" s="13" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -12479,6 +12736,9 @@
       </c>
       <c r="AS109" s="13" t="n">
         <v>12.59</v>
+      </c>
+      <c r="AT109" s="13" t="n">
+        <v>10.02</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -12569,6 +12829,9 @@
       <c r="AS110" s="13" t="n">
         <v>749.27</v>
       </c>
+      <c r="AT110" s="13" t="n">
+        <v>742.5599999999999</v>
+      </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
       <c r="A111" s="3" t="n">
@@ -12664,6 +12927,7 @@
       <c r="AQ111" s="13" t="n"/>
       <c r="AR111" s="13" t="n"/>
       <c r="AS111" s="13" t="n"/>
+      <c r="AT111" s="13" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -12800,6 +13064,9 @@
       </c>
       <c r="AS112" s="13" t="n">
         <v>79.61</v>
+      </c>
+      <c r="AT112" s="13" t="n">
+        <v>77.73999999999999</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -12890,6 +13157,9 @@
       <c r="AS113" s="13" t="n">
         <v>3393.05</v>
       </c>
+      <c r="AT113" s="13" t="n">
+        <v>3392.2</v>
+      </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
       <c r="A114" s="3" t="n">
@@ -12985,6 +13255,7 @@
       <c r="AQ114" s="13" t="n"/>
       <c r="AR114" s="13" t="n"/>
       <c r="AS114" s="13" t="n"/>
+      <c r="AT114" s="13" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -13121,6 +13392,9 @@
       </c>
       <c r="AS115" s="13" t="n">
         <v>30.88</v>
+      </c>
+      <c r="AT115" s="13" t="n">
+        <v>27.7</v>
       </c>
     </row>
     <row r="116">
@@ -13195,6 +13469,9 @@
       </c>
       <c r="AS116" s="13" t="n">
         <v>4070.85</v>
+      </c>
+      <c r="AT116" s="13" t="n">
+        <v>3966.04</v>
       </c>
     </row>
     <row r="117">
@@ -13246,6 +13523,7 @@
       <c r="AQ117" s="13" t="n"/>
       <c r="AR117" s="13" t="n"/>
       <c r="AS117" s="13" t="n"/>
+      <c r="AT117" s="13" t="n"/>
     </row>
     <row r="118">
       <c r="P118" s="13" t="n">
@@ -13338,6 +13616,9 @@
       <c r="AS118" s="13" t="n">
         <v>29.02</v>
       </c>
+      <c r="AT118" s="13" t="n">
+        <v>29.02</v>
+      </c>
     </row>
     <row r="119">
       <c r="Y119" s="13" t="n">
@@ -13402,6 +13683,9 @@
       </c>
       <c r="AS119" s="13" t="n">
         <v>2792.96</v>
+      </c>
+      <c r="AT119" s="13" t="n">
+        <v>2758.42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-04-30 06:18:40]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT119"/>
+  <dimension ref="A1:AU119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="15"/>
@@ -563,6 +563,7 @@
     <col width="15" customWidth="1" min="44" max="44"/>
     <col width="15" customWidth="1" min="45" max="45"/>
     <col width="15" customWidth="1" min="46" max="46"/>
+    <col width="15" customWidth="1" min="47" max="47"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -796,6 +797,11 @@
           <t>2026/04/27</t>
         </is>
       </c>
+      <c r="AU1" s="13" t="inlineStr">
+        <is>
+          <t>2026/04/30</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1028,6 +1034,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="AU2" s="14" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1168,6 +1179,9 @@
       <c r="AT3" s="13" t="n">
         <v>69.06</v>
       </c>
+      <c r="AU3" s="13" t="n">
+        <v>69.28</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1307,6 +1321,9 @@
       </c>
       <c r="AT4" s="13" t="n">
         <v>4083.03</v>
+      </c>
+      <c r="AU4" s="13" t="n">
+        <v>4113.74</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1356,6 +1373,7 @@
       <c r="AR5" s="13" t="n"/>
       <c r="AS5" s="13" t="n"/>
       <c r="AT5" s="13" t="n"/>
+      <c r="AU5" s="13" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1452,6 +1470,7 @@
       <c r="AR6" s="13" t="n"/>
       <c r="AS6" s="13" t="n"/>
       <c r="AT6" s="13" t="n"/>
+      <c r="AU6" s="13" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1591,6 +1610,9 @@
       </c>
       <c r="AT7" s="13" t="n">
         <v>67.44</v>
+      </c>
+      <c r="AU7" s="13" t="n">
+        <v>67.94</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -1684,6 +1706,9 @@
       <c r="AT8" s="13" t="n">
         <v>5960.28</v>
       </c>
+      <c r="AU8" s="13" t="n">
+        <v>6017.67</v>
+      </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -1780,6 +1805,7 @@
       <c r="AR9" s="13" t="n"/>
       <c r="AS9" s="13" t="n"/>
       <c r="AT9" s="13" t="n"/>
+      <c r="AU9" s="13" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -1919,6 +1945,9 @@
       </c>
       <c r="AT10" s="13" t="n">
         <v>59.07</v>
+      </c>
+      <c r="AU10" s="13" t="n">
+        <v>59.95</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2012,6 +2041,9 @@
       <c r="AT11" s="13" t="n">
         <v>4765.91</v>
       </c>
+      <c r="AU11" s="13" t="n">
+        <v>4806.97</v>
+      </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -2108,6 +2140,7 @@
       <c r="AR12" s="13" t="n"/>
       <c r="AS12" s="13" t="n"/>
       <c r="AT12" s="13" t="n"/>
+      <c r="AU12" s="13" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2247,6 +2280,9 @@
       </c>
       <c r="AT13" s="13" t="n">
         <v>66.51000000000001</v>
+      </c>
+      <c r="AU13" s="13" t="n">
+        <v>67.03</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -2340,6 +2376,9 @@
       <c r="AT14" s="13" t="n">
         <v>8296.5</v>
       </c>
+      <c r="AU14" s="13" t="n">
+        <v>8346.370000000001</v>
+      </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -2436,6 +2475,7 @@
       <c r="AR15" s="13" t="n"/>
       <c r="AS15" s="13" t="n"/>
       <c r="AT15" s="13" t="n"/>
+      <c r="AU15" s="13" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -2575,6 +2615,9 @@
       </c>
       <c r="AT16" s="13" t="n">
         <v>39.94</v>
+      </c>
+      <c r="AU16" s="13" t="n">
+        <v>40.39</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -2668,6 +2711,9 @@
       <c r="AT17" s="13" t="n">
         <v>2630.77</v>
       </c>
+      <c r="AU17" s="13" t="n">
+        <v>2670.8</v>
+      </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="3" t="n">
@@ -2764,6 +2810,7 @@
       <c r="AR18" s="13" t="n"/>
       <c r="AS18" s="13" t="n"/>
       <c r="AT18" s="13" t="n"/>
+      <c r="AU18" s="13" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -2903,6 +2950,9 @@
       </c>
       <c r="AT19" s="13" t="n">
         <v>97.05</v>
+      </c>
+      <c r="AU19" s="13" t="n">
+        <v>94.06999999999999</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -2996,6 +3046,9 @@
       <c r="AT20" s="13" t="n">
         <v>7165.08</v>
       </c>
+      <c r="AU20" s="13" t="n">
+        <v>7135.95</v>
+      </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -3092,6 +3145,7 @@
       <c r="AR21" s="13" t="n"/>
       <c r="AS21" s="13" t="n"/>
       <c r="AT21" s="13" t="n"/>
+      <c r="AU21" s="13" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -3229,6 +3283,9 @@
       </c>
       <c r="AT22" s="13" t="n">
         <v>43.07</v>
+      </c>
+      <c r="AU22" s="13" t="n">
+        <v>43.74</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1">
@@ -3322,6 +3379,9 @@
       <c r="AT23" s="13" t="n">
         <v>77099.42999999999</v>
       </c>
+      <c r="AU23" s="13" t="n">
+        <v>76355.50999999999</v>
+      </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="3" t="n">
@@ -3418,6 +3478,7 @@
       <c r="AR24" s="13" t="n"/>
       <c r="AS24" s="13" t="n"/>
       <c r="AT24" s="13" t="n"/>
+      <c r="AU24" s="13" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -3557,6 +3618,9 @@
       </c>
       <c r="AT25" s="13" t="n">
         <v>50.17</v>
+      </c>
+      <c r="AU25" s="13" t="n">
+        <v>75.43000000000001</v>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="1">
@@ -3648,6 +3712,7 @@
       <c r="AT26" s="13" t="n">
         <v>24128.98</v>
       </c>
+      <c r="AU26" s="13" t="inlineStr"/>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -3744,6 +3809,7 @@
       <c r="AR27" s="13" t="n"/>
       <c r="AS27" s="13" t="n"/>
       <c r="AT27" s="13" t="n"/>
+      <c r="AU27" s="13" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -3883,6 +3949,9 @@
       </c>
       <c r="AT28" s="13" t="n">
         <v>87.04000000000001</v>
+      </c>
+      <c r="AU28" s="13" t="n">
+        <v>87.3</v>
       </c>
     </row>
     <row r="29" ht="14.25" customHeight="1">
@@ -3976,6 +4045,9 @@
       <c r="AT29" s="13" t="n">
         <v>60469.86</v>
       </c>
+      <c r="AU29" s="13" t="n">
+        <v>59132.74</v>
+      </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="3" t="n">
@@ -4072,6 +4144,7 @@
       <c r="AR30" s="13" t="n"/>
       <c r="AS30" s="13" t="n"/>
       <c r="AT30" s="13" t="n"/>
+      <c r="AU30" s="13" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -4211,6 +4284,9 @@
       </c>
       <c r="AT31" s="13" t="n">
         <v>53.32</v>
+      </c>
+      <c r="AU31" s="13" t="n">
+        <v>51.89</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -4304,6 +4380,9 @@
       <c r="AT32" s="13" t="n">
         <v>5766.97</v>
       </c>
+      <c r="AU32" s="13" t="n">
+        <v>5858.45</v>
+      </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
       <c r="A33" s="3" t="n">
@@ -4400,6 +4479,7 @@
       <c r="AR33" s="13" t="n"/>
       <c r="AS33" s="13" t="n"/>
       <c r="AT33" s="13" t="n"/>
+      <c r="AU33" s="13" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -4539,6 +4619,9 @@
       </c>
       <c r="AT34" s="13" t="n">
         <v>4.77</v>
+      </c>
+      <c r="AU34" s="13" t="n">
+        <v>5.79</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -4632,6 +4715,9 @@
       <c r="AT35" s="13" t="n">
         <v>34421.37</v>
       </c>
+      <c r="AU35" s="13" t="n">
+        <v>35006.18</v>
+      </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="3" t="n">
@@ -4728,6 +4814,7 @@
       <c r="AR36" s="13" t="n"/>
       <c r="AS36" s="13" t="n"/>
       <c r="AT36" s="13" t="n"/>
+      <c r="AU36" s="13" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -4867,6 +4954,9 @@
       </c>
       <c r="AT37" s="13" t="n">
         <v>54.58</v>
+      </c>
+      <c r="AU37" s="13" t="n">
+        <v>57.09</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -4960,6 +5050,9 @@
       <c r="AT38" s="13" t="n">
         <v>3880.56</v>
       </c>
+      <c r="AU38" s="13" t="n">
+        <v>3910.85</v>
+      </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
       <c r="A39" s="3" t="n">
@@ -5056,6 +5149,7 @@
       <c r="AR39" s="13" t="n"/>
       <c r="AS39" s="13" t="n"/>
       <c r="AT39" s="13" t="n"/>
+      <c r="AU39" s="13" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -5195,6 +5289,9 @@
       </c>
       <c r="AT40" s="13" t="n">
         <v>56.5</v>
+      </c>
+      <c r="AU40" s="13" t="n">
+        <v>58.05</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -5288,6 +5385,9 @@
       <c r="AT41" s="13" t="n">
         <v>3646.36</v>
       </c>
+      <c r="AU41" s="13" t="n">
+        <v>3680</v>
+      </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
       <c r="A42" s="3" t="n">
@@ -5384,6 +5484,7 @@
       <c r="AR42" s="13" t="n"/>
       <c r="AS42" s="13" t="n"/>
       <c r="AT42" s="13" t="n"/>
+      <c r="AU42" s="13" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -5523,6 +5624,9 @@
       </c>
       <c r="AT43" s="13" t="n">
         <v>9.56</v>
+      </c>
+      <c r="AU43" s="13" t="n">
+        <v>10.16</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -5616,6 +5720,9 @@
       <c r="AT44" s="13" t="n">
         <v>6626.55</v>
       </c>
+      <c r="AU44" s="13" t="n">
+        <v>6683.55</v>
+      </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
       <c r="A45" s="3" t="n">
@@ -5712,6 +5819,7 @@
       <c r="AR45" s="13" t="n"/>
       <c r="AS45" s="13" t="n"/>
       <c r="AT45" s="13" t="n"/>
+      <c r="AU45" s="13" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -5851,6 +5959,9 @@
       </c>
       <c r="AT46" s="13" t="n">
         <v>12.46</v>
+      </c>
+      <c r="AU46" s="13" t="n">
+        <v>33.23</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -5944,6 +6055,9 @@
       <c r="AT47" s="13" t="n">
         <v>7877.83</v>
       </c>
+      <c r="AU47" s="13" t="n">
+        <v>8011.84</v>
+      </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
       <c r="A48" s="3" t="n">
@@ -6040,6 +6154,7 @@
       <c r="AR48" s="13" t="n"/>
       <c r="AS48" s="13" t="n"/>
       <c r="AT48" s="13" t="n"/>
+      <c r="AU48" s="13" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -6179,6 +6294,9 @@
       </c>
       <c r="AT49" s="13" t="n">
         <v>7.42</v>
+      </c>
+      <c r="AU49" s="13" t="n">
+        <v>8.619999999999999</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -6272,6 +6390,9 @@
       <c r="AT50" s="13" t="n">
         <v>11568.45</v>
       </c>
+      <c r="AU50" s="13" t="n">
+        <v>11574.14</v>
+      </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
       <c r="A51" s="3" t="n">
@@ -6368,6 +6489,7 @@
       <c r="AR51" s="13" t="n"/>
       <c r="AS51" s="13" t="n"/>
       <c r="AT51" s="13" t="n"/>
+      <c r="AU51" s="13" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -6507,6 +6629,9 @@
       </c>
       <c r="AT52" s="13" t="n">
         <v>21.97</v>
+      </c>
+      <c r="AU52" s="13" t="n">
+        <v>43.02</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -6600,6 +6725,9 @@
       <c r="AT53" s="13" t="n">
         <v>12206.39</v>
       </c>
+      <c r="AU53" s="13" t="n">
+        <v>12151.29</v>
+      </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
       <c r="A54" s="3" t="n">
@@ -6696,6 +6824,7 @@
       <c r="AR54" s="13" t="n"/>
       <c r="AS54" s="13" t="n"/>
       <c r="AT54" s="13" t="n"/>
+      <c r="AU54" s="13" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -6835,6 +6964,9 @@
       </c>
       <c r="AT55" s="13" t="n">
         <v>14.98</v>
+      </c>
+      <c r="AU55" s="13" t="n">
+        <v>13.3</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -6928,6 +7060,9 @@
       <c r="AT56" s="13" t="n">
         <v>7640.52</v>
       </c>
+      <c r="AU56" s="13" t="n">
+        <v>7648.91</v>
+      </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
       <c r="A57" s="3" t="n">
@@ -7024,6 +7159,7 @@
       <c r="AR57" s="13" t="n"/>
       <c r="AS57" s="13" t="n"/>
       <c r="AT57" s="13" t="n"/>
+      <c r="AU57" s="13" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -7163,6 +7299,9 @@
       </c>
       <c r="AT58" s="13" t="n">
         <v>19.03</v>
+      </c>
+      <c r="AU58" s="13" t="n">
+        <v>18.94</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -7256,6 +7395,9 @@
       <c r="AT59" s="13" t="n">
         <v>14049.18</v>
       </c>
+      <c r="AU59" s="13" t="n">
+        <v>14367.98</v>
+      </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
       <c r="A60" s="3" t="n">
@@ -7352,6 +7494,7 @@
       <c r="AR60" s="13" t="n"/>
       <c r="AS60" s="13" t="n"/>
       <c r="AT60" s="13" t="n"/>
+      <c r="AU60" s="13" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -7491,6 +7634,9 @@
       </c>
       <c r="AT61" s="13" t="n">
         <v>64.86</v>
+      </c>
+      <c r="AU61" s="13" t="n">
+        <v>62.21</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -7584,6 +7730,9 @@
       <c r="AT62" s="13" t="n">
         <v>15569.82</v>
       </c>
+      <c r="AU62" s="13" t="n">
+        <v>14687.84</v>
+      </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
       <c r="A63" s="3" t="n">
@@ -7680,6 +7829,7 @@
       <c r="AR63" s="13" t="n"/>
       <c r="AS63" s="13" t="n"/>
       <c r="AT63" s="13" t="n"/>
+      <c r="AU63" s="13" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -7819,6 +7969,9 @@
       </c>
       <c r="AT64" s="13" t="n">
         <v>5.95</v>
+      </c>
+      <c r="AU64" s="13" t="n">
+        <v>4.58</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -7912,6 +8065,9 @@
       <c r="AT65" s="13" t="n">
         <v>7776.03</v>
       </c>
+      <c r="AU65" s="13" t="n">
+        <v>8010.29</v>
+      </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
       <c r="A66" s="3" t="n">
@@ -8008,6 +8164,7 @@
       <c r="AR66" s="13" t="n"/>
       <c r="AS66" s="13" t="n"/>
       <c r="AT66" s="13" t="n"/>
+      <c r="AU66" s="13" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -8147,6 +8304,9 @@
       </c>
       <c r="AT67" s="13" t="n">
         <v>4.31</v>
+      </c>
+      <c r="AU67" s="13" t="n">
+        <v>2.11</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -8240,6 +8400,9 @@
       <c r="AT68" s="13" t="n">
         <v>8970.6</v>
       </c>
+      <c r="AU68" s="13" t="n">
+        <v>9067.51</v>
+      </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
       <c r="A69" s="3" t="n">
@@ -8336,6 +8499,7 @@
       <c r="AR69" s="13" t="n"/>
       <c r="AS69" s="13" t="n"/>
       <c r="AT69" s="13" t="n"/>
+      <c r="AU69" s="13" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -8475,6 +8639,9 @@
       </c>
       <c r="AT70" s="13" t="n">
         <v>22.27</v>
+      </c>
+      <c r="AU70" s="13" t="n">
+        <v>20.44</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -8568,6 +8735,9 @@
       <c r="AT71" s="13" t="n">
         <v>2498.12</v>
       </c>
+      <c r="AU71" s="13" t="n">
+        <v>2631.9</v>
+      </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
       <c r="A72" s="3" t="n">
@@ -8664,6 +8834,7 @@
       <c r="AR72" s="13" t="n"/>
       <c r="AS72" s="13" t="n"/>
       <c r="AT72" s="13" t="n"/>
+      <c r="AU72" s="13" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -8803,6 +8974,9 @@
       </c>
       <c r="AT73" s="13" t="n">
         <v>32.66</v>
+      </c>
+      <c r="AU73" s="13" t="n">
+        <v>32.77</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -8896,6 +9070,9 @@
       <c r="AT74" s="13" t="n">
         <v>4932.77</v>
       </c>
+      <c r="AU74" s="13" t="n">
+        <v>5075.31</v>
+      </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
       <c r="A75" s="3" t="n">
@@ -8992,6 +9169,7 @@
       <c r="AR75" s="13" t="n"/>
       <c r="AS75" s="13" t="n"/>
       <c r="AT75" s="13" t="n"/>
+      <c r="AU75" s="13" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -9131,6 +9309,9 @@
       </c>
       <c r="AT76" s="13" t="n">
         <v>16.33</v>
+      </c>
+      <c r="AU76" s="13" t="n">
+        <v>20.79</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -9224,6 +9405,9 @@
       <c r="AT77" s="13" t="n">
         <v>8545.09</v>
       </c>
+      <c r="AU77" s="13" t="n">
+        <v>8626.67</v>
+      </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
       <c r="A78" s="3" t="n">
@@ -9320,6 +9504,7 @@
       <c r="AR78" s="13" t="n"/>
       <c r="AS78" s="13" t="n"/>
       <c r="AT78" s="13" t="n"/>
+      <c r="AU78" s="13" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -9459,6 +9644,9 @@
       </c>
       <c r="AT79" s="13" t="n">
         <v>9.630000000000001</v>
+      </c>
+      <c r="AU79" s="13" t="n">
+        <v>10.19</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -9552,6 +9740,9 @@
       <c r="AT80" s="13" t="n">
         <v>1275.33</v>
       </c>
+      <c r="AU80" s="13" t="n">
+        <v>1307.49</v>
+      </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
       <c r="A81" s="3" t="n">
@@ -9648,6 +9839,7 @@
       <c r="AR81" s="13" t="n"/>
       <c r="AS81" s="13" t="n"/>
       <c r="AT81" s="13" t="n"/>
+      <c r="AU81" s="13" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -9787,6 +9979,9 @@
       </c>
       <c r="AT82" s="13" t="n">
         <v>13.22</v>
+      </c>
+      <c r="AU82" s="13" t="n">
+        <v>11.73</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -9880,6 +10075,9 @@
       <c r="AT83" s="13" t="n">
         <v>15803.31</v>
       </c>
+      <c r="AU83" s="13" t="n">
+        <v>15684.77</v>
+      </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
       <c r="A84" s="3" t="n">
@@ -9976,6 +10174,7 @@
       <c r="AR84" s="13" t="n"/>
       <c r="AS84" s="13" t="n"/>
       <c r="AT84" s="13" t="n"/>
+      <c r="AU84" s="13" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -10115,6 +10314,9 @@
       </c>
       <c r="AT85" s="13" t="n">
         <v>69.94</v>
+      </c>
+      <c r="AU85" s="13" t="n">
+        <v>68.40000000000001</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -10208,6 +10410,9 @@
       <c r="AT86" s="13" t="n">
         <v>3168.41</v>
       </c>
+      <c r="AU86" s="13" t="n">
+        <v>3221.02</v>
+      </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
       <c r="A87" s="3" t="n">
@@ -10304,6 +10509,7 @@
       <c r="AR87" s="13" t="n"/>
       <c r="AS87" s="13" t="n"/>
       <c r="AT87" s="13" t="n"/>
+      <c r="AU87" s="13" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -10443,6 +10649,9 @@
       </c>
       <c r="AT88" s="13" t="n">
         <v>73.77</v>
+      </c>
+      <c r="AU88" s="13" t="n">
+        <v>73.92</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -10536,6 +10745,9 @@
       <c r="AT89" s="13" t="n">
         <v>3164.38</v>
       </c>
+      <c r="AU89" s="13" t="n">
+        <v>3157.1</v>
+      </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
       <c r="A90" s="3" t="n">
@@ -10632,6 +10844,7 @@
       <c r="AR90" s="13" t="n"/>
       <c r="AS90" s="13" t="n"/>
       <c r="AT90" s="13" t="n"/>
+      <c r="AU90" s="13" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -10771,6 +10984,9 @@
       </c>
       <c r="AT91" s="13" t="n">
         <v>59.31</v>
+      </c>
+      <c r="AU91" s="13" t="n">
+        <v>62.23</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -10864,6 +11080,9 @@
       <c r="AT92" s="13" t="n">
         <v>3357.7</v>
       </c>
+      <c r="AU92" s="13" t="n">
+        <v>3461.45</v>
+      </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
       <c r="A93" s="3" t="n">
@@ -10960,6 +11179,7 @@
       <c r="AR93" s="13" t="n"/>
       <c r="AS93" s="13" t="n"/>
       <c r="AT93" s="13" t="n"/>
+      <c r="AU93" s="13" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -11099,6 +11319,9 @@
       </c>
       <c r="AT94" s="13" t="n">
         <v>42.7</v>
+      </c>
+      <c r="AU94" s="13" t="n">
+        <v>55.52</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -11192,6 +11415,9 @@
       <c r="AT95" s="13" t="n">
         <v>1881.97</v>
       </c>
+      <c r="AU95" s="13" t="n">
+        <v>1898.04</v>
+      </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
       <c r="A96" s="3" t="n">
@@ -11288,6 +11514,7 @@
       <c r="AR96" s="13" t="n"/>
       <c r="AS96" s="13" t="n"/>
       <c r="AT96" s="13" t="n"/>
+      <c r="AU96" s="13" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -11427,6 +11654,9 @@
       </c>
       <c r="AT97" s="13" t="n">
         <v>26.24</v>
+      </c>
+      <c r="AU97" s="13" t="n">
+        <v>26.59</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -11520,6 +11750,9 @@
       <c r="AT98" s="13" t="n">
         <v>9774.690000000001</v>
       </c>
+      <c r="AU98" s="13" t="n">
+        <v>9641.110000000001</v>
+      </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
       <c r="A99" s="3" t="n">
@@ -11616,6 +11849,7 @@
       <c r="AR99" s="13" t="n"/>
       <c r="AS99" s="13" t="n"/>
       <c r="AT99" s="13" t="n"/>
+      <c r="AU99" s="13" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -11755,6 +11989,9 @@
       </c>
       <c r="AT100" s="13" t="n">
         <v>91.48999999999999</v>
+      </c>
+      <c r="AU100" s="13" t="n">
+        <v>90.73</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -11848,6 +12085,9 @@
       <c r="AT101" s="13" t="n">
         <v>11044.82</v>
       </c>
+      <c r="AU101" s="13" t="n">
+        <v>11484.59</v>
+      </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
       <c r="A102" s="3" t="n">
@@ -11944,6 +12184,7 @@
       <c r="AR102" s="13" t="n"/>
       <c r="AS102" s="13" t="n"/>
       <c r="AT102" s="13" t="n"/>
+      <c r="AU102" s="13" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -12083,6 +12324,9 @@
       </c>
       <c r="AT103" s="13" t="n">
         <v>77.61</v>
+      </c>
+      <c r="AU103" s="13" t="n">
+        <v>71.40000000000001</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -12176,6 +12420,9 @@
       <c r="AT104" s="13" t="n">
         <v>14214.98</v>
       </c>
+      <c r="AU104" s="13" t="n">
+        <v>14295.66</v>
+      </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
       <c r="A105" s="3" t="n">
@@ -12272,6 +12519,7 @@
       <c r="AR105" s="13" t="n"/>
       <c r="AS105" s="13" t="n"/>
       <c r="AT105" s="13" t="n"/>
+      <c r="AU105" s="13" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -12411,6 +12659,9 @@
       </c>
       <c r="AT106" s="13" t="n">
         <v>21.85</v>
+      </c>
+      <c r="AU106" s="13" t="n">
+        <v>32.16</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -12504,6 +12755,9 @@
       <c r="AT107" s="13" t="n">
         <v>2096.41</v>
       </c>
+      <c r="AU107" s="13" t="n">
+        <v>2161.17</v>
+      </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
       <c r="A108" s="3" t="n">
@@ -12600,6 +12854,7 @@
       <c r="AR108" s="13" t="n"/>
       <c r="AS108" s="13" t="n"/>
       <c r="AT108" s="13" t="n"/>
+      <c r="AU108" s="13" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -12739,6 +12994,9 @@
       </c>
       <c r="AT109" s="13" t="n">
         <v>10.02</v>
+      </c>
+      <c r="AU109" s="13" t="n">
+        <v>11.97</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -12832,6 +13090,9 @@
       <c r="AT110" s="13" t="n">
         <v>742.5599999999999</v>
       </c>
+      <c r="AU110" s="13" t="n">
+        <v>756.7</v>
+      </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
       <c r="A111" s="3" t="n">
@@ -12928,6 +13189,7 @@
       <c r="AR111" s="13" t="n"/>
       <c r="AS111" s="13" t="n"/>
       <c r="AT111" s="13" t="n"/>
+      <c r="AU111" s="13" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -13067,6 +13329,9 @@
       </c>
       <c r="AT112" s="13" t="n">
         <v>77.73999999999999</v>
+      </c>
+      <c r="AU112" s="13" t="n">
+        <v>76.23999999999999</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -13160,6 +13425,9 @@
       <c r="AT113" s="13" t="n">
         <v>3392.2</v>
       </c>
+      <c r="AU113" s="13" t="n">
+        <v>3442.74</v>
+      </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
       <c r="A114" s="3" t="n">
@@ -13256,6 +13524,7 @@
       <c r="AR114" s="13" t="n"/>
       <c r="AS114" s="13" t="n"/>
       <c r="AT114" s="13" t="n"/>
+      <c r="AU114" s="13" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -13395,6 +13664,9 @@
       </c>
       <c r="AT115" s="13" t="n">
         <v>27.7</v>
+      </c>
+      <c r="AU115" s="13" t="n">
+        <v>25.98</v>
       </c>
     </row>
     <row r="116">
@@ -13472,6 +13744,9 @@
       </c>
       <c r="AT116" s="13" t="n">
         <v>3966.04</v>
+      </c>
+      <c r="AU116" s="13" t="n">
+        <v>3971.38</v>
       </c>
     </row>
     <row r="117">
@@ -13524,6 +13799,7 @@
       <c r="AR117" s="13" t="n"/>
       <c r="AS117" s="13" t="n"/>
       <c r="AT117" s="13" t="n"/>
+      <c r="AU117" s="13" t="n"/>
     </row>
     <row r="118">
       <c r="P118" s="13" t="n">
@@ -13619,6 +13895,9 @@
       <c r="AT118" s="13" t="n">
         <v>29.02</v>
       </c>
+      <c r="AU118" s="13" t="n">
+        <v>29.02</v>
+      </c>
     </row>
     <row r="119">
       <c r="Y119" s="13" t="n">
@@ -13686,6 +13965,9 @@
       </c>
       <c r="AT119" s="13" t="n">
         <v>2758.42</v>
+      </c>
+      <c r="AU119" s="13" t="n">
+        <v>2797.47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-05-04 06:28:26]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU119"/>
+  <dimension ref="A1:AV119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="15"/>
@@ -564,6 +564,7 @@
     <col width="15" customWidth="1" min="45" max="45"/>
     <col width="15" customWidth="1" min="46" max="46"/>
     <col width="15" customWidth="1" min="47" max="47"/>
+    <col width="15" customWidth="1" min="48" max="48"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -802,6 +803,11 @@
           <t>2026/04/30</t>
         </is>
       </c>
+      <c r="AV1" s="13" t="inlineStr">
+        <is>
+          <t>2026/05/04</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1039,6 +1045,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="AV2" s="14" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1182,6 +1193,9 @@
       <c r="AU3" s="13" t="n">
         <v>69.28</v>
       </c>
+      <c r="AV3" s="13" t="n">
+        <v>69.06</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1324,6 +1338,9 @@
       </c>
       <c r="AU4" s="13" t="n">
         <v>4113.74</v>
+      </c>
+      <c r="AV4" s="13" t="n">
+        <v>4112.16</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1374,6 +1391,7 @@
       <c r="AS5" s="13" t="n"/>
       <c r="AT5" s="13" t="n"/>
       <c r="AU5" s="13" t="n"/>
+      <c r="AV5" s="13" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1471,6 +1489,7 @@
       <c r="AS6" s="13" t="n"/>
       <c r="AT6" s="13" t="n"/>
       <c r="AU6" s="13" t="n"/>
+      <c r="AV6" s="13" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1613,6 +1632,9 @@
       </c>
       <c r="AU7" s="13" t="n">
         <v>67.94</v>
+      </c>
+      <c r="AV7" s="13" t="n">
+        <v>66.28</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -1709,6 +1731,9 @@
       <c r="AU8" s="13" t="n">
         <v>6017.67</v>
       </c>
+      <c r="AV8" s="13" t="n">
+        <v>6020.44</v>
+      </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -1806,6 +1831,7 @@
       <c r="AS9" s="13" t="n"/>
       <c r="AT9" s="13" t="n"/>
       <c r="AU9" s="13" t="n"/>
+      <c r="AV9" s="13" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -1948,6 +1974,9 @@
       </c>
       <c r="AU10" s="13" t="n">
         <v>59.95</v>
+      </c>
+      <c r="AV10" s="13" t="n">
+        <v>56.85</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2044,6 +2073,9 @@
       <c r="AU11" s="13" t="n">
         <v>4806.97</v>
       </c>
+      <c r="AV11" s="13" t="n">
+        <v>4807.31</v>
+      </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -2141,6 +2173,7 @@
       <c r="AS12" s="13" t="n"/>
       <c r="AT12" s="13" t="n"/>
       <c r="AU12" s="13" t="n"/>
+      <c r="AV12" s="13" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2283,6 +2316,9 @@
       </c>
       <c r="AU13" s="13" t="n">
         <v>67.03</v>
+      </c>
+      <c r="AV13" s="13" t="n">
+        <v>66.5</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -2379,6 +2415,9 @@
       <c r="AU14" s="13" t="n">
         <v>8346.370000000001</v>
       </c>
+      <c r="AV14" s="13" t="n">
+        <v>8349.51</v>
+      </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -2476,6 +2515,7 @@
       <c r="AS15" s="13" t="n"/>
       <c r="AT15" s="13" t="n"/>
       <c r="AU15" s="13" t="n"/>
+      <c r="AV15" s="13" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -2618,6 +2658,9 @@
       </c>
       <c r="AU16" s="13" t="n">
         <v>40.39</v>
+      </c>
+      <c r="AV16" s="13" t="n">
+        <v>37.41</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -2714,6 +2757,9 @@
       <c r="AU17" s="13" t="n">
         <v>2670.8</v>
       </c>
+      <c r="AV17" s="13" t="n">
+        <v>2679.37</v>
+      </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="3" t="n">
@@ -2811,6 +2857,7 @@
       <c r="AS18" s="13" t="n"/>
       <c r="AT18" s="13" t="n"/>
       <c r="AU18" s="13" t="n"/>
+      <c r="AV18" s="13" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -2953,6 +3000,9 @@
       </c>
       <c r="AU19" s="13" t="n">
         <v>94.06999999999999</v>
+      </c>
+      <c r="AV19" s="13" t="n">
+        <v>94.84999999999999</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -3049,6 +3099,9 @@
       <c r="AU20" s="13" t="n">
         <v>7135.95</v>
       </c>
+      <c r="AV20" s="13" t="n">
+        <v>7230.12</v>
+      </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -3146,6 +3199,7 @@
       <c r="AS21" s="13" t="n"/>
       <c r="AT21" s="13" t="n"/>
       <c r="AU21" s="13" t="n"/>
+      <c r="AV21" s="13" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -3286,6 +3340,9 @@
       </c>
       <c r="AU22" s="13" t="n">
         <v>43.74</v>
+      </c>
+      <c r="AV22" s="13" t="n">
+        <v>42.85</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1">
@@ -3382,6 +3439,9 @@
       <c r="AU23" s="13" t="n">
         <v>76355.50999999999</v>
       </c>
+      <c r="AV23" s="13" t="n">
+        <v>77669.92</v>
+      </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="3" t="n">
@@ -3479,6 +3539,7 @@
       <c r="AS24" s="13" t="n"/>
       <c r="AT24" s="13" t="n"/>
       <c r="AU24" s="13" t="n"/>
+      <c r="AV24" s="13" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -3621,6 +3682,9 @@
       </c>
       <c r="AU25" s="13" t="n">
         <v>75.43000000000001</v>
+      </c>
+      <c r="AV25" s="13" t="n">
+        <v>48.64</v>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="1">
@@ -3713,6 +3777,9 @@
         <v>24128.98</v>
       </c>
       <c r="AU26" s="13" t="inlineStr"/>
+      <c r="AV26" s="13" t="n">
+        <v>24292.38</v>
+      </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -3810,6 +3877,7 @@
       <c r="AS27" s="13" t="n"/>
       <c r="AT27" s="13" t="n"/>
       <c r="AU27" s="13" t="n"/>
+      <c r="AV27" s="13" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -3951,6 +4019,9 @@
         <v>87.04000000000001</v>
       </c>
       <c r="AU28" s="13" t="n">
+        <v>87.3</v>
+      </c>
+      <c r="AV28" s="13" t="n">
         <v>87.3</v>
       </c>
     </row>
@@ -4048,6 +4119,9 @@
       <c r="AU29" s="13" t="n">
         <v>59132.74</v>
       </c>
+      <c r="AV29" s="13" t="n">
+        <v>59513.12</v>
+      </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="3" t="n">
@@ -4145,6 +4219,7 @@
       <c r="AS30" s="13" t="n"/>
       <c r="AT30" s="13" t="n"/>
       <c r="AU30" s="13" t="n"/>
+      <c r="AV30" s="13" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -4287,6 +4362,9 @@
       </c>
       <c r="AU31" s="13" t="n">
         <v>51.89</v>
+      </c>
+      <c r="AV31" s="13" t="n">
+        <v>51.56</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -4383,6 +4461,9 @@
       <c r="AU32" s="13" t="n">
         <v>5858.45</v>
       </c>
+      <c r="AV32" s="13" t="n">
+        <v>5865.07</v>
+      </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
       <c r="A33" s="3" t="n">
@@ -4480,6 +4561,7 @@
       <c r="AS33" s="13" t="n"/>
       <c r="AT33" s="13" t="n"/>
       <c r="AU33" s="13" t="n"/>
+      <c r="AV33" s="13" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -4622,6 +4704,9 @@
       </c>
       <c r="AU34" s="13" t="n">
         <v>5.79</v>
+      </c>
+      <c r="AV34" s="13" t="n">
+        <v>4.58</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -4718,6 +4803,9 @@
       <c r="AU35" s="13" t="n">
         <v>35006.18</v>
       </c>
+      <c r="AV35" s="13" t="n">
+        <v>34957.44</v>
+      </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="3" t="n">
@@ -4815,6 +4903,7 @@
       <c r="AS36" s="13" t="n"/>
       <c r="AT36" s="13" t="n"/>
       <c r="AU36" s="13" t="n"/>
+      <c r="AV36" s="13" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -4957,6 +5046,9 @@
       </c>
       <c r="AU37" s="13" t="n">
         <v>57.09</v>
+      </c>
+      <c r="AV37" s="13" t="n">
+        <v>56.64</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -5053,6 +5145,9 @@
       <c r="AU38" s="13" t="n">
         <v>3910.85</v>
       </c>
+      <c r="AV38" s="13" t="n">
+        <v>3908.45</v>
+      </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
       <c r="A39" s="3" t="n">
@@ -5150,6 +5245,7 @@
       <c r="AS39" s="13" t="n"/>
       <c r="AT39" s="13" t="n"/>
       <c r="AU39" s="13" t="n"/>
+      <c r="AV39" s="13" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -5292,6 +5388,9 @@
       </c>
       <c r="AU40" s="13" t="n">
         <v>58.05</v>
+      </c>
+      <c r="AV40" s="13" t="n">
+        <v>57.55</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -5388,6 +5487,9 @@
       <c r="AU41" s="13" t="n">
         <v>3680</v>
       </c>
+      <c r="AV41" s="13" t="n">
+        <v>3677.15</v>
+      </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
       <c r="A42" s="3" t="n">
@@ -5485,6 +5587,7 @@
       <c r="AS42" s="13" t="n"/>
       <c r="AT42" s="13" t="n"/>
       <c r="AU42" s="13" t="n"/>
+      <c r="AV42" s="13" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -5627,6 +5730,9 @@
       </c>
       <c r="AU43" s="13" t="n">
         <v>10.16</v>
+      </c>
+      <c r="AV43" s="13" t="n">
+        <v>9.08</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -5723,6 +5829,9 @@
       <c r="AU44" s="13" t="n">
         <v>6683.55</v>
       </c>
+      <c r="AV44" s="13" t="n">
+        <v>6687.22</v>
+      </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
       <c r="A45" s="3" t="n">
@@ -5820,6 +5929,7 @@
       <c r="AS45" s="13" t="n"/>
       <c r="AT45" s="13" t="n"/>
       <c r="AU45" s="13" t="n"/>
+      <c r="AV45" s="13" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -5962,6 +6072,9 @@
       </c>
       <c r="AU46" s="13" t="n">
         <v>33.23</v>
+      </c>
+      <c r="AV46" s="13" t="n">
+        <v>33.07</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -6058,6 +6171,9 @@
       <c r="AU47" s="13" t="n">
         <v>8011.84</v>
       </c>
+      <c r="AV47" s="13" t="n">
+        <v>8013.49</v>
+      </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
       <c r="A48" s="3" t="n">
@@ -6155,6 +6271,7 @@
       <c r="AS48" s="13" t="n"/>
       <c r="AT48" s="13" t="n"/>
       <c r="AU48" s="13" t="n"/>
+      <c r="AV48" s="13" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -6297,6 +6414,9 @@
       </c>
       <c r="AU49" s="13" t="n">
         <v>8.619999999999999</v>
+      </c>
+      <c r="AV49" s="13" t="n">
+        <v>6.91</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -6393,6 +6513,9 @@
       <c r="AU50" s="13" t="n">
         <v>11574.14</v>
       </c>
+      <c r="AV50" s="13" t="n">
+        <v>11783.4</v>
+      </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
       <c r="A51" s="3" t="n">
@@ -6490,6 +6613,7 @@
       <c r="AS51" s="13" t="n"/>
       <c r="AT51" s="13" t="n"/>
       <c r="AU51" s="13" t="n"/>
+      <c r="AV51" s="13" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -6632,6 +6756,9 @@
       </c>
       <c r="AU52" s="13" t="n">
         <v>43.02</v>
+      </c>
+      <c r="AV52" s="13" t="n">
+        <v>42.56</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -6728,6 +6855,9 @@
       <c r="AU53" s="13" t="n">
         <v>12151.29</v>
       </c>
+      <c r="AV53" s="13" t="n">
+        <v>12176.59</v>
+      </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
       <c r="A54" s="3" t="n">
@@ -6825,6 +6955,7 @@
       <c r="AS54" s="13" t="n"/>
       <c r="AT54" s="13" t="n"/>
       <c r="AU54" s="13" t="n"/>
+      <c r="AV54" s="13" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -6967,6 +7098,9 @@
       </c>
       <c r="AU55" s="13" t="n">
         <v>13.3</v>
+      </c>
+      <c r="AV55" s="13" t="n">
+        <v>12.96</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -7063,6 +7197,9 @@
       <c r="AU56" s="13" t="n">
         <v>7648.91</v>
       </c>
+      <c r="AV56" s="13" t="n">
+        <v>7640.03</v>
+      </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
       <c r="A57" s="3" t="n">
@@ -7160,6 +7297,7 @@
       <c r="AS57" s="13" t="n"/>
       <c r="AT57" s="13" t="n"/>
       <c r="AU57" s="13" t="n"/>
+      <c r="AV57" s="13" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -7302,6 +7440,9 @@
       </c>
       <c r="AU58" s="13" t="n">
         <v>18.94</v>
+      </c>
+      <c r="AV58" s="13" t="n">
+        <v>17.73</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -7398,6 +7539,9 @@
       <c r="AU59" s="13" t="n">
         <v>14367.98</v>
       </c>
+      <c r="AV59" s="13" t="n">
+        <v>14358.23</v>
+      </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
       <c r="A60" s="3" t="n">
@@ -7495,6 +7639,7 @@
       <c r="AS60" s="13" t="n"/>
       <c r="AT60" s="13" t="n"/>
       <c r="AU60" s="13" t="n"/>
+      <c r="AV60" s="13" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -7637,6 +7782,9 @@
       </c>
       <c r="AU61" s="13" t="n">
         <v>62.21</v>
+      </c>
+      <c r="AV61" s="13" t="n">
+        <v>61.11</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -7733,6 +7881,9 @@
       <c r="AU62" s="13" t="n">
         <v>14687.84</v>
       </c>
+      <c r="AV62" s="13" t="n">
+        <v>15569.82</v>
+      </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
       <c r="A63" s="3" t="n">
@@ -7830,6 +7981,7 @@
       <c r="AS63" s="13" t="n"/>
       <c r="AT63" s="13" t="n"/>
       <c r="AU63" s="13" t="n"/>
+      <c r="AV63" s="13" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -7972,6 +8124,9 @@
       </c>
       <c r="AU64" s="13" t="n">
         <v>4.58</v>
+      </c>
+      <c r="AV64" s="13" t="n">
+        <v>3.38</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -8068,6 +8223,9 @@
       <c r="AU65" s="13" t="n">
         <v>8010.29</v>
       </c>
+      <c r="AV65" s="13" t="n">
+        <v>7632.93</v>
+      </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
       <c r="A66" s="3" t="n">
@@ -8165,6 +8323,7 @@
       <c r="AS66" s="13" t="n"/>
       <c r="AT66" s="13" t="n"/>
       <c r="AU66" s="13" t="n"/>
+      <c r="AV66" s="13" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -8307,6 +8466,9 @@
       </c>
       <c r="AU67" s="13" t="n">
         <v>2.11</v>
+      </c>
+      <c r="AV67" s="13" t="n">
+        <v>3.33</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -8403,6 +8565,9 @@
       <c r="AU68" s="13" t="n">
         <v>9067.51</v>
       </c>
+      <c r="AV68" s="13" t="n">
+        <v>9049.690000000001</v>
+      </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
       <c r="A69" s="3" t="n">
@@ -8500,6 +8665,7 @@
       <c r="AS69" s="13" t="n"/>
       <c r="AT69" s="13" t="n"/>
       <c r="AU69" s="13" t="n"/>
+      <c r="AV69" s="13" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -8642,6 +8808,9 @@
       </c>
       <c r="AU70" s="13" t="n">
         <v>20.44</v>
+      </c>
+      <c r="AV70" s="13" t="n">
+        <v>18.55</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -8738,6 +8907,9 @@
       <c r="AU71" s="13" t="n">
         <v>2631.9</v>
       </c>
+      <c r="AV71" s="13" t="n">
+        <v>2519.52</v>
+      </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
       <c r="A72" s="3" t="n">
@@ -8835,6 +9007,7 @@
       <c r="AS72" s="13" t="n"/>
       <c r="AT72" s="13" t="n"/>
       <c r="AU72" s="13" t="n"/>
+      <c r="AV72" s="13" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -8977,6 +9150,9 @@
       </c>
       <c r="AU73" s="13" t="n">
         <v>32.77</v>
+      </c>
+      <c r="AV73" s="13" t="n">
+        <v>28.46</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -9073,6 +9249,9 @@
       <c r="AU74" s="13" t="n">
         <v>5075.31</v>
       </c>
+      <c r="AV74" s="13" t="n">
+        <v>5002.37</v>
+      </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
       <c r="A75" s="3" t="n">
@@ -9170,6 +9349,7 @@
       <c r="AS75" s="13" t="n"/>
       <c r="AT75" s="13" t="n"/>
       <c r="AU75" s="13" t="n"/>
+      <c r="AV75" s="13" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -9312,6 +9492,9 @@
       </c>
       <c r="AU76" s="13" t="n">
         <v>20.79</v>
+      </c>
+      <c r="AV76" s="13" t="n">
+        <v>20.25</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -9408,6 +9591,9 @@
       <c r="AU77" s="13" t="n">
         <v>8626.67</v>
       </c>
+      <c r="AV77" s="13" t="n">
+        <v>8629.6</v>
+      </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
       <c r="A78" s="3" t="n">
@@ -9505,6 +9691,7 @@
       <c r="AS78" s="13" t="n"/>
       <c r="AT78" s="13" t="n"/>
       <c r="AU78" s="13" t="n"/>
+      <c r="AV78" s="13" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -9647,6 +9834,9 @@
       </c>
       <c r="AU79" s="13" t="n">
         <v>10.19</v>
+      </c>
+      <c r="AV79" s="13" t="n">
+        <v>10.05</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -9743,6 +9933,9 @@
       <c r="AU80" s="13" t="n">
         <v>1307.49</v>
       </c>
+      <c r="AV80" s="13" t="n">
+        <v>1305.07</v>
+      </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
       <c r="A81" s="3" t="n">
@@ -9840,6 +10033,7 @@
       <c r="AS81" s="13" t="n"/>
       <c r="AT81" s="13" t="n"/>
       <c r="AU81" s="13" t="n"/>
+      <c r="AV81" s="13" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -9982,6 +10176,9 @@
       </c>
       <c r="AU82" s="13" t="n">
         <v>11.73</v>
+      </c>
+      <c r="AV82" s="13" t="n">
+        <v>8.09</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -10078,6 +10275,9 @@
       <c r="AU83" s="13" t="n">
         <v>15684.77</v>
       </c>
+      <c r="AV83" s="13" t="n">
+        <v>15609.46</v>
+      </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
       <c r="A84" s="3" t="n">
@@ -10175,6 +10375,7 @@
       <c r="AS84" s="13" t="n"/>
       <c r="AT84" s="13" t="n"/>
       <c r="AU84" s="13" t="n"/>
+      <c r="AV84" s="13" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -10317,6 +10518,9 @@
       </c>
       <c r="AU85" s="13" t="n">
         <v>68.40000000000001</v>
+      </c>
+      <c r="AV85" s="13" t="n">
+        <v>66.90000000000001</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -10413,6 +10617,9 @@
       <c r="AU86" s="13" t="n">
         <v>3221.02</v>
       </c>
+      <c r="AV86" s="13" t="n">
+        <v>3228.56</v>
+      </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
       <c r="A87" s="3" t="n">
@@ -10510,6 +10717,7 @@
       <c r="AS87" s="13" t="n"/>
       <c r="AT87" s="13" t="n"/>
       <c r="AU87" s="13" t="n"/>
+      <c r="AV87" s="13" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -10652,6 +10860,9 @@
       </c>
       <c r="AU88" s="13" t="n">
         <v>73.92</v>
+      </c>
+      <c r="AV88" s="13" t="n">
+        <v>74.12</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -10748,6 +10959,9 @@
       <c r="AU89" s="13" t="n">
         <v>3157.1</v>
       </c>
+      <c r="AV89" s="13" t="n">
+        <v>3161.09</v>
+      </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
       <c r="A90" s="3" t="n">
@@ -10845,6 +11059,7 @@
       <c r="AS90" s="13" t="n"/>
       <c r="AT90" s="13" t="n"/>
       <c r="AU90" s="13" t="n"/>
+      <c r="AV90" s="13" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -10987,6 +11202,9 @@
       </c>
       <c r="AU91" s="13" t="n">
         <v>62.23</v>
+      </c>
+      <c r="AV91" s="13" t="n">
+        <v>59.59</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -11083,6 +11301,9 @@
       <c r="AU92" s="13" t="n">
         <v>3461.45</v>
       </c>
+      <c r="AV92" s="13" t="n">
+        <v>3461</v>
+      </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
       <c r="A93" s="3" t="n">
@@ -11180,6 +11401,7 @@
       <c r="AS93" s="13" t="n"/>
       <c r="AT93" s="13" t="n"/>
       <c r="AU93" s="13" t="n"/>
+      <c r="AV93" s="13" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -11322,6 +11544,9 @@
       </c>
       <c r="AU94" s="13" t="n">
         <v>55.52</v>
+      </c>
+      <c r="AV94" s="13" t="n">
+        <v>54.61</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -11418,6 +11643,9 @@
       <c r="AU95" s="13" t="n">
         <v>1898.04</v>
       </c>
+      <c r="AV95" s="13" t="n">
+        <v>1938.72</v>
+      </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
       <c r="A96" s="3" t="n">
@@ -11515,6 +11743,7 @@
       <c r="AS96" s="13" t="n"/>
       <c r="AT96" s="13" t="n"/>
       <c r="AU96" s="13" t="n"/>
+      <c r="AV96" s="13" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -11657,6 +11886,9 @@
       </c>
       <c r="AU97" s="13" t="n">
         <v>26.59</v>
+      </c>
+      <c r="AV97" s="13" t="n">
+        <v>26.71</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -11753,6 +11985,9 @@
       <c r="AU98" s="13" t="n">
         <v>9641.110000000001</v>
       </c>
+      <c r="AV98" s="13" t="n">
+        <v>9644.700000000001</v>
+      </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
       <c r="A99" s="3" t="n">
@@ -11850,6 +12085,7 @@
       <c r="AS99" s="13" t="n"/>
       <c r="AT99" s="13" t="n"/>
       <c r="AU99" s="13" t="n"/>
+      <c r="AV99" s="13" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -11992,6 +12228,9 @@
       </c>
       <c r="AU100" s="13" t="n">
         <v>90.73</v>
+      </c>
+      <c r="AV100" s="13" t="n">
+        <v>90.78</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -12088,6 +12327,9 @@
       <c r="AU101" s="13" t="n">
         <v>11484.59</v>
       </c>
+      <c r="AV101" s="13" t="n">
+        <v>11451.16</v>
+      </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
       <c r="A102" s="3" t="n">
@@ -12185,6 +12427,7 @@
       <c r="AS102" s="13" t="n"/>
       <c r="AT102" s="13" t="n"/>
       <c r="AU102" s="13" t="n"/>
+      <c r="AV102" s="13" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -12327,6 +12570,9 @@
       </c>
       <c r="AU103" s="13" t="n">
         <v>71.40000000000001</v>
+      </c>
+      <c r="AV103" s="13" t="n">
+        <v>71.12</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -12423,6 +12669,9 @@
       <c r="AU104" s="13" t="n">
         <v>14295.66</v>
       </c>
+      <c r="AV104" s="13" t="n">
+        <v>14301.36</v>
+      </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
       <c r="A105" s="3" t="n">
@@ -12520,6 +12769,7 @@
       <c r="AS105" s="13" t="n"/>
       <c r="AT105" s="13" t="n"/>
       <c r="AU105" s="13" t="n"/>
+      <c r="AV105" s="13" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -12662,6 +12912,9 @@
       </c>
       <c r="AU106" s="13" t="n">
         <v>32.16</v>
+      </c>
+      <c r="AV106" s="13" t="n">
+        <v>34.93</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -12758,6 +13011,9 @@
       <c r="AU107" s="13" t="n">
         <v>2161.17</v>
       </c>
+      <c r="AV107" s="13" t="n">
+        <v>2165.75</v>
+      </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
       <c r="A108" s="3" t="n">
@@ -12855,6 +13111,7 @@
       <c r="AS108" s="13" t="n"/>
       <c r="AT108" s="13" t="n"/>
       <c r="AU108" s="13" t="n"/>
+      <c r="AV108" s="13" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -12997,6 +13254,9 @@
       </c>
       <c r="AU109" s="13" t="n">
         <v>11.97</v>
+      </c>
+      <c r="AV109" s="13" t="n">
+        <v>10.94</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -13093,6 +13353,9 @@
       <c r="AU110" s="13" t="n">
         <v>756.7</v>
       </c>
+      <c r="AV110" s="13" t="n">
+        <v>757.08</v>
+      </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
       <c r="A111" s="3" t="n">
@@ -13190,6 +13453,7 @@
       <c r="AS111" s="13" t="n"/>
       <c r="AT111" s="13" t="n"/>
       <c r="AU111" s="13" t="n"/>
+      <c r="AV111" s="13" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -13332,6 +13596,9 @@
       </c>
       <c r="AU112" s="13" t="n">
         <v>76.23999999999999</v>
+      </c>
+      <c r="AV112" s="13" t="n">
+        <v>75.17</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -13428,6 +13695,9 @@
       <c r="AU113" s="13" t="n">
         <v>3442.74</v>
       </c>
+      <c r="AV113" s="13" t="n">
+        <v>3419.76</v>
+      </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
       <c r="A114" s="3" t="n">
@@ -13525,6 +13795,7 @@
       <c r="AS114" s="13" t="n"/>
       <c r="AT114" s="13" t="n"/>
       <c r="AU114" s="13" t="n"/>
+      <c r="AV114" s="13" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -13667,6 +13938,9 @@
       </c>
       <c r="AU115" s="13" t="n">
         <v>25.98</v>
+      </c>
+      <c r="AV115" s="13" t="n">
+        <v>24.72</v>
       </c>
     </row>
     <row r="116">
@@ -13747,6 +14021,9 @@
       </c>
       <c r="AU116" s="13" t="n">
         <v>3971.38</v>
+      </c>
+      <c r="AV116" s="13" t="n">
+        <v>3971.44</v>
       </c>
     </row>
     <row r="117">
@@ -13800,6 +14077,7 @@
       <c r="AS117" s="13" t="n"/>
       <c r="AT117" s="13" t="n"/>
       <c r="AU117" s="13" t="n"/>
+      <c r="AV117" s="13" t="n"/>
     </row>
     <row r="118">
       <c r="P118" s="13" t="n">
@@ -13898,6 +14176,9 @@
       <c r="AU118" s="13" t="n">
         <v>29.02</v>
       </c>
+      <c r="AV118" s="13" t="n">
+        <v>29.02</v>
+      </c>
     </row>
     <row r="119">
       <c r="Y119" s="13" t="n">
@@ -13968,6 +14249,9 @@
       </c>
       <c r="AU119" s="13" t="n">
         <v>2797.47</v>
+      </c>
+      <c r="AV119" s="13" t="n">
+        <v>2864.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-05-11 06:56:37]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV119"/>
+  <dimension ref="A1:AW137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="15"/>
@@ -565,6 +565,7 @@
     <col width="15" customWidth="1" min="46" max="46"/>
     <col width="15" customWidth="1" min="47" max="47"/>
     <col width="15" customWidth="1" min="48" max="48"/>
+    <col width="15" customWidth="1" min="49" max="49"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -808,6 +809,11 @@
           <t>2026/05/04</t>
         </is>
       </c>
+      <c r="AW1" s="13" t="inlineStr">
+        <is>
+          <t>2026/05/11</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1050,6 +1056,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="AW2" s="14" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1196,6 +1207,9 @@
       <c r="AV3" s="13" t="n">
         <v>69.06</v>
       </c>
+      <c r="AW3" s="13" t="n">
+        <v>71.53</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1341,6 +1355,9 @@
       </c>
       <c r="AV4" s="13" t="n">
         <v>4112.16</v>
+      </c>
+      <c r="AW4" s="13" t="n">
+        <v>4224.44</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1392,6 +1409,7 @@
       <c r="AT5" s="13" t="n"/>
       <c r="AU5" s="13" t="n"/>
       <c r="AV5" s="13" t="n"/>
+      <c r="AW5" s="13" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1490,6 +1508,7 @@
       <c r="AT6" s="13" t="n"/>
       <c r="AU6" s="13" t="n"/>
       <c r="AV6" s="13" t="n"/>
+      <c r="AW6" s="13" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1635,6 +1654,9 @@
       </c>
       <c r="AV7" s="13" t="n">
         <v>66.28</v>
+      </c>
+      <c r="AW7" s="13" t="n">
+        <v>68.45</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -1734,6 +1756,9 @@
       <c r="AV8" s="13" t="n">
         <v>6020.44</v>
       </c>
+      <c r="AW8" s="13" t="n">
+        <v>6262.7</v>
+      </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -1832,6 +1857,7 @@
       <c r="AT9" s="13" t="n"/>
       <c r="AU9" s="13" t="n"/>
       <c r="AV9" s="13" t="n"/>
+      <c r="AW9" s="13" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -1977,6 +2003,9 @@
       </c>
       <c r="AV10" s="13" t="n">
         <v>56.85</v>
+      </c>
+      <c r="AW10" s="13" t="n">
+        <v>57.92</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2076,6 +2105,9 @@
       <c r="AV11" s="13" t="n">
         <v>4807.31</v>
       </c>
+      <c r="AW11" s="13" t="n">
+        <v>4952.31</v>
+      </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -2174,6 +2206,7 @@
       <c r="AT12" s="13" t="n"/>
       <c r="AU12" s="13" t="n"/>
       <c r="AV12" s="13" t="n"/>
+      <c r="AW12" s="13" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2319,6 +2352,9 @@
       </c>
       <c r="AV13" s="13" t="n">
         <v>66.5</v>
+      </c>
+      <c r="AW13" s="13" t="n">
+        <v>68.97</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -2418,6 +2454,9 @@
       <c r="AV14" s="13" t="n">
         <v>8349.51</v>
       </c>
+      <c r="AW14" s="13" t="n">
+        <v>8840.23</v>
+      </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -2516,6 +2555,7 @@
       <c r="AT15" s="13" t="n"/>
       <c r="AU15" s="13" t="n"/>
       <c r="AV15" s="13" t="n"/>
+      <c r="AW15" s="13" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -2661,6 +2701,9 @@
       </c>
       <c r="AV16" s="13" t="n">
         <v>37.41</v>
+      </c>
+      <c r="AW16" s="13" t="n">
+        <v>38.8</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -2760,6 +2803,9 @@
       <c r="AV17" s="13" t="n">
         <v>2679.37</v>
       </c>
+      <c r="AW17" s="13" t="n">
+        <v>2724.65</v>
+      </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="3" t="n">
@@ -2858,6 +2904,7 @@
       <c r="AT18" s="13" t="n"/>
       <c r="AU18" s="13" t="n"/>
       <c r="AV18" s="13" t="n"/>
+      <c r="AW18" s="13" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -3003,6 +3050,9 @@
       </c>
       <c r="AV19" s="13" t="n">
         <v>94.84999999999999</v>
+      </c>
+      <c r="AW19" s="13" t="n">
+        <v>96.31</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -3102,6 +3152,9 @@
       <c r="AV20" s="13" t="n">
         <v>7230.12</v>
       </c>
+      <c r="AW20" s="13" t="n">
+        <v>7398.93</v>
+      </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -3200,6 +3253,7 @@
       <c r="AT21" s="13" t="n"/>
       <c r="AU21" s="13" t="n"/>
       <c r="AV21" s="13" t="n"/>
+      <c r="AW21" s="13" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -3343,6 +3397,9 @@
       </c>
       <c r="AV22" s="13" t="n">
         <v>42.85</v>
+      </c>
+      <c r="AW22" s="13" t="n">
+        <v>41.58</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1">
@@ -3442,6 +3499,9 @@
       <c r="AV23" s="13" t="n">
         <v>77669.92</v>
       </c>
+      <c r="AW23" s="13" t="n">
+        <v>76466.28</v>
+      </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="3" t="n">
@@ -3540,6 +3600,7 @@
       <c r="AT24" s="13" t="n"/>
       <c r="AU24" s="13" t="n"/>
       <c r="AV24" s="13" t="n"/>
+      <c r="AW24" s="13" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -3685,6 +3746,9 @@
       </c>
       <c r="AV25" s="13" t="n">
         <v>48.64</v>
+      </c>
+      <c r="AW25" s="13" t="n">
+        <v>52.14</v>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="1">
@@ -3780,6 +3844,9 @@
       <c r="AV26" s="13" t="n">
         <v>24292.38</v>
       </c>
+      <c r="AW26" s="13" t="n">
+        <v>24338.63</v>
+      </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -3878,6 +3945,7 @@
       <c r="AT27" s="13" t="n"/>
       <c r="AU27" s="13" t="n"/>
       <c r="AV27" s="13" t="n"/>
+      <c r="AW27" s="13" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -4023,6 +4091,9 @@
       </c>
       <c r="AV28" s="13" t="n">
         <v>87.3</v>
+      </c>
+      <c r="AW28" s="13" t="n">
+        <v>92.91</v>
       </c>
     </row>
     <row r="29" ht="14.25" customHeight="1">
@@ -4122,6 +4193,9 @@
       <c r="AV29" s="13" t="n">
         <v>59513.12</v>
       </c>
+      <c r="AW29" s="13" t="n">
+        <v>62417.88</v>
+      </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="3" t="n">
@@ -4220,6 +4294,7 @@
       <c r="AT30" s="13" t="n"/>
       <c r="AU30" s="13" t="n"/>
       <c r="AV30" s="13" t="n"/>
+      <c r="AW30" s="13" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -4365,6 +4440,9 @@
       </c>
       <c r="AV31" s="13" t="n">
         <v>51.56</v>
+      </c>
+      <c r="AW31" s="13" t="n">
+        <v>49.91</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -4464,6 +4542,9 @@
       <c r="AV32" s="13" t="n">
         <v>5865.07</v>
       </c>
+      <c r="AW32" s="13" t="n">
+        <v>5784.43</v>
+      </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
       <c r="A33" s="3" t="n">
@@ -4562,6 +4643,7 @@
       <c r="AT33" s="13" t="n"/>
       <c r="AU33" s="13" t="n"/>
       <c r="AV33" s="13" t="n"/>
+      <c r="AW33" s="13" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -4707,6 +4789,9 @@
       </c>
       <c r="AV34" s="13" t="n">
         <v>4.58</v>
+      </c>
+      <c r="AW34" s="13" t="n">
+        <v>62.6</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -4806,6 +4891,9 @@
       <c r="AV35" s="13" t="n">
         <v>34957.44</v>
       </c>
+      <c r="AW35" s="13" t="n">
+        <v>11898.62</v>
+      </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="3" t="n">
@@ -4904,6 +4992,7 @@
       <c r="AT36" s="13" t="n"/>
       <c r="AU36" s="13" t="n"/>
       <c r="AV36" s="13" t="n"/>
+      <c r="AW36" s="13" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -5049,6 +5138,9 @@
       </c>
       <c r="AV37" s="13" t="n">
         <v>56.64</v>
+      </c>
+      <c r="AW37" s="13" t="n">
+        <v>48.44</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -5148,6 +5240,9 @@
       <c r="AV38" s="13" t="n">
         <v>3908.45</v>
       </c>
+      <c r="AW38" s="13" t="n">
+        <v>11222.04</v>
+      </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
       <c r="A39" s="3" t="n">
@@ -5246,6 +5341,7 @@
       <c r="AT39" s="13" t="n"/>
       <c r="AU39" s="13" t="n"/>
       <c r="AV39" s="13" t="n"/>
+      <c r="AW39" s="13" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -5391,6 +5487,9 @@
       </c>
       <c r="AV40" s="13" t="n">
         <v>57.55</v>
+      </c>
+      <c r="AW40" s="13" t="n">
+        <v>51.77</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -5490,6 +5589,9 @@
       <c r="AV41" s="13" t="n">
         <v>3677.15</v>
       </c>
+      <c r="AW41" s="13" t="n">
+        <v>3254.14</v>
+      </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
       <c r="A42" s="3" t="n">
@@ -5588,6 +5690,7 @@
       <c r="AT42" s="13" t="n"/>
       <c r="AU42" s="13" t="n"/>
       <c r="AV42" s="13" t="n"/>
+      <c r="AW42" s="13" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -5733,6 +5836,9 @@
       </c>
       <c r="AV43" s="13" t="n">
         <v>9.08</v>
+      </c>
+      <c r="AW43" s="13" t="n">
+        <v>64.09999999999999</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -5832,6 +5938,9 @@
       <c r="AV44" s="13" t="n">
         <v>6687.22</v>
       </c>
+      <c r="AW44" s="13" t="n">
+        <v>7195.6</v>
+      </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
       <c r="A45" s="3" t="n">
@@ -5930,6 +6039,7 @@
       <c r="AT45" s="13" t="n"/>
       <c r="AU45" s="13" t="n"/>
       <c r="AV45" s="13" t="n"/>
+      <c r="AW45" s="13" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -6075,6 +6185,9 @@
       </c>
       <c r="AV46" s="13" t="n">
         <v>33.07</v>
+      </c>
+      <c r="AW46" s="13" t="n">
+        <v>2.32</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -6174,6 +6287,9 @@
       <c r="AV47" s="13" t="n">
         <v>8013.49</v>
       </c>
+      <c r="AW47" s="13" t="n">
+        <v>35770.43</v>
+      </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
       <c r="A48" s="3" t="n">
@@ -6272,6 +6388,7 @@
       <c r="AT48" s="13" t="n"/>
       <c r="AU48" s="13" t="n"/>
       <c r="AV48" s="13" t="n"/>
+      <c r="AW48" s="13" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -6417,6 +6534,9 @@
       </c>
       <c r="AV49" s="13" t="n">
         <v>6.91</v>
+      </c>
+      <c r="AW49" s="13" t="n">
+        <v>59.25</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -6516,6 +6636,9 @@
       <c r="AV50" s="13" t="n">
         <v>11783.4</v>
       </c>
+      <c r="AW50" s="13" t="n">
+        <v>4198.12</v>
+      </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
       <c r="A51" s="3" t="n">
@@ -6614,6 +6737,7 @@
       <c r="AT51" s="13" t="n"/>
       <c r="AU51" s="13" t="n"/>
       <c r="AV51" s="13" t="n"/>
+      <c r="AW51" s="13" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -6759,6 +6883,9 @@
       </c>
       <c r="AV52" s="13" t="n">
         <v>42.56</v>
+      </c>
+      <c r="AW52" s="13" t="n">
+        <v>59.74</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -6858,6 +6985,9 @@
       <c r="AV53" s="13" t="n">
         <v>12176.59</v>
       </c>
+      <c r="AW53" s="13" t="n">
+        <v>3929.58</v>
+      </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
       <c r="A54" s="3" t="n">
@@ -6956,6 +7086,7 @@
       <c r="AT54" s="13" t="n"/>
       <c r="AU54" s="13" t="n"/>
       <c r="AV54" s="13" t="n"/>
+      <c r="AW54" s="13" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -7101,6 +7232,9 @@
       </c>
       <c r="AV55" s="13" t="n">
         <v>12.96</v>
+      </c>
+      <c r="AW55" s="13" t="n">
+        <v>8.85</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -7200,6 +7334,9 @@
       <c r="AV56" s="13" t="n">
         <v>7640.03</v>
       </c>
+      <c r="AW56" s="13" t="n">
+        <v>6794.19</v>
+      </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
       <c r="A57" s="3" t="n">
@@ -7298,6 +7435,7 @@
       <c r="AT57" s="13" t="n"/>
       <c r="AU57" s="13" t="n"/>
       <c r="AV57" s="13" t="n"/>
+      <c r="AW57" s="13" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -7443,6 +7581,9 @@
       </c>
       <c r="AV58" s="13" t="n">
         <v>17.73</v>
+      </c>
+      <c r="AW58" s="13" t="n">
+        <v>31.66</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -7542,6 +7683,9 @@
       <c r="AV59" s="13" t="n">
         <v>14358.23</v>
       </c>
+      <c r="AW59" s="13" t="n">
+        <v>8009.66</v>
+      </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
       <c r="A60" s="3" t="n">
@@ -7640,6 +7784,7 @@
       <c r="AT60" s="13" t="n"/>
       <c r="AU60" s="13" t="n"/>
       <c r="AV60" s="13" t="n"/>
+      <c r="AW60" s="13" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -7785,6 +7930,9 @@
       </c>
       <c r="AV61" s="13" t="n">
         <v>61.11</v>
+      </c>
+      <c r="AW61" s="13" t="n">
+        <v>6.62</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -7884,6 +8032,9 @@
       <c r="AV62" s="13" t="n">
         <v>15569.82</v>
       </c>
+      <c r="AW62" s="13" t="n">
+        <v>11786.27</v>
+      </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
       <c r="A63" s="3" t="n">
@@ -7982,6 +8133,7 @@
       <c r="AT63" s="13" t="n"/>
       <c r="AU63" s="13" t="n"/>
       <c r="AV63" s="13" t="n"/>
+      <c r="AW63" s="13" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -8127,6 +8279,9 @@
       </c>
       <c r="AV64" s="13" t="n">
         <v>3.38</v>
+      </c>
+      <c r="AW64" s="13" t="n">
+        <v>44.7</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -8226,6 +8381,9 @@
       <c r="AV65" s="13" t="n">
         <v>7632.93</v>
       </c>
+      <c r="AW65" s="13" t="n">
+        <v>12833.42</v>
+      </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
       <c r="A66" s="3" t="n">
@@ -8324,6 +8482,7 @@
       <c r="AT66" s="13" t="n"/>
       <c r="AU66" s="13" t="n"/>
       <c r="AV66" s="13" t="n"/>
+      <c r="AW66" s="13" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -8469,6 +8628,9 @@
       </c>
       <c r="AV67" s="13" t="n">
         <v>3.33</v>
+      </c>
+      <c r="AW67" s="13" t="n">
+        <v>19.61</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -8568,6 +8730,9 @@
       <c r="AV68" s="13" t="n">
         <v>9049.690000000001</v>
       </c>
+      <c r="AW68" s="13" t="n">
+        <v>7518.38</v>
+      </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
       <c r="A69" s="3" t="n">
@@ -8666,6 +8831,7 @@
       <c r="AT69" s="13" t="n"/>
       <c r="AU69" s="13" t="n"/>
       <c r="AV69" s="13" t="n"/>
+      <c r="AW69" s="13" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -8811,6 +8977,9 @@
       </c>
       <c r="AV70" s="13" t="n">
         <v>18.55</v>
+      </c>
+      <c r="AW70" s="13" t="n">
+        <v>18.63</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -8910,6 +9079,9 @@
       <c r="AV71" s="13" t="n">
         <v>2519.52</v>
       </c>
+      <c r="AW71" s="13" t="n">
+        <v>14144.86</v>
+      </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
       <c r="A72" s="3" t="n">
@@ -9008,6 +9180,7 @@
       <c r="AT72" s="13" t="n"/>
       <c r="AU72" s="13" t="n"/>
       <c r="AV72" s="13" t="n"/>
+      <c r="AW72" s="13" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -9153,6 +9326,9 @@
       </c>
       <c r="AV73" s="13" t="n">
         <v>28.46</v>
+      </c>
+      <c r="AW73" s="13" t="n">
+        <v>60.24</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -9252,6 +9428,9 @@
       <c r="AV74" s="13" t="n">
         <v>5002.37</v>
       </c>
+      <c r="AW74" s="13" t="n">
+        <v>14675.81</v>
+      </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
       <c r="A75" s="3" t="n">
@@ -9350,6 +9529,7 @@
       <c r="AT75" s="13" t="n"/>
       <c r="AU75" s="13" t="n"/>
       <c r="AV75" s="13" t="n"/>
+      <c r="AW75" s="13" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -9495,6 +9675,9 @@
       </c>
       <c r="AV76" s="13" t="n">
         <v>20.25</v>
+      </c>
+      <c r="AW76" s="13" t="n">
+        <v>7.41</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -9594,6 +9777,9 @@
       <c r="AV77" s="13" t="n">
         <v>8629.6</v>
       </c>
+      <c r="AW77" s="13" t="n">
+        <v>7782.72</v>
+      </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
       <c r="A78" s="3" t="n">
@@ -9692,6 +9878,7 @@
       <c r="AT78" s="13" t="n"/>
       <c r="AU78" s="13" t="n"/>
       <c r="AV78" s="13" t="n"/>
+      <c r="AW78" s="13" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -9837,6 +10024,9 @@
       </c>
       <c r="AV79" s="13" t="n">
         <v>10.05</v>
+      </c>
+      <c r="AW79" s="13" t="n">
+        <v>3.53</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -9936,6 +10126,9 @@
       <c r="AV80" s="13" t="n">
         <v>1305.07</v>
       </c>
+      <c r="AW80" s="13" t="n">
+        <v>9102.610000000001</v>
+      </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
       <c r="A81" s="3" t="n">
@@ -10034,6 +10227,7 @@
       <c r="AT81" s="13" t="n"/>
       <c r="AU81" s="13" t="n"/>
       <c r="AV81" s="13" t="n"/>
+      <c r="AW81" s="13" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -10179,6 +10373,9 @@
       </c>
       <c r="AV82" s="13" t="n">
         <v>8.09</v>
+      </c>
+      <c r="AW82" s="13" t="n">
+        <v>23.3</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -10278,6 +10475,9 @@
       <c r="AV83" s="13" t="n">
         <v>15609.46</v>
       </c>
+      <c r="AW83" s="13" t="n">
+        <v>2631.9</v>
+      </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
       <c r="A84" s="3" t="n">
@@ -10376,6 +10576,7 @@
       <c r="AT84" s="13" t="n"/>
       <c r="AU84" s="13" t="n"/>
       <c r="AV84" s="13" t="n"/>
+      <c r="AW84" s="13" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -10521,6 +10722,9 @@
       </c>
       <c r="AV85" s="13" t="n">
         <v>66.90000000000001</v>
+      </c>
+      <c r="AW85" s="13" t="n">
+        <v>35.17</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -10620,6 +10824,9 @@
       <c r="AV86" s="13" t="n">
         <v>3228.56</v>
       </c>
+      <c r="AW86" s="13" t="n">
+        <v>5102.94</v>
+      </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
       <c r="A87" s="3" t="n">
@@ -10718,6 +10925,7 @@
       <c r="AT87" s="13" t="n"/>
       <c r="AU87" s="13" t="n"/>
       <c r="AV87" s="13" t="n"/>
+      <c r="AW87" s="13" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -10863,6 +11071,9 @@
       </c>
       <c r="AV88" s="13" t="n">
         <v>74.12</v>
+      </c>
+      <c r="AW88" s="13" t="n">
+        <v>19.44</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -10962,6 +11173,9 @@
       <c r="AV89" s="13" t="n">
         <v>3161.09</v>
       </c>
+      <c r="AW89" s="13" t="n">
+        <v>8697.82</v>
+      </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
       <c r="A90" s="3" t="n">
@@ -11060,6 +11274,7 @@
       <c r="AT90" s="13" t="n"/>
       <c r="AU90" s="13" t="n"/>
       <c r="AV90" s="13" t="n"/>
+      <c r="AW90" s="13" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -11205,6 +11420,9 @@
       </c>
       <c r="AV91" s="13" t="n">
         <v>59.59</v>
+      </c>
+      <c r="AW91" s="13" t="n">
+        <v>10.45</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -11304,6 +11522,9 @@
       <c r="AV92" s="13" t="n">
         <v>3461</v>
       </c>
+      <c r="AW92" s="13" t="n">
+        <v>1317.29</v>
+      </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
       <c r="A93" s="3" t="n">
@@ -11402,6 +11623,7 @@
       <c r="AT93" s="13" t="n"/>
       <c r="AU93" s="13" t="n"/>
       <c r="AV93" s="13" t="n"/>
+      <c r="AW93" s="13" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -11547,6 +11769,9 @@
       </c>
       <c r="AV94" s="13" t="n">
         <v>54.61</v>
+      </c>
+      <c r="AW94" s="13" t="n">
+        <v>12.3</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -11646,6 +11871,9 @@
       <c r="AV95" s="13" t="n">
         <v>1938.72</v>
       </c>
+      <c r="AW95" s="13" t="n">
+        <v>15432.27</v>
+      </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
       <c r="A96" s="3" t="n">
@@ -11744,6 +11972,7 @@
       <c r="AT96" s="13" t="n"/>
       <c r="AU96" s="13" t="n"/>
       <c r="AV96" s="13" t="n"/>
+      <c r="AW96" s="13" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -11889,6 +12118,9 @@
       </c>
       <c r="AV97" s="13" t="n">
         <v>26.71</v>
+      </c>
+      <c r="AW97" s="13" t="n">
+        <v>35.93</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -11988,6 +12220,9 @@
       <c r="AV98" s="13" t="n">
         <v>9644.700000000001</v>
       </c>
+      <c r="AW98" s="13" t="n">
+        <v>3229.09</v>
+      </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
       <c r="A99" s="3" t="n">
@@ -12086,6 +12321,7 @@
       <c r="AT99" s="13" t="n"/>
       <c r="AU99" s="13" t="n"/>
       <c r="AV99" s="13" t="n"/>
+      <c r="AW99" s="13" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -12231,6 +12467,9 @@
       </c>
       <c r="AV100" s="13" t="n">
         <v>90.78</v>
+      </c>
+      <c r="AW100" s="13" t="n">
+        <v>67.48</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -12330,6 +12569,9 @@
       <c r="AV101" s="13" t="n">
         <v>11451.16</v>
       </c>
+      <c r="AW101" s="13" t="n">
+        <v>3286.91</v>
+      </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
       <c r="A102" s="3" t="n">
@@ -12428,6 +12670,7 @@
       <c r="AT102" s="13" t="n"/>
       <c r="AU102" s="13" t="n"/>
       <c r="AV102" s="13" t="n"/>
+      <c r="AW102" s="13" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -12573,6 +12816,9 @@
       </c>
       <c r="AV103" s="13" t="n">
         <v>71.12</v>
+      </c>
+      <c r="AW103" s="13" t="n">
+        <v>75.44</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -12672,6 +12918,9 @@
       <c r="AV104" s="13" t="n">
         <v>14301.36</v>
       </c>
+      <c r="AW104" s="13" t="n">
+        <v>3263.56</v>
+      </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
       <c r="A105" s="3" t="n">
@@ -12770,6 +13019,7 @@
       <c r="AT105" s="13" t="n"/>
       <c r="AU105" s="13" t="n"/>
       <c r="AV105" s="13" t="n"/>
+      <c r="AW105" s="13" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -12915,6 +13165,9 @@
       </c>
       <c r="AV106" s="13" t="n">
         <v>34.93</v>
+      </c>
+      <c r="AW106" s="13" t="n">
+        <v>58.88</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -13014,6 +13267,9 @@
       <c r="AV107" s="13" t="n">
         <v>2165.75</v>
       </c>
+      <c r="AW107" s="13" t="n">
+        <v>3475.88</v>
+      </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
       <c r="A108" s="3" t="n">
@@ -13112,6 +13368,7 @@
       <c r="AT108" s="13" t="n"/>
       <c r="AU108" s="13" t="n"/>
       <c r="AV108" s="13" t="n"/>
+      <c r="AW108" s="13" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -13257,6 +13514,9 @@
       </c>
       <c r="AV109" s="13" t="n">
         <v>10.94</v>
+      </c>
+      <c r="AW109" s="13" t="n">
+        <v>52.78</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -13356,6 +13616,9 @@
       <c r="AV110" s="13" t="n">
         <v>757.08</v>
       </c>
+      <c r="AW110" s="13" t="n">
+        <v>1922.27</v>
+      </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
       <c r="A111" s="3" t="n">
@@ -13454,6 +13717,7 @@
       <c r="AT111" s="13" t="n"/>
       <c r="AU111" s="13" t="n"/>
       <c r="AV111" s="13" t="n"/>
+      <c r="AW111" s="13" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -13599,6 +13863,9 @@
       </c>
       <c r="AV112" s="13" t="n">
         <v>75.17</v>
+      </c>
+      <c r="AW112" s="13" t="n">
+        <v>27.8</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -13698,6 +13965,9 @@
       <c r="AV113" s="13" t="n">
         <v>3419.76</v>
       </c>
+      <c r="AW113" s="13" t="n">
+        <v>9959.57</v>
+      </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
       <c r="A114" s="3" t="n">
@@ -13796,6 +14066,7 @@
       <c r="AT114" s="13" t="n"/>
       <c r="AU114" s="13" t="n"/>
       <c r="AV114" s="13" t="n"/>
+      <c r="AW114" s="13" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -13941,6 +14212,9 @@
       </c>
       <c r="AV115" s="13" t="n">
         <v>24.72</v>
+      </c>
+      <c r="AW115" s="13" t="n">
+        <v>93.41</v>
       </c>
     </row>
     <row r="116">
@@ -14024,6 +14298,9 @@
       </c>
       <c r="AV116" s="13" t="n">
         <v>3971.44</v>
+      </c>
+      <c r="AW116" s="13" t="n">
+        <v>12676.57</v>
       </c>
     </row>
     <row r="117">
@@ -14078,6 +14355,7 @@
       <c r="AT117" s="13" t="n"/>
       <c r="AU117" s="13" t="n"/>
       <c r="AV117" s="13" t="n"/>
+      <c r="AW117" s="13" t="n"/>
     </row>
     <row r="118">
       <c r="P118" s="13" t="n">
@@ -14179,6 +14457,9 @@
       <c r="AV118" s="13" t="n">
         <v>29.02</v>
       </c>
+      <c r="AW118" s="13" t="n">
+        <v>77.90000000000001</v>
+      </c>
     </row>
     <row r="119">
       <c r="Y119" s="13" t="n">
@@ -14252,6 +14533,87 @@
       </c>
       <c r="AV119" s="13" t="n">
         <v>2864.2</v>
+      </c>
+      <c r="AW119" s="13" t="n">
+        <v>15167.63</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="AW120" s="13" t="n"/>
+    </row>
+    <row r="121">
+      <c r="AW121" s="13" t="n">
+        <v>32.69</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="AW122" s="13" t="n">
+        <v>2118.78</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="AW123" s="13" t="n"/>
+    </row>
+    <row r="124">
+      <c r="AW124" s="13" t="n">
+        <v>10.87</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="AW125" s="13" t="n">
+        <v>772.05</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="AW126" s="13" t="n"/>
+    </row>
+    <row r="127">
+      <c r="AW127" s="13" t="n">
+        <v>77.79000000000001</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="AW128" s="13" t="n">
+        <v>3609.88</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="AW129" s="13" t="n"/>
+    </row>
+    <row r="130">
+      <c r="AW130" s="13" t="n">
+        <v>28.56</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="AW131" s="13" t="n">
+        <v>4137.73</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="AW132" s="13" t="n"/>
+    </row>
+    <row r="133">
+      <c r="AW133" s="13" t="n">
+        <v>29.02</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="AW134" s="13" t="n">
+        <v>3019.41</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="AW135" s="13" t="n"/>
+    </row>
+    <row r="136">
+      <c r="AW136" s="13" t="n">
+        <v>60.91</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="AW137" s="13" t="n">
+        <v>7695.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-05-18 07:12:48]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW137"/>
+  <dimension ref="A1:AX137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="15"/>
@@ -566,6 +566,7 @@
     <col width="15" customWidth="1" min="47" max="47"/>
     <col width="15" customWidth="1" min="48" max="48"/>
     <col width="15" customWidth="1" min="49" max="49"/>
+    <col width="15" customWidth="1" min="50" max="50"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -814,6 +815,11 @@
           <t>2026/05/11</t>
         </is>
       </c>
+      <c r="AX1" s="13" t="inlineStr">
+        <is>
+          <t>2026/05/18</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1061,6 +1067,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="AX2" s="14" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1210,6 +1221,9 @@
       <c r="AW3" s="13" t="n">
         <v>71.53</v>
       </c>
+      <c r="AX3" s="13" t="n">
+        <v>70.78</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1358,6 +1372,9 @@
       </c>
       <c r="AW4" s="13" t="n">
         <v>4224.44</v>
+      </c>
+      <c r="AX4" s="13" t="n">
+        <v>4131.53</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1410,6 +1427,7 @@
       <c r="AU5" s="13" t="n"/>
       <c r="AV5" s="13" t="n"/>
       <c r="AW5" s="13" t="n"/>
+      <c r="AX5" s="13" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1509,6 +1527,7 @@
       <c r="AU6" s="13" t="n"/>
       <c r="AV6" s="13" t="n"/>
       <c r="AW6" s="13" t="n"/>
+      <c r="AX6" s="13" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1657,6 +1676,9 @@
       </c>
       <c r="AW7" s="13" t="n">
         <v>68.45</v>
+      </c>
+      <c r="AX7" s="13" t="n">
+        <v>67.09</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -1759,6 +1781,9 @@
       <c r="AW8" s="13" t="n">
         <v>6262.7</v>
       </c>
+      <c r="AX8" s="13" t="n">
+        <v>6084.51</v>
+      </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -1858,6 +1883,7 @@
       <c r="AU9" s="13" t="n"/>
       <c r="AV9" s="13" t="n"/>
       <c r="AW9" s="13" t="n"/>
+      <c r="AX9" s="13" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2006,6 +2032,9 @@
       </c>
       <c r="AW10" s="13" t="n">
         <v>57.92</v>
+      </c>
+      <c r="AX10" s="13" t="n">
+        <v>56.7</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2108,6 +2137,9 @@
       <c r="AW11" s="13" t="n">
         <v>4952.31</v>
       </c>
+      <c r="AX11" s="13" t="n">
+        <v>4833.52</v>
+      </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -2207,6 +2239,7 @@
       <c r="AU12" s="13" t="n"/>
       <c r="AV12" s="13" t="n"/>
       <c r="AW12" s="13" t="n"/>
+      <c r="AX12" s="13" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2355,6 +2388,9 @@
       </c>
       <c r="AW13" s="13" t="n">
         <v>68.97</v>
+      </c>
+      <c r="AX13" s="13" t="n">
+        <v>67.84999999999999</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -2457,6 +2493,9 @@
       <c r="AW14" s="13" t="n">
         <v>8840.23</v>
       </c>
+      <c r="AX14" s="13" t="n">
+        <v>8554.24</v>
+      </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -2556,6 +2595,7 @@
       <c r="AU15" s="13" t="n"/>
       <c r="AV15" s="13" t="n"/>
       <c r="AW15" s="13" t="n"/>
+      <c r="AX15" s="13" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -2704,6 +2744,9 @@
       </c>
       <c r="AW16" s="13" t="n">
         <v>38.8</v>
+      </c>
+      <c r="AX16" s="13" t="n">
+        <v>36.72</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -2806,6 +2849,9 @@
       <c r="AW17" s="13" t="n">
         <v>2724.65</v>
       </c>
+      <c r="AX17" s="13" t="n">
+        <v>2673.14</v>
+      </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="3" t="n">
@@ -2905,6 +2951,7 @@
       <c r="AU18" s="13" t="n"/>
       <c r="AV18" s="13" t="n"/>
       <c r="AW18" s="13" t="n"/>
+      <c r="AX18" s="13" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -3053,6 +3100,9 @@
       </c>
       <c r="AW19" s="13" t="n">
         <v>96.31</v>
+      </c>
+      <c r="AX19" s="13" t="n">
+        <v>96.2</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -3155,6 +3205,9 @@
       <c r="AW20" s="13" t="n">
         <v>7398.93</v>
       </c>
+      <c r="AX20" s="13" t="n">
+        <v>7408.5</v>
+      </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -3254,6 +3307,7 @@
       <c r="AU21" s="13" t="n"/>
       <c r="AV21" s="13" t="n"/>
       <c r="AW21" s="13" t="n"/>
+      <c r="AX21" s="13" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -3400,6 +3454,9 @@
       </c>
       <c r="AW22" s="13" t="n">
         <v>41.58</v>
+      </c>
+      <c r="AX22" s="13" t="n">
+        <v>36.34</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1">
@@ -3502,6 +3559,9 @@
       <c r="AW23" s="13" t="n">
         <v>76466.28</v>
       </c>
+      <c r="AX23" s="13" t="n">
+        <v>74936.33</v>
+      </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="3" t="n">
@@ -3601,6 +3661,7 @@
       <c r="AU24" s="13" t="n"/>
       <c r="AV24" s="13" t="n"/>
       <c r="AW24" s="13" t="n"/>
+      <c r="AX24" s="13" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -3749,6 +3810,9 @@
       </c>
       <c r="AW25" s="13" t="n">
         <v>52.14</v>
+      </c>
+      <c r="AX25" s="13" t="n">
+        <v>49.88</v>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="1">
@@ -3847,6 +3911,9 @@
       <c r="AW26" s="13" t="n">
         <v>24338.63</v>
       </c>
+      <c r="AX26" s="13" t="n">
+        <v>23950.57</v>
+      </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -3946,6 +4013,7 @@
       <c r="AU27" s="13" t="n"/>
       <c r="AV27" s="13" t="n"/>
       <c r="AW27" s="13" t="n"/>
+      <c r="AX27" s="13" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -4094,6 +4162,9 @@
       </c>
       <c r="AW28" s="13" t="n">
         <v>92.91</v>
+      </c>
+      <c r="AX28" s="13" t="n">
+        <v>92.09</v>
       </c>
     </row>
     <row r="29" ht="14.25" customHeight="1">
@@ -4196,6 +4267,9 @@
       <c r="AW29" s="13" t="n">
         <v>62417.88</v>
       </c>
+      <c r="AX29" s="13" t="n">
+        <v>60815.95</v>
+      </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="3" t="n">
@@ -4295,6 +4369,7 @@
       <c r="AU30" s="13" t="n"/>
       <c r="AV30" s="13" t="n"/>
       <c r="AW30" s="13" t="n"/>
+      <c r="AX30" s="13" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -4443,6 +4518,9 @@
       </c>
       <c r="AW31" s="13" t="n">
         <v>49.91</v>
+      </c>
+      <c r="AX31" s="13" t="n">
+        <v>56.35</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -4545,6 +4623,9 @@
       <c r="AW32" s="13" t="n">
         <v>5784.43</v>
       </c>
+      <c r="AX32" s="13" t="n">
+        <v>5654.2</v>
+      </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
       <c r="A33" s="3" t="n">
@@ -4644,6 +4725,7 @@
       <c r="AU33" s="13" t="n"/>
       <c r="AV33" s="13" t="n"/>
       <c r="AW33" s="13" t="n"/>
+      <c r="AX33" s="13" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -4792,6 +4874,9 @@
       </c>
       <c r="AW34" s="13" t="n">
         <v>62.6</v>
+      </c>
+      <c r="AX34" s="13" t="n">
+        <v>70.95999999999999</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -4894,6 +4979,9 @@
       <c r="AW35" s="13" t="n">
         <v>11898.62</v>
       </c>
+      <c r="AX35" s="13" t="n">
+        <v>11809.5</v>
+      </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="3" t="n">
@@ -4993,6 +5081,7 @@
       <c r="AU36" s="13" t="n"/>
       <c r="AV36" s="13" t="n"/>
       <c r="AW36" s="13" t="n"/>
+      <c r="AX36" s="13" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -5141,6 +5230,9 @@
       </c>
       <c r="AW37" s="13" t="n">
         <v>48.44</v>
+      </c>
+      <c r="AX37" s="13" t="n">
+        <v>56.17</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -5243,6 +5335,9 @@
       <c r="AW38" s="13" t="n">
         <v>11222.04</v>
       </c>
+      <c r="AX38" s="13" t="n">
+        <v>11115.82</v>
+      </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
       <c r="A39" s="3" t="n">
@@ -5342,6 +5437,7 @@
       <c r="AU39" s="13" t="n"/>
       <c r="AV39" s="13" t="n"/>
       <c r="AW39" s="13" t="n"/>
+      <c r="AX39" s="13" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -5490,6 +5586,9 @@
       </c>
       <c r="AW40" s="13" t="n">
         <v>51.77</v>
+      </c>
+      <c r="AX40" s="13" t="n">
+        <v>60.19</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -5592,6 +5691,9 @@
       <c r="AW41" s="13" t="n">
         <v>3254.14</v>
       </c>
+      <c r="AX41" s="13" t="n">
+        <v>3210.36</v>
+      </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
       <c r="A42" s="3" t="n">
@@ -5691,6 +5793,7 @@
       <c r="AU42" s="13" t="n"/>
       <c r="AV42" s="13" t="n"/>
       <c r="AW42" s="13" t="n"/>
+      <c r="AX42" s="13" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -5839,6 +5942,9 @@
       </c>
       <c r="AW43" s="13" t="n">
         <v>64.09999999999999</v>
+      </c>
+      <c r="AX43" s="13" t="n">
+        <v>78.56</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -5941,6 +6047,9 @@
       <c r="AW44" s="13" t="n">
         <v>7195.6</v>
       </c>
+      <c r="AX44" s="13" t="n">
+        <v>7183.28</v>
+      </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
       <c r="A45" s="3" t="n">
@@ -6040,6 +6149,7 @@
       <c r="AU45" s="13" t="n"/>
       <c r="AV45" s="13" t="n"/>
       <c r="AW45" s="13" t="n"/>
+      <c r="AX45" s="13" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -6188,6 +6298,9 @@
       </c>
       <c r="AW46" s="13" t="n">
         <v>2.32</v>
+      </c>
+      <c r="AX46" s="13" t="n">
+        <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -6290,6 +6403,9 @@
       <c r="AW47" s="13" t="n">
         <v>35770.43</v>
       </c>
+      <c r="AX47" s="13" t="n">
+        <v>34481.36</v>
+      </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
       <c r="A48" s="3" t="n">
@@ -6389,6 +6505,7 @@
       <c r="AU48" s="13" t="n"/>
       <c r="AV48" s="13" t="n"/>
       <c r="AW48" s="13" t="n"/>
+      <c r="AX48" s="13" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -6537,6 +6654,9 @@
       </c>
       <c r="AW49" s="13" t="n">
         <v>59.25</v>
+      </c>
+      <c r="AX49" s="13" t="n">
+        <v>61.98</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -6639,6 +6759,9 @@
       <c r="AW50" s="13" t="n">
         <v>4198.12</v>
       </c>
+      <c r="AX50" s="13" t="n">
+        <v>4196.08</v>
+      </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
       <c r="A51" s="3" t="n">
@@ -6738,6 +6861,7 @@
       <c r="AU51" s="13" t="n"/>
       <c r="AV51" s="13" t="n"/>
       <c r="AW51" s="13" t="n"/>
+      <c r="AX51" s="13" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -6886,6 +7010,9 @@
       </c>
       <c r="AW52" s="13" t="n">
         <v>59.74</v>
+      </c>
+      <c r="AX52" s="13" t="n">
+        <v>62.17</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -6988,6 +7115,9 @@
       <c r="AW53" s="13" t="n">
         <v>3929.58</v>
       </c>
+      <c r="AX53" s="13" t="n">
+        <v>3914.88</v>
+      </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
       <c r="A54" s="3" t="n">
@@ -7087,6 +7217,7 @@
       <c r="AU54" s="13" t="n"/>
       <c r="AV54" s="13" t="n"/>
       <c r="AW54" s="13" t="n"/>
+      <c r="AX54" s="13" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -7235,6 +7366,9 @@
       </c>
       <c r="AW55" s="13" t="n">
         <v>8.85</v>
+      </c>
+      <c r="AX55" s="13" t="n">
+        <v>5.94</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -7337,6 +7471,9 @@
       <c r="AW56" s="13" t="n">
         <v>6794.19</v>
       </c>
+      <c r="AX56" s="13" t="n">
+        <v>6413.74</v>
+      </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
       <c r="A57" s="3" t="n">
@@ -7436,6 +7573,7 @@
       <c r="AU57" s="13" t="n"/>
       <c r="AV57" s="13" t="n"/>
       <c r="AW57" s="13" t="n"/>
+      <c r="AX57" s="13" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -7584,6 +7722,9 @@
       </c>
       <c r="AW58" s="13" t="n">
         <v>31.66</v>
+      </c>
+      <c r="AX58" s="13" t="n">
+        <v>28.8</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -7686,6 +7827,9 @@
       <c r="AW59" s="13" t="n">
         <v>8009.66</v>
       </c>
+      <c r="AX59" s="13" t="n">
+        <v>7565.53</v>
+      </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
       <c r="A60" s="3" t="n">
@@ -7785,6 +7929,7 @@
       <c r="AU60" s="13" t="n"/>
       <c r="AV60" s="13" t="n"/>
       <c r="AW60" s="13" t="n"/>
+      <c r="AX60" s="13" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -7933,6 +8078,9 @@
       </c>
       <c r="AW61" s="13" t="n">
         <v>6.62</v>
+      </c>
+      <c r="AX61" s="13" t="n">
+        <v>5.41</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -8035,6 +8183,9 @@
       <c r="AW62" s="13" t="n">
         <v>11786.27</v>
       </c>
+      <c r="AX62" s="13" t="n">
+        <v>11490.66</v>
+      </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
       <c r="A63" s="3" t="n">
@@ -8134,6 +8285,7 @@
       <c r="AU63" s="13" t="n"/>
       <c r="AV63" s="13" t="n"/>
       <c r="AW63" s="13" t="n"/>
+      <c r="AX63" s="13" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -8282,6 +8434,9 @@
       </c>
       <c r="AW64" s="13" t="n">
         <v>44.7</v>
+      </c>
+      <c r="AX64" s="13" t="n">
+        <v>32.89</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -8384,6 +8539,9 @@
       <c r="AW65" s="13" t="n">
         <v>12833.42</v>
       </c>
+      <c r="AX65" s="13" t="n">
+        <v>12734.33</v>
+      </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
       <c r="A66" s="3" t="n">
@@ -8483,6 +8641,7 @@
       <c r="AU66" s="13" t="n"/>
       <c r="AV66" s="13" t="n"/>
       <c r="AW66" s="13" t="n"/>
+      <c r="AX66" s="13" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -8631,6 +8790,9 @@
       </c>
       <c r="AW67" s="13" t="n">
         <v>19.61</v>
+      </c>
+      <c r="AX67" s="13" t="n">
+        <v>16.91</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -8733,6 +8895,9 @@
       <c r="AW68" s="13" t="n">
         <v>7518.38</v>
       </c>
+      <c r="AX68" s="13" t="n">
+        <v>7076.51</v>
+      </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
       <c r="A69" s="3" t="n">
@@ -8832,6 +8997,7 @@
       <c r="AU69" s="13" t="n"/>
       <c r="AV69" s="13" t="n"/>
       <c r="AW69" s="13" t="n"/>
+      <c r="AX69" s="13" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -8980,6 +9146,9 @@
       </c>
       <c r="AW70" s="13" t="n">
         <v>18.63</v>
+      </c>
+      <c r="AX70" s="13" t="n">
+        <v>15.84</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -9082,6 +9251,9 @@
       <c r="AW71" s="13" t="n">
         <v>14144.86</v>
       </c>
+      <c r="AX71" s="13" t="n">
+        <v>13467.57</v>
+      </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
       <c r="A72" s="3" t="n">
@@ -9181,6 +9353,7 @@
       <c r="AU72" s="13" t="n"/>
       <c r="AV72" s="13" t="n"/>
       <c r="AW72" s="13" t="n"/>
+      <c r="AX72" s="13" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -9329,6 +9502,9 @@
       </c>
       <c r="AW73" s="13" t="n">
         <v>60.24</v>
+      </c>
+      <c r="AX73" s="13" t="n">
+        <v>56.16</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -9431,6 +9607,9 @@
       <c r="AW74" s="13" t="n">
         <v>14675.81</v>
       </c>
+      <c r="AX74" s="13" t="n">
+        <v>13445.7</v>
+      </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
       <c r="A75" s="3" t="n">
@@ -9530,6 +9709,7 @@
       <c r="AU75" s="13" t="n"/>
       <c r="AV75" s="13" t="n"/>
       <c r="AW75" s="13" t="n"/>
+      <c r="AX75" s="13" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -9678,6 +9858,9 @@
       </c>
       <c r="AW76" s="13" t="n">
         <v>7.41</v>
+      </c>
+      <c r="AX76" s="13" t="n">
+        <v>3.22</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -9780,6 +9963,9 @@
       <c r="AW77" s="13" t="n">
         <v>7782.72</v>
       </c>
+      <c r="AX77" s="13" t="n">
+        <v>7569.61</v>
+      </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
       <c r="A78" s="3" t="n">
@@ -9879,6 +10065,7 @@
       <c r="AU78" s="13" t="n"/>
       <c r="AV78" s="13" t="n"/>
       <c r="AW78" s="13" t="n"/>
+      <c r="AX78" s="13" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -10027,6 +10214,9 @@
       </c>
       <c r="AW79" s="13" t="n">
         <v>3.53</v>
+      </c>
+      <c r="AX79" s="13" t="n">
+        <v>2.5</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -10129,6 +10319,9 @@
       <c r="AW80" s="13" t="n">
         <v>9102.610000000001</v>
       </c>
+      <c r="AX80" s="13" t="n">
+        <v>8778.969999999999</v>
+      </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
       <c r="A81" s="3" t="n">
@@ -10228,6 +10421,7 @@
       <c r="AU81" s="13" t="n"/>
       <c r="AV81" s="13" t="n"/>
       <c r="AW81" s="13" t="n"/>
+      <c r="AX81" s="13" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -10376,6 +10570,9 @@
       </c>
       <c r="AW82" s="13" t="n">
         <v>23.3</v>
+      </c>
+      <c r="AX82" s="13" t="n">
+        <v>16.73</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -10478,6 +10675,9 @@
       <c r="AW83" s="13" t="n">
         <v>2631.9</v>
       </c>
+      <c r="AX83" s="13" t="n">
+        <v>2468.92</v>
+      </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
       <c r="A84" s="3" t="n">
@@ -10577,6 +10777,7 @@
       <c r="AU84" s="13" t="n"/>
       <c r="AV84" s="13" t="n"/>
       <c r="AW84" s="13" t="n"/>
+      <c r="AX84" s="13" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -10725,6 +10926,9 @@
       </c>
       <c r="AW85" s="13" t="n">
         <v>35.17</v>
+      </c>
+      <c r="AX85" s="13" t="n">
+        <v>25.09</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -10827,6 +11031,9 @@
       <c r="AW86" s="13" t="n">
         <v>5102.94</v>
       </c>
+      <c r="AX86" s="13" t="n">
+        <v>4833.36</v>
+      </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
       <c r="A87" s="3" t="n">
@@ -10926,6 +11133,7 @@
       <c r="AU87" s="13" t="n"/>
       <c r="AV87" s="13" t="n"/>
       <c r="AW87" s="13" t="n"/>
+      <c r="AX87" s="13" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -11074,6 +11282,9 @@
       </c>
       <c r="AW88" s="13" t="n">
         <v>19.44</v>
+      </c>
+      <c r="AX88" s="13" t="n">
+        <v>17.43</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -11176,6 +11387,9 @@
       <c r="AW89" s="13" t="n">
         <v>8697.82</v>
       </c>
+      <c r="AX89" s="13" t="n">
+        <v>8199.790000000001</v>
+      </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
       <c r="A90" s="3" t="n">
@@ -11275,6 +11489,7 @@
       <c r="AU90" s="13" t="n"/>
       <c r="AV90" s="13" t="n"/>
       <c r="AW90" s="13" t="n"/>
+      <c r="AX90" s="13" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -11423,6 +11638,9 @@
       </c>
       <c r="AW91" s="13" t="n">
         <v>10.45</v>
+      </c>
+      <c r="AX91" s="13" t="n">
+        <v>6.24</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -11525,6 +11743,9 @@
       <c r="AW92" s="13" t="n">
         <v>1317.29</v>
       </c>
+      <c r="AX92" s="13" t="n">
+        <v>1223.69</v>
+      </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
       <c r="A93" s="3" t="n">
@@ -11624,6 +11845,7 @@
       <c r="AU93" s="13" t="n"/>
       <c r="AV93" s="13" t="n"/>
       <c r="AW93" s="13" t="n"/>
+      <c r="AX93" s="13" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -11772,6 +11994,9 @@
       </c>
       <c r="AW94" s="13" t="n">
         <v>12.3</v>
+      </c>
+      <c r="AX94" s="13" t="n">
+        <v>10.15</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -11874,6 +12099,9 @@
       <c r="AW95" s="13" t="n">
         <v>15432.27</v>
       </c>
+      <c r="AX95" s="13" t="n">
+        <v>14950.45</v>
+      </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
       <c r="A96" s="3" t="n">
@@ -11973,6 +12201,7 @@
       <c r="AU96" s="13" t="n"/>
       <c r="AV96" s="13" t="n"/>
       <c r="AW96" s="13" t="n"/>
+      <c r="AX96" s="13" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -12121,6 +12350,9 @@
       </c>
       <c r="AW97" s="13" t="n">
         <v>35.93</v>
+      </c>
+      <c r="AX97" s="13" t="n">
+        <v>32.52</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -12223,6 +12455,9 @@
       <c r="AW98" s="13" t="n">
         <v>3229.09</v>
       </c>
+      <c r="AX98" s="13" t="n">
+        <v>3132.33</v>
+      </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
       <c r="A99" s="3" t="n">
@@ -12322,6 +12557,7 @@
       <c r="AU99" s="13" t="n"/>
       <c r="AV99" s="13" t="n"/>
       <c r="AW99" s="13" t="n"/>
+      <c r="AX99" s="13" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -12470,6 +12706,9 @@
       </c>
       <c r="AW100" s="13" t="n">
         <v>67.48</v>
+      </c>
+      <c r="AX100" s="13" t="n">
+        <v>63.19</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -12572,6 +12811,9 @@
       <c r="AW101" s="13" t="n">
         <v>3286.91</v>
       </c>
+      <c r="AX101" s="13" t="n">
+        <v>3139.55</v>
+      </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
       <c r="A102" s="3" t="n">
@@ -12671,6 +12913,7 @@
       <c r="AU102" s="13" t="n"/>
       <c r="AV102" s="13" t="n"/>
       <c r="AW102" s="13" t="n"/>
+      <c r="AX102" s="13" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -12819,6 +13062,9 @@
       </c>
       <c r="AW103" s="13" t="n">
         <v>75.44</v>
+      </c>
+      <c r="AX103" s="13" t="n">
+        <v>75.65000000000001</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -12921,6 +13167,9 @@
       <c r="AW104" s="13" t="n">
         <v>3263.56</v>
       </c>
+      <c r="AX104" s="13" t="n">
+        <v>3279.56</v>
+      </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
       <c r="A105" s="3" t="n">
@@ -13020,6 +13269,7 @@
       <c r="AU105" s="13" t="n"/>
       <c r="AV105" s="13" t="n"/>
       <c r="AW105" s="13" t="n"/>
+      <c r="AX105" s="13" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -13168,6 +13418,9 @@
       </c>
       <c r="AW106" s="13" t="n">
         <v>58.88</v>
+      </c>
+      <c r="AX106" s="13" t="n">
+        <v>53.88</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -13270,6 +13523,9 @@
       <c r="AW107" s="13" t="n">
         <v>3475.88</v>
       </c>
+      <c r="AX107" s="13" t="n">
+        <v>3282.37</v>
+      </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
       <c r="A108" s="3" t="n">
@@ -13369,6 +13625,7 @@
       <c r="AU108" s="13" t="n"/>
       <c r="AV108" s="13" t="n"/>
       <c r="AW108" s="13" t="n"/>
+      <c r="AX108" s="13" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -13517,6 +13774,9 @@
       </c>
       <c r="AW109" s="13" t="n">
         <v>52.78</v>
+      </c>
+      <c r="AX109" s="13" t="n">
+        <v>50.11</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -13619,6 +13879,9 @@
       <c r="AW110" s="13" t="n">
         <v>1922.27</v>
       </c>
+      <c r="AX110" s="13" t="n">
+        <v>1779.7</v>
+      </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
       <c r="A111" s="3" t="n">
@@ -13718,6 +13981,7 @@
       <c r="AU111" s="13" t="n"/>
       <c r="AV111" s="13" t="n"/>
       <c r="AW111" s="13" t="n"/>
+      <c r="AX111" s="13" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -13866,6 +14130,9 @@
       </c>
       <c r="AW112" s="13" t="n">
         <v>27.8</v>
+      </c>
+      <c r="AX112" s="13" t="n">
+        <v>25.97</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -13968,6 +14235,9 @@
       <c r="AW113" s="13" t="n">
         <v>9959.57</v>
       </c>
+      <c r="AX113" s="13" t="n">
+        <v>9745.35</v>
+      </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
       <c r="A114" s="3" t="n">
@@ -14067,6 +14337,7 @@
       <c r="AU114" s="13" t="n"/>
       <c r="AV114" s="13" t="n"/>
       <c r="AW114" s="13" t="n"/>
+      <c r="AX114" s="13" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -14215,6 +14486,9 @@
       </c>
       <c r="AW115" s="13" t="n">
         <v>93.41</v>
+      </c>
+      <c r="AX115" s="13" t="n">
+        <v>95.47</v>
       </c>
     </row>
     <row r="116">
@@ -14301,6 +14575,9 @@
       </c>
       <c r="AW116" s="13" t="n">
         <v>12676.57</v>
+      </c>
+      <c r="AX116" s="13" t="n">
+        <v>12981.75</v>
       </c>
     </row>
     <row r="117">
@@ -14356,6 +14633,7 @@
       <c r="AU117" s="13" t="n"/>
       <c r="AV117" s="13" t="n"/>
       <c r="AW117" s="13" t="n"/>
+      <c r="AX117" s="13" t="n"/>
     </row>
     <row r="118">
       <c r="P118" s="13" t="n">
@@ -14460,6 +14738,9 @@
       <c r="AW118" s="13" t="n">
         <v>77.90000000000001</v>
       </c>
+      <c r="AX118" s="13" t="n">
+        <v>70.16</v>
+      </c>
     </row>
     <row r="119">
       <c r="Y119" s="13" t="n">
@@ -14537,83 +14818,128 @@
       <c r="AW119" s="13" t="n">
         <v>15167.63</v>
       </c>
+      <c r="AX119" s="13" t="n">
+        <v>14075.06</v>
+      </c>
     </row>
     <row r="120">
       <c r="AW120" s="13" t="n"/>
+      <c r="AX120" s="13" t="n"/>
     </row>
     <row r="121">
       <c r="AW121" s="13" t="n">
         <v>32.69</v>
       </c>
+      <c r="AX121" s="13" t="n">
+        <v>31.05</v>
+      </c>
     </row>
     <row r="122">
       <c r="AW122" s="13" t="n">
         <v>2118.78</v>
       </c>
+      <c r="AX122" s="13" t="n">
+        <v>2026.92</v>
+      </c>
     </row>
     <row r="123">
       <c r="AW123" s="13" t="n"/>
+      <c r="AX123" s="13" t="n"/>
     </row>
     <row r="124">
       <c r="AW124" s="13" t="n">
         <v>10.87</v>
       </c>
+      <c r="AX124" s="13" t="n">
+        <v>7.93</v>
+      </c>
     </row>
     <row r="125">
       <c r="AW125" s="13" t="n">
         <v>772.05</v>
       </c>
+      <c r="AX125" s="13" t="n">
+        <v>735.75</v>
+      </c>
     </row>
     <row r="126">
       <c r="AW126" s="13" t="n"/>
+      <c r="AX126" s="13" t="n"/>
     </row>
     <row r="127">
       <c r="AW127" s="13" t="n">
         <v>77.79000000000001</v>
       </c>
+      <c r="AX127" s="13" t="n">
+        <v>72.61</v>
+      </c>
     </row>
     <row r="128">
       <c r="AW128" s="13" t="n">
         <v>3609.88</v>
       </c>
+      <c r="AX128" s="13" t="n">
+        <v>3253.01</v>
+      </c>
     </row>
     <row r="129">
       <c r="AW129" s="13" t="n"/>
+      <c r="AX129" s="13" t="n"/>
     </row>
     <row r="130">
       <c r="AW130" s="13" t="n">
         <v>28.56</v>
       </c>
+      <c r="AX130" s="13" t="n">
+        <v>26.47</v>
+      </c>
     </row>
     <row r="131">
       <c r="AW131" s="13" t="n">
         <v>4137.73</v>
       </c>
+      <c r="AX131" s="13" t="n">
+        <v>4005.12</v>
+      </c>
     </row>
     <row r="132">
       <c r="AW132" s="13" t="n"/>
+      <c r="AX132" s="13" t="n"/>
     </row>
     <row r="133">
       <c r="AW133" s="13" t="n">
         <v>29.02</v>
       </c>
+      <c r="AX133" s="13" t="n">
+        <v>29.02</v>
+      </c>
     </row>
     <row r="134">
       <c r="AW134" s="13" t="n">
         <v>3019.41</v>
       </c>
+      <c r="AX134" s="13" t="n">
+        <v>2829.72</v>
+      </c>
     </row>
     <row r="135">
       <c r="AW135" s="13" t="n"/>
+      <c r="AX135" s="13" t="n"/>
     </row>
     <row r="136">
       <c r="AW136" s="13" t="n">
         <v>60.91</v>
       </c>
+      <c r="AX136" s="13" t="n">
+        <v>37.4</v>
+      </c>
     </row>
     <row r="137">
       <c r="AW137" s="13" t="n">
         <v>7695.1</v>
+      </c>
+      <c r="AX137" s="13" t="n">
+        <v>7193.45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-07-13 06:36:33]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX137"/>
+  <dimension ref="A1:AY137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="15"/>
@@ -567,6 +567,7 @@
     <col width="15" customWidth="1" min="48" max="48"/>
     <col width="15" customWidth="1" min="49" max="49"/>
     <col width="15" customWidth="1" min="50" max="50"/>
+    <col width="15" customWidth="1" min="51" max="51"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -820,6 +821,11 @@
           <t>2026/05/18</t>
         </is>
       </c>
+      <c r="AY1" s="13" t="inlineStr">
+        <is>
+          <t>2026/07/13</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1072,6 +1078,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="AY2" s="14" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1224,6 +1235,9 @@
       <c r="AX3" s="13" t="n">
         <v>70.78</v>
       </c>
+      <c r="AY3" s="13" t="n">
+        <v>66.86</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1375,6 +1389,9 @@
       </c>
       <c r="AX4" s="13" t="n">
         <v>4131.53</v>
+      </c>
+      <c r="AY4" s="13" t="n">
+        <v>3906.6</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1428,6 +1445,7 @@
       <c r="AV5" s="13" t="n"/>
       <c r="AW5" s="13" t="n"/>
       <c r="AX5" s="13" t="n"/>
+      <c r="AY5" s="13" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1528,6 +1546,7 @@
       <c r="AV6" s="13" t="n"/>
       <c r="AW6" s="13" t="n"/>
       <c r="AX6" s="13" t="n"/>
+      <c r="AY6" s="13" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1679,6 +1698,9 @@
       </c>
       <c r="AX7" s="13" t="n">
         <v>67.09</v>
+      </c>
+      <c r="AY7" s="13" t="n">
+        <v>64.93000000000001</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -1784,6 +1806,9 @@
       <c r="AX8" s="13" t="n">
         <v>6084.51</v>
       </c>
+      <c r="AY8" s="13" t="n">
+        <v>5822.41</v>
+      </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -1884,6 +1909,7 @@
       <c r="AV9" s="13" t="n"/>
       <c r="AW9" s="13" t="n"/>
       <c r="AX9" s="13" t="n"/>
+      <c r="AY9" s="13" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2035,6 +2061,9 @@
       </c>
       <c r="AX10" s="13" t="n">
         <v>56.7</v>
+      </c>
+      <c r="AY10" s="13" t="n">
+        <v>55.74</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2140,6 +2169,9 @@
       <c r="AX11" s="13" t="n">
         <v>4833.52</v>
       </c>
+      <c r="AY11" s="13" t="n">
+        <v>4676.43</v>
+      </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -2240,6 +2272,7 @@
       <c r="AV12" s="13" t="n"/>
       <c r="AW12" s="13" t="n"/>
       <c r="AX12" s="13" t="n"/>
+      <c r="AY12" s="13" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2391,6 +2424,9 @@
       </c>
       <c r="AX13" s="13" t="n">
         <v>67.84999999999999</v>
+      </c>
+      <c r="AY13" s="13" t="n">
+        <v>70.51000000000001</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -2496,6 +2532,9 @@
       <c r="AX14" s="13" t="n">
         <v>8554.24</v>
       </c>
+      <c r="AY14" s="13" t="n">
+        <v>8107.06</v>
+      </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -2596,6 +2635,7 @@
       <c r="AV15" s="13" t="n"/>
       <c r="AW15" s="13" t="n"/>
       <c r="AX15" s="13" t="n"/>
+      <c r="AY15" s="13" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -2747,6 +2787,9 @@
       </c>
       <c r="AX16" s="13" t="n">
         <v>36.72</v>
+      </c>
+      <c r="AY16" s="13" t="n">
+        <v>33.74</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -2852,6 +2895,9 @@
       <c r="AX17" s="13" t="n">
         <v>2673.14</v>
       </c>
+      <c r="AY17" s="13" t="n">
+        <v>2557.81</v>
+      </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="3" t="n">
@@ -2952,6 +2998,7 @@
       <c r="AV18" s="13" t="n"/>
       <c r="AW18" s="13" t="n"/>
       <c r="AX18" s="13" t="n"/>
+      <c r="AY18" s="13" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -3103,6 +3150,9 @@
       </c>
       <c r="AX19" s="13" t="n">
         <v>96.2</v>
+      </c>
+      <c r="AY19" s="13" t="n">
+        <v>87.13</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -3208,6 +3258,9 @@
       <c r="AX20" s="13" t="n">
         <v>7408.5</v>
       </c>
+      <c r="AY20" s="13" t="n">
+        <v>7575.39</v>
+      </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -3308,6 +3361,7 @@
       <c r="AV21" s="13" t="n"/>
       <c r="AW21" s="13" t="n"/>
       <c r="AX21" s="13" t="n"/>
+      <c r="AY21" s="13" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -3456,6 +3510,9 @@
         <v>41.58</v>
       </c>
       <c r="AX22" s="13" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="AY22" s="13" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -3562,6 +3619,9 @@
       <c r="AX23" s="13" t="n">
         <v>74936.33</v>
       </c>
+      <c r="AY23" s="13" t="n">
+        <v>77381.41</v>
+      </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="3" t="n">
@@ -3662,6 +3722,7 @@
       <c r="AV24" s="13" t="n"/>
       <c r="AW24" s="13" t="n"/>
       <c r="AX24" s="13" t="n"/>
+      <c r="AY24" s="13" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -3812,6 +3873,9 @@
         <v>52.14</v>
       </c>
       <c r="AX25" s="13" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="AY25" s="13" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -3914,6 +3978,9 @@
       <c r="AX26" s="13" t="n">
         <v>23950.57</v>
       </c>
+      <c r="AY26" s="13" t="n">
+        <v>25067.09</v>
+      </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -4014,6 +4081,7 @@
       <c r="AV27" s="13" t="n"/>
       <c r="AW27" s="13" t="n"/>
       <c r="AX27" s="13" t="n"/>
+      <c r="AY27" s="13" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -4164,6 +4232,9 @@
         <v>92.91</v>
       </c>
       <c r="AX28" s="13" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="AY28" s="13" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -4270,6 +4341,9 @@
       <c r="AX29" s="13" t="n">
         <v>60815.95</v>
       </c>
+      <c r="AY29" s="13" t="n">
+        <v>67242.73</v>
+      </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="3" t="n">
@@ -4370,6 +4444,7 @@
       <c r="AV30" s="13" t="n"/>
       <c r="AW30" s="13" t="n"/>
       <c r="AX30" s="13" t="n"/>
+      <c r="AY30" s="13" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -4521,6 +4596,9 @@
       </c>
       <c r="AX31" s="13" t="n">
         <v>56.35</v>
+      </c>
+      <c r="AY31" s="13" t="n">
+        <v>51.18</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -4626,6 +4704,9 @@
       <c r="AX32" s="13" t="n">
         <v>5654.2</v>
       </c>
+      <c r="AY32" s="13" t="n">
+        <v>5190.42</v>
+      </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
       <c r="A33" s="3" t="n">
@@ -4726,6 +4807,7 @@
       <c r="AV33" s="13" t="n"/>
       <c r="AW33" s="13" t="n"/>
       <c r="AX33" s="13" t="n"/>
+      <c r="AY33" s="13" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -4877,6 +4959,9 @@
       </c>
       <c r="AX34" s="13" t="n">
         <v>70.95999999999999</v>
+      </c>
+      <c r="AY34" s="13" t="n">
+        <v>72.67</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -4982,6 +5067,9 @@
       <c r="AX35" s="13" t="n">
         <v>11809.5</v>
       </c>
+      <c r="AY35" s="13" t="n">
+        <v>10929.97</v>
+      </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="3" t="n">
@@ -5082,6 +5170,7 @@
       <c r="AV36" s="13" t="n"/>
       <c r="AW36" s="13" t="n"/>
       <c r="AX36" s="13" t="n"/>
+      <c r="AY36" s="13" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -5233,6 +5322,9 @@
       </c>
       <c r="AX37" s="13" t="n">
         <v>56.17</v>
+      </c>
+      <c r="AY37" s="13" t="n">
+        <v>58.26</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -5338,6 +5430,9 @@
       <c r="AX38" s="13" t="n">
         <v>11115.82</v>
       </c>
+      <c r="AY38" s="13" t="n">
+        <v>10327.58</v>
+      </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
       <c r="A39" s="3" t="n">
@@ -5438,6 +5533,7 @@
       <c r="AV39" s="13" t="n"/>
       <c r="AW39" s="13" t="n"/>
       <c r="AX39" s="13" t="n"/>
+      <c r="AY39" s="13" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -5589,6 +5685,9 @@
       </c>
       <c r="AX40" s="13" t="n">
         <v>60.19</v>
+      </c>
+      <c r="AY40" s="13" t="n">
+        <v>53.87</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -5694,6 +5793,9 @@
       <c r="AX41" s="13" t="n">
         <v>3210.36</v>
       </c>
+      <c r="AY41" s="13" t="n">
+        <v>2979.1</v>
+      </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
       <c r="A42" s="3" t="n">
@@ -5794,6 +5896,7 @@
       <c r="AV42" s="13" t="n"/>
       <c r="AW42" s="13" t="n"/>
       <c r="AX42" s="13" t="n"/>
+      <c r="AY42" s="13" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -5945,6 +6048,9 @@
       </c>
       <c r="AX43" s="13" t="n">
         <v>78.56</v>
+      </c>
+      <c r="AY43" s="13" t="n">
+        <v>67.11</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -6050,6 +6156,9 @@
       <c r="AX44" s="13" t="n">
         <v>7183.28</v>
       </c>
+      <c r="AY44" s="13" t="n">
+        <v>6698.78</v>
+      </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
       <c r="A45" s="3" t="n">
@@ -6150,6 +6259,7 @@
       <c r="AV45" s="13" t="n"/>
       <c r="AW45" s="13" t="n"/>
       <c r="AX45" s="13" t="n"/>
+      <c r="AY45" s="13" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -6301,6 +6411,9 @@
       </c>
       <c r="AX46" s="13" t="n">
         <v>0.6899999999999999</v>
+      </c>
+      <c r="AY46" s="13" t="n">
+        <v>21.69</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -6406,6 +6519,9 @@
       <c r="AX47" s="13" t="n">
         <v>34481.36</v>
       </c>
+      <c r="AY47" s="13" t="n">
+        <v>31877.53</v>
+      </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
       <c r="A48" s="3" t="n">
@@ -6506,6 +6622,7 @@
       <c r="AV48" s="13" t="n"/>
       <c r="AW48" s="13" t="n"/>
       <c r="AX48" s="13" t="n"/>
+      <c r="AY48" s="13" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -6657,6 +6774,9 @@
       </c>
       <c r="AX49" s="13" t="n">
         <v>61.98</v>
+      </c>
+      <c r="AY49" s="13" t="n">
+        <v>58.25</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -6762,6 +6882,9 @@
       <c r="AX50" s="13" t="n">
         <v>4196.08</v>
       </c>
+      <c r="AY50" s="13" t="n">
+        <v>3916.3</v>
+      </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
       <c r="A51" s="3" t="n">
@@ -6862,6 +6985,7 @@
       <c r="AV51" s="13" t="n"/>
       <c r="AW51" s="13" t="n"/>
       <c r="AX51" s="13" t="n"/>
+      <c r="AY51" s="13" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -7013,6 +7137,9 @@
       </c>
       <c r="AX52" s="13" t="n">
         <v>62.17</v>
+      </c>
+      <c r="AY52" s="13" t="n">
+        <v>66.40000000000001</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -7118,6 +7245,9 @@
       <c r="AX53" s="13" t="n">
         <v>3914.88</v>
       </c>
+      <c r="AY53" s="13" t="n">
+        <v>3693.2</v>
+      </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
       <c r="A54" s="3" t="n">
@@ -7218,6 +7348,7 @@
       <c r="AV54" s="13" t="n"/>
       <c r="AW54" s="13" t="n"/>
       <c r="AX54" s="13" t="n"/>
+      <c r="AY54" s="13" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -7369,6 +7500,9 @@
       </c>
       <c r="AX55" s="13" t="n">
         <v>5.94</v>
+      </c>
+      <c r="AY55" s="13" t="n">
+        <v>7.35</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -7474,6 +7608,9 @@
       <c r="AX56" s="13" t="n">
         <v>6413.74</v>
       </c>
+      <c r="AY56" s="13" t="n">
+        <v>6118.22</v>
+      </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
       <c r="A57" s="3" t="n">
@@ -7574,6 +7711,7 @@
       <c r="AV57" s="13" t="n"/>
       <c r="AW57" s="13" t="n"/>
       <c r="AX57" s="13" t="n"/>
+      <c r="AY57" s="13" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -7725,6 +7863,9 @@
       </c>
       <c r="AX58" s="13" t="n">
         <v>28.8</v>
+      </c>
+      <c r="AY58" s="13" t="n">
+        <v>29.26</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -7830,6 +7971,9 @@
       <c r="AX59" s="13" t="n">
         <v>7565.53</v>
       </c>
+      <c r="AY59" s="13" t="n">
+        <v>7734.35</v>
+      </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
       <c r="A60" s="3" t="n">
@@ -7930,6 +8074,7 @@
       <c r="AV60" s="13" t="n"/>
       <c r="AW60" s="13" t="n"/>
       <c r="AX60" s="13" t="n"/>
+      <c r="AY60" s="13" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -8081,6 +8226,9 @@
       </c>
       <c r="AX61" s="13" t="n">
         <v>5.41</v>
+      </c>
+      <c r="AY61" s="13" t="n">
+        <v>0.86</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -8186,6 +8334,9 @@
       <c r="AX62" s="13" t="n">
         <v>11490.66</v>
       </c>
+      <c r="AY62" s="13" t="n">
+        <v>10285.78</v>
+      </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
       <c r="A63" s="3" t="n">
@@ -8286,6 +8437,7 @@
       <c r="AV63" s="13" t="n"/>
       <c r="AW63" s="13" t="n"/>
       <c r="AX63" s="13" t="n"/>
+      <c r="AY63" s="13" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -8437,6 +8589,9 @@
       </c>
       <c r="AX64" s="13" t="n">
         <v>32.89</v>
+      </c>
+      <c r="AY64" s="13" t="n">
+        <v>17.66</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -8542,6 +8697,9 @@
       <c r="AX65" s="13" t="n">
         <v>12734.33</v>
       </c>
+      <c r="AY65" s="13" t="n">
+        <v>11475.31</v>
+      </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
       <c r="A66" s="3" t="n">
@@ -8642,6 +8800,7 @@
       <c r="AV66" s="13" t="n"/>
       <c r="AW66" s="13" t="n"/>
       <c r="AX66" s="13" t="n"/>
+      <c r="AY66" s="13" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -8793,6 +8952,9 @@
       </c>
       <c r="AX67" s="13" t="n">
         <v>16.91</v>
+      </c>
+      <c r="AY67" s="13" t="n">
+        <v>6.17</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -8898,6 +9060,9 @@
       <c r="AX68" s="13" t="n">
         <v>7076.51</v>
       </c>
+      <c r="AY68" s="13" t="n">
+        <v>6080.72</v>
+      </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
       <c r="A69" s="3" t="n">
@@ -8998,6 +9163,7 @@
       <c r="AV69" s="13" t="n"/>
       <c r="AW69" s="13" t="n"/>
       <c r="AX69" s="13" t="n"/>
+      <c r="AY69" s="13" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -9149,6 +9315,9 @@
       </c>
       <c r="AX70" s="13" t="n">
         <v>15.84</v>
+      </c>
+      <c r="AY70" s="13" t="n">
+        <v>7.8</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -9254,6 +9423,9 @@
       <c r="AX71" s="13" t="n">
         <v>13467.57</v>
       </c>
+      <c r="AY71" s="13" t="n">
+        <v>11956.6</v>
+      </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
       <c r="A72" s="3" t="n">
@@ -9354,6 +9526,7 @@
       <c r="AV72" s="13" t="n"/>
       <c r="AW72" s="13" t="n"/>
       <c r="AX72" s="13" t="n"/>
+      <c r="AY72" s="13" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -9505,6 +9678,9 @@
       </c>
       <c r="AX73" s="13" t="n">
         <v>56.16</v>
+      </c>
+      <c r="AY73" s="13" t="n">
+        <v>52.15</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -9610,6 +9786,9 @@
       <c r="AX74" s="13" t="n">
         <v>13445.7</v>
       </c>
+      <c r="AY74" s="13" t="n">
+        <v>15569.82</v>
+      </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
       <c r="A75" s="3" t="n">
@@ -9710,6 +9889,7 @@
       <c r="AV75" s="13" t="n"/>
       <c r="AW75" s="13" t="n"/>
       <c r="AX75" s="13" t="n"/>
+      <c r="AY75" s="13" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -9861,6 +10041,9 @@
       </c>
       <c r="AX76" s="13" t="n">
         <v>3.22</v>
+      </c>
+      <c r="AY76" s="13" t="n">
+        <v>3.29</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -9966,6 +10149,9 @@
       <c r="AX77" s="13" t="n">
         <v>7569.61</v>
       </c>
+      <c r="AY77" s="13" t="n">
+        <v>6926.32</v>
+      </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
       <c r="A78" s="3" t="n">
@@ -10066,6 +10252,7 @@
       <c r="AV78" s="13" t="n"/>
       <c r="AW78" s="13" t="n"/>
       <c r="AX78" s="13" t="n"/>
+      <c r="AY78" s="13" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -10217,6 +10404,9 @@
       </c>
       <c r="AX79" s="13" t="n">
         <v>2.5</v>
+      </c>
+      <c r="AY79" s="13" t="n">
+        <v>2.44</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -10322,6 +10512,9 @@
       <c r="AX80" s="13" t="n">
         <v>8778.969999999999</v>
       </c>
+      <c r="AY80" s="13" t="n">
+        <v>8619.530000000001</v>
+      </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
       <c r="A81" s="3" t="n">
@@ -10422,6 +10615,7 @@
       <c r="AV81" s="13" t="n"/>
       <c r="AW81" s="13" t="n"/>
       <c r="AX81" s="13" t="n"/>
+      <c r="AY81" s="13" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -10573,6 +10767,9 @@
       </c>
       <c r="AX82" s="13" t="n">
         <v>16.73</v>
+      </c>
+      <c r="AY82" s="13" t="n">
+        <v>12.36</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -10678,6 +10875,9 @@
       <c r="AX83" s="13" t="n">
         <v>2468.92</v>
       </c>
+      <c r="AY83" s="13" t="n">
+        <v>2237.93</v>
+      </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
       <c r="A84" s="3" t="n">
@@ -10778,6 +10978,7 @@
       <c r="AV84" s="13" t="n"/>
       <c r="AW84" s="13" t="n"/>
       <c r="AX84" s="13" t="n"/>
+      <c r="AY84" s="13" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -10929,6 +11130,9 @@
       </c>
       <c r="AX85" s="13" t="n">
         <v>25.09</v>
+      </c>
+      <c r="AY85" s="13" t="n">
+        <v>26.7</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -11034,6 +11238,9 @@
       <c r="AX86" s="13" t="n">
         <v>4833.36</v>
       </c>
+      <c r="AY86" s="13" t="n">
+        <v>5075.31</v>
+      </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
       <c r="A87" s="3" t="n">
@@ -11134,6 +11341,7 @@
       <c r="AV87" s="13" t="n"/>
       <c r="AW87" s="13" t="n"/>
       <c r="AX87" s="13" t="n"/>
+      <c r="AY87" s="13" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -11286,6 +11494,7 @@
       <c r="AX88" s="13" t="n">
         <v>17.43</v>
       </c>
+      <c r="AY88" s="13" t="n"/>
     </row>
     <row r="89" ht="14.25" customHeight="1">
       <c r="A89" s="1" t="n"/>
@@ -11390,6 +11599,7 @@
       <c r="AX89" s="13" t="n">
         <v>8199.790000000001</v>
       </c>
+      <c r="AY89" s="13" t="n"/>
     </row>
     <row r="90" ht="14.25" customHeight="1">
       <c r="A90" s="3" t="n">
@@ -11490,6 +11700,7 @@
       <c r="AV90" s="13" t="n"/>
       <c r="AW90" s="13" t="n"/>
       <c r="AX90" s="13" t="n"/>
+      <c r="AY90" s="13" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -11641,6 +11852,9 @@
       </c>
       <c r="AX91" s="13" t="n">
         <v>6.24</v>
+      </c>
+      <c r="AY91" s="13" t="n">
+        <v>3.1</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -11746,6 +11960,9 @@
       <c r="AX92" s="13" t="n">
         <v>1223.69</v>
       </c>
+      <c r="AY92" s="13" t="n">
+        <v>1113.51</v>
+      </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
       <c r="A93" s="3" t="n">
@@ -11846,6 +12063,7 @@
       <c r="AV93" s="13" t="n"/>
       <c r="AW93" s="13" t="n"/>
       <c r="AX93" s="13" t="n"/>
+      <c r="AY93" s="13" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -11997,6 +12215,9 @@
       </c>
       <c r="AX94" s="13" t="n">
         <v>10.15</v>
+      </c>
+      <c r="AY94" s="13" t="n">
+        <v>4.1</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -12102,6 +12323,9 @@
       <c r="AX95" s="13" t="n">
         <v>14950.45</v>
       </c>
+      <c r="AY95" s="13" t="n">
+        <v>13217.34</v>
+      </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
       <c r="A96" s="3" t="n">
@@ -12202,6 +12426,7 @@
       <c r="AV96" s="13" t="n"/>
       <c r="AW96" s="13" t="n"/>
       <c r="AX96" s="13" t="n"/>
+      <c r="AY96" s="13" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -12353,6 +12578,9 @@
       </c>
       <c r="AX97" s="13" t="n">
         <v>32.52</v>
+      </c>
+      <c r="AY97" s="13" t="n">
+        <v>45.23</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -12458,6 +12686,9 @@
       <c r="AX98" s="13" t="n">
         <v>3132.33</v>
       </c>
+      <c r="AY98" s="13" t="n">
+        <v>3167.36</v>
+      </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
       <c r="A99" s="3" t="n">
@@ -12558,6 +12789,7 @@
       <c r="AV99" s="13" t="n"/>
       <c r="AW99" s="13" t="n"/>
       <c r="AX99" s="13" t="n"/>
+      <c r="AY99" s="13" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -12709,6 +12941,9 @@
       </c>
       <c r="AX100" s="13" t="n">
         <v>63.19</v>
+      </c>
+      <c r="AY100" s="13" t="n">
+        <v>39.34</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -12814,6 +13049,9 @@
       <c r="AX101" s="13" t="n">
         <v>3139.55</v>
       </c>
+      <c r="AY101" s="13" t="n">
+        <v>2414.86</v>
+      </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
       <c r="A102" s="3" t="n">
@@ -12914,6 +13152,7 @@
       <c r="AV102" s="13" t="n"/>
       <c r="AW102" s="13" t="n"/>
       <c r="AX102" s="13" t="n"/>
+      <c r="AY102" s="13" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -13065,6 +13304,9 @@
       </c>
       <c r="AX103" s="13" t="n">
         <v>75.65000000000001</v>
+      </c>
+      <c r="AY103" s="13" t="n">
+        <v>18.94</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -13170,6 +13412,9 @@
       <c r="AX104" s="13" t="n">
         <v>3279.56</v>
       </c>
+      <c r="AY104" s="13" t="n">
+        <v>2705.1</v>
+      </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
       <c r="A105" s="3" t="n">
@@ -13270,6 +13515,7 @@
       <c r="AV105" s="13" t="n"/>
       <c r="AW105" s="13" t="n"/>
       <c r="AX105" s="13" t="n"/>
+      <c r="AY105" s="13" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -13421,6 +13667,9 @@
       </c>
       <c r="AX106" s="13" t="n">
         <v>53.88</v>
+      </c>
+      <c r="AY106" s="13" t="n">
+        <v>38.53</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -13526,6 +13775,9 @@
       <c r="AX107" s="13" t="n">
         <v>3282.37</v>
       </c>
+      <c r="AY107" s="13" t="n">
+        <v>2601.88</v>
+      </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
       <c r="A108" s="3" t="n">
@@ -13626,6 +13878,7 @@
       <c r="AV108" s="13" t="n"/>
       <c r="AW108" s="13" t="n"/>
       <c r="AX108" s="13" t="n"/>
+      <c r="AY108" s="13" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -13777,6 +14030,9 @@
       </c>
       <c r="AX109" s="13" t="n">
         <v>50.11</v>
+      </c>
+      <c r="AY109" s="13" t="n">
+        <v>59.53</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -13882,6 +14138,9 @@
       <c r="AX110" s="13" t="n">
         <v>1779.7</v>
       </c>
+      <c r="AY110" s="13" t="n">
+        <v>1908.79</v>
+      </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
       <c r="A111" s="3" t="n">
@@ -13982,6 +14241,7 @@
       <c r="AV111" s="13" t="n"/>
       <c r="AW111" s="13" t="n"/>
       <c r="AX111" s="13" t="n"/>
+      <c r="AY111" s="13" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -14133,6 +14393,9 @@
       </c>
       <c r="AX112" s="13" t="n">
         <v>25.97</v>
+      </c>
+      <c r="AY112" s="13" t="n">
+        <v>20.44</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -14238,6 +14501,9 @@
       <c r="AX113" s="13" t="n">
         <v>9745.35</v>
       </c>
+      <c r="AY113" s="13" t="n">
+        <v>8566.25</v>
+      </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
       <c r="A114" s="3" t="n">
@@ -14338,6 +14604,7 @@
       <c r="AV114" s="13" t="n"/>
       <c r="AW114" s="13" t="n"/>
       <c r="AX114" s="13" t="n"/>
+      <c r="AY114" s="13" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -14489,6 +14756,9 @@
       </c>
       <c r="AX115" s="13" t="n">
         <v>95.47</v>
+      </c>
+      <c r="AY115" s="13" t="n">
+        <v>99.28</v>
       </c>
     </row>
     <row r="116">
@@ -14578,6 +14848,9 @@
       </c>
       <c r="AX116" s="13" t="n">
         <v>12981.75</v>
+      </c>
+      <c r="AY116" s="13" t="n">
+        <v>16304.17</v>
       </c>
     </row>
     <row r="117">
@@ -14634,6 +14907,7 @@
       <c r="AV117" s="13" t="n"/>
       <c r="AW117" s="13" t="n"/>
       <c r="AX117" s="13" t="n"/>
+      <c r="AY117" s="13" t="n"/>
     </row>
     <row r="118">
       <c r="P118" s="13" t="n">
@@ -14741,6 +15015,9 @@
       <c r="AX118" s="13" t="n">
         <v>70.16</v>
       </c>
+      <c r="AY118" s="13" t="n">
+        <v>62.89</v>
+      </c>
     </row>
     <row r="119">
       <c r="Y119" s="13" t="n">
@@ -14821,10 +15098,14 @@
       <c r="AX119" s="13" t="n">
         <v>14075.06</v>
       </c>
+      <c r="AY119" s="13" t="n">
+        <v>12165.01</v>
+      </c>
     </row>
     <row r="120">
       <c r="AW120" s="13" t="n"/>
       <c r="AX120" s="13" t="n"/>
+      <c r="AY120" s="13" t="n"/>
     </row>
     <row r="121">
       <c r="AW121" s="13" t="n">
@@ -14833,6 +15114,9 @@
       <c r="AX121" s="13" t="n">
         <v>31.05</v>
       </c>
+      <c r="AY121" s="13" t="n">
+        <v>27.69</v>
+      </c>
     </row>
     <row r="122">
       <c r="AW122" s="13" t="n">
@@ -14841,10 +15125,14 @@
       <c r="AX122" s="13" t="n">
         <v>2026.92</v>
       </c>
+      <c r="AY122" s="13" t="n">
+        <v>1821.31</v>
+      </c>
     </row>
     <row r="123">
       <c r="AW123" s="13" t="n"/>
       <c r="AX123" s="13" t="n"/>
+      <c r="AY123" s="13" t="n"/>
     </row>
     <row r="124">
       <c r="AW124" s="13" t="n">
@@ -14853,6 +15141,9 @@
       <c r="AX124" s="13" t="n">
         <v>7.93</v>
       </c>
+      <c r="AY124" s="13" t="n">
+        <v>15.54</v>
+      </c>
     </row>
     <row r="125">
       <c r="AW125" s="13" t="n">
@@ -14861,10 +15152,14 @@
       <c r="AX125" s="13" t="n">
         <v>735.75</v>
       </c>
+      <c r="AY125" s="13" t="n">
+        <v>768.65</v>
+      </c>
     </row>
     <row r="126">
       <c r="AW126" s="13" t="n"/>
       <c r="AX126" s="13" t="n"/>
+      <c r="AY126" s="13" t="n"/>
     </row>
     <row r="127">
       <c r="AW127" s="13" t="n">
@@ -14873,6 +15168,9 @@
       <c r="AX127" s="13" t="n">
         <v>72.61</v>
       </c>
+      <c r="AY127" s="13" t="n">
+        <v>58.22</v>
+      </c>
     </row>
     <row r="128">
       <c r="AW128" s="13" t="n">
@@ -14881,10 +15179,14 @@
       <c r="AX128" s="13" t="n">
         <v>3253.01</v>
       </c>
+      <c r="AY128" s="13" t="n">
+        <v>2678.46</v>
+      </c>
     </row>
     <row r="129">
       <c r="AW129" s="13" t="n"/>
       <c r="AX129" s="13" t="n"/>
+      <c r="AY129" s="13" t="n"/>
     </row>
     <row r="130">
       <c r="AW130" s="13" t="n">
@@ -14893,6 +15195,9 @@
       <c r="AX130" s="13" t="n">
         <v>26.47</v>
       </c>
+      <c r="AY130" s="13" t="n">
+        <v>20.78</v>
+      </c>
     </row>
     <row r="131">
       <c r="AW131" s="13" t="n">
@@ -14901,10 +15206,14 @@
       <c r="AX131" s="13" t="n">
         <v>4005.12</v>
       </c>
+      <c r="AY131" s="13" t="n">
+        <v>3568.39</v>
+      </c>
     </row>
     <row r="132">
       <c r="AW132" s="13" t="n"/>
       <c r="AX132" s="13" t="n"/>
+      <c r="AY132" s="13" t="n"/>
     </row>
     <row r="133">
       <c r="AW133" s="13" t="n">
@@ -14913,6 +15222,9 @@
       <c r="AX133" s="13" t="n">
         <v>29.02</v>
       </c>
+      <c r="AY133" s="13" t="n">
+        <v>2.09</v>
+      </c>
     </row>
     <row r="134">
       <c r="AW134" s="13" t="n">
@@ -14921,10 +15233,14 @@
       <c r="AX134" s="13" t="n">
         <v>2829.72</v>
       </c>
+      <c r="AY134" s="13" t="n">
+        <v>2362.93</v>
+      </c>
     </row>
     <row r="135">
       <c r="AW135" s="13" t="n"/>
       <c r="AX135" s="13" t="n"/>
+      <c r="AY135" s="13" t="n"/>
     </row>
     <row r="136">
       <c r="AW136" s="13" t="n">
@@ -14933,6 +15249,9 @@
       <c r="AX136" s="13" t="n">
         <v>37.4</v>
       </c>
+      <c r="AY136" s="13" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="137">
       <c r="AW137" s="13" t="n">
@@ -14940,6 +15259,9 @@
       </c>
       <c r="AX137" s="13" t="n">
         <v>7193.45</v>
+      </c>
+      <c r="AY137" s="13" t="n">
+        <v>6280.28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-07-13 06:40:23]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY137"/>
+  <dimension ref="A1:AZ137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="15"/>
@@ -568,6 +568,7 @@
     <col width="15" customWidth="1" min="49" max="49"/>
     <col width="15" customWidth="1" min="50" max="50"/>
     <col width="15" customWidth="1" min="51" max="51"/>
+    <col width="15" customWidth="1" min="52" max="52"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -826,6 +827,11 @@
           <t>2026/07/13</t>
         </is>
       </c>
+      <c r="AZ1" s="13" t="inlineStr">
+        <is>
+          <t>2026/07/13</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1083,6 +1089,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="AZ2" s="14" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1238,6 +1249,9 @@
       <c r="AY3" s="13" t="n">
         <v>66.86</v>
       </c>
+      <c r="AZ3" s="13" t="n">
+        <v>66.86</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1392,6 +1406,9 @@
       </c>
       <c r="AY4" s="13" t="n">
         <v>3906.6</v>
+      </c>
+      <c r="AZ4" s="13" t="n">
+        <v>3914.85</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1446,6 +1463,7 @@
       <c r="AW5" s="13" t="n"/>
       <c r="AX5" s="13" t="n"/>
       <c r="AY5" s="13" t="n"/>
+      <c r="AZ5" s="13" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1547,6 +1565,7 @@
       <c r="AW6" s="13" t="n"/>
       <c r="AX6" s="13" t="n"/>
       <c r="AY6" s="13" t="n"/>
+      <c r="AZ6" s="13" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1700,6 +1719,9 @@
         <v>67.09</v>
       </c>
       <c r="AY7" s="13" t="n">
+        <v>64.93000000000001</v>
+      </c>
+      <c r="AZ7" s="13" t="n">
         <v>64.93000000000001</v>
       </c>
     </row>
@@ -1809,6 +1831,9 @@
       <c r="AY8" s="13" t="n">
         <v>5822.41</v>
       </c>
+      <c r="AZ8" s="13" t="n">
+        <v>5841.28</v>
+      </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -1910,6 +1935,7 @@
       <c r="AW9" s="13" t="n"/>
       <c r="AX9" s="13" t="n"/>
       <c r="AY9" s="13" t="n"/>
+      <c r="AZ9" s="13" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2063,6 +2089,9 @@
         <v>56.7</v>
       </c>
       <c r="AY10" s="13" t="n">
+        <v>55.74</v>
+      </c>
+      <c r="AZ10" s="13" t="n">
         <v>55.74</v>
       </c>
     </row>
@@ -2172,6 +2201,9 @@
       <c r="AY11" s="13" t="n">
         <v>4676.43</v>
       </c>
+      <c r="AZ11" s="13" t="n">
+        <v>4685.33</v>
+      </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -2273,6 +2305,7 @@
       <c r="AW12" s="13" t="n"/>
       <c r="AX12" s="13" t="n"/>
       <c r="AY12" s="13" t="n"/>
+      <c r="AZ12" s="13" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2426,6 +2459,9 @@
         <v>67.84999999999999</v>
       </c>
       <c r="AY13" s="13" t="n">
+        <v>70.51000000000001</v>
+      </c>
+      <c r="AZ13" s="13" t="n">
         <v>70.51000000000001</v>
       </c>
     </row>
@@ -2535,6 +2571,9 @@
       <c r="AY14" s="13" t="n">
         <v>8107.06</v>
       </c>
+      <c r="AZ14" s="13" t="n">
+        <v>8135.86</v>
+      </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -2636,6 +2675,7 @@
       <c r="AW15" s="13" t="n"/>
       <c r="AX15" s="13" t="n"/>
       <c r="AY15" s="13" t="n"/>
+      <c r="AZ15" s="13" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -2789,6 +2829,9 @@
         <v>36.72</v>
       </c>
       <c r="AY16" s="13" t="n">
+        <v>33.74</v>
+      </c>
+      <c r="AZ16" s="13" t="n">
         <v>33.74</v>
       </c>
     </row>
@@ -2898,6 +2941,9 @@
       <c r="AY17" s="13" t="n">
         <v>2557.81</v>
       </c>
+      <c r="AZ17" s="13" t="n">
+        <v>2563.76</v>
+      </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="3" t="n">
@@ -2999,6 +3045,7 @@
       <c r="AW18" s="13" t="n"/>
       <c r="AX18" s="13" t="n"/>
       <c r="AY18" s="13" t="n"/>
+      <c r="AZ18" s="13" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -3152,6 +3199,9 @@
         <v>96.2</v>
       </c>
       <c r="AY19" s="13" t="n">
+        <v>87.13</v>
+      </c>
+      <c r="AZ19" s="13" t="n">
         <v>87.13</v>
       </c>
     </row>
@@ -3261,6 +3311,9 @@
       <c r="AY20" s="13" t="n">
         <v>7575.39</v>
       </c>
+      <c r="AZ20" s="13" t="n">
+        <v>7575.39</v>
+      </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -3362,6 +3415,7 @@
       <c r="AW21" s="13" t="n"/>
       <c r="AX21" s="13" t="n"/>
       <c r="AY21" s="13" t="n"/>
+      <c r="AZ21" s="13" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -3513,6 +3567,9 @@
         <v>36.34</v>
       </c>
       <c r="AY22" s="13" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="AZ22" s="13" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -3622,6 +3679,9 @@
       <c r="AY23" s="13" t="n">
         <v>77381.41</v>
       </c>
+      <c r="AZ23" s="13" t="n">
+        <v>77411.88</v>
+      </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="3" t="n">
@@ -3723,6 +3783,7 @@
       <c r="AW24" s="13" t="n"/>
       <c r="AX24" s="13" t="n"/>
       <c r="AY24" s="13" t="n"/>
+      <c r="AZ24" s="13" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -3876,6 +3937,9 @@
         <v>49.88</v>
       </c>
       <c r="AY25" s="13" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="AZ25" s="13" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -3981,6 +4045,9 @@
       <c r="AY26" s="13" t="n">
         <v>25067.09</v>
       </c>
+      <c r="AZ26" s="13" t="n">
+        <v>25067.09</v>
+      </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -4082,6 +4149,7 @@
       <c r="AW27" s="13" t="n"/>
       <c r="AX27" s="13" t="n"/>
       <c r="AY27" s="13" t="n"/>
+      <c r="AZ27" s="13" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -4235,6 +4303,9 @@
         <v>92.09</v>
       </c>
       <c r="AY28" s="13" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="AZ28" s="13" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -4344,6 +4415,9 @@
       <c r="AY29" s="13" t="n">
         <v>67242.73</v>
       </c>
+      <c r="AZ29" s="13" t="n">
+        <v>67242.73</v>
+      </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="3" t="n">
@@ -4445,6 +4519,7 @@
       <c r="AW30" s="13" t="n"/>
       <c r="AX30" s="13" t="n"/>
       <c r="AY30" s="13" t="n"/>
+      <c r="AZ30" s="13" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -4598,6 +4673,9 @@
         <v>56.35</v>
       </c>
       <c r="AY31" s="13" t="n">
+        <v>51.18</v>
+      </c>
+      <c r="AZ31" s="13" t="n">
         <v>51.18</v>
       </c>
     </row>
@@ -4707,6 +4785,9 @@
       <c r="AY32" s="13" t="n">
         <v>5190.42</v>
       </c>
+      <c r="AZ32" s="13" t="n">
+        <v>5198.15</v>
+      </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
       <c r="A33" s="3" t="n">
@@ -4808,6 +4889,7 @@
       <c r="AW33" s="13" t="n"/>
       <c r="AX33" s="13" t="n"/>
       <c r="AY33" s="13" t="n"/>
+      <c r="AZ33" s="13" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -4961,6 +5043,9 @@
         <v>70.95999999999999</v>
       </c>
       <c r="AY34" s="13" t="n">
+        <v>72.67</v>
+      </c>
+      <c r="AZ34" s="13" t="n">
         <v>72.67</v>
       </c>
     </row>
@@ -5070,6 +5155,9 @@
       <c r="AY35" s="13" t="n">
         <v>10929.97</v>
       </c>
+      <c r="AZ35" s="13" t="n">
+        <v>10999.18</v>
+      </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="3" t="n">
@@ -5171,6 +5259,7 @@
       <c r="AW36" s="13" t="n"/>
       <c r="AX36" s="13" t="n"/>
       <c r="AY36" s="13" t="n"/>
+      <c r="AZ36" s="13" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -5324,6 +5413,9 @@
         <v>56.17</v>
       </c>
       <c r="AY37" s="13" t="n">
+        <v>58.26</v>
+      </c>
+      <c r="AZ37" s="13" t="n">
         <v>58.26</v>
       </c>
     </row>
@@ -5433,6 +5525,9 @@
       <c r="AY38" s="13" t="n">
         <v>10327.58</v>
       </c>
+      <c r="AZ38" s="13" t="n">
+        <v>10327.58</v>
+      </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
       <c r="A39" s="3" t="n">
@@ -5534,6 +5629,7 @@
       <c r="AW39" s="13" t="n"/>
       <c r="AX39" s="13" t="n"/>
       <c r="AY39" s="13" t="n"/>
+      <c r="AZ39" s="13" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -5687,6 +5783,9 @@
         <v>60.19</v>
       </c>
       <c r="AY40" s="13" t="n">
+        <v>53.87</v>
+      </c>
+      <c r="AZ40" s="13" t="n">
         <v>53.87</v>
       </c>
     </row>
@@ -5796,6 +5895,9 @@
       <c r="AY41" s="13" t="n">
         <v>2979.1</v>
       </c>
+      <c r="AZ41" s="13" t="n">
+        <v>2979.1</v>
+      </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
       <c r="A42" s="3" t="n">
@@ -5897,6 +5999,7 @@
       <c r="AW42" s="13" t="n"/>
       <c r="AX42" s="13" t="n"/>
       <c r="AY42" s="13" t="n"/>
+      <c r="AZ42" s="13" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -6050,6 +6153,9 @@
         <v>78.56</v>
       </c>
       <c r="AY43" s="13" t="n">
+        <v>67.11</v>
+      </c>
+      <c r="AZ43" s="13" t="n">
         <v>67.11</v>
       </c>
     </row>
@@ -6159,6 +6265,9 @@
       <c r="AY44" s="13" t="n">
         <v>6698.78</v>
       </c>
+      <c r="AZ44" s="13" t="n">
+        <v>6698.78</v>
+      </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
       <c r="A45" s="3" t="n">
@@ -6260,6 +6369,7 @@
       <c r="AW45" s="13" t="n"/>
       <c r="AX45" s="13" t="n"/>
       <c r="AY45" s="13" t="n"/>
+      <c r="AZ45" s="13" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -6413,6 +6523,9 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="AY46" s="13" t="n">
+        <v>21.69</v>
+      </c>
+      <c r="AZ46" s="13" t="n">
         <v>21.69</v>
       </c>
     </row>
@@ -6522,6 +6635,9 @@
       <c r="AY47" s="13" t="n">
         <v>31877.53</v>
       </c>
+      <c r="AZ47" s="13" t="n">
+        <v>31877.53</v>
+      </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
       <c r="A48" s="3" t="n">
@@ -6623,6 +6739,7 @@
       <c r="AW48" s="13" t="n"/>
       <c r="AX48" s="13" t="n"/>
       <c r="AY48" s="13" t="n"/>
+      <c r="AZ48" s="13" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -6776,6 +6893,9 @@
         <v>61.98</v>
       </c>
       <c r="AY49" s="13" t="n">
+        <v>58.25</v>
+      </c>
+      <c r="AZ49" s="13" t="n">
         <v>58.25</v>
       </c>
     </row>
@@ -6885,6 +7005,9 @@
       <c r="AY50" s="13" t="n">
         <v>3916.3</v>
       </c>
+      <c r="AZ50" s="13" t="n">
+        <v>3934.46</v>
+      </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
       <c r="A51" s="3" t="n">
@@ -6986,6 +7109,7 @@
       <c r="AW51" s="13" t="n"/>
       <c r="AX51" s="13" t="n"/>
       <c r="AY51" s="13" t="n"/>
+      <c r="AZ51" s="13" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -7139,6 +7263,9 @@
         <v>62.17</v>
       </c>
       <c r="AY52" s="13" t="n">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="AZ52" s="13" t="n">
         <v>66.40000000000001</v>
       </c>
     </row>
@@ -7248,6 +7375,9 @@
       <c r="AY53" s="13" t="n">
         <v>3693.2</v>
       </c>
+      <c r="AZ53" s="13" t="n">
+        <v>3711.83</v>
+      </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
       <c r="A54" s="3" t="n">
@@ -7349,6 +7479,7 @@
       <c r="AW54" s="13" t="n"/>
       <c r="AX54" s="13" t="n"/>
       <c r="AY54" s="13" t="n"/>
+      <c r="AZ54" s="13" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -7502,6 +7633,9 @@
         <v>5.94</v>
       </c>
       <c r="AY55" s="13" t="n">
+        <v>7.35</v>
+      </c>
+      <c r="AZ55" s="13" t="n">
         <v>7.35</v>
       </c>
     </row>
@@ -7611,6 +7745,9 @@
       <c r="AY56" s="13" t="n">
         <v>6118.22</v>
       </c>
+      <c r="AZ56" s="13" t="n">
+        <v>6124.59</v>
+      </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
       <c r="A57" s="3" t="n">
@@ -7712,6 +7849,7 @@
       <c r="AW57" s="13" t="n"/>
       <c r="AX57" s="13" t="n"/>
       <c r="AY57" s="13" t="n"/>
+      <c r="AZ57" s="13" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -7865,6 +8003,9 @@
         <v>28.8</v>
       </c>
       <c r="AY58" s="13" t="n">
+        <v>29.26</v>
+      </c>
+      <c r="AZ58" s="13" t="n">
         <v>29.26</v>
       </c>
     </row>
@@ -7974,6 +8115,9 @@
       <c r="AY59" s="13" t="n">
         <v>7734.35</v>
       </c>
+      <c r="AZ59" s="13" t="n">
+        <v>7744.71</v>
+      </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
       <c r="A60" s="3" t="n">
@@ -8075,6 +8219,7 @@
       <c r="AW60" s="13" t="n"/>
       <c r="AX60" s="13" t="n"/>
       <c r="AY60" s="13" t="n"/>
+      <c r="AZ60" s="13" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -8228,6 +8373,9 @@
         <v>5.41</v>
       </c>
       <c r="AY61" s="13" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="AZ61" s="13" t="n">
         <v>0.86</v>
       </c>
     </row>
@@ -8337,6 +8485,9 @@
       <c r="AY62" s="13" t="n">
         <v>10285.78</v>
       </c>
+      <c r="AZ62" s="13" t="n">
+        <v>10291</v>
+      </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
       <c r="A63" s="3" t="n">
@@ -8438,6 +8589,7 @@
       <c r="AW63" s="13" t="n"/>
       <c r="AX63" s="13" t="n"/>
       <c r="AY63" s="13" t="n"/>
+      <c r="AZ63" s="13" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -8591,6 +8743,9 @@
         <v>32.89</v>
       </c>
       <c r="AY64" s="13" t="n">
+        <v>17.66</v>
+      </c>
+      <c r="AZ64" s="13" t="n">
         <v>17.66</v>
       </c>
     </row>
@@ -8700,6 +8855,9 @@
       <c r="AY65" s="13" t="n">
         <v>11475.31</v>
       </c>
+      <c r="AZ65" s="13" t="n">
+        <v>11482.55</v>
+      </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
       <c r="A66" s="3" t="n">
@@ -8801,6 +8959,7 @@
       <c r="AW66" s="13" t="n"/>
       <c r="AX66" s="13" t="n"/>
       <c r="AY66" s="13" t="n"/>
+      <c r="AZ66" s="13" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -8954,6 +9113,9 @@
         <v>16.91</v>
       </c>
       <c r="AY67" s="13" t="n">
+        <v>6.17</v>
+      </c>
+      <c r="AZ67" s="13" t="n">
         <v>6.17</v>
       </c>
     </row>
@@ -9063,6 +9225,9 @@
       <c r="AY68" s="13" t="n">
         <v>6080.72</v>
       </c>
+      <c r="AZ68" s="13" t="n">
+        <v>6082.38</v>
+      </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
       <c r="A69" s="3" t="n">
@@ -9164,6 +9329,7 @@
       <c r="AW69" s="13" t="n"/>
       <c r="AX69" s="13" t="n"/>
       <c r="AY69" s="13" t="n"/>
+      <c r="AZ69" s="13" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -9317,6 +9483,9 @@
         <v>15.84</v>
       </c>
       <c r="AY70" s="13" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="AZ70" s="13" t="n">
         <v>7.8</v>
       </c>
     </row>
@@ -9426,6 +9595,9 @@
       <c r="AY71" s="13" t="n">
         <v>11956.6</v>
       </c>
+      <c r="AZ71" s="13" t="n">
+        <v>11958.88</v>
+      </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
       <c r="A72" s="3" t="n">
@@ -9527,6 +9699,7 @@
       <c r="AW72" s="13" t="n"/>
       <c r="AX72" s="13" t="n"/>
       <c r="AY72" s="13" t="n"/>
+      <c r="AZ72" s="13" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -9680,6 +9853,9 @@
         <v>56.16</v>
       </c>
       <c r="AY73" s="13" t="n">
+        <v>52.15</v>
+      </c>
+      <c r="AZ73" s="13" t="n">
         <v>52.15</v>
       </c>
     </row>
@@ -9789,6 +9965,9 @@
       <c r="AY74" s="13" t="n">
         <v>15569.82</v>
       </c>
+      <c r="AZ74" s="13" t="n">
+        <v>13733.6</v>
+      </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
       <c r="A75" s="3" t="n">
@@ -9890,6 +10069,7 @@
       <c r="AW75" s="13" t="n"/>
       <c r="AX75" s="13" t="n"/>
       <c r="AY75" s="13" t="n"/>
+      <c r="AZ75" s="13" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -10043,6 +10223,9 @@
         <v>3.22</v>
       </c>
       <c r="AY76" s="13" t="n">
+        <v>3.29</v>
+      </c>
+      <c r="AZ76" s="13" t="n">
         <v>3.29</v>
       </c>
     </row>
@@ -10152,6 +10335,9 @@
       <c r="AY77" s="13" t="n">
         <v>6926.32</v>
       </c>
+      <c r="AZ77" s="13" t="n">
+        <v>6926.37</v>
+      </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
       <c r="A78" s="3" t="n">
@@ -10253,6 +10439,7 @@
       <c r="AW78" s="13" t="n"/>
       <c r="AX78" s="13" t="n"/>
       <c r="AY78" s="13" t="n"/>
+      <c r="AZ78" s="13" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -10406,6 +10593,9 @@
         <v>2.5</v>
       </c>
       <c r="AY79" s="13" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="AZ79" s="13" t="n">
         <v>2.44</v>
       </c>
     </row>
@@ -10515,6 +10705,9 @@
       <c r="AY80" s="13" t="n">
         <v>8619.530000000001</v>
       </c>
+      <c r="AZ80" s="13" t="n">
+        <v>8632.85</v>
+      </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
       <c r="A81" s="3" t="n">
@@ -10616,6 +10809,7 @@
       <c r="AW81" s="13" t="n"/>
       <c r="AX81" s="13" t="n"/>
       <c r="AY81" s="13" t="n"/>
+      <c r="AZ81" s="13" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -10769,6 +10963,9 @@
         <v>16.73</v>
       </c>
       <c r="AY82" s="13" t="n">
+        <v>12.36</v>
+      </c>
+      <c r="AZ82" s="13" t="n">
         <v>12.36</v>
       </c>
     </row>
@@ -10878,6 +11075,9 @@
       <c r="AY83" s="13" t="n">
         <v>2237.93</v>
       </c>
+      <c r="AZ83" s="13" t="n">
+        <v>2631.9</v>
+      </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
       <c r="A84" s="3" t="n">
@@ -10979,6 +11179,7 @@
       <c r="AW84" s="13" t="n"/>
       <c r="AX84" s="13" t="n"/>
       <c r="AY84" s="13" t="n"/>
+      <c r="AZ84" s="13" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -11132,6 +11333,9 @@
         <v>25.09</v>
       </c>
       <c r="AY85" s="13" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="AZ85" s="13" t="n">
         <v>26.7</v>
       </c>
     </row>
@@ -11241,6 +11445,9 @@
       <c r="AY86" s="13" t="n">
         <v>5075.31</v>
       </c>
+      <c r="AZ86" s="13" t="n">
+        <v>5075.31</v>
+      </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
       <c r="A87" s="3" t="n">
@@ -11342,6 +11549,7 @@
       <c r="AW87" s="13" t="n"/>
       <c r="AX87" s="13" t="n"/>
       <c r="AY87" s="13" t="n"/>
+      <c r="AZ87" s="13" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -11495,6 +11703,9 @@
         <v>17.43</v>
       </c>
       <c r="AY88" s="13" t="n"/>
+      <c r="AZ88" s="13" t="n">
+        <v>19.84</v>
+      </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
       <c r="A89" s="1" t="n"/>
@@ -11600,6 +11811,9 @@
         <v>8199.790000000001</v>
       </c>
       <c r="AY89" s="13" t="n"/>
+      <c r="AZ89" s="13" t="n">
+        <v>8282.82</v>
+      </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
       <c r="A90" s="3" t="n">
@@ -11701,6 +11915,7 @@
       <c r="AW90" s="13" t="n"/>
       <c r="AX90" s="13" t="n"/>
       <c r="AY90" s="13" t="n"/>
+      <c r="AZ90" s="13" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -11854,6 +12069,9 @@
         <v>6.24</v>
       </c>
       <c r="AY91" s="13" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="AZ91" s="13" t="n">
         <v>3.1</v>
       </c>
     </row>
@@ -11963,6 +12181,9 @@
       <c r="AY92" s="13" t="n">
         <v>1113.51</v>
       </c>
+      <c r="AZ92" s="13" t="n">
+        <v>1113.51</v>
+      </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
       <c r="A93" s="3" t="n">
@@ -12064,6 +12285,7 @@
       <c r="AW93" s="13" t="n"/>
       <c r="AX93" s="13" t="n"/>
       <c r="AY93" s="13" t="n"/>
+      <c r="AZ93" s="13" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -12217,6 +12439,9 @@
         <v>10.15</v>
       </c>
       <c r="AY94" s="13" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="AZ94" s="13" t="n">
         <v>4.1</v>
       </c>
     </row>
@@ -12326,6 +12551,9 @@
       <c r="AY95" s="13" t="n">
         <v>13217.34</v>
       </c>
+      <c r="AZ95" s="13" t="n">
+        <v>13217.34</v>
+      </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
       <c r="A96" s="3" t="n">
@@ -12427,6 +12655,7 @@
       <c r="AW96" s="13" t="n"/>
       <c r="AX96" s="13" t="n"/>
       <c r="AY96" s="13" t="n"/>
+      <c r="AZ96" s="13" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -12580,6 +12809,9 @@
         <v>32.52</v>
       </c>
       <c r="AY97" s="13" t="n">
+        <v>45.23</v>
+      </c>
+      <c r="AZ97" s="13" t="n">
         <v>45.23</v>
       </c>
     </row>
@@ -12689,6 +12921,9 @@
       <c r="AY98" s="13" t="n">
         <v>3167.36</v>
       </c>
+      <c r="AZ98" s="13" t="n">
+        <v>3167.36</v>
+      </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
       <c r="A99" s="3" t="n">
@@ -12790,6 +13025,7 @@
       <c r="AW99" s="13" t="n"/>
       <c r="AX99" s="13" t="n"/>
       <c r="AY99" s="13" t="n"/>
+      <c r="AZ99" s="13" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -12943,6 +13179,9 @@
         <v>63.19</v>
       </c>
       <c r="AY100" s="13" t="n">
+        <v>39.34</v>
+      </c>
+      <c r="AZ100" s="13" t="n">
         <v>39.34</v>
       </c>
     </row>
@@ -13052,6 +13291,9 @@
       <c r="AY101" s="13" t="n">
         <v>2414.86</v>
       </c>
+      <c r="AZ101" s="13" t="n">
+        <v>2408.06</v>
+      </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
       <c r="A102" s="3" t="n">
@@ -13153,6 +13395,7 @@
       <c r="AW102" s="13" t="n"/>
       <c r="AX102" s="13" t="n"/>
       <c r="AY102" s="13" t="n"/>
+      <c r="AZ102" s="13" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -13306,6 +13549,9 @@
         <v>75.65000000000001</v>
       </c>
       <c r="AY103" s="13" t="n">
+        <v>18.94</v>
+      </c>
+      <c r="AZ103" s="13" t="n">
         <v>18.94</v>
       </c>
     </row>
@@ -13415,6 +13661,9 @@
       <c r="AY104" s="13" t="n">
         <v>2705.1</v>
       </c>
+      <c r="AZ104" s="13" t="n">
+        <v>2515.51</v>
+      </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
       <c r="A105" s="3" t="n">
@@ -13516,6 +13765,7 @@
       <c r="AW105" s="13" t="n"/>
       <c r="AX105" s="13" t="n"/>
       <c r="AY105" s="13" t="n"/>
+      <c r="AZ105" s="13" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -13669,6 +13919,9 @@
         <v>53.88</v>
       </c>
       <c r="AY106" s="13" t="n">
+        <v>38.53</v>
+      </c>
+      <c r="AZ106" s="13" t="n">
         <v>38.53</v>
       </c>
     </row>
@@ -13778,6 +14031,9 @@
       <c r="AY107" s="13" t="n">
         <v>2601.88</v>
       </c>
+      <c r="AZ107" s="13" t="n">
+        <v>2685.35</v>
+      </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
       <c r="A108" s="3" t="n">
@@ -13879,6 +14135,7 @@
       <c r="AW108" s="13" t="n"/>
       <c r="AX108" s="13" t="n"/>
       <c r="AY108" s="13" t="n"/>
+      <c r="AZ108" s="13" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -14032,6 +14289,9 @@
         <v>50.11</v>
       </c>
       <c r="AY109" s="13" t="n">
+        <v>59.53</v>
+      </c>
+      <c r="AZ109" s="13" t="n">
         <v>59.53</v>
       </c>
     </row>
@@ -14141,6 +14401,9 @@
       <c r="AY110" s="13" t="n">
         <v>1908.79</v>
       </c>
+      <c r="AZ110" s="13" t="n">
+        <v>1908.95</v>
+      </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
       <c r="A111" s="3" t="n">
@@ -14242,6 +14505,7 @@
       <c r="AW111" s="13" t="n"/>
       <c r="AX111" s="13" t="n"/>
       <c r="AY111" s="13" t="n"/>
+      <c r="AZ111" s="13" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -14395,6 +14659,9 @@
         <v>25.97</v>
       </c>
       <c r="AY112" s="13" t="n">
+        <v>20.44</v>
+      </c>
+      <c r="AZ112" s="13" t="n">
         <v>20.44</v>
       </c>
     </row>
@@ -14504,6 +14771,9 @@
       <c r="AY113" s="13" t="n">
         <v>8566.25</v>
       </c>
+      <c r="AZ113" s="13" t="n">
+        <v>8566.25</v>
+      </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
       <c r="A114" s="3" t="n">
@@ -14605,6 +14875,7 @@
       <c r="AW114" s="13" t="n"/>
       <c r="AX114" s="13" t="n"/>
       <c r="AY114" s="13" t="n"/>
+      <c r="AZ114" s="13" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -14758,6 +15029,9 @@
         <v>95.47</v>
       </c>
       <c r="AY115" s="13" t="n">
+        <v>99.28</v>
+      </c>
+      <c r="AZ115" s="13" t="n">
         <v>99.28</v>
       </c>
     </row>
@@ -14851,6 +15125,9 @@
       </c>
       <c r="AY116" s="13" t="n">
         <v>16304.17</v>
+      </c>
+      <c r="AZ116" s="13" t="n">
+        <v>16269.28</v>
       </c>
     </row>
     <row r="117">
@@ -14908,6 +15185,7 @@
       <c r="AW117" s="13" t="n"/>
       <c r="AX117" s="13" t="n"/>
       <c r="AY117" s="13" t="n"/>
+      <c r="AZ117" s="13" t="n"/>
     </row>
     <row r="118">
       <c r="P118" s="13" t="n">
@@ -15018,6 +15296,9 @@
       <c r="AY118" s="13" t="n">
         <v>62.89</v>
       </c>
+      <c r="AZ118" s="13" t="n">
+        <v>62.89</v>
+      </c>
     </row>
     <row r="119">
       <c r="Y119" s="13" t="n">
@@ -15100,12 +15381,16 @@
       </c>
       <c r="AY119" s="13" t="n">
         <v>12165.01</v>
+      </c>
+      <c r="AZ119" s="13" t="n">
+        <v>12152.43</v>
       </c>
     </row>
     <row r="120">
       <c r="AW120" s="13" t="n"/>
       <c r="AX120" s="13" t="n"/>
       <c r="AY120" s="13" t="n"/>
+      <c r="AZ120" s="13" t="n"/>
     </row>
     <row r="121">
       <c r="AW121" s="13" t="n">
@@ -15117,6 +15402,9 @@
       <c r="AY121" s="13" t="n">
         <v>27.69</v>
       </c>
+      <c r="AZ121" s="13" t="n">
+        <v>27.69</v>
+      </c>
     </row>
     <row r="122">
       <c r="AW122" s="13" t="n">
@@ -15127,12 +15415,16 @@
       </c>
       <c r="AY122" s="13" t="n">
         <v>1821.31</v>
+      </c>
+      <c r="AZ122" s="13" t="n">
+        <v>1817.47</v>
       </c>
     </row>
     <row r="123">
       <c r="AW123" s="13" t="n"/>
       <c r="AX123" s="13" t="n"/>
       <c r="AY123" s="13" t="n"/>
+      <c r="AZ123" s="13" t="n"/>
     </row>
     <row r="124">
       <c r="AW124" s="13" t="n">
@@ -15144,6 +15436,9 @@
       <c r="AY124" s="13" t="n">
         <v>15.54</v>
       </c>
+      <c r="AZ124" s="13" t="n">
+        <v>15.54</v>
+      </c>
     </row>
     <row r="125">
       <c r="AW125" s="13" t="n">
@@ -15154,12 +15449,16 @@
       </c>
       <c r="AY125" s="13" t="n">
         <v>768.65</v>
+      </c>
+      <c r="AZ125" s="13" t="n">
+        <v>768.13</v>
       </c>
     </row>
     <row r="126">
       <c r="AW126" s="13" t="n"/>
       <c r="AX126" s="13" t="n"/>
       <c r="AY126" s="13" t="n"/>
+      <c r="AZ126" s="13" t="n"/>
     </row>
     <row r="127">
       <c r="AW127" s="13" t="n">
@@ -15171,6 +15470,9 @@
       <c r="AY127" s="13" t="n">
         <v>58.22</v>
       </c>
+      <c r="AZ127" s="13" t="n">
+        <v>58.22</v>
+      </c>
     </row>
     <row r="128">
       <c r="AW128" s="13" t="n">
@@ -15181,12 +15483,16 @@
       </c>
       <c r="AY128" s="13" t="n">
         <v>2678.46</v>
+      </c>
+      <c r="AZ128" s="13" t="n">
+        <v>2674.72</v>
       </c>
     </row>
     <row r="129">
       <c r="AW129" s="13" t="n"/>
       <c r="AX129" s="13" t="n"/>
       <c r="AY129" s="13" t="n"/>
+      <c r="AZ129" s="13" t="n"/>
     </row>
     <row r="130">
       <c r="AW130" s="13" t="n">
@@ -15198,6 +15504,9 @@
       <c r="AY130" s="13" t="n">
         <v>20.78</v>
       </c>
+      <c r="AZ130" s="13" t="n">
+        <v>20.78</v>
+      </c>
     </row>
     <row r="131">
       <c r="AW131" s="13" t="n">
@@ -15208,12 +15517,16 @@
       </c>
       <c r="AY131" s="13" t="n">
         <v>3568.39</v>
+      </c>
+      <c r="AZ131" s="13" t="n">
+        <v>3567.08</v>
       </c>
     </row>
     <row r="132">
       <c r="AW132" s="13" t="n"/>
       <c r="AX132" s="13" t="n"/>
       <c r="AY132" s="13" t="n"/>
+      <c r="AZ132" s="13" t="n"/>
     </row>
     <row r="133">
       <c r="AW133" s="13" t="n">
@@ -15225,6 +15538,7 @@
       <c r="AY133" s="13" t="n">
         <v>2.09</v>
       </c>
+      <c r="AZ133" s="13" t="n"/>
     </row>
     <row r="134">
       <c r="AW134" s="13" t="n">
@@ -15236,11 +15550,13 @@
       <c r="AY134" s="13" t="n">
         <v>2362.93</v>
       </c>
+      <c r="AZ134" s="13" t="n"/>
     </row>
     <row r="135">
       <c r="AW135" s="13" t="n"/>
       <c r="AX135" s="13" t="n"/>
       <c r="AY135" s="13" t="n"/>
+      <c r="AZ135" s="13" t="n"/>
     </row>
     <row r="136">
       <c r="AW136" s="13" t="n">
@@ -15252,6 +15568,9 @@
       <c r="AY136" s="13" t="n">
         <v>15</v>
       </c>
+      <c r="AZ136" s="13" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="137">
       <c r="AW137" s="13" t="n">
@@ -15261,6 +15580,9 @@
         <v>7193.45</v>
       </c>
       <c r="AY137" s="13" t="n">
+        <v>6280.28</v>
+      </c>
+      <c r="AZ137" s="13" t="n">
         <v>6280.28</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-07-13 07:33:59]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ137"/>
+  <dimension ref="A1:BA137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="15"/>
@@ -569,6 +569,7 @@
     <col width="15" customWidth="1" min="50" max="50"/>
     <col width="15" customWidth="1" min="51" max="51"/>
     <col width="15" customWidth="1" min="52" max="52"/>
+    <col width="15" customWidth="1" min="53" max="53"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -832,6 +833,11 @@
           <t>2026/07/13</t>
         </is>
       </c>
+      <c r="BA1" s="13" t="inlineStr">
+        <is>
+          <t>2026/07/13</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1094,6 +1100,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BA2" s="14" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1252,6 +1263,9 @@
       <c r="AZ3" s="13" t="n">
         <v>66.86</v>
       </c>
+      <c r="BA3" s="13" t="n">
+        <v>66.86</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1409,6 +1423,9 @@
       </c>
       <c r="AZ4" s="13" t="n">
         <v>3914.85</v>
+      </c>
+      <c r="BA4" s="13" t="n">
+        <v>3913.79</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1464,6 +1481,7 @@
       <c r="AX5" s="13" t="n"/>
       <c r="AY5" s="13" t="n"/>
       <c r="AZ5" s="13" t="n"/>
+      <c r="BA5" s="13" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1566,6 +1584,7 @@
       <c r="AX6" s="13" t="n"/>
       <c r="AY6" s="13" t="n"/>
       <c r="AZ6" s="13" t="n"/>
+      <c r="BA6" s="13" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1722,6 +1741,9 @@
         <v>64.93000000000001</v>
       </c>
       <c r="AZ7" s="13" t="n">
+        <v>64.93000000000001</v>
+      </c>
+      <c r="BA7" s="13" t="n">
         <v>64.93000000000001</v>
       </c>
     </row>
@@ -1834,6 +1856,9 @@
       <c r="AZ8" s="13" t="n">
         <v>5841.28</v>
       </c>
+      <c r="BA8" s="13" t="n">
+        <v>5851.82</v>
+      </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -1936,6 +1961,7 @@
       <c r="AX9" s="13" t="n"/>
       <c r="AY9" s="13" t="n"/>
       <c r="AZ9" s="13" t="n"/>
+      <c r="BA9" s="13" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2092,6 +2118,9 @@
         <v>55.74</v>
       </c>
       <c r="AZ10" s="13" t="n">
+        <v>55.74</v>
+      </c>
+      <c r="BA10" s="13" t="n">
         <v>55.74</v>
       </c>
     </row>
@@ -2204,6 +2233,9 @@
       <c r="AZ11" s="13" t="n">
         <v>4685.33</v>
       </c>
+      <c r="BA11" s="13" t="n">
+        <v>4695.38</v>
+      </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -2306,6 +2338,7 @@
       <c r="AX12" s="13" t="n"/>
       <c r="AY12" s="13" t="n"/>
       <c r="AZ12" s="13" t="n"/>
+      <c r="BA12" s="13" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2462,6 +2495,9 @@
         <v>70.51000000000001</v>
       </c>
       <c r="AZ13" s="13" t="n">
+        <v>70.51000000000001</v>
+      </c>
+      <c r="BA13" s="13" t="n">
         <v>70.51000000000001</v>
       </c>
     </row>
@@ -2574,6 +2610,9 @@
       <c r="AZ14" s="13" t="n">
         <v>8135.86</v>
       </c>
+      <c r="BA14" s="13" t="n">
+        <v>8138.14</v>
+      </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -2676,6 +2715,7 @@
       <c r="AX15" s="13" t="n"/>
       <c r="AY15" s="13" t="n"/>
       <c r="AZ15" s="13" t="n"/>
+      <c r="BA15" s="13" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -2832,6 +2872,9 @@
         <v>33.74</v>
       </c>
       <c r="AZ16" s="13" t="n">
+        <v>33.74</v>
+      </c>
+      <c r="BA16" s="13" t="n">
         <v>33.74</v>
       </c>
     </row>
@@ -2944,6 +2987,9 @@
       <c r="AZ17" s="13" t="n">
         <v>2563.76</v>
       </c>
+      <c r="BA17" s="13" t="n">
+        <v>2568.26</v>
+      </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="3" t="n">
@@ -3046,6 +3092,7 @@
       <c r="AX18" s="13" t="n"/>
       <c r="AY18" s="13" t="n"/>
       <c r="AZ18" s="13" t="n"/>
+      <c r="BA18" s="13" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -3202,6 +3249,9 @@
         <v>87.13</v>
       </c>
       <c r="AZ19" s="13" t="n">
+        <v>87.13</v>
+      </c>
+      <c r="BA19" s="13" t="n">
         <v>87.13</v>
       </c>
     </row>
@@ -3314,6 +3364,9 @@
       <c r="AZ20" s="13" t="n">
         <v>7575.39</v>
       </c>
+      <c r="BA20" s="13" t="n">
+        <v>7575.39</v>
+      </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -3416,6 +3469,7 @@
       <c r="AX21" s="13" t="n"/>
       <c r="AY21" s="13" t="n"/>
       <c r="AZ21" s="13" t="n"/>
+      <c r="BA21" s="13" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -3570,6 +3624,9 @@
         <v>36.34</v>
       </c>
       <c r="AZ22" s="13" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BA22" s="13" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -3682,6 +3739,9 @@
       <c r="AZ23" s="13" t="n">
         <v>77411.88</v>
       </c>
+      <c r="BA23" s="13" t="n">
+        <v>77632.78999999999</v>
+      </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="3" t="n">
@@ -3784,6 +3844,7 @@
       <c r="AX24" s="13" t="n"/>
       <c r="AY24" s="13" t="n"/>
       <c r="AZ24" s="13" t="n"/>
+      <c r="BA24" s="13" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -3940,6 +4001,9 @@
         <v>49.88</v>
       </c>
       <c r="AZ25" s="13" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BA25" s="13" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -4048,6 +4112,9 @@
       <c r="AZ26" s="13" t="n">
         <v>25067.09</v>
       </c>
+      <c r="BA26" s="13" t="n">
+        <v>25041.78</v>
+      </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -4150,6 +4217,7 @@
       <c r="AX27" s="13" t="n"/>
       <c r="AY27" s="13" t="n"/>
       <c r="AZ27" s="13" t="n"/>
+      <c r="BA27" s="13" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -4306,6 +4374,9 @@
         <v>92.09</v>
       </c>
       <c r="AZ28" s="13" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BA28" s="13" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -4418,6 +4489,9 @@
       <c r="AZ29" s="13" t="n">
         <v>67242.73</v>
       </c>
+      <c r="BA29" s="13" t="n">
+        <v>67242.73</v>
+      </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="3" t="n">
@@ -4520,6 +4594,7 @@
       <c r="AX30" s="13" t="n"/>
       <c r="AY30" s="13" t="n"/>
       <c r="AZ30" s="13" t="n"/>
+      <c r="BA30" s="13" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -4676,6 +4751,9 @@
         <v>51.18</v>
       </c>
       <c r="AZ31" s="13" t="n">
+        <v>51.18</v>
+      </c>
+      <c r="BA31" s="13" t="n">
         <v>51.18</v>
       </c>
     </row>
@@ -4788,6 +4866,9 @@
       <c r="AZ32" s="13" t="n">
         <v>5198.15</v>
       </c>
+      <c r="BA32" s="13" t="n">
+        <v>5198.11</v>
+      </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
       <c r="A33" s="3" t="n">
@@ -4890,6 +4971,7 @@
       <c r="AX33" s="13" t="n"/>
       <c r="AY33" s="13" t="n"/>
       <c r="AZ33" s="13" t="n"/>
+      <c r="BA33" s="13" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -5046,6 +5128,9 @@
         <v>72.67</v>
       </c>
       <c r="AZ34" s="13" t="n">
+        <v>72.67</v>
+      </c>
+      <c r="BA34" s="13" t="n">
         <v>72.67</v>
       </c>
     </row>
@@ -5158,6 +5243,9 @@
       <c r="AZ35" s="13" t="n">
         <v>10999.18</v>
       </c>
+      <c r="BA35" s="13" t="n">
+        <v>11025.22</v>
+      </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="3" t="n">
@@ -5260,6 +5348,7 @@
       <c r="AX36" s="13" t="n"/>
       <c r="AY36" s="13" t="n"/>
       <c r="AZ36" s="13" t="n"/>
+      <c r="BA36" s="13" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -5416,6 +5505,9 @@
         <v>58.26</v>
       </c>
       <c r="AZ37" s="13" t="n">
+        <v>58.26</v>
+      </c>
+      <c r="BA37" s="13" t="n">
         <v>58.26</v>
       </c>
     </row>
@@ -5528,6 +5620,9 @@
       <c r="AZ38" s="13" t="n">
         <v>10327.58</v>
       </c>
+      <c r="BA38" s="13" t="n">
+        <v>10327.58</v>
+      </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
       <c r="A39" s="3" t="n">
@@ -5630,6 +5725,7 @@
       <c r="AX39" s="13" t="n"/>
       <c r="AY39" s="13" t="n"/>
       <c r="AZ39" s="13" t="n"/>
+      <c r="BA39" s="13" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -5786,6 +5882,9 @@
         <v>53.87</v>
       </c>
       <c r="AZ40" s="13" t="n">
+        <v>53.87</v>
+      </c>
+      <c r="BA40" s="13" t="n">
         <v>53.87</v>
       </c>
     </row>
@@ -5898,6 +5997,9 @@
       <c r="AZ41" s="13" t="n">
         <v>2979.1</v>
       </c>
+      <c r="BA41" s="13" t="n">
+        <v>2979.1</v>
+      </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
       <c r="A42" s="3" t="n">
@@ -6000,6 +6102,7 @@
       <c r="AX42" s="13" t="n"/>
       <c r="AY42" s="13" t="n"/>
       <c r="AZ42" s="13" t="n"/>
+      <c r="BA42" s="13" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -6156,6 +6259,9 @@
         <v>67.11</v>
       </c>
       <c r="AZ43" s="13" t="n">
+        <v>67.11</v>
+      </c>
+      <c r="BA43" s="13" t="n">
         <v>67.11</v>
       </c>
     </row>
@@ -6268,6 +6374,9 @@
       <c r="AZ44" s="13" t="n">
         <v>6698.78</v>
       </c>
+      <c r="BA44" s="13" t="n">
+        <v>6698.78</v>
+      </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
       <c r="A45" s="3" t="n">
@@ -6370,6 +6479,7 @@
       <c r="AX45" s="13" t="n"/>
       <c r="AY45" s="13" t="n"/>
       <c r="AZ45" s="13" t="n"/>
+      <c r="BA45" s="13" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -6526,6 +6636,9 @@
         <v>21.69</v>
       </c>
       <c r="AZ46" s="13" t="n">
+        <v>21.69</v>
+      </c>
+      <c r="BA46" s="13" t="n">
         <v>21.69</v>
       </c>
     </row>
@@ -6638,6 +6751,9 @@
       <c r="AZ47" s="13" t="n">
         <v>31877.53</v>
       </c>
+      <c r="BA47" s="13" t="n">
+        <v>32587.01</v>
+      </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
       <c r="A48" s="3" t="n">
@@ -6740,6 +6856,7 @@
       <c r="AX48" s="13" t="n"/>
       <c r="AY48" s="13" t="n"/>
       <c r="AZ48" s="13" t="n"/>
+      <c r="BA48" s="13" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -6896,6 +7013,9 @@
         <v>58.25</v>
       </c>
       <c r="AZ49" s="13" t="n">
+        <v>58.25</v>
+      </c>
+      <c r="BA49" s="13" t="n">
         <v>58.25</v>
       </c>
     </row>
@@ -7008,6 +7128,9 @@
       <c r="AZ50" s="13" t="n">
         <v>3934.46</v>
       </c>
+      <c r="BA50" s="13" t="n">
+        <v>3952.48</v>
+      </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
       <c r="A51" s="3" t="n">
@@ -7110,6 +7233,7 @@
       <c r="AX51" s="13" t="n"/>
       <c r="AY51" s="13" t="n"/>
       <c r="AZ51" s="13" t="n"/>
+      <c r="BA51" s="13" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -7266,6 +7390,9 @@
         <v>66.40000000000001</v>
       </c>
       <c r="AZ52" s="13" t="n">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="BA52" s="13" t="n">
         <v>66.40000000000001</v>
       </c>
     </row>
@@ -7378,6 +7505,9 @@
       <c r="AZ53" s="13" t="n">
         <v>3711.83</v>
       </c>
+      <c r="BA53" s="13" t="n">
+        <v>3723.52</v>
+      </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
       <c r="A54" s="3" t="n">
@@ -7480,6 +7610,7 @@
       <c r="AX54" s="13" t="n"/>
       <c r="AY54" s="13" t="n"/>
       <c r="AZ54" s="13" t="n"/>
+      <c r="BA54" s="13" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -7636,6 +7767,9 @@
         <v>7.35</v>
       </c>
       <c r="AZ55" s="13" t="n">
+        <v>7.35</v>
+      </c>
+      <c r="BA55" s="13" t="n">
         <v>7.35</v>
       </c>
     </row>
@@ -7748,6 +7882,9 @@
       <c r="AZ56" s="13" t="n">
         <v>6124.59</v>
       </c>
+      <c r="BA56" s="13" t="n">
+        <v>6128.38</v>
+      </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
       <c r="A57" s="3" t="n">
@@ -7850,6 +7987,7 @@
       <c r="AX57" s="13" t="n"/>
       <c r="AY57" s="13" t="n"/>
       <c r="AZ57" s="13" t="n"/>
+      <c r="BA57" s="13" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -8006,6 +8144,9 @@
         <v>29.26</v>
       </c>
       <c r="AZ58" s="13" t="n">
+        <v>29.26</v>
+      </c>
+      <c r="BA58" s="13" t="n">
         <v>29.26</v>
       </c>
     </row>
@@ -8118,6 +8259,9 @@
       <c r="AZ59" s="13" t="n">
         <v>7744.71</v>
       </c>
+      <c r="BA59" s="13" t="n">
+        <v>7756.03</v>
+      </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
       <c r="A60" s="3" t="n">
@@ -8220,6 +8364,7 @@
       <c r="AX60" s="13" t="n"/>
       <c r="AY60" s="13" t="n"/>
       <c r="AZ60" s="13" t="n"/>
+      <c r="BA60" s="13" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -8376,6 +8521,9 @@
         <v>0.86</v>
       </c>
       <c r="AZ61" s="13" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="BA61" s="13" t="n">
         <v>0.86</v>
       </c>
     </row>
@@ -8488,6 +8636,9 @@
       <c r="AZ62" s="13" t="n">
         <v>10291</v>
       </c>
+      <c r="BA62" s="13" t="n">
+        <v>10288.32</v>
+      </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
       <c r="A63" s="3" t="n">
@@ -8590,6 +8741,7 @@
       <c r="AX63" s="13" t="n"/>
       <c r="AY63" s="13" t="n"/>
       <c r="AZ63" s="13" t="n"/>
+      <c r="BA63" s="13" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -8746,6 +8898,9 @@
         <v>17.66</v>
       </c>
       <c r="AZ64" s="13" t="n">
+        <v>17.66</v>
+      </c>
+      <c r="BA64" s="13" t="n">
         <v>17.66</v>
       </c>
     </row>
@@ -8858,6 +9013,9 @@
       <c r="AZ65" s="13" t="n">
         <v>11482.55</v>
       </c>
+      <c r="BA65" s="13" t="n">
+        <v>11482.55</v>
+      </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
       <c r="A66" s="3" t="n">
@@ -8960,6 +9118,7 @@
       <c r="AX66" s="13" t="n"/>
       <c r="AY66" s="13" t="n"/>
       <c r="AZ66" s="13" t="n"/>
+      <c r="BA66" s="13" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -9116,6 +9275,9 @@
         <v>6.17</v>
       </c>
       <c r="AZ67" s="13" t="n">
+        <v>6.17</v>
+      </c>
+      <c r="BA67" s="13" t="n">
         <v>6.17</v>
       </c>
     </row>
@@ -9228,6 +9390,9 @@
       <c r="AZ68" s="13" t="n">
         <v>6082.38</v>
       </c>
+      <c r="BA68" s="13" t="n">
+        <v>6085.19</v>
+      </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
       <c r="A69" s="3" t="n">
@@ -9330,6 +9495,7 @@
       <c r="AX69" s="13" t="n"/>
       <c r="AY69" s="13" t="n"/>
       <c r="AZ69" s="13" t="n"/>
+      <c r="BA69" s="13" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -9486,6 +9652,9 @@
         <v>7.8</v>
       </c>
       <c r="AZ70" s="13" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="BA70" s="13" t="n">
         <v>7.8</v>
       </c>
     </row>
@@ -9598,6 +9767,9 @@
       <c r="AZ71" s="13" t="n">
         <v>11958.88</v>
       </c>
+      <c r="BA71" s="13" t="n">
+        <v>11953.61</v>
+      </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
       <c r="A72" s="3" t="n">
@@ -9700,6 +9872,7 @@
       <c r="AX72" s="13" t="n"/>
       <c r="AY72" s="13" t="n"/>
       <c r="AZ72" s="13" t="n"/>
+      <c r="BA72" s="13" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -9856,6 +10029,9 @@
         <v>52.15</v>
       </c>
       <c r="AZ73" s="13" t="n">
+        <v>52.15</v>
+      </c>
+      <c r="BA73" s="13" t="n">
         <v>52.15</v>
       </c>
     </row>
@@ -9968,6 +10144,9 @@
       <c r="AZ74" s="13" t="n">
         <v>13733.6</v>
       </c>
+      <c r="BA74" s="13" t="n">
+        <v>13897.48</v>
+      </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
       <c r="A75" s="3" t="n">
@@ -10070,6 +10249,7 @@
       <c r="AX75" s="13" t="n"/>
       <c r="AY75" s="13" t="n"/>
       <c r="AZ75" s="13" t="n"/>
+      <c r="BA75" s="13" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -10226,6 +10406,9 @@
         <v>3.29</v>
       </c>
       <c r="AZ76" s="13" t="n">
+        <v>3.29</v>
+      </c>
+      <c r="BA76" s="13" t="n">
         <v>3.29</v>
       </c>
     </row>
@@ -10338,6 +10521,9 @@
       <c r="AZ77" s="13" t="n">
         <v>6926.37</v>
       </c>
+      <c r="BA77" s="13" t="n">
+        <v>6926.37</v>
+      </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
       <c r="A78" s="3" t="n">
@@ -10440,6 +10626,7 @@
       <c r="AX78" s="13" t="n"/>
       <c r="AY78" s="13" t="n"/>
       <c r="AZ78" s="13" t="n"/>
+      <c r="BA78" s="13" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -10596,6 +10783,9 @@
         <v>2.44</v>
       </c>
       <c r="AZ79" s="13" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="BA79" s="13" t="n">
         <v>2.44</v>
       </c>
     </row>
@@ -10708,6 +10898,9 @@
       <c r="AZ80" s="13" t="n">
         <v>8632.85</v>
       </c>
+      <c r="BA80" s="13" t="n">
+        <v>8669.1</v>
+      </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
       <c r="A81" s="3" t="n">
@@ -10810,6 +11003,7 @@
       <c r="AX81" s="13" t="n"/>
       <c r="AY81" s="13" t="n"/>
       <c r="AZ81" s="13" t="n"/>
+      <c r="BA81" s="13" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -10966,6 +11160,9 @@
         <v>12.36</v>
       </c>
       <c r="AZ82" s="13" t="n">
+        <v>12.36</v>
+      </c>
+      <c r="BA82" s="13" t="n">
         <v>12.36</v>
       </c>
     </row>
@@ -11078,6 +11275,9 @@
       <c r="AZ83" s="13" t="n">
         <v>2631.9</v>
       </c>
+      <c r="BA83" s="13" t="n">
+        <v>2631.9</v>
+      </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
       <c r="A84" s="3" t="n">
@@ -11180,6 +11380,7 @@
       <c r="AX84" s="13" t="n"/>
       <c r="AY84" s="13" t="n"/>
       <c r="AZ84" s="13" t="n"/>
+      <c r="BA84" s="13" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -11336,6 +11537,9 @@
         <v>26.7</v>
       </c>
       <c r="AZ85" s="13" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="BA85" s="13" t="n">
         <v>26.7</v>
       </c>
     </row>
@@ -11448,6 +11652,9 @@
       <c r="AZ86" s="13" t="n">
         <v>5075.31</v>
       </c>
+      <c r="BA86" s="13" t="n">
+        <v>5075.31</v>
+      </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
       <c r="A87" s="3" t="n">
@@ -11550,6 +11757,7 @@
       <c r="AX87" s="13" t="n"/>
       <c r="AY87" s="13" t="n"/>
       <c r="AZ87" s="13" t="n"/>
+      <c r="BA87" s="13" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -11704,6 +11912,9 @@
       </c>
       <c r="AY88" s="13" t="n"/>
       <c r="AZ88" s="13" t="n">
+        <v>19.84</v>
+      </c>
+      <c r="BA88" s="13" t="n">
         <v>19.84</v>
       </c>
     </row>
@@ -11814,6 +12025,9 @@
       <c r="AZ89" s="13" t="n">
         <v>8282.82</v>
       </c>
+      <c r="BA89" s="13" t="n">
+        <v>8293.110000000001</v>
+      </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
       <c r="A90" s="3" t="n">
@@ -11916,6 +12130,7 @@
       <c r="AX90" s="13" t="n"/>
       <c r="AY90" s="13" t="n"/>
       <c r="AZ90" s="13" t="n"/>
+      <c r="BA90" s="13" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -12072,6 +12287,9 @@
         <v>3.1</v>
       </c>
       <c r="AZ91" s="13" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="BA91" s="13" t="n">
         <v>3.1</v>
       </c>
     </row>
@@ -12184,6 +12402,9 @@
       <c r="AZ92" s="13" t="n">
         <v>1113.51</v>
       </c>
+      <c r="BA92" s="13" t="n">
+        <v>1113.51</v>
+      </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
       <c r="A93" s="3" t="n">
@@ -12286,6 +12507,7 @@
       <c r="AX93" s="13" t="n"/>
       <c r="AY93" s="13" t="n"/>
       <c r="AZ93" s="13" t="n"/>
+      <c r="BA93" s="13" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -12442,6 +12664,9 @@
         <v>4.1</v>
       </c>
       <c r="AZ94" s="13" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="BA94" s="13" t="n">
         <v>4.1</v>
       </c>
     </row>
@@ -12554,6 +12779,9 @@
       <c r="AZ95" s="13" t="n">
         <v>13217.34</v>
       </c>
+      <c r="BA95" s="13" t="n">
+        <v>13217.34</v>
+      </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
       <c r="A96" s="3" t="n">
@@ -12656,6 +12884,7 @@
       <c r="AX96" s="13" t="n"/>
       <c r="AY96" s="13" t="n"/>
       <c r="AZ96" s="13" t="n"/>
+      <c r="BA96" s="13" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -12812,6 +13041,9 @@
         <v>45.23</v>
       </c>
       <c r="AZ97" s="13" t="n">
+        <v>45.23</v>
+      </c>
+      <c r="BA97" s="13" t="n">
         <v>45.23</v>
       </c>
     </row>
@@ -12924,6 +13156,9 @@
       <c r="AZ98" s="13" t="n">
         <v>3167.36</v>
       </c>
+      <c r="BA98" s="13" t="n">
+        <v>3167.36</v>
+      </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
       <c r="A99" s="3" t="n">
@@ -13026,6 +13261,7 @@
       <c r="AX99" s="13" t="n"/>
       <c r="AY99" s="13" t="n"/>
       <c r="AZ99" s="13" t="n"/>
+      <c r="BA99" s="13" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -13182,6 +13418,9 @@
         <v>39.34</v>
       </c>
       <c r="AZ100" s="13" t="n">
+        <v>39.34</v>
+      </c>
+      <c r="BA100" s="13" t="n">
         <v>39.34</v>
       </c>
     </row>
@@ -13294,6 +13533,9 @@
       <c r="AZ101" s="13" t="n">
         <v>2408.06</v>
       </c>
+      <c r="BA101" s="13" t="n">
+        <v>2412.49</v>
+      </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
       <c r="A102" s="3" t="n">
@@ -13396,6 +13638,7 @@
       <c r="AX102" s="13" t="n"/>
       <c r="AY102" s="13" t="n"/>
       <c r="AZ102" s="13" t="n"/>
+      <c r="BA102" s="13" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -13552,6 +13795,9 @@
         <v>18.94</v>
       </c>
       <c r="AZ103" s="13" t="n">
+        <v>18.94</v>
+      </c>
+      <c r="BA103" s="13" t="n">
         <v>18.94</v>
       </c>
     </row>
@@ -13664,6 +13910,9 @@
       <c r="AZ104" s="13" t="n">
         <v>2515.51</v>
       </c>
+      <c r="BA104" s="13" t="n">
+        <v>2554.52</v>
+      </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
       <c r="A105" s="3" t="n">
@@ -13766,6 +14015,7 @@
       <c r="AX105" s="13" t="n"/>
       <c r="AY105" s="13" t="n"/>
       <c r="AZ105" s="13" t="n"/>
+      <c r="BA105" s="13" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -13922,6 +14172,9 @@
         <v>38.53</v>
       </c>
       <c r="AZ106" s="13" t="n">
+        <v>38.53</v>
+      </c>
+      <c r="BA106" s="13" t="n">
         <v>38.53</v>
       </c>
     </row>
@@ -14034,6 +14287,9 @@
       <c r="AZ107" s="13" t="n">
         <v>2685.35</v>
       </c>
+      <c r="BA107" s="13" t="n">
+        <v>2571.96</v>
+      </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
       <c r="A108" s="3" t="n">
@@ -14136,6 +14392,7 @@
       <c r="AX108" s="13" t="n"/>
       <c r="AY108" s="13" t="n"/>
       <c r="AZ108" s="13" t="n"/>
+      <c r="BA108" s="13" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -14292,6 +14549,9 @@
         <v>59.53</v>
       </c>
       <c r="AZ109" s="13" t="n">
+        <v>59.53</v>
+      </c>
+      <c r="BA109" s="13" t="n">
         <v>59.53</v>
       </c>
     </row>
@@ -14404,6 +14664,9 @@
       <c r="AZ110" s="13" t="n">
         <v>1908.95</v>
       </c>
+      <c r="BA110" s="13" t="n">
+        <v>1925.27</v>
+      </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
       <c r="A111" s="3" t="n">
@@ -14506,6 +14769,7 @@
       <c r="AX111" s="13" t="n"/>
       <c r="AY111" s="13" t="n"/>
       <c r="AZ111" s="13" t="n"/>
+      <c r="BA111" s="13" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -14662,6 +14926,9 @@
         <v>20.44</v>
       </c>
       <c r="AZ112" s="13" t="n">
+        <v>20.44</v>
+      </c>
+      <c r="BA112" s="13" t="n">
         <v>20.44</v>
       </c>
     </row>
@@ -14774,6 +15041,9 @@
       <c r="AZ113" s="13" t="n">
         <v>8566.25</v>
       </c>
+      <c r="BA113" s="13" t="n">
+        <v>8321.969999999999</v>
+      </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
       <c r="A114" s="3" t="n">
@@ -14876,6 +15146,7 @@
       <c r="AX114" s="13" t="n"/>
       <c r="AY114" s="13" t="n"/>
       <c r="AZ114" s="13" t="n"/>
+      <c r="BA114" s="13" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -15032,6 +15303,9 @@
         <v>99.28</v>
       </c>
       <c r="AZ115" s="13" t="n">
+        <v>99.28</v>
+      </c>
+      <c r="BA115" s="13" t="n">
         <v>99.28</v>
       </c>
     </row>
@@ -15128,6 +15402,9 @@
       </c>
       <c r="AZ116" s="13" t="n">
         <v>16269.28</v>
+      </c>
+      <c r="BA116" s="13" t="n">
+        <v>16321</v>
       </c>
     </row>
     <row r="117">
@@ -15186,6 +15463,7 @@
       <c r="AX117" s="13" t="n"/>
       <c r="AY117" s="13" t="n"/>
       <c r="AZ117" s="13" t="n"/>
+      <c r="BA117" s="13" t="n"/>
     </row>
     <row r="118">
       <c r="P118" s="13" t="n">
@@ -15299,6 +15577,9 @@
       <c r="AZ118" s="13" t="n">
         <v>62.89</v>
       </c>
+      <c r="BA118" s="13" t="n">
+        <v>62.89</v>
+      </c>
     </row>
     <row r="119">
       <c r="Y119" s="13" t="n">
@@ -15384,6 +15665,9 @@
       </c>
       <c r="AZ119" s="13" t="n">
         <v>12152.43</v>
+      </c>
+      <c r="BA119" s="13" t="n">
+        <v>12103.66</v>
       </c>
     </row>
     <row r="120">
@@ -15391,6 +15675,7 @@
       <c r="AX120" s="13" t="n"/>
       <c r="AY120" s="13" t="n"/>
       <c r="AZ120" s="13" t="n"/>
+      <c r="BA120" s="13" t="n"/>
     </row>
     <row r="121">
       <c r="AW121" s="13" t="n">
@@ -15405,6 +15690,9 @@
       <c r="AZ121" s="13" t="n">
         <v>27.69</v>
       </c>
+      <c r="BA121" s="13" t="n">
+        <v>27.69</v>
+      </c>
     </row>
     <row r="122">
       <c r="AW122" s="13" t="n">
@@ -15417,6 +15705,9 @@
         <v>1821.31</v>
       </c>
       <c r="AZ122" s="13" t="n">
+        <v>1817.47</v>
+      </c>
+      <c r="BA122" s="13" t="n">
         <v>1817.47</v>
       </c>
     </row>
@@ -15425,6 +15716,7 @@
       <c r="AX123" s="13" t="n"/>
       <c r="AY123" s="13" t="n"/>
       <c r="AZ123" s="13" t="n"/>
+      <c r="BA123" s="13" t="n"/>
     </row>
     <row r="124">
       <c r="AW124" s="13" t="n">
@@ -15439,6 +15731,9 @@
       <c r="AZ124" s="13" t="n">
         <v>15.54</v>
       </c>
+      <c r="BA124" s="13" t="n">
+        <v>15.54</v>
+      </c>
     </row>
     <row r="125">
       <c r="AW125" s="13" t="n">
@@ -15452,6 +15747,9 @@
       </c>
       <c r="AZ125" s="13" t="n">
         <v>768.13</v>
+      </c>
+      <c r="BA125" s="13" t="n">
+        <v>769.1799999999999</v>
       </c>
     </row>
     <row r="126">
@@ -15459,6 +15757,7 @@
       <c r="AX126" s="13" t="n"/>
       <c r="AY126" s="13" t="n"/>
       <c r="AZ126" s="13" t="n"/>
+      <c r="BA126" s="13" t="n"/>
     </row>
     <row r="127">
       <c r="AW127" s="13" t="n">
@@ -15473,6 +15772,9 @@
       <c r="AZ127" s="13" t="n">
         <v>58.22</v>
       </c>
+      <c r="BA127" s="13" t="n">
+        <v>58.22</v>
+      </c>
     </row>
     <row r="128">
       <c r="AW128" s="13" t="n">
@@ -15486,6 +15788,9 @@
       </c>
       <c r="AZ128" s="13" t="n">
         <v>2674.72</v>
+      </c>
+      <c r="BA128" s="13" t="n">
+        <v>2674.28</v>
       </c>
     </row>
     <row r="129">
@@ -15493,6 +15798,7 @@
       <c r="AX129" s="13" t="n"/>
       <c r="AY129" s="13" t="n"/>
       <c r="AZ129" s="13" t="n"/>
+      <c r="BA129" s="13" t="n"/>
     </row>
     <row r="130">
       <c r="AW130" s="13" t="n">
@@ -15507,6 +15813,9 @@
       <c r="AZ130" s="13" t="n">
         <v>20.78</v>
       </c>
+      <c r="BA130" s="13" t="n">
+        <v>20.78</v>
+      </c>
     </row>
     <row r="131">
       <c r="AW131" s="13" t="n">
@@ -15520,6 +15829,9 @@
       </c>
       <c r="AZ131" s="13" t="n">
         <v>3567.08</v>
+      </c>
+      <c r="BA131" s="13" t="n">
+        <v>3566.03</v>
       </c>
     </row>
     <row r="132">
@@ -15527,6 +15839,7 @@
       <c r="AX132" s="13" t="n"/>
       <c r="AY132" s="13" t="n"/>
       <c r="AZ132" s="13" t="n"/>
+      <c r="BA132" s="13" t="n"/>
     </row>
     <row r="133">
       <c r="AW133" s="13" t="n">
@@ -15539,6 +15852,9 @@
         <v>2.09</v>
       </c>
       <c r="AZ133" s="13" t="n"/>
+      <c r="BA133" s="13" t="n">
+        <v>2.09</v>
+      </c>
     </row>
     <row r="134">
       <c r="AW134" s="13" t="n">
@@ -15551,12 +15867,16 @@
         <v>2362.93</v>
       </c>
       <c r="AZ134" s="13" t="n"/>
+      <c r="BA134" s="13" t="n">
+        <v>2343.65</v>
+      </c>
     </row>
     <row r="135">
       <c r="AW135" s="13" t="n"/>
       <c r="AX135" s="13" t="n"/>
       <c r="AY135" s="13" t="n"/>
       <c r="AZ135" s="13" t="n"/>
+      <c r="BA135" s="13" t="n"/>
     </row>
     <row r="136">
       <c r="AW136" s="13" t="n">
@@ -15571,6 +15891,9 @@
       <c r="AZ136" s="13" t="n">
         <v>15</v>
       </c>
+      <c r="BA136" s="13" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="137">
       <c r="AW137" s="13" t="n">
@@ -15583,6 +15906,9 @@
         <v>6280.28</v>
       </c>
       <c r="AZ137" s="13" t="n">
+        <v>6280.28</v>
+      </c>
+      <c r="BA137" s="13" t="n">
         <v>6280.28</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-07-20 06:38:13]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ137"/>
+  <dimension ref="A1:BA137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -586,6 +586,7 @@
     <col width="15" customWidth="1" min="50" max="50"/>
     <col width="15" customWidth="1" min="51" max="51"/>
     <col width="15" customWidth="1" min="52" max="52"/>
+    <col width="15" customWidth="1" min="53" max="53"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -849,6 +850,11 @@
           <t>2026/07/16</t>
         </is>
       </c>
+      <c r="BA1" s="15" t="inlineStr">
+        <is>
+          <t>2026/07/20</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1111,6 +1117,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BA2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1269,6 +1280,9 @@
       <c r="AZ3" s="15" t="n">
         <v>65.25</v>
       </c>
+      <c r="BA3" s="15" t="n">
+        <v>21.73</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1426,6 +1440,9 @@
       </c>
       <c r="AZ4" s="15" t="n">
         <v>3897.06</v>
+      </c>
+      <c r="BA4" s="15" t="n">
+        <v>3752.46</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1481,6 +1498,7 @@
       <c r="AX5" s="13" t="n"/>
       <c r="AY5" s="13" t="n"/>
       <c r="AZ5" s="15" t="n"/>
+      <c r="BA5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1583,6 +1601,7 @@
       <c r="AX6" s="13" t="n"/>
       <c r="AY6" s="13" t="n"/>
       <c r="AZ6" s="15" t="n"/>
+      <c r="BA6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1740,6 +1759,9 @@
       </c>
       <c r="AZ7" s="15" t="n">
         <v>65.8</v>
+      </c>
+      <c r="BA7" s="15" t="n">
+        <v>57.38</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -1851,6 +1873,9 @@
       <c r="AZ8" s="15" t="n">
         <v>5844.35</v>
       </c>
+      <c r="BA8" s="15" t="n">
+        <v>5525.38</v>
+      </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -1953,6 +1978,7 @@
       <c r="AX9" s="13" t="n"/>
       <c r="AY9" s="13" t="n"/>
       <c r="AZ9" s="15" t="n"/>
+      <c r="BA9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2110,6 +2136,9 @@
       </c>
       <c r="AZ10" s="15" t="n">
         <v>57.07</v>
+      </c>
+      <c r="BA10" s="15" t="n">
+        <v>49.2</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2221,6 +2250,9 @@
       <c r="AZ11" s="15" t="n">
         <v>4711.47</v>
       </c>
+      <c r="BA11" s="15" t="n">
+        <v>4530.75</v>
+      </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -2323,6 +2355,7 @@
       <c r="AX12" s="13" t="n"/>
       <c r="AY12" s="13" t="n"/>
       <c r="AZ12" s="15" t="n"/>
+      <c r="BA12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2480,6 +2513,9 @@
       </c>
       <c r="AZ13" s="15" t="n">
         <v>68.5</v>
+      </c>
+      <c r="BA13" s="15" t="n">
+        <v>62.77</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -2591,6 +2627,9 @@
       <c r="AZ14" s="15" t="n">
         <v>7998.03</v>
       </c>
+      <c r="BA14" s="15" t="n">
+        <v>7274.34</v>
+      </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -2693,6 +2732,7 @@
       <c r="AX15" s="13" t="n"/>
       <c r="AY15" s="13" t="n"/>
       <c r="AZ15" s="15" t="n"/>
+      <c r="BA15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -2850,6 +2890,9 @@
       </c>
       <c r="AZ16" s="15" t="n">
         <v>35.69</v>
+      </c>
+      <c r="BA16" s="15" t="n">
+        <v>28.43</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -2961,6 +3004,9 @@
       <c r="AZ17" s="15" t="n">
         <v>2620.36</v>
       </c>
+      <c r="BA17" s="15" t="n">
+        <v>2536.29</v>
+      </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="3" t="n">
@@ -3063,6 +3109,7 @@
       <c r="AX18" s="13" t="n"/>
       <c r="AY18" s="13" t="n"/>
       <c r="AZ18" s="15" t="n"/>
+      <c r="BA18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -3220,6 +3267,9 @@
       </c>
       <c r="AZ19" s="15" t="n">
         <v>86.06</v>
+      </c>
+      <c r="BA19" s="15" t="n">
+        <v>86.56</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -3331,6 +3381,9 @@
       <c r="AZ20" s="15" t="n">
         <v>7572.4</v>
       </c>
+      <c r="BA20" s="15" t="n">
+        <v>7457.69</v>
+      </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -3433,6 +3486,7 @@
       <c r="AX21" s="13" t="n"/>
       <c r="AY21" s="13" t="n"/>
       <c r="AZ21" s="15" t="n"/>
+      <c r="BA21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -3587,6 +3641,9 @@
         <v>36.34</v>
       </c>
       <c r="AZ22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BA22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -3699,6 +3756,9 @@
       <c r="AZ23" s="15" t="n">
         <v>77483.42</v>
       </c>
+      <c r="BA23" s="15" t="n">
+        <v>77579.10000000001</v>
+      </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="3" t="n">
@@ -3801,6 +3861,7 @@
       <c r="AX24" s="13" t="n"/>
       <c r="AY24" s="13" t="n"/>
       <c r="AZ24" s="15" t="n"/>
+      <c r="BA24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -3957,6 +4018,9 @@
         <v>49.88</v>
       </c>
       <c r="AZ25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BA25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -4063,6 +4127,9 @@
         <v>25041.78</v>
       </c>
       <c r="AZ26" s="15" t="inlineStr"/>
+      <c r="BA26" s="15" t="n">
+        <v>24830.98</v>
+      </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -4165,6 +4232,7 @@
       <c r="AX27" s="13" t="n"/>
       <c r="AY27" s="13" t="n"/>
       <c r="AZ27" s="15" t="n"/>
+      <c r="BA27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -4321,6 +4389,9 @@
         <v>92.09</v>
       </c>
       <c r="AZ28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BA28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -4433,6 +4504,9 @@
       <c r="AZ29" s="15" t="n">
         <v>66625.48</v>
       </c>
+      <c r="BA29" s="15" t="n">
+        <v>64141.12</v>
+      </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="3" t="n">
@@ -4535,6 +4609,7 @@
       <c r="AX30" s="13" t="n"/>
       <c r="AY30" s="13" t="n"/>
       <c r="AZ30" s="15" t="n"/>
+      <c r="BA30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -4692,6 +4767,9 @@
       </c>
       <c r="AZ31" s="15" t="n">
         <v>47.54</v>
+      </c>
+      <c r="BA31" s="15" t="n">
+        <v>48.88</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -4803,6 +4881,9 @@
       <c r="AZ32" s="15" t="n">
         <v>5330.25</v>
       </c>
+      <c r="BA32" s="15" t="n">
+        <v>5410.42</v>
+      </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
       <c r="A33" s="3" t="n">
@@ -4905,6 +4986,7 @@
       <c r="AX33" s="13" t="n"/>
       <c r="AY33" s="13" t="n"/>
       <c r="AZ33" s="15" t="n"/>
+      <c r="BA33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -5062,6 +5144,9 @@
       </c>
       <c r="AZ34" s="15" t="n">
         <v>63.03</v>
+      </c>
+      <c r="BA34" s="15" t="n">
+        <v>66.13</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -5173,6 +5258,9 @@
       <c r="AZ35" s="15" t="n">
         <v>11297.34</v>
       </c>
+      <c r="BA35" s="15" t="n">
+        <v>11245.35</v>
+      </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="3" t="n">
@@ -5275,6 +5363,7 @@
       <c r="AX36" s="13" t="n"/>
       <c r="AY36" s="13" t="n"/>
       <c r="AZ36" s="15" t="n"/>
+      <c r="BA36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -5432,6 +5521,9 @@
       </c>
       <c r="AZ37" s="15" t="n">
         <v>52.3</v>
+      </c>
+      <c r="BA37" s="15" t="n">
+        <v>53.09</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -5543,6 +5635,9 @@
       <c r="AZ38" s="15" t="n">
         <v>10709.77</v>
       </c>
+      <c r="BA38" s="15" t="n">
+        <v>10633.93</v>
+      </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
       <c r="A39" s="3" t="n">
@@ -5645,6 +5740,7 @@
       <c r="AX39" s="13" t="n"/>
       <c r="AY39" s="13" t="n"/>
       <c r="AZ39" s="15" t="n"/>
+      <c r="BA39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -5802,6 +5898,9 @@
       </c>
       <c r="AZ40" s="15" t="n">
         <v>51.92</v>
+      </c>
+      <c r="BA40" s="15" t="n">
+        <v>51.89</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -5913,6 +6012,9 @@
       <c r="AZ41" s="15" t="n">
         <v>3115.39</v>
       </c>
+      <c r="BA41" s="15" t="n">
+        <v>3059.91</v>
+      </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
       <c r="A42" s="3" t="n">
@@ -6015,6 +6117,7 @@
       <c r="AX42" s="13" t="n"/>
       <c r="AY42" s="13" t="n"/>
       <c r="AZ42" s="15" t="n"/>
+      <c r="BA42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -6172,6 +6275,9 @@
       </c>
       <c r="AZ43" s="15" t="n">
         <v>59.91</v>
+      </c>
+      <c r="BA43" s="15" t="n">
+        <v>66.31999999999999</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -6283,6 +6389,9 @@
       <c r="AZ44" s="15" t="n">
         <v>6881.29</v>
       </c>
+      <c r="BA44" s="15" t="n">
+        <v>6869.73</v>
+      </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
       <c r="A45" s="3" t="n">
@@ -6385,6 +6494,7 @@
       <c r="AX45" s="13" t="n"/>
       <c r="AY45" s="13" t="n"/>
       <c r="AZ45" s="15" t="n"/>
+      <c r="BA45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -6542,6 +6652,9 @@
       </c>
       <c r="AZ46" s="15" t="n">
         <v>26.01</v>
+      </c>
+      <c r="BA46" s="15" t="n">
+        <v>18.6</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -6653,6 +6766,9 @@
       <c r="AZ47" s="15" t="n">
         <v>33002.06</v>
       </c>
+      <c r="BA47" s="15" t="n">
+        <v>32082.79</v>
+      </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
       <c r="A48" s="3" t="n">
@@ -6755,6 +6871,7 @@
       <c r="AX48" s="13" t="n"/>
       <c r="AY48" s="13" t="n"/>
       <c r="AZ48" s="15" t="n"/>
+      <c r="BA48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -6912,6 +7029,9 @@
       </c>
       <c r="AZ49" s="15" t="n">
         <v>57.51</v>
+      </c>
+      <c r="BA49" s="15" t="n">
+        <v>48.51</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -7023,6 +7143,9 @@
       <c r="AZ50" s="15" t="n">
         <v>3947.32</v>
       </c>
+      <c r="BA50" s="15" t="n">
+        <v>3563.25</v>
+      </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
       <c r="A51" s="3" t="n">
@@ -7125,6 +7248,7 @@
       <c r="AX51" s="13" t="n"/>
       <c r="AY51" s="13" t="n"/>
       <c r="AZ51" s="15" t="n"/>
+      <c r="BA51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -7282,6 +7406,9 @@
       </c>
       <c r="AZ52" s="15" t="n">
         <v>65.44</v>
+      </c>
+      <c r="BA52" s="15" t="n">
+        <v>57.72</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -7393,6 +7520,9 @@
       <c r="AZ53" s="15" t="n">
         <v>3709.59</v>
       </c>
+      <c r="BA53" s="15" t="n">
+        <v>3340.48</v>
+      </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
       <c r="A54" s="3" t="n">
@@ -7495,6 +7625,7 @@
       <c r="AX54" s="13" t="n"/>
       <c r="AY54" s="13" t="n"/>
       <c r="AZ54" s="15" t="n"/>
+      <c r="BA54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -7652,6 +7783,9 @@
       </c>
       <c r="AZ55" s="15" t="n">
         <v>13.16</v>
+      </c>
+      <c r="BA55" s="15" t="n">
+        <v>7.68</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -7763,6 +7897,9 @@
       <c r="AZ56" s="15" t="n">
         <v>6633.43</v>
       </c>
+      <c r="BA56" s="15" t="n">
+        <v>6325.73</v>
+      </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
       <c r="A57" s="3" t="n">
@@ -7865,6 +8002,7 @@
       <c r="AX57" s="13" t="n"/>
       <c r="AY57" s="13" t="n"/>
       <c r="AZ57" s="15" t="n"/>
+      <c r="BA57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -8022,6 +8160,9 @@
       </c>
       <c r="AZ58" s="15" t="n">
         <v>37.84</v>
+      </c>
+      <c r="BA58" s="15" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -8133,6 +8274,9 @@
       <c r="AZ59" s="15" t="n">
         <v>8201.309999999999</v>
       </c>
+      <c r="BA59" s="15" t="n">
+        <v>8000.89</v>
+      </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
       <c r="A60" s="3" t="n">
@@ -8235,6 +8379,7 @@
       <c r="AX60" s="13" t="n"/>
       <c r="AY60" s="13" t="n"/>
       <c r="AZ60" s="15" t="n"/>
+      <c r="BA60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -8392,6 +8537,9 @@
       </c>
       <c r="AZ61" s="15" t="n">
         <v>2.18</v>
+      </c>
+      <c r="BA61" s="15" t="n">
+        <v>1.94</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -8503,6 +8651,9 @@
       <c r="AZ62" s="15" t="n">
         <v>10285.78</v>
       </c>
+      <c r="BA62" s="15" t="n">
+        <v>10771.99</v>
+      </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
       <c r="A63" s="3" t="n">
@@ -8605,6 +8756,7 @@
       <c r="AX63" s="13" t="n"/>
       <c r="AY63" s="13" t="n"/>
       <c r="AZ63" s="15" t="n"/>
+      <c r="BA63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -8762,6 +8914,9 @@
       </c>
       <c r="AZ64" s="15" t="n">
         <v>21.27</v>
+      </c>
+      <c r="BA64" s="15" t="n">
+        <v>15.07</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -8873,6 +9028,9 @@
       <c r="AZ65" s="15" t="n">
         <v>11608.72</v>
       </c>
+      <c r="BA65" s="15" t="n">
+        <v>10992.6</v>
+      </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
       <c r="A66" s="3" t="n">
@@ -8975,6 +9133,7 @@
       <c r="AX66" s="13" t="n"/>
       <c r="AY66" s="13" t="n"/>
       <c r="AZ66" s="15" t="n"/>
+      <c r="BA66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -9132,6 +9291,9 @@
       </c>
       <c r="AZ67" s="15" t="n">
         <v>10.9</v>
+      </c>
+      <c r="BA67" s="15" t="n">
+        <v>10.61</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -9243,6 +9405,9 @@
       <c r="AZ68" s="15" t="n">
         <v>6505.27</v>
       </c>
+      <c r="BA68" s="15" t="n">
+        <v>6620.96</v>
+      </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
       <c r="A69" s="3" t="n">
@@ -9345,6 +9510,7 @@
       <c r="AX69" s="13" t="n"/>
       <c r="AY69" s="13" t="n"/>
       <c r="AZ69" s="15" t="n"/>
+      <c r="BA69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -9502,6 +9668,9 @@
       </c>
       <c r="AZ70" s="15" t="n">
         <v>11.62</v>
+      </c>
+      <c r="BA70" s="15" t="n">
+        <v>11.5</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -9613,6 +9782,9 @@
       <c r="AZ71" s="15" t="n">
         <v>12553.75</v>
       </c>
+      <c r="BA71" s="15" t="n">
+        <v>12666.14</v>
+      </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
       <c r="A72" s="3" t="n">
@@ -9715,6 +9887,7 @@
       <c r="AX72" s="13" t="n"/>
       <c r="AY72" s="13" t="n"/>
       <c r="AZ72" s="15" t="n"/>
+      <c r="BA72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -9872,6 +10045,9 @@
       </c>
       <c r="AZ73" s="15" t="n">
         <v>53.17</v>
+      </c>
+      <c r="BA73" s="15" t="n">
+        <v>51.77</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -9983,6 +10159,9 @@
       <c r="AZ74" s="15" t="n">
         <v>14637.99</v>
       </c>
+      <c r="BA74" s="15" t="n">
+        <v>14021.77</v>
+      </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
       <c r="A75" s="3" t="n">
@@ -10085,6 +10264,7 @@
       <c r="AX75" s="13" t="n"/>
       <c r="AY75" s="13" t="n"/>
       <c r="AZ75" s="15" t="n"/>
+      <c r="BA75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -10242,6 +10422,9 @@
       </c>
       <c r="AZ76" s="15" t="n">
         <v>3.71</v>
+      </c>
+      <c r="BA76" s="15" t="n">
+        <v>3.66</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -10353,6 +10536,9 @@
       <c r="AZ77" s="15" t="n">
         <v>7296.99</v>
       </c>
+      <c r="BA77" s="15" t="n">
+        <v>7047.55</v>
+      </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
       <c r="A78" s="3" t="n">
@@ -10455,6 +10641,7 @@
       <c r="AX78" s="13" t="n"/>
       <c r="AY78" s="13" t="n"/>
       <c r="AZ78" s="15" t="n"/>
+      <c r="BA78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -10612,6 +10799,9 @@
       </c>
       <c r="AZ79" s="15" t="n">
         <v>4.12</v>
+      </c>
+      <c r="BA79" s="15" t="n">
+        <v>4.04</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -10723,6 +10913,9 @@
       <c r="AZ80" s="15" t="n">
         <v>9188.450000000001</v>
       </c>
+      <c r="BA80" s="15" t="n">
+        <v>9140.83</v>
+      </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
       <c r="A81" s="3" t="n">
@@ -10825,6 +11018,7 @@
       <c r="AX81" s="13" t="n"/>
       <c r="AY81" s="13" t="n"/>
       <c r="AZ81" s="15" t="n"/>
+      <c r="BA81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -10982,6 +11176,9 @@
       </c>
       <c r="AZ82" s="15" t="n">
         <v>13.11</v>
+      </c>
+      <c r="BA82" s="15" t="n">
+        <v>12.66</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -11093,6 +11290,9 @@
       <c r="AZ83" s="15" t="n">
         <v>2631.9</v>
       </c>
+      <c r="BA83" s="15" t="n">
+        <v>2335.88</v>
+      </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
       <c r="A84" s="3" t="n">
@@ -11195,6 +11395,7 @@
       <c r="AX84" s="13" t="n"/>
       <c r="AY84" s="13" t="n"/>
       <c r="AZ84" s="15" t="n"/>
+      <c r="BA84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -11352,6 +11553,9 @@
       </c>
       <c r="AZ85" s="15" t="n">
         <v>28.88</v>
+      </c>
+      <c r="BA85" s="15" t="n">
+        <v>24.17</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -11463,6 +11667,9 @@
       <c r="AZ86" s="15" t="n">
         <v>4886.04</v>
       </c>
+      <c r="BA86" s="15" t="n">
+        <v>4735.38</v>
+      </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
       <c r="A87" s="3" t="n">
@@ -11565,6 +11772,7 @@
       <c r="AX87" s="13" t="n"/>
       <c r="AY87" s="13" t="n"/>
       <c r="AZ87" s="15" t="n"/>
+      <c r="BA87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -11722,6 +11930,9 @@
       </c>
       <c r="AZ88" s="15" t="n">
         <v>26.8</v>
+      </c>
+      <c r="BA88" s="15" t="n">
+        <v>19.87</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -11833,6 +12044,9 @@
       <c r="AZ89" s="15" t="n">
         <v>8841.83</v>
       </c>
+      <c r="BA89" s="15" t="n">
+        <v>8485.110000000001</v>
+      </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
       <c r="A90" s="3" t="n">
@@ -11935,6 +12149,7 @@
       <c r="AX90" s="13" t="n"/>
       <c r="AY90" s="13" t="n"/>
       <c r="AZ90" s="15" t="n"/>
+      <c r="BA90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -12092,6 +12307,9 @@
       </c>
       <c r="AZ91" s="15" t="n">
         <v>4.37</v>
+      </c>
+      <c r="BA91" s="15" t="n">
+        <v>3.72</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -12203,6 +12421,9 @@
       <c r="AZ92" s="15" t="n">
         <v>1156.67</v>
       </c>
+      <c r="BA92" s="15" t="n">
+        <v>1137.96</v>
+      </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
       <c r="A93" s="3" t="n">
@@ -12305,6 +12526,7 @@
       <c r="AX93" s="13" t="n"/>
       <c r="AY93" s="13" t="n"/>
       <c r="AZ93" s="15" t="n"/>
+      <c r="BA93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -12462,6 +12684,9 @@
       </c>
       <c r="AZ94" s="15" t="n">
         <v>5.44</v>
+      </c>
+      <c r="BA94" s="15" t="n">
+        <v>4.96</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -12573,6 +12798,9 @@
       <c r="AZ95" s="15" t="n">
         <v>13737.48</v>
       </c>
+      <c r="BA95" s="15" t="n">
+        <v>13576.65</v>
+      </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
       <c r="A96" s="3" t="n">
@@ -12675,6 +12903,7 @@
       <c r="AX96" s="13" t="n"/>
       <c r="AY96" s="13" t="n"/>
       <c r="AZ96" s="15" t="n"/>
+      <c r="BA96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -12832,6 +13061,9 @@
       </c>
       <c r="AZ97" s="15" t="n">
         <v>50.16</v>
+      </c>
+      <c r="BA97" s="15" t="n">
+        <v>41.28</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -12943,6 +13175,9 @@
       <c r="AZ98" s="15" t="n">
         <v>3316.81</v>
       </c>
+      <c r="BA98" s="15" t="n">
+        <v>3091.16</v>
+      </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
       <c r="A99" s="3" t="n">
@@ -13045,6 +13280,7 @@
       <c r="AX99" s="13" t="n"/>
       <c r="AY99" s="13" t="n"/>
       <c r="AZ99" s="15" t="n"/>
+      <c r="BA99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -13202,6 +13438,9 @@
       </c>
       <c r="AZ100" s="15" t="n">
         <v>39.05</v>
+      </c>
+      <c r="BA100" s="15" t="n">
+        <v>35.04</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -13313,6 +13552,9 @@
       <c r="AZ101" s="15" t="n">
         <v>2387.93</v>
       </c>
+      <c r="BA101" s="15" t="n">
+        <v>2231.52</v>
+      </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
       <c r="A102" s="3" t="n">
@@ -13415,6 +13657,7 @@
       <c r="AX102" s="13" t="n"/>
       <c r="AY102" s="13" t="n"/>
       <c r="AZ102" s="15" t="n"/>
+      <c r="BA102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -13572,6 +13815,9 @@
       </c>
       <c r="AZ103" s="15" t="n">
         <v>16.96</v>
+      </c>
+      <c r="BA103" s="15" t="n">
+        <v>12.26</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -13683,6 +13929,9 @@
       <c r="AZ104" s="15" t="n">
         <v>2456.84</v>
       </c>
+      <c r="BA104" s="15" t="n">
+        <v>2286.4</v>
+      </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
       <c r="A105" s="3" t="n">
@@ -13785,6 +14034,7 @@
       <c r="AX105" s="13" t="n"/>
       <c r="AY105" s="13" t="n"/>
       <c r="AZ105" s="15" t="n"/>
+      <c r="BA105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -13942,6 +14192,9 @@
       </c>
       <c r="AZ106" s="15" t="n">
         <v>38.89</v>
+      </c>
+      <c r="BA106" s="15" t="n">
+        <v>37.08</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -14053,6 +14306,9 @@
       <c r="AZ107" s="15" t="n">
         <v>2581.26</v>
       </c>
+      <c r="BA107" s="15" t="n">
+        <v>2391.38</v>
+      </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
       <c r="A108" s="3" t="n">
@@ -14155,6 +14411,7 @@
       <c r="AX108" s="13" t="n"/>
       <c r="AY108" s="13" t="n"/>
       <c r="AZ108" s="15" t="n"/>
+      <c r="BA108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -14312,6 +14569,9 @@
       </c>
       <c r="AZ109" s="15" t="n">
         <v>66.65000000000001</v>
+      </c>
+      <c r="BA109" s="15" t="n">
+        <v>56.72</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -14423,6 +14683,9 @@
       <c r="AZ110" s="15" t="n">
         <v>2053.63</v>
       </c>
+      <c r="BA110" s="15" t="n">
+        <v>1935.08</v>
+      </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
       <c r="A111" s="3" t="n">
@@ -14525,6 +14788,7 @@
       <c r="AX111" s="13" t="n"/>
       <c r="AY111" s="13" t="n"/>
       <c r="AZ111" s="15" t="n"/>
+      <c r="BA111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -14682,6 +14946,9 @@
       </c>
       <c r="AZ112" s="15" t="n">
         <v>21.99</v>
+      </c>
+      <c r="BA112" s="15" t="n">
+        <v>20.8</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -14793,6 +15060,9 @@
       <c r="AZ113" s="15" t="n">
         <v>8856.83</v>
       </c>
+      <c r="BA113" s="15" t="n">
+        <v>8403.35</v>
+      </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
       <c r="A114" s="3" t="n">
@@ -14895,6 +15165,7 @@
       <c r="AX114" s="13" t="n"/>
       <c r="AY114" s="13" t="n"/>
       <c r="AZ114" s="15" t="n"/>
+      <c r="BA114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -15052,6 +15323,9 @@
       </c>
       <c r="AZ115" s="15" t="n">
         <v>98.43000000000001</v>
+      </c>
+      <c r="BA115" s="15" t="n">
+        <v>96.63</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -15147,6 +15421,9 @@
       </c>
       <c r="AZ116" s="15" t="n">
         <v>15189.12</v>
+      </c>
+      <c r="BA116" s="15" t="n">
+        <v>12766.26</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -15205,6 +15482,7 @@
       <c r="AX117" s="13" t="n"/>
       <c r="AY117" s="13" t="n"/>
       <c r="AZ117" s="15" t="n"/>
+      <c r="BA117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -15318,6 +15596,9 @@
       <c r="AZ118" s="15" t="n">
         <v>48.69</v>
       </c>
+      <c r="BA118" s="15" t="n">
+        <v>37.22</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -15403,6 +15684,9 @@
       </c>
       <c r="AZ119" s="15" t="n">
         <v>11407.26</v>
+      </c>
+      <c r="BA119" s="15" t="n">
+        <v>10528.94</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -15410,6 +15694,7 @@
       <c r="AX120" s="13" t="n"/>
       <c r="AY120" s="13" t="n"/>
       <c r="AZ120" s="15" t="n"/>
+      <c r="BA120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -15424,6 +15709,9 @@
       <c r="AZ121" s="15" t="n">
         <v>28.33</v>
       </c>
+      <c r="BA121" s="15" t="n">
+        <v>28.34</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -15437,6 +15725,9 @@
       </c>
       <c r="AZ122" s="15" t="n">
         <v>1897.79</v>
+      </c>
+      <c r="BA122" s="15" t="n">
+        <v>1843.85</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -15444,6 +15735,7 @@
       <c r="AX123" s="13" t="n"/>
       <c r="AY123" s="13" t="n"/>
       <c r="AZ123" s="15" t="n"/>
+      <c r="BA123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -15458,6 +15750,9 @@
       <c r="AZ124" s="15" t="n">
         <v>17.99</v>
       </c>
+      <c r="BA124" s="15" t="n">
+        <v>13.99</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -15471,6 +15766,9 @@
       </c>
       <c r="AZ125" s="15" t="n">
         <v>779.23</v>
+      </c>
+      <c r="BA125" s="15" t="n">
+        <v>773.9</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -15478,6 +15776,7 @@
       <c r="AX126" s="13" t="n"/>
       <c r="AY126" s="13" t="n"/>
       <c r="AZ126" s="15" t="n"/>
+      <c r="BA126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -15492,6 +15791,9 @@
       <c r="AZ127" s="15" t="n">
         <v>56.16</v>
       </c>
+      <c r="BA127" s="15" t="n">
+        <v>49.31</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -15504,6 +15806,9 @@
         <v>2674.28</v>
       </c>
       <c r="AZ128" s="15" t="n">
+        <v>2674.28</v>
+      </c>
+      <c r="BA128" s="15" t="n">
         <v>2674.28</v>
       </c>
     </row>
@@ -15512,6 +15817,7 @@
       <c r="AX129" s="13" t="n"/>
       <c r="AY129" s="13" t="n"/>
       <c r="AZ129" s="15" t="n"/>
+      <c r="BA129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -15526,6 +15832,9 @@
       <c r="AZ130" s="15" t="n">
         <v>20.68</v>
       </c>
+      <c r="BA130" s="15" t="n">
+        <v>19.71</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -15539,6 +15848,9 @@
       </c>
       <c r="AZ131" s="15" t="n">
         <v>3545.76</v>
+      </c>
+      <c r="BA131" s="15" t="n">
+        <v>3449.02</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -15546,6 +15858,7 @@
       <c r="AX132" s="13" t="n"/>
       <c r="AY132" s="13" t="n"/>
       <c r="AZ132" s="15" t="n"/>
+      <c r="BA132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -15560,6 +15873,9 @@
       <c r="AZ133" s="15" t="n">
         <v>1.87</v>
       </c>
+      <c r="BA133" s="15" t="n">
+        <v>1.52</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -15573,6 +15889,9 @@
       </c>
       <c r="AZ134" s="15" t="n">
         <v>2388.21</v>
+      </c>
+      <c r="BA134" s="15" t="n">
+        <v>2269.39</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -15580,6 +15899,7 @@
       <c r="AX135" s="13" t="n"/>
       <c r="AY135" s="13" t="n"/>
       <c r="AZ135" s="15" t="n"/>
+      <c r="BA135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -15594,6 +15914,9 @@
       <c r="AZ136" s="15" t="n">
         <v>6.2</v>
       </c>
+      <c r="BA136" s="15" t="n">
+        <v>4.95</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -15607,6 +15930,9 @@
       </c>
       <c r="AZ137" s="15" t="n">
         <v>5616.84</v>
+      </c>
+      <c r="BA137" s="15" t="n">
+        <v>5197.16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-07-23 06:21:01]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA137"/>
+  <dimension ref="A1:BB137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -587,6 +587,7 @@
     <col width="15" customWidth="1" min="51" max="51"/>
     <col width="15" customWidth="1" min="52" max="52"/>
     <col width="15" customWidth="1" min="53" max="53"/>
+    <col width="15" customWidth="1" min="54" max="54"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -855,6 +856,11 @@
           <t>2026/07/20</t>
         </is>
       </c>
+      <c r="BB1" s="15" t="inlineStr">
+        <is>
+          <t>2026/07/23</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1122,6 +1128,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BB2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1283,6 +1294,9 @@
       <c r="BA3" s="15" t="n">
         <v>21.73</v>
       </c>
+      <c r="BB3" s="15" t="n">
+        <v>61.97</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1443,6 +1457,9 @@
       </c>
       <c r="BA4" s="15" t="n">
         <v>3752.46</v>
+      </c>
+      <c r="BB4" s="15" t="n">
+        <v>3869.94</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1499,6 +1516,7 @@
       <c r="AY5" s="13" t="n"/>
       <c r="AZ5" s="15" t="n"/>
       <c r="BA5" s="15" t="n"/>
+      <c r="BB5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1602,6 +1620,7 @@
       <c r="AY6" s="13" t="n"/>
       <c r="AZ6" s="15" t="n"/>
       <c r="BA6" s="15" t="n"/>
+      <c r="BB6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1762,6 +1781,9 @@
       </c>
       <c r="BA7" s="15" t="n">
         <v>57.38</v>
+      </c>
+      <c r="BB7" s="15" t="n">
+        <v>64.72</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -1875,6 +1897,9 @@
       </c>
       <c r="BA8" s="15" t="n">
         <v>5525.38</v>
+      </c>
+      <c r="BB8" s="15" t="n">
+        <v>5804.21</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -1979,6 +2004,7 @@
       <c r="AY9" s="13" t="n"/>
       <c r="AZ9" s="15" t="n"/>
       <c r="BA9" s="15" t="n"/>
+      <c r="BB9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2139,6 +2165,9 @@
       </c>
       <c r="BA10" s="15" t="n">
         <v>49.2</v>
+      </c>
+      <c r="BB10" s="15" t="n">
+        <v>58.9</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2252,6 +2281,9 @@
       </c>
       <c r="BA11" s="15" t="n">
         <v>4530.75</v>
+      </c>
+      <c r="BB11" s="15" t="n">
+        <v>4719.71</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -2356,6 +2388,7 @@
       <c r="AY12" s="13" t="n"/>
       <c r="AZ12" s="15" t="n"/>
       <c r="BA12" s="15" t="n"/>
+      <c r="BB12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2516,6 +2549,9 @@
       </c>
       <c r="BA13" s="15" t="n">
         <v>62.77</v>
+      </c>
+      <c r="BB13" s="15" t="n">
+        <v>65.84</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -2629,6 +2665,9 @@
       </c>
       <c r="BA14" s="15" t="n">
         <v>7274.34</v>
+      </c>
+      <c r="BB14" s="15" t="n">
+        <v>7718.78</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -2733,6 +2772,7 @@
       <c r="AY15" s="13" t="n"/>
       <c r="AZ15" s="15" t="n"/>
       <c r="BA15" s="15" t="n"/>
+      <c r="BB15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -2893,6 +2933,9 @@
       </c>
       <c r="BA16" s="15" t="n">
         <v>28.43</v>
+      </c>
+      <c r="BB16" s="15" t="n">
+        <v>37.71</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -3006,6 +3049,9 @@
       </c>
       <c r="BA17" s="15" t="n">
         <v>2536.29</v>
+      </c>
+      <c r="BB17" s="15" t="n">
+        <v>2609.87</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -3110,6 +3156,7 @@
       <c r="AY18" s="13" t="n"/>
       <c r="AZ18" s="15" t="n"/>
       <c r="BA18" s="15" t="n"/>
+      <c r="BB18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -3270,6 +3317,9 @@
       </c>
       <c r="BA19" s="15" t="n">
         <v>86.56</v>
+      </c>
+      <c r="BB19" s="15" t="n">
+        <v>86.2</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -3383,6 +3433,9 @@
       </c>
       <c r="BA20" s="15" t="n">
         <v>7457.69</v>
+      </c>
+      <c r="BB20" s="15" t="n">
+        <v>7498.96</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -3487,6 +3540,7 @@
       <c r="AY21" s="13" t="n"/>
       <c r="AZ21" s="15" t="n"/>
       <c r="BA21" s="15" t="n"/>
+      <c r="BB21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -3644,6 +3698,9 @@
         <v>36.34</v>
       </c>
       <c r="BA22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BB22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -3758,6 +3815,9 @@
       </c>
       <c r="BA23" s="15" t="n">
         <v>77579.10000000001</v>
+      </c>
+      <c r="BB23" s="15" t="n">
+        <v>76562.36</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -3862,6 +3922,7 @@
       <c r="AY24" s="13" t="n"/>
       <c r="AZ24" s="15" t="n"/>
       <c r="BA24" s="15" t="n"/>
+      <c r="BB24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -4021,6 +4082,9 @@
         <v>49.88</v>
       </c>
       <c r="BA25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BB25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -4130,6 +4194,7 @@
       <c r="BA26" s="15" t="n">
         <v>24830.98</v>
       </c>
+      <c r="BB26" s="15" t="inlineStr"/>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -4233,6 +4298,7 @@
       <c r="AY27" s="13" t="n"/>
       <c r="AZ27" s="15" t="n"/>
       <c r="BA27" s="15" t="n"/>
+      <c r="BB27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -4392,6 +4458,9 @@
         <v>92.09</v>
       </c>
       <c r="BA28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BB28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -4506,6 +4575,9 @@
       </c>
       <c r="BA29" s="15" t="n">
         <v>64141.12</v>
+      </c>
+      <c r="BB29" s="15" t="n">
+        <v>66218.11</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -4610,6 +4682,7 @@
       <c r="AY30" s="13" t="n"/>
       <c r="AZ30" s="15" t="n"/>
       <c r="BA30" s="15" t="n"/>
+      <c r="BB30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -4770,6 +4843,9 @@
       </c>
       <c r="BA31" s="15" t="n">
         <v>48.88</v>
+      </c>
+      <c r="BB31" s="15" t="n">
+        <v>45.65</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -4883,6 +4959,9 @@
       </c>
       <c r="BA32" s="15" t="n">
         <v>5410.42</v>
+      </c>
+      <c r="BB32" s="15" t="n">
+        <v>5501.53</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -4987,6 +5066,7 @@
       <c r="AY33" s="13" t="n"/>
       <c r="AZ33" s="15" t="n"/>
       <c r="BA33" s="15" t="n"/>
+      <c r="BB33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -5147,6 +5227,9 @@
       </c>
       <c r="BA34" s="15" t="n">
         <v>66.13</v>
+      </c>
+      <c r="BB34" s="15" t="n">
+        <v>60.39</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -5260,6 +5343,9 @@
       </c>
       <c r="BA35" s="15" t="n">
         <v>11245.35</v>
+      </c>
+      <c r="BB35" s="15" t="n">
+        <v>11459.52</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -5364,6 +5450,7 @@
       <c r="AY36" s="13" t="n"/>
       <c r="AZ36" s="15" t="n"/>
       <c r="BA36" s="15" t="n"/>
+      <c r="BB36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -5524,6 +5611,9 @@
       </c>
       <c r="BA37" s="15" t="n">
         <v>53.09</v>
+      </c>
+      <c r="BB37" s="15" t="n">
+        <v>50.33</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -5637,6 +5727,9 @@
       </c>
       <c r="BA38" s="15" t="n">
         <v>10633.93</v>
+      </c>
+      <c r="BB38" s="15" t="n">
+        <v>10824.3</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -5741,6 +5834,7 @@
       <c r="AY39" s="13" t="n"/>
       <c r="AZ39" s="15" t="n"/>
       <c r="BA39" s="15" t="n"/>
+      <c r="BB39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -5901,6 +5995,9 @@
       </c>
       <c r="BA40" s="15" t="n">
         <v>51.89</v>
+      </c>
+      <c r="BB40" s="15" t="n">
+        <v>50.04</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -6014,6 +6111,9 @@
       </c>
       <c r="BA41" s="15" t="n">
         <v>3059.91</v>
+      </c>
+      <c r="BB41" s="15" t="n">
+        <v>3178.04</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -6118,6 +6218,7 @@
       <c r="AY42" s="13" t="n"/>
       <c r="AZ42" s="15" t="n"/>
       <c r="BA42" s="15" t="n"/>
+      <c r="BB42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -6278,6 +6379,9 @@
       </c>
       <c r="BA43" s="15" t="n">
         <v>66.31999999999999</v>
+      </c>
+      <c r="BB43" s="15" t="n">
+        <v>58.34</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -6391,6 +6495,9 @@
       </c>
       <c r="BA44" s="15" t="n">
         <v>6869.73</v>
+      </c>
+      <c r="BB44" s="15" t="n">
+        <v>7018.33</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -6495,6 +6602,7 @@
       <c r="AY45" s="13" t="n"/>
       <c r="AZ45" s="15" t="n"/>
       <c r="BA45" s="15" t="n"/>
+      <c r="BB45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -6655,6 +6763,9 @@
       </c>
       <c r="BA46" s="15" t="n">
         <v>18.6</v>
+      </c>
+      <c r="BB46" s="15" t="n">
+        <v>29.76</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -6768,6 +6879,9 @@
       </c>
       <c r="BA47" s="15" t="n">
         <v>32082.79</v>
+      </c>
+      <c r="BB47" s="15" t="n">
+        <v>33050.75</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -6872,6 +6986,7 @@
       <c r="AY48" s="13" t="n"/>
       <c r="AZ48" s="15" t="n"/>
       <c r="BA48" s="15" t="n"/>
+      <c r="BB48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -7032,6 +7147,9 @@
       </c>
       <c r="BA49" s="15" t="n">
         <v>48.51</v>
+      </c>
+      <c r="BB49" s="15" t="n">
+        <v>51.95</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -7145,6 +7263,9 @@
       </c>
       <c r="BA50" s="15" t="n">
         <v>3563.25</v>
+      </c>
+      <c r="BB50" s="15" t="n">
+        <v>3794.8</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -7249,6 +7370,7 @@
       <c r="AY51" s="13" t="n"/>
       <c r="AZ51" s="15" t="n"/>
       <c r="BA51" s="15" t="n"/>
+      <c r="BB51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -7409,6 +7531,9 @@
       </c>
       <c r="BA52" s="15" t="n">
         <v>57.72</v>
+      </c>
+      <c r="BB52" s="15" t="n">
+        <v>61.41</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -7522,6 +7647,9 @@
       </c>
       <c r="BA53" s="15" t="n">
         <v>3340.48</v>
+      </c>
+      <c r="BB53" s="15" t="n">
+        <v>3563.63</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -7626,6 +7754,7 @@
       <c r="AY54" s="13" t="n"/>
       <c r="AZ54" s="15" t="n"/>
       <c r="BA54" s="15" t="n"/>
+      <c r="BB54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -7786,6 +7915,9 @@
       </c>
       <c r="BA55" s="15" t="n">
         <v>7.68</v>
+      </c>
+      <c r="BB55" s="15" t="n">
+        <v>11.14</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -7899,6 +8031,9 @@
       </c>
       <c r="BA56" s="15" t="n">
         <v>6325.73</v>
+      </c>
+      <c r="BB56" s="15" t="n">
+        <v>6430</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -8003,6 +8138,7 @@
       <c r="AY57" s="13" t="n"/>
       <c r="AZ57" s="15" t="n"/>
       <c r="BA57" s="15" t="n"/>
+      <c r="BB57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -8163,6 +8299,9 @@
       </c>
       <c r="BA58" s="15" t="n">
         <v>31</v>
+      </c>
+      <c r="BB58" s="15" t="n">
+        <v>38.12</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -8276,6 +8415,9 @@
       </c>
       <c r="BA59" s="15" t="n">
         <v>8000.89</v>
+      </c>
+      <c r="BB59" s="15" t="n">
+        <v>8133.25</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -8380,6 +8522,7 @@
       <c r="AY60" s="13" t="n"/>
       <c r="AZ60" s="15" t="n"/>
       <c r="BA60" s="15" t="n"/>
+      <c r="BB60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -8540,6 +8683,9 @@
       </c>
       <c r="BA61" s="15" t="n">
         <v>1.94</v>
+      </c>
+      <c r="BB61" s="15" t="n">
+        <v>3.25</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -8653,6 +8799,9 @@
       </c>
       <c r="BA62" s="15" t="n">
         <v>10771.99</v>
+      </c>
+      <c r="BB62" s="15" t="n">
+        <v>10831.37</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -8757,6 +8906,7 @@
       <c r="AY63" s="13" t="n"/>
       <c r="AZ63" s="15" t="n"/>
       <c r="BA63" s="15" t="n"/>
+      <c r="BB63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -8917,6 +9067,9 @@
       </c>
       <c r="BA64" s="15" t="n">
         <v>15.07</v>
+      </c>
+      <c r="BB64" s="15" t="n">
+        <v>17.11</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -9030,6 +9183,9 @@
       </c>
       <c r="BA65" s="15" t="n">
         <v>10992.6</v>
+      </c>
+      <c r="BB65" s="15" t="n">
+        <v>11200.76</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -9134,6 +9290,7 @@
       <c r="AY66" s="13" t="n"/>
       <c r="AZ66" s="15" t="n"/>
       <c r="BA66" s="15" t="n"/>
+      <c r="BB66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -9294,6 +9451,9 @@
       </c>
       <c r="BA67" s="15" t="n">
         <v>10.61</v>
+      </c>
+      <c r="BB67" s="15" t="n">
+        <v>15.12</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -9407,6 +9567,9 @@
       </c>
       <c r="BA68" s="15" t="n">
         <v>6620.96</v>
+      </c>
+      <c r="BB68" s="15" t="n">
+        <v>6563.87</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -9511,6 +9674,7 @@
       <c r="AY69" s="13" t="n"/>
       <c r="AZ69" s="15" t="n"/>
       <c r="BA69" s="15" t="n"/>
+      <c r="BB69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -9671,6 +9835,9 @@
       </c>
       <c r="BA70" s="15" t="n">
         <v>11.5</v>
+      </c>
+      <c r="BB70" s="15" t="n">
+        <v>14.69</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -9784,6 +9951,9 @@
       </c>
       <c r="BA71" s="15" t="n">
         <v>12666.14</v>
+      </c>
+      <c r="BB71" s="15" t="n">
+        <v>12643.91</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -9888,6 +10058,7 @@
       <c r="AY72" s="13" t="n"/>
       <c r="AZ72" s="15" t="n"/>
       <c r="BA72" s="15" t="n"/>
+      <c r="BB72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -10048,6 +10219,9 @@
       </c>
       <c r="BA73" s="15" t="n">
         <v>51.77</v>
+      </c>
+      <c r="BB73" s="15" t="n">
+        <v>52.61</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -10161,6 +10335,9 @@
       </c>
       <c r="BA74" s="15" t="n">
         <v>14021.77</v>
+      </c>
+      <c r="BB74" s="15" t="n">
+        <v>15569.82</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -10265,6 +10442,7 @@
       <c r="AY75" s="13" t="n"/>
       <c r="AZ75" s="15" t="n"/>
       <c r="BA75" s="15" t="n"/>
+      <c r="BB75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -10425,6 +10603,9 @@
       </c>
       <c r="BA76" s="15" t="n">
         <v>3.66</v>
+      </c>
+      <c r="BB76" s="15" t="n">
+        <v>3.04</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -10538,6 +10719,9 @@
       </c>
       <c r="BA77" s="15" t="n">
         <v>7047.55</v>
+      </c>
+      <c r="BB77" s="15" t="n">
+        <v>7031.82</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
@@ -10642,6 +10826,7 @@
       <c r="AY78" s="13" t="n"/>
       <c r="AZ78" s="15" t="n"/>
       <c r="BA78" s="15" t="n"/>
+      <c r="BB78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -10802,6 +10987,9 @@
       </c>
       <c r="BA79" s="15" t="n">
         <v>4.04</v>
+      </c>
+      <c r="BB79" s="15" t="n">
+        <v>4.12</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -10915,6 +11103,9 @@
       </c>
       <c r="BA80" s="15" t="n">
         <v>9140.83</v>
+      </c>
+      <c r="BB80" s="15" t="n">
+        <v>8861.790000000001</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -11019,6 +11210,7 @@
       <c r="AY81" s="13" t="n"/>
       <c r="AZ81" s="15" t="n"/>
       <c r="BA81" s="15" t="n"/>
+      <c r="BB81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -11179,6 +11371,9 @@
       </c>
       <c r="BA82" s="15" t="n">
         <v>12.66</v>
+      </c>
+      <c r="BB82" s="15" t="n">
+        <v>11.98</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -11292,6 +11487,9 @@
       </c>
       <c r="BA83" s="15" t="n">
         <v>2335.88</v>
+      </c>
+      <c r="BB83" s="15" t="n">
+        <v>2277.45</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -11396,6 +11594,7 @@
       <c r="AY84" s="13" t="n"/>
       <c r="AZ84" s="15" t="n"/>
       <c r="BA84" s="15" t="n"/>
+      <c r="BB84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -11556,6 +11755,9 @@
       </c>
       <c r="BA85" s="15" t="n">
         <v>24.17</v>
+      </c>
+      <c r="BB85" s="15" t="n">
+        <v>23.94</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -11669,6 +11871,9 @@
       </c>
       <c r="BA86" s="15" t="n">
         <v>4735.38</v>
+      </c>
+      <c r="BB86" s="15" t="n">
+        <v>4697.35</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -11773,6 +11978,7 @@
       <c r="AY87" s="13" t="n"/>
       <c r="AZ87" s="15" t="n"/>
       <c r="BA87" s="15" t="n"/>
+      <c r="BB87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -11933,6 +12139,9 @@
       </c>
       <c r="BA88" s="15" t="n">
         <v>19.87</v>
+      </c>
+      <c r="BB88" s="15" t="n">
+        <v>24.45</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -12046,6 +12255,9 @@
       </c>
       <c r="BA89" s="15" t="n">
         <v>8485.110000000001</v>
+      </c>
+      <c r="BB89" s="15" t="n">
+        <v>8615.799999999999</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -12150,6 +12362,7 @@
       <c r="AY90" s="13" t="n"/>
       <c r="AZ90" s="15" t="n"/>
       <c r="BA90" s="15" t="n"/>
+      <c r="BB90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -12310,6 +12523,9 @@
       </c>
       <c r="BA91" s="15" t="n">
         <v>3.72</v>
+      </c>
+      <c r="BB91" s="15" t="n">
+        <v>7.06</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -12423,6 +12639,9 @@
       </c>
       <c r="BA92" s="15" t="n">
         <v>1137.96</v>
+      </c>
+      <c r="BB92" s="15" t="n">
+        <v>1212.18</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -12527,6 +12746,7 @@
       <c r="AY93" s="13" t="n"/>
       <c r="AZ93" s="15" t="n"/>
       <c r="BA93" s="15" t="n"/>
+      <c r="BB93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -12687,6 +12907,9 @@
       </c>
       <c r="BA94" s="15" t="n">
         <v>4.96</v>
+      </c>
+      <c r="BB94" s="15" t="n">
+        <v>6.32</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -12800,6 +13023,9 @@
       </c>
       <c r="BA95" s="15" t="n">
         <v>13576.65</v>
+      </c>
+      <c r="BB95" s="15" t="n">
+        <v>13990.39</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -12904,6 +13130,7 @@
       <c r="AY96" s="13" t="n"/>
       <c r="AZ96" s="15" t="n"/>
       <c r="BA96" s="15" t="n"/>
+      <c r="BB96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -13064,6 +13291,9 @@
       </c>
       <c r="BA97" s="15" t="n">
         <v>41.28</v>
+      </c>
+      <c r="BB97" s="15" t="n">
+        <v>47.05</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -13177,6 +13407,9 @@
       </c>
       <c r="BA98" s="15" t="n">
         <v>3091.16</v>
+      </c>
+      <c r="BB98" s="15" t="n">
+        <v>3215.1</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -13281,6 +13514,7 @@
       <c r="AY99" s="13" t="n"/>
       <c r="AZ99" s="15" t="n"/>
       <c r="BA99" s="15" t="n"/>
+      <c r="BB99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -13441,6 +13675,9 @@
       </c>
       <c r="BA100" s="15" t="n">
         <v>35.04</v>
+      </c>
+      <c r="BB100" s="15" t="n">
+        <v>36.95</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -13554,6 +13791,9 @@
       </c>
       <c r="BA101" s="15" t="n">
         <v>2231.52</v>
+      </c>
+      <c r="BB101" s="15" t="n">
+        <v>2415.31</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -13658,6 +13898,7 @@
       <c r="AY102" s="13" t="n"/>
       <c r="AZ102" s="15" t="n"/>
       <c r="BA102" s="15" t="n"/>
+      <c r="BB102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -13818,6 +14059,9 @@
       </c>
       <c r="BA103" s="15" t="n">
         <v>12.26</v>
+      </c>
+      <c r="BB103" s="15" t="n">
+        <v>14.55</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -13931,6 +14175,9 @@
       </c>
       <c r="BA104" s="15" t="n">
         <v>2286.4</v>
+      </c>
+      <c r="BB104" s="15" t="n">
+        <v>2483.24</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -14035,6 +14282,7 @@
       <c r="AY105" s="13" t="n"/>
       <c r="AZ105" s="15" t="n"/>
       <c r="BA105" s="15" t="n"/>
+      <c r="BB105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -14195,6 +14443,9 @@
       </c>
       <c r="BA106" s="15" t="n">
         <v>37.08</v>
+      </c>
+      <c r="BB106" s="15" t="n">
+        <v>37.41</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -14308,6 +14559,9 @@
       </c>
       <c r="BA107" s="15" t="n">
         <v>2391.38</v>
+      </c>
+      <c r="BB107" s="15" t="n">
+        <v>2560.91</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -14412,6 +14666,7 @@
       <c r="AY108" s="13" t="n"/>
       <c r="AZ108" s="15" t="n"/>
       <c r="BA108" s="15" t="n"/>
+      <c r="BB108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -14572,6 +14827,9 @@
       </c>
       <c r="BA109" s="15" t="n">
         <v>56.72</v>
+      </c>
+      <c r="BB109" s="15" t="n">
+        <v>63.25</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -14685,6 +14943,9 @@
       </c>
       <c r="BA110" s="15" t="n">
         <v>1935.08</v>
+      </c>
+      <c r="BB110" s="15" t="n">
+        <v>1974.24</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -14789,6 +15050,7 @@
       <c r="AY111" s="13" t="n"/>
       <c r="AZ111" s="15" t="n"/>
       <c r="BA111" s="15" t="n"/>
+      <c r="BB111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -14949,6 +15211,9 @@
       </c>
       <c r="BA112" s="15" t="n">
         <v>20.8</v>
+      </c>
+      <c r="BB112" s="15" t="n">
+        <v>21.26</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -15062,6 +15327,9 @@
       </c>
       <c r="BA113" s="15" t="n">
         <v>8403.35</v>
+      </c>
+      <c r="BB113" s="15" t="n">
+        <v>8636.68</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -15166,6 +15434,7 @@
       <c r="AY114" s="13" t="n"/>
       <c r="AZ114" s="15" t="n"/>
       <c r="BA114" s="15" t="n"/>
+      <c r="BB114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -15326,6 +15595,9 @@
       </c>
       <c r="BA115" s="15" t="n">
         <v>96.63</v>
+      </c>
+      <c r="BB115" s="15" t="n">
+        <v>97.84999999999999</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -15424,6 +15696,9 @@
       </c>
       <c r="BA116" s="15" t="n">
         <v>12766.26</v>
+      </c>
+      <c r="BB116" s="15" t="n">
+        <v>14154.58</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -15483,6 +15758,7 @@
       <c r="AY117" s="13" t="n"/>
       <c r="AZ117" s="15" t="n"/>
       <c r="BA117" s="15" t="n"/>
+      <c r="BB117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -15599,6 +15875,9 @@
       <c r="BA118" s="15" t="n">
         <v>37.22</v>
       </c>
+      <c r="BB118" s="15" t="n">
+        <v>41.63</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -15687,6 +15966,9 @@
       </c>
       <c r="BA119" s="15" t="n">
         <v>10528.94</v>
+      </c>
+      <c r="BB119" s="15" t="n">
+        <v>11141.11</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -15695,6 +15977,7 @@
       <c r="AY120" s="13" t="n"/>
       <c r="AZ120" s="15" t="n"/>
       <c r="BA120" s="15" t="n"/>
+      <c r="BB120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -15712,6 +15995,9 @@
       <c r="BA121" s="15" t="n">
         <v>28.34</v>
       </c>
+      <c r="BB121" s="15" t="n">
+        <v>28.23</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -15728,6 +16014,9 @@
       </c>
       <c r="BA122" s="15" t="n">
         <v>1843.85</v>
+      </c>
+      <c r="BB122" s="15" t="n">
+        <v>1842.78</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -15736,6 +16025,7 @@
       <c r="AY123" s="13" t="n"/>
       <c r="AZ123" s="15" t="n"/>
       <c r="BA123" s="15" t="n"/>
+      <c r="BB123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -15753,6 +16043,9 @@
       <c r="BA124" s="15" t="n">
         <v>13.99</v>
       </c>
+      <c r="BB124" s="15" t="n">
+        <v>15.89</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -15769,6 +16062,9 @@
       </c>
       <c r="BA125" s="15" t="n">
         <v>773.9</v>
+      </c>
+      <c r="BB125" s="15" t="n">
+        <v>785.35</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -15777,6 +16073,7 @@
       <c r="AY126" s="13" t="n"/>
       <c r="AZ126" s="15" t="n"/>
       <c r="BA126" s="15" t="n"/>
+      <c r="BB126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -15794,6 +16091,9 @@
       <c r="BA127" s="15" t="n">
         <v>49.31</v>
       </c>
+      <c r="BB127" s="15" t="n">
+        <v>62.08</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -15810,6 +16110,9 @@
       </c>
       <c r="BA128" s="15" t="n">
         <v>2674.28</v>
+      </c>
+      <c r="BB128" s="15" t="n">
+        <v>2871.1</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -15818,6 +16121,7 @@
       <c r="AY129" s="13" t="n"/>
       <c r="AZ129" s="15" t="n"/>
       <c r="BA129" s="15" t="n"/>
+      <c r="BB129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -15835,6 +16139,9 @@
       <c r="BA130" s="15" t="n">
         <v>19.71</v>
       </c>
+      <c r="BB130" s="15" t="n">
+        <v>20.38</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -15851,6 +16158,9 @@
       </c>
       <c r="BA131" s="15" t="n">
         <v>3449.02</v>
+      </c>
+      <c r="BB131" s="15" t="n">
+        <v>3561.99</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -15859,6 +16169,7 @@
       <c r="AY132" s="13" t="n"/>
       <c r="AZ132" s="15" t="n"/>
       <c r="BA132" s="15" t="n"/>
+      <c r="BB132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -15876,6 +16187,9 @@
       <c r="BA133" s="15" t="n">
         <v>1.52</v>
       </c>
+      <c r="BB133" s="15" t="n">
+        <v>1.52</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -15892,6 +16206,9 @@
       </c>
       <c r="BA134" s="15" t="n">
         <v>2269.39</v>
+      </c>
+      <c r="BB134" s="15" t="n">
+        <v>2287.24</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -15900,6 +16217,7 @@
       <c r="AY135" s="13" t="n"/>
       <c r="AZ135" s="15" t="n"/>
       <c r="BA135" s="15" t="n"/>
+      <c r="BB135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -15917,6 +16235,9 @@
       <c r="BA136" s="15" t="n">
         <v>4.95</v>
       </c>
+      <c r="BB136" s="15" t="n">
+        <v>6.54</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -15933,6 +16254,9 @@
       </c>
       <c r="BA137" s="15" t="n">
         <v>5197.16</v>
+      </c>
+      <c r="BB137" s="15" t="n">
+        <v>5251.87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-07-27 06:54:38]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB137"/>
+  <dimension ref="A1:BC137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -588,6 +588,7 @@
     <col width="15" customWidth="1" min="52" max="52"/>
     <col width="15" customWidth="1" min="53" max="53"/>
     <col width="15" customWidth="1" min="54" max="54"/>
+    <col width="15" customWidth="1" min="55" max="55"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -861,6 +862,11 @@
           <t>2026/07/23</t>
         </is>
       </c>
+      <c r="BC1" s="15" t="inlineStr">
+        <is>
+          <t>2026/07/27</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1133,6 +1139,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BC2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1297,6 +1308,9 @@
       <c r="BB3" s="15" t="n">
         <v>61.97</v>
       </c>
+      <c r="BC3" s="15" t="n">
+        <v>60.12</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1460,6 +1474,9 @@
       </c>
       <c r="BB4" s="15" t="n">
         <v>3869.94</v>
+      </c>
+      <c r="BC4" s="15" t="n">
+        <v>3854.07</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1517,6 +1534,7 @@
       <c r="AZ5" s="15" t="n"/>
       <c r="BA5" s="15" t="n"/>
       <c r="BB5" s="15" t="n"/>
+      <c r="BC5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1621,6 +1639,7 @@
       <c r="AZ6" s="15" t="n"/>
       <c r="BA6" s="15" t="n"/>
       <c r="BB6" s="15" t="n"/>
+      <c r="BC6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1784,6 +1803,9 @@
       </c>
       <c r="BB7" s="15" t="n">
         <v>64.72</v>
+      </c>
+      <c r="BC7" s="15" t="n">
+        <v>62.02</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -1900,6 +1922,9 @@
       </c>
       <c r="BB8" s="15" t="n">
         <v>5804.21</v>
+      </c>
+      <c r="BC8" s="15" t="n">
+        <v>5784.23</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2005,6 +2030,7 @@
       <c r="AZ9" s="15" t="n"/>
       <c r="BA9" s="15" t="n"/>
       <c r="BB9" s="15" t="n"/>
+      <c r="BC9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2168,6 +2194,9 @@
       </c>
       <c r="BB10" s="15" t="n">
         <v>58.9</v>
+      </c>
+      <c r="BC10" s="15" t="n">
+        <v>54.9</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2284,6 +2313,9 @@
       </c>
       <c r="BB11" s="15" t="n">
         <v>4719.71</v>
+      </c>
+      <c r="BC11" s="15" t="n">
+        <v>4696.85</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -2389,6 +2421,7 @@
       <c r="AZ12" s="15" t="n"/>
       <c r="BA12" s="15" t="n"/>
       <c r="BB12" s="15" t="n"/>
+      <c r="BC12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2552,6 +2585,9 @@
       </c>
       <c r="BB13" s="15" t="n">
         <v>65.84</v>
+      </c>
+      <c r="BC13" s="15" t="n">
+        <v>63.42</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -2668,6 +2704,9 @@
       </c>
       <c r="BB14" s="15" t="n">
         <v>7718.78</v>
+      </c>
+      <c r="BC14" s="15" t="n">
+        <v>7713.98</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -2773,6 +2812,7 @@
       <c r="AZ15" s="15" t="n"/>
       <c r="BA15" s="15" t="n"/>
       <c r="BB15" s="15" t="n"/>
+      <c r="BC15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -2936,6 +2976,9 @@
       </c>
       <c r="BB16" s="15" t="n">
         <v>37.71</v>
+      </c>
+      <c r="BC16" s="15" t="n">
+        <v>35.12</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -3052,6 +3095,9 @@
       </c>
       <c r="BB17" s="15" t="n">
         <v>2609.87</v>
+      </c>
+      <c r="BC17" s="15" t="n">
+        <v>2601.82</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -3157,6 +3203,7 @@
       <c r="AZ18" s="15" t="n"/>
       <c r="BA18" s="15" t="n"/>
       <c r="BB18" s="15" t="n"/>
+      <c r="BC18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -3320,6 +3367,9 @@
       </c>
       <c r="BB19" s="15" t="n">
         <v>86.2</v>
+      </c>
+      <c r="BC19" s="15" t="n">
+        <v>81.86</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -3436,6 +3486,9 @@
       </c>
       <c r="BB20" s="15" t="n">
         <v>7498.96</v>
+      </c>
+      <c r="BC20" s="15" t="n">
+        <v>7411.98</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -3541,6 +3594,7 @@
       <c r="AZ21" s="15" t="n"/>
       <c r="BA21" s="15" t="n"/>
       <c r="BB21" s="15" t="n"/>
+      <c r="BC21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -3701,6 +3755,9 @@
         <v>36.34</v>
       </c>
       <c r="BB22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BC22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -3818,6 +3875,9 @@
       </c>
       <c r="BB23" s="15" t="n">
         <v>76562.36</v>
+      </c>
+      <c r="BC23" s="15" t="n">
+        <v>76719.09</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -3923,6 +3983,7 @@
       <c r="AZ24" s="15" t="n"/>
       <c r="BA24" s="15" t="n"/>
       <c r="BB24" s="15" t="n"/>
+      <c r="BC24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -4085,6 +4146,9 @@
         <v>49.88</v>
       </c>
       <c r="BB25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BC25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -4195,6 +4259,9 @@
         <v>24830.98</v>
       </c>
       <c r="BB26" s="15" t="inlineStr"/>
+      <c r="BC26" s="15" t="n">
+        <v>25099</v>
+      </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -4299,6 +4366,7 @@
       <c r="AZ27" s="15" t="n"/>
       <c r="BA27" s="15" t="n"/>
       <c r="BB27" s="15" t="n"/>
+      <c r="BC27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -4461,6 +4529,9 @@
         <v>92.09</v>
       </c>
       <c r="BB28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BC28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -4578,6 +4649,9 @@
       </c>
       <c r="BB29" s="15" t="n">
         <v>66218.11</v>
+      </c>
+      <c r="BC29" s="15" t="n">
+        <v>64931.19</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -4683,6 +4757,7 @@
       <c r="AZ30" s="15" t="n"/>
       <c r="BA30" s="15" t="n"/>
       <c r="BB30" s="15" t="n"/>
+      <c r="BC30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -4846,6 +4921,9 @@
       </c>
       <c r="BB31" s="15" t="n">
         <v>45.65</v>
+      </c>
+      <c r="BC31" s="15" t="n">
+        <v>46.21</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -4962,6 +5040,9 @@
       </c>
       <c r="BB32" s="15" t="n">
         <v>5501.53</v>
+      </c>
+      <c r="BC32" s="15" t="n">
+        <v>5433.84</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -5067,6 +5148,7 @@
       <c r="AZ33" s="15" t="n"/>
       <c r="BA33" s="15" t="n"/>
       <c r="BB33" s="15" t="n"/>
+      <c r="BC33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -5230,6 +5312,9 @@
       </c>
       <c r="BB34" s="15" t="n">
         <v>60.39</v>
+      </c>
+      <c r="BC34" s="15" t="n">
+        <v>59.14</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -5346,6 +5431,9 @@
       </c>
       <c r="BB35" s="15" t="n">
         <v>11459.52</v>
+      </c>
+      <c r="BC35" s="15" t="n">
+        <v>11383.25</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -5451,6 +5539,7 @@
       <c r="AZ36" s="15" t="n"/>
       <c r="BA36" s="15" t="n"/>
       <c r="BB36" s="15" t="n"/>
+      <c r="BC36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -5614,6 +5703,9 @@
       </c>
       <c r="BB37" s="15" t="n">
         <v>50.33</v>
+      </c>
+      <c r="BC37" s="15" t="n">
+        <v>50.24</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -5730,6 +5822,9 @@
       </c>
       <c r="BB38" s="15" t="n">
         <v>10824.3</v>
+      </c>
+      <c r="BC38" s="15" t="n">
+        <v>10775.41</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -5835,6 +5930,7 @@
       <c r="AZ39" s="15" t="n"/>
       <c r="BA39" s="15" t="n"/>
       <c r="BB39" s="15" t="n"/>
+      <c r="BC39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -5998,6 +6094,9 @@
       </c>
       <c r="BB40" s="15" t="n">
         <v>50.04</v>
+      </c>
+      <c r="BC40" s="15" t="n">
+        <v>51.01</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -6114,6 +6213,9 @@
       </c>
       <c r="BB41" s="15" t="n">
         <v>3178.04</v>
+      </c>
+      <c r="BC41" s="15" t="n">
+        <v>3140.45</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -6219,6 +6321,7 @@
       <c r="AZ42" s="15" t="n"/>
       <c r="BA42" s="15" t="n"/>
       <c r="BB42" s="15" t="n"/>
+      <c r="BC42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -6382,6 +6485,9 @@
       </c>
       <c r="BB43" s="15" t="n">
         <v>58.34</v>
+      </c>
+      <c r="BC43" s="15" t="n">
+        <v>57.84</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -6498,6 +6604,9 @@
       </c>
       <c r="BB44" s="15" t="n">
         <v>7018.33</v>
+      </c>
+      <c r="BC44" s="15" t="n">
+        <v>7000.09</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -6603,6 +6712,7 @@
       <c r="AZ45" s="15" t="n"/>
       <c r="BA45" s="15" t="n"/>
       <c r="BB45" s="15" t="n"/>
+      <c r="BC45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -6766,6 +6876,9 @@
       </c>
       <c r="BB46" s="15" t="n">
         <v>29.76</v>
+      </c>
+      <c r="BC46" s="15" t="n">
+        <v>26.48</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -6882,6 +6995,9 @@
       </c>
       <c r="BB47" s="15" t="n">
         <v>33050.75</v>
+      </c>
+      <c r="BC47" s="15" t="n">
+        <v>32210.4</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -6987,6 +7103,7 @@
       <c r="AZ48" s="15" t="n"/>
       <c r="BA48" s="15" t="n"/>
       <c r="BB48" s="15" t="n"/>
+      <c r="BC48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -7150,6 +7267,9 @@
       </c>
       <c r="BB49" s="15" t="n">
         <v>51.95</v>
+      </c>
+      <c r="BC49" s="15" t="n">
+        <v>47.45</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -7266,6 +7386,9 @@
       </c>
       <c r="BB50" s="15" t="n">
         <v>3794.8</v>
+      </c>
+      <c r="BC50" s="15" t="n">
+        <v>3815.48</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -7371,6 +7494,7 @@
       <c r="AZ51" s="15" t="n"/>
       <c r="BA51" s="15" t="n"/>
       <c r="BB51" s="15" t="n"/>
+      <c r="BC51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -7534,6 +7658,9 @@
       </c>
       <c r="BB52" s="15" t="n">
         <v>61.41</v>
+      </c>
+      <c r="BC52" s="15" t="n">
+        <v>55.86</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -7650,6 +7777,9 @@
       </c>
       <c r="BB53" s="15" t="n">
         <v>3563.63</v>
+      </c>
+      <c r="BC53" s="15" t="n">
+        <v>3584.35</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -7755,6 +7885,7 @@
       <c r="AZ54" s="15" t="n"/>
       <c r="BA54" s="15" t="n"/>
       <c r="BB54" s="15" t="n"/>
+      <c r="BC54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -7918,6 +8049,9 @@
       </c>
       <c r="BB55" s="15" t="n">
         <v>11.14</v>
+      </c>
+      <c r="BC55" s="15" t="n">
+        <v>7.68</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -8034,6 +8168,9 @@
       </c>
       <c r="BB56" s="15" t="n">
         <v>6430</v>
+      </c>
+      <c r="BC56" s="15" t="n">
+        <v>6360.11</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -8139,6 +8276,7 @@
       <c r="AZ57" s="15" t="n"/>
       <c r="BA57" s="15" t="n"/>
       <c r="BB57" s="15" t="n"/>
+      <c r="BC57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -8302,6 +8440,9 @@
       </c>
       <c r="BB58" s="15" t="n">
         <v>38.12</v>
+      </c>
+      <c r="BC58" s="15" t="n">
+        <v>31.45</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -8418,6 +8559,9 @@
       </c>
       <c r="BB59" s="15" t="n">
         <v>8133.25</v>
+      </c>
+      <c r="BC59" s="15" t="n">
+        <v>7928.36</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -8523,6 +8667,7 @@
       <c r="AZ60" s="15" t="n"/>
       <c r="BA60" s="15" t="n"/>
       <c r="BB60" s="15" t="n"/>
+      <c r="BC60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -8686,6 +8831,9 @@
       </c>
       <c r="BB61" s="15" t="n">
         <v>3.25</v>
+      </c>
+      <c r="BC61" s="15" t="n">
+        <v>2.6</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -8802,6 +8950,9 @@
       </c>
       <c r="BB62" s="15" t="n">
         <v>10831.37</v>
+      </c>
+      <c r="BC62" s="15" t="n">
+        <v>10720.79</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -8907,6 +9058,7 @@
       <c r="AZ63" s="15" t="n"/>
       <c r="BA63" s="15" t="n"/>
       <c r="BB63" s="15" t="n"/>
+      <c r="BC63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -9070,6 +9222,9 @@
       </c>
       <c r="BB64" s="15" t="n">
         <v>17.11</v>
+      </c>
+      <c r="BC64" s="15" t="n">
+        <v>13.34</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -9186,6 +9341,9 @@
       </c>
       <c r="BB65" s="15" t="n">
         <v>11200.76</v>
+      </c>
+      <c r="BC65" s="15" t="n">
+        <v>11178.06</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -9291,6 +9449,7 @@
       <c r="AZ66" s="15" t="n"/>
       <c r="BA66" s="15" t="n"/>
       <c r="BB66" s="15" t="n"/>
+      <c r="BC66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -9454,6 +9613,9 @@
       </c>
       <c r="BB67" s="15" t="n">
         <v>15.12</v>
+      </c>
+      <c r="BC67" s="15" t="n">
+        <v>13.54</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -9570,6 +9732,9 @@
       </c>
       <c r="BB68" s="15" t="n">
         <v>6563.87</v>
+      </c>
+      <c r="BC68" s="15" t="n">
+        <v>6469.83</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -9675,6 +9840,7 @@
       <c r="AZ69" s="15" t="n"/>
       <c r="BA69" s="15" t="n"/>
       <c r="BB69" s="15" t="n"/>
+      <c r="BC69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -9838,6 +10004,9 @@
       </c>
       <c r="BB70" s="15" t="n">
         <v>14.69</v>
+      </c>
+      <c r="BC70" s="15" t="n">
+        <v>12.96</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -9954,6 +10123,9 @@
       </c>
       <c r="BB71" s="15" t="n">
         <v>12643.91</v>
+      </c>
+      <c r="BC71" s="15" t="n">
+        <v>12470.65</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -10059,6 +10231,7 @@
       <c r="AZ72" s="15" t="n"/>
       <c r="BA72" s="15" t="n"/>
       <c r="BB72" s="15" t="n"/>
+      <c r="BC72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -10222,6 +10395,9 @@
       </c>
       <c r="BB73" s="15" t="n">
         <v>52.61</v>
+      </c>
+      <c r="BC73" s="15" t="n">
+        <v>52.27</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -10338,6 +10514,9 @@
       </c>
       <c r="BB74" s="15" t="n">
         <v>15569.82</v>
+      </c>
+      <c r="BC74" s="15" t="n">
+        <v>14099.43</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -10443,6 +10622,7 @@
       <c r="AZ75" s="15" t="n"/>
       <c r="BA75" s="15" t="n"/>
       <c r="BB75" s="15" t="n"/>
+      <c r="BC75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -10606,6 +10786,9 @@
       </c>
       <c r="BB76" s="15" t="n">
         <v>3.04</v>
+      </c>
+      <c r="BC76" s="15" t="n">
+        <v>2.86</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -10722,6 +10905,9 @@
       </c>
       <c r="BB77" s="15" t="n">
         <v>7031.82</v>
+      </c>
+      <c r="BC77" s="15" t="n">
+        <v>6818.12</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
@@ -10827,6 +11013,7 @@
       <c r="AZ78" s="15" t="n"/>
       <c r="BA78" s="15" t="n"/>
       <c r="BB78" s="15" t="n"/>
+      <c r="BC78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -10990,6 +11177,9 @@
       </c>
       <c r="BB79" s="15" t="n">
         <v>4.12</v>
+      </c>
+      <c r="BC79" s="15" t="n">
+        <v>3.09</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -11106,6 +11296,9 @@
       </c>
       <c r="BB80" s="15" t="n">
         <v>8861.790000000001</v>
+      </c>
+      <c r="BC80" s="15" t="n">
+        <v>8831.42</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -11211,6 +11404,7 @@
       <c r="AZ81" s="15" t="n"/>
       <c r="BA81" s="15" t="n"/>
       <c r="BB81" s="15" t="n"/>
+      <c r="BC81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -11374,6 +11568,9 @@
       </c>
       <c r="BB82" s="15" t="n">
         <v>11.98</v>
+      </c>
+      <c r="BC82" s="15" t="n">
+        <v>11.34</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -11490,6 +11687,9 @@
       </c>
       <c r="BB83" s="15" t="n">
         <v>2277.45</v>
+      </c>
+      <c r="BC83" s="15" t="n">
+        <v>2280.38</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -11595,6 +11795,7 @@
       <c r="AZ84" s="15" t="n"/>
       <c r="BA84" s="15" t="n"/>
       <c r="BB84" s="15" t="n"/>
+      <c r="BC84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -11758,6 +11959,9 @@
       </c>
       <c r="BB85" s="15" t="n">
         <v>23.94</v>
+      </c>
+      <c r="BC85" s="15" t="n">
+        <v>23.08</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -11874,6 +12078,9 @@
       </c>
       <c r="BB86" s="15" t="n">
         <v>4697.35</v>
+      </c>
+      <c r="BC86" s="15" t="n">
+        <v>4713.64</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -11979,6 +12186,7 @@
       <c r="AZ87" s="15" t="n"/>
       <c r="BA87" s="15" t="n"/>
       <c r="BB87" s="15" t="n"/>
+      <c r="BC87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -12142,6 +12350,9 @@
       </c>
       <c r="BB88" s="15" t="n">
         <v>24.45</v>
+      </c>
+      <c r="BC88" s="15" t="n">
+        <v>19.73</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -12258,6 +12469,9 @@
       </c>
       <c r="BB89" s="15" t="n">
         <v>8615.799999999999</v>
+      </c>
+      <c r="BC89" s="15" t="n">
+        <v>8476.440000000001</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -12363,6 +12577,7 @@
       <c r="AZ90" s="15" t="n"/>
       <c r="BA90" s="15" t="n"/>
       <c r="BB90" s="15" t="n"/>
+      <c r="BC90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -12526,6 +12741,9 @@
       </c>
       <c r="BB91" s="15" t="n">
         <v>7.06</v>
+      </c>
+      <c r="BC91" s="15" t="n">
+        <v>6.58</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -12642,6 +12860,9 @@
       </c>
       <c r="BB92" s="15" t="n">
         <v>1212.18</v>
+      </c>
+      <c r="BC92" s="15" t="n">
+        <v>1204.84</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -12747,6 +12968,7 @@
       <c r="AZ93" s="15" t="n"/>
       <c r="BA93" s="15" t="n"/>
       <c r="BB93" s="15" t="n"/>
+      <c r="BC93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -12910,6 +13132,9 @@
       </c>
       <c r="BB94" s="15" t="n">
         <v>6.32</v>
+      </c>
+      <c r="BC94" s="15" t="n">
+        <v>5.51</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -13026,6 +13251,9 @@
       </c>
       <c r="BB95" s="15" t="n">
         <v>13990.39</v>
+      </c>
+      <c r="BC95" s="15" t="n">
+        <v>13757.19</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -13131,6 +13359,7 @@
       <c r="AZ96" s="15" t="n"/>
       <c r="BA96" s="15" t="n"/>
       <c r="BB96" s="15" t="n"/>
+      <c r="BC96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -13294,6 +13523,9 @@
       </c>
       <c r="BB97" s="15" t="n">
         <v>47.05</v>
+      </c>
+      <c r="BC97" s="15" t="n">
+        <v>43.06</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -13410,6 +13642,9 @@
       </c>
       <c r="BB98" s="15" t="n">
         <v>3215.1</v>
+      </c>
+      <c r="BC98" s="15" t="n">
+        <v>3093.89</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -13515,6 +13750,7 @@
       <c r="AZ99" s="15" t="n"/>
       <c r="BA99" s="15" t="n"/>
       <c r="BB99" s="15" t="n"/>
+      <c r="BC99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -13678,6 +13914,9 @@
       </c>
       <c r="BB100" s="15" t="n">
         <v>36.95</v>
+      </c>
+      <c r="BC100" s="15" t="n">
+        <v>34.75</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -13794,6 +14033,9 @@
       </c>
       <c r="BB101" s="15" t="n">
         <v>2415.31</v>
+      </c>
+      <c r="BC101" s="15" t="n">
+        <v>2414.39</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -13899,6 +14141,7 @@
       <c r="AZ102" s="15" t="n"/>
       <c r="BA102" s="15" t="n"/>
       <c r="BB102" s="15" t="n"/>
+      <c r="BC102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -14062,6 +14305,9 @@
       </c>
       <c r="BB103" s="15" t="n">
         <v>14.55</v>
+      </c>
+      <c r="BC103" s="15" t="n">
+        <v>14.06</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -14177,6 +14423,9 @@
         <v>2286.4</v>
       </c>
       <c r="BB104" s="15" t="n">
+        <v>2483.24</v>
+      </c>
+      <c r="BC104" s="15" t="n">
         <v>2483.24</v>
       </c>
     </row>
@@ -14283,6 +14532,7 @@
       <c r="AZ105" s="15" t="n"/>
       <c r="BA105" s="15" t="n"/>
       <c r="BB105" s="15" t="n"/>
+      <c r="BC105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -14446,6 +14696,9 @@
       </c>
       <c r="BB106" s="15" t="n">
         <v>37.41</v>
+      </c>
+      <c r="BC106" s="15" t="n">
+        <v>35.95</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -14562,6 +14815,9 @@
       </c>
       <c r="BB107" s="15" t="n">
         <v>2560.91</v>
+      </c>
+      <c r="BC107" s="15" t="n">
+        <v>2561.13</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -14667,6 +14923,7 @@
       <c r="AZ108" s="15" t="n"/>
       <c r="BA108" s="15" t="n"/>
       <c r="BB108" s="15" t="n"/>
+      <c r="BC108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -14830,6 +15087,9 @@
       </c>
       <c r="BB109" s="15" t="n">
         <v>63.25</v>
+      </c>
+      <c r="BC109" s="15" t="n">
+        <v>57.98</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -14946,6 +15206,9 @@
       </c>
       <c r="BB110" s="15" t="n">
         <v>1974.24</v>
+      </c>
+      <c r="BC110" s="15" t="n">
+        <v>1894.98</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -15051,6 +15314,7 @@
       <c r="AZ111" s="15" t="n"/>
       <c r="BA111" s="15" t="n"/>
       <c r="BB111" s="15" t="n"/>
+      <c r="BC111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -15214,6 +15478,9 @@
       </c>
       <c r="BB112" s="15" t="n">
         <v>21.26</v>
+      </c>
+      <c r="BC112" s="15" t="n">
+        <v>19.6</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -15330,6 +15597,9 @@
       </c>
       <c r="BB113" s="15" t="n">
         <v>8636.68</v>
+      </c>
+      <c r="BC113" s="15" t="n">
+        <v>8516.059999999999</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -15435,6 +15705,7 @@
       <c r="AZ114" s="15" t="n"/>
       <c r="BA114" s="15" t="n"/>
       <c r="BB114" s="15" t="n"/>
+      <c r="BC114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -15598,6 +15869,9 @@
       </c>
       <c r="BB115" s="15" t="n">
         <v>97.84999999999999</v>
+      </c>
+      <c r="BC115" s="15" t="n">
+        <v>97.22</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -15699,6 +15973,9 @@
       </c>
       <c r="BB116" s="15" t="n">
         <v>14154.58</v>
+      </c>
+      <c r="BC116" s="15" t="n">
+        <v>14152.29</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -15759,6 +16036,7 @@
       <c r="AZ117" s="15" t="n"/>
       <c r="BA117" s="15" t="n"/>
       <c r="BB117" s="15" t="n"/>
+      <c r="BC117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -15878,6 +16156,9 @@
       <c r="BB118" s="15" t="n">
         <v>41.63</v>
       </c>
+      <c r="BC118" s="15" t="n">
+        <v>40.41</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -15969,6 +16250,9 @@
       </c>
       <c r="BB119" s="15" t="n">
         <v>11141.11</v>
+      </c>
+      <c r="BC119" s="15" t="n">
+        <v>11182.8</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -15978,6 +16262,7 @@
       <c r="AZ120" s="15" t="n"/>
       <c r="BA120" s="15" t="n"/>
       <c r="BB120" s="15" t="n"/>
+      <c r="BC120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -15998,6 +16283,9 @@
       <c r="BB121" s="15" t="n">
         <v>28.23</v>
       </c>
+      <c r="BC121" s="15" t="n">
+        <v>27.4</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -16017,6 +16305,9 @@
       </c>
       <c r="BB122" s="15" t="n">
         <v>1842.78</v>
+      </c>
+      <c r="BC122" s="15" t="n">
+        <v>1810.95</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -16026,6 +16317,7 @@
       <c r="AZ123" s="15" t="n"/>
       <c r="BA123" s="15" t="n"/>
       <c r="BB123" s="15" t="n"/>
+      <c r="BC123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -16046,6 +16338,9 @@
       <c r="BB124" s="15" t="n">
         <v>15.89</v>
       </c>
+      <c r="BC124" s="15" t="n">
+        <v>13.93</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -16065,6 +16360,9 @@
       </c>
       <c r="BB125" s="15" t="n">
         <v>785.35</v>
+      </c>
+      <c r="BC125" s="15" t="n">
+        <v>770.9</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -16074,6 +16372,7 @@
       <c r="AZ126" s="15" t="n"/>
       <c r="BA126" s="15" t="n"/>
       <c r="BB126" s="15" t="n"/>
+      <c r="BC126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -16094,6 +16393,9 @@
       <c r="BB127" s="15" t="n">
         <v>62.08</v>
       </c>
+      <c r="BC127" s="15" t="n">
+        <v>59.52</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -16113,6 +16415,9 @@
       </c>
       <c r="BB128" s="15" t="n">
         <v>2871.1</v>
+      </c>
+      <c r="BC128" s="15" t="n">
+        <v>2745.29</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -16122,6 +16427,7 @@
       <c r="AZ129" s="15" t="n"/>
       <c r="BA129" s="15" t="n"/>
       <c r="BB129" s="15" t="n"/>
+      <c r="BC129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -16142,6 +16448,9 @@
       <c r="BB130" s="15" t="n">
         <v>20.38</v>
       </c>
+      <c r="BC130" s="15" t="n">
+        <v>19.84</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -16161,6 +16470,9 @@
       </c>
       <c r="BB131" s="15" t="n">
         <v>3561.99</v>
+      </c>
+      <c r="BC131" s="15" t="n">
+        <v>3542.49</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -16170,6 +16482,7 @@
       <c r="AZ132" s="15" t="n"/>
       <c r="BA132" s="15" t="n"/>
       <c r="BB132" s="15" t="n"/>
+      <c r="BC132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -16190,6 +16503,9 @@
       <c r="BB133" s="15" t="n">
         <v>1.52</v>
       </c>
+      <c r="BC133" s="15" t="n">
+        <v>1.36</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -16209,6 +16525,9 @@
       </c>
       <c r="BB134" s="15" t="n">
         <v>2287.24</v>
+      </c>
+      <c r="BC134" s="15" t="n">
+        <v>2273.63</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -16218,6 +16537,7 @@
       <c r="AZ135" s="15" t="n"/>
       <c r="BA135" s="15" t="n"/>
       <c r="BB135" s="15" t="n"/>
+      <c r="BC135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -16238,6 +16558,9 @@
       <c r="BB136" s="15" t="n">
         <v>6.54</v>
       </c>
+      <c r="BC136" s="15" t="n">
+        <v>7.41</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -16257,6 +16580,9 @@
       </c>
       <c r="BB137" s="15" t="n">
         <v>5251.87</v>
+      </c>
+      <c r="BC137" s="15" t="n">
+        <v>5272.37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-07-30 06:13:17]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BC137"/>
+  <dimension ref="A1:BD137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -589,6 +589,7 @@
     <col width="15" customWidth="1" min="53" max="53"/>
     <col width="15" customWidth="1" min="54" max="54"/>
     <col width="15" customWidth="1" min="55" max="55"/>
+    <col width="15" customWidth="1" min="56" max="56"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -867,6 +868,11 @@
           <t>2026/07/27</t>
         </is>
       </c>
+      <c r="BD1" s="15" t="inlineStr">
+        <is>
+          <t>2026/07/30</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1144,6 +1150,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BD2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1311,6 +1322,9 @@
       <c r="BC3" s="15" t="n">
         <v>60.12</v>
       </c>
+      <c r="BD3" s="15" t="n">
+        <v>59.47</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1477,6 +1491,9 @@
       </c>
       <c r="BC4" s="15" t="n">
         <v>3854.07</v>
+      </c>
+      <c r="BD4" s="15" t="n">
+        <v>3811.7</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1535,6 +1552,7 @@
       <c r="BA5" s="15" t="n"/>
       <c r="BB5" s="15" t="n"/>
       <c r="BC5" s="15" t="n"/>
+      <c r="BD5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1640,6 +1658,7 @@
       <c r="BA6" s="15" t="n"/>
       <c r="BB6" s="15" t="n"/>
       <c r="BC6" s="15" t="n"/>
+      <c r="BD6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1806,6 +1825,9 @@
       </c>
       <c r="BC7" s="15" t="n">
         <v>62.02</v>
+      </c>
+      <c r="BD7" s="15" t="n">
+        <v>61.92</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -1925,6 +1947,9 @@
       </c>
       <c r="BC8" s="15" t="n">
         <v>5784.23</v>
+      </c>
+      <c r="BD8" s="15" t="n">
+        <v>5591.62</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2031,6 +2056,7 @@
       <c r="BA9" s="15" t="n"/>
       <c r="BB9" s="15" t="n"/>
       <c r="BC9" s="15" t="n"/>
+      <c r="BD9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2197,6 +2223,9 @@
       </c>
       <c r="BC10" s="15" t="n">
         <v>54.9</v>
+      </c>
+      <c r="BD10" s="15" t="n">
+        <v>55.48</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2316,6 +2345,9 @@
       </c>
       <c r="BC11" s="15" t="n">
         <v>4696.85</v>
+      </c>
+      <c r="BD11" s="15" t="n">
+        <v>4571.35</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -2422,6 +2454,7 @@
       <c r="BA12" s="15" t="n"/>
       <c r="BB12" s="15" t="n"/>
       <c r="BC12" s="15" t="n"/>
+      <c r="BD12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2588,6 +2621,9 @@
       </c>
       <c r="BC13" s="15" t="n">
         <v>63.42</v>
+      </c>
+      <c r="BD13" s="15" t="n">
+        <v>63.03</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -2707,6 +2743,9 @@
       </c>
       <c r="BC14" s="15" t="n">
         <v>7713.98</v>
+      </c>
+      <c r="BD14" s="15" t="n">
+        <v>7364.04</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -2813,6 +2852,7 @@
       <c r="BA15" s="15" t="n"/>
       <c r="BB15" s="15" t="n"/>
       <c r="BC15" s="15" t="n"/>
+      <c r="BD15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -2979,6 +3019,9 @@
       </c>
       <c r="BC16" s="15" t="n">
         <v>35.12</v>
+      </c>
+      <c r="BD16" s="15" t="n">
+        <v>35.67</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -3098,6 +3141,9 @@
       </c>
       <c r="BC17" s="15" t="n">
         <v>2601.82</v>
+      </c>
+      <c r="BD17" s="15" t="n">
+        <v>2536.29</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -3204,6 +3250,7 @@
       <c r="BA18" s="15" t="n"/>
       <c r="BB18" s="15" t="n"/>
       <c r="BC18" s="15" t="n"/>
+      <c r="BD18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -3370,6 +3417,9 @@
       </c>
       <c r="BC19" s="15" t="n">
         <v>81.86</v>
+      </c>
+      <c r="BD19" s="15" t="n">
+        <v>81.75</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -3489,6 +3539,9 @@
       </c>
       <c r="BC20" s="15" t="n">
         <v>7411.98</v>
+      </c>
+      <c r="BD20" s="15" t="n">
+        <v>7316.15</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -3595,6 +3648,7 @@
       <c r="BA21" s="15" t="n"/>
       <c r="BB21" s="15" t="n"/>
       <c r="BC21" s="15" t="n"/>
+      <c r="BD21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -3758,6 +3812,9 @@
         <v>36.34</v>
       </c>
       <c r="BC22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BD22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -3878,6 +3935,9 @@
       </c>
       <c r="BC23" s="15" t="n">
         <v>76719.09</v>
+      </c>
+      <c r="BD23" s="15" t="n">
+        <v>77689.99000000001</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -3984,6 +4044,7 @@
       <c r="BA24" s="15" t="n"/>
       <c r="BB24" s="15" t="n"/>
       <c r="BC24" s="15" t="n"/>
+      <c r="BD24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -4149,6 +4210,9 @@
         <v>49.88</v>
       </c>
       <c r="BC25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BD25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -4262,6 +4326,7 @@
       <c r="BC26" s="15" t="n">
         <v>25099</v>
       </c>
+      <c r="BD26" s="15" t="inlineStr"/>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -4367,6 +4432,7 @@
       <c r="BA27" s="15" t="n"/>
       <c r="BB27" s="15" t="n"/>
       <c r="BC27" s="15" t="n"/>
+      <c r="BD27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -4532,6 +4598,9 @@
         <v>92.09</v>
       </c>
       <c r="BC28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BD28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -4652,6 +4721,9 @@
       </c>
       <c r="BC29" s="15" t="n">
         <v>64931.19</v>
+      </c>
+      <c r="BD29" s="15" t="n">
+        <v>61950.01</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -4758,6 +4830,7 @@
       <c r="BA30" s="15" t="n"/>
       <c r="BB30" s="15" t="n"/>
       <c r="BC30" s="15" t="n"/>
+      <c r="BD30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -4924,6 +4997,9 @@
       </c>
       <c r="BC31" s="15" t="n">
         <v>46.21</v>
+      </c>
+      <c r="BD31" s="15" t="n">
+        <v>45.62</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -5043,6 +5119,9 @@
       </c>
       <c r="BC32" s="15" t="n">
         <v>5433.84</v>
+      </c>
+      <c r="BD32" s="15" t="n">
+        <v>5556.65</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -5149,6 +5228,7 @@
       <c r="BA33" s="15" t="n"/>
       <c r="BB33" s="15" t="n"/>
       <c r="BC33" s="15" t="n"/>
+      <c r="BD33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -5315,6 +5395,9 @@
       </c>
       <c r="BC34" s="15" t="n">
         <v>59.14</v>
+      </c>
+      <c r="BD34" s="15" t="n">
+        <v>55.78</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -5434,6 +5517,9 @@
       </c>
       <c r="BC35" s="15" t="n">
         <v>11383.25</v>
+      </c>
+      <c r="BD35" s="15" t="n">
+        <v>11736.42</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -5540,6 +5626,7 @@
       <c r="BA36" s="15" t="n"/>
       <c r="BB36" s="15" t="n"/>
       <c r="BC36" s="15" t="n"/>
+      <c r="BD36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -5706,6 +5793,9 @@
       </c>
       <c r="BC37" s="15" t="n">
         <v>50.24</v>
+      </c>
+      <c r="BD37" s="15" t="n">
+        <v>50.85</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -5825,6 +5915,9 @@
       </c>
       <c r="BC38" s="15" t="n">
         <v>10775.41</v>
+      </c>
+      <c r="BD38" s="15" t="n">
+        <v>11000.28</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -5931,6 +6024,7 @@
       <c r="BA39" s="15" t="n"/>
       <c r="BB39" s="15" t="n"/>
       <c r="BC39" s="15" t="n"/>
+      <c r="BD39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -6097,6 +6191,9 @@
       </c>
       <c r="BC40" s="15" t="n">
         <v>51.01</v>
+      </c>
+      <c r="BD40" s="15" t="n">
+        <v>50.14</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -6216,6 +6313,9 @@
       </c>
       <c r="BC41" s="15" t="n">
         <v>3140.45</v>
+      </c>
+      <c r="BD41" s="15" t="n">
+        <v>3191</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -6322,6 +6422,7 @@
       <c r="BA42" s="15" t="n"/>
       <c r="BB42" s="15" t="n"/>
       <c r="BC42" s="15" t="n"/>
+      <c r="BD42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -6488,6 +6589,9 @@
       </c>
       <c r="BC43" s="15" t="n">
         <v>57.84</v>
+      </c>
+      <c r="BD43" s="15" t="n">
+        <v>55.25</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -6607,6 +6711,9 @@
       </c>
       <c r="BC44" s="15" t="n">
         <v>7000.09</v>
+      </c>
+      <c r="BD44" s="15" t="n">
+        <v>7125.2</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -6713,6 +6820,7 @@
       <c r="BA45" s="15" t="n"/>
       <c r="BB45" s="15" t="n"/>
       <c r="BC45" s="15" t="n"/>
+      <c r="BD45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -6879,6 +6987,9 @@
       </c>
       <c r="BC46" s="15" t="n">
         <v>26.48</v>
+      </c>
+      <c r="BD46" s="15" t="n">
+        <v>25.66</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -6998,6 +7109,9 @@
       </c>
       <c r="BC47" s="15" t="n">
         <v>32210.4</v>
+      </c>
+      <c r="BD47" s="15" t="n">
+        <v>33039.38</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -7104,6 +7218,7 @@
       <c r="BA48" s="15" t="n"/>
       <c r="BB48" s="15" t="n"/>
       <c r="BC48" s="15" t="n"/>
+      <c r="BD48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -7270,6 +7385,9 @@
       </c>
       <c r="BC49" s="15" t="n">
         <v>47.45</v>
+      </c>
+      <c r="BD49" s="15" t="n">
+        <v>44.78</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -7389,6 +7507,9 @@
       </c>
       <c r="BC50" s="15" t="n">
         <v>3815.48</v>
+      </c>
+      <c r="BD50" s="15" t="n">
+        <v>3468.12</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -7495,6 +7616,7 @@
       <c r="BA51" s="15" t="n"/>
       <c r="BB51" s="15" t="n"/>
       <c r="BC51" s="15" t="n"/>
+      <c r="BD51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -7661,6 +7783,9 @@
       </c>
       <c r="BC52" s="15" t="n">
         <v>55.86</v>
+      </c>
+      <c r="BD52" s="15" t="n">
+        <v>52.77</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -7780,6 +7905,9 @@
       </c>
       <c r="BC53" s="15" t="n">
         <v>3584.35</v>
+      </c>
+      <c r="BD53" s="15" t="n">
+        <v>3289.13</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -7886,6 +8014,7 @@
       <c r="BA54" s="15" t="n"/>
       <c r="BB54" s="15" t="n"/>
       <c r="BC54" s="15" t="n"/>
+      <c r="BD54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -8052,6 +8181,9 @@
       </c>
       <c r="BC55" s="15" t="n">
         <v>7.68</v>
+      </c>
+      <c r="BD55" s="15" t="n">
+        <v>10.7</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -8171,6 +8303,9 @@
       </c>
       <c r="BC56" s="15" t="n">
         <v>6360.11</v>
+      </c>
+      <c r="BD56" s="15" t="n">
+        <v>6402.17</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -8277,6 +8412,7 @@
       <c r="BA57" s="15" t="n"/>
       <c r="BB57" s="15" t="n"/>
       <c r="BC57" s="15" t="n"/>
+      <c r="BD57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -8443,6 +8579,9 @@
       </c>
       <c r="BC58" s="15" t="n">
         <v>31.45</v>
+      </c>
+      <c r="BD58" s="15" t="n">
+        <v>35.31</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -8562,6 +8701,9 @@
       </c>
       <c r="BC59" s="15" t="n">
         <v>7928.36</v>
+      </c>
+      <c r="BD59" s="15" t="n">
+        <v>8052.16</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -8668,6 +8810,7 @@
       <c r="BA60" s="15" t="n"/>
       <c r="BB60" s="15" t="n"/>
       <c r="BC60" s="15" t="n"/>
+      <c r="BD60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -8834,6 +8977,9 @@
       </c>
       <c r="BC61" s="15" t="n">
         <v>2.6</v>
+      </c>
+      <c r="BD61" s="15" t="n">
+        <v>5.04</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -8953,6 +9099,9 @@
       </c>
       <c r="BC62" s="15" t="n">
         <v>10720.79</v>
+      </c>
+      <c r="BD62" s="15" t="n">
+        <v>11319.41</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -9059,6 +9208,7 @@
       <c r="BA63" s="15" t="n"/>
       <c r="BB63" s="15" t="n"/>
       <c r="BC63" s="15" t="n"/>
+      <c r="BD63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -9225,6 +9375,9 @@
       </c>
       <c r="BC64" s="15" t="n">
         <v>13.34</v>
+      </c>
+      <c r="BD64" s="15" t="n">
+        <v>20.39</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -9344,6 +9497,9 @@
       </c>
       <c r="BC65" s="15" t="n">
         <v>11178.06</v>
+      </c>
+      <c r="BD65" s="15" t="n">
+        <v>11333.16</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -9450,6 +9606,7 @@
       <c r="BA66" s="15" t="n"/>
       <c r="BB66" s="15" t="n"/>
       <c r="BC66" s="15" t="n"/>
+      <c r="BD66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -9616,6 +9773,9 @@
       </c>
       <c r="BC67" s="15" t="n">
         <v>13.54</v>
+      </c>
+      <c r="BD67" s="15" t="n">
+        <v>16.37</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -9735,6 +9895,9 @@
       </c>
       <c r="BC68" s="15" t="n">
         <v>6469.83</v>
+      </c>
+      <c r="BD68" s="15" t="n">
+        <v>6944.81</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -9841,6 +10004,7 @@
       <c r="BA69" s="15" t="n"/>
       <c r="BB69" s="15" t="n"/>
       <c r="BC69" s="15" t="n"/>
+      <c r="BD69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -10007,6 +10171,9 @@
       </c>
       <c r="BC70" s="15" t="n">
         <v>12.96</v>
+      </c>
+      <c r="BD70" s="15" t="n">
+        <v>16.3</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -10126,6 +10293,9 @@
       </c>
       <c r="BC71" s="15" t="n">
         <v>12470.65</v>
+      </c>
+      <c r="BD71" s="15" t="n">
+        <v>13096.88</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -10232,6 +10402,7 @@
       <c r="BA72" s="15" t="n"/>
       <c r="BB72" s="15" t="n"/>
       <c r="BC72" s="15" t="n"/>
+      <c r="BD72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -10398,6 +10569,9 @@
       </c>
       <c r="BC73" s="15" t="n">
         <v>52.27</v>
+      </c>
+      <c r="BD73" s="15" t="n">
+        <v>52.71</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -10517,6 +10691,9 @@
       </c>
       <c r="BC74" s="15" t="n">
         <v>14099.43</v>
+      </c>
+      <c r="BD74" s="15" t="n">
+        <v>15569.82</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -10623,6 +10800,7 @@
       <c r="BA75" s="15" t="n"/>
       <c r="BB75" s="15" t="n"/>
       <c r="BC75" s="15" t="n"/>
+      <c r="BD75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -10789,6 +10967,9 @@
       </c>
       <c r="BC76" s="15" t="n">
         <v>2.86</v>
+      </c>
+      <c r="BD76" s="15" t="n">
+        <v>4.57</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -10908,6 +11089,9 @@
       </c>
       <c r="BC77" s="15" t="n">
         <v>6818.12</v>
+      </c>
+      <c r="BD77" s="15" t="n">
+        <v>7263.47</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
@@ -11014,6 +11198,7 @@
       <c r="BA78" s="15" t="n"/>
       <c r="BB78" s="15" t="n"/>
       <c r="BC78" s="15" t="n"/>
+      <c r="BD78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -11180,6 +11365,9 @@
       </c>
       <c r="BC79" s="15" t="n">
         <v>3.09</v>
+      </c>
+      <c r="BD79" s="15" t="n">
+        <v>4.19</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -11299,6 +11487,9 @@
       </c>
       <c r="BC80" s="15" t="n">
         <v>8831.42</v>
+      </c>
+      <c r="BD80" s="15" t="n">
+        <v>8905.889999999999</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -11405,6 +11596,7 @@
       <c r="BA81" s="15" t="n"/>
       <c r="BB81" s="15" t="n"/>
       <c r="BC81" s="15" t="n"/>
+      <c r="BD81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -11571,6 +11763,9 @@
       </c>
       <c r="BC82" s="15" t="n">
         <v>11.34</v>
+      </c>
+      <c r="BD82" s="15" t="n">
+        <v>14.04</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -11690,6 +11885,9 @@
       </c>
       <c r="BC83" s="15" t="n">
         <v>2280.38</v>
+      </c>
+      <c r="BD83" s="15" t="n">
+        <v>2376.64</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -11796,6 +11994,7 @@
       <c r="BA84" s="15" t="n"/>
       <c r="BB84" s="15" t="n"/>
       <c r="BC84" s="15" t="n"/>
+      <c r="BD84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -11962,6 +12161,9 @@
       </c>
       <c r="BC85" s="15" t="n">
         <v>23.08</v>
+      </c>
+      <c r="BD85" s="15" t="n">
+        <v>27.92</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -12081,6 +12283,9 @@
       </c>
       <c r="BC86" s="15" t="n">
         <v>4713.64</v>
+      </c>
+      <c r="BD86" s="15" t="n">
+        <v>4804.46</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -12187,6 +12392,7 @@
       <c r="BA87" s="15" t="n"/>
       <c r="BB87" s="15" t="n"/>
       <c r="BC87" s="15" t="n"/>
+      <c r="BD87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -12353,6 +12559,9 @@
       </c>
       <c r="BC88" s="15" t="n">
         <v>19.73</v>
+      </c>
+      <c r="BD88" s="15" t="n">
+        <v>21.98</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -12472,6 +12681,9 @@
       </c>
       <c r="BC89" s="15" t="n">
         <v>8476.440000000001</v>
+      </c>
+      <c r="BD89" s="15" t="n">
+        <v>8455.41</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -12578,6 +12790,7 @@
       <c r="BA90" s="15" t="n"/>
       <c r="BB90" s="15" t="n"/>
       <c r="BC90" s="15" t="n"/>
+      <c r="BD90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -12744,6 +12957,9 @@
       </c>
       <c r="BC91" s="15" t="n">
         <v>6.58</v>
+      </c>
+      <c r="BD91" s="15" t="n">
+        <v>6.68</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -12863,6 +13079,9 @@
       </c>
       <c r="BC92" s="15" t="n">
         <v>1204.84</v>
+      </c>
+      <c r="BD92" s="15" t="n">
+        <v>1206.57</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -12969,6 +13188,7 @@
       <c r="BA93" s="15" t="n"/>
       <c r="BB93" s="15" t="n"/>
       <c r="BC93" s="15" t="n"/>
+      <c r="BD93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -13135,6 +13355,9 @@
       </c>
       <c r="BC94" s="15" t="n">
         <v>5.51</v>
+      </c>
+      <c r="BD94" s="15" t="n">
+        <v>7.5</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -13254,6 +13477,9 @@
       </c>
       <c r="BC95" s="15" t="n">
         <v>13757.19</v>
+      </c>
+      <c r="BD95" s="15" t="n">
+        <v>14253.77</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -13360,6 +13586,7 @@
       <c r="BA96" s="15" t="n"/>
       <c r="BB96" s="15" t="n"/>
       <c r="BC96" s="15" t="n"/>
+      <c r="BD96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -13526,6 +13753,9 @@
       </c>
       <c r="BC97" s="15" t="n">
         <v>43.06</v>
+      </c>
+      <c r="BD97" s="15" t="n">
+        <v>45.04</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -13645,6 +13875,9 @@
       </c>
       <c r="BC98" s="15" t="n">
         <v>3093.89</v>
+      </c>
+      <c r="BD98" s="15" t="n">
+        <v>3163.62</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -13751,6 +13984,7 @@
       <c r="BA99" s="15" t="n"/>
       <c r="BB99" s="15" t="n"/>
       <c r="BC99" s="15" t="n"/>
+      <c r="BD99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -13917,6 +14151,9 @@
       </c>
       <c r="BC100" s="15" t="n">
         <v>34.75</v>
+      </c>
+      <c r="BD100" s="15" t="n">
+        <v>36.41</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -14036,6 +14273,9 @@
       </c>
       <c r="BC101" s="15" t="n">
         <v>2414.39</v>
+      </c>
+      <c r="BD101" s="15" t="n">
+        <v>2361.96</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -14142,6 +14382,7 @@
       <c r="BA102" s="15" t="n"/>
       <c r="BB102" s="15" t="n"/>
       <c r="BC102" s="15" t="n"/>
+      <c r="BD102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -14308,6 +14549,9 @@
       </c>
       <c r="BC103" s="15" t="n">
         <v>14.06</v>
+      </c>
+      <c r="BD103" s="15" t="n">
+        <v>13.82</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -14427,6 +14671,9 @@
       </c>
       <c r="BC104" s="15" t="n">
         <v>2483.24</v>
+      </c>
+      <c r="BD104" s="15" t="n">
+        <v>2372.03</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -14533,6 +14780,7 @@
       <c r="BA105" s="15" t="n"/>
       <c r="BB105" s="15" t="n"/>
       <c r="BC105" s="15" t="n"/>
+      <c r="BD105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -14699,6 +14947,9 @@
       </c>
       <c r="BC106" s="15" t="n">
         <v>35.95</v>
+      </c>
+      <c r="BD106" s="15" t="n">
+        <v>37.73</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -14818,6 +15069,9 @@
       </c>
       <c r="BC107" s="15" t="n">
         <v>2561.13</v>
+      </c>
+      <c r="BD107" s="15" t="n">
+        <v>2566.6</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -14924,6 +15178,7 @@
       <c r="BA108" s="15" t="n"/>
       <c r="BB108" s="15" t="n"/>
       <c r="BC108" s="15" t="n"/>
+      <c r="BD108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -15090,6 +15345,9 @@
       </c>
       <c r="BC109" s="15" t="n">
         <v>57.98</v>
+      </c>
+      <c r="BD109" s="15" t="n">
+        <v>58.79</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -15209,6 +15467,9 @@
       </c>
       <c r="BC110" s="15" t="n">
         <v>1894.98</v>
+      </c>
+      <c r="BD110" s="15" t="n">
+        <v>1875.8</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -15315,6 +15576,7 @@
       <c r="BA111" s="15" t="n"/>
       <c r="BB111" s="15" t="n"/>
       <c r="BC111" s="15" t="n"/>
+      <c r="BD111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -15481,6 +15743,9 @@
       </c>
       <c r="BC112" s="15" t="n">
         <v>19.6</v>
+      </c>
+      <c r="BD112" s="15" t="n">
+        <v>21.7</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -15600,6 +15865,9 @@
       </c>
       <c r="BC113" s="15" t="n">
         <v>8516.059999999999</v>
+      </c>
+      <c r="BD113" s="15" t="n">
+        <v>8486.91</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -15706,6 +15974,7 @@
       <c r="BA114" s="15" t="n"/>
       <c r="BB114" s="15" t="n"/>
       <c r="BC114" s="15" t="n"/>
+      <c r="BD114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -15872,6 +16141,9 @@
       </c>
       <c r="BC115" s="15" t="n">
         <v>97.22</v>
+      </c>
+      <c r="BD115" s="15" t="n">
+        <v>94.84</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -15976,6 +16248,9 @@
       </c>
       <c r="BC116" s="15" t="n">
         <v>14152.29</v>
+      </c>
+      <c r="BD116" s="15" t="n">
+        <v>12339.33</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -16037,6 +16312,7 @@
       <c r="BA117" s="15" t="n"/>
       <c r="BB117" s="15" t="n"/>
       <c r="BC117" s="15" t="n"/>
+      <c r="BD117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -16159,6 +16435,9 @@
       <c r="BC118" s="15" t="n">
         <v>40.41</v>
       </c>
+      <c r="BD118" s="15" t="n">
+        <v>42.87</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -16253,6 +16532,9 @@
       </c>
       <c r="BC119" s="15" t="n">
         <v>11182.8</v>
+      </c>
+      <c r="BD119" s="15" t="n">
+        <v>10872.42</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -16263,6 +16545,7 @@
       <c r="BA120" s="15" t="n"/>
       <c r="BB120" s="15" t="n"/>
       <c r="BC120" s="15" t="n"/>
+      <c r="BD120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -16286,6 +16569,9 @@
       <c r="BC121" s="15" t="n">
         <v>27.4</v>
       </c>
+      <c r="BD121" s="15" t="n">
+        <v>27.74</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -16308,6 +16594,9 @@
       </c>
       <c r="BC122" s="15" t="n">
         <v>1810.95</v>
+      </c>
+      <c r="BD122" s="15" t="n">
+        <v>1823.14</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -16318,6 +16607,7 @@
       <c r="BA123" s="15" t="n"/>
       <c r="BB123" s="15" t="n"/>
       <c r="BC123" s="15" t="n"/>
+      <c r="BD123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -16341,6 +16631,9 @@
       <c r="BC124" s="15" t="n">
         <v>13.93</v>
       </c>
+      <c r="BD124" s="15" t="n">
+        <v>15.15</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -16363,6 +16656,9 @@
       </c>
       <c r="BC125" s="15" t="n">
         <v>770.9</v>
+      </c>
+      <c r="BD125" s="15" t="n">
+        <v>772.16</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -16373,6 +16669,7 @@
       <c r="BA126" s="15" t="n"/>
       <c r="BB126" s="15" t="n"/>
       <c r="BC126" s="15" t="n"/>
+      <c r="BD126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -16396,6 +16693,9 @@
       <c r="BC127" s="15" t="n">
         <v>59.52</v>
       </c>
+      <c r="BD127" s="15" t="n">
+        <v>62.09</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -16417,6 +16717,9 @@
         <v>2871.1</v>
       </c>
       <c r="BC128" s="15" t="n">
+        <v>2745.29</v>
+      </c>
+      <c r="BD128" s="15" t="n">
         <v>2745.29</v>
       </c>
     </row>
@@ -16428,6 +16731,7 @@
       <c r="BA129" s="15" t="n"/>
       <c r="BB129" s="15" t="n"/>
       <c r="BC129" s="15" t="n"/>
+      <c r="BD129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -16451,6 +16755,9 @@
       <c r="BC130" s="15" t="n">
         <v>19.84</v>
       </c>
+      <c r="BD130" s="15" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -16473,6 +16780,9 @@
       </c>
       <c r="BC131" s="15" t="n">
         <v>3542.49</v>
+      </c>
+      <c r="BD131" s="15" t="n">
+        <v>3517.4</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -16483,6 +16793,7 @@
       <c r="BA132" s="15" t="n"/>
       <c r="BB132" s="15" t="n"/>
       <c r="BC132" s="15" t="n"/>
+      <c r="BD132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -16506,6 +16817,9 @@
       <c r="BC133" s="15" t="n">
         <v>1.36</v>
       </c>
+      <c r="BD133" s="15" t="n">
+        <v>2.09</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -16528,6 +16842,9 @@
       </c>
       <c r="BC134" s="15" t="n">
         <v>2273.63</v>
+      </c>
+      <c r="BD134" s="15" t="n">
+        <v>2326.06</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -16538,6 +16855,7 @@
       <c r="BA135" s="15" t="n"/>
       <c r="BB135" s="15" t="n"/>
       <c r="BC135" s="15" t="n"/>
+      <c r="BD135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -16561,6 +16879,9 @@
       <c r="BC136" s="15" t="n">
         <v>7.41</v>
       </c>
+      <c r="BD136" s="15" t="n">
+        <v>8.92</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -16583,6 +16904,9 @@
       </c>
       <c r="BC137" s="15" t="n">
         <v>5272.37</v>
+      </c>
+      <c r="BD137" s="15" t="n">
+        <v>5391.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-07-31 06:11:48]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BD137"/>
+  <dimension ref="A1:BE143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -590,6 +590,7 @@
     <col width="15" customWidth="1" min="54" max="54"/>
     <col width="15" customWidth="1" min="55" max="55"/>
     <col width="15" customWidth="1" min="56" max="56"/>
+    <col width="15" customWidth="1" min="57" max="57"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -873,6 +874,11 @@
           <t>2026/07/30</t>
         </is>
       </c>
+      <c r="BE1" s="15" t="inlineStr">
+        <is>
+          <t>2026/07/31</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1155,6 +1161,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BE2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1325,6 +1336,9 @@
       <c r="BD3" s="15" t="n">
         <v>59.47</v>
       </c>
+      <c r="BE3" s="15" t="n">
+        <v>57.36</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1494,6 +1508,9 @@
       </c>
       <c r="BD4" s="15" t="n">
         <v>3811.7</v>
+      </c>
+      <c r="BE4" s="15" t="n">
+        <v>3837.11</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1553,6 +1570,7 @@
       <c r="BB5" s="15" t="n"/>
       <c r="BC5" s="15" t="n"/>
       <c r="BD5" s="15" t="n"/>
+      <c r="BE5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1659,6 +1677,7 @@
       <c r="BB6" s="15" t="n"/>
       <c r="BC6" s="15" t="n"/>
       <c r="BD6" s="15" t="n"/>
+      <c r="BE6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1828,6 +1847,9 @@
       </c>
       <c r="BD7" s="15" t="n">
         <v>61.92</v>
+      </c>
+      <c r="BE7" s="15" t="n">
+        <v>61.19</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -1950,6 +1972,9 @@
       </c>
       <c r="BD8" s="15" t="n">
         <v>5591.62</v>
+      </c>
+      <c r="BE8" s="15" t="n">
+        <v>5656.33</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2057,6 +2082,7 @@
       <c r="BB9" s="15" t="n"/>
       <c r="BC9" s="15" t="n"/>
       <c r="BD9" s="15" t="n"/>
+      <c r="BE9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2226,6 +2252,9 @@
       </c>
       <c r="BD10" s="15" t="n">
         <v>55.48</v>
+      </c>
+      <c r="BE10" s="15" t="n">
+        <v>55.67</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2348,6 +2377,9 @@
       </c>
       <c r="BD11" s="15" t="n">
         <v>4571.35</v>
+      </c>
+      <c r="BE11" s="15" t="n">
+        <v>4604.58</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -2455,6 +2487,7 @@
       <c r="BB12" s="15" t="n"/>
       <c r="BC12" s="15" t="n"/>
       <c r="BD12" s="15" t="n"/>
+      <c r="BE12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2624,6 +2657,9 @@
       </c>
       <c r="BD13" s="15" t="n">
         <v>63.03</v>
+      </c>
+      <c r="BE13" s="15" t="n">
+        <v>60.19</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -2746,6 +2782,9 @@
       </c>
       <c r="BD14" s="15" t="n">
         <v>7364.04</v>
+      </c>
+      <c r="BE14" s="15" t="n">
+        <v>7545.62</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -2853,6 +2892,7 @@
       <c r="BB15" s="15" t="n"/>
       <c r="BC15" s="15" t="n"/>
       <c r="BD15" s="15" t="n"/>
+      <c r="BE15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -3022,6 +3062,9 @@
       </c>
       <c r="BD16" s="15" t="n">
         <v>35.67</v>
+      </c>
+      <c r="BE16" s="15" t="n">
+        <v>36.64</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -3143,6 +3186,9 @@
         <v>2601.82</v>
       </c>
       <c r="BD17" s="15" t="n">
+        <v>2536.29</v>
+      </c>
+      <c r="BE17" s="15" t="n">
         <v>2536.29</v>
       </c>
     </row>
@@ -3251,6 +3297,7 @@
       <c r="BB18" s="15" t="n"/>
       <c r="BC18" s="15" t="n"/>
       <c r="BD18" s="15" t="n"/>
+      <c r="BE18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -3420,6 +3467,9 @@
       </c>
       <c r="BD19" s="15" t="n">
         <v>81.75</v>
+      </c>
+      <c r="BE19" s="15" t="n">
+        <v>80.76000000000001</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -3542,6 +3592,9 @@
       </c>
       <c r="BD20" s="15" t="n">
         <v>7316.15</v>
+      </c>
+      <c r="BE20" s="15" t="n">
+        <v>7437.63</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -3649,6 +3702,7 @@
       <c r="BB21" s="15" t="n"/>
       <c r="BC21" s="15" t="n"/>
       <c r="BD21" s="15" t="n"/>
+      <c r="BE21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -3815,6 +3869,9 @@
         <v>36.34</v>
       </c>
       <c r="BD22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BE22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -3938,6 +3995,9 @@
       </c>
       <c r="BD23" s="15" t="n">
         <v>77689.99000000001</v>
+      </c>
+      <c r="BE23" s="15" t="n">
+        <v>78041.48</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -4045,6 +4105,7 @@
       <c r="BB24" s="15" t="n"/>
       <c r="BC24" s="15" t="n"/>
       <c r="BD24" s="15" t="n"/>
+      <c r="BE24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -4213,6 +4274,9 @@
         <v>49.88</v>
       </c>
       <c r="BD25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BE25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -4327,6 +4391,7 @@
         <v>25099</v>
       </c>
       <c r="BD26" s="15" t="inlineStr"/>
+      <c r="BE26" s="15" t="inlineStr"/>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -4433,6 +4498,7 @@
       <c r="BB27" s="15" t="n"/>
       <c r="BC27" s="15" t="n"/>
       <c r="BD27" s="15" t="n"/>
+      <c r="BE27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -4601,6 +4667,9 @@
         <v>92.09</v>
       </c>
       <c r="BD28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BE28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -4724,6 +4793,9 @@
       </c>
       <c r="BD29" s="15" t="n">
         <v>61950.01</v>
+      </c>
+      <c r="BE29" s="15" t="n">
+        <v>64409.39</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -4831,6 +4903,7 @@
       <c r="BB30" s="15" t="n"/>
       <c r="BC30" s="15" t="n"/>
       <c r="BD30" s="15" t="n"/>
+      <c r="BE30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -5000,6 +5073,9 @@
       </c>
       <c r="BD31" s="15" t="n">
         <v>45.62</v>
+      </c>
+      <c r="BE31" s="15" t="n">
+        <v>46.99</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -5122,6 +5198,9 @@
       </c>
       <c r="BD32" s="15" t="n">
         <v>5556.65</v>
+      </c>
+      <c r="BE32" s="15" t="n">
+        <v>5548.06</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -5229,6 +5308,7 @@
       <c r="BB33" s="15" t="n"/>
       <c r="BC33" s="15" t="n"/>
       <c r="BD33" s="15" t="n"/>
+      <c r="BE33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -5398,6 +5478,9 @@
       </c>
       <c r="BD34" s="15" t="n">
         <v>55.78</v>
+      </c>
+      <c r="BE34" s="15" t="n">
+        <v>55.98</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -5520,6 +5603,9 @@
       </c>
       <c r="BD35" s="15" t="n">
         <v>11736.42</v>
+      </c>
+      <c r="BE35" s="15" t="n">
+        <v>11692.35</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -5627,6 +5713,7 @@
       <c r="BB36" s="15" t="n"/>
       <c r="BC36" s="15" t="n"/>
       <c r="BD36" s="15" t="n"/>
+      <c r="BE36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -5796,6 +5883,9 @@
       </c>
       <c r="BD37" s="15" t="n">
         <v>50.85</v>
+      </c>
+      <c r="BE37" s="15" t="n">
+        <v>50.44</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -5918,6 +6008,9 @@
       </c>
       <c r="BD38" s="15" t="n">
         <v>11000.28</v>
+      </c>
+      <c r="BE38" s="15" t="n">
+        <v>11171.66</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -6025,6 +6118,7 @@
       <c r="BB39" s="15" t="n"/>
       <c r="BC39" s="15" t="n"/>
       <c r="BD39" s="15" t="n"/>
+      <c r="BE39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -6194,6 +6288,9 @@
       </c>
       <c r="BD40" s="15" t="n">
         <v>50.14</v>
+      </c>
+      <c r="BE40" s="15" t="n">
+        <v>50.19</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -6316,6 +6413,9 @@
       </c>
       <c r="BD41" s="15" t="n">
         <v>3191</v>
+      </c>
+      <c r="BE41" s="15" t="n">
+        <v>3227.27</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -6423,6 +6523,7 @@
       <c r="BB42" s="15" t="n"/>
       <c r="BC42" s="15" t="n"/>
       <c r="BD42" s="15" t="n"/>
+      <c r="BE42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -6592,6 +6693,9 @@
       </c>
       <c r="BD43" s="15" t="n">
         <v>55.25</v>
+      </c>
+      <c r="BE43" s="15" t="n">
+        <v>58.6</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -6714,6 +6818,9 @@
       </c>
       <c r="BD44" s="15" t="n">
         <v>7125.2</v>
+      </c>
+      <c r="BE44" s="15" t="n">
+        <v>7244.78</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -6821,6 +6928,7 @@
       <c r="BB45" s="15" t="n"/>
       <c r="BC45" s="15" t="n"/>
       <c r="BD45" s="15" t="n"/>
+      <c r="BE45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -6990,6 +7098,9 @@
       </c>
       <c r="BD46" s="15" t="n">
         <v>25.66</v>
+      </c>
+      <c r="BE46" s="15" t="n">
+        <v>27.08</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -7112,6 +7223,9 @@
       </c>
       <c r="BD47" s="15" t="n">
         <v>33039.38</v>
+      </c>
+      <c r="BE47" s="15" t="n">
+        <v>33613.32</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -7219,6 +7333,7 @@
       <c r="BB48" s="15" t="n"/>
       <c r="BC48" s="15" t="n"/>
       <c r="BD48" s="15" t="n"/>
+      <c r="BE48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -7388,6 +7503,9 @@
       </c>
       <c r="BD49" s="15" t="n">
         <v>44.78</v>
+      </c>
+      <c r="BE49" s="15" t="n">
+        <v>41.67</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -7510,6 +7628,9 @@
       </c>
       <c r="BD50" s="15" t="n">
         <v>3468.12</v>
+      </c>
+      <c r="BE50" s="15" t="n">
+        <v>3566.54</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -7617,6 +7738,7 @@
       <c r="BB51" s="15" t="n"/>
       <c r="BC51" s="15" t="n"/>
       <c r="BD51" s="15" t="n"/>
+      <c r="BE51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -7786,6 +7908,9 @@
       </c>
       <c r="BD52" s="15" t="n">
         <v>52.77</v>
+      </c>
+      <c r="BE52" s="15" t="n">
+        <v>49.08</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -7908,6 +8033,9 @@
       </c>
       <c r="BD53" s="15" t="n">
         <v>3289.13</v>
+      </c>
+      <c r="BE53" s="15" t="n">
+        <v>3387.38</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -8015,6 +8143,7 @@
       <c r="BB54" s="15" t="n"/>
       <c r="BC54" s="15" t="n"/>
       <c r="BD54" s="15" t="n"/>
+      <c r="BE54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -8184,6 +8313,9 @@
       </c>
       <c r="BD55" s="15" t="n">
         <v>10.7</v>
+      </c>
+      <c r="BE55" s="15" t="n">
+        <v>10.42</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -8306,6 +8438,9 @@
       </c>
       <c r="BD56" s="15" t="n">
         <v>6402.17</v>
+      </c>
+      <c r="BE56" s="15" t="n">
+        <v>6520.71</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -8413,6 +8548,7 @@
       <c r="BB57" s="15" t="n"/>
       <c r="BC57" s="15" t="n"/>
       <c r="BD57" s="15" t="n"/>
+      <c r="BE57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -8582,6 +8718,9 @@
       </c>
       <c r="BD58" s="15" t="n">
         <v>35.31</v>
+      </c>
+      <c r="BE58" s="15" t="n">
+        <v>37.16</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -8704,6 +8843,9 @@
       </c>
       <c r="BD59" s="15" t="n">
         <v>8052.16</v>
+      </c>
+      <c r="BE59" s="15" t="n">
+        <v>8084.53</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -8811,6 +8953,7 @@
       <c r="BB60" s="15" t="n"/>
       <c r="BC60" s="15" t="n"/>
       <c r="BD60" s="15" t="n"/>
+      <c r="BE60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -8980,6 +9123,9 @@
       </c>
       <c r="BD61" s="15" t="n">
         <v>5.04</v>
+      </c>
+      <c r="BE61" s="15" t="n">
+        <v>7.29</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -9102,6 +9248,9 @@
       </c>
       <c r="BD62" s="15" t="n">
         <v>11319.41</v>
+      </c>
+      <c r="BE62" s="15" t="n">
+        <v>11337.21</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -9209,6 +9358,7 @@
       <c r="BB63" s="15" t="n"/>
       <c r="BC63" s="15" t="n"/>
       <c r="BD63" s="15" t="n"/>
+      <c r="BE63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -9378,6 +9528,9 @@
       </c>
       <c r="BD64" s="15" t="n">
         <v>20.39</v>
+      </c>
+      <c r="BE64" s="15" t="n">
+        <v>22.07</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -9500,6 +9653,9 @@
       </c>
       <c r="BD65" s="15" t="n">
         <v>11333.16</v>
+      </c>
+      <c r="BE65" s="15" t="n">
+        <v>11429.35</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -9607,6 +9763,7 @@
       <c r="BB66" s="15" t="n"/>
       <c r="BC66" s="15" t="n"/>
       <c r="BD66" s="15" t="n"/>
+      <c r="BE66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -9776,6 +9933,9 @@
       </c>
       <c r="BD67" s="15" t="n">
         <v>16.37</v>
+      </c>
+      <c r="BE67" s="15" t="n">
+        <v>20.16</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -9898,6 +10058,9 @@
       </c>
       <c r="BD68" s="15" t="n">
         <v>6944.81</v>
+      </c>
+      <c r="BE68" s="15" t="n">
+        <v>6918.68</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -10005,6 +10168,7 @@
       <c r="BB69" s="15" t="n"/>
       <c r="BC69" s="15" t="n"/>
       <c r="BD69" s="15" t="n"/>
+      <c r="BE69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -10174,6 +10338,9 @@
       </c>
       <c r="BD70" s="15" t="n">
         <v>16.3</v>
+      </c>
+      <c r="BE70" s="15" t="n">
+        <v>18.57</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -10296,6 +10463,9 @@
       </c>
       <c r="BD71" s="15" t="n">
         <v>13096.88</v>
+      </c>
+      <c r="BE71" s="15" t="n">
+        <v>13006.35</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -10403,6 +10573,7 @@
       <c r="BB72" s="15" t="n"/>
       <c r="BC72" s="15" t="n"/>
       <c r="BD72" s="15" t="n"/>
+      <c r="BE72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -10572,6 +10743,9 @@
       </c>
       <c r="BD73" s="15" t="n">
         <v>52.71</v>
+      </c>
+      <c r="BE73" s="15" t="n">
+        <v>52.02</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -10694,6 +10868,9 @@
       </c>
       <c r="BD74" s="15" t="n">
         <v>15569.82</v>
+      </c>
+      <c r="BE74" s="15" t="n">
+        <v>13850.53</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -10801,6 +10978,7 @@
       <c r="BB75" s="15" t="n"/>
       <c r="BC75" s="15" t="n"/>
       <c r="BD75" s="15" t="n"/>
+      <c r="BE75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -10970,6 +11148,9 @@
       </c>
       <c r="BD76" s="15" t="n">
         <v>4.57</v>
+      </c>
+      <c r="BE76" s="15" t="n">
+        <v>4.82</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -11092,6 +11273,9 @@
       </c>
       <c r="BD77" s="15" t="n">
         <v>7263.47</v>
+      </c>
+      <c r="BE77" s="15" t="n">
+        <v>7294.46</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
@@ -11199,6 +11383,7 @@
       <c r="BB78" s="15" t="n"/>
       <c r="BC78" s="15" t="n"/>
       <c r="BD78" s="15" t="n"/>
+      <c r="BE78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -11368,6 +11553,9 @@
       </c>
       <c r="BD79" s="15" t="n">
         <v>4.19</v>
+      </c>
+      <c r="BE79" s="15" t="n">
+        <v>4.58</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -11490,6 +11678,9 @@
       </c>
       <c r="BD80" s="15" t="n">
         <v>8905.889999999999</v>
+      </c>
+      <c r="BE80" s="15" t="n">
+        <v>8937.27</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -11597,6 +11788,7 @@
       <c r="BB81" s="15" t="n"/>
       <c r="BC81" s="15" t="n"/>
       <c r="BD81" s="15" t="n"/>
+      <c r="BE81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -11765,6 +11957,9 @@
         <v>11.34</v>
       </c>
       <c r="BD82" s="15" t="n">
+        <v>14.04</v>
+      </c>
+      <c r="BE82" s="15" t="n">
         <v>14.04</v>
       </c>
     </row>
@@ -11888,6 +12083,9 @@
       </c>
       <c r="BD83" s="15" t="n">
         <v>2376.64</v>
+      </c>
+      <c r="BE83" s="15" t="n">
+        <v>2631.9</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -11995,6 +12193,7 @@
       <c r="BB84" s="15" t="n"/>
       <c r="BC84" s="15" t="n"/>
       <c r="BD84" s="15" t="n"/>
+      <c r="BE84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -12164,6 +12363,9 @@
       </c>
       <c r="BD85" s="15" t="n">
         <v>27.92</v>
+      </c>
+      <c r="BE85" s="15" t="n">
+        <v>26.7</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -12286,6 +12488,9 @@
       </c>
       <c r="BD86" s="15" t="n">
         <v>4804.46</v>
+      </c>
+      <c r="BE86" s="15" t="n">
+        <v>5075.31</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -12393,6 +12598,7 @@
       <c r="BB87" s="15" t="n"/>
       <c r="BC87" s="15" t="n"/>
       <c r="BD87" s="15" t="n"/>
+      <c r="BE87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -12562,6 +12768,9 @@
       </c>
       <c r="BD88" s="15" t="n">
         <v>21.98</v>
+      </c>
+      <c r="BE88" s="15" t="n">
+        <v>21.3</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -12684,6 +12893,9 @@
       </c>
       <c r="BD89" s="15" t="n">
         <v>8455.41</v>
+      </c>
+      <c r="BE89" s="15" t="n">
+        <v>8534.889999999999</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -12791,6 +13003,7 @@
       <c r="BB90" s="15" t="n"/>
       <c r="BC90" s="15" t="n"/>
       <c r="BD90" s="15" t="n"/>
+      <c r="BE90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -12960,6 +13173,9 @@
       </c>
       <c r="BD91" s="15" t="n">
         <v>6.68</v>
+      </c>
+      <c r="BE91" s="15" t="n">
+        <v>7.74</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -13082,6 +13298,9 @@
       </c>
       <c r="BD92" s="15" t="n">
         <v>1206.57</v>
+      </c>
+      <c r="BE92" s="15" t="n">
+        <v>1235.42</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -13189,6 +13408,7 @@
       <c r="BB93" s="15" t="n"/>
       <c r="BC93" s="15" t="n"/>
       <c r="BD93" s="15" t="n"/>
+      <c r="BE93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -13358,6 +13578,9 @@
       </c>
       <c r="BD94" s="15" t="n">
         <v>7.5</v>
+      </c>
+      <c r="BE94" s="15" t="n">
+        <v>9.02</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -13480,6 +13703,9 @@
       </c>
       <c r="BD95" s="15" t="n">
         <v>14253.77</v>
+      </c>
+      <c r="BE95" s="15" t="n">
+        <v>14613.3</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -13587,6 +13813,7 @@
       <c r="BB96" s="15" t="n"/>
       <c r="BC96" s="15" t="n"/>
       <c r="BD96" s="15" t="n"/>
+      <c r="BE96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -13756,6 +13983,9 @@
       </c>
       <c r="BD97" s="15" t="n">
         <v>45.04</v>
+      </c>
+      <c r="BE97" s="15" t="n">
+        <v>43.5</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -13878,6 +14108,9 @@
       </c>
       <c r="BD98" s="15" t="n">
         <v>3163.62</v>
+      </c>
+      <c r="BE98" s="15" t="n">
+        <v>3137.74</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -13985,6 +14218,7 @@
       <c r="BB99" s="15" t="n"/>
       <c r="BC99" s="15" t="n"/>
       <c r="BD99" s="15" t="n"/>
+      <c r="BE99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -14154,6 +14388,9 @@
       </c>
       <c r="BD100" s="15" t="n">
         <v>36.41</v>
+      </c>
+      <c r="BE100" s="15" t="n">
+        <v>36</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -14276,6 +14513,9 @@
       </c>
       <c r="BD101" s="15" t="n">
         <v>2361.96</v>
+      </c>
+      <c r="BE101" s="15" t="n">
+        <v>2382.13</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -14383,6 +14623,7 @@
       <c r="BB102" s="15" t="n"/>
       <c r="BC102" s="15" t="n"/>
       <c r="BD102" s="15" t="n"/>
+      <c r="BE102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -14552,6 +14793,9 @@
       </c>
       <c r="BD103" s="15" t="n">
         <v>13.82</v>
+      </c>
+      <c r="BE103" s="15" t="n">
+        <v>12.66</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -14674,6 +14918,9 @@
       </c>
       <c r="BD104" s="15" t="n">
         <v>2372.03</v>
+      </c>
+      <c r="BE104" s="15" t="n">
+        <v>2401.79</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -14781,6 +15028,7 @@
       <c r="BB105" s="15" t="n"/>
       <c r="BC105" s="15" t="n"/>
       <c r="BD105" s="15" t="n"/>
+      <c r="BE105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -14950,6 +15198,9 @@
       </c>
       <c r="BD106" s="15" t="n">
         <v>37.73</v>
+      </c>
+      <c r="BE106" s="15" t="n">
+        <v>38.03</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -15072,6 +15323,9 @@
       </c>
       <c r="BD107" s="15" t="n">
         <v>2566.6</v>
+      </c>
+      <c r="BE107" s="15" t="n">
+        <v>2585.79</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -15179,6 +15433,7 @@
       <c r="BB108" s="15" t="n"/>
       <c r="BC108" s="15" t="n"/>
       <c r="BD108" s="15" t="n"/>
+      <c r="BE108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -15348,6 +15603,9 @@
       </c>
       <c r="BD109" s="15" t="n">
         <v>58.79</v>
+      </c>
+      <c r="BE109" s="15" t="n">
+        <v>56.46</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -15470,6 +15728,9 @@
       </c>
       <c r="BD110" s="15" t="n">
         <v>1875.8</v>
+      </c>
+      <c r="BE110" s="15" t="n">
+        <v>1897.58</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -15577,6 +15838,7 @@
       <c r="BB111" s="15" t="n"/>
       <c r="BC111" s="15" t="n"/>
       <c r="BD111" s="15" t="n"/>
+      <c r="BE111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -15746,6 +16008,9 @@
       </c>
       <c r="BD112" s="15" t="n">
         <v>21.7</v>
+      </c>
+      <c r="BE112" s="15" t="n">
+        <v>21.78</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -15868,6 +16133,9 @@
       </c>
       <c r="BD113" s="15" t="n">
         <v>8486.91</v>
+      </c>
+      <c r="BE113" s="15" t="n">
+        <v>8517.129999999999</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -15975,6 +16243,7 @@
       <c r="BB114" s="15" t="n"/>
       <c r="BC114" s="15" t="n"/>
       <c r="BD114" s="15" t="n"/>
+      <c r="BE114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -16144,6 +16413,9 @@
       </c>
       <c r="BD115" s="15" t="n">
         <v>94.84</v>
+      </c>
+      <c r="BE115" s="15" t="n">
+        <v>92.34</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -16251,6 +16523,9 @@
       </c>
       <c r="BD116" s="15" t="n">
         <v>12339.33</v>
+      </c>
+      <c r="BE116" s="15" t="n">
+        <v>12724.46</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -16313,6 +16588,7 @@
       <c r="BB117" s="15" t="n"/>
       <c r="BC117" s="15" t="n"/>
       <c r="BD117" s="15" t="n"/>
+      <c r="BE117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -16438,6 +16714,9 @@
       <c r="BD118" s="15" t="n">
         <v>42.87</v>
       </c>
+      <c r="BE118" s="15" t="n">
+        <v>25.2</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -16535,6 +16814,9 @@
       </c>
       <c r="BD119" s="15" t="n">
         <v>10872.42</v>
+      </c>
+      <c r="BE119" s="15" t="n">
+        <v>1170.06</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -16546,6 +16828,7 @@
       <c r="BB120" s="15" t="n"/>
       <c r="BC120" s="15" t="n"/>
       <c r="BD120" s="15" t="n"/>
+      <c r="BE120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -16572,6 +16855,9 @@
       <c r="BD121" s="15" t="n">
         <v>27.74</v>
       </c>
+      <c r="BE121" s="15" t="n">
+        <v>40.2</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -16597,6 +16883,9 @@
       </c>
       <c r="BD122" s="15" t="n">
         <v>1823.14</v>
+      </c>
+      <c r="BE122" s="15" t="n">
+        <v>11096.98</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -16608,6 +16897,7 @@
       <c r="BB123" s="15" t="n"/>
       <c r="BC123" s="15" t="n"/>
       <c r="BD123" s="15" t="n"/>
+      <c r="BE123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -16634,6 +16924,9 @@
       <c r="BD124" s="15" t="n">
         <v>15.15</v>
       </c>
+      <c r="BE124" s="15" t="n">
+        <v>28.35</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -16659,6 +16952,9 @@
       </c>
       <c r="BD125" s="15" t="n">
         <v>772.16</v>
+      </c>
+      <c r="BE125" s="15" t="n">
+        <v>1810.76</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -16670,6 +16966,7 @@
       <c r="BB126" s="15" t="n"/>
       <c r="BC126" s="15" t="n"/>
       <c r="BD126" s="15" t="n"/>
+      <c r="BE126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -16696,6 +16993,9 @@
       <c r="BD127" s="15" t="n">
         <v>62.09</v>
       </c>
+      <c r="BE127" s="15" t="n">
+        <v>15.32</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -16721,6 +17021,9 @@
       </c>
       <c r="BD128" s="15" t="n">
         <v>2745.29</v>
+      </c>
+      <c r="BE128" s="15" t="n">
+        <v>773.47</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -16732,6 +17035,7 @@
       <c r="BB129" s="15" t="n"/>
       <c r="BC129" s="15" t="n"/>
       <c r="BD129" s="15" t="n"/>
+      <c r="BE129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -16758,6 +17062,9 @@
       <c r="BD130" s="15" t="n">
         <v>20.34</v>
       </c>
+      <c r="BE130" s="15" t="n">
+        <v>60.86</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -16783,6 +17090,9 @@
       </c>
       <c r="BD131" s="15" t="n">
         <v>3517.4</v>
+      </c>
+      <c r="BE131" s="15" t="n">
+        <v>2745.29</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -16794,6 +17104,7 @@
       <c r="BB132" s="15" t="n"/>
       <c r="BC132" s="15" t="n"/>
       <c r="BD132" s="15" t="n"/>
+      <c r="BE132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -16820,6 +17131,9 @@
       <c r="BD133" s="15" t="n">
         <v>2.09</v>
       </c>
+      <c r="BE133" s="15" t="n">
+        <v>20.32</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -16845,6 +17159,9 @@
       </c>
       <c r="BD134" s="15" t="n">
         <v>2326.06</v>
+      </c>
+      <c r="BE134" s="15" t="n">
+        <v>3563.82</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -16856,6 +17173,7 @@
       <c r="BB135" s="15" t="n"/>
       <c r="BC135" s="15" t="n"/>
       <c r="BD135" s="15" t="n"/>
+      <c r="BE135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -16882,6 +17200,9 @@
       <c r="BD136" s="15" t="n">
         <v>8.92</v>
       </c>
+      <c r="BE136" s="15" t="n">
+        <v>2.06</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -16907,6 +17228,35 @@
       </c>
       <c r="BD137" s="15" t="n">
         <v>5391.4</v>
+      </c>
+      <c r="BE137" s="15" t="n">
+        <v>2332.03</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="BE138" s="15" t="n"/>
+    </row>
+    <row r="139">
+      <c r="BE139" s="15" t="n">
+        <v>7.98</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="BE140" s="15" t="n">
+        <v>5307.49</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="BE141" s="15" t="n"/>
+    </row>
+    <row r="142">
+      <c r="BE142" s="15" t="n">
+        <v>25.61</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="BE143" s="15" t="n">
+        <v>2330.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-08-03 06:52:56]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE143"/>
+  <dimension ref="A1:BF143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -591,6 +591,7 @@
     <col width="15" customWidth="1" min="55" max="55"/>
     <col width="15" customWidth="1" min="56" max="56"/>
     <col width="15" customWidth="1" min="57" max="57"/>
+    <col width="15" customWidth="1" min="58" max="58"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -879,6 +880,11 @@
           <t>2026/07/31</t>
         </is>
       </c>
+      <c r="BF1" s="15" t="inlineStr">
+        <is>
+          <t>2026/08/03</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1166,6 +1172,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BF2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1339,6 +1350,9 @@
       <c r="BE3" s="15" t="n">
         <v>57.36</v>
       </c>
+      <c r="BF3" s="15" t="n">
+        <v>58.97</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1511,6 +1525,9 @@
       </c>
       <c r="BE4" s="15" t="n">
         <v>3837.11</v>
+      </c>
+      <c r="BF4" s="15" t="n">
+        <v>3804.48</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1571,6 +1588,7 @@
       <c r="BC5" s="15" t="n"/>
       <c r="BD5" s="15" t="n"/>
       <c r="BE5" s="15" t="n"/>
+      <c r="BF5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1678,6 +1696,7 @@
       <c r="BC6" s="15" t="n"/>
       <c r="BD6" s="15" t="n"/>
       <c r="BE6" s="15" t="n"/>
+      <c r="BF6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1850,6 +1869,9 @@
       </c>
       <c r="BE7" s="15" t="n">
         <v>61.19</v>
+      </c>
+      <c r="BF7" s="15" t="n">
+        <v>61.98</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -1975,6 +1997,9 @@
       </c>
       <c r="BE8" s="15" t="n">
         <v>5656.33</v>
+      </c>
+      <c r="BF8" s="15" t="n">
+        <v>5564.1</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2083,6 +2108,7 @@
       <c r="BC9" s="15" t="n"/>
       <c r="BD9" s="15" t="n"/>
       <c r="BE9" s="15" t="n"/>
+      <c r="BF9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2255,6 +2281,9 @@
       </c>
       <c r="BE10" s="15" t="n">
         <v>55.67</v>
+      </c>
+      <c r="BF10" s="15" t="n">
+        <v>57.54</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2380,6 +2409,9 @@
       </c>
       <c r="BE11" s="15" t="n">
         <v>4604.58</v>
+      </c>
+      <c r="BF11" s="15" t="n">
+        <v>4537.63</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -2488,6 +2520,7 @@
       <c r="BC12" s="15" t="n"/>
       <c r="BD12" s="15" t="n"/>
       <c r="BE12" s="15" t="n"/>
+      <c r="BF12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2660,6 +2693,9 @@
       </c>
       <c r="BE13" s="15" t="n">
         <v>60.19</v>
+      </c>
+      <c r="BF13" s="15" t="n">
+        <v>62.19</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -2785,6 +2821,9 @@
       </c>
       <c r="BE14" s="15" t="n">
         <v>7545.62</v>
+      </c>
+      <c r="BF14" s="15" t="n">
+        <v>7408.74</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -2893,6 +2932,7 @@
       <c r="BC15" s="15" t="n"/>
       <c r="BD15" s="15" t="n"/>
       <c r="BE15" s="15" t="n"/>
+      <c r="BF15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -3065,6 +3105,9 @@
       </c>
       <c r="BE16" s="15" t="n">
         <v>36.64</v>
+      </c>
+      <c r="BF16" s="15" t="n">
+        <v>36.34</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -3190,6 +3233,9 @@
       </c>
       <c r="BE17" s="15" t="n">
         <v>2536.29</v>
+      </c>
+      <c r="BF17" s="15" t="n">
+        <v>2583.02</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -3298,6 +3344,7 @@
       <c r="BC18" s="15" t="n"/>
       <c r="BD18" s="15" t="n"/>
       <c r="BE18" s="15" t="n"/>
+      <c r="BF18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -3470,6 +3517,9 @@
       </c>
       <c r="BE19" s="15" t="n">
         <v>80.76000000000001</v>
+      </c>
+      <c r="BF19" s="15" t="n">
+        <v>81.09999999999999</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -3595,6 +3645,9 @@
       </c>
       <c r="BE20" s="15" t="n">
         <v>7437.63</v>
+      </c>
+      <c r="BF20" s="15" t="n">
+        <v>7489.72</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -3703,6 +3756,7 @@
       <c r="BC21" s="15" t="n"/>
       <c r="BD21" s="15" t="n"/>
       <c r="BE21" s="15" t="n"/>
+      <c r="BF21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -3872,6 +3926,9 @@
         <v>36.34</v>
       </c>
       <c r="BE22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BF22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -3998,6 +4055,9 @@
       </c>
       <c r="BE23" s="15" t="n">
         <v>78041.48</v>
+      </c>
+      <c r="BF23" s="15" t="n">
+        <v>78731.5</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -4106,6 +4166,7 @@
       <c r="BC24" s="15" t="n"/>
       <c r="BD24" s="15" t="n"/>
       <c r="BE24" s="15" t="n"/>
+      <c r="BF24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -4277,6 +4338,9 @@
         <v>49.88</v>
       </c>
       <c r="BE25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BF25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -4392,6 +4456,9 @@
       </c>
       <c r="BD26" s="15" t="inlineStr"/>
       <c r="BE26" s="15" t="inlineStr"/>
+      <c r="BF26" s="15" t="n">
+        <v>25629.24</v>
+      </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -4499,6 +4566,7 @@
       <c r="BC27" s="15" t="n"/>
       <c r="BD27" s="15" t="n"/>
       <c r="BE27" s="15" t="n"/>
+      <c r="BF27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -4670,6 +4738,9 @@
         <v>92.09</v>
       </c>
       <c r="BE28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BF28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -4796,6 +4867,9 @@
       </c>
       <c r="BE29" s="15" t="n">
         <v>64409.39</v>
+      </c>
+      <c r="BF29" s="15" t="n">
+        <v>63754.9</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -4904,6 +4978,7 @@
       <c r="BC30" s="15" t="n"/>
       <c r="BD30" s="15" t="n"/>
       <c r="BE30" s="15" t="n"/>
+      <c r="BF30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -5076,6 +5151,9 @@
       </c>
       <c r="BE31" s="15" t="n">
         <v>46.99</v>
+      </c>
+      <c r="BF31" s="15" t="n">
+        <v>46.51</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -5201,6 +5279,9 @@
       </c>
       <c r="BE32" s="15" t="n">
         <v>5548.06</v>
+      </c>
+      <c r="BF32" s="15" t="n">
+        <v>5548.54</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -5309,6 +5390,7 @@
       <c r="BC33" s="15" t="n"/>
       <c r="BD33" s="15" t="n"/>
       <c r="BE33" s="15" t="n"/>
+      <c r="BF33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -5481,6 +5563,9 @@
       </c>
       <c r="BE34" s="15" t="n">
         <v>55.98</v>
+      </c>
+      <c r="BF34" s="15" t="n">
+        <v>56.88</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -5606,6 +5691,9 @@
       </c>
       <c r="BE35" s="15" t="n">
         <v>11692.35</v>
+      </c>
+      <c r="BF35" s="15" t="n">
+        <v>11782.42</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -5714,6 +5802,7 @@
       <c r="BC36" s="15" t="n"/>
       <c r="BD36" s="15" t="n"/>
       <c r="BE36" s="15" t="n"/>
+      <c r="BF36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -5886,6 +5975,9 @@
       </c>
       <c r="BE37" s="15" t="n">
         <v>50.44</v>
+      </c>
+      <c r="BF37" s="15" t="n">
+        <v>51.02</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -6011,6 +6103,9 @@
       </c>
       <c r="BE38" s="15" t="n">
         <v>11171.66</v>
+      </c>
+      <c r="BF38" s="15" t="n">
+        <v>11125.28</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -6119,6 +6214,7 @@
       <c r="BC39" s="15" t="n"/>
       <c r="BD39" s="15" t="n"/>
       <c r="BE39" s="15" t="n"/>
+      <c r="BF39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -6291,6 +6387,9 @@
       </c>
       <c r="BE40" s="15" t="n">
         <v>50.19</v>
+      </c>
+      <c r="BF40" s="15" t="n">
+        <v>50.72</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -6416,6 +6515,9 @@
       </c>
       <c r="BE41" s="15" t="n">
         <v>3227.27</v>
+      </c>
+      <c r="BF41" s="15" t="n">
+        <v>3220.68</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -6524,6 +6626,7 @@
       <c r="BC42" s="15" t="n"/>
       <c r="BD42" s="15" t="n"/>
       <c r="BE42" s="15" t="n"/>
+      <c r="BF42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -6696,6 +6799,9 @@
       </c>
       <c r="BE43" s="15" t="n">
         <v>58.6</v>
+      </c>
+      <c r="BF43" s="15" t="n">
+        <v>58.65</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -6821,6 +6927,9 @@
       </c>
       <c r="BE44" s="15" t="n">
         <v>7244.78</v>
+      </c>
+      <c r="BF44" s="15" t="n">
+        <v>7165.05</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -6929,6 +7038,7 @@
       <c r="BC45" s="15" t="n"/>
       <c r="BD45" s="15" t="n"/>
       <c r="BE45" s="15" t="n"/>
+      <c r="BF45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -7101,6 +7211,9 @@
       </c>
       <c r="BE46" s="15" t="n">
         <v>27.08</v>
+      </c>
+      <c r="BF46" s="15" t="n">
+        <v>27.96</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -7226,6 +7339,9 @@
       </c>
       <c r="BE47" s="15" t="n">
         <v>33613.32</v>
+      </c>
+      <c r="BF47" s="15" t="n">
+        <v>33503.52</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -7334,6 +7450,7 @@
       <c r="BC48" s="15" t="n"/>
       <c r="BD48" s="15" t="n"/>
       <c r="BE48" s="15" t="n"/>
+      <c r="BF48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -7506,6 +7623,9 @@
       </c>
       <c r="BE49" s="15" t="n">
         <v>41.67</v>
+      </c>
+      <c r="BF49" s="15" t="n">
+        <v>44.37</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -7631,6 +7751,9 @@
       </c>
       <c r="BE50" s="15" t="n">
         <v>3566.54</v>
+      </c>
+      <c r="BF50" s="15" t="n">
+        <v>3492.47</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -7739,6 +7862,7 @@
       <c r="BC51" s="15" t="n"/>
       <c r="BD51" s="15" t="n"/>
       <c r="BE51" s="15" t="n"/>
+      <c r="BF51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -7911,6 +8035,9 @@
       </c>
       <c r="BE52" s="15" t="n">
         <v>49.08</v>
+      </c>
+      <c r="BF52" s="15" t="n">
+        <v>52.67</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -8036,6 +8163,9 @@
       </c>
       <c r="BE53" s="15" t="n">
         <v>3387.38</v>
+      </c>
+      <c r="BF53" s="15" t="n">
+        <v>3301.05</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -8144,6 +8274,7 @@
       <c r="BC54" s="15" t="n"/>
       <c r="BD54" s="15" t="n"/>
       <c r="BE54" s="15" t="n"/>
+      <c r="BF54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -8316,6 +8447,9 @@
       </c>
       <c r="BE55" s="15" t="n">
         <v>10.42</v>
+      </c>
+      <c r="BF55" s="15" t="n">
+        <v>12.51</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -8441,6 +8575,9 @@
       </c>
       <c r="BE56" s="15" t="n">
         <v>6520.71</v>
+      </c>
+      <c r="BF56" s="15" t="n">
+        <v>6456.47</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -8549,6 +8686,7 @@
       <c r="BC57" s="15" t="n"/>
       <c r="BD57" s="15" t="n"/>
       <c r="BE57" s="15" t="n"/>
+      <c r="BF57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -8721,6 +8859,9 @@
       </c>
       <c r="BE58" s="15" t="n">
         <v>37.16</v>
+      </c>
+      <c r="BF58" s="15" t="n">
+        <v>36.95</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -8846,6 +8987,9 @@
       </c>
       <c r="BE59" s="15" t="n">
         <v>8084.53</v>
+      </c>
+      <c r="BF59" s="15" t="n">
+        <v>8019.07</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -8954,6 +9098,7 @@
       <c r="BC60" s="15" t="n"/>
       <c r="BD60" s="15" t="n"/>
       <c r="BE60" s="15" t="n"/>
+      <c r="BF60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -9126,6 +9271,9 @@
       </c>
       <c r="BE61" s="15" t="n">
         <v>7.29</v>
+      </c>
+      <c r="BF61" s="15" t="n">
+        <v>6.54</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -9251,6 +9399,9 @@
       </c>
       <c r="BE62" s="15" t="n">
         <v>11337.21</v>
+      </c>
+      <c r="BF62" s="15" t="n">
+        <v>11144.58</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -9359,6 +9510,7 @@
       <c r="BC63" s="15" t="n"/>
       <c r="BD63" s="15" t="n"/>
       <c r="BE63" s="15" t="n"/>
+      <c r="BF63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -9531,6 +9683,9 @@
       </c>
       <c r="BE64" s="15" t="n">
         <v>22.07</v>
+      </c>
+      <c r="BF64" s="15" t="n">
+        <v>22.94</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -9656,6 +9811,9 @@
       </c>
       <c r="BE65" s="15" t="n">
         <v>11429.35</v>
+      </c>
+      <c r="BF65" s="15" t="n">
+        <v>11328.53</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -9764,6 +9922,7 @@
       <c r="BC66" s="15" t="n"/>
       <c r="BD66" s="15" t="n"/>
       <c r="BE66" s="15" t="n"/>
+      <c r="BF66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -9936,6 +10095,9 @@
       </c>
       <c r="BE67" s="15" t="n">
         <v>20.16</v>
+      </c>
+      <c r="BF67" s="15" t="n">
+        <v>19.68</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -10061,6 +10223,9 @@
       </c>
       <c r="BE68" s="15" t="n">
         <v>6918.68</v>
+      </c>
+      <c r="BF68" s="15" t="n">
+        <v>6863.21</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -10169,6 +10334,7 @@
       <c r="BC69" s="15" t="n"/>
       <c r="BD69" s="15" t="n"/>
       <c r="BE69" s="15" t="n"/>
+      <c r="BF69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -10341,6 +10507,9 @@
       </c>
       <c r="BE70" s="15" t="n">
         <v>18.57</v>
+      </c>
+      <c r="BF70" s="15" t="n">
+        <v>18.36</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -10466,6 +10635,9 @@
       </c>
       <c r="BE71" s="15" t="n">
         <v>13006.35</v>
+      </c>
+      <c r="BF71" s="15" t="n">
+        <v>12975.39</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -10574,6 +10746,7 @@
       <c r="BC72" s="15" t="n"/>
       <c r="BD72" s="15" t="n"/>
       <c r="BE72" s="15" t="n"/>
+      <c r="BF72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -10746,6 +10919,9 @@
       </c>
       <c r="BE73" s="15" t="n">
         <v>52.02</v>
+      </c>
+      <c r="BF73" s="15" t="n">
+        <v>53.26</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -10871,6 +11047,9 @@
       </c>
       <c r="BE74" s="15" t="n">
         <v>13850.53</v>
+      </c>
+      <c r="BF74" s="15" t="n">
+        <v>13655.35</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -10979,6 +11158,7 @@
       <c r="BC75" s="15" t="n"/>
       <c r="BD75" s="15" t="n"/>
       <c r="BE75" s="15" t="n"/>
+      <c r="BF75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -11151,6 +11331,9 @@
       </c>
       <c r="BE76" s="15" t="n">
         <v>4.82</v>
+      </c>
+      <c r="BF76" s="15" t="n">
+        <v>5.08</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -11276,6 +11459,9 @@
       </c>
       <c r="BE77" s="15" t="n">
         <v>7294.46</v>
+      </c>
+      <c r="BF77" s="15" t="n">
+        <v>7319.35</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
@@ -11384,6 +11570,7 @@
       <c r="BC78" s="15" t="n"/>
       <c r="BD78" s="15" t="n"/>
       <c r="BE78" s="15" t="n"/>
+      <c r="BF78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -11556,6 +11743,9 @@
       </c>
       <c r="BE79" s="15" t="n">
         <v>4.58</v>
+      </c>
+      <c r="BF79" s="15" t="n">
+        <v>4.96</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -11681,6 +11871,9 @@
       </c>
       <c r="BE80" s="15" t="n">
         <v>8937.27</v>
+      </c>
+      <c r="BF80" s="15" t="n">
+        <v>8996.5</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -11789,6 +11982,7 @@
       <c r="BC81" s="15" t="n"/>
       <c r="BD81" s="15" t="n"/>
       <c r="BE81" s="15" t="n"/>
+      <c r="BF81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -11961,6 +12155,9 @@
       </c>
       <c r="BE82" s="15" t="n">
         <v>14.04</v>
+      </c>
+      <c r="BF82" s="15" t="n">
+        <v>14.57</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -12085,6 +12282,9 @@
         <v>2376.64</v>
       </c>
       <c r="BE83" s="15" t="n">
+        <v>2631.9</v>
+      </c>
+      <c r="BF83" s="15" t="n">
         <v>2631.9</v>
       </c>
     </row>
@@ -12194,6 +12394,7 @@
       <c r="BC84" s="15" t="n"/>
       <c r="BD84" s="15" t="n"/>
       <c r="BE84" s="15" t="n"/>
+      <c r="BF84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -12366,6 +12567,9 @@
       </c>
       <c r="BE85" s="15" t="n">
         <v>26.7</v>
+      </c>
+      <c r="BF85" s="15" t="n">
+        <v>28.41</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -12491,6 +12695,9 @@
       </c>
       <c r="BE86" s="15" t="n">
         <v>5075.31</v>
+      </c>
+      <c r="BF86" s="15" t="n">
+        <v>4857.7</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -12599,6 +12806,7 @@
       <c r="BC87" s="15" t="n"/>
       <c r="BD87" s="15" t="n"/>
       <c r="BE87" s="15" t="n"/>
+      <c r="BF87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -12771,6 +12979,9 @@
       </c>
       <c r="BE88" s="15" t="n">
         <v>21.3</v>
+      </c>
+      <c r="BF88" s="15" t="n">
+        <v>21.9</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -12896,6 +13107,9 @@
       </c>
       <c r="BE89" s="15" t="n">
         <v>8534.889999999999</v>
+      </c>
+      <c r="BF89" s="15" t="n">
+        <v>8449.16</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -13004,6 +13218,7 @@
       <c r="BC90" s="15" t="n"/>
       <c r="BD90" s="15" t="n"/>
       <c r="BE90" s="15" t="n"/>
+      <c r="BF90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -13176,6 +13391,9 @@
       </c>
       <c r="BE91" s="15" t="n">
         <v>7.74</v>
+      </c>
+      <c r="BF91" s="15" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -13301,6 +13519,9 @@
       </c>
       <c r="BE92" s="15" t="n">
         <v>1235.42</v>
+      </c>
+      <c r="BF92" s="15" t="n">
+        <v>1218.35</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -13409,6 +13630,7 @@
       <c r="BC93" s="15" t="n"/>
       <c r="BD93" s="15" t="n"/>
       <c r="BE93" s="15" t="n"/>
+      <c r="BF93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -13581,6 +13803,9 @@
       </c>
       <c r="BE94" s="15" t="n">
         <v>9.02</v>
+      </c>
+      <c r="BF94" s="15" t="n">
+        <v>8.619999999999999</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -13706,6 +13931,9 @@
       </c>
       <c r="BE95" s="15" t="n">
         <v>14613.3</v>
+      </c>
+      <c r="BF95" s="15" t="n">
+        <v>14532.99</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -13814,6 +14042,7 @@
       <c r="BC96" s="15" t="n"/>
       <c r="BD96" s="15" t="n"/>
       <c r="BE96" s="15" t="n"/>
+      <c r="BF96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -13986,6 +14215,9 @@
       </c>
       <c r="BE97" s="15" t="n">
         <v>43.5</v>
+      </c>
+      <c r="BF97" s="15" t="n">
+        <v>44.05</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -14111,6 +14343,9 @@
       </c>
       <c r="BE98" s="15" t="n">
         <v>3137.74</v>
+      </c>
+      <c r="BF98" s="15" t="n">
+        <v>3162.76</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -14219,6 +14454,7 @@
       <c r="BC99" s="15" t="n"/>
       <c r="BD99" s="15" t="n"/>
       <c r="BE99" s="15" t="n"/>
+      <c r="BF99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -14391,6 +14627,9 @@
       </c>
       <c r="BE100" s="15" t="n">
         <v>36</v>
+      </c>
+      <c r="BF100" s="15" t="n">
+        <v>36.08</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -14516,6 +14755,9 @@
       </c>
       <c r="BE101" s="15" t="n">
         <v>2382.13</v>
+      </c>
+      <c r="BF101" s="15" t="n">
+        <v>2384.92</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -14624,6 +14866,7 @@
       <c r="BC102" s="15" t="n"/>
       <c r="BD102" s="15" t="n"/>
       <c r="BE102" s="15" t="n"/>
+      <c r="BF102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -14796,6 +15039,9 @@
       </c>
       <c r="BE103" s="15" t="n">
         <v>12.66</v>
+      </c>
+      <c r="BF103" s="15" t="n">
+        <v>14.05</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -14921,6 +15167,9 @@
       </c>
       <c r="BE104" s="15" t="n">
         <v>2401.79</v>
+      </c>
+      <c r="BF104" s="15" t="n">
+        <v>2444.22</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -15029,6 +15278,7 @@
       <c r="BC105" s="15" t="n"/>
       <c r="BD105" s="15" t="n"/>
       <c r="BE105" s="15" t="n"/>
+      <c r="BF105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -15201,6 +15451,9 @@
       </c>
       <c r="BE106" s="15" t="n">
         <v>38.03</v>
+      </c>
+      <c r="BF106" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -15326,6 +15579,9 @@
       </c>
       <c r="BE107" s="15" t="n">
         <v>2585.79</v>
+      </c>
+      <c r="BF107" s="15" t="n">
+        <v>2573.31</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -15434,6 +15690,7 @@
       <c r="BC108" s="15" t="n"/>
       <c r="BD108" s="15" t="n"/>
       <c r="BE108" s="15" t="n"/>
+      <c r="BF108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -15606,6 +15863,9 @@
       </c>
       <c r="BE109" s="15" t="n">
         <v>56.46</v>
+      </c>
+      <c r="BF109" s="15" t="n">
+        <v>57</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -15731,6 +15991,9 @@
       </c>
       <c r="BE110" s="15" t="n">
         <v>1897.58</v>
+      </c>
+      <c r="BF110" s="15" t="n">
+        <v>1898.59</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -15839,6 +16102,7 @@
       <c r="BC111" s="15" t="n"/>
       <c r="BD111" s="15" t="n"/>
       <c r="BE111" s="15" t="n"/>
+      <c r="BF111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -16011,6 +16275,9 @@
       </c>
       <c r="BE112" s="15" t="n">
         <v>21.78</v>
+      </c>
+      <c r="BF112" s="15" t="n">
+        <v>22.54</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -16136,6 +16403,9 @@
       </c>
       <c r="BE113" s="15" t="n">
         <v>8517.129999999999</v>
+      </c>
+      <c r="BF113" s="15" t="n">
+        <v>8486.91</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -16244,6 +16514,7 @@
       <c r="BC114" s="15" t="n"/>
       <c r="BD114" s="15" t="n"/>
       <c r="BE114" s="15" t="n"/>
+      <c r="BF114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -16416,6 +16687,9 @@
       </c>
       <c r="BE115" s="15" t="n">
         <v>92.34</v>
+      </c>
+      <c r="BF115" s="15" t="n">
+        <v>93.19</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -16526,6 +16800,9 @@
       </c>
       <c r="BE116" s="15" t="n">
         <v>12724.46</v>
+      </c>
+      <c r="BF116" s="15" t="n">
+        <v>11627.83</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -16589,6 +16866,7 @@
       <c r="BC117" s="15" t="n"/>
       <c r="BD117" s="15" t="n"/>
       <c r="BE117" s="15" t="n"/>
+      <c r="BF117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -16717,6 +16995,9 @@
       <c r="BE118" s="15" t="n">
         <v>25.2</v>
       </c>
+      <c r="BF118" s="15" t="n">
+        <v>31.69</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -16817,6 +17098,9 @@
       </c>
       <c r="BE119" s="15" t="n">
         <v>1170.06</v>
+      </c>
+      <c r="BF119" s="15" t="n">
+        <v>1243.02</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -16829,6 +17113,7 @@
       <c r="BC120" s="15" t="n"/>
       <c r="BD120" s="15" t="n"/>
       <c r="BE120" s="15" t="n"/>
+      <c r="BF120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -16858,6 +17143,9 @@
       <c r="BE121" s="15" t="n">
         <v>40.2</v>
       </c>
+      <c r="BF121" s="15" t="n">
+        <v>42.69</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -16886,6 +17174,9 @@
       </c>
       <c r="BE122" s="15" t="n">
         <v>11096.98</v>
+      </c>
+      <c r="BF122" s="15" t="n">
+        <v>11146.58</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -16898,6 +17189,7 @@
       <c r="BC123" s="15" t="n"/>
       <c r="BD123" s="15" t="n"/>
       <c r="BE123" s="15" t="n"/>
+      <c r="BF123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -16927,6 +17219,9 @@
       <c r="BE124" s="15" t="n">
         <v>28.35</v>
       </c>
+      <c r="BF124" s="15" t="n">
+        <v>28.34</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -16955,6 +17250,9 @@
       </c>
       <c r="BE125" s="15" t="n">
         <v>1810.76</v>
+      </c>
+      <c r="BF125" s="15" t="n">
+        <v>1864.85</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -16967,6 +17265,7 @@
       <c r="BC126" s="15" t="n"/>
       <c r="BD126" s="15" t="n"/>
       <c r="BE126" s="15" t="n"/>
+      <c r="BF126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -16996,6 +17295,9 @@
       <c r="BE127" s="15" t="n">
         <v>15.32</v>
       </c>
+      <c r="BF127" s="15" t="n">
+        <v>14.68</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -17024,6 +17326,9 @@
       </c>
       <c r="BE128" s="15" t="n">
         <v>773.47</v>
+      </c>
+      <c r="BF128" s="15" t="n">
+        <v>769.83</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -17036,6 +17341,7 @@
       <c r="BC129" s="15" t="n"/>
       <c r="BD129" s="15" t="n"/>
       <c r="BE129" s="15" t="n"/>
+      <c r="BF129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -17065,6 +17371,9 @@
       <c r="BE130" s="15" t="n">
         <v>60.86</v>
       </c>
+      <c r="BF130" s="15" t="n">
+        <v>63.65</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -17093,6 +17402,9 @@
       </c>
       <c r="BE131" s="15" t="n">
         <v>2745.29</v>
+      </c>
+      <c r="BF131" s="15" t="n">
+        <v>2815.99</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -17105,6 +17417,7 @@
       <c r="BC132" s="15" t="n"/>
       <c r="BD132" s="15" t="n"/>
       <c r="BE132" s="15" t="n"/>
+      <c r="BF132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -17134,6 +17447,9 @@
       <c r="BE133" s="15" t="n">
         <v>20.32</v>
       </c>
+      <c r="BF133" s="15" t="n">
+        <v>20.84</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -17162,6 +17478,9 @@
       </c>
       <c r="BE134" s="15" t="n">
         <v>3563.82</v>
+      </c>
+      <c r="BF134" s="15" t="n">
+        <v>3576.02</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -17174,6 +17493,7 @@
       <c r="BC135" s="15" t="n"/>
       <c r="BD135" s="15" t="n"/>
       <c r="BE135" s="15" t="n"/>
+      <c r="BF135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -17203,6 +17523,9 @@
       <c r="BE136" s="15" t="n">
         <v>2.06</v>
       </c>
+      <c r="BF136" s="15" t="n">
+        <v>2.43</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -17232,31 +17555,48 @@
       <c r="BE137" s="15" t="n">
         <v>2332.03</v>
       </c>
+      <c r="BF137" s="15" t="n">
+        <v>2350.74</v>
+      </c>
     </row>
     <row r="138">
       <c r="BE138" s="15" t="n"/>
+      <c r="BF138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
         <v>7.98</v>
       </c>
+      <c r="BF139" s="15" t="n">
+        <v>8.960000000000001</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
         <v>5307.49</v>
       </c>
+      <c r="BF140" s="15" t="n">
+        <v>5375.74</v>
+      </c>
     </row>
     <row r="141">
       <c r="BE141" s="15" t="n"/>
+      <c r="BF141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
         <v>25.61</v>
       </c>
+      <c r="BF142" s="15" t="n">
+        <v>25.87</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
         <v>2330.3</v>
+      </c>
+      <c r="BF143" s="15" t="n">
+        <v>2353.44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-08-06 06:17:07]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BF143"/>
+  <dimension ref="A1:BG143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -592,6 +592,7 @@
     <col width="15" customWidth="1" min="56" max="56"/>
     <col width="15" customWidth="1" min="57" max="57"/>
     <col width="15" customWidth="1" min="58" max="58"/>
+    <col width="15" customWidth="1" min="59" max="59"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -885,6 +886,11 @@
           <t>2026/08/03</t>
         </is>
       </c>
+      <c r="BG1" s="15" t="inlineStr">
+        <is>
+          <t>2026/08/06</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1177,6 +1183,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BG2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1353,6 +1364,9 @@
       <c r="BF3" s="15" t="n">
         <v>58.97</v>
       </c>
+      <c r="BG3" s="15" t="n">
+        <v>62.6</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1528,6 +1542,9 @@
       </c>
       <c r="BF4" s="15" t="n">
         <v>3804.48</v>
+      </c>
+      <c r="BG4" s="15" t="n">
+        <v>3881.78</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1589,6 +1606,7 @@
       <c r="BD5" s="15" t="n"/>
       <c r="BE5" s="15" t="n"/>
       <c r="BF5" s="15" t="n"/>
+      <c r="BG5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1697,6 +1715,7 @@
       <c r="BD6" s="15" t="n"/>
       <c r="BE6" s="15" t="n"/>
       <c r="BF6" s="15" t="n"/>
+      <c r="BG6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1872,6 +1891,9 @@
       </c>
       <c r="BF7" s="15" t="n">
         <v>61.98</v>
+      </c>
+      <c r="BG7" s="15" t="n">
+        <v>62.27</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -2000,6 +2022,9 @@
       </c>
       <c r="BF8" s="15" t="n">
         <v>5564.1</v>
+      </c>
+      <c r="BG8" s="15" t="n">
+        <v>5716.01</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2109,6 +2134,7 @@
       <c r="BD9" s="15" t="n"/>
       <c r="BE9" s="15" t="n"/>
       <c r="BF9" s="15" t="n"/>
+      <c r="BG9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2284,6 +2310,9 @@
       </c>
       <c r="BF10" s="15" t="n">
         <v>57.54</v>
+      </c>
+      <c r="BG10" s="15" t="n">
+        <v>55.62</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2412,6 +2441,9 @@
       </c>
       <c r="BF11" s="15" t="n">
         <v>4537.63</v>
+      </c>
+      <c r="BG11" s="15" t="n">
+        <v>4626.78</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -2521,6 +2553,7 @@
       <c r="BD12" s="15" t="n"/>
       <c r="BE12" s="15" t="n"/>
       <c r="BF12" s="15" t="n"/>
+      <c r="BG12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2696,6 +2729,9 @@
       </c>
       <c r="BF13" s="15" t="n">
         <v>62.19</v>
+      </c>
+      <c r="BG13" s="15" t="n">
+        <v>65.56</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -2824,6 +2860,9 @@
       </c>
       <c r="BF14" s="15" t="n">
         <v>7408.74</v>
+      </c>
+      <c r="BG14" s="15" t="n">
+        <v>7757.44</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -2933,6 +2972,7 @@
       <c r="BD15" s="15" t="n"/>
       <c r="BE15" s="15" t="n"/>
       <c r="BF15" s="15" t="n"/>
+      <c r="BG15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -3108,6 +3148,9 @@
       </c>
       <c r="BF16" s="15" t="n">
         <v>36.34</v>
+      </c>
+      <c r="BG16" s="15" t="n">
+        <v>35.5</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -3236,6 +3279,9 @@
       </c>
       <c r="BF17" s="15" t="n">
         <v>2583.02</v>
+      </c>
+      <c r="BG17" s="15" t="n">
+        <v>2594.58</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -3345,6 +3391,7 @@
       <c r="BD18" s="15" t="n"/>
       <c r="BE18" s="15" t="n"/>
       <c r="BF18" s="15" t="n"/>
+      <c r="BG18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -3520,6 +3567,9 @@
       </c>
       <c r="BF19" s="15" t="n">
         <v>81.09999999999999</v>
+      </c>
+      <c r="BG19" s="15" t="n">
+        <v>82.34999999999999</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -3648,6 +3698,9 @@
       </c>
       <c r="BF20" s="15" t="n">
         <v>7489.72</v>
+      </c>
+      <c r="BG20" s="15" t="n">
+        <v>7723.55</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -3757,6 +3810,7 @@
       <c r="BD21" s="15" t="n"/>
       <c r="BE21" s="15" t="n"/>
       <c r="BF21" s="15" t="n"/>
+      <c r="BG21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -3929,6 +3983,9 @@
         <v>36.34</v>
       </c>
       <c r="BF22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BG22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -4058,6 +4115,9 @@
       </c>
       <c r="BF23" s="15" t="n">
         <v>78731.5</v>
+      </c>
+      <c r="BG23" s="15" t="n">
+        <v>78859.21000000001</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -4167,6 +4227,7 @@
       <c r="BD24" s="15" t="n"/>
       <c r="BE24" s="15" t="n"/>
       <c r="BF24" s="15" t="n"/>
+      <c r="BG24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -4341,6 +4402,9 @@
         <v>49.88</v>
       </c>
       <c r="BF25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BG25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -4459,6 +4523,7 @@
       <c r="BF26" s="15" t="n">
         <v>25629.24</v>
       </c>
+      <c r="BG26" s="15" t="inlineStr"/>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -4567,6 +4632,7 @@
       <c r="BD27" s="15" t="n"/>
       <c r="BE27" s="15" t="n"/>
       <c r="BF27" s="15" t="n"/>
+      <c r="BG27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -4741,6 +4807,9 @@
         <v>92.09</v>
       </c>
       <c r="BF28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BG28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -4870,6 +4939,9 @@
       </c>
       <c r="BF29" s="15" t="n">
         <v>63754.9</v>
+      </c>
+      <c r="BG29" s="15" t="n">
+        <v>65678.78999999999</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -4979,6 +5051,7 @@
       <c r="BD30" s="15" t="n"/>
       <c r="BE30" s="15" t="n"/>
       <c r="BF30" s="15" t="n"/>
+      <c r="BG30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -5154,6 +5227,9 @@
       </c>
       <c r="BF31" s="15" t="n">
         <v>46.51</v>
+      </c>
+      <c r="BG31" s="15" t="n">
+        <v>45.43</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -5282,6 +5358,9 @@
       </c>
       <c r="BF32" s="15" t="n">
         <v>5548.54</v>
+      </c>
+      <c r="BG32" s="15" t="n">
+        <v>5526.25</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -5391,6 +5470,7 @@
       <c r="BD33" s="15" t="n"/>
       <c r="BE33" s="15" t="n"/>
       <c r="BF33" s="15" t="n"/>
+      <c r="BG33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -5566,6 +5646,9 @@
       </c>
       <c r="BF34" s="15" t="n">
         <v>56.88</v>
+      </c>
+      <c r="BG34" s="15" t="n">
+        <v>58.75</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -5694,6 +5777,9 @@
       </c>
       <c r="BF35" s="15" t="n">
         <v>11782.42</v>
+      </c>
+      <c r="BG35" s="15" t="n">
+        <v>11306.07</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -5803,6 +5889,7 @@
       <c r="BD36" s="15" t="n"/>
       <c r="BE36" s="15" t="n"/>
       <c r="BF36" s="15" t="n"/>
+      <c r="BG36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -5978,6 +6065,9 @@
       </c>
       <c r="BF37" s="15" t="n">
         <v>51.02</v>
+      </c>
+      <c r="BG37" s="15" t="n">
+        <v>49.75</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -6106,6 +6196,9 @@
       </c>
       <c r="BF38" s="15" t="n">
         <v>11125.28</v>
+      </c>
+      <c r="BG38" s="15" t="n">
+        <v>10766.13</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -6215,6 +6308,7 @@
       <c r="BD39" s="15" t="n"/>
       <c r="BE39" s="15" t="n"/>
       <c r="BF39" s="15" t="n"/>
+      <c r="BG39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -6390,6 +6484,9 @@
       </c>
       <c r="BF40" s="15" t="n">
         <v>50.72</v>
+      </c>
+      <c r="BG40" s="15" t="n">
+        <v>49.12</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -6518,6 +6615,9 @@
       </c>
       <c r="BF41" s="15" t="n">
         <v>3220.68</v>
+      </c>
+      <c r="BG41" s="15" t="n">
+        <v>3141.46</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -6627,6 +6727,7 @@
       <c r="BD42" s="15" t="n"/>
       <c r="BE42" s="15" t="n"/>
       <c r="BF42" s="15" t="n"/>
+      <c r="BG42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -6802,6 +6903,9 @@
       </c>
       <c r="BF43" s="15" t="n">
         <v>58.65</v>
+      </c>
+      <c r="BG43" s="15" t="n">
+        <v>57.33</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -6930,6 +7034,9 @@
       </c>
       <c r="BF44" s="15" t="n">
         <v>7165.05</v>
+      </c>
+      <c r="BG44" s="15" t="n">
+        <v>6944.22</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -7039,6 +7146,7 @@
       <c r="BD45" s="15" t="n"/>
       <c r="BE45" s="15" t="n"/>
       <c r="BF45" s="15" t="n"/>
+      <c r="BG45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -7214,6 +7322,9 @@
       </c>
       <c r="BF46" s="15" t="n">
         <v>27.96</v>
+      </c>
+      <c r="BG46" s="15" t="n">
+        <v>27.08</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -7341,6 +7452,9 @@
         <v>33613.32</v>
       </c>
       <c r="BF47" s="15" t="n">
+        <v>33503.52</v>
+      </c>
+      <c r="BG47" s="15" t="n">
         <v>33503.52</v>
       </c>
     </row>
@@ -7451,6 +7565,7 @@
       <c r="BD48" s="15" t="n"/>
       <c r="BE48" s="15" t="n"/>
       <c r="BF48" s="15" t="n"/>
+      <c r="BG48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -7626,6 +7741,9 @@
       </c>
       <c r="BF49" s="15" t="n">
         <v>44.37</v>
+      </c>
+      <c r="BG49" s="15" t="n">
+        <v>48.97</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -7754,6 +7872,9 @@
       </c>
       <c r="BF50" s="15" t="n">
         <v>3492.47</v>
+      </c>
+      <c r="BG50" s="15" t="n">
+        <v>3674.04</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -7863,6 +7984,7 @@
       <c r="BD51" s="15" t="n"/>
       <c r="BE51" s="15" t="n"/>
       <c r="BF51" s="15" t="n"/>
+      <c r="BG51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -8038,6 +8160,9 @@
       </c>
       <c r="BF52" s="15" t="n">
         <v>52.67</v>
+      </c>
+      <c r="BG52" s="15" t="n">
+        <v>59.21</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -8166,6 +8291,9 @@
       </c>
       <c r="BF53" s="15" t="n">
         <v>3301.05</v>
+      </c>
+      <c r="BG53" s="15" t="n">
+        <v>3486.45</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -8275,6 +8403,7 @@
       <c r="BD54" s="15" t="n"/>
       <c r="BE54" s="15" t="n"/>
       <c r="BF54" s="15" t="n"/>
+      <c r="BG54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -8450,6 +8579,9 @@
       </c>
       <c r="BF55" s="15" t="n">
         <v>12.51</v>
+      </c>
+      <c r="BG55" s="15" t="n">
+        <v>14.69</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -8578,6 +8710,9 @@
       </c>
       <c r="BF56" s="15" t="n">
         <v>6456.47</v>
+      </c>
+      <c r="BG56" s="15" t="n">
+        <v>6550.13</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -8687,6 +8822,7 @@
       <c r="BD57" s="15" t="n"/>
       <c r="BE57" s="15" t="n"/>
       <c r="BF57" s="15" t="n"/>
+      <c r="BG57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -8862,6 +8998,9 @@
       </c>
       <c r="BF58" s="15" t="n">
         <v>36.95</v>
+      </c>
+      <c r="BG58" s="15" t="n">
+        <v>36.06</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -8990,6 +9129,9 @@
       </c>
       <c r="BF59" s="15" t="n">
         <v>8019.07</v>
+      </c>
+      <c r="BG59" s="15" t="n">
+        <v>8167.59</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -9099,6 +9241,7 @@
       <c r="BD60" s="15" t="n"/>
       <c r="BE60" s="15" t="n"/>
       <c r="BF60" s="15" t="n"/>
+      <c r="BG60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -9274,6 +9417,9 @@
       </c>
       <c r="BF61" s="15" t="n">
         <v>6.54</v>
+      </c>
+      <c r="BG61" s="15" t="n">
+        <v>4.17</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -9402,6 +9548,9 @@
       </c>
       <c r="BF62" s="15" t="n">
         <v>11144.58</v>
+      </c>
+      <c r="BG62" s="15" t="n">
+        <v>10898.57</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -9511,6 +9660,7 @@
       <c r="BD63" s="15" t="n"/>
       <c r="BE63" s="15" t="n"/>
       <c r="BF63" s="15" t="n"/>
+      <c r="BG63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -9686,6 +9836,9 @@
       </c>
       <c r="BF64" s="15" t="n">
         <v>22.94</v>
+      </c>
+      <c r="BG64" s="15" t="n">
+        <v>21.93</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -9814,6 +9967,9 @@
       </c>
       <c r="BF65" s="15" t="n">
         <v>11328.53</v>
+      </c>
+      <c r="BG65" s="15" t="n">
+        <v>11368.1</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -9923,6 +10079,7 @@
       <c r="BD66" s="15" t="n"/>
       <c r="BE66" s="15" t="n"/>
       <c r="BF66" s="15" t="n"/>
+      <c r="BG66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -10098,6 +10255,9 @@
       </c>
       <c r="BF67" s="15" t="n">
         <v>19.68</v>
+      </c>
+      <c r="BG67" s="15" t="n">
+        <v>15.61</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -10226,6 +10386,9 @@
       </c>
       <c r="BF68" s="15" t="n">
         <v>6863.21</v>
+      </c>
+      <c r="BG68" s="15" t="n">
+        <v>6678.51</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -10335,6 +10498,7 @@
       <c r="BD69" s="15" t="n"/>
       <c r="BE69" s="15" t="n"/>
       <c r="BF69" s="15" t="n"/>
+      <c r="BG69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -10510,6 +10674,9 @@
       </c>
       <c r="BF70" s="15" t="n">
         <v>18.36</v>
+      </c>
+      <c r="BG70" s="15" t="n">
+        <v>15.11</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -10638,6 +10805,9 @@
       </c>
       <c r="BF71" s="15" t="n">
         <v>12975.39</v>
+      </c>
+      <c r="BG71" s="15" t="n">
+        <v>12623.13</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -10747,6 +10917,7 @@
       <c r="BD72" s="15" t="n"/>
       <c r="BE72" s="15" t="n"/>
       <c r="BF72" s="15" t="n"/>
+      <c r="BG72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -10922,6 +11093,9 @@
       </c>
       <c r="BF73" s="15" t="n">
         <v>53.26</v>
+      </c>
+      <c r="BG73" s="15" t="n">
+        <v>53.74</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -11050,6 +11224,9 @@
       </c>
       <c r="BF74" s="15" t="n">
         <v>13655.35</v>
+      </c>
+      <c r="BG74" s="15" t="n">
+        <v>14297.63</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -11159,6 +11336,7 @@
       <c r="BD75" s="15" t="n"/>
       <c r="BE75" s="15" t="n"/>
       <c r="BF75" s="15" t="n"/>
+      <c r="BG75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -11334,6 +11512,9 @@
       </c>
       <c r="BF76" s="15" t="n">
         <v>5.08</v>
+      </c>
+      <c r="BG76" s="15" t="n">
+        <v>6.91</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -11462,6 +11643,9 @@
       </c>
       <c r="BF77" s="15" t="n">
         <v>7319.35</v>
+      </c>
+      <c r="BG77" s="15" t="n">
+        <v>7441.91</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
@@ -11571,6 +11755,7 @@
       <c r="BD78" s="15" t="n"/>
       <c r="BE78" s="15" t="n"/>
       <c r="BF78" s="15" t="n"/>
+      <c r="BG78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -11746,6 +11931,9 @@
       </c>
       <c r="BF79" s="15" t="n">
         <v>4.96</v>
+      </c>
+      <c r="BG79" s="15" t="n">
+        <v>3.93</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -11874,6 +12062,9 @@
       </c>
       <c r="BF80" s="15" t="n">
         <v>8996.5</v>
+      </c>
+      <c r="BG80" s="15" t="n">
+        <v>8803.23</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -11983,6 +12174,7 @@
       <c r="BD81" s="15" t="n"/>
       <c r="BE81" s="15" t="n"/>
       <c r="BF81" s="15" t="n"/>
+      <c r="BG81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -12158,6 +12350,9 @@
       </c>
       <c r="BF82" s="15" t="n">
         <v>14.57</v>
+      </c>
+      <c r="BG82" s="15" t="n">
+        <v>16.18</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -12286,6 +12481,9 @@
       </c>
       <c r="BF83" s="15" t="n">
         <v>2631.9</v>
+      </c>
+      <c r="BG83" s="15" t="n">
+        <v>2406.99</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -12395,6 +12593,7 @@
       <c r="BD84" s="15" t="n"/>
       <c r="BE84" s="15" t="n"/>
       <c r="BF84" s="15" t="n"/>
+      <c r="BG84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -12570,6 +12769,9 @@
       </c>
       <c r="BF85" s="15" t="n">
         <v>28.41</v>
+      </c>
+      <c r="BG85" s="15" t="n">
+        <v>31.54</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -12698,6 +12900,9 @@
       </c>
       <c r="BF86" s="15" t="n">
         <v>4857.7</v>
+      </c>
+      <c r="BG86" s="15" t="n">
+        <v>5075.31</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -12807,6 +13012,7 @@
       <c r="BD87" s="15" t="n"/>
       <c r="BE87" s="15" t="n"/>
       <c r="BF87" s="15" t="n"/>
+      <c r="BG87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -12982,6 +13188,9 @@
       </c>
       <c r="BF88" s="15" t="n">
         <v>21.9</v>
+      </c>
+      <c r="BG88" s="15" t="n">
+        <v>23.09</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -13110,6 +13319,9 @@
       </c>
       <c r="BF89" s="15" t="n">
         <v>8449.16</v>
+      </c>
+      <c r="BG89" s="15" t="n">
+        <v>8551.719999999999</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -13219,6 +13431,7 @@
       <c r="BD90" s="15" t="n"/>
       <c r="BE90" s="15" t="n"/>
       <c r="BF90" s="15" t="n"/>
+      <c r="BG90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -13394,6 +13607,9 @@
       </c>
       <c r="BF91" s="15" t="n">
         <v>7</v>
+      </c>
+      <c r="BG91" s="15" t="n">
+        <v>6.12</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -13522,6 +13738,9 @@
       </c>
       <c r="BF92" s="15" t="n">
         <v>1218.35</v>
+      </c>
+      <c r="BG92" s="15" t="n">
+        <v>1198.71</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -13631,6 +13850,7 @@
       <c r="BD93" s="15" t="n"/>
       <c r="BE93" s="15" t="n"/>
       <c r="BF93" s="15" t="n"/>
+      <c r="BG93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -13806,6 +14026,9 @@
       </c>
       <c r="BF94" s="15" t="n">
         <v>8.619999999999999</v>
+      </c>
+      <c r="BG94" s="15" t="n">
+        <v>7.17</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -13934,6 +14157,9 @@
       </c>
       <c r="BF95" s="15" t="n">
         <v>14532.99</v>
+      </c>
+      <c r="BG95" s="15" t="n">
+        <v>14147.93</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -14043,6 +14269,7 @@
       <c r="BD96" s="15" t="n"/>
       <c r="BE96" s="15" t="n"/>
       <c r="BF96" s="15" t="n"/>
+      <c r="BG96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -14218,6 +14445,9 @@
       </c>
       <c r="BF97" s="15" t="n">
         <v>44.05</v>
+      </c>
+      <c r="BG97" s="15" t="n">
+        <v>45.81</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -14346,6 +14576,9 @@
       </c>
       <c r="BF98" s="15" t="n">
         <v>3162.76</v>
+      </c>
+      <c r="BG98" s="15" t="n">
+        <v>3243.66</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -14455,6 +14688,7 @@
       <c r="BD99" s="15" t="n"/>
       <c r="BE99" s="15" t="n"/>
       <c r="BF99" s="15" t="n"/>
+      <c r="BG99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -14630,6 +14864,9 @@
       </c>
       <c r="BF100" s="15" t="n">
         <v>36.08</v>
+      </c>
+      <c r="BG100" s="15" t="n">
+        <v>39.09</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -14758,6 +14995,9 @@
       </c>
       <c r="BF101" s="15" t="n">
         <v>2384.92</v>
+      </c>
+      <c r="BG101" s="15" t="n">
+        <v>2429.82</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -14867,6 +15107,7 @@
       <c r="BD102" s="15" t="n"/>
       <c r="BE102" s="15" t="n"/>
       <c r="BF102" s="15" t="n"/>
+      <c r="BG102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -15042,6 +15283,9 @@
       </c>
       <c r="BF103" s="15" t="n">
         <v>14.05</v>
+      </c>
+      <c r="BG103" s="15" t="n">
+        <v>16.68</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -15170,6 +15414,9 @@
       </c>
       <c r="BF104" s="15" t="n">
         <v>2444.22</v>
+      </c>
+      <c r="BG104" s="15" t="n">
+        <v>2483.41</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -15279,6 +15526,7 @@
       <c r="BD105" s="15" t="n"/>
       <c r="BE105" s="15" t="n"/>
       <c r="BF105" s="15" t="n"/>
+      <c r="BG105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -15454,6 +15702,9 @@
       </c>
       <c r="BF106" s="15" t="n">
         <v>0</v>
+      </c>
+      <c r="BG106" s="15" t="n">
+        <v>39.17</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -15582,6 +15833,9 @@
       </c>
       <c r="BF107" s="15" t="n">
         <v>2573.31</v>
+      </c>
+      <c r="BG107" s="15" t="n">
+        <v>2598.34</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -15691,6 +15945,7 @@
       <c r="BD108" s="15" t="n"/>
       <c r="BE108" s="15" t="n"/>
       <c r="BF108" s="15" t="n"/>
+      <c r="BG108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -15866,6 +16121,9 @@
       </c>
       <c r="BF109" s="15" t="n">
         <v>57</v>
+      </c>
+      <c r="BG109" s="15" t="n">
+        <v>59.95</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -15994,6 +16252,9 @@
       </c>
       <c r="BF110" s="15" t="n">
         <v>1898.59</v>
+      </c>
+      <c r="BG110" s="15" t="n">
+        <v>1918.14</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -16103,6 +16364,7 @@
       <c r="BD111" s="15" t="n"/>
       <c r="BE111" s="15" t="n"/>
       <c r="BF111" s="15" t="n"/>
+      <c r="BG111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -16278,6 +16540,9 @@
       </c>
       <c r="BF112" s="15" t="n">
         <v>22.54</v>
+      </c>
+      <c r="BG112" s="15" t="n">
+        <v>22.7</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -16407,6 +16672,7 @@
       <c r="BF113" s="15" t="n">
         <v>8486.91</v>
       </c>
+      <c r="BG113" s="15" t="inlineStr"/>
     </row>
     <row r="114" ht="14.25" customHeight="1">
       <c r="A114" s="3" t="n">
@@ -16515,6 +16781,7 @@
       <c r="BD114" s="15" t="n"/>
       <c r="BE114" s="15" t="n"/>
       <c r="BF114" s="15" t="n"/>
+      <c r="BG114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -16690,6 +16957,9 @@
       </c>
       <c r="BF115" s="15" t="n">
         <v>93.19</v>
+      </c>
+      <c r="BG115" s="15" t="n">
+        <v>94.78</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -16803,6 +17073,9 @@
       </c>
       <c r="BF116" s="15" t="n">
         <v>11627.83</v>
+      </c>
+      <c r="BG116" s="15" t="n">
+        <v>13072.56</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -16867,6 +17140,7 @@
       <c r="BD117" s="15" t="n"/>
       <c r="BE117" s="15" t="n"/>
       <c r="BF117" s="15" t="n"/>
+      <c r="BG117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -16998,6 +17272,9 @@
       <c r="BF118" s="15" t="n">
         <v>31.69</v>
       </c>
+      <c r="BG118" s="15" t="n">
+        <v>36.7</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -17101,6 +17378,9 @@
       </c>
       <c r="BF119" s="15" t="n">
         <v>1243.02</v>
+      </c>
+      <c r="BG119" s="15" t="n">
+        <v>1300.63</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -17114,6 +17394,7 @@
       <c r="BD120" s="15" t="n"/>
       <c r="BE120" s="15" t="n"/>
       <c r="BF120" s="15" t="n"/>
+      <c r="BG120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -17146,6 +17427,9 @@
       <c r="BF121" s="15" t="n">
         <v>42.69</v>
       </c>
+      <c r="BG121" s="15" t="n">
+        <v>49.41</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -17177,6 +17461,9 @@
       </c>
       <c r="BF122" s="15" t="n">
         <v>11146.58</v>
+      </c>
+      <c r="BG122" s="15" t="n">
+        <v>11444.18</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -17190,6 +17477,7 @@
       <c r="BD123" s="15" t="n"/>
       <c r="BE123" s="15" t="n"/>
       <c r="BF123" s="15" t="n"/>
+      <c r="BG123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -17222,6 +17510,9 @@
       <c r="BF124" s="15" t="n">
         <v>28.34</v>
       </c>
+      <c r="BG124" s="15" t="n">
+        <v>27.59</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -17253,6 +17544,9 @@
       </c>
       <c r="BF125" s="15" t="n">
         <v>1864.85</v>
+      </c>
+      <c r="BG125" s="15" t="n">
+        <v>1857.71</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -17266,6 +17560,7 @@
       <c r="BD126" s="15" t="n"/>
       <c r="BE126" s="15" t="n"/>
       <c r="BF126" s="15" t="n"/>
+      <c r="BG126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -17298,6 +17593,9 @@
       <c r="BF127" s="15" t="n">
         <v>14.68</v>
       </c>
+      <c r="BG127" s="15" t="n">
+        <v>15.05</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -17329,6 +17627,9 @@
       </c>
       <c r="BF128" s="15" t="n">
         <v>769.83</v>
+      </c>
+      <c r="BG128" s="15" t="n">
+        <v>764.42</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -17342,6 +17643,7 @@
       <c r="BD129" s="15" t="n"/>
       <c r="BE129" s="15" t="n"/>
       <c r="BF129" s="15" t="n"/>
+      <c r="BG129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -17374,6 +17676,9 @@
       <c r="BF130" s="15" t="n">
         <v>63.65</v>
       </c>
+      <c r="BG130" s="15" t="n">
+        <v>70.63</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -17405,6 +17710,9 @@
       </c>
       <c r="BF131" s="15" t="n">
         <v>2815.99</v>
+      </c>
+      <c r="BG131" s="15" t="n">
+        <v>3014.01</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -17418,6 +17726,7 @@
       <c r="BD132" s="15" t="n"/>
       <c r="BE132" s="15" t="n"/>
       <c r="BF132" s="15" t="n"/>
+      <c r="BG132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -17450,6 +17759,9 @@
       <c r="BF133" s="15" t="n">
         <v>20.84</v>
       </c>
+      <c r="BG133" s="15" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -17481,6 +17793,9 @@
       </c>
       <c r="BF134" s="15" t="n">
         <v>3576.02</v>
+      </c>
+      <c r="BG134" s="15" t="n">
+        <v>3605.55</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -17494,6 +17809,7 @@
       <c r="BD135" s="15" t="n"/>
       <c r="BE135" s="15" t="n"/>
       <c r="BF135" s="15" t="n"/>
+      <c r="BG135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -17526,6 +17842,9 @@
       <c r="BF136" s="15" t="n">
         <v>2.43</v>
       </c>
+      <c r="BG136" s="15" t="n">
+        <v>2.67</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -17558,10 +17877,14 @@
       <c r="BF137" s="15" t="n">
         <v>2350.74</v>
       </c>
+      <c r="BG137" s="15" t="n">
+        <v>2402.55</v>
+      </c>
     </row>
     <row r="138">
       <c r="BE138" s="15" t="n"/>
       <c r="BF138" s="15" t="n"/>
+      <c r="BG138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -17570,6 +17893,9 @@
       <c r="BF139" s="15" t="n">
         <v>8.960000000000001</v>
       </c>
+      <c r="BG139" s="15" t="n">
+        <v>11.2</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -17578,10 +17904,14 @@
       <c r="BF140" s="15" t="n">
         <v>5375.74</v>
       </c>
+      <c r="BG140" s="15" t="n">
+        <v>5572.78</v>
+      </c>
     </row>
     <row r="141">
       <c r="BE141" s="15" t="n"/>
       <c r="BF141" s="15" t="n"/>
+      <c r="BG141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -17590,6 +17920,9 @@
       <c r="BF142" s="15" t="n">
         <v>25.87</v>
       </c>
+      <c r="BG142" s="15" t="n">
+        <v>25.79</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -17597,6 +17930,9 @@
       </c>
       <c r="BF143" s="15" t="n">
         <v>2353.44</v>
+      </c>
+      <c r="BG143" s="15" t="n">
+        <v>2338.52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-08-10 05:11:30]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BG143"/>
+  <dimension ref="A1:BH143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -593,6 +593,7 @@
     <col width="15" customWidth="1" min="57" max="57"/>
     <col width="15" customWidth="1" min="58" max="58"/>
     <col width="15" customWidth="1" min="59" max="59"/>
+    <col width="15" customWidth="1" min="60" max="60"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -891,6 +892,11 @@
           <t>2026/08/06</t>
         </is>
       </c>
+      <c r="BH1" s="15" t="inlineStr">
+        <is>
+          <t>2026/08/10</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1188,6 +1194,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BH2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1367,6 +1378,9 @@
       <c r="BG3" s="15" t="n">
         <v>62.6</v>
       </c>
+      <c r="BH3" s="15" t="n">
+        <v>64.02</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1545,6 +1559,9 @@
       </c>
       <c r="BG4" s="15" t="n">
         <v>3881.78</v>
+      </c>
+      <c r="BH4" s="15" t="n">
+        <v>3946.93</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1607,6 +1624,7 @@
       <c r="BE5" s="15" t="n"/>
       <c r="BF5" s="15" t="n"/>
       <c r="BG5" s="15" t="n"/>
+      <c r="BH5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1716,6 +1734,7 @@
       <c r="BE6" s="15" t="n"/>
       <c r="BF6" s="15" t="n"/>
       <c r="BG6" s="15" t="n"/>
+      <c r="BH6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1894,6 +1913,9 @@
       </c>
       <c r="BG7" s="15" t="n">
         <v>62.27</v>
+      </c>
+      <c r="BH7" s="15" t="n">
+        <v>65.19</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -2025,6 +2047,9 @@
       </c>
       <c r="BG8" s="15" t="n">
         <v>5716.01</v>
+      </c>
+      <c r="BH8" s="15" t="n">
+        <v>5793.73</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2135,6 +2160,7 @@
       <c r="BE9" s="15" t="n"/>
       <c r="BF9" s="15" t="n"/>
       <c r="BG9" s="15" t="n"/>
+      <c r="BH9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2313,6 +2339,9 @@
       </c>
       <c r="BG10" s="15" t="n">
         <v>55.62</v>
+      </c>
+      <c r="BH10" s="15" t="n">
+        <v>57</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2444,6 +2473,9 @@
       </c>
       <c r="BG11" s="15" t="n">
         <v>4626.78</v>
+      </c>
+      <c r="BH11" s="15" t="n">
+        <v>4670.53</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -2554,6 +2586,7 @@
       <c r="BE12" s="15" t="n"/>
       <c r="BF12" s="15" t="n"/>
       <c r="BG12" s="15" t="n"/>
+      <c r="BH12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2732,6 +2765,9 @@
       </c>
       <c r="BG13" s="15" t="n">
         <v>65.56</v>
+      </c>
+      <c r="BH13" s="15" t="n">
+        <v>67.12</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -2863,6 +2899,9 @@
       </c>
       <c r="BG14" s="15" t="n">
         <v>7757.44</v>
+      </c>
+      <c r="BH14" s="15" t="n">
+        <v>7941.06</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -2973,6 +3012,7 @@
       <c r="BE15" s="15" t="n"/>
       <c r="BF15" s="15" t="n"/>
       <c r="BG15" s="15" t="n"/>
+      <c r="BH15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -3151,6 +3191,9 @@
       </c>
       <c r="BG16" s="15" t="n">
         <v>35.5</v>
+      </c>
+      <c r="BH16" s="15" t="n">
+        <v>36.65</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -3282,6 +3325,9 @@
       </c>
       <c r="BG17" s="15" t="n">
         <v>2594.58</v>
+      </c>
+      <c r="BH17" s="15" t="n">
+        <v>2623.4</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -3392,6 +3438,7 @@
       <c r="BE18" s="15" t="n"/>
       <c r="BF18" s="15" t="n"/>
       <c r="BG18" s="15" t="n"/>
+      <c r="BH18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -3570,6 +3617,9 @@
       </c>
       <c r="BG19" s="15" t="n">
         <v>82.34999999999999</v>
+      </c>
+      <c r="BH19" s="15" t="n">
+        <v>82.09</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -3701,6 +3751,9 @@
       </c>
       <c r="BG20" s="15" t="n">
         <v>7723.55</v>
+      </c>
+      <c r="BH20" s="15" t="n">
+        <v>7757.64</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -3811,6 +3864,7 @@
       <c r="BE21" s="15" t="n"/>
       <c r="BF21" s="15" t="n"/>
       <c r="BG21" s="15" t="n"/>
+      <c r="BH21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -3986,6 +4040,9 @@
         <v>36.34</v>
       </c>
       <c r="BG22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BH22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -4118,6 +4175,9 @@
       </c>
       <c r="BG23" s="15" t="n">
         <v>78859.21000000001</v>
+      </c>
+      <c r="BH23" s="15" t="n">
+        <v>78561.49000000001</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -4228,6 +4288,7 @@
       <c r="BE24" s="15" t="n"/>
       <c r="BF24" s="15" t="n"/>
       <c r="BG24" s="15" t="n"/>
+      <c r="BH24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -4405,6 +4466,9 @@
         <v>49.88</v>
       </c>
       <c r="BG25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BH25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -4524,6 +4588,9 @@
         <v>25629.24</v>
       </c>
       <c r="BG26" s="15" t="inlineStr"/>
+      <c r="BH26" s="15" t="n">
+        <v>26319.45</v>
+      </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -4633,6 +4700,7 @@
       <c r="BE27" s="15" t="n"/>
       <c r="BF27" s="15" t="n"/>
       <c r="BG27" s="15" t="n"/>
+      <c r="BH27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -4810,6 +4878,9 @@
         <v>92.09</v>
       </c>
       <c r="BG28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BH28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -4942,6 +5013,9 @@
       </c>
       <c r="BG29" s="15" t="n">
         <v>65678.78999999999</v>
+      </c>
+      <c r="BH29" s="15" t="n">
+        <v>66863.55</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -5052,6 +5126,7 @@
       <c r="BE30" s="15" t="n"/>
       <c r="BF30" s="15" t="n"/>
       <c r="BG30" s="15" t="n"/>
+      <c r="BH30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -5230,6 +5305,9 @@
       </c>
       <c r="BG31" s="15" t="n">
         <v>45.43</v>
+      </c>
+      <c r="BH31" s="15" t="n">
+        <v>45.66</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -5361,6 +5439,9 @@
       </c>
       <c r="BG32" s="15" t="n">
         <v>5526.25</v>
+      </c>
+      <c r="BH32" s="15" t="n">
+        <v>5569.2</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -5471,6 +5552,7 @@
       <c r="BE33" s="15" t="n"/>
       <c r="BF33" s="15" t="n"/>
       <c r="BG33" s="15" t="n"/>
+      <c r="BH33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -5649,6 +5731,9 @@
       </c>
       <c r="BG34" s="15" t="n">
         <v>58.75</v>
+      </c>
+      <c r="BH34" s="15" t="n">
+        <v>58.68</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -5780,6 +5865,9 @@
       </c>
       <c r="BG35" s="15" t="n">
         <v>11306.07</v>
+      </c>
+      <c r="BH35" s="15" t="n">
+        <v>11291.49</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -5890,6 +5978,7 @@
       <c r="BE36" s="15" t="n"/>
       <c r="BF36" s="15" t="n"/>
       <c r="BG36" s="15" t="n"/>
+      <c r="BH36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -6068,6 +6157,9 @@
       </c>
       <c r="BG37" s="15" t="n">
         <v>49.75</v>
+      </c>
+      <c r="BH37" s="15" t="n">
+        <v>50.05</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -6199,6 +6291,9 @@
       </c>
       <c r="BG38" s="15" t="n">
         <v>10766.13</v>
+      </c>
+      <c r="BH38" s="15" t="n">
+        <v>10715.06</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -6309,6 +6404,7 @@
       <c r="BE39" s="15" t="n"/>
       <c r="BF39" s="15" t="n"/>
       <c r="BG39" s="15" t="n"/>
+      <c r="BH39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -6487,6 +6583,9 @@
       </c>
       <c r="BG40" s="15" t="n">
         <v>49.12</v>
+      </c>
+      <c r="BH40" s="15" t="n">
+        <v>49.92</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -6618,6 +6717,9 @@
       </c>
       <c r="BG41" s="15" t="n">
         <v>3141.46</v>
+      </c>
+      <c r="BH41" s="15" t="n">
+        <v>3197.71</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -6728,6 +6830,7 @@
       <c r="BE42" s="15" t="n"/>
       <c r="BF42" s="15" t="n"/>
       <c r="BG42" s="15" t="n"/>
+      <c r="BH42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -6906,6 +7009,9 @@
       </c>
       <c r="BG43" s="15" t="n">
         <v>57.33</v>
+      </c>
+      <c r="BH43" s="15" t="n">
+        <v>58.97</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -7037,6 +7143,9 @@
       </c>
       <c r="BG44" s="15" t="n">
         <v>6944.22</v>
+      </c>
+      <c r="BH44" s="15" t="n">
+        <v>6884.36</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -7147,6 +7256,7 @@
       <c r="BE45" s="15" t="n"/>
       <c r="BF45" s="15" t="n"/>
       <c r="BG45" s="15" t="n"/>
+      <c r="BH45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -7325,6 +7435,9 @@
       </c>
       <c r="BG46" s="15" t="n">
         <v>27.08</v>
+      </c>
+      <c r="BH46" s="15" t="n">
+        <v>29.75</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -7456,6 +7569,9 @@
       </c>
       <c r="BG47" s="15" t="n">
         <v>33503.52</v>
+      </c>
+      <c r="BH47" s="15" t="n">
+        <v>34417.12</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -7566,6 +7682,7 @@
       <c r="BE48" s="15" t="n"/>
       <c r="BF48" s="15" t="n"/>
       <c r="BG48" s="15" t="n"/>
+      <c r="BH48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -7744,6 +7861,9 @@
       </c>
       <c r="BG49" s="15" t="n">
         <v>48.97</v>
+      </c>
+      <c r="BH49" s="15" t="n">
+        <v>49.02</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -7875,6 +7995,9 @@
       </c>
       <c r="BG50" s="15" t="n">
         <v>3674.04</v>
+      </c>
+      <c r="BH50" s="15" t="n">
+        <v>3631.6</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -7985,6 +8108,7 @@
       <c r="BE51" s="15" t="n"/>
       <c r="BF51" s="15" t="n"/>
       <c r="BG51" s="15" t="n"/>
+      <c r="BH51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -8163,6 +8287,9 @@
       </c>
       <c r="BG52" s="15" t="n">
         <v>59.21</v>
+      </c>
+      <c r="BH52" s="15" t="n">
+        <v>60.23</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -8294,6 +8421,9 @@
       </c>
       <c r="BG53" s="15" t="n">
         <v>3486.45</v>
+      </c>
+      <c r="BH53" s="15" t="n">
+        <v>3486.72</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -8404,6 +8534,7 @@
       <c r="BE54" s="15" t="n"/>
       <c r="BF54" s="15" t="n"/>
       <c r="BG54" s="15" t="n"/>
+      <c r="BH54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -8582,6 +8713,9 @@
       </c>
       <c r="BG55" s="15" t="n">
         <v>14.69</v>
+      </c>
+      <c r="BH55" s="15" t="n">
+        <v>18.15</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -8713,6 +8847,9 @@
       </c>
       <c r="BG56" s="15" t="n">
         <v>6550.13</v>
+      </c>
+      <c r="BH56" s="15" t="n">
+        <v>6962.91</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -8823,6 +8960,7 @@
       <c r="BE57" s="15" t="n"/>
       <c r="BF57" s="15" t="n"/>
       <c r="BG57" s="15" t="n"/>
+      <c r="BH57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -9001,6 +9139,9 @@
       </c>
       <c r="BG58" s="15" t="n">
         <v>36.06</v>
+      </c>
+      <c r="BH58" s="15" t="n">
+        <v>39.99</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -9132,6 +9273,9 @@
       </c>
       <c r="BG59" s="15" t="n">
         <v>8167.59</v>
+      </c>
+      <c r="BH59" s="15" t="n">
+        <v>8679.719999999999</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -9242,6 +9386,7 @@
       <c r="BE60" s="15" t="n"/>
       <c r="BF60" s="15" t="n"/>
       <c r="BG60" s="15" t="n"/>
+      <c r="BH60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -9420,6 +9565,9 @@
       </c>
       <c r="BG61" s="15" t="n">
         <v>4.17</v>
+      </c>
+      <c r="BH61" s="15" t="n">
+        <v>3.55</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -9551,6 +9699,9 @@
       </c>
       <c r="BG62" s="15" t="n">
         <v>10898.57</v>
+      </c>
+      <c r="BH62" s="15" t="n">
+        <v>11034.71</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -9661,6 +9812,7 @@
       <c r="BE63" s="15" t="n"/>
       <c r="BF63" s="15" t="n"/>
       <c r="BG63" s="15" t="n"/>
+      <c r="BH63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -9839,6 +9991,9 @@
       </c>
       <c r="BG64" s="15" t="n">
         <v>21.93</v>
+      </c>
+      <c r="BH64" s="15" t="n">
+        <v>19.46</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -9969,6 +10124,9 @@
         <v>11328.53</v>
       </c>
       <c r="BG65" s="15" t="n">
+        <v>11368.1</v>
+      </c>
+      <c r="BH65" s="15" t="n">
         <v>11368.1</v>
       </c>
     </row>
@@ -10080,6 +10238,7 @@
       <c r="BE66" s="15" t="n"/>
       <c r="BF66" s="15" t="n"/>
       <c r="BG66" s="15" t="n"/>
+      <c r="BH66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -10258,6 +10417,9 @@
       </c>
       <c r="BG67" s="15" t="n">
         <v>15.61</v>
+      </c>
+      <c r="BH67" s="15" t="n">
+        <v>15.7</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -10389,6 +10551,9 @@
       </c>
       <c r="BG68" s="15" t="n">
         <v>6678.51</v>
+      </c>
+      <c r="BH68" s="15" t="n">
+        <v>6908.63</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -10499,6 +10664,7 @@
       <c r="BE69" s="15" t="n"/>
       <c r="BF69" s="15" t="n"/>
       <c r="BG69" s="15" t="n"/>
+      <c r="BH69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -10677,6 +10843,9 @@
       </c>
       <c r="BG70" s="15" t="n">
         <v>15.11</v>
+      </c>
+      <c r="BH70" s="15" t="n">
+        <v>15.07</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -10808,6 +10977,9 @@
       </c>
       <c r="BG71" s="15" t="n">
         <v>12623.13</v>
+      </c>
+      <c r="BH71" s="15" t="n">
+        <v>12964.85</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -10918,6 +11090,7 @@
       <c r="BE72" s="15" t="n"/>
       <c r="BF72" s="15" t="n"/>
       <c r="BG72" s="15" t="n"/>
+      <c r="BH72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -11096,6 +11269,9 @@
       </c>
       <c r="BG73" s="15" t="n">
         <v>53.74</v>
+      </c>
+      <c r="BH73" s="15" t="n">
+        <v>55.12</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -11227,6 +11403,9 @@
       </c>
       <c r="BG74" s="15" t="n">
         <v>14297.63</v>
+      </c>
+      <c r="BH74" s="15" t="n">
+        <v>15569.82</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -11337,6 +11516,7 @@
       <c r="BE75" s="15" t="n"/>
       <c r="BF75" s="15" t="n"/>
       <c r="BG75" s="15" t="n"/>
+      <c r="BH75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -11515,6 +11695,9 @@
       </c>
       <c r="BG76" s="15" t="n">
         <v>6.91</v>
+      </c>
+      <c r="BH76" s="15" t="n">
+        <v>5.71</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -11646,6 +11829,9 @@
       </c>
       <c r="BG77" s="15" t="n">
         <v>7441.91</v>
+      </c>
+      <c r="BH77" s="15" t="n">
+        <v>7439.15</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
@@ -11756,6 +11942,7 @@
       <c r="BE78" s="15" t="n"/>
       <c r="BF78" s="15" t="n"/>
       <c r="BG78" s="15" t="n"/>
+      <c r="BH78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -11934,6 +12121,9 @@
       </c>
       <c r="BG79" s="15" t="n">
         <v>3.93</v>
+      </c>
+      <c r="BH79" s="15" t="n">
+        <v>4.37</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -12065,6 +12255,9 @@
       </c>
       <c r="BG80" s="15" t="n">
         <v>8803.23</v>
+      </c>
+      <c r="BH80" s="15" t="n">
+        <v>8970.24</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -12175,6 +12368,7 @@
       <c r="BE81" s="15" t="n"/>
       <c r="BF81" s="15" t="n"/>
       <c r="BG81" s="15" t="n"/>
+      <c r="BH81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -12353,6 +12547,9 @@
       </c>
       <c r="BG82" s="15" t="n">
         <v>16.18</v>
+      </c>
+      <c r="BH82" s="15" t="n">
+        <v>15.22</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -12484,6 +12681,9 @@
       </c>
       <c r="BG83" s="15" t="n">
         <v>2406.99</v>
+      </c>
+      <c r="BH83" s="15" t="n">
+        <v>2424.82</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -12594,6 +12794,7 @@
       <c r="BE84" s="15" t="n"/>
       <c r="BF84" s="15" t="n"/>
       <c r="BG84" s="15" t="n"/>
+      <c r="BH84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -12772,6 +12973,9 @@
       </c>
       <c r="BG85" s="15" t="n">
         <v>31.54</v>
+      </c>
+      <c r="BH85" s="15" t="n">
+        <v>30.44</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -12903,6 +13107,9 @@
       </c>
       <c r="BG86" s="15" t="n">
         <v>5075.31</v>
+      </c>
+      <c r="BH86" s="15" t="n">
+        <v>4876.2</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -13013,6 +13220,7 @@
       <c r="BE87" s="15" t="n"/>
       <c r="BF87" s="15" t="n"/>
       <c r="BG87" s="15" t="n"/>
+      <c r="BH87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -13191,6 +13399,9 @@
       </c>
       <c r="BG88" s="15" t="n">
         <v>23.09</v>
+      </c>
+      <c r="BH88" s="15" t="n">
+        <v>28.71</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -13322,6 +13533,9 @@
       </c>
       <c r="BG89" s="15" t="n">
         <v>8551.719999999999</v>
+      </c>
+      <c r="BH89" s="15" t="n">
+        <v>9047.34</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -13432,6 +13646,7 @@
       <c r="BE90" s="15" t="n"/>
       <c r="BF90" s="15" t="n"/>
       <c r="BG90" s="15" t="n"/>
+      <c r="BH90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -13610,6 +13825,9 @@
       </c>
       <c r="BG91" s="15" t="n">
         <v>6.12</v>
+      </c>
+      <c r="BH91" s="15" t="n">
+        <v>5.43</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -13741,6 +13959,9 @@
       </c>
       <c r="BG92" s="15" t="n">
         <v>1198.71</v>
+      </c>
+      <c r="BH92" s="15" t="n">
+        <v>1183.83</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -13851,6 +14072,7 @@
       <c r="BE93" s="15" t="n"/>
       <c r="BF93" s="15" t="n"/>
       <c r="BG93" s="15" t="n"/>
+      <c r="BH93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -14029,6 +14251,9 @@
       </c>
       <c r="BG94" s="15" t="n">
         <v>7.17</v>
+      </c>
+      <c r="BH94" s="15" t="n">
+        <v>7.29</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -14160,6 +14385,9 @@
       </c>
       <c r="BG95" s="15" t="n">
         <v>14147.93</v>
+      </c>
+      <c r="BH95" s="15" t="n">
+        <v>14131.94</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -14270,6 +14498,7 @@
       <c r="BE96" s="15" t="n"/>
       <c r="BF96" s="15" t="n"/>
       <c r="BG96" s="15" t="n"/>
+      <c r="BH96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -14448,6 +14677,9 @@
       </c>
       <c r="BG97" s="15" t="n">
         <v>45.81</v>
+      </c>
+      <c r="BH97" s="15" t="n">
+        <v>51.45</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -14579,6 +14811,9 @@
       </c>
       <c r="BG98" s="15" t="n">
         <v>3243.66</v>
+      </c>
+      <c r="BH98" s="15" t="n">
+        <v>3370.1</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -14689,6 +14924,7 @@
       <c r="BE99" s="15" t="n"/>
       <c r="BF99" s="15" t="n"/>
       <c r="BG99" s="15" t="n"/>
+      <c r="BH99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -14867,6 +15103,9 @@
       </c>
       <c r="BG100" s="15" t="n">
         <v>39.09</v>
+      </c>
+      <c r="BH100" s="15" t="n">
+        <v>38.09</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -14998,6 +15237,9 @@
       </c>
       <c r="BG101" s="15" t="n">
         <v>2429.82</v>
+      </c>
+      <c r="BH101" s="15" t="n">
+        <v>2482.15</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -15108,6 +15350,7 @@
       <c r="BE102" s="15" t="n"/>
       <c r="BF102" s="15" t="n"/>
       <c r="BG102" s="15" t="n"/>
+      <c r="BH102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -15286,6 +15529,9 @@
       </c>
       <c r="BG103" s="15" t="n">
         <v>16.68</v>
+      </c>
+      <c r="BH103" s="15" t="n">
+        <v>17.15</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -15417,6 +15663,9 @@
       </c>
       <c r="BG104" s="15" t="n">
         <v>2483.41</v>
+      </c>
+      <c r="BH104" s="15" t="n">
+        <v>2494.23</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -15527,6 +15776,7 @@
       <c r="BE105" s="15" t="n"/>
       <c r="BF105" s="15" t="n"/>
       <c r="BG105" s="15" t="n"/>
+      <c r="BH105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -15705,6 +15955,9 @@
       </c>
       <c r="BG106" s="15" t="n">
         <v>39.17</v>
+      </c>
+      <c r="BH106" s="15" t="n">
+        <v>38.13</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -15835,6 +16088,9 @@
         <v>2573.31</v>
       </c>
       <c r="BG107" s="15" t="n">
+        <v>2598.34</v>
+      </c>
+      <c r="BH107" s="15" t="n">
         <v>2598.34</v>
       </c>
     </row>
@@ -15946,6 +16202,7 @@
       <c r="BE108" s="15" t="n"/>
       <c r="BF108" s="15" t="n"/>
       <c r="BG108" s="15" t="n"/>
+      <c r="BH108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -16124,6 +16381,9 @@
       </c>
       <c r="BG109" s="15" t="n">
         <v>59.95</v>
+      </c>
+      <c r="BH109" s="15" t="n">
+        <v>66.81999999999999</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -16255,6 +16515,9 @@
       </c>
       <c r="BG110" s="15" t="n">
         <v>1918.14</v>
+      </c>
+      <c r="BH110" s="15" t="n">
+        <v>2057.72</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -16365,6 +16628,7 @@
       <c r="BE111" s="15" t="n"/>
       <c r="BF111" s="15" t="n"/>
       <c r="BG111" s="15" t="n"/>
+      <c r="BH111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -16543,6 +16807,9 @@
       </c>
       <c r="BG112" s="15" t="n">
         <v>22.7</v>
+      </c>
+      <c r="BH112" s="15" t="n">
+        <v>23.65</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -16673,6 +16940,9 @@
         <v>8486.91</v>
       </c>
       <c r="BG113" s="15" t="inlineStr"/>
+      <c r="BH113" s="15" t="n">
+        <v>8939.18</v>
+      </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
       <c r="A114" s="3" t="n">
@@ -16782,6 +17052,7 @@
       <c r="BE114" s="15" t="n"/>
       <c r="BF114" s="15" t="n"/>
       <c r="BG114" s="15" t="n"/>
+      <c r="BH114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -16960,6 +17231,9 @@
       </c>
       <c r="BG115" s="15" t="n">
         <v>94.78</v>
+      </c>
+      <c r="BH115" s="15" t="n">
+        <v>96.03</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -17076,6 +17350,9 @@
       </c>
       <c r="BG116" s="15" t="n">
         <v>13072.56</v>
+      </c>
+      <c r="BH116" s="15" t="n">
+        <v>13403.42</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -17141,6 +17418,7 @@
       <c r="BE117" s="15" t="n"/>
       <c r="BF117" s="15" t="n"/>
       <c r="BG117" s="15" t="n"/>
+      <c r="BH117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -17275,6 +17553,9 @@
       <c r="BG118" s="15" t="n">
         <v>36.7</v>
       </c>
+      <c r="BH118" s="15" t="n">
+        <v>34.3</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -17381,6 +17662,9 @@
       </c>
       <c r="BG119" s="15" t="n">
         <v>1300.63</v>
+      </c>
+      <c r="BH119" s="15" t="n">
+        <v>1278.85</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -17395,6 +17679,7 @@
       <c r="BE120" s="15" t="n"/>
       <c r="BF120" s="15" t="n"/>
       <c r="BG120" s="15" t="n"/>
+      <c r="BH120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -17430,6 +17715,9 @@
       <c r="BG121" s="15" t="n">
         <v>49.41</v>
       </c>
+      <c r="BH121" s="15" t="n">
+        <v>51.17</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -17464,6 +17752,9 @@
       </c>
       <c r="BG122" s="15" t="n">
         <v>11444.18</v>
+      </c>
+      <c r="BH122" s="15" t="n">
+        <v>11672.22</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -17478,6 +17769,7 @@
       <c r="BE123" s="15" t="n"/>
       <c r="BF123" s="15" t="n"/>
       <c r="BG123" s="15" t="n"/>
+      <c r="BH123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -17513,6 +17805,9 @@
       <c r="BG124" s="15" t="n">
         <v>27.59</v>
       </c>
+      <c r="BH124" s="15" t="n">
+        <v>27.49</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -17547,6 +17842,9 @@
       </c>
       <c r="BG125" s="15" t="n">
         <v>1857.71</v>
+      </c>
+      <c r="BH125" s="15" t="n">
+        <v>1839.6</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -17561,6 +17859,7 @@
       <c r="BE126" s="15" t="n"/>
       <c r="BF126" s="15" t="n"/>
       <c r="BG126" s="15" t="n"/>
+      <c r="BH126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -17596,6 +17895,9 @@
       <c r="BG127" s="15" t="n">
         <v>15.05</v>
       </c>
+      <c r="BH127" s="15" t="n">
+        <v>14.49</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -17630,6 +17932,9 @@
       </c>
       <c r="BG128" s="15" t="n">
         <v>764.42</v>
+      </c>
+      <c r="BH128" s="15" t="n">
+        <v>764.2</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -17644,6 +17949,7 @@
       <c r="BE129" s="15" t="n"/>
       <c r="BF129" s="15" t="n"/>
       <c r="BG129" s="15" t="n"/>
+      <c r="BH129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -17679,6 +17985,9 @@
       <c r="BG130" s="15" t="n">
         <v>70.63</v>
       </c>
+      <c r="BH130" s="15" t="n">
+        <v>74.37</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -17713,6 +18022,9 @@
       </c>
       <c r="BG131" s="15" t="n">
         <v>3014.01</v>
+      </c>
+      <c r="BH131" s="15" t="n">
+        <v>3146.97</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -17727,6 +18039,7 @@
       <c r="BE132" s="15" t="n"/>
       <c r="BF132" s="15" t="n"/>
       <c r="BG132" s="15" t="n"/>
+      <c r="BH132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -17762,6 +18075,9 @@
       <c r="BG133" s="15" t="n">
         <v>21</v>
       </c>
+      <c r="BH133" s="15" t="n">
+        <v>20.92</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -17796,6 +18112,9 @@
       </c>
       <c r="BG134" s="15" t="n">
         <v>3605.55</v>
+      </c>
+      <c r="BH134" s="15" t="n">
+        <v>3623.95</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -17810,6 +18129,7 @@
       <c r="BE135" s="15" t="n"/>
       <c r="BF135" s="15" t="n"/>
       <c r="BG135" s="15" t="n"/>
+      <c r="BH135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -17845,6 +18165,9 @@
       <c r="BG136" s="15" t="n">
         <v>2.67</v>
       </c>
+      <c r="BH136" s="15" t="n">
+        <v>2.86</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -17879,12 +18202,16 @@
       </c>
       <c r="BG137" s="15" t="n">
         <v>2402.55</v>
+      </c>
+      <c r="BH137" s="15" t="n">
+        <v>2422.8</v>
       </c>
     </row>
     <row r="138">
       <c r="BE138" s="15" t="n"/>
       <c r="BF138" s="15" t="n"/>
       <c r="BG138" s="15" t="n"/>
+      <c r="BH138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -17896,6 +18223,9 @@
       <c r="BG139" s="15" t="n">
         <v>11.2</v>
       </c>
+      <c r="BH139" s="15" t="n">
+        <v>11.57</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -17906,12 +18236,16 @@
       </c>
       <c r="BG140" s="15" t="n">
         <v>5572.78</v>
+      </c>
+      <c r="BH140" s="15" t="n">
+        <v>5637.76</v>
       </c>
     </row>
     <row r="141">
       <c r="BE141" s="15" t="n"/>
       <c r="BF141" s="15" t="n"/>
       <c r="BG141" s="15" t="n"/>
+      <c r="BH141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -17923,6 +18257,9 @@
       <c r="BG142" s="15" t="n">
         <v>25.79</v>
       </c>
+      <c r="BH142" s="15" t="n">
+        <v>25.18</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -17933,6 +18270,9 @@
       </c>
       <c r="BG143" s="15" t="n">
         <v>2338.52</v>
+      </c>
+      <c r="BH143" s="15" t="n">
+        <v>2312.19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-08-13 05:23:37]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BH143"/>
+  <dimension ref="A1:BI143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -594,6 +594,7 @@
     <col width="15" customWidth="1" min="58" max="58"/>
     <col width="15" customWidth="1" min="59" max="59"/>
     <col width="15" customWidth="1" min="60" max="60"/>
+    <col width="15" customWidth="1" min="61" max="61"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -897,6 +898,11 @@
           <t>2026/08/10</t>
         </is>
       </c>
+      <c r="BI1" s="15" t="inlineStr">
+        <is>
+          <t>2026/08/13</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1199,6 +1205,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BI2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1381,6 +1392,9 @@
       <c r="BH3" s="15" t="n">
         <v>64.02</v>
       </c>
+      <c r="BI3" s="15" t="n">
+        <v>67.7</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1562,6 +1576,9 @@
       </c>
       <c r="BH4" s="15" t="n">
         <v>3946.93</v>
+      </c>
+      <c r="BI4" s="15" t="n">
+        <v>3962.6</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1625,6 +1642,7 @@
       <c r="BF5" s="15" t="n"/>
       <c r="BG5" s="15" t="n"/>
       <c r="BH5" s="15" t="n"/>
+      <c r="BI5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1735,6 +1753,7 @@
       <c r="BF6" s="15" t="n"/>
       <c r="BG6" s="15" t="n"/>
       <c r="BH6" s="15" t="n"/>
+      <c r="BI6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1916,6 +1935,9 @@
       </c>
       <c r="BH7" s="15" t="n">
         <v>65.19</v>
+      </c>
+      <c r="BI7" s="15" t="n">
+        <v>64.98</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -2050,6 +2072,9 @@
       </c>
       <c r="BH8" s="15" t="n">
         <v>5793.73</v>
+      </c>
+      <c r="BI8" s="15" t="n">
+        <v>5869.06</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2161,6 +2186,7 @@
       <c r="BF9" s="15" t="n"/>
       <c r="BG9" s="15" t="n"/>
       <c r="BH9" s="15" t="n"/>
+      <c r="BI9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2342,6 +2368,9 @@
       </c>
       <c r="BH10" s="15" t="n">
         <v>57</v>
+      </c>
+      <c r="BI10" s="15" t="n">
+        <v>56.65</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2476,6 +2505,9 @@
       </c>
       <c r="BH11" s="15" t="n">
         <v>4670.53</v>
+      </c>
+      <c r="BI11" s="15" t="n">
+        <v>4715.45</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -2587,6 +2619,7 @@
       <c r="BF12" s="15" t="n"/>
       <c r="BG12" s="15" t="n"/>
       <c r="BH12" s="15" t="n"/>
+      <c r="BI12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2768,6 +2801,9 @@
       </c>
       <c r="BH13" s="15" t="n">
         <v>67.12</v>
+      </c>
+      <c r="BI13" s="15" t="n">
+        <v>67.26000000000001</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -2902,6 +2938,9 @@
       </c>
       <c r="BH14" s="15" t="n">
         <v>7941.06</v>
+      </c>
+      <c r="BI14" s="15" t="n">
+        <v>8106.32</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -3013,6 +3052,7 @@
       <c r="BF15" s="15" t="n"/>
       <c r="BG15" s="15" t="n"/>
       <c r="BH15" s="15" t="n"/>
+      <c r="BI15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -3194,6 +3234,9 @@
       </c>
       <c r="BH16" s="15" t="n">
         <v>36.65</v>
+      </c>
+      <c r="BI16" s="15" t="n">
+        <v>36.18</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -3328,6 +3371,9 @@
       </c>
       <c r="BH17" s="15" t="n">
         <v>2623.4</v>
+      </c>
+      <c r="BI17" s="15" t="n">
+        <v>2623.75</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -3439,6 +3485,7 @@
       <c r="BF18" s="15" t="n"/>
       <c r="BG18" s="15" t="n"/>
       <c r="BH18" s="15" t="n"/>
+      <c r="BI18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -3620,6 +3667,9 @@
       </c>
       <c r="BH19" s="15" t="n">
         <v>82.09</v>
+      </c>
+      <c r="BI19" s="15" t="n">
+        <v>81.59</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -3754,6 +3804,9 @@
       </c>
       <c r="BH20" s="15" t="n">
         <v>7757.64</v>
+      </c>
+      <c r="BI20" s="15" t="n">
+        <v>7748.5</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -3865,6 +3918,7 @@
       <c r="BF21" s="15" t="n"/>
       <c r="BG21" s="15" t="n"/>
       <c r="BH21" s="15" t="n"/>
+      <c r="BI21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -4043,6 +4097,9 @@
         <v>36.34</v>
       </c>
       <c r="BH22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BI22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -4178,6 +4235,9 @@
       </c>
       <c r="BH23" s="15" t="n">
         <v>78561.49000000001</v>
+      </c>
+      <c r="BI23" s="15" t="n">
+        <v>77719.11</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -4289,6 +4349,7 @@
       <c r="BF24" s="15" t="n"/>
       <c r="BG24" s="15" t="n"/>
       <c r="BH24" s="15" t="n"/>
+      <c r="BI24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -4469,6 +4530,9 @@
         <v>49.88</v>
       </c>
       <c r="BH25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BI25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -4590,6 +4654,9 @@
       <c r="BG26" s="15" t="inlineStr"/>
       <c r="BH26" s="15" t="n">
         <v>26319.45</v>
+      </c>
+      <c r="BI26" s="15" t="n">
+        <v>26331.07</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -4701,6 +4768,7 @@
       <c r="BF27" s="15" t="n"/>
       <c r="BG27" s="15" t="n"/>
       <c r="BH27" s="15" t="n"/>
+      <c r="BI27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -4881,6 +4949,9 @@
         <v>92.09</v>
       </c>
       <c r="BH28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BI28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -5016,6 +5087,9 @@
       </c>
       <c r="BH29" s="15" t="n">
         <v>66863.55</v>
+      </c>
+      <c r="BI29" s="15" t="n">
+        <v>68668.50999999999</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -5127,6 +5201,7 @@
       <c r="BF30" s="15" t="n"/>
       <c r="BG30" s="15" t="n"/>
       <c r="BH30" s="15" t="n"/>
+      <c r="BI30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -5308,6 +5383,9 @@
       </c>
       <c r="BH31" s="15" t="n">
         <v>45.66</v>
+      </c>
+      <c r="BI31" s="15" t="n">
+        <v>45.46</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -5442,6 +5520,9 @@
       </c>
       <c r="BH32" s="15" t="n">
         <v>5569.2</v>
+      </c>
+      <c r="BI32" s="15" t="n">
+        <v>5474.47</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -5553,6 +5634,7 @@
       <c r="BF33" s="15" t="n"/>
       <c r="BG33" s="15" t="n"/>
       <c r="BH33" s="15" t="n"/>
+      <c r="BI33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -5734,6 +5816,9 @@
       </c>
       <c r="BH34" s="15" t="n">
         <v>58.68</v>
+      </c>
+      <c r="BI34" s="15" t="n">
+        <v>59.37</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -5868,6 +5953,9 @@
       </c>
       <c r="BH35" s="15" t="n">
         <v>11291.49</v>
+      </c>
+      <c r="BI35" s="15" t="n">
+        <v>11311.12</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -5979,6 +6067,7 @@
       <c r="BF36" s="15" t="n"/>
       <c r="BG36" s="15" t="n"/>
       <c r="BH36" s="15" t="n"/>
+      <c r="BI36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -6160,6 +6249,9 @@
       </c>
       <c r="BH37" s="15" t="n">
         <v>50.05</v>
+      </c>
+      <c r="BI37" s="15" t="n">
+        <v>50.07</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -6294,6 +6386,9 @@
       </c>
       <c r="BH38" s="15" t="n">
         <v>10715.06</v>
+      </c>
+      <c r="BI38" s="15" t="n">
+        <v>10709.62</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -6405,6 +6500,7 @@
       <c r="BF39" s="15" t="n"/>
       <c r="BG39" s="15" t="n"/>
       <c r="BH39" s="15" t="n"/>
+      <c r="BI39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -6586,6 +6682,9 @@
       </c>
       <c r="BH40" s="15" t="n">
         <v>49.92</v>
+      </c>
+      <c r="BI40" s="15" t="n">
+        <v>50.19</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -6720,6 +6819,9 @@
       </c>
       <c r="BH41" s="15" t="n">
         <v>3197.71</v>
+      </c>
+      <c r="BI41" s="15" t="n">
+        <v>3212.36</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -6831,6 +6933,7 @@
       <c r="BF42" s="15" t="n"/>
       <c r="BG42" s="15" t="n"/>
       <c r="BH42" s="15" t="n"/>
+      <c r="BI42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -7012,6 +7115,9 @@
       </c>
       <c r="BH43" s="15" t="n">
         <v>58.97</v>
+      </c>
+      <c r="BI43" s="15" t="n">
+        <v>59.88</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -7146,6 +7252,9 @@
       </c>
       <c r="BH44" s="15" t="n">
         <v>6884.36</v>
+      </c>
+      <c r="BI44" s="15" t="n">
+        <v>6896.49</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -7257,6 +7366,7 @@
       <c r="BF45" s="15" t="n"/>
       <c r="BG45" s="15" t="n"/>
       <c r="BH45" s="15" t="n"/>
+      <c r="BI45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -7438,6 +7548,9 @@
       </c>
       <c r="BH46" s="15" t="n">
         <v>29.75</v>
+      </c>
+      <c r="BI46" s="15" t="n">
+        <v>31.15</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -7572,6 +7685,9 @@
       </c>
       <c r="BH47" s="15" t="n">
         <v>34417.12</v>
+      </c>
+      <c r="BI47" s="15" t="n">
+        <v>34236.96</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -7683,6 +7799,7 @@
       <c r="BF48" s="15" t="n"/>
       <c r="BG48" s="15" t="n"/>
       <c r="BH48" s="15" t="n"/>
+      <c r="BI48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -7864,6 +7981,9 @@
       </c>
       <c r="BH49" s="15" t="n">
         <v>49.02</v>
+      </c>
+      <c r="BI49" s="15" t="n">
+        <v>48.53</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -7998,6 +8118,9 @@
       </c>
       <c r="BH50" s="15" t="n">
         <v>3631.6</v>
+      </c>
+      <c r="BI50" s="15" t="n">
+        <v>3844.57</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -8109,6 +8232,7 @@
       <c r="BF51" s="15" t="n"/>
       <c r="BG51" s="15" t="n"/>
       <c r="BH51" s="15" t="n"/>
+      <c r="BI51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -8290,6 +8414,9 @@
       </c>
       <c r="BH52" s="15" t="n">
         <v>60.23</v>
+      </c>
+      <c r="BI52" s="15" t="n">
+        <v>60.46</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -8424,6 +8551,9 @@
       </c>
       <c r="BH53" s="15" t="n">
         <v>3486.72</v>
+      </c>
+      <c r="BI53" s="15" t="n">
+        <v>3664.34</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -8535,6 +8665,7 @@
       <c r="BF54" s="15" t="n"/>
       <c r="BG54" s="15" t="n"/>
       <c r="BH54" s="15" t="n"/>
+      <c r="BI54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -8716,6 +8847,9 @@
       </c>
       <c r="BH55" s="15" t="n">
         <v>18.15</v>
+      </c>
+      <c r="BI55" s="15" t="n">
+        <v>19.79</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -8850,6 +8984,9 @@
       </c>
       <c r="BH56" s="15" t="n">
         <v>6962.91</v>
+      </c>
+      <c r="BI56" s="15" t="n">
+        <v>7120.25</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -8961,6 +9098,7 @@
       <c r="BF57" s="15" t="n"/>
       <c r="BG57" s="15" t="n"/>
       <c r="BH57" s="15" t="n"/>
+      <c r="BI57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -9142,6 +9280,9 @@
       </c>
       <c r="BH58" s="15" t="n">
         <v>39.99</v>
+      </c>
+      <c r="BI58" s="15" t="n">
+        <v>40.96</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -9276,6 +9417,9 @@
       </c>
       <c r="BH59" s="15" t="n">
         <v>8679.719999999999</v>
+      </c>
+      <c r="BI59" s="15" t="n">
+        <v>8742.67</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -9387,6 +9531,7 @@
       <c r="BF60" s="15" t="n"/>
       <c r="BG60" s="15" t="n"/>
       <c r="BH60" s="15" t="n"/>
+      <c r="BI60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -9568,6 +9713,9 @@
       </c>
       <c r="BH61" s="15" t="n">
         <v>3.55</v>
+      </c>
+      <c r="BI61" s="15" t="n">
+        <v>4.62</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -9702,6 +9850,9 @@
       </c>
       <c r="BH62" s="15" t="n">
         <v>11034.71</v>
+      </c>
+      <c r="BI62" s="15" t="n">
+        <v>10948.81</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -9813,6 +9964,7 @@
       <c r="BF63" s="15" t="n"/>
       <c r="BG63" s="15" t="n"/>
       <c r="BH63" s="15" t="n"/>
+      <c r="BI63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -9994,6 +10146,9 @@
       </c>
       <c r="BH64" s="15" t="n">
         <v>19.46</v>
+      </c>
+      <c r="BI64" s="15" t="n">
+        <v>21.57</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -10128,6 +10283,9 @@
       </c>
       <c r="BH65" s="15" t="n">
         <v>11368.1</v>
+      </c>
+      <c r="BI65" s="15" t="n">
+        <v>11572.3</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -10239,6 +10397,7 @@
       <c r="BF66" s="15" t="n"/>
       <c r="BG66" s="15" t="n"/>
       <c r="BH66" s="15" t="n"/>
+      <c r="BI66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -10420,6 +10579,9 @@
       </c>
       <c r="BH67" s="15" t="n">
         <v>15.7</v>
+      </c>
+      <c r="BI67" s="15" t="n">
+        <v>18.75</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -10554,6 +10716,9 @@
       </c>
       <c r="BH68" s="15" t="n">
         <v>6908.63</v>
+      </c>
+      <c r="BI68" s="15" t="n">
+        <v>6978.61</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -10665,6 +10830,7 @@
       <c r="BF69" s="15" t="n"/>
       <c r="BG69" s="15" t="n"/>
       <c r="BH69" s="15" t="n"/>
+      <c r="BI69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -10846,6 +11012,9 @@
       </c>
       <c r="BH70" s="15" t="n">
         <v>15.07</v>
+      </c>
+      <c r="BI70" s="15" t="n">
+        <v>17.32</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -10980,6 +11149,9 @@
       </c>
       <c r="BH71" s="15" t="n">
         <v>12964.85</v>
+      </c>
+      <c r="BI71" s="15" t="n">
+        <v>12872.53</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -11091,6 +11263,7 @@
       <c r="BF72" s="15" t="n"/>
       <c r="BG72" s="15" t="n"/>
       <c r="BH72" s="15" t="n"/>
+      <c r="BI72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -11272,6 +11445,9 @@
       </c>
       <c r="BH73" s="15" t="n">
         <v>55.12</v>
+      </c>
+      <c r="BI73" s="15" t="n">
+        <v>55.28</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -11405,6 +11581,9 @@
         <v>14297.63</v>
       </c>
       <c r="BH74" s="15" t="n">
+        <v>15569.82</v>
+      </c>
+      <c r="BI74" s="15" t="n">
         <v>15569.82</v>
       </c>
     </row>
@@ -11517,6 +11696,7 @@
       <c r="BF75" s="15" t="n"/>
       <c r="BG75" s="15" t="n"/>
       <c r="BH75" s="15" t="n"/>
+      <c r="BI75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -11698,6 +11878,9 @@
       </c>
       <c r="BH76" s="15" t="n">
         <v>5.71</v>
+      </c>
+      <c r="BI76" s="15" t="n">
+        <v>4.36</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -11832,6 +12015,9 @@
       </c>
       <c r="BH77" s="15" t="n">
         <v>7439.15</v>
+      </c>
+      <c r="BI77" s="15" t="n">
+        <v>7319.35</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
@@ -11943,6 +12129,7 @@
       <c r="BF78" s="15" t="n"/>
       <c r="BG78" s="15" t="n"/>
       <c r="BH78" s="15" t="n"/>
+      <c r="BI78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -12124,6 +12311,9 @@
       </c>
       <c r="BH79" s="15" t="n">
         <v>4.37</v>
+      </c>
+      <c r="BI79" s="15" t="n">
+        <v>3.92</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -12258,6 +12448,9 @@
       </c>
       <c r="BH80" s="15" t="n">
         <v>8970.24</v>
+      </c>
+      <c r="BI80" s="15" t="n">
+        <v>9010</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -12369,6 +12562,7 @@
       <c r="BF81" s="15" t="n"/>
       <c r="BG81" s="15" t="n"/>
       <c r="BH81" s="15" t="n"/>
+      <c r="BI81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -12550,6 +12744,9 @@
       </c>
       <c r="BH82" s="15" t="n">
         <v>15.22</v>
+      </c>
+      <c r="BI82" s="15" t="n">
+        <v>13.75</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -12684,6 +12881,9 @@
       </c>
       <c r="BH83" s="15" t="n">
         <v>2424.82</v>
+      </c>
+      <c r="BI83" s="15" t="n">
+        <v>2328.48</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -12795,6 +12995,7 @@
       <c r="BF84" s="15" t="n"/>
       <c r="BG84" s="15" t="n"/>
       <c r="BH84" s="15" t="n"/>
+      <c r="BI84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -12976,6 +13177,9 @@
       </c>
       <c r="BH85" s="15" t="n">
         <v>30.44</v>
+      </c>
+      <c r="BI85" s="15" t="n">
+        <v>28.05</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -13110,6 +13314,9 @@
       </c>
       <c r="BH86" s="15" t="n">
         <v>4876.2</v>
+      </c>
+      <c r="BI86" s="15" t="n">
+        <v>5075.31</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -13221,6 +13428,7 @@
       <c r="BF87" s="15" t="n"/>
       <c r="BG87" s="15" t="n"/>
       <c r="BH87" s="15" t="n"/>
+      <c r="BI87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -13402,6 +13610,9 @@
       </c>
       <c r="BH88" s="15" t="n">
         <v>28.71</v>
+      </c>
+      <c r="BI88" s="15" t="n">
+        <v>29.42</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -13536,6 +13747,9 @@
       </c>
       <c r="BH89" s="15" t="n">
         <v>9047.34</v>
+      </c>
+      <c r="BI89" s="15" t="n">
+        <v>9212.370000000001</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -13647,6 +13861,7 @@
       <c r="BF90" s="15" t="n"/>
       <c r="BG90" s="15" t="n"/>
       <c r="BH90" s="15" t="n"/>
+      <c r="BI90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -13828,6 +14043,9 @@
       </c>
       <c r="BH91" s="15" t="n">
         <v>5.43</v>
+      </c>
+      <c r="BI91" s="15" t="n">
+        <v>4.58</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -13962,6 +14180,9 @@
       </c>
       <c r="BH92" s="15" t="n">
         <v>1183.83</v>
+      </c>
+      <c r="BI92" s="15" t="n">
+        <v>1161.26</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -14073,6 +14294,7 @@
       <c r="BF93" s="15" t="n"/>
       <c r="BG93" s="15" t="n"/>
       <c r="BH93" s="15" t="n"/>
+      <c r="BI93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -14254,6 +14476,9 @@
       </c>
       <c r="BH94" s="15" t="n">
         <v>7.29</v>
+      </c>
+      <c r="BI94" s="15" t="n">
+        <v>8.449999999999999</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -14388,6 +14613,9 @@
       </c>
       <c r="BH95" s="15" t="n">
         <v>14131.94</v>
+      </c>
+      <c r="BI95" s="15" t="n">
+        <v>14441.62</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -14499,6 +14727,7 @@
       <c r="BF96" s="15" t="n"/>
       <c r="BG96" s="15" t="n"/>
       <c r="BH96" s="15" t="n"/>
+      <c r="BI96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -14680,6 +14909,9 @@
       </c>
       <c r="BH97" s="15" t="n">
         <v>51.45</v>
+      </c>
+      <c r="BI97" s="15" t="n">
+        <v>52.61</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -14814,6 +15046,9 @@
       </c>
       <c r="BH98" s="15" t="n">
         <v>3370.1</v>
+      </c>
+      <c r="BI98" s="15" t="n">
+        <v>3423.26</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -14925,6 +15160,7 @@
       <c r="BF99" s="15" t="n"/>
       <c r="BG99" s="15" t="n"/>
       <c r="BH99" s="15" t="n"/>
+      <c r="BI99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -15106,6 +15342,9 @@
       </c>
       <c r="BH100" s="15" t="n">
         <v>38.09</v>
+      </c>
+      <c r="BI100" s="15" t="n">
+        <v>39.45</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -15240,6 +15479,9 @@
       </c>
       <c r="BH101" s="15" t="n">
         <v>2482.15</v>
+      </c>
+      <c r="BI101" s="15" t="n">
+        <v>2534.8</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -15351,6 +15593,7 @@
       <c r="BF102" s="15" t="n"/>
       <c r="BG102" s="15" t="n"/>
       <c r="BH102" s="15" t="n"/>
+      <c r="BI102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -15532,6 +15775,9 @@
       </c>
       <c r="BH103" s="15" t="n">
         <v>17.15</v>
+      </c>
+      <c r="BI103" s="15" t="n">
+        <v>17.87</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -15665,6 +15911,9 @@
         <v>2483.41</v>
       </c>
       <c r="BH104" s="15" t="n">
+        <v>2494.23</v>
+      </c>
+      <c r="BI104" s="15" t="n">
         <v>2494.23</v>
       </c>
     </row>
@@ -15777,6 +16026,7 @@
       <c r="BF105" s="15" t="n"/>
       <c r="BG105" s="15" t="n"/>
       <c r="BH105" s="15" t="n"/>
+      <c r="BI105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -15958,6 +16208,9 @@
       </c>
       <c r="BH106" s="15" t="n">
         <v>38.13</v>
+      </c>
+      <c r="BI106" s="15" t="n">
+        <v>39.1</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -16091,6 +16344,9 @@
         <v>2598.34</v>
       </c>
       <c r="BH107" s="15" t="n">
+        <v>2598.34</v>
+      </c>
+      <c r="BI107" s="15" t="n">
         <v>2598.34</v>
       </c>
     </row>
@@ -16203,6 +16459,7 @@
       <c r="BF108" s="15" t="n"/>
       <c r="BG108" s="15" t="n"/>
       <c r="BH108" s="15" t="n"/>
+      <c r="BI108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -16384,6 +16641,9 @@
       </c>
       <c r="BH109" s="15" t="n">
         <v>66.81999999999999</v>
+      </c>
+      <c r="BI109" s="15" t="n">
+        <v>67.25</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -16518,6 +16778,9 @@
       </c>
       <c r="BH110" s="15" t="n">
         <v>2057.72</v>
+      </c>
+      <c r="BI110" s="15" t="n">
+        <v>2134.5</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -16629,6 +16892,7 @@
       <c r="BF111" s="15" t="n"/>
       <c r="BG111" s="15" t="n"/>
       <c r="BH111" s="15" t="n"/>
+      <c r="BI111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -16810,6 +17074,9 @@
       </c>
       <c r="BH112" s="15" t="n">
         <v>23.65</v>
+      </c>
+      <c r="BI112" s="15" t="n">
+        <v>23.8</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -16942,6 +17209,9 @@
       <c r="BG113" s="15" t="inlineStr"/>
       <c r="BH113" s="15" t="n">
         <v>8939.18</v>
+      </c>
+      <c r="BI113" s="15" t="n">
+        <v>9091</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -17053,6 +17323,7 @@
       <c r="BF114" s="15" t="n"/>
       <c r="BG114" s="15" t="n"/>
       <c r="BH114" s="15" t="n"/>
+      <c r="BI114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -17234,6 +17505,9 @@
       </c>
       <c r="BH115" s="15" t="n">
         <v>96.03</v>
+      </c>
+      <c r="BI115" s="15" t="n">
+        <v>95.92</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -17353,6 +17627,9 @@
       </c>
       <c r="BH116" s="15" t="n">
         <v>13403.42</v>
+      </c>
+      <c r="BI116" s="15" t="n">
+        <v>13945.49</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -17419,6 +17696,7 @@
       <c r="BF117" s="15" t="n"/>
       <c r="BG117" s="15" t="n"/>
       <c r="BH117" s="15" t="n"/>
+      <c r="BI117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -17556,6 +17834,9 @@
       <c r="BH118" s="15" t="n">
         <v>34.3</v>
       </c>
+      <c r="BI118" s="15" t="n">
+        <v>35.77</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -17665,6 +17946,9 @@
       </c>
       <c r="BH119" s="15" t="n">
         <v>1278.85</v>
+      </c>
+      <c r="BI119" s="15" t="n">
+        <v>1291.63</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -17680,6 +17964,7 @@
       <c r="BF120" s="15" t="n"/>
       <c r="BG120" s="15" t="n"/>
       <c r="BH120" s="15" t="n"/>
+      <c r="BI120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -17718,6 +18003,9 @@
       <c r="BH121" s="15" t="n">
         <v>51.17</v>
       </c>
+      <c r="BI121" s="15" t="n">
+        <v>51.38</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -17755,6 +18043,9 @@
       </c>
       <c r="BH122" s="15" t="n">
         <v>11672.22</v>
+      </c>
+      <c r="BI122" s="15" t="n">
+        <v>11787.57</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -17770,6 +18061,7 @@
       <c r="BF123" s="15" t="n"/>
       <c r="BG123" s="15" t="n"/>
       <c r="BH123" s="15" t="n"/>
+      <c r="BI123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -17808,6 +18100,9 @@
       <c r="BH124" s="15" t="n">
         <v>27.49</v>
       </c>
+      <c r="BI124" s="15" t="n">
+        <v>28.6</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -17845,6 +18140,9 @@
       </c>
       <c r="BH125" s="15" t="n">
         <v>1839.6</v>
+      </c>
+      <c r="BI125" s="15" t="n">
+        <v>1879.97</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -17860,6 +18158,7 @@
       <c r="BF126" s="15" t="n"/>
       <c r="BG126" s="15" t="n"/>
       <c r="BH126" s="15" t="n"/>
+      <c r="BI126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -17898,6 +18197,9 @@
       <c r="BH127" s="15" t="n">
         <v>14.49</v>
       </c>
+      <c r="BI127" s="15" t="n">
+        <v>13.96</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -17935,6 +18237,9 @@
       </c>
       <c r="BH128" s="15" t="n">
         <v>764.2</v>
+      </c>
+      <c r="BI128" s="15" t="n">
+        <v>770.39</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -17950,6 +18255,7 @@
       <c r="BF129" s="15" t="n"/>
       <c r="BG129" s="15" t="n"/>
       <c r="BH129" s="15" t="n"/>
+      <c r="BI129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -17988,6 +18294,9 @@
       <c r="BH130" s="15" t="n">
         <v>74.37</v>
       </c>
+      <c r="BI130" s="15" t="n">
+        <v>72.28</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -18025,6 +18334,9 @@
       </c>
       <c r="BH131" s="15" t="n">
         <v>3146.97</v>
+      </c>
+      <c r="BI131" s="15" t="n">
+        <v>3096.16</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -18040,6 +18352,7 @@
       <c r="BF132" s="15" t="n"/>
       <c r="BG132" s="15" t="n"/>
       <c r="BH132" s="15" t="n"/>
+      <c r="BI132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -18078,6 +18391,9 @@
       <c r="BH133" s="15" t="n">
         <v>20.92</v>
       </c>
+      <c r="BI133" s="15" t="n">
+        <v>21.01</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -18115,6 +18431,9 @@
       </c>
       <c r="BH134" s="15" t="n">
         <v>3623.95</v>
+      </c>
+      <c r="BI134" s="15" t="n">
+        <v>3635.06</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -18130,6 +18449,7 @@
       <c r="BF135" s="15" t="n"/>
       <c r="BG135" s="15" t="n"/>
       <c r="BH135" s="15" t="n"/>
+      <c r="BI135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -18168,6 +18488,9 @@
       <c r="BH136" s="15" t="n">
         <v>2.86</v>
       </c>
+      <c r="BI136" s="15" t="n">
+        <v>3.83</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -18205,6 +18528,9 @@
       </c>
       <c r="BH137" s="15" t="n">
         <v>2422.8</v>
+      </c>
+      <c r="BI137" s="15" t="n">
+        <v>2402.55</v>
       </c>
     </row>
     <row r="138">
@@ -18212,6 +18538,7 @@
       <c r="BF138" s="15" t="n"/>
       <c r="BG138" s="15" t="n"/>
       <c r="BH138" s="15" t="n"/>
+      <c r="BI138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -18226,6 +18553,9 @@
       <c r="BH139" s="15" t="n">
         <v>11.57</v>
       </c>
+      <c r="BI139" s="15" t="n">
+        <v>12.31</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -18239,6 +18569,9 @@
       </c>
       <c r="BH140" s="15" t="n">
         <v>5637.76</v>
+      </c>
+      <c r="BI140" s="15" t="n">
+        <v>5685.23</v>
       </c>
     </row>
     <row r="141">
@@ -18246,6 +18579,7 @@
       <c r="BF141" s="15" t="n"/>
       <c r="BG141" s="15" t="n"/>
       <c r="BH141" s="15" t="n"/>
+      <c r="BI141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -18260,6 +18594,9 @@
       <c r="BH142" s="15" t="n">
         <v>25.18</v>
       </c>
+      <c r="BI142" s="15" t="n">
+        <v>25.13</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -18273,6 +18610,9 @@
       </c>
       <c r="BH143" s="15" t="n">
         <v>2312.19</v>
+      </c>
+      <c r="BI143" s="15" t="n">
+        <v>2328.16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-08-14 07:51:02]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BI143"/>
+  <dimension ref="A1:BJ146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -595,6 +595,7 @@
     <col width="15" customWidth="1" min="59" max="59"/>
     <col width="15" customWidth="1" min="60" max="60"/>
     <col width="15" customWidth="1" min="61" max="61"/>
+    <col width="15" customWidth="1" min="62" max="62"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -903,6 +904,11 @@
           <t>2026/08/13</t>
         </is>
       </c>
+      <c r="BJ1" s="15" t="inlineStr">
+        <is>
+          <t>2026/08/14</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1210,6 +1216,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BJ2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1395,6 +1406,9 @@
       <c r="BI3" s="15" t="n">
         <v>67.7</v>
       </c>
+      <c r="BJ3" s="15" t="n">
+        <v>67.23</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1579,6 +1593,9 @@
       </c>
       <c r="BI4" s="15" t="n">
         <v>3962.6</v>
+      </c>
+      <c r="BJ4" s="15" t="n">
+        <v>3927.18</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1643,6 +1660,7 @@
       <c r="BG5" s="15" t="n"/>
       <c r="BH5" s="15" t="n"/>
       <c r="BI5" s="15" t="n"/>
+      <c r="BJ5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1754,6 +1772,7 @@
       <c r="BG6" s="15" t="n"/>
       <c r="BH6" s="15" t="n"/>
       <c r="BI6" s="15" t="n"/>
+      <c r="BJ6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1938,6 +1957,9 @@
       </c>
       <c r="BI7" s="15" t="n">
         <v>64.98</v>
+      </c>
+      <c r="BJ7" s="15" t="n">
+        <v>64.78</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -2075,6 +2097,9 @@
       </c>
       <c r="BI8" s="15" t="n">
         <v>5869.06</v>
+      </c>
+      <c r="BJ8" s="15" t="n">
+        <v>5801.17</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2187,6 +2212,7 @@
       <c r="BG9" s="15" t="n"/>
       <c r="BH9" s="15" t="n"/>
       <c r="BI9" s="15" t="n"/>
+      <c r="BJ9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2371,6 +2397,9 @@
       </c>
       <c r="BI10" s="15" t="n">
         <v>56.65</v>
+      </c>
+      <c r="BJ10" s="15" t="n">
+        <v>56.7</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2508,6 +2537,9 @@
       </c>
       <c r="BI11" s="15" t="n">
         <v>4715.45</v>
+      </c>
+      <c r="BJ11" s="15" t="n">
+        <v>4665.88</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -2620,6 +2652,7 @@
       <c r="BG12" s="15" t="n"/>
       <c r="BH12" s="15" t="n"/>
       <c r="BI12" s="15" t="n"/>
+      <c r="BJ12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2804,6 +2837,9 @@
       </c>
       <c r="BI13" s="15" t="n">
         <v>67.26000000000001</v>
+      </c>
+      <c r="BJ13" s="15" t="n">
+        <v>66.66</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -2941,6 +2977,9 @@
       </c>
       <c r="BI14" s="15" t="n">
         <v>8106.32</v>
+      </c>
+      <c r="BJ14" s="15" t="n">
+        <v>7990.33</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -3053,6 +3092,7 @@
       <c r="BG15" s="15" t="n"/>
       <c r="BH15" s="15" t="n"/>
       <c r="BI15" s="15" t="n"/>
+      <c r="BJ15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -3237,6 +3277,9 @@
       </c>
       <c r="BI16" s="15" t="n">
         <v>36.18</v>
+      </c>
+      <c r="BJ16" s="15" t="n">
+        <v>35.04</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -3374,6 +3417,9 @@
       </c>
       <c r="BI17" s="15" t="n">
         <v>2623.75</v>
+      </c>
+      <c r="BJ17" s="15" t="n">
+        <v>2600.68</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -3486,6 +3532,7 @@
       <c r="BG18" s="15" t="n"/>
       <c r="BH18" s="15" t="n"/>
       <c r="BI18" s="15" t="n"/>
+      <c r="BJ18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -3670,6 +3717,9 @@
       </c>
       <c r="BI19" s="15" t="n">
         <v>81.59</v>
+      </c>
+      <c r="BJ19" s="15" t="n">
+        <v>81.72</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -3807,6 +3857,9 @@
       </c>
       <c r="BI20" s="15" t="n">
         <v>7748.5</v>
+      </c>
+      <c r="BJ20" s="15" t="n">
+        <v>7798.99</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -3919,6 +3972,7 @@
       <c r="BG21" s="15" t="n"/>
       <c r="BH21" s="15" t="n"/>
       <c r="BI21" s="15" t="n"/>
+      <c r="BJ21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -4100,6 +4154,9 @@
         <v>36.34</v>
       </c>
       <c r="BI22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BJ22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -4238,6 +4295,9 @@
       </c>
       <c r="BI23" s="15" t="n">
         <v>77719.11</v>
+      </c>
+      <c r="BJ23" s="15" t="n">
+        <v>77848.63</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -4350,6 +4410,7 @@
       <c r="BG24" s="15" t="n"/>
       <c r="BH24" s="15" t="n"/>
       <c r="BI24" s="15" t="n"/>
+      <c r="BJ24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -4533,6 +4594,9 @@
         <v>49.88</v>
       </c>
       <c r="BI25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BJ25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -4657,6 +4721,9 @@
       </c>
       <c r="BI26" s="15" t="n">
         <v>26331.07</v>
+      </c>
+      <c r="BJ26" s="15" t="n">
+        <v>26451.25</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -4769,6 +4836,7 @@
       <c r="BG27" s="15" t="n"/>
       <c r="BH27" s="15" t="n"/>
       <c r="BI27" s="15" t="n"/>
+      <c r="BJ27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -4952,6 +5020,9 @@
         <v>92.09</v>
       </c>
       <c r="BI28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BJ28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -5090,6 +5161,9 @@
       </c>
       <c r="BI29" s="15" t="n">
         <v>68668.50999999999</v>
+      </c>
+      <c r="BJ29" s="15" t="n">
+        <v>68713.8</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -5202,6 +5276,7 @@
       <c r="BG30" s="15" t="n"/>
       <c r="BH30" s="15" t="n"/>
       <c r="BI30" s="15" t="n"/>
+      <c r="BJ30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -5386,6 +5461,9 @@
       </c>
       <c r="BI31" s="15" t="n">
         <v>45.46</v>
+      </c>
+      <c r="BJ31" s="15" t="n">
+        <v>97.44</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
@@ -5523,6 +5601,9 @@
       </c>
       <c r="BI32" s="15" t="n">
         <v>5474.47</v>
+      </c>
+      <c r="BJ32" s="15" t="n">
+        <v>6977.94</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -5635,6 +5716,7 @@
       <c r="BG33" s="15" t="n"/>
       <c r="BH33" s="15" t="n"/>
       <c r="BI33" s="15" t="n"/>
+      <c r="BJ33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -5819,6 +5901,9 @@
       </c>
       <c r="BI34" s="15" t="n">
         <v>59.37</v>
+      </c>
+      <c r="BJ34" s="15" t="n">
+        <v>45.55</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -5956,6 +6041,9 @@
       </c>
       <c r="BI35" s="15" t="n">
         <v>11311.12</v>
+      </c>
+      <c r="BJ35" s="15" t="n">
+        <v>5478.39</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -6068,6 +6156,7 @@
       <c r="BG36" s="15" t="n"/>
       <c r="BH36" s="15" t="n"/>
       <c r="BI36" s="15" t="n"/>
+      <c r="BJ36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -6252,6 +6341,9 @@
       </c>
       <c r="BI37" s="15" t="n">
         <v>50.07</v>
+      </c>
+      <c r="BJ37" s="15" t="n">
+        <v>59.07</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -6389,6 +6481,9 @@
       </c>
       <c r="BI38" s="15" t="n">
         <v>10709.62</v>
+      </c>
+      <c r="BJ38" s="15" t="n">
+        <v>11245.24</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -6501,6 +6596,7 @@
       <c r="BG39" s="15" t="n"/>
       <c r="BH39" s="15" t="n"/>
       <c r="BI39" s="15" t="n"/>
+      <c r="BJ39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -6685,6 +6781,9 @@
       </c>
       <c r="BI40" s="15" t="n">
         <v>50.19</v>
+      </c>
+      <c r="BJ40" s="15" t="n">
+        <v>49.93</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -6822,6 +6921,9 @@
       </c>
       <c r="BI41" s="15" t="n">
         <v>3212.36</v>
+      </c>
+      <c r="BJ41" s="15" t="n">
+        <v>10695.18</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -6934,6 +7036,7 @@
       <c r="BG42" s="15" t="n"/>
       <c r="BH42" s="15" t="n"/>
       <c r="BI42" s="15" t="n"/>
+      <c r="BJ42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -7118,6 +7221,9 @@
       </c>
       <c r="BI43" s="15" t="n">
         <v>59.88</v>
+      </c>
+      <c r="BJ43" s="15" t="n">
+        <v>50.08</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -7255,6 +7361,9 @@
       </c>
       <c r="BI44" s="15" t="n">
         <v>6896.49</v>
+      </c>
+      <c r="BJ44" s="15" t="n">
+        <v>3187.46</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -7367,6 +7476,7 @@
       <c r="BG45" s="15" t="n"/>
       <c r="BH45" s="15" t="n"/>
       <c r="BI45" s="15" t="n"/>
+      <c r="BJ45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -7551,6 +7661,9 @@
       </c>
       <c r="BI46" s="15" t="n">
         <v>31.15</v>
+      </c>
+      <c r="BJ46" s="15" t="n">
+        <v>59.29</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -7688,6 +7801,9 @@
       </c>
       <c r="BI47" s="15" t="n">
         <v>34236.96</v>
+      </c>
+      <c r="BJ47" s="15" t="n">
+        <v>6894.77</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -7800,6 +7916,7 @@
       <c r="BG48" s="15" t="n"/>
       <c r="BH48" s="15" t="n"/>
       <c r="BI48" s="15" t="n"/>
+      <c r="BJ48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -7984,6 +8101,9 @@
       </c>
       <c r="BI49" s="15" t="n">
         <v>48.53</v>
+      </c>
+      <c r="BJ49" s="15" t="n">
+        <v>29.48</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -8121,6 +8241,9 @@
       </c>
       <c r="BI50" s="15" t="n">
         <v>3844.57</v>
+      </c>
+      <c r="BJ50" s="15" t="n">
+        <v>34036.07</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -8233,6 +8356,7 @@
       <c r="BG51" s="15" t="n"/>
       <c r="BH51" s="15" t="n"/>
       <c r="BI51" s="15" t="n"/>
+      <c r="BJ51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -8417,6 +8541,9 @@
       </c>
       <c r="BI52" s="15" t="n">
         <v>60.46</v>
+      </c>
+      <c r="BJ52" s="15" t="n">
+        <v>48.36</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -8554,6 +8681,9 @@
       </c>
       <c r="BI53" s="15" t="n">
         <v>3664.34</v>
+      </c>
+      <c r="BJ53" s="15" t="n">
+        <v>3807.97</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -8666,6 +8796,7 @@
       <c r="BG54" s="15" t="n"/>
       <c r="BH54" s="15" t="n"/>
       <c r="BI54" s="15" t="n"/>
+      <c r="BJ54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -8850,6 +8981,9 @@
       </c>
       <c r="BI55" s="15" t="n">
         <v>19.79</v>
+      </c>
+      <c r="BJ55" s="15" t="n">
+        <v>59.94</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -8987,6 +9121,9 @@
       </c>
       <c r="BI56" s="15" t="n">
         <v>7120.25</v>
+      </c>
+      <c r="BJ56" s="15" t="n">
+        <v>3626.3</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -9099,6 +9236,7 @@
       <c r="BG57" s="15" t="n"/>
       <c r="BH57" s="15" t="n"/>
       <c r="BI57" s="15" t="n"/>
+      <c r="BJ57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -9283,6 +9421,9 @@
       </c>
       <c r="BI58" s="15" t="n">
         <v>40.96</v>
+      </c>
+      <c r="BJ58" s="15" t="n">
+        <v>21.3</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -9420,6 +9561,9 @@
       </c>
       <c r="BI59" s="15" t="n">
         <v>8742.67</v>
+      </c>
+      <c r="BJ59" s="15" t="n">
+        <v>6949.47</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -9532,6 +9676,7 @@
       <c r="BG60" s="15" t="n"/>
       <c r="BH60" s="15" t="n"/>
       <c r="BI60" s="15" t="n"/>
+      <c r="BJ60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -9716,6 +9861,9 @@
       </c>
       <c r="BI61" s="15" t="n">
         <v>4.62</v>
+      </c>
+      <c r="BJ61" s="15" t="n">
+        <v>40.71</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -9853,6 +10001,9 @@
       </c>
       <c r="BI62" s="15" t="n">
         <v>10948.81</v>
+      </c>
+      <c r="BJ62" s="15" t="n">
+        <v>8487.139999999999</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -9965,6 +10116,7 @@
       <c r="BG63" s="15" t="n"/>
       <c r="BH63" s="15" t="n"/>
       <c r="BI63" s="15" t="n"/>
+      <c r="BJ63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -10149,6 +10301,9 @@
       </c>
       <c r="BI64" s="15" t="n">
         <v>21.57</v>
+      </c>
+      <c r="BJ64" s="15" t="n">
+        <v>4.75</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -10286,6 +10441,9 @@
       </c>
       <c r="BI65" s="15" t="n">
         <v>11572.3</v>
+      </c>
+      <c r="BJ65" s="15" t="n">
+        <v>10787.19</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -10398,6 +10556,7 @@
       <c r="BG66" s="15" t="n"/>
       <c r="BH66" s="15" t="n"/>
       <c r="BI66" s="15" t="n"/>
+      <c r="BJ66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -10582,6 +10741,9 @@
       </c>
       <c r="BI67" s="15" t="n">
         <v>18.75</v>
+      </c>
+      <c r="BJ67" s="15" t="n">
+        <v>20.6</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -10719,6 +10881,9 @@
       </c>
       <c r="BI68" s="15" t="n">
         <v>6978.61</v>
+      </c>
+      <c r="BJ68" s="15" t="n">
+        <v>11572.3</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -10831,6 +10996,7 @@
       <c r="BG69" s="15" t="n"/>
       <c r="BH69" s="15" t="n"/>
       <c r="BI69" s="15" t="n"/>
+      <c r="BJ69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -11015,6 +11181,9 @@
       </c>
       <c r="BI70" s="15" t="n">
         <v>17.32</v>
+      </c>
+      <c r="BJ70" s="15" t="n">
+        <v>19.85</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -11152,6 +11321,9 @@
       </c>
       <c r="BI71" s="15" t="n">
         <v>12872.53</v>
+      </c>
+      <c r="BJ71" s="15" t="n">
+        <v>6804.46</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -11264,6 +11436,7 @@
       <c r="BG72" s="15" t="n"/>
       <c r="BH72" s="15" t="n"/>
       <c r="BI72" s="15" t="n"/>
+      <c r="BJ72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -11448,6 +11621,9 @@
       </c>
       <c r="BI73" s="15" t="n">
         <v>55.28</v>
+      </c>
+      <c r="BJ73" s="15" t="n">
+        <v>17.61</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -11585,6 +11761,9 @@
       </c>
       <c r="BI74" s="15" t="n">
         <v>15569.82</v>
+      </c>
+      <c r="BJ74" s="15" t="n">
+        <v>12658.53</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -11697,6 +11876,7 @@
       <c r="BG75" s="15" t="n"/>
       <c r="BH75" s="15" t="n"/>
       <c r="BI75" s="15" t="n"/>
+      <c r="BJ75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -11881,6 +12061,9 @@
       </c>
       <c r="BI76" s="15" t="n">
         <v>4.36</v>
+      </c>
+      <c r="BJ76" s="15" t="n">
+        <v>55.55</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -12018,6 +12201,9 @@
       </c>
       <c r="BI77" s="15" t="n">
         <v>7319.35</v>
+      </c>
+      <c r="BJ77" s="15" t="n">
+        <v>15569.82</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
@@ -12130,6 +12316,7 @@
       <c r="BG78" s="15" t="n"/>
       <c r="BH78" s="15" t="n"/>
       <c r="BI78" s="15" t="n"/>
+      <c r="BJ78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -12314,6 +12501,9 @@
       </c>
       <c r="BI79" s="15" t="n">
         <v>3.92</v>
+      </c>
+      <c r="BJ79" s="15" t="n">
+        <v>3.61</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -12451,6 +12641,9 @@
       </c>
       <c r="BI80" s="15" t="n">
         <v>9010</v>
+      </c>
+      <c r="BJ80" s="15" t="n">
+        <v>6982.18</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -12563,6 +12756,7 @@
       <c r="BG81" s="15" t="n"/>
       <c r="BH81" s="15" t="n"/>
       <c r="BI81" s="15" t="n"/>
+      <c r="BJ81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -12747,6 +12941,9 @@
       </c>
       <c r="BI82" s="15" t="n">
         <v>13.75</v>
+      </c>
+      <c r="BJ82" s="15" t="n">
+        <v>4.43</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -12884,6 +13081,9 @@
       </c>
       <c r="BI83" s="15" t="n">
         <v>2328.48</v>
+      </c>
+      <c r="BJ83" s="15" t="n">
+        <v>8851.09</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -12996,6 +13196,7 @@
       <c r="BG84" s="15" t="n"/>
       <c r="BH84" s="15" t="n"/>
       <c r="BI84" s="15" t="n"/>
+      <c r="BJ84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -13180,6 +13381,9 @@
       </c>
       <c r="BI85" s="15" t="n">
         <v>28.05</v>
+      </c>
+      <c r="BJ85" s="15" t="n">
+        <v>12.66</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -13317,6 +13521,9 @@
       </c>
       <c r="BI86" s="15" t="n">
         <v>5075.31</v>
+      </c>
+      <c r="BJ86" s="15" t="n">
+        <v>2631.9</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -13429,6 +13636,7 @@
       <c r="BG87" s="15" t="n"/>
       <c r="BH87" s="15" t="n"/>
       <c r="BI87" s="15" t="n"/>
+      <c r="BJ87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -13613,6 +13821,9 @@
       </c>
       <c r="BI88" s="15" t="n">
         <v>29.42</v>
+      </c>
+      <c r="BJ88" s="15" t="n">
+        <v>28.98</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -13750,6 +13961,9 @@
       </c>
       <c r="BI89" s="15" t="n">
         <v>9212.370000000001</v>
+      </c>
+      <c r="BJ89" s="15" t="n">
+        <v>5075.31</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -13862,6 +14076,7 @@
       <c r="BG90" s="15" t="n"/>
       <c r="BH90" s="15" t="n"/>
       <c r="BI90" s="15" t="n"/>
+      <c r="BJ90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -14046,6 +14261,9 @@
       </c>
       <c r="BI91" s="15" t="n">
         <v>4.58</v>
+      </c>
+      <c r="BJ91" s="15" t="n">
+        <v>30.03</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -14183,6 +14401,9 @@
       </c>
       <c r="BI92" s="15" t="n">
         <v>1161.26</v>
+      </c>
+      <c r="BJ92" s="15" t="n">
+        <v>8977.57</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -14295,6 +14516,7 @@
       <c r="BG93" s="15" t="n"/>
       <c r="BH93" s="15" t="n"/>
       <c r="BI93" s="15" t="n"/>
+      <c r="BJ93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -14479,6 +14701,9 @@
       </c>
       <c r="BI94" s="15" t="n">
         <v>8.449999999999999</v>
+      </c>
+      <c r="BJ94" s="15" t="n">
+        <v>4.84</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -14616,6 +14841,9 @@
       </c>
       <c r="BI95" s="15" t="n">
         <v>14441.62</v>
+      </c>
+      <c r="BJ95" s="15" t="n">
+        <v>1164.31</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -14728,6 +14956,7 @@
       <c r="BG96" s="15" t="n"/>
       <c r="BH96" s="15" t="n"/>
       <c r="BI96" s="15" t="n"/>
+      <c r="BJ96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -14912,6 +15141,9 @@
       </c>
       <c r="BI97" s="15" t="n">
         <v>52.61</v>
+      </c>
+      <c r="BJ97" s="15" t="n">
+        <v>8.68</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -15049,6 +15281,9 @@
       </c>
       <c r="BI98" s="15" t="n">
         <v>3423.26</v>
+      </c>
+      <c r="BJ98" s="15" t="n">
+        <v>14490.77</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -15161,6 +15396,7 @@
       <c r="BG99" s="15" t="n"/>
       <c r="BH99" s="15" t="n"/>
       <c r="BI99" s="15" t="n"/>
+      <c r="BJ99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -15345,6 +15581,9 @@
       </c>
       <c r="BI100" s="15" t="n">
         <v>39.45</v>
+      </c>
+      <c r="BJ100" s="15" t="n">
+        <v>53.6</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -15482,6 +15721,9 @@
       </c>
       <c r="BI101" s="15" t="n">
         <v>2534.8</v>
+      </c>
+      <c r="BJ101" s="15" t="n">
+        <v>3464.35</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -15594,6 +15836,7 @@
       <c r="BG102" s="15" t="n"/>
       <c r="BH102" s="15" t="n"/>
       <c r="BI102" s="15" t="n"/>
+      <c r="BJ102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -15778,6 +16021,9 @@
       </c>
       <c r="BI103" s="15" t="n">
         <v>17.87</v>
+      </c>
+      <c r="BJ103" s="15" t="n">
+        <v>38.98</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -15915,6 +16161,9 @@
       </c>
       <c r="BI104" s="15" t="n">
         <v>2494.23</v>
+      </c>
+      <c r="BJ104" s="15" t="n">
+        <v>2512.5</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -16027,6 +16276,7 @@
       <c r="BG105" s="15" t="n"/>
       <c r="BH105" s="15" t="n"/>
       <c r="BI105" s="15" t="n"/>
+      <c r="BJ105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -16211,6 +16461,9 @@
       </c>
       <c r="BI106" s="15" t="n">
         <v>39.1</v>
+      </c>
+      <c r="BJ106" s="15" t="n">
+        <v>17.08</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -16348,6 +16601,9 @@
       </c>
       <c r="BI107" s="15" t="n">
         <v>2598.34</v>
+      </c>
+      <c r="BJ107" s="15" t="n">
+        <v>2494.23</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -16460,6 +16716,7 @@
       <c r="BG108" s="15" t="n"/>
       <c r="BH108" s="15" t="n"/>
       <c r="BI108" s="15" t="n"/>
+      <c r="BJ108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -16644,6 +16901,9 @@
       </c>
       <c r="BI109" s="15" t="n">
         <v>67.25</v>
+      </c>
+      <c r="BJ109" s="15" t="n">
+        <v>38.79</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -16781,6 +17041,9 @@
       </c>
       <c r="BI110" s="15" t="n">
         <v>2134.5</v>
+      </c>
+      <c r="BJ110" s="15" t="n">
+        <v>2663.1</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -16893,6 +17156,7 @@
       <c r="BG111" s="15" t="n"/>
       <c r="BH111" s="15" t="n"/>
       <c r="BI111" s="15" t="n"/>
+      <c r="BJ111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -17077,6 +17341,9 @@
       </c>
       <c r="BI112" s="15" t="n">
         <v>23.8</v>
+      </c>
+      <c r="BJ112" s="15" t="n">
+        <v>68.48</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -17212,6 +17479,9 @@
       </c>
       <c r="BI113" s="15" t="n">
         <v>9091</v>
+      </c>
+      <c r="BJ113" s="15" t="n">
+        <v>2098.35</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -17324,6 +17594,7 @@
       <c r="BG114" s="15" t="n"/>
       <c r="BH114" s="15" t="n"/>
       <c r="BI114" s="15" t="n"/>
+      <c r="BJ114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -17508,6 +17779,9 @@
       </c>
       <c r="BI115" s="15" t="n">
         <v>95.92</v>
+      </c>
+      <c r="BJ115" s="15" t="n">
+        <v>23.93</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -17630,6 +17904,9 @@
       </c>
       <c r="BI116" s="15" t="n">
         <v>13945.49</v>
+      </c>
+      <c r="BJ116" s="15" t="n">
+        <v>8929.530000000001</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -17697,6 +17974,7 @@
       <c r="BG117" s="15" t="n"/>
       <c r="BH117" s="15" t="n"/>
       <c r="BI117" s="15" t="n"/>
+      <c r="BJ117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -17837,6 +18115,9 @@
       <c r="BI118" s="15" t="n">
         <v>35.77</v>
       </c>
+      <c r="BJ118" s="15" t="n">
+        <v>95.43000000000001</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -17949,6 +18230,9 @@
       </c>
       <c r="BI119" s="15" t="n">
         <v>1291.63</v>
+      </c>
+      <c r="BJ119" s="15" t="n">
+        <v>13493.35</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -17965,6 +18249,7 @@
       <c r="BG120" s="15" t="n"/>
       <c r="BH120" s="15" t="n"/>
       <c r="BI120" s="15" t="n"/>
+      <c r="BJ120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -18006,6 +18291,9 @@
       <c r="BI121" s="15" t="n">
         <v>51.38</v>
       </c>
+      <c r="BJ121" s="15" t="n">
+        <v>33.08</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -18046,6 +18334,9 @@
       </c>
       <c r="BI122" s="15" t="n">
         <v>11787.57</v>
+      </c>
+      <c r="BJ122" s="15" t="n">
+        <v>1267.69</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -18062,6 +18353,7 @@
       <c r="BG123" s="15" t="n"/>
       <c r="BH123" s="15" t="n"/>
       <c r="BI123" s="15" t="n"/>
+      <c r="BJ123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -18103,6 +18395,9 @@
       <c r="BI124" s="15" t="n">
         <v>28.6</v>
       </c>
+      <c r="BJ124" s="15" t="n">
+        <v>50.05</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -18143,6 +18438,9 @@
       </c>
       <c r="BI125" s="15" t="n">
         <v>1879.97</v>
+      </c>
+      <c r="BJ125" s="15" t="n">
+        <v>11659.75</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -18159,6 +18457,7 @@
       <c r="BG126" s="15" t="n"/>
       <c r="BH126" s="15" t="n"/>
       <c r="BI126" s="15" t="n"/>
+      <c r="BJ126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -18200,6 +18499,9 @@
       <c r="BI127" s="15" t="n">
         <v>13.96</v>
       </c>
+      <c r="BJ127" s="15" t="n">
+        <v>28.6</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -18240,6 +18542,9 @@
       </c>
       <c r="BI128" s="15" t="n">
         <v>770.39</v>
+      </c>
+      <c r="BJ128" s="15" t="n">
+        <v>1848.91</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -18256,6 +18561,7 @@
       <c r="BG129" s="15" t="n"/>
       <c r="BH129" s="15" t="n"/>
       <c r="BI129" s="15" t="n"/>
+      <c r="BJ129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -18297,6 +18603,9 @@
       <c r="BI130" s="15" t="n">
         <v>72.28</v>
       </c>
+      <c r="BJ130" s="15" t="n">
+        <v>15.65</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -18337,6 +18646,9 @@
       </c>
       <c r="BI131" s="15" t="n">
         <v>3096.16</v>
+      </c>
+      <c r="BJ131" s="15" t="n">
+        <v>756.25</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -18353,6 +18665,7 @@
       <c r="BG132" s="15" t="n"/>
       <c r="BH132" s="15" t="n"/>
       <c r="BI132" s="15" t="n"/>
+      <c r="BJ132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -18394,6 +18707,9 @@
       <c r="BI133" s="15" t="n">
         <v>21.01</v>
       </c>
+      <c r="BJ133" s="15" t="n">
+        <v>68.02</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -18434,6 +18750,9 @@
       </c>
       <c r="BI134" s="15" t="n">
         <v>3635.06</v>
+      </c>
+      <c r="BJ134" s="15" t="n">
+        <v>3078.44</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -18450,6 +18769,7 @@
       <c r="BG135" s="15" t="n"/>
       <c r="BH135" s="15" t="n"/>
       <c r="BI135" s="15" t="n"/>
+      <c r="BJ135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -18491,6 +18811,9 @@
       <c r="BI136" s="15" t="n">
         <v>3.83</v>
       </c>
+      <c r="BJ136" s="15" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -18531,6 +18854,9 @@
       </c>
       <c r="BI137" s="15" t="n">
         <v>2402.55</v>
+      </c>
+      <c r="BJ137" s="15" t="n">
+        <v>3603.48</v>
       </c>
     </row>
     <row r="138">
@@ -18539,6 +18865,7 @@
       <c r="BG138" s="15" t="n"/>
       <c r="BH138" s="15" t="n"/>
       <c r="BI138" s="15" t="n"/>
+      <c r="BJ138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -18556,6 +18883,9 @@
       <c r="BI139" s="15" t="n">
         <v>12.31</v>
       </c>
+      <c r="BJ139" s="15" t="n">
+        <v>3.57</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -18572,6 +18902,9 @@
       </c>
       <c r="BI140" s="15" t="n">
         <v>5685.23</v>
+      </c>
+      <c r="BJ140" s="15" t="n">
+        <v>2408.81</v>
       </c>
     </row>
     <row r="141">
@@ -18580,6 +18913,7 @@
       <c r="BG141" s="15" t="n"/>
       <c r="BH141" s="15" t="n"/>
       <c r="BI141" s="15" t="n"/>
+      <c r="BJ141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -18597,6 +18931,9 @@
       <c r="BI142" s="15" t="n">
         <v>25.13</v>
       </c>
+      <c r="BJ142" s="15" t="n">
+        <v>12.27</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -18613,6 +18950,22 @@
       </c>
       <c r="BI143" s="15" t="n">
         <v>2328.16</v>
+      </c>
+      <c r="BJ143" s="15" t="n">
+        <v>5685.23</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="BJ144" s="15" t="n"/>
+    </row>
+    <row r="145">
+      <c r="BJ145" s="15" t="n">
+        <v>24.82</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="BJ146" s="15" t="n">
+        <v>2304.53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-08-17 04:24:52]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BJ146"/>
+  <dimension ref="A1:BK146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -596,6 +596,7 @@
     <col width="15" customWidth="1" min="60" max="60"/>
     <col width="15" customWidth="1" min="61" max="61"/>
     <col width="15" customWidth="1" min="62" max="62"/>
+    <col width="15" customWidth="1" min="63" max="63"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -909,6 +910,11 @@
           <t>2026/08/14</t>
         </is>
       </c>
+      <c r="BK1" s="15" t="inlineStr">
+        <is>
+          <t>2026/08/17</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1221,6 +1227,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BK2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1409,6 +1420,9 @@
       <c r="BJ3" s="15" t="n">
         <v>67.23</v>
       </c>
+      <c r="BK3" s="15" t="n">
+        <v>67.41</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1596,6 +1610,9 @@
       </c>
       <c r="BJ4" s="15" t="n">
         <v>3927.18</v>
+      </c>
+      <c r="BK4" s="15" t="n">
+        <v>3960.19</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1661,6 +1678,7 @@
       <c r="BH5" s="15" t="n"/>
       <c r="BI5" s="15" t="n"/>
       <c r="BJ5" s="15" t="n"/>
+      <c r="BK5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1773,6 +1791,7 @@
       <c r="BH6" s="15" t="n"/>
       <c r="BI6" s="15" t="n"/>
       <c r="BJ6" s="15" t="n"/>
+      <c r="BK6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1960,6 +1979,9 @@
       </c>
       <c r="BJ7" s="15" t="n">
         <v>64.78</v>
+      </c>
+      <c r="BK7" s="15" t="n">
+        <v>63.26</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -2100,6 +2122,9 @@
       </c>
       <c r="BJ8" s="15" t="n">
         <v>5801.17</v>
+      </c>
+      <c r="BK8" s="15" t="n">
+        <v>5860.01</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2213,6 +2238,7 @@
       <c r="BH9" s="15" t="n"/>
       <c r="BI9" s="15" t="n"/>
       <c r="BJ9" s="15" t="n"/>
+      <c r="BK9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2400,6 +2426,9 @@
       </c>
       <c r="BJ10" s="15" t="n">
         <v>56.7</v>
+      </c>
+      <c r="BK10" s="15" t="n">
+        <v>54.67</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2540,6 +2569,9 @@
       </c>
       <c r="BJ11" s="15" t="n">
         <v>4665.88</v>
+      </c>
+      <c r="BK11" s="15" t="n">
+        <v>4701.19</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -2653,6 +2685,7 @@
       <c r="BH12" s="15" t="n"/>
       <c r="BI12" s="15" t="n"/>
       <c r="BJ12" s="15" t="n"/>
+      <c r="BK12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2840,6 +2873,9 @@
       </c>
       <c r="BJ13" s="15" t="n">
         <v>66.66</v>
+      </c>
+      <c r="BK13" s="15" t="n">
+        <v>66.69</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -2980,6 +3016,9 @@
       </c>
       <c r="BJ14" s="15" t="n">
         <v>7990.33</v>
+      </c>
+      <c r="BK14" s="15" t="n">
+        <v>8119.26</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -3093,6 +3132,7 @@
       <c r="BH15" s="15" t="n"/>
       <c r="BI15" s="15" t="n"/>
       <c r="BJ15" s="15" t="n"/>
+      <c r="BK15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -3280,6 +3320,9 @@
       </c>
       <c r="BJ16" s="15" t="n">
         <v>35.04</v>
+      </c>
+      <c r="BK16" s="15" t="n">
+        <v>35.16</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -3419,6 +3462,9 @@
         <v>2623.75</v>
       </c>
       <c r="BJ17" s="15" t="n">
+        <v>2600.68</v>
+      </c>
+      <c r="BK17" s="15" t="n">
         <v>2600.68</v>
       </c>
     </row>
@@ -3533,6 +3579,7 @@
       <c r="BH18" s="15" t="n"/>
       <c r="BI18" s="15" t="n"/>
       <c r="BJ18" s="15" t="n"/>
+      <c r="BK18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -3720,6 +3767,9 @@
       </c>
       <c r="BJ19" s="15" t="n">
         <v>81.72</v>
+      </c>
+      <c r="BK19" s="15" t="n">
+        <v>81.91</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -3860,6 +3910,9 @@
       </c>
       <c r="BJ20" s="15" t="n">
         <v>7798.99</v>
+      </c>
+      <c r="BK20" s="15" t="n">
+        <v>7785.76</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -3973,6 +4026,7 @@
       <c r="BH21" s="15" t="n"/>
       <c r="BI21" s="15" t="n"/>
       <c r="BJ21" s="15" t="n"/>
+      <c r="BK21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -4157,6 +4211,9 @@
         <v>36.34</v>
       </c>
       <c r="BJ22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BK22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -4298,6 +4355,9 @@
       </c>
       <c r="BJ23" s="15" t="n">
         <v>77848.63</v>
+      </c>
+      <c r="BK23" s="15" t="n">
+        <v>77661.00999999999</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -4411,6 +4471,7 @@
       <c r="BH24" s="15" t="n"/>
       <c r="BI24" s="15" t="n"/>
       <c r="BJ24" s="15" t="n"/>
+      <c r="BK24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -4597,6 +4658,9 @@
         <v>49.88</v>
       </c>
       <c r="BJ25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BK25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -4724,6 +4788,9 @@
       </c>
       <c r="BJ26" s="15" t="n">
         <v>26451.25</v>
+      </c>
+      <c r="BK26" s="15" t="n">
+        <v>26440.31</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -4837,6 +4904,7 @@
       <c r="BH27" s="15" t="n"/>
       <c r="BI27" s="15" t="n"/>
       <c r="BJ27" s="15" t="n"/>
+      <c r="BK27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -5023,6 +5091,9 @@
         <v>92.09</v>
       </c>
       <c r="BJ28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BK28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -5164,6 +5235,9 @@
       </c>
       <c r="BJ29" s="15" t="n">
         <v>68713.8</v>
+      </c>
+      <c r="BK29" s="15" t="n">
+        <v>68922.84</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -5277,6 +5351,7 @@
       <c r="BH30" s="15" t="n"/>
       <c r="BI30" s="15" t="n"/>
       <c r="BJ30" s="15" t="n"/>
+      <c r="BK30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -5463,6 +5538,9 @@
         <v>45.46</v>
       </c>
       <c r="BJ31" s="15" t="n">
+        <v>97.44</v>
+      </c>
+      <c r="BK31" s="15" t="n">
         <v>97.44</v>
       </c>
     </row>
@@ -5603,6 +5681,9 @@
         <v>5474.47</v>
       </c>
       <c r="BJ32" s="15" t="n">
+        <v>6977.94</v>
+      </c>
+      <c r="BK32" s="15" t="n">
         <v>6977.94</v>
       </c>
     </row>
@@ -5717,6 +5798,7 @@
       <c r="BH33" s="15" t="n"/>
       <c r="BI33" s="15" t="n"/>
       <c r="BJ33" s="15" t="n"/>
+      <c r="BK33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -5904,6 +5986,9 @@
       </c>
       <c r="BJ34" s="15" t="n">
         <v>45.55</v>
+      </c>
+      <c r="BK34" s="15" t="n">
+        <v>45.28</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -6044,6 +6129,9 @@
       </c>
       <c r="BJ35" s="15" t="n">
         <v>5478.39</v>
+      </c>
+      <c r="BK35" s="15" t="n">
+        <v>5488.93</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -6157,6 +6245,7 @@
       <c r="BH36" s="15" t="n"/>
       <c r="BI36" s="15" t="n"/>
       <c r="BJ36" s="15" t="n"/>
+      <c r="BK36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -6344,6 +6433,9 @@
       </c>
       <c r="BJ37" s="15" t="n">
         <v>59.07</v>
+      </c>
+      <c r="BK37" s="15" t="n">
+        <v>59.88</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -6484,6 +6576,9 @@
       </c>
       <c r="BJ38" s="15" t="n">
         <v>11245.24</v>
+      </c>
+      <c r="BK38" s="15" t="n">
+        <v>11206.89</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -6597,6 +6692,7 @@
       <c r="BH39" s="15" t="n"/>
       <c r="BI39" s="15" t="n"/>
       <c r="BJ39" s="15" t="n"/>
+      <c r="BK39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -6784,6 +6880,9 @@
       </c>
       <c r="BJ40" s="15" t="n">
         <v>49.93</v>
+      </c>
+      <c r="BK40" s="15" t="n">
+        <v>49.99</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -6924,6 +7023,9 @@
       </c>
       <c r="BJ41" s="15" t="n">
         <v>10695.18</v>
+      </c>
+      <c r="BK41" s="15" t="n">
+        <v>10655.59</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -7037,6 +7139,7 @@
       <c r="BH42" s="15" t="n"/>
       <c r="BI42" s="15" t="n"/>
       <c r="BJ42" s="15" t="n"/>
+      <c r="BK42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -7224,6 +7327,9 @@
       </c>
       <c r="BJ43" s="15" t="n">
         <v>50.08</v>
+      </c>
+      <c r="BK43" s="15" t="n">
+        <v>50.16</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -7364,6 +7470,9 @@
       </c>
       <c r="BJ44" s="15" t="n">
         <v>3187.46</v>
+      </c>
+      <c r="BK44" s="15" t="n">
+        <v>3206.98</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -7477,6 +7586,7 @@
       <c r="BH45" s="15" t="n"/>
       <c r="BI45" s="15" t="n"/>
       <c r="BJ45" s="15" t="n"/>
+      <c r="BK45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -7664,6 +7774,9 @@
       </c>
       <c r="BJ46" s="15" t="n">
         <v>59.29</v>
+      </c>
+      <c r="BK46" s="15" t="n">
+        <v>59.64</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -7804,6 +7917,9 @@
       </c>
       <c r="BJ47" s="15" t="n">
         <v>6894.77</v>
+      </c>
+      <c r="BK47" s="15" t="n">
+        <v>6863.63</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -7917,6 +8033,7 @@
       <c r="BH48" s="15" t="n"/>
       <c r="BI48" s="15" t="n"/>
       <c r="BJ48" s="15" t="n"/>
+      <c r="BK48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -8104,6 +8221,9 @@
       </c>
       <c r="BJ49" s="15" t="n">
         <v>29.48</v>
+      </c>
+      <c r="BK49" s="15" t="n">
+        <v>28.6</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -8243,6 +8363,9 @@
         <v>3844.57</v>
       </c>
       <c r="BJ50" s="15" t="n">
+        <v>34036.07</v>
+      </c>
+      <c r="BK50" s="15" t="n">
         <v>34036.07</v>
       </c>
     </row>
@@ -8357,6 +8480,7 @@
       <c r="BH51" s="15" t="n"/>
       <c r="BI51" s="15" t="n"/>
       <c r="BJ51" s="15" t="n"/>
+      <c r="BK51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -8544,6 +8668,9 @@
       </c>
       <c r="BJ52" s="15" t="n">
         <v>48.36</v>
+      </c>
+      <c r="BK52" s="15" t="n">
+        <v>49.24</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -8684,6 +8811,9 @@
       </c>
       <c r="BJ53" s="15" t="n">
         <v>3807.97</v>
+      </c>
+      <c r="BK53" s="15" t="n">
+        <v>3853.98</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -8797,6 +8927,7 @@
       <c r="BH54" s="15" t="n"/>
       <c r="BI54" s="15" t="n"/>
       <c r="BJ54" s="15" t="n"/>
+      <c r="BK54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -8984,6 +9115,9 @@
       </c>
       <c r="BJ55" s="15" t="n">
         <v>59.94</v>
+      </c>
+      <c r="BK55" s="15" t="n">
+        <v>60.76</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -9124,6 +9258,9 @@
       </c>
       <c r="BJ56" s="15" t="n">
         <v>3626.3</v>
+      </c>
+      <c r="BK56" s="15" t="n">
+        <v>3674.68</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -9237,6 +9374,7 @@
       <c r="BH57" s="15" t="n"/>
       <c r="BI57" s="15" t="n"/>
       <c r="BJ57" s="15" t="n"/>
+      <c r="BK57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -9424,6 +9562,9 @@
       </c>
       <c r="BJ58" s="15" t="n">
         <v>21.3</v>
+      </c>
+      <c r="BK58" s="15" t="n">
+        <v>19.34</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -9564,6 +9705,9 @@
       </c>
       <c r="BJ59" s="15" t="n">
         <v>6949.47</v>
+      </c>
+      <c r="BK59" s="15" t="n">
+        <v>6982.33</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -9677,6 +9821,7 @@
       <c r="BH60" s="15" t="n"/>
       <c r="BI60" s="15" t="n"/>
       <c r="BJ60" s="15" t="n"/>
+      <c r="BK60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -9864,6 +10009,9 @@
       </c>
       <c r="BJ61" s="15" t="n">
         <v>40.71</v>
+      </c>
+      <c r="BK61" s="15" t="n">
+        <v>37.99</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -10004,6 +10152,9 @@
       </c>
       <c r="BJ62" s="15" t="n">
         <v>8487.139999999999</v>
+      </c>
+      <c r="BK62" s="15" t="n">
+        <v>8616.85</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -10117,6 +10268,7 @@
       <c r="BH63" s="15" t="n"/>
       <c r="BI63" s="15" t="n"/>
       <c r="BJ63" s="15" t="n"/>
+      <c r="BK63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -10304,6 +10456,9 @@
       </c>
       <c r="BJ64" s="15" t="n">
         <v>4.75</v>
+      </c>
+      <c r="BK64" s="15" t="n">
+        <v>3.92</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -10444,6 +10599,9 @@
       </c>
       <c r="BJ65" s="15" t="n">
         <v>10787.19</v>
+      </c>
+      <c r="BK65" s="15" t="n">
+        <v>10666.47</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -10557,6 +10715,7 @@
       <c r="BH66" s="15" t="n"/>
       <c r="BI66" s="15" t="n"/>
       <c r="BJ66" s="15" t="n"/>
+      <c r="BK66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -10744,6 +10903,9 @@
       </c>
       <c r="BJ67" s="15" t="n">
         <v>20.6</v>
+      </c>
+      <c r="BK67" s="15" t="n">
+        <v>18.93</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -10884,6 +11046,9 @@
       </c>
       <c r="BJ68" s="15" t="n">
         <v>11572.3</v>
+      </c>
+      <c r="BK68" s="15" t="n">
+        <v>11436</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -10997,6 +11162,7 @@
       <c r="BH69" s="15" t="n"/>
       <c r="BI69" s="15" t="n"/>
       <c r="BJ69" s="15" t="n"/>
+      <c r="BK69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -11184,6 +11350,9 @@
       </c>
       <c r="BJ70" s="15" t="n">
         <v>19.85</v>
+      </c>
+      <c r="BK70" s="15" t="n">
+        <v>18.54</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -11324,6 +11493,9 @@
       </c>
       <c r="BJ71" s="15" t="n">
         <v>6804.46</v>
+      </c>
+      <c r="BK71" s="15" t="n">
+        <v>6582.58</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -11437,6 +11609,7 @@
       <c r="BH72" s="15" t="n"/>
       <c r="BI72" s="15" t="n"/>
       <c r="BJ72" s="15" t="n"/>
+      <c r="BK72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -11624,6 +11797,9 @@
       </c>
       <c r="BJ73" s="15" t="n">
         <v>17.61</v>
+      </c>
+      <c r="BK73" s="15" t="n">
+        <v>15.7</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -11764,6 +11940,9 @@
       </c>
       <c r="BJ74" s="15" t="n">
         <v>12658.53</v>
+      </c>
+      <c r="BK74" s="15" t="n">
+        <v>12465.92</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -11877,6 +12056,7 @@
       <c r="BH75" s="15" t="n"/>
       <c r="BI75" s="15" t="n"/>
       <c r="BJ75" s="15" t="n"/>
+      <c r="BK75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -12064,6 +12244,9 @@
       </c>
       <c r="BJ76" s="15" t="n">
         <v>55.55</v>
+      </c>
+      <c r="BK76" s="15" t="n">
+        <v>54.25</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -12203,6 +12386,9 @@
         <v>7319.35</v>
       </c>
       <c r="BJ77" s="15" t="n">
+        <v>15569.82</v>
+      </c>
+      <c r="BK77" s="15" t="n">
         <v>15569.82</v>
       </c>
     </row>
@@ -12317,6 +12503,7 @@
       <c r="BH78" s="15" t="n"/>
       <c r="BI78" s="15" t="n"/>
       <c r="BJ78" s="15" t="n"/>
+      <c r="BK78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -12504,6 +12691,9 @@
       </c>
       <c r="BJ79" s="15" t="n">
         <v>3.61</v>
+      </c>
+      <c r="BK79" s="15" t="n">
+        <v>3.05</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -12644,6 +12834,9 @@
       </c>
       <c r="BJ80" s="15" t="n">
         <v>6982.18</v>
+      </c>
+      <c r="BK80" s="15" t="n">
+        <v>7086.33</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -12757,6 +12950,7 @@
       <c r="BH81" s="15" t="n"/>
       <c r="BI81" s="15" t="n"/>
       <c r="BJ81" s="15" t="n"/>
+      <c r="BK81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -12944,6 +13138,9 @@
       </c>
       <c r="BJ82" s="15" t="n">
         <v>4.43</v>
+      </c>
+      <c r="BK82" s="15" t="n">
+        <v>5.4</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -13083,6 +13280,9 @@
         <v>2328.48</v>
       </c>
       <c r="BJ83" s="15" t="n">
+        <v>8851.09</v>
+      </c>
+      <c r="BK83" s="15" t="n">
         <v>8851.09</v>
       </c>
     </row>
@@ -13197,6 +13397,7 @@
       <c r="BH84" s="15" t="n"/>
       <c r="BI84" s="15" t="n"/>
       <c r="BJ84" s="15" t="n"/>
+      <c r="BK84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -13384,6 +13585,9 @@
       </c>
       <c r="BJ85" s="15" t="n">
         <v>12.66</v>
+      </c>
+      <c r="BK85" s="15" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -13523,6 +13727,9 @@
         <v>5075.31</v>
       </c>
       <c r="BJ86" s="15" t="n">
+        <v>2631.9</v>
+      </c>
+      <c r="BK86" s="15" t="n">
         <v>2631.9</v>
       </c>
     </row>
@@ -13637,6 +13844,7 @@
       <c r="BH87" s="15" t="n"/>
       <c r="BI87" s="15" t="n"/>
       <c r="BJ87" s="15" t="n"/>
+      <c r="BK87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -13824,6 +14032,9 @@
       </c>
       <c r="BJ88" s="15" t="n">
         <v>28.98</v>
+      </c>
+      <c r="BK88" s="15" t="n">
+        <v>26.31</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -13963,6 +14174,9 @@
         <v>9212.370000000001</v>
       </c>
       <c r="BJ89" s="15" t="n">
+        <v>5075.31</v>
+      </c>
+      <c r="BK89" s="15" t="n">
         <v>5075.31</v>
       </c>
     </row>
@@ -14077,6 +14291,7 @@
       <c r="BH90" s="15" t="n"/>
       <c r="BI90" s="15" t="n"/>
       <c r="BJ90" s="15" t="n"/>
+      <c r="BK90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -14264,6 +14479,9 @@
       </c>
       <c r="BJ91" s="15" t="n">
         <v>30.03</v>
+      </c>
+      <c r="BK91" s="15" t="n">
+        <v>28.97</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -14404,6 +14622,9 @@
       </c>
       <c r="BJ92" s="15" t="n">
         <v>8977.57</v>
+      </c>
+      <c r="BK92" s="15" t="n">
+        <v>9038.370000000001</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -14517,6 +14738,7 @@
       <c r="BH93" s="15" t="n"/>
       <c r="BI93" s="15" t="n"/>
       <c r="BJ93" s="15" t="n"/>
+      <c r="BK93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -14704,6 +14926,9 @@
       </c>
       <c r="BJ94" s="15" t="n">
         <v>4.84</v>
+      </c>
+      <c r="BK94" s="15" t="n">
+        <v>4.08</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -14844,6 +15069,9 @@
       </c>
       <c r="BJ95" s="15" t="n">
         <v>1164.31</v>
+      </c>
+      <c r="BK95" s="15" t="n">
+        <v>1142.31</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -14957,6 +15185,7 @@
       <c r="BH96" s="15" t="n"/>
       <c r="BI96" s="15" t="n"/>
       <c r="BJ96" s="15" t="n"/>
+      <c r="BK96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -15144,6 +15373,9 @@
       </c>
       <c r="BJ97" s="15" t="n">
         <v>8.68</v>
+      </c>
+      <c r="BK97" s="15" t="n">
+        <v>7.95</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -15284,6 +15516,9 @@
       </c>
       <c r="BJ98" s="15" t="n">
         <v>14490.77</v>
+      </c>
+      <c r="BK98" s="15" t="n">
+        <v>14328.89</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -15397,6 +15632,7 @@
       <c r="BH99" s="15" t="n"/>
       <c r="BI99" s="15" t="n"/>
       <c r="BJ99" s="15" t="n"/>
+      <c r="BK99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -15584,6 +15820,9 @@
       </c>
       <c r="BJ100" s="15" t="n">
         <v>53.6</v>
+      </c>
+      <c r="BK100" s="15" t="n">
+        <v>51.84</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -15724,6 +15963,9 @@
       </c>
       <c r="BJ101" s="15" t="n">
         <v>3464.35</v>
+      </c>
+      <c r="BK101" s="15" t="n">
+        <v>3424.68</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -15837,6 +16079,7 @@
       <c r="BH102" s="15" t="n"/>
       <c r="BI102" s="15" t="n"/>
       <c r="BJ102" s="15" t="n"/>
+      <c r="BK102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -16024,6 +16267,9 @@
       </c>
       <c r="BJ103" s="15" t="n">
         <v>38.98</v>
+      </c>
+      <c r="BK103" s="15" t="n">
+        <v>39</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -16164,6 +16410,9 @@
       </c>
       <c r="BJ104" s="15" t="n">
         <v>2512.5</v>
+      </c>
+      <c r="BK104" s="15" t="n">
+        <v>2534.57</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -16277,6 +16526,7 @@
       <c r="BH105" s="15" t="n"/>
       <c r="BI105" s="15" t="n"/>
       <c r="BJ105" s="15" t="n"/>
+      <c r="BK105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -16464,6 +16714,9 @@
       </c>
       <c r="BJ106" s="15" t="n">
         <v>17.08</v>
+      </c>
+      <c r="BK106" s="15" t="n">
+        <v>17.1</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -16604,6 +16857,9 @@
       </c>
       <c r="BJ107" s="15" t="n">
         <v>2494.23</v>
+      </c>
+      <c r="BK107" s="15" t="n">
+        <v>2595.64</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -16717,6 +16973,7 @@
       <c r="BH108" s="15" t="n"/>
       <c r="BI108" s="15" t="n"/>
       <c r="BJ108" s="15" t="n"/>
+      <c r="BK108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -16904,6 +17161,9 @@
       </c>
       <c r="BJ109" s="15" t="n">
         <v>38.79</v>
+      </c>
+      <c r="BK109" s="15" t="n">
+        <v>38.55</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -17044,6 +17304,9 @@
       </c>
       <c r="BJ110" s="15" t="n">
         <v>2663.1</v>
+      </c>
+      <c r="BK110" s="15" t="n">
+        <v>2682.47</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -17157,6 +17420,7 @@
       <c r="BH111" s="15" t="n"/>
       <c r="BI111" s="15" t="n"/>
       <c r="BJ111" s="15" t="n"/>
+      <c r="BK111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -17344,6 +17608,9 @@
       </c>
       <c r="BJ112" s="15" t="n">
         <v>68.48</v>
+      </c>
+      <c r="BK112" s="15" t="n">
+        <v>66.44</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -17482,6 +17749,9 @@
       </c>
       <c r="BJ113" s="15" t="n">
         <v>2098.35</v>
+      </c>
+      <c r="BK113" s="15" t="n">
+        <v>2058.92</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -17595,6 +17865,7 @@
       <c r="BH114" s="15" t="n"/>
       <c r="BI114" s="15" t="n"/>
       <c r="BJ114" s="15" t="n"/>
+      <c r="BK114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -17782,6 +18053,9 @@
       </c>
       <c r="BJ115" s="15" t="n">
         <v>23.93</v>
+      </c>
+      <c r="BK115" s="15" t="n">
+        <v>23.36</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -17907,6 +18181,9 @@
       </c>
       <c r="BJ116" s="15" t="n">
         <v>8929.530000000001</v>
+      </c>
+      <c r="BK116" s="15" t="n">
+        <v>8885.33</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -17975,6 +18252,7 @@
       <c r="BH117" s="15" t="n"/>
       <c r="BI117" s="15" t="n"/>
       <c r="BJ117" s="15" t="n"/>
+      <c r="BK117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -18118,6 +18396,9 @@
       <c r="BJ118" s="15" t="n">
         <v>95.43000000000001</v>
       </c>
+      <c r="BK118" s="15" t="n">
+        <v>95.28</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -18233,6 +18514,9 @@
       </c>
       <c r="BJ119" s="15" t="n">
         <v>13493.35</v>
+      </c>
+      <c r="BK119" s="15" t="n">
+        <v>14112.07</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -18250,6 +18534,7 @@
       <c r="BH120" s="15" t="n"/>
       <c r="BI120" s="15" t="n"/>
       <c r="BJ120" s="15" t="n"/>
+      <c r="BK120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -18294,6 +18579,9 @@
       <c r="BJ121" s="15" t="n">
         <v>33.08</v>
       </c>
+      <c r="BK121" s="15" t="n">
+        <v>32.84</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -18337,6 +18625,9 @@
       </c>
       <c r="BJ122" s="15" t="n">
         <v>1267.69</v>
+      </c>
+      <c r="BK122" s="15" t="n">
+        <v>1268.16</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -18354,6 +18645,7 @@
       <c r="BH123" s="15" t="n"/>
       <c r="BI123" s="15" t="n"/>
       <c r="BJ123" s="15" t="n"/>
+      <c r="BK123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -18398,6 +18690,9 @@
       <c r="BJ124" s="15" t="n">
         <v>50.05</v>
       </c>
+      <c r="BK124" s="15" t="n">
+        <v>51.09</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -18441,6 +18736,9 @@
       </c>
       <c r="BJ125" s="15" t="n">
         <v>11659.75</v>
+      </c>
+      <c r="BK125" s="15" t="n">
+        <v>11798.3</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -18458,6 +18756,7 @@
       <c r="BH126" s="15" t="n"/>
       <c r="BI126" s="15" t="n"/>
       <c r="BJ126" s="15" t="n"/>
+      <c r="BK126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -18502,6 +18801,9 @@
       <c r="BJ127" s="15" t="n">
         <v>28.6</v>
       </c>
+      <c r="BK127" s="15" t="n">
+        <v>28.25</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -18544,6 +18846,9 @@
         <v>770.39</v>
       </c>
       <c r="BJ128" s="15" t="n">
+        <v>1848.91</v>
+      </c>
+      <c r="BK128" s="15" t="n">
         <v>1848.91</v>
       </c>
     </row>
@@ -18562,6 +18867,7 @@
       <c r="BH129" s="15" t="n"/>
       <c r="BI129" s="15" t="n"/>
       <c r="BJ129" s="15" t="n"/>
+      <c r="BK129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -18606,6 +18912,9 @@
       <c r="BJ130" s="15" t="n">
         <v>15.65</v>
       </c>
+      <c r="BK130" s="15" t="n">
+        <v>13.49</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -18649,6 +18958,9 @@
       </c>
       <c r="BJ131" s="15" t="n">
         <v>756.25</v>
+      </c>
+      <c r="BK131" s="15" t="n">
+        <v>757.58</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -18666,6 +18978,7 @@
       <c r="BH132" s="15" t="n"/>
       <c r="BI132" s="15" t="n"/>
       <c r="BJ132" s="15" t="n"/>
+      <c r="BK132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -18710,6 +19023,9 @@
       <c r="BJ133" s="15" t="n">
         <v>68.02</v>
       </c>
+      <c r="BK133" s="15" t="n">
+        <v>69.27</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -18753,6 +19069,9 @@
       </c>
       <c r="BJ134" s="15" t="n">
         <v>3078.44</v>
+      </c>
+      <c r="BK134" s="15" t="n">
+        <v>3038.41</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -18770,6 +19089,7 @@
       <c r="BH135" s="15" t="n"/>
       <c r="BI135" s="15" t="n"/>
       <c r="BJ135" s="15" t="n"/>
+      <c r="BK135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -18814,6 +19134,9 @@
       <c r="BJ136" s="15" t="n">
         <v>20.8</v>
       </c>
+      <c r="BK136" s="15" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -18857,6 +19180,9 @@
       </c>
       <c r="BJ137" s="15" t="n">
         <v>3603.48</v>
+      </c>
+      <c r="BK137" s="15" t="n">
+        <v>3635.5</v>
       </c>
     </row>
     <row r="138">
@@ -18866,6 +19192,7 @@
       <c r="BH138" s="15" t="n"/>
       <c r="BI138" s="15" t="n"/>
       <c r="BJ138" s="15" t="n"/>
+      <c r="BK138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -18886,6 +19213,9 @@
       <c r="BJ139" s="15" t="n">
         <v>3.57</v>
       </c>
+      <c r="BK139" s="15" t="n">
+        <v>3.61</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -18904,6 +19234,9 @@
         <v>5685.23</v>
       </c>
       <c r="BJ140" s="15" t="n">
+        <v>2408.81</v>
+      </c>
+      <c r="BK140" s="15" t="n">
         <v>2408.81</v>
       </c>
     </row>
@@ -18914,6 +19247,7 @@
       <c r="BH141" s="15" t="n"/>
       <c r="BI141" s="15" t="n"/>
       <c r="BJ141" s="15" t="n"/>
+      <c r="BK141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -18934,6 +19268,9 @@
       <c r="BJ142" s="15" t="n">
         <v>12.27</v>
       </c>
+      <c r="BK142" s="15" t="n">
+        <v>12.88</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -18954,18 +19291,28 @@
       <c r="BJ143" s="15" t="n">
         <v>5685.23</v>
       </c>
+      <c r="BK143" s="15" t="n">
+        <v>5692.93</v>
+      </c>
     </row>
     <row r="144">
       <c r="BJ144" s="15" t="n"/>
+      <c r="BK144" s="15" t="n"/>
     </row>
     <row r="145">
       <c r="BJ145" s="15" t="n">
         <v>24.82</v>
       </c>
+      <c r="BK145" s="15" t="n">
+        <v>24.53</v>
+      </c>
     </row>
     <row r="146">
       <c r="BJ146" s="15" t="n">
         <v>2304.53</v>
+      </c>
+      <c r="BK146" s="15" t="n">
+        <v>2279.97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-08-20 04:14:56]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BK146"/>
+  <dimension ref="A1:BL146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -597,6 +597,7 @@
     <col width="15" customWidth="1" min="61" max="61"/>
     <col width="15" customWidth="1" min="62" max="62"/>
     <col width="15" customWidth="1" min="63" max="63"/>
+    <col width="15" customWidth="1" min="64" max="64"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -915,6 +916,11 @@
           <t>2026/08/17</t>
         </is>
       </c>
+      <c r="BL1" s="15" t="inlineStr">
+        <is>
+          <t>2026/08/20</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1232,6 +1238,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BL2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1423,6 +1434,9 @@
       <c r="BK3" s="15" t="n">
         <v>67.41</v>
       </c>
+      <c r="BL3" s="15" t="n">
+        <v>67.75</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1613,6 +1627,9 @@
       </c>
       <c r="BK4" s="15" t="n">
         <v>3960.19</v>
+      </c>
+      <c r="BL4" s="15" t="n">
+        <v>3905.23</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1679,6 +1696,7 @@
       <c r="BI5" s="15" t="n"/>
       <c r="BJ5" s="15" t="n"/>
       <c r="BK5" s="15" t="n"/>
+      <c r="BL5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1792,6 +1810,7 @@
       <c r="BI6" s="15" t="n"/>
       <c r="BJ6" s="15" t="n"/>
       <c r="BK6" s="15" t="n"/>
+      <c r="BL6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -1982,6 +2001,9 @@
       </c>
       <c r="BK7" s="15" t="n">
         <v>63.26</v>
+      </c>
+      <c r="BL7" s="15" t="n">
+        <v>61.88</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -2125,6 +2147,9 @@
       </c>
       <c r="BK8" s="15" t="n">
         <v>5860.01</v>
+      </c>
+      <c r="BL8" s="15" t="n">
+        <v>5708.49</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2239,6 +2264,7 @@
       <c r="BI9" s="15" t="n"/>
       <c r="BJ9" s="15" t="n"/>
       <c r="BK9" s="15" t="n"/>
+      <c r="BL9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2429,6 +2455,9 @@
       </c>
       <c r="BK10" s="15" t="n">
         <v>54.67</v>
+      </c>
+      <c r="BL10" s="15" t="n">
+        <v>54.69</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2572,6 +2601,9 @@
       </c>
       <c r="BK11" s="15" t="n">
         <v>4701.19</v>
+      </c>
+      <c r="BL11" s="15" t="n">
+        <v>4593.48</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -2686,6 +2718,7 @@
       <c r="BI12" s="15" t="n"/>
       <c r="BJ12" s="15" t="n"/>
       <c r="BK12" s="15" t="n"/>
+      <c r="BL12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2876,6 +2909,9 @@
       </c>
       <c r="BK13" s="15" t="n">
         <v>66.69</v>
+      </c>
+      <c r="BL13" s="15" t="n">
+        <v>64.73999999999999</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -3019,6 +3055,9 @@
       </c>
       <c r="BK14" s="15" t="n">
         <v>8119.26</v>
+      </c>
+      <c r="BL14" s="15" t="n">
+        <v>7880.34</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -3133,6 +3172,7 @@
       <c r="BI15" s="15" t="n"/>
       <c r="BJ15" s="15" t="n"/>
       <c r="BK15" s="15" t="n"/>
+      <c r="BL15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -3323,6 +3363,9 @@
       </c>
       <c r="BK16" s="15" t="n">
         <v>35.16</v>
+      </c>
+      <c r="BL16" s="15" t="n">
+        <v>36.73</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -3466,6 +3509,9 @@
       </c>
       <c r="BK17" s="15" t="n">
         <v>2600.68</v>
+      </c>
+      <c r="BL17" s="15" t="n">
+        <v>2623.75</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -3580,6 +3626,7 @@
       <c r="BI18" s="15" t="n"/>
       <c r="BJ18" s="15" t="n"/>
       <c r="BK18" s="15" t="n"/>
+      <c r="BL18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -3770,6 +3817,9 @@
       </c>
       <c r="BK19" s="15" t="n">
         <v>81.91</v>
+      </c>
+      <c r="BL19" s="15" t="n">
+        <v>81.95999999999999</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -3913,6 +3963,9 @@
       </c>
       <c r="BK20" s="15" t="n">
         <v>7785.76</v>
+      </c>
+      <c r="BL20" s="15" t="n">
+        <v>7707.98</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -4027,6 +4080,7 @@
       <c r="BI21" s="15" t="n"/>
       <c r="BJ21" s="15" t="n"/>
       <c r="BK21" s="15" t="n"/>
+      <c r="BL21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -4214,6 +4268,9 @@
         <v>36.34</v>
       </c>
       <c r="BK22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BL22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -4358,6 +4415,9 @@
       </c>
       <c r="BK23" s="15" t="n">
         <v>77661.00999999999</v>
+      </c>
+      <c r="BL23" s="15" t="n">
+        <v>77400.38</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -4472,6 +4532,7 @@
       <c r="BI24" s="15" t="n"/>
       <c r="BJ24" s="15" t="n"/>
       <c r="BK24" s="15" t="n"/>
+      <c r="BL24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -4661,6 +4722,9 @@
         <v>49.88</v>
       </c>
       <c r="BK25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BL25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -4791,6 +4855,9 @@
       </c>
       <c r="BK26" s="15" t="n">
         <v>26440.31</v>
+      </c>
+      <c r="BL26" s="15" t="n">
+        <v>26091.33</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -4905,6 +4972,7 @@
       <c r="BI27" s="15" t="n"/>
       <c r="BJ27" s="15" t="n"/>
       <c r="BK27" s="15" t="n"/>
+      <c r="BL27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -5094,6 +5162,9 @@
         <v>92.09</v>
       </c>
       <c r="BK28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BL28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -5238,6 +5309,9 @@
       </c>
       <c r="BK29" s="15" t="n">
         <v>68922.84</v>
+      </c>
+      <c r="BL29" s="15" t="n">
+        <v>66057.83</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -5352,6 +5426,7 @@
       <c r="BI30" s="15" t="n"/>
       <c r="BJ30" s="15" t="n"/>
       <c r="BK30" s="15" t="n"/>
+      <c r="BL30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -5541,6 +5616,9 @@
         <v>97.44</v>
       </c>
       <c r="BK31" s="15" t="n">
+        <v>97.44</v>
+      </c>
+      <c r="BL31" s="15" t="n">
         <v>97.44</v>
       </c>
     </row>
@@ -5685,6 +5763,9 @@
       </c>
       <c r="BK32" s="15" t="n">
         <v>6977.94</v>
+      </c>
+      <c r="BL32" s="15" t="n">
+        <v>6890.82</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -5799,6 +5880,7 @@
       <c r="BI33" s="15" t="n"/>
       <c r="BJ33" s="15" t="n"/>
       <c r="BK33" s="15" t="n"/>
+      <c r="BL33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -5989,6 +6071,9 @@
       </c>
       <c r="BK34" s="15" t="n">
         <v>45.28</v>
+      </c>
+      <c r="BL34" s="15" t="n">
+        <v>46.36</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -6132,6 +6217,9 @@
       </c>
       <c r="BK35" s="15" t="n">
         <v>5488.93</v>
+      </c>
+      <c r="BL35" s="15" t="n">
+        <v>5552.27</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -6246,6 +6334,7 @@
       <c r="BI36" s="15" t="n"/>
       <c r="BJ36" s="15" t="n"/>
       <c r="BK36" s="15" t="n"/>
+      <c r="BL36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -6436,6 +6525,9 @@
       </c>
       <c r="BK37" s="15" t="n">
         <v>59.88</v>
+      </c>
+      <c r="BL37" s="15" t="n">
+        <v>57.2</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -6579,6 +6671,9 @@
       </c>
       <c r="BK38" s="15" t="n">
         <v>11206.89</v>
+      </c>
+      <c r="BL38" s="15" t="n">
+        <v>11289.09</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -6693,6 +6788,7 @@
       <c r="BI39" s="15" t="n"/>
       <c r="BJ39" s="15" t="n"/>
       <c r="BK39" s="15" t="n"/>
+      <c r="BL39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -6883,6 +6979,9 @@
       </c>
       <c r="BK40" s="15" t="n">
         <v>49.99</v>
+      </c>
+      <c r="BL40" s="15" t="n">
+        <v>51.05</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -7026,6 +7125,9 @@
       </c>
       <c r="BK41" s="15" t="n">
         <v>10655.59</v>
+      </c>
+      <c r="BL41" s="15" t="n">
+        <v>10852.25</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -7140,6 +7242,7 @@
       <c r="BI42" s="15" t="n"/>
       <c r="BJ42" s="15" t="n"/>
       <c r="BK42" s="15" t="n"/>
+      <c r="BL42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -7330,6 +7433,9 @@
       </c>
       <c r="BK43" s="15" t="n">
         <v>50.16</v>
+      </c>
+      <c r="BL43" s="15" t="n">
+        <v>50.47</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -7473,6 +7579,9 @@
       </c>
       <c r="BK44" s="15" t="n">
         <v>3206.98</v>
+      </c>
+      <c r="BL44" s="15" t="n">
+        <v>3279.14</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -7587,6 +7696,7 @@
       <c r="BI45" s="15" t="n"/>
       <c r="BJ45" s="15" t="n"/>
       <c r="BK45" s="15" t="n"/>
+      <c r="BL45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -7777,6 +7887,9 @@
       </c>
       <c r="BK46" s="15" t="n">
         <v>59.64</v>
+      </c>
+      <c r="BL46" s="15" t="n">
+        <v>58.78</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -7920,6 +8033,9 @@
       </c>
       <c r="BK47" s="15" t="n">
         <v>6863.63</v>
+      </c>
+      <c r="BL47" s="15" t="n">
+        <v>6943.53</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -8034,6 +8150,7 @@
       <c r="BI48" s="15" t="n"/>
       <c r="BJ48" s="15" t="n"/>
       <c r="BK48" s="15" t="n"/>
+      <c r="BL48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -8224,6 +8341,9 @@
       </c>
       <c r="BK49" s="15" t="n">
         <v>28.6</v>
+      </c>
+      <c r="BL49" s="15" t="n">
+        <v>27.79</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -8367,6 +8487,9 @@
       </c>
       <c r="BK50" s="15" t="n">
         <v>34036.07</v>
+      </c>
+      <c r="BL50" s="15" t="n">
+        <v>34069.12</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -8481,6 +8604,7 @@
       <c r="BI51" s="15" t="n"/>
       <c r="BJ51" s="15" t="n"/>
       <c r="BK51" s="15" t="n"/>
+      <c r="BL51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -8671,6 +8795,9 @@
       </c>
       <c r="BK52" s="15" t="n">
         <v>49.24</v>
+      </c>
+      <c r="BL52" s="15" t="n">
+        <v>45.97</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -8814,6 +8941,9 @@
       </c>
       <c r="BK53" s="15" t="n">
         <v>3853.98</v>
+      </c>
+      <c r="BL53" s="15" t="n">
+        <v>3672.37</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -8928,6 +9058,7 @@
       <c r="BI54" s="15" t="n"/>
       <c r="BJ54" s="15" t="n"/>
       <c r="BK54" s="15" t="n"/>
+      <c r="BL54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -9118,6 +9249,9 @@
       </c>
       <c r="BK55" s="15" t="n">
         <v>60.76</v>
+      </c>
+      <c r="BL55" s="15" t="n">
+        <v>54.56</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -9261,6 +9395,9 @@
       </c>
       <c r="BK56" s="15" t="n">
         <v>3674.68</v>
+      </c>
+      <c r="BL56" s="15" t="n">
+        <v>3509.44</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -9375,6 +9512,7 @@
       <c r="BI57" s="15" t="n"/>
       <c r="BJ57" s="15" t="n"/>
       <c r="BK57" s="15" t="n"/>
+      <c r="BL57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -9565,6 +9703,9 @@
       </c>
       <c r="BK58" s="15" t="n">
         <v>19.34</v>
+      </c>
+      <c r="BL58" s="15" t="n">
+        <v>18.1</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -9708,6 +9849,9 @@
       </c>
       <c r="BK59" s="15" t="n">
         <v>6982.33</v>
+      </c>
+      <c r="BL59" s="15" t="n">
+        <v>7188</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -9822,6 +9966,7 @@
       <c r="BI60" s="15" t="n"/>
       <c r="BJ60" s="15" t="n"/>
       <c r="BK60" s="15" t="n"/>
+      <c r="BL60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -10012,6 +10157,9 @@
       </c>
       <c r="BK61" s="15" t="n">
         <v>37.99</v>
+      </c>
+      <c r="BL61" s="15" t="n">
+        <v>37.71</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -10155,6 +10303,9 @@
       </c>
       <c r="BK62" s="15" t="n">
         <v>8616.85</v>
+      </c>
+      <c r="BL62" s="15" t="n">
+        <v>8728.530000000001</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -10269,6 +10420,7 @@
       <c r="BI63" s="15" t="n"/>
       <c r="BJ63" s="15" t="n"/>
       <c r="BK63" s="15" t="n"/>
+      <c r="BL63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -10459,6 +10611,9 @@
       </c>
       <c r="BK64" s="15" t="n">
         <v>3.92</v>
+      </c>
+      <c r="BL64" s="15" t="n">
+        <v>3.59</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -10602,6 +10757,9 @@
       </c>
       <c r="BK65" s="15" t="n">
         <v>10666.47</v>
+      </c>
+      <c r="BL65" s="15" t="n">
+        <v>10763.09</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -10716,6 +10874,7 @@
       <c r="BI66" s="15" t="n"/>
       <c r="BJ66" s="15" t="n"/>
       <c r="BK66" s="15" t="n"/>
+      <c r="BL66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -10906,6 +11065,9 @@
       </c>
       <c r="BK67" s="15" t="n">
         <v>18.93</v>
+      </c>
+      <c r="BL67" s="15" t="n">
+        <v>19.99</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -11049,6 +11211,9 @@
       </c>
       <c r="BK68" s="15" t="n">
         <v>11436</v>
+      </c>
+      <c r="BL68" s="15" t="n">
+        <v>11366.98</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -11163,6 +11328,7 @@
       <c r="BI69" s="15" t="n"/>
       <c r="BJ69" s="15" t="n"/>
       <c r="BK69" s="15" t="n"/>
+      <c r="BL69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -11353,6 +11519,9 @@
       </c>
       <c r="BK70" s="15" t="n">
         <v>18.54</v>
+      </c>
+      <c r="BL70" s="15" t="n">
+        <v>14.89</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -11496,6 +11665,9 @@
       </c>
       <c r="BK71" s="15" t="n">
         <v>6582.58</v>
+      </c>
+      <c r="BL71" s="15" t="n">
+        <v>6537.61</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -11610,6 +11782,7 @@
       <c r="BI72" s="15" t="n"/>
       <c r="BJ72" s="15" t="n"/>
       <c r="BK72" s="15" t="n"/>
+      <c r="BL72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -11800,6 +11973,9 @@
       </c>
       <c r="BK73" s="15" t="n">
         <v>15.7</v>
+      </c>
+      <c r="BL73" s="15" t="n">
+        <v>13.71</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -11943,6 +12119,9 @@
       </c>
       <c r="BK74" s="15" t="n">
         <v>12465.92</v>
+      </c>
+      <c r="BL74" s="15" t="n">
+        <v>12503.52</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -12057,6 +12236,7 @@
       <c r="BI75" s="15" t="n"/>
       <c r="BJ75" s="15" t="n"/>
       <c r="BK75" s="15" t="n"/>
+      <c r="BL75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -12247,6 +12427,9 @@
       </c>
       <c r="BK76" s="15" t="n">
         <v>54.25</v>
+      </c>
+      <c r="BL76" s="15" t="n">
+        <v>55.03</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -12389,6 +12572,9 @@
         <v>15569.82</v>
       </c>
       <c r="BK77" s="15" t="n">
+        <v>15569.82</v>
+      </c>
+      <c r="BL77" s="15" t="n">
         <v>15569.82</v>
       </c>
     </row>
@@ -12504,6 +12690,7 @@
       <c r="BI78" s="15" t="n"/>
       <c r="BJ78" s="15" t="n"/>
       <c r="BK78" s="15" t="n"/>
+      <c r="BL78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -12694,6 +12881,9 @@
       </c>
       <c r="BK79" s="15" t="n">
         <v>3.05</v>
+      </c>
+      <c r="BL79" s="15" t="n">
+        <v>3.42</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -12837,6 +13027,9 @@
       </c>
       <c r="BK80" s="15" t="n">
         <v>7086.33</v>
+      </c>
+      <c r="BL80" s="15" t="n">
+        <v>7254.7</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -12951,6 +13144,7 @@
       <c r="BI81" s="15" t="n"/>
       <c r="BJ81" s="15" t="n"/>
       <c r="BK81" s="15" t="n"/>
+      <c r="BL81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -13141,6 +13335,9 @@
       </c>
       <c r="BK82" s="15" t="n">
         <v>5.4</v>
+      </c>
+      <c r="BL82" s="15" t="n">
+        <v>4.42</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -13284,6 +13481,9 @@
       </c>
       <c r="BK83" s="15" t="n">
         <v>8851.09</v>
+      </c>
+      <c r="BL83" s="15" t="n">
+        <v>8669.940000000001</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -13398,6 +13598,7 @@
       <c r="BI84" s="15" t="n"/>
       <c r="BJ84" s="15" t="n"/>
       <c r="BK84" s="15" t="n"/>
+      <c r="BL84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -13588,6 +13789,9 @@
       </c>
       <c r="BK85" s="15" t="n">
         <v>12</v>
+      </c>
+      <c r="BL85" s="15" t="n">
+        <v>12.77</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -13730,6 +13934,9 @@
         <v>2631.9</v>
       </c>
       <c r="BK86" s="15" t="n">
+        <v>2631.9</v>
+      </c>
+      <c r="BL86" s="15" t="n">
         <v>2631.9</v>
       </c>
     </row>
@@ -13845,6 +14052,7 @@
       <c r="BI87" s="15" t="n"/>
       <c r="BJ87" s="15" t="n"/>
       <c r="BK87" s="15" t="n"/>
+      <c r="BL87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -14035,6 +14243,9 @@
       </c>
       <c r="BK88" s="15" t="n">
         <v>26.31</v>
+      </c>
+      <c r="BL88" s="15" t="n">
+        <v>27.99</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -14177,6 +14388,9 @@
         <v>5075.31</v>
       </c>
       <c r="BK89" s="15" t="n">
+        <v>5075.31</v>
+      </c>
+      <c r="BL89" s="15" t="n">
         <v>5075.31</v>
       </c>
     </row>
@@ -14292,6 +14506,7 @@
       <c r="BI90" s="15" t="n"/>
       <c r="BJ90" s="15" t="n"/>
       <c r="BK90" s="15" t="n"/>
+      <c r="BL90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -14482,6 +14697,9 @@
       </c>
       <c r="BK91" s="15" t="n">
         <v>28.97</v>
+      </c>
+      <c r="BL91" s="15" t="n">
+        <v>25.76</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -14625,6 +14843,9 @@
       </c>
       <c r="BK92" s="15" t="n">
         <v>9038.370000000001</v>
+      </c>
+      <c r="BL92" s="15" t="n">
+        <v>9209.950000000001</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -14739,6 +14960,7 @@
       <c r="BI93" s="15" t="n"/>
       <c r="BJ93" s="15" t="n"/>
       <c r="BK93" s="15" t="n"/>
+      <c r="BL93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -14929,6 +15151,9 @@
       </c>
       <c r="BK94" s="15" t="n">
         <v>4.08</v>
+      </c>
+      <c r="BL94" s="15" t="n">
+        <v>4.04</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -15072,6 +15297,9 @@
       </c>
       <c r="BK95" s="15" t="n">
         <v>1142.31</v>
+      </c>
+      <c r="BL95" s="15" t="n">
+        <v>1148.76</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -15186,6 +15414,7 @@
       <c r="BI96" s="15" t="n"/>
       <c r="BJ96" s="15" t="n"/>
       <c r="BK96" s="15" t="n"/>
+      <c r="BL96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -15376,6 +15605,9 @@
       </c>
       <c r="BK97" s="15" t="n">
         <v>7.95</v>
+      </c>
+      <c r="BL97" s="15" t="n">
+        <v>6.9</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -15519,6 +15751,9 @@
       </c>
       <c r="BK98" s="15" t="n">
         <v>14328.89</v>
+      </c>
+      <c r="BL98" s="15" t="n">
+        <v>14018.67</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -15633,6 +15868,7 @@
       <c r="BI99" s="15" t="n"/>
       <c r="BJ99" s="15" t="n"/>
       <c r="BK99" s="15" t="n"/>
+      <c r="BL99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -15823,6 +16059,9 @@
       </c>
       <c r="BK100" s="15" t="n">
         <v>51.84</v>
+      </c>
+      <c r="BL100" s="15" t="n">
+        <v>50.19</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -15966,6 +16205,9 @@
       </c>
       <c r="BK101" s="15" t="n">
         <v>3424.68</v>
+      </c>
+      <c r="BL101" s="15" t="n">
+        <v>3354.61</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -16080,6 +16322,7 @@
       <c r="BI102" s="15" t="n"/>
       <c r="BJ102" s="15" t="n"/>
       <c r="BK102" s="15" t="n"/>
+      <c r="BL102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -16270,6 +16513,9 @@
       </c>
       <c r="BK103" s="15" t="n">
         <v>39</v>
+      </c>
+      <c r="BL103" s="15" t="n">
+        <v>36.5</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -16413,6 +16659,9 @@
       </c>
       <c r="BK104" s="15" t="n">
         <v>2534.57</v>
+      </c>
+      <c r="BL104" s="15" t="n">
+        <v>2446.66</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -16527,6 +16776,7 @@
       <c r="BI105" s="15" t="n"/>
       <c r="BJ105" s="15" t="n"/>
       <c r="BK105" s="15" t="n"/>
+      <c r="BL105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -16717,6 +16967,9 @@
       </c>
       <c r="BK106" s="15" t="n">
         <v>17.1</v>
+      </c>
+      <c r="BL106" s="15" t="n">
+        <v>14.65</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -16859,6 +17112,9 @@
         <v>2494.23</v>
       </c>
       <c r="BK107" s="15" t="n">
+        <v>2595.64</v>
+      </c>
+      <c r="BL107" s="15" t="n">
         <v>2595.64</v>
       </c>
     </row>
@@ -16974,6 +17230,7 @@
       <c r="BI108" s="15" t="n"/>
       <c r="BJ108" s="15" t="n"/>
       <c r="BK108" s="15" t="n"/>
+      <c r="BL108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -17164,6 +17421,9 @@
       </c>
       <c r="BK109" s="15" t="n">
         <v>38.55</v>
+      </c>
+      <c r="BL109" s="15" t="n">
+        <v>36.81</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -17307,6 +17567,9 @@
       </c>
       <c r="BK110" s="15" t="n">
         <v>2682.47</v>
+      </c>
+      <c r="BL110" s="15" t="n">
+        <v>2591.86</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -17421,6 +17684,7 @@
       <c r="BI111" s="15" t="n"/>
       <c r="BJ111" s="15" t="n"/>
       <c r="BK111" s="15" t="n"/>
+      <c r="BL111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -17611,6 +17875,9 @@
       </c>
       <c r="BK112" s="15" t="n">
         <v>66.44</v>
+      </c>
+      <c r="BL112" s="15" t="n">
+        <v>64.62</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -17752,6 +18019,9 @@
       </c>
       <c r="BK113" s="15" t="n">
         <v>2058.92</v>
+      </c>
+      <c r="BL113" s="15" t="n">
+        <v>2116.41</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -17866,6 +18136,7 @@
       <c r="BI114" s="15" t="n"/>
       <c r="BJ114" s="15" t="n"/>
       <c r="BK114" s="15" t="n"/>
+      <c r="BL114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -18056,6 +18327,9 @@
       </c>
       <c r="BK115" s="15" t="n">
         <v>23.36</v>
+      </c>
+      <c r="BL115" s="15" t="n">
+        <v>21.36</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -18184,6 +18458,9 @@
       </c>
       <c r="BK116" s="15" t="n">
         <v>8885.33</v>
+      </c>
+      <c r="BL116" s="15" t="n">
+        <v>9144.950000000001</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -18253,6 +18530,7 @@
       <c r="BI117" s="15" t="n"/>
       <c r="BJ117" s="15" t="n"/>
       <c r="BK117" s="15" t="n"/>
+      <c r="BL117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -18399,6 +18677,9 @@
       <c r="BK118" s="15" t="n">
         <v>95.28</v>
       </c>
+      <c r="BL118" s="15" t="n">
+        <v>90.3</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -18517,6 +18798,9 @@
       </c>
       <c r="BK119" s="15" t="n">
         <v>14112.07</v>
+      </c>
+      <c r="BL119" s="15" t="n">
+        <v>13057.27</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -18535,6 +18819,7 @@
       <c r="BI120" s="15" t="n"/>
       <c r="BJ120" s="15" t="n"/>
       <c r="BK120" s="15" t="n"/>
+      <c r="BL120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -18582,6 +18867,9 @@
       <c r="BK121" s="15" t="n">
         <v>32.84</v>
       </c>
+      <c r="BL121" s="15" t="n">
+        <v>26.66</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -18628,6 +18916,9 @@
       </c>
       <c r="BK122" s="15" t="n">
         <v>1268.16</v>
+      </c>
+      <c r="BL122" s="15" t="n">
+        <v>1192.72</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -18646,6 +18937,7 @@
       <c r="BI123" s="15" t="n"/>
       <c r="BJ123" s="15" t="n"/>
       <c r="BK123" s="15" t="n"/>
+      <c r="BL123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -18693,6 +18985,9 @@
       <c r="BK124" s="15" t="n">
         <v>51.09</v>
       </c>
+      <c r="BL124" s="15" t="n">
+        <v>43.31</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -18739,6 +19034,9 @@
       </c>
       <c r="BK125" s="15" t="n">
         <v>11798.3</v>
+      </c>
+      <c r="BL125" s="15" t="n">
+        <v>11216.97</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -18757,6 +19055,7 @@
       <c r="BI126" s="15" t="n"/>
       <c r="BJ126" s="15" t="n"/>
       <c r="BK126" s="15" t="n"/>
+      <c r="BL126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -18804,6 +19103,9 @@
       <c r="BK127" s="15" t="n">
         <v>28.25</v>
       </c>
+      <c r="BL127" s="15" t="n">
+        <v>28.17</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -18850,6 +19152,9 @@
       </c>
       <c r="BK128" s="15" t="n">
         <v>1848.91</v>
+      </c>
+      <c r="BL128" s="15" t="n">
+        <v>1862.02</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -18868,6 +19173,7 @@
       <c r="BI129" s="15" t="n"/>
       <c r="BJ129" s="15" t="n"/>
       <c r="BK129" s="15" t="n"/>
+      <c r="BL129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -18915,6 +19221,9 @@
       <c r="BK130" s="15" t="n">
         <v>13.49</v>
       </c>
+      <c r="BL130" s="15" t="n">
+        <v>9.640000000000001</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -18961,6 +19270,9 @@
       </c>
       <c r="BK131" s="15" t="n">
         <v>757.58</v>
+      </c>
+      <c r="BL131" s="15" t="n">
+        <v>736.96</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -18979,6 +19291,7 @@
       <c r="BI132" s="15" t="n"/>
       <c r="BJ132" s="15" t="n"/>
       <c r="BK132" s="15" t="n"/>
+      <c r="BL132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -19026,6 +19339,9 @@
       <c r="BK133" s="15" t="n">
         <v>69.27</v>
       </c>
+      <c r="BL133" s="15" t="n">
+        <v>68.45999999999999</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -19072,6 +19388,9 @@
       </c>
       <c r="BK134" s="15" t="n">
         <v>3038.41</v>
+      </c>
+      <c r="BL134" s="15" t="n">
+        <v>2974.54</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -19090,6 +19409,7 @@
       <c r="BI135" s="15" t="n"/>
       <c r="BJ135" s="15" t="n"/>
       <c r="BK135" s="15" t="n"/>
+      <c r="BL135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -19137,6 +19457,9 @@
       <c r="BK136" s="15" t="n">
         <v>20.69</v>
       </c>
+      <c r="BL136" s="15" t="n">
+        <v>19.62</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -19183,6 +19506,9 @@
       </c>
       <c r="BK137" s="15" t="n">
         <v>3635.5</v>
+      </c>
+      <c r="BL137" s="15" t="n">
+        <v>3556.93</v>
       </c>
     </row>
     <row r="138">
@@ -19193,6 +19519,7 @@
       <c r="BI138" s="15" t="n"/>
       <c r="BJ138" s="15" t="n"/>
       <c r="BK138" s="15" t="n"/>
+      <c r="BL138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -19216,6 +19543,9 @@
       <c r="BK139" s="15" t="n">
         <v>3.61</v>
       </c>
+      <c r="BL139" s="15" t="n">
+        <v>3.33</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -19238,6 +19568,9 @@
       </c>
       <c r="BK140" s="15" t="n">
         <v>2408.81</v>
+      </c>
+      <c r="BL140" s="15" t="n">
+        <v>2400.76</v>
       </c>
     </row>
     <row r="141">
@@ -19248,6 +19581,7 @@
       <c r="BI141" s="15" t="n"/>
       <c r="BJ141" s="15" t="n"/>
       <c r="BK141" s="15" t="n"/>
+      <c r="BL141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -19271,6 +19605,9 @@
       <c r="BK142" s="15" t="n">
         <v>12.88</v>
       </c>
+      <c r="BL142" s="15" t="n">
+        <v>13.57</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -19294,10 +19631,14 @@
       <c r="BK143" s="15" t="n">
         <v>5692.93</v>
       </c>
+      <c r="BL143" s="15" t="n">
+        <v>5746.4</v>
+      </c>
     </row>
     <row r="144">
       <c r="BJ144" s="15" t="n"/>
       <c r="BK144" s="15" t="n"/>
+      <c r="BL144" s="15" t="n"/>
     </row>
     <row r="145">
       <c r="BJ145" s="15" t="n">
@@ -19306,6 +19647,9 @@
       <c r="BK145" s="15" t="n">
         <v>24.53</v>
       </c>
+      <c r="BL145" s="15" t="n">
+        <v>23.96</v>
+      </c>
     </row>
     <row r="146">
       <c r="BJ146" s="15" t="n">
@@ -19313,6 +19657,9 @@
       </c>
       <c r="BK146" s="15" t="n">
         <v>2279.97</v>
+      </c>
+      <c r="BL146" s="15" t="n">
+        <v>2240.49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-08-24 04:27:49]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BL146"/>
+  <dimension ref="A1:BM146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -598,6 +598,7 @@
     <col width="15" customWidth="1" min="62" max="62"/>
     <col width="15" customWidth="1" min="63" max="63"/>
     <col width="15" customWidth="1" min="64" max="64"/>
+    <col width="15" customWidth="1" min="65" max="65"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -921,6 +922,11 @@
           <t>2026/08/20</t>
         </is>
       </c>
+      <c r="BM1" s="15" t="inlineStr">
+        <is>
+          <t>2026/08/24</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1243,6 +1249,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BM2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1437,6 +1448,9 @@
       <c r="BL3" s="15" t="n">
         <v>67.75</v>
       </c>
+      <c r="BM3" s="15" t="n">
+        <v>65.34</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1630,6 +1644,9 @@
       </c>
       <c r="BL4" s="15" t="n">
         <v>3905.23</v>
+      </c>
+      <c r="BM4" s="15" t="n">
+        <v>3877.3</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1697,6 +1714,7 @@
       <c r="BJ5" s="15" t="n"/>
       <c r="BK5" s="15" t="n"/>
       <c r="BL5" s="15" t="n"/>
+      <c r="BM5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1811,6 +1829,7 @@
       <c r="BJ6" s="15" t="n"/>
       <c r="BK6" s="15" t="n"/>
       <c r="BL6" s="15" t="n"/>
+      <c r="BM6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -2004,6 +2023,9 @@
       </c>
       <c r="BL7" s="15" t="n">
         <v>61.88</v>
+      </c>
+      <c r="BM7" s="15" t="n">
+        <v>61.63</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -2150,6 +2172,9 @@
       </c>
       <c r="BL8" s="15" t="n">
         <v>5708.49</v>
+      </c>
+      <c r="BM8" s="15" t="n">
+        <v>5631.5</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2265,6 +2290,7 @@
       <c r="BJ9" s="15" t="n"/>
       <c r="BK9" s="15" t="n"/>
       <c r="BL9" s="15" t="n"/>
+      <c r="BM9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2458,6 +2484,9 @@
       </c>
       <c r="BL10" s="15" t="n">
         <v>54.69</v>
+      </c>
+      <c r="BM10" s="15" t="n">
+        <v>53.15</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2604,6 +2633,9 @@
       </c>
       <c r="BL11" s="15" t="n">
         <v>4593.48</v>
+      </c>
+      <c r="BM11" s="15" t="n">
+        <v>4560.85</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -2719,6 +2751,7 @@
       <c r="BJ12" s="15" t="n"/>
       <c r="BK12" s="15" t="n"/>
       <c r="BL12" s="15" t="n"/>
+      <c r="BM12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2912,6 +2945,9 @@
       </c>
       <c r="BL13" s="15" t="n">
         <v>64.73999999999999</v>
+      </c>
+      <c r="BM13" s="15" t="n">
+        <v>64.66</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -3058,6 +3094,9 @@
       </c>
       <c r="BL14" s="15" t="n">
         <v>7880.34</v>
+      </c>
+      <c r="BM14" s="15" t="n">
+        <v>7692.53</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -3173,6 +3212,7 @@
       <c r="BJ15" s="15" t="n"/>
       <c r="BK15" s="15" t="n"/>
       <c r="BL15" s="15" t="n"/>
+      <c r="BM15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -3366,6 +3406,9 @@
       </c>
       <c r="BL16" s="15" t="n">
         <v>36.73</v>
+      </c>
+      <c r="BM16" s="15" t="n">
+        <v>34.68</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -3512,6 +3555,9 @@
       </c>
       <c r="BL17" s="15" t="n">
         <v>2623.75</v>
+      </c>
+      <c r="BM17" s="15" t="n">
+        <v>2562.04</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -3627,6 +3673,7 @@
       <c r="BJ18" s="15" t="n"/>
       <c r="BK18" s="15" t="n"/>
       <c r="BL18" s="15" t="n"/>
+      <c r="BM18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -3820,6 +3867,9 @@
       </c>
       <c r="BL19" s="15" t="n">
         <v>81.95999999999999</v>
+      </c>
+      <c r="BM19" s="15" t="n">
+        <v>81.02</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -3966,6 +4016,9 @@
       </c>
       <c r="BL20" s="15" t="n">
         <v>7707.98</v>
+      </c>
+      <c r="BM20" s="15" t="n">
+        <v>7674.37</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -4081,6 +4134,7 @@
       <c r="BJ21" s="15" t="n"/>
       <c r="BK21" s="15" t="n"/>
       <c r="BL21" s="15" t="n"/>
+      <c r="BM21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -4271,6 +4325,9 @@
         <v>36.34</v>
       </c>
       <c r="BL22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BM22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -4418,6 +4475,9 @@
       </c>
       <c r="BL23" s="15" t="n">
         <v>77400.38</v>
+      </c>
+      <c r="BM23" s="15" t="n">
+        <v>77678.35000000001</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -4533,6 +4593,7 @@
       <c r="BJ24" s="15" t="n"/>
       <c r="BK24" s="15" t="n"/>
       <c r="BL24" s="15" t="n"/>
+      <c r="BM24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -4725,6 +4786,9 @@
         <v>49.88</v>
       </c>
       <c r="BL25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BM25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -4858,6 +4922,9 @@
       </c>
       <c r="BL26" s="15" t="n">
         <v>26091.33</v>
+      </c>
+      <c r="BM26" s="15" t="n">
+        <v>26136.56</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -4973,6 +5040,7 @@
       <c r="BJ27" s="15" t="n"/>
       <c r="BK27" s="15" t="n"/>
       <c r="BL27" s="15" t="n"/>
+      <c r="BM27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -5165,6 +5233,9 @@
         <v>92.09</v>
       </c>
       <c r="BL28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BM28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -5312,6 +5383,9 @@
       </c>
       <c r="BL29" s="15" t="n">
         <v>66057.83</v>
+      </c>
+      <c r="BM29" s="15" t="n">
+        <v>65751.64999999999</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -5427,6 +5501,7 @@
       <c r="BJ30" s="15" t="n"/>
       <c r="BK30" s="15" t="n"/>
       <c r="BL30" s="15" t="n"/>
+      <c r="BM30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -5619,6 +5694,9 @@
         <v>97.44</v>
       </c>
       <c r="BL31" s="15" t="n">
+        <v>97.44</v>
+      </c>
+      <c r="BM31" s="15" t="n">
         <v>97.44</v>
       </c>
     </row>
@@ -5766,6 +5844,9 @@
       </c>
       <c r="BL32" s="15" t="n">
         <v>6890.82</v>
+      </c>
+      <c r="BM32" s="15" t="n">
+        <v>6706.38</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -5881,6 +5962,7 @@
       <c r="BJ33" s="15" t="n"/>
       <c r="BK33" s="15" t="n"/>
       <c r="BL33" s="15" t="n"/>
+      <c r="BM33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -6074,6 +6156,9 @@
       </c>
       <c r="BL34" s="15" t="n">
         <v>46.36</v>
+      </c>
+      <c r="BM34" s="15" t="n">
+        <v>45.4</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -6220,6 +6305,9 @@
       </c>
       <c r="BL35" s="15" t="n">
         <v>5552.27</v>
+      </c>
+      <c r="BM35" s="15" t="n">
+        <v>5647.76</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -6335,6 +6423,7 @@
       <c r="BJ36" s="15" t="n"/>
       <c r="BK36" s="15" t="n"/>
       <c r="BL36" s="15" t="n"/>
+      <c r="BM36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -6528,6 +6617,9 @@
       </c>
       <c r="BL37" s="15" t="n">
         <v>57.2</v>
+      </c>
+      <c r="BM37" s="15" t="n">
+        <v>59.25</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -6674,6 +6766,9 @@
       </c>
       <c r="BL38" s="15" t="n">
         <v>11289.09</v>
+      </c>
+      <c r="BM38" s="15" t="n">
+        <v>11266.26</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -6789,6 +6884,7 @@
       <c r="BJ39" s="15" t="n"/>
       <c r="BK39" s="15" t="n"/>
       <c r="BL39" s="15" t="n"/>
+      <c r="BM39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -6982,6 +7078,9 @@
       </c>
       <c r="BL40" s="15" t="n">
         <v>51.05</v>
+      </c>
+      <c r="BM40" s="15" t="n">
+        <v>50.39</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -7128,6 +7227,9 @@
       </c>
       <c r="BL41" s="15" t="n">
         <v>10852.25</v>
+      </c>
+      <c r="BM41" s="15" t="n">
+        <v>10858.77</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -7243,6 +7345,7 @@
       <c r="BJ42" s="15" t="n"/>
       <c r="BK42" s="15" t="n"/>
       <c r="BL42" s="15" t="n"/>
+      <c r="BM42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -7436,6 +7539,9 @@
       </c>
       <c r="BL43" s="15" t="n">
         <v>50.47</v>
+      </c>
+      <c r="BM43" s="15" t="n">
+        <v>50.43</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -7582,6 +7688,9 @@
       </c>
       <c r="BL44" s="15" t="n">
         <v>3279.14</v>
+      </c>
+      <c r="BM44" s="15" t="n">
+        <v>3300.46</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -7697,6 +7806,7 @@
       <c r="BJ45" s="15" t="n"/>
       <c r="BK45" s="15" t="n"/>
       <c r="BL45" s="15" t="n"/>
+      <c r="BM45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -7890,6 +8000,9 @@
       </c>
       <c r="BL46" s="15" t="n">
         <v>58.78</v>
+      </c>
+      <c r="BM46" s="15" t="n">
+        <v>60.95</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -8036,6 +8149,9 @@
       </c>
       <c r="BL47" s="15" t="n">
         <v>6943.53</v>
+      </c>
+      <c r="BM47" s="15" t="n">
+        <v>6897.89</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -8151,6 +8267,7 @@
       <c r="BJ48" s="15" t="n"/>
       <c r="BK48" s="15" t="n"/>
       <c r="BL48" s="15" t="n"/>
+      <c r="BM48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -8344,6 +8461,9 @@
       </c>
       <c r="BL49" s="15" t="n">
         <v>27.79</v>
+      </c>
+      <c r="BM49" s="15" t="n">
+        <v>28.11</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -8490,6 +8610,9 @@
       </c>
       <c r="BL50" s="15" t="n">
         <v>34069.12</v>
+      </c>
+      <c r="BM50" s="15" t="n">
+        <v>33771.36</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -8605,6 +8728,7 @@
       <c r="BJ51" s="15" t="n"/>
       <c r="BK51" s="15" t="n"/>
       <c r="BL51" s="15" t="n"/>
+      <c r="BM51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -8798,6 +8922,9 @@
       </c>
       <c r="BL52" s="15" t="n">
         <v>45.97</v>
+      </c>
+      <c r="BM52" s="15" t="n">
+        <v>45.9</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -8944,6 +9071,9 @@
       </c>
       <c r="BL53" s="15" t="n">
         <v>3672.37</v>
+      </c>
+      <c r="BM53" s="15" t="n">
+        <v>3595.24</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -9059,6 +9189,7 @@
       <c r="BJ54" s="15" t="n"/>
       <c r="BK54" s="15" t="n"/>
       <c r="BL54" s="15" t="n"/>
+      <c r="BM54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -9252,6 +9383,9 @@
       </c>
       <c r="BL55" s="15" t="n">
         <v>54.56</v>
+      </c>
+      <c r="BM55" s="15" t="n">
+        <v>52.72</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -9398,6 +9532,9 @@
       </c>
       <c r="BL56" s="15" t="n">
         <v>3509.44</v>
+      </c>
+      <c r="BM56" s="15" t="n">
+        <v>3421.5</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -9513,6 +9650,7 @@
       <c r="BJ57" s="15" t="n"/>
       <c r="BK57" s="15" t="n"/>
       <c r="BL57" s="15" t="n"/>
+      <c r="BM57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -9706,6 +9844,9 @@
       </c>
       <c r="BL58" s="15" t="n">
         <v>18.1</v>
+      </c>
+      <c r="BM58" s="15" t="n">
+        <v>19.8</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -9852,6 +9993,9 @@
       </c>
       <c r="BL59" s="15" t="n">
         <v>7188</v>
+      </c>
+      <c r="BM59" s="15" t="n">
+        <v>6702.38</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -9967,6 +10111,7 @@
       <c r="BJ60" s="15" t="n"/>
       <c r="BK60" s="15" t="n"/>
       <c r="BL60" s="15" t="n"/>
+      <c r="BM60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -10160,6 +10305,9 @@
       </c>
       <c r="BL61" s="15" t="n">
         <v>37.71</v>
+      </c>
+      <c r="BM61" s="15" t="n">
+        <v>33.27</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -10306,6 +10454,9 @@
       </c>
       <c r="BL62" s="15" t="n">
         <v>8728.530000000001</v>
+      </c>
+      <c r="BM62" s="15" t="n">
+        <v>8119.02</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -10421,6 +10572,7 @@
       <c r="BJ63" s="15" t="n"/>
       <c r="BK63" s="15" t="n"/>
       <c r="BL63" s="15" t="n"/>
+      <c r="BM63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -10614,6 +10766,9 @@
       </c>
       <c r="BL64" s="15" t="n">
         <v>3.59</v>
+      </c>
+      <c r="BM64" s="15" t="n">
+        <v>6.62</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -10760,6 +10915,9 @@
       </c>
       <c r="BL65" s="15" t="n">
         <v>10763.09</v>
+      </c>
+      <c r="BM65" s="15" t="n">
+        <v>10733.97</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -10875,6 +11033,7 @@
       <c r="BJ66" s="15" t="n"/>
       <c r="BK66" s="15" t="n"/>
       <c r="BL66" s="15" t="n"/>
+      <c r="BM66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -11068,6 +11227,9 @@
       </c>
       <c r="BL67" s="15" t="n">
         <v>19.99</v>
+      </c>
+      <c r="BM67" s="15" t="n">
+        <v>19.59</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -11214,6 +11376,9 @@
       </c>
       <c r="BL68" s="15" t="n">
         <v>11366.98</v>
+      </c>
+      <c r="BM68" s="15" t="n">
+        <v>11209.32</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -11329,6 +11494,7 @@
       <c r="BJ69" s="15" t="n"/>
       <c r="BK69" s="15" t="n"/>
       <c r="BL69" s="15" t="n"/>
+      <c r="BM69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -11522,6 +11688,9 @@
       </c>
       <c r="BL70" s="15" t="n">
         <v>14.89</v>
+      </c>
+      <c r="BM70" s="15" t="n">
+        <v>12.52</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -11668,6 +11837,9 @@
       </c>
       <c r="BL71" s="15" t="n">
         <v>6537.61</v>
+      </c>
+      <c r="BM71" s="15" t="n">
+        <v>6533.35</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -11783,6 +11955,7 @@
       <c r="BJ72" s="15" t="n"/>
       <c r="BK72" s="15" t="n"/>
       <c r="BL72" s="15" t="n"/>
+      <c r="BM72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -11976,6 +12149,9 @@
       </c>
       <c r="BL73" s="15" t="n">
         <v>13.71</v>
+      </c>
+      <c r="BM73" s="15" t="n">
+        <v>15.04</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -12122,6 +12298,9 @@
       </c>
       <c r="BL74" s="15" t="n">
         <v>12503.52</v>
+      </c>
+      <c r="BM74" s="15" t="n">
+        <v>12426.07</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -12237,6 +12416,7 @@
       <c r="BJ75" s="15" t="n"/>
       <c r="BK75" s="15" t="n"/>
       <c r="BL75" s="15" t="n"/>
+      <c r="BM75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -12430,6 +12610,9 @@
       </c>
       <c r="BL76" s="15" t="n">
         <v>55.03</v>
+      </c>
+      <c r="BM76" s="15" t="n">
+        <v>52.81</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -12576,6 +12759,9 @@
       </c>
       <c r="BL77" s="15" t="n">
         <v>15569.82</v>
+      </c>
+      <c r="BM77" s="15" t="n">
+        <v>15598.74</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
@@ -12691,6 +12877,7 @@
       <c r="BJ78" s="15" t="n"/>
       <c r="BK78" s="15" t="n"/>
       <c r="BL78" s="15" t="n"/>
+      <c r="BM78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -12884,6 +13071,9 @@
       </c>
       <c r="BL79" s="15" t="n">
         <v>3.42</v>
+      </c>
+      <c r="BM79" s="15" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -13030,6 +13220,9 @@
       </c>
       <c r="BL80" s="15" t="n">
         <v>7254.7</v>
+      </c>
+      <c r="BM80" s="15" t="n">
+        <v>6841.68</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -13145,6 +13338,7 @@
       <c r="BJ81" s="15" t="n"/>
       <c r="BK81" s="15" t="n"/>
       <c r="BL81" s="15" t="n"/>
+      <c r="BM81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -13337,6 +13531,9 @@
         <v>5.4</v>
       </c>
       <c r="BL82" s="15" t="n">
+        <v>4.42</v>
+      </c>
+      <c r="BM82" s="15" t="n">
         <v>4.42</v>
       </c>
     </row>
@@ -13484,6 +13681,9 @@
       </c>
       <c r="BL83" s="15" t="n">
         <v>8669.940000000001</v>
+      </c>
+      <c r="BM83" s="15" t="n">
+        <v>8384.68</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -13599,6 +13799,7 @@
       <c r="BJ84" s="15" t="n"/>
       <c r="BK84" s="15" t="n"/>
       <c r="BL84" s="15" t="n"/>
+      <c r="BM84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -13792,6 +13993,9 @@
       </c>
       <c r="BL85" s="15" t="n">
         <v>12.77</v>
+      </c>
+      <c r="BM85" s="15" t="n">
+        <v>18.43</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -13938,6 +14142,9 @@
       </c>
       <c r="BL86" s="15" t="n">
         <v>2631.9</v>
+      </c>
+      <c r="BM86" s="15" t="n">
+        <v>2194.69</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -14053,6 +14260,7 @@
       <c r="BJ87" s="15" t="n"/>
       <c r="BK87" s="15" t="n"/>
       <c r="BL87" s="15" t="n"/>
+      <c r="BM87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -14246,6 +14454,9 @@
       </c>
       <c r="BL88" s="15" t="n">
         <v>27.99</v>
+      </c>
+      <c r="BM88" s="15" t="n">
+        <v>34.41</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -14391,6 +14602,9 @@
         <v>5075.31</v>
       </c>
       <c r="BL89" s="15" t="n">
+        <v>5075.31</v>
+      </c>
+      <c r="BM89" s="15" t="n">
         <v>5075.31</v>
       </c>
     </row>
@@ -14507,6 +14721,7 @@
       <c r="BJ90" s="15" t="n"/>
       <c r="BK90" s="15" t="n"/>
       <c r="BL90" s="15" t="n"/>
+      <c r="BM90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -14700,6 +14915,9 @@
       </c>
       <c r="BL91" s="15" t="n">
         <v>25.76</v>
+      </c>
+      <c r="BM91" s="15" t="n">
+        <v>24.96</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -14846,6 +15064,9 @@
       </c>
       <c r="BL92" s="15" t="n">
         <v>9209.950000000001</v>
+      </c>
+      <c r="BM92" s="15" t="n">
+        <v>8524.129999999999</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -14961,6 +15182,7 @@
       <c r="BJ93" s="15" t="n"/>
       <c r="BK93" s="15" t="n"/>
       <c r="BL93" s="15" t="n"/>
+      <c r="BM93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -15154,6 +15376,9 @@
       </c>
       <c r="BL94" s="15" t="n">
         <v>4.04</v>
+      </c>
+      <c r="BM94" s="15" t="n">
+        <v>4.85</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -15300,6 +15525,9 @@
       </c>
       <c r="BL95" s="15" t="n">
         <v>1148.76</v>
+      </c>
+      <c r="BM95" s="15" t="n">
+        <v>1171.89</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -15415,6 +15643,7 @@
       <c r="BJ96" s="15" t="n"/>
       <c r="BK96" s="15" t="n"/>
       <c r="BL96" s="15" t="n"/>
+      <c r="BM96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -15608,6 +15837,9 @@
       </c>
       <c r="BL97" s="15" t="n">
         <v>6.9</v>
+      </c>
+      <c r="BM97" s="15" t="n">
+        <v>6.04</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -15754,6 +15986,9 @@
       </c>
       <c r="BL98" s="15" t="n">
         <v>14018.67</v>
+      </c>
+      <c r="BM98" s="15" t="n">
+        <v>13788.89</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -15869,6 +16104,7 @@
       <c r="BJ99" s="15" t="n"/>
       <c r="BK99" s="15" t="n"/>
       <c r="BL99" s="15" t="n"/>
+      <c r="BM99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -16062,6 +16298,9 @@
       </c>
       <c r="BL100" s="15" t="n">
         <v>50.19</v>
+      </c>
+      <c r="BM100" s="15" t="n">
+        <v>50.62</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -16208,6 +16447,9 @@
       </c>
       <c r="BL101" s="15" t="n">
         <v>3354.61</v>
+      </c>
+      <c r="BM101" s="15" t="n">
+        <v>3390.67</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -16323,6 +16565,7 @@
       <c r="BJ102" s="15" t="n"/>
       <c r="BK102" s="15" t="n"/>
       <c r="BL102" s="15" t="n"/>
+      <c r="BM102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -16516,6 +16759,9 @@
       </c>
       <c r="BL103" s="15" t="n">
         <v>36.5</v>
+      </c>
+      <c r="BM103" s="15" t="n">
+        <v>35.49</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -16662,6 +16908,9 @@
       </c>
       <c r="BL104" s="15" t="n">
         <v>2446.66</v>
+      </c>
+      <c r="BM104" s="15" t="n">
+        <v>2440.72</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -16777,6 +17026,7 @@
       <c r="BJ105" s="15" t="n"/>
       <c r="BK105" s="15" t="n"/>
       <c r="BL105" s="15" t="n"/>
+      <c r="BM105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -16970,6 +17220,9 @@
       </c>
       <c r="BL106" s="15" t="n">
         <v>14.65</v>
+      </c>
+      <c r="BM106" s="15" t="n">
+        <v>15.62</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -17116,6 +17369,9 @@
       </c>
       <c r="BL107" s="15" t="n">
         <v>2595.64</v>
+      </c>
+      <c r="BM107" s="15" t="n">
+        <v>2520.37</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -17231,6 +17487,7 @@
       <c r="BJ108" s="15" t="n"/>
       <c r="BK108" s="15" t="n"/>
       <c r="BL108" s="15" t="n"/>
+      <c r="BM108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -17424,6 +17681,9 @@
       </c>
       <c r="BL109" s="15" t="n">
         <v>36.81</v>
+      </c>
+      <c r="BM109" s="15" t="n">
+        <v>37.34</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -17570,6 +17830,9 @@
       </c>
       <c r="BL110" s="15" t="n">
         <v>2591.86</v>
+      </c>
+      <c r="BM110" s="15" t="n">
+        <v>2602.14</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -17685,6 +17948,7 @@
       <c r="BJ111" s="15" t="n"/>
       <c r="BK111" s="15" t="n"/>
       <c r="BL111" s="15" t="n"/>
+      <c r="BM111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -17878,6 +18142,9 @@
       </c>
       <c r="BL112" s="15" t="n">
         <v>64.62</v>
+      </c>
+      <c r="BM112" s="15" t="n">
+        <v>63.16</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -18022,6 +18289,9 @@
       </c>
       <c r="BL113" s="15" t="n">
         <v>2116.41</v>
+      </c>
+      <c r="BM113" s="15" t="n">
+        <v>1925.5</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -18137,6 +18407,7 @@
       <c r="BJ114" s="15" t="n"/>
       <c r="BK114" s="15" t="n"/>
       <c r="BL114" s="15" t="n"/>
+      <c r="BM114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -18330,6 +18601,9 @@
       </c>
       <c r="BL115" s="15" t="n">
         <v>21.36</v>
+      </c>
+      <c r="BM115" s="15" t="n">
+        <v>23.15</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -18460,6 +18734,9 @@
         <v>8885.33</v>
       </c>
       <c r="BL116" s="15" t="n">
+        <v>9144.950000000001</v>
+      </c>
+      <c r="BM116" s="15" t="n">
         <v>9144.950000000001</v>
       </c>
     </row>
@@ -18531,6 +18808,7 @@
       <c r="BJ117" s="15" t="n"/>
       <c r="BK117" s="15" t="n"/>
       <c r="BL117" s="15" t="n"/>
+      <c r="BM117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -18680,6 +18958,9 @@
       <c r="BL118" s="15" t="n">
         <v>90.3</v>
       </c>
+      <c r="BM118" s="15" t="n">
+        <v>87.91</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -18801,6 +19082,9 @@
       </c>
       <c r="BL119" s="15" t="n">
         <v>13057.27</v>
+      </c>
+      <c r="BM119" s="15" t="n">
+        <v>12684.9</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -18820,6 +19104,7 @@
       <c r="BJ120" s="15" t="n"/>
       <c r="BK120" s="15" t="n"/>
       <c r="BL120" s="15" t="n"/>
+      <c r="BM120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -18870,6 +19155,9 @@
       <c r="BL121" s="15" t="n">
         <v>26.66</v>
       </c>
+      <c r="BM121" s="15" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -18919,6 +19207,9 @@
       </c>
       <c r="BL122" s="15" t="n">
         <v>1192.72</v>
+      </c>
+      <c r="BM122" s="15" t="n">
+        <v>1191.8</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -18938,6 +19229,7 @@
       <c r="BJ123" s="15" t="n"/>
       <c r="BK123" s="15" t="n"/>
       <c r="BL123" s="15" t="n"/>
+      <c r="BM123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -18988,6 +19280,9 @@
       <c r="BL124" s="15" t="n">
         <v>43.31</v>
       </c>
+      <c r="BM124" s="15" t="n">
+        <v>42.82</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -19037,6 +19332,9 @@
       </c>
       <c r="BL125" s="15" t="n">
         <v>11216.97</v>
+      </c>
+      <c r="BM125" s="15" t="n">
+        <v>11033.11</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -19056,6 +19354,7 @@
       <c r="BJ126" s="15" t="n"/>
       <c r="BK126" s="15" t="n"/>
       <c r="BL126" s="15" t="n"/>
+      <c r="BM126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -19106,6 +19405,9 @@
       <c r="BL127" s="15" t="n">
         <v>28.17</v>
       </c>
+      <c r="BM127" s="15" t="n">
+        <v>1.7</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -19155,6 +19457,9 @@
       </c>
       <c r="BL128" s="15" t="n">
         <v>1862.02</v>
+      </c>
+      <c r="BM128" s="15" t="n">
+        <v>1839.18</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -19174,6 +19479,7 @@
       <c r="BJ129" s="15" t="n"/>
       <c r="BK129" s="15" t="n"/>
       <c r="BL129" s="15" t="n"/>
+      <c r="BM129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -19224,6 +19530,9 @@
       <c r="BL130" s="15" t="n">
         <v>9.640000000000001</v>
       </c>
+      <c r="BM130" s="15" t="n">
+        <v>8.609999999999999</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -19273,6 +19582,9 @@
       </c>
       <c r="BL131" s="15" t="n">
         <v>736.96</v>
+      </c>
+      <c r="BM131" s="15" t="n">
+        <v>742.41</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -19292,6 +19604,7 @@
       <c r="BJ132" s="15" t="n"/>
       <c r="BK132" s="15" t="n"/>
       <c r="BL132" s="15" t="n"/>
+      <c r="BM132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -19342,6 +19655,9 @@
       <c r="BL133" s="15" t="n">
         <v>68.45999999999999</v>
       </c>
+      <c r="BM133" s="15" t="n">
+        <v>70.17</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -19391,6 +19707,9 @@
       </c>
       <c r="BL134" s="15" t="n">
         <v>2974.54</v>
+      </c>
+      <c r="BM134" s="15" t="n">
+        <v>3081.52</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -19410,6 +19729,7 @@
       <c r="BJ135" s="15" t="n"/>
       <c r="BK135" s="15" t="n"/>
       <c r="BL135" s="15" t="n"/>
+      <c r="BM135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -19460,6 +19780,9 @@
       <c r="BL136" s="15" t="n">
         <v>19.62</v>
       </c>
+      <c r="BM136" s="15" t="n">
+        <v>19.92</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -19509,6 +19832,9 @@
       </c>
       <c r="BL137" s="15" t="n">
         <v>3556.93</v>
+      </c>
+      <c r="BM137" s="15" t="n">
+        <v>3539.37</v>
       </c>
     </row>
     <row r="138">
@@ -19520,6 +19846,7 @@
       <c r="BJ138" s="15" t="n"/>
       <c r="BK138" s="15" t="n"/>
       <c r="BL138" s="15" t="n"/>
+      <c r="BM138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -19546,6 +19873,9 @@
       <c r="BL139" s="15" t="n">
         <v>3.33</v>
       </c>
+      <c r="BM139" s="15" t="n">
+        <v>2.69</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -19571,6 +19901,9 @@
       </c>
       <c r="BL140" s="15" t="n">
         <v>2400.76</v>
+      </c>
+      <c r="BM140" s="15" t="n">
+        <v>2394.09</v>
       </c>
     </row>
     <row r="141">
@@ -19582,6 +19915,7 @@
       <c r="BJ141" s="15" t="n"/>
       <c r="BK141" s="15" t="n"/>
       <c r="BL141" s="15" t="n"/>
+      <c r="BM141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -19608,6 +19942,9 @@
       <c r="BL142" s="15" t="n">
         <v>13.57</v>
       </c>
+      <c r="BM142" s="15" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -19633,12 +19970,16 @@
       </c>
       <c r="BL143" s="15" t="n">
         <v>5746.4</v>
+      </c>
+      <c r="BM143" s="15" t="n">
+        <v>5410.93</v>
       </c>
     </row>
     <row r="144">
       <c r="BJ144" s="15" t="n"/>
       <c r="BK144" s="15" t="n"/>
       <c r="BL144" s="15" t="n"/>
+      <c r="BM144" s="15" t="n"/>
     </row>
     <row r="145">
       <c r="BJ145" s="15" t="n">
@@ -19650,6 +19991,9 @@
       <c r="BL145" s="15" t="n">
         <v>23.96</v>
       </c>
+      <c r="BM145" s="15" t="n">
+        <v>23.82</v>
+      </c>
     </row>
     <row r="146">
       <c r="BJ146" s="15" t="n">
@@ -19660,6 +20004,9 @@
       </c>
       <c r="BL146" s="15" t="n">
         <v>2240.49</v>
+      </c>
+      <c r="BM146" s="15" t="n">
+        <v>2253.12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-08-27 14:36:36]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BM146"/>
+  <dimension ref="A1:BN146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -599,6 +599,7 @@
     <col width="15" customWidth="1" min="63" max="63"/>
     <col width="15" customWidth="1" min="64" max="64"/>
     <col width="15" customWidth="1" min="65" max="65"/>
+    <col width="15" customWidth="1" min="66" max="66"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -927,6 +928,11 @@
           <t>2026/08/24</t>
         </is>
       </c>
+      <c r="BN1" s="15" t="inlineStr">
+        <is>
+          <t>2026/08/27</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1254,6 +1260,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BN2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1451,6 +1462,9 @@
       <c r="BM3" s="15" t="n">
         <v>65.34</v>
       </c>
+      <c r="BN3" s="15" t="n">
+        <v>63.94</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1647,6 +1661,9 @@
       </c>
       <c r="BM4" s="15" t="n">
         <v>3877.3</v>
+      </c>
+      <c r="BN4" s="15" t="n">
+        <v>3956.57</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1715,6 +1732,7 @@
       <c r="BK5" s="15" t="n"/>
       <c r="BL5" s="15" t="n"/>
       <c r="BM5" s="15" t="n"/>
+      <c r="BN5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1830,6 +1848,7 @@
       <c r="BK6" s="15" t="n"/>
       <c r="BL6" s="15" t="n"/>
       <c r="BM6" s="15" t="n"/>
+      <c r="BN6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -2026,6 +2045,9 @@
       </c>
       <c r="BM7" s="15" t="n">
         <v>61.63</v>
+      </c>
+      <c r="BN7" s="15" t="n">
+        <v>60.77</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -2175,6 +2197,9 @@
       </c>
       <c r="BM8" s="15" t="n">
         <v>5631.5</v>
+      </c>
+      <c r="BN8" s="15" t="n">
+        <v>5740.88</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2291,6 +2316,7 @@
       <c r="BK9" s="15" t="n"/>
       <c r="BL9" s="15" t="n"/>
       <c r="BM9" s="15" t="n"/>
+      <c r="BN9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2487,6 +2513,9 @@
       </c>
       <c r="BM10" s="15" t="n">
         <v>53.15</v>
+      </c>
+      <c r="BN10" s="15" t="n">
+        <v>53.9</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2636,6 +2665,9 @@
       </c>
       <c r="BM11" s="15" t="n">
         <v>4560.85</v>
+      </c>
+      <c r="BN11" s="15" t="n">
+        <v>4630.28</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -2752,6 +2784,7 @@
       <c r="BK12" s="15" t="n"/>
       <c r="BL12" s="15" t="n"/>
       <c r="BM12" s="15" t="n"/>
+      <c r="BN12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2948,6 +2981,9 @@
       </c>
       <c r="BM13" s="15" t="n">
         <v>64.66</v>
+      </c>
+      <c r="BN13" s="15" t="n">
+        <v>62.54</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -3097,6 +3133,9 @@
       </c>
       <c r="BM14" s="15" t="n">
         <v>7692.53</v>
+      </c>
+      <c r="BN14" s="15" t="n">
+        <v>7946.33</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -3213,6 +3252,7 @@
       <c r="BK15" s="15" t="n"/>
       <c r="BL15" s="15" t="n"/>
       <c r="BM15" s="15" t="n"/>
+      <c r="BN15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -3409,6 +3449,9 @@
       </c>
       <c r="BM16" s="15" t="n">
         <v>34.68</v>
+      </c>
+      <c r="BN16" s="15" t="n">
+        <v>33.7</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -3558,6 +3601,9 @@
       </c>
       <c r="BM17" s="15" t="n">
         <v>2562.04</v>
+      </c>
+      <c r="BN17" s="15" t="n">
+        <v>2594.35</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -3674,6 +3720,7 @@
       <c r="BK18" s="15" t="n"/>
       <c r="BL18" s="15" t="n"/>
       <c r="BM18" s="15" t="n"/>
+      <c r="BN18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -3870,6 +3917,9 @@
       </c>
       <c r="BM19" s="15" t="n">
         <v>81.02</v>
+      </c>
+      <c r="BN19" s="15" t="n">
+        <v>81.34</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -4019,6 +4069,9 @@
       </c>
       <c r="BM20" s="15" t="n">
         <v>7674.37</v>
+      </c>
+      <c r="BN20" s="15" t="n">
+        <v>7713.55</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -4135,6 +4188,7 @@
       <c r="BK21" s="15" t="n"/>
       <c r="BL21" s="15" t="n"/>
       <c r="BM21" s="15" t="n"/>
+      <c r="BN21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -4328,6 +4382,9 @@
         <v>36.34</v>
       </c>
       <c r="BM22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BN22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -4478,6 +4535,9 @@
       </c>
       <c r="BM23" s="15" t="n">
         <v>77678.35000000001</v>
+      </c>
+      <c r="BN23" s="15" t="n">
+        <v>76933.59</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -4594,6 +4654,7 @@
       <c r="BK24" s="15" t="n"/>
       <c r="BL24" s="15" t="n"/>
       <c r="BM24" s="15" t="n"/>
+      <c r="BN24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -4789,6 +4850,9 @@
         <v>49.88</v>
       </c>
       <c r="BM25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BN25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -4925,6 +4989,9 @@
       </c>
       <c r="BM26" s="15" t="n">
         <v>26136.56</v>
+      </c>
+      <c r="BN26" s="15" t="n">
+        <v>26253.99</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -5041,6 +5108,7 @@
       <c r="BK27" s="15" t="n"/>
       <c r="BL27" s="15" t="n"/>
       <c r="BM27" s="15" t="n"/>
+      <c r="BN27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -5236,6 +5304,9 @@
         <v>92.09</v>
       </c>
       <c r="BM28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BN28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -5386,6 +5457,9 @@
       </c>
       <c r="BM29" s="15" t="n">
         <v>65751.64999999999</v>
+      </c>
+      <c r="BN29" s="15" t="n">
+        <v>66131.98</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -5502,6 +5576,7 @@
       <c r="BK30" s="15" t="n"/>
       <c r="BL30" s="15" t="n"/>
       <c r="BM30" s="15" t="n"/>
+      <c r="BN30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -5697,6 +5772,9 @@
         <v>97.44</v>
       </c>
       <c r="BM31" s="15" t="n">
+        <v>97.44</v>
+      </c>
+      <c r="BN31" s="15" t="n">
         <v>97.44</v>
       </c>
     </row>
@@ -5847,6 +5925,9 @@
       </c>
       <c r="BM32" s="15" t="n">
         <v>6706.38</v>
+      </c>
+      <c r="BN32" s="15" t="n">
+        <v>6912.37</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -5963,6 +6044,7 @@
       <c r="BK33" s="15" t="n"/>
       <c r="BL33" s="15" t="n"/>
       <c r="BM33" s="15" t="n"/>
+      <c r="BN33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -6159,6 +6241,9 @@
       </c>
       <c r="BM34" s="15" t="n">
         <v>45.4</v>
+      </c>
+      <c r="BN34" s="15" t="n">
+        <v>45.88</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -6308,6 +6393,9 @@
       </c>
       <c r="BM35" s="15" t="n">
         <v>5647.76</v>
+      </c>
+      <c r="BN35" s="15" t="n">
+        <v>5676.05</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -6424,6 +6512,7 @@
       <c r="BK36" s="15" t="n"/>
       <c r="BL36" s="15" t="n"/>
       <c r="BM36" s="15" t="n"/>
+      <c r="BN36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -6620,6 +6709,9 @@
       </c>
       <c r="BM37" s="15" t="n">
         <v>59.25</v>
+      </c>
+      <c r="BN37" s="15" t="n">
+        <v>57.33</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -6769,6 +6861,9 @@
       </c>
       <c r="BM38" s="15" t="n">
         <v>11266.26</v>
+      </c>
+      <c r="BN38" s="15" t="n">
+        <v>11306.87</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -6885,6 +6980,7 @@
       <c r="BK39" s="15" t="n"/>
       <c r="BL39" s="15" t="n"/>
       <c r="BM39" s="15" t="n"/>
+      <c r="BN39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -7081,6 +7177,9 @@
       </c>
       <c r="BM40" s="15" t="n">
         <v>50.39</v>
+      </c>
+      <c r="BN40" s="15" t="n">
+        <v>50.52</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -7230,6 +7329,9 @@
       </c>
       <c r="BM41" s="15" t="n">
         <v>10858.77</v>
+      </c>
+      <c r="BN41" s="15" t="n">
+        <v>11002.01</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -7346,6 +7448,7 @@
       <c r="BK42" s="15" t="n"/>
       <c r="BL42" s="15" t="n"/>
       <c r="BM42" s="15" t="n"/>
+      <c r="BN42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -7542,6 +7645,9 @@
       </c>
       <c r="BM43" s="15" t="n">
         <v>50.43</v>
+      </c>
+      <c r="BN43" s="15" t="n">
+        <v>50.26</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -7691,6 +7797,9 @@
       </c>
       <c r="BM44" s="15" t="n">
         <v>3300.46</v>
+      </c>
+      <c r="BN44" s="15" t="n">
+        <v>3351.48</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -7807,6 +7916,7 @@
       <c r="BK45" s="15" t="n"/>
       <c r="BL45" s="15" t="n"/>
       <c r="BM45" s="15" t="n"/>
+      <c r="BN45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -8003,6 +8113,9 @@
       </c>
       <c r="BM46" s="15" t="n">
         <v>60.95</v>
+      </c>
+      <c r="BN46" s="15" t="n">
+        <v>59.12</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -8152,6 +8265,9 @@
       </c>
       <c r="BM47" s="15" t="n">
         <v>6897.89</v>
+      </c>
+      <c r="BN47" s="15" t="n">
+        <v>7033.51</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -8268,6 +8384,7 @@
       <c r="BK48" s="15" t="n"/>
       <c r="BL48" s="15" t="n"/>
       <c r="BM48" s="15" t="n"/>
+      <c r="BN48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -8464,6 +8581,9 @@
       </c>
       <c r="BM49" s="15" t="n">
         <v>28.11</v>
+      </c>
+      <c r="BN49" s="15" t="n">
+        <v>25.33</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -8613,6 +8733,9 @@
       </c>
       <c r="BM50" s="15" t="n">
         <v>33771.36</v>
+      </c>
+      <c r="BN50" s="15" t="n">
+        <v>33541.54</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -8729,6 +8852,7 @@
       <c r="BK51" s="15" t="n"/>
       <c r="BL51" s="15" t="n"/>
       <c r="BM51" s="15" t="n"/>
+      <c r="BN51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -8925,6 +9049,9 @@
       </c>
       <c r="BM52" s="15" t="n">
         <v>45.9</v>
+      </c>
+      <c r="BN52" s="15" t="n">
+        <v>42.98</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -9074,6 +9201,9 @@
       </c>
       <c r="BM53" s="15" t="n">
         <v>3595.24</v>
+      </c>
+      <c r="BN53" s="15" t="n">
+        <v>3634.34</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -9190,6 +9320,7 @@
       <c r="BK54" s="15" t="n"/>
       <c r="BL54" s="15" t="n"/>
       <c r="BM54" s="15" t="n"/>
+      <c r="BN54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -9386,6 +9517,9 @@
       </c>
       <c r="BM55" s="15" t="n">
         <v>52.72</v>
+      </c>
+      <c r="BN55" s="15" t="n">
+        <v>49.17</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -9535,6 +9669,9 @@
       </c>
       <c r="BM56" s="15" t="n">
         <v>3421.5</v>
+      </c>
+      <c r="BN56" s="15" t="n">
+        <v>3473.35</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -9651,6 +9788,7 @@
       <c r="BK57" s="15" t="n"/>
       <c r="BL57" s="15" t="n"/>
       <c r="BM57" s="15" t="n"/>
+      <c r="BN57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -9847,6 +9985,9 @@
       </c>
       <c r="BM58" s="15" t="n">
         <v>19.8</v>
+      </c>
+      <c r="BN58" s="15" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -9996,6 +10137,9 @@
       </c>
       <c r="BM59" s="15" t="n">
         <v>6702.38</v>
+      </c>
+      <c r="BN59" s="15" t="n">
+        <v>6842.42</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -10112,6 +10256,7 @@
       <c r="BK60" s="15" t="n"/>
       <c r="BL60" s="15" t="n"/>
       <c r="BM60" s="15" t="n"/>
+      <c r="BN60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -10308,6 +10453,9 @@
       </c>
       <c r="BM61" s="15" t="n">
         <v>33.27</v>
+      </c>
+      <c r="BN61" s="15" t="n">
+        <v>31.95</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -10457,6 +10605,9 @@
       </c>
       <c r="BM62" s="15" t="n">
         <v>8119.02</v>
+      </c>
+      <c r="BN62" s="15" t="n">
+        <v>8289.290000000001</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -10573,6 +10724,7 @@
       <c r="BK63" s="15" t="n"/>
       <c r="BL63" s="15" t="n"/>
       <c r="BM63" s="15" t="n"/>
+      <c r="BN63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -10769,6 +10921,9 @@
       </c>
       <c r="BM64" s="15" t="n">
         <v>6.62</v>
+      </c>
+      <c r="BN64" s="15" t="n">
+        <v>8.710000000000001</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -10918,6 +11073,9 @@
       </c>
       <c r="BM65" s="15" t="n">
         <v>10733.97</v>
+      </c>
+      <c r="BN65" s="15" t="n">
+        <v>10752.99</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -11034,6 +11192,7 @@
       <c r="BK66" s="15" t="n"/>
       <c r="BL66" s="15" t="n"/>
       <c r="BM66" s="15" t="n"/>
+      <c r="BN66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -11230,6 +11389,9 @@
       </c>
       <c r="BM67" s="15" t="n">
         <v>19.59</v>
+      </c>
+      <c r="BN67" s="15" t="n">
+        <v>20.38</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -11379,6 +11541,9 @@
       </c>
       <c r="BM68" s="15" t="n">
         <v>11209.32</v>
+      </c>
+      <c r="BN68" s="15" t="n">
+        <v>11413.66</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -11495,6 +11660,7 @@
       <c r="BK69" s="15" t="n"/>
       <c r="BL69" s="15" t="n"/>
       <c r="BM69" s="15" t="n"/>
+      <c r="BN69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -11691,6 +11857,9 @@
       </c>
       <c r="BM70" s="15" t="n">
         <v>12.52</v>
+      </c>
+      <c r="BN70" s="15" t="n">
+        <v>16.7</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -11840,6 +12009,9 @@
       </c>
       <c r="BM71" s="15" t="n">
         <v>6533.35</v>
+      </c>
+      <c r="BN71" s="15" t="n">
+        <v>6460.01</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -11956,6 +12128,7 @@
       <c r="BK72" s="15" t="n"/>
       <c r="BL72" s="15" t="n"/>
       <c r="BM72" s="15" t="n"/>
+      <c r="BN72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -12152,6 +12325,9 @@
       </c>
       <c r="BM73" s="15" t="n">
         <v>15.04</v>
+      </c>
+      <c r="BN73" s="15" t="n">
+        <v>17.53</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -12301,6 +12477,9 @@
       </c>
       <c r="BM74" s="15" t="n">
         <v>12426.07</v>
+      </c>
+      <c r="BN74" s="15" t="n">
+        <v>12489.39</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -12417,6 +12596,7 @@
       <c r="BK75" s="15" t="n"/>
       <c r="BL75" s="15" t="n"/>
       <c r="BM75" s="15" t="n"/>
+      <c r="BN75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -12613,6 +12793,9 @@
       </c>
       <c r="BM76" s="15" t="n">
         <v>52.81</v>
+      </c>
+      <c r="BN76" s="15" t="n">
+        <v>51.33</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -12762,6 +12945,9 @@
       </c>
       <c r="BM77" s="15" t="n">
         <v>15598.74</v>
+      </c>
+      <c r="BN77" s="15" t="n">
+        <v>16268.73</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
@@ -12878,6 +13064,7 @@
       <c r="BK78" s="15" t="n"/>
       <c r="BL78" s="15" t="n"/>
       <c r="BM78" s="15" t="n"/>
+      <c r="BN78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -13074,6 +13261,9 @@
       </c>
       <c r="BM79" s="15" t="n">
         <v>8</v>
+      </c>
+      <c r="BN79" s="15" t="n">
+        <v>5.49</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -13223,6 +13413,9 @@
       </c>
       <c r="BM80" s="15" t="n">
         <v>6841.68</v>
+      </c>
+      <c r="BN80" s="15" t="n">
+        <v>6955.02</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -13339,6 +13532,7 @@
       <c r="BK81" s="15" t="n"/>
       <c r="BL81" s="15" t="n"/>
       <c r="BM81" s="15" t="n"/>
+      <c r="BN81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -13535,6 +13729,9 @@
       </c>
       <c r="BM82" s="15" t="n">
         <v>4.42</v>
+      </c>
+      <c r="BN82" s="15" t="n">
+        <v>5.04</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -13684,6 +13881,9 @@
       </c>
       <c r="BM83" s="15" t="n">
         <v>8384.68</v>
+      </c>
+      <c r="BN83" s="15" t="n">
+        <v>8661.26</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -13800,6 +14000,7 @@
       <c r="BK84" s="15" t="n"/>
       <c r="BL84" s="15" t="n"/>
       <c r="BM84" s="15" t="n"/>
+      <c r="BN84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -13996,6 +14197,9 @@
       </c>
       <c r="BM85" s="15" t="n">
         <v>18.43</v>
+      </c>
+      <c r="BN85" s="15" t="n">
+        <v>17.02</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -14145,6 +14349,9 @@
       </c>
       <c r="BM86" s="15" t="n">
         <v>2194.69</v>
+      </c>
+      <c r="BN86" s="15" t="n">
+        <v>2631.9</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -14261,6 +14468,7 @@
       <c r="BK87" s="15" t="n"/>
       <c r="BL87" s="15" t="n"/>
       <c r="BM87" s="15" t="n"/>
+      <c r="BN87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -14457,6 +14665,9 @@
       </c>
       <c r="BM88" s="15" t="n">
         <v>34.41</v>
+      </c>
+      <c r="BN88" s="15" t="n">
+        <v>33.41</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -14605,6 +14816,9 @@
         <v>5075.31</v>
       </c>
       <c r="BM89" s="15" t="n">
+        <v>5075.31</v>
+      </c>
+      <c r="BN89" s="15" t="n">
         <v>5075.31</v>
       </c>
     </row>
@@ -14722,6 +14936,7 @@
       <c r="BK90" s="15" t="n"/>
       <c r="BL90" s="15" t="n"/>
       <c r="BM90" s="15" t="n"/>
+      <c r="BN90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -14918,6 +15133,9 @@
       </c>
       <c r="BM91" s="15" t="n">
         <v>24.96</v>
+      </c>
+      <c r="BN91" s="15" t="n">
+        <v>19.14</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -15067,6 +15285,9 @@
       </c>
       <c r="BM92" s="15" t="n">
         <v>8524.129999999999</v>
+      </c>
+      <c r="BN92" s="15" t="n">
+        <v>8723.85</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -15183,6 +15404,7 @@
       <c r="BK93" s="15" t="n"/>
       <c r="BL93" s="15" t="n"/>
       <c r="BM93" s="15" t="n"/>
+      <c r="BN93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -15379,6 +15601,9 @@
       </c>
       <c r="BM94" s="15" t="n">
         <v>4.85</v>
+      </c>
+      <c r="BN94" s="15" t="n">
+        <v>7.73</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -15528,6 +15753,9 @@
       </c>
       <c r="BM95" s="15" t="n">
         <v>1171.89</v>
+      </c>
+      <c r="BN95" s="15" t="n">
+        <v>1230.57</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -15644,6 +15872,7 @@
       <c r="BK96" s="15" t="n"/>
       <c r="BL96" s="15" t="n"/>
       <c r="BM96" s="15" t="n"/>
+      <c r="BN96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -15840,6 +16069,9 @@
       </c>
       <c r="BM97" s="15" t="n">
         <v>6.04</v>
+      </c>
+      <c r="BN97" s="15" t="n">
+        <v>6.77</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -15989,6 +16221,9 @@
       </c>
       <c r="BM98" s="15" t="n">
         <v>13788.89</v>
+      </c>
+      <c r="BN98" s="15" t="n">
+        <v>13943.49</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -16105,6 +16340,7 @@
       <c r="BK99" s="15" t="n"/>
       <c r="BL99" s="15" t="n"/>
       <c r="BM99" s="15" t="n"/>
+      <c r="BN99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -16301,6 +16537,9 @@
       </c>
       <c r="BM100" s="15" t="n">
         <v>50.62</v>
+      </c>
+      <c r="BN100" s="15" t="n">
+        <v>39.95</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -16450,6 +16689,9 @@
       </c>
       <c r="BM101" s="15" t="n">
         <v>3390.67</v>
+      </c>
+      <c r="BN101" s="15" t="n">
+        <v>3318.54</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -16566,6 +16808,7 @@
       <c r="BK102" s="15" t="n"/>
       <c r="BL102" s="15" t="n"/>
       <c r="BM102" s="15" t="n"/>
+      <c r="BN102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -16762,6 +17005,9 @@
       </c>
       <c r="BM103" s="15" t="n">
         <v>35.49</v>
+      </c>
+      <c r="BN103" s="15" t="n">
+        <v>33.67</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -16911,6 +17157,9 @@
       </c>
       <c r="BM104" s="15" t="n">
         <v>2440.72</v>
+      </c>
+      <c r="BN104" s="15" t="n">
+        <v>2424.25</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -17027,6 +17276,7 @@
       <c r="BK105" s="15" t="n"/>
       <c r="BL105" s="15" t="n"/>
       <c r="BM105" s="15" t="n"/>
+      <c r="BN105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -17223,6 +17473,9 @@
       </c>
       <c r="BM106" s="15" t="n">
         <v>15.62</v>
+      </c>
+      <c r="BN106" s="15" t="n">
+        <v>16.21</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -17372,6 +17625,9 @@
       </c>
       <c r="BM107" s="15" t="n">
         <v>2520.37</v>
+      </c>
+      <c r="BN107" s="15" t="n">
+        <v>2494.19</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -17488,6 +17744,7 @@
       <c r="BK108" s="15" t="n"/>
       <c r="BL108" s="15" t="n"/>
       <c r="BM108" s="15" t="n"/>
+      <c r="BN108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -17684,6 +17941,9 @@
       </c>
       <c r="BM109" s="15" t="n">
         <v>37.34</v>
+      </c>
+      <c r="BN109" s="15" t="n">
+        <v>35.69</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -17833,6 +18093,9 @@
       </c>
       <c r="BM110" s="15" t="n">
         <v>2602.14</v>
+      </c>
+      <c r="BN110" s="15" t="n">
+        <v>2602.09</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -17949,6 +18212,7 @@
       <c r="BK111" s="15" t="n"/>
       <c r="BL111" s="15" t="n"/>
       <c r="BM111" s="15" t="n"/>
+      <c r="BN111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -18145,6 +18409,9 @@
       </c>
       <c r="BM112" s="15" t="n">
         <v>63.16</v>
+      </c>
+      <c r="BN112" s="15" t="n">
+        <v>54.26</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -18292,6 +18559,9 @@
       </c>
       <c r="BM113" s="15" t="n">
         <v>1925.5</v>
+      </c>
+      <c r="BN113" s="15" t="n">
+        <v>1971.87</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -18408,6 +18678,7 @@
       <c r="BK114" s="15" t="n"/>
       <c r="BL114" s="15" t="n"/>
       <c r="BM114" s="15" t="n"/>
+      <c r="BN114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -18604,6 +18875,9 @@
       </c>
       <c r="BM115" s="15" t="n">
         <v>23.15</v>
+      </c>
+      <c r="BN115" s="15" t="n">
+        <v>17.88</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -18738,6 +19012,9 @@
       </c>
       <c r="BM116" s="15" t="n">
         <v>9144.950000000001</v>
+      </c>
+      <c r="BN116" s="15" t="n">
+        <v>8915.129999999999</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -18809,6 +19086,7 @@
       <c r="BK117" s="15" t="n"/>
       <c r="BL117" s="15" t="n"/>
       <c r="BM117" s="15" t="n"/>
+      <c r="BN117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -18961,6 +19239,9 @@
       <c r="BM118" s="15" t="n">
         <v>87.91</v>
       </c>
+      <c r="BN118" s="15" t="n">
+        <v>83.54000000000001</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -19085,6 +19366,9 @@
       </c>
       <c r="BM119" s="15" t="n">
         <v>12684.9</v>
+      </c>
+      <c r="BN119" s="15" t="n">
+        <v>13386.38</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -19105,6 +19389,7 @@
       <c r="BK120" s="15" t="n"/>
       <c r="BL120" s="15" t="n"/>
       <c r="BM120" s="15" t="n"/>
+      <c r="BN120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -19158,6 +19443,9 @@
       <c r="BM121" s="15" t="n">
         <v>24.25</v>
       </c>
+      <c r="BN121" s="15" t="n">
+        <v>23.67</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -19210,6 +19498,9 @@
       </c>
       <c r="BM122" s="15" t="n">
         <v>1191.8</v>
+      </c>
+      <c r="BN122" s="15" t="n">
+        <v>1191.9</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -19230,6 +19521,7 @@
       <c r="BK123" s="15" t="n"/>
       <c r="BL123" s="15" t="n"/>
       <c r="BM123" s="15" t="n"/>
+      <c r="BN123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -19283,6 +19575,9 @@
       <c r="BM124" s="15" t="n">
         <v>42.82</v>
       </c>
+      <c r="BN124" s="15" t="n">
+        <v>41.8</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -19335,6 +19630,9 @@
       </c>
       <c r="BM125" s="15" t="n">
         <v>11033.11</v>
+      </c>
+      <c r="BN125" s="15" t="n">
+        <v>11350.16</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -19355,6 +19653,7 @@
       <c r="BK126" s="15" t="n"/>
       <c r="BL126" s="15" t="n"/>
       <c r="BM126" s="15" t="n"/>
+      <c r="BN126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -19408,6 +19707,9 @@
       <c r="BM127" s="15" t="n">
         <v>1.7</v>
       </c>
+      <c r="BN127" s="15" t="n">
+        <v>3.4</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -19460,6 +19762,9 @@
       </c>
       <c r="BM128" s="15" t="n">
         <v>1839.18</v>
+      </c>
+      <c r="BN128" s="15" t="n">
+        <v>1861.56</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -19480,6 +19785,7 @@
       <c r="BK129" s="15" t="n"/>
       <c r="BL129" s="15" t="n"/>
       <c r="BM129" s="15" t="n"/>
+      <c r="BN129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -19533,6 +19839,9 @@
       <c r="BM130" s="15" t="n">
         <v>8.609999999999999</v>
       </c>
+      <c r="BN130" s="15" t="n">
+        <v>12.63</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -19585,6 +19894,9 @@
       </c>
       <c r="BM131" s="15" t="n">
         <v>742.41</v>
+      </c>
+      <c r="BN131" s="15" t="n">
+        <v>769.36</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -19605,6 +19917,7 @@
       <c r="BK132" s="15" t="n"/>
       <c r="BL132" s="15" t="n"/>
       <c r="BM132" s="15" t="n"/>
+      <c r="BN132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -19658,6 +19971,9 @@
       <c r="BM133" s="15" t="n">
         <v>70.17</v>
       </c>
+      <c r="BN133" s="15" t="n">
+        <v>68.69</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -19710,6 +20026,9 @@
       </c>
       <c r="BM134" s="15" t="n">
         <v>3081.52</v>
+      </c>
+      <c r="BN134" s="15" t="n">
+        <v>3112.31</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -19730,6 +20049,7 @@
       <c r="BK135" s="15" t="n"/>
       <c r="BL135" s="15" t="n"/>
       <c r="BM135" s="15" t="n"/>
+      <c r="BN135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -19783,6 +20103,9 @@
       <c r="BM136" s="15" t="n">
         <v>19.92</v>
       </c>
+      <c r="BN136" s="15" t="n">
+        <v>21.01</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -19835,6 +20158,9 @@
       </c>
       <c r="BM137" s="15" t="n">
         <v>3539.37</v>
+      </c>
+      <c r="BN137" s="15" t="n">
+        <v>3608.61</v>
       </c>
     </row>
     <row r="138">
@@ -19847,6 +20173,7 @@
       <c r="BK138" s="15" t="n"/>
       <c r="BL138" s="15" t="n"/>
       <c r="BM138" s="15" t="n"/>
+      <c r="BN138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -19876,6 +20203,9 @@
       <c r="BM139" s="15" t="n">
         <v>2.69</v>
       </c>
+      <c r="BN139" s="15" t="n">
+        <v>3.72</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -19904,6 +20234,9 @@
       </c>
       <c r="BM140" s="15" t="n">
         <v>2394.09</v>
+      </c>
+      <c r="BN140" s="15" t="n">
+        <v>2443.4</v>
       </c>
     </row>
     <row r="141">
@@ -19916,6 +20249,7 @@
       <c r="BK141" s="15" t="n"/>
       <c r="BL141" s="15" t="n"/>
       <c r="BM141" s="15" t="n"/>
+      <c r="BN141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -19945,6 +20279,9 @@
       <c r="BM142" s="15" t="n">
         <v>10</v>
       </c>
+      <c r="BN142" s="15" t="n">
+        <v>12.27</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -19973,6 +20310,9 @@
       </c>
       <c r="BM143" s="15" t="n">
         <v>5410.93</v>
+      </c>
+      <c r="BN143" s="15" t="n">
+        <v>5446.1</v>
       </c>
     </row>
     <row r="144">
@@ -19980,6 +20320,7 @@
       <c r="BK144" s="15" t="n"/>
       <c r="BL144" s="15" t="n"/>
       <c r="BM144" s="15" t="n"/>
+      <c r="BN144" s="15" t="n"/>
     </row>
     <row r="145">
       <c r="BJ145" s="15" t="n">
@@ -19994,6 +20335,9 @@
       <c r="BM145" s="15" t="n">
         <v>23.82</v>
       </c>
+      <c r="BN145" s="15" t="n">
+        <v>25.55</v>
+      </c>
     </row>
     <row r="146">
       <c r="BJ146" s="15" t="n">
@@ -20007,6 +20351,9 @@
       </c>
       <c r="BM146" s="15" t="n">
         <v>2253.12</v>
+      </c>
+      <c r="BN146" s="15" t="n">
+        <v>2305.74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-08-31 10:07:16]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BN146"/>
+  <dimension ref="A1:BO146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -600,6 +600,7 @@
     <col width="15" customWidth="1" min="64" max="64"/>
     <col width="15" customWidth="1" min="65" max="65"/>
     <col width="15" customWidth="1" min="66" max="66"/>
+    <col width="15" customWidth="1" min="67" max="67"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -933,6 +934,11 @@
           <t>2026/08/27</t>
         </is>
       </c>
+      <c r="BO1" s="15" t="inlineStr">
+        <is>
+          <t>2026/08/31</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1265,6 +1271,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BO2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1465,6 +1476,9 @@
       <c r="BN3" s="15" t="n">
         <v>63.94</v>
       </c>
+      <c r="BO3" s="15" t="n">
+        <v>65.77</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1664,6 +1678,9 @@
       </c>
       <c r="BN4" s="15" t="n">
         <v>3956.57</v>
+      </c>
+      <c r="BO4" s="15" t="n">
+        <v>3986.3</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1733,6 +1750,7 @@
       <c r="BL5" s="15" t="n"/>
       <c r="BM5" s="15" t="n"/>
       <c r="BN5" s="15" t="n"/>
+      <c r="BO5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1849,6 +1867,7 @@
       <c r="BL6" s="15" t="n"/>
       <c r="BM6" s="15" t="n"/>
       <c r="BN6" s="15" t="n"/>
+      <c r="BO6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -2048,6 +2067,9 @@
       </c>
       <c r="BN7" s="15" t="n">
         <v>60.77</v>
+      </c>
+      <c r="BO7" s="15" t="n">
+        <v>56.39</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -2200,6 +2222,9 @@
       </c>
       <c r="BN8" s="15" t="n">
         <v>5740.88</v>
+      </c>
+      <c r="BO8" s="15" t="n">
+        <v>5729.95</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2317,6 +2342,7 @@
       <c r="BL9" s="15" t="n"/>
       <c r="BM9" s="15" t="n"/>
       <c r="BN9" s="15" t="n"/>
+      <c r="BO9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2516,6 +2542,9 @@
       </c>
       <c r="BN10" s="15" t="n">
         <v>53.9</v>
+      </c>
+      <c r="BO10" s="15" t="n">
+        <v>50.78</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2668,6 +2697,9 @@
       </c>
       <c r="BN11" s="15" t="n">
         <v>4630.28</v>
+      </c>
+      <c r="BO11" s="15" t="n">
+        <v>4625.09</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -2785,6 +2817,7 @@
       <c r="BL12" s="15" t="n"/>
       <c r="BM12" s="15" t="n"/>
       <c r="BN12" s="15" t="n"/>
+      <c r="BO12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -2984,6 +3017,9 @@
       </c>
       <c r="BN13" s="15" t="n">
         <v>62.54</v>
+      </c>
+      <c r="BO13" s="15" t="n">
+        <v>62.03</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -3136,6 +3172,9 @@
       </c>
       <c r="BN14" s="15" t="n">
         <v>7946.33</v>
+      </c>
+      <c r="BO14" s="15" t="n">
+        <v>7952.1</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -3253,6 +3292,7 @@
       <c r="BL15" s="15" t="n"/>
       <c r="BM15" s="15" t="n"/>
       <c r="BN15" s="15" t="n"/>
+      <c r="BO15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -3452,6 +3492,9 @@
       </c>
       <c r="BN16" s="15" t="n">
         <v>33.7</v>
+      </c>
+      <c r="BO16" s="15" t="n">
+        <v>31.55</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -3604,6 +3647,9 @@
       </c>
       <c r="BN17" s="15" t="n">
         <v>2594.35</v>
+      </c>
+      <c r="BO17" s="15" t="n">
+        <v>2562.04</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -3721,6 +3767,7 @@
       <c r="BL18" s="15" t="n"/>
       <c r="BM18" s="15" t="n"/>
       <c r="BN18" s="15" t="n"/>
+      <c r="BO18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -3920,6 +3967,9 @@
       </c>
       <c r="BN19" s="15" t="n">
         <v>81.34</v>
+      </c>
+      <c r="BO19" s="15" t="n">
+        <v>80.75</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -4072,6 +4122,9 @@
       </c>
       <c r="BN20" s="15" t="n">
         <v>7713.55</v>
+      </c>
+      <c r="BO20" s="15" t="n">
+        <v>7711.76</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -4189,6 +4242,7 @@
       <c r="BL21" s="15" t="n"/>
       <c r="BM21" s="15" t="n"/>
       <c r="BN21" s="15" t="n"/>
+      <c r="BO21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -4385,6 +4439,9 @@
         <v>36.34</v>
       </c>
       <c r="BN22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BO22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -4538,6 +4595,9 @@
       </c>
       <c r="BN23" s="15" t="n">
         <v>76933.59</v>
+      </c>
+      <c r="BO23" s="15" t="n">
+        <v>76924.92999999999</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -4655,6 +4715,7 @@
       <c r="BL24" s="15" t="n"/>
       <c r="BM24" s="15" t="n"/>
       <c r="BN24" s="15" t="n"/>
+      <c r="BO24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -4853,6 +4914,9 @@
         <v>49.88</v>
       </c>
       <c r="BN25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BO25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -4992,6 +5056,9 @@
       </c>
       <c r="BN26" s="15" t="n">
         <v>26253.99</v>
+      </c>
+      <c r="BO26" s="15" t="n">
+        <v>26400.58</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -5109,6 +5176,7 @@
       <c r="BL27" s="15" t="n"/>
       <c r="BM27" s="15" t="n"/>
       <c r="BN27" s="15" t="n"/>
+      <c r="BO27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -5307,6 +5375,9 @@
         <v>92.09</v>
       </c>
       <c r="BN28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BO28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -5460,6 +5531,9 @@
       </c>
       <c r="BN29" s="15" t="n">
         <v>66131.98</v>
+      </c>
+      <c r="BO29" s="15" t="n">
+        <v>66311.92999999999</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -5577,6 +5651,7 @@
       <c r="BL30" s="15" t="n"/>
       <c r="BM30" s="15" t="n"/>
       <c r="BN30" s="15" t="n"/>
+      <c r="BO30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -5775,6 +5850,9 @@
         <v>97.44</v>
       </c>
       <c r="BN31" s="15" t="n">
+        <v>97.44</v>
+      </c>
+      <c r="BO31" s="15" t="n">
         <v>97.44</v>
       </c>
     </row>
@@ -5928,6 +6006,9 @@
       </c>
       <c r="BN32" s="15" t="n">
         <v>6912.37</v>
+      </c>
+      <c r="BO32" s="15" t="n">
+        <v>6820.02</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -6045,6 +6126,7 @@
       <c r="BL33" s="15" t="n"/>
       <c r="BM33" s="15" t="n"/>
       <c r="BN33" s="15" t="n"/>
+      <c r="BO33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -6244,6 +6326,9 @@
       </c>
       <c r="BN34" s="15" t="n">
         <v>45.88</v>
+      </c>
+      <c r="BO34" s="15" t="n">
+        <v>45.48</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -6396,6 +6481,9 @@
       </c>
       <c r="BN35" s="15" t="n">
         <v>5676.05</v>
+      </c>
+      <c r="BO35" s="15" t="n">
+        <v>5718.42</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -6513,6 +6601,7 @@
       <c r="BL36" s="15" t="n"/>
       <c r="BM36" s="15" t="n"/>
       <c r="BN36" s="15" t="n"/>
+      <c r="BO36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -6712,6 +6801,9 @@
       </c>
       <c r="BN37" s="15" t="n">
         <v>57.33</v>
+      </c>
+      <c r="BO37" s="15" t="n">
+        <v>59.29</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -6864,6 +6956,9 @@
       </c>
       <c r="BN38" s="15" t="n">
         <v>11306.87</v>
+      </c>
+      <c r="BO38" s="15" t="n">
+        <v>11317.65</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -6981,6 +7076,7 @@
       <c r="BL39" s="15" t="n"/>
       <c r="BM39" s="15" t="n"/>
       <c r="BN39" s="15" t="n"/>
+      <c r="BO39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -7180,6 +7276,9 @@
       </c>
       <c r="BN40" s="15" t="n">
         <v>50.52</v>
+      </c>
+      <c r="BO40" s="15" t="n">
+        <v>50.7</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -7332,6 +7431,9 @@
       </c>
       <c r="BN41" s="15" t="n">
         <v>11002.01</v>
+      </c>
+      <c r="BO41" s="15" t="n">
+        <v>10941.54</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -7449,6 +7551,7 @@
       <c r="BL42" s="15" t="n"/>
       <c r="BM42" s="15" t="n"/>
       <c r="BN42" s="15" t="n"/>
+      <c r="BO42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -7648,6 +7751,9 @@
       </c>
       <c r="BN43" s="15" t="n">
         <v>50.26</v>
+      </c>
+      <c r="BO43" s="15" t="n">
+        <v>49.33</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -7800,6 +7906,9 @@
       </c>
       <c r="BN44" s="15" t="n">
         <v>3351.48</v>
+      </c>
+      <c r="BO44" s="15" t="n">
+        <v>3372</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -7917,6 +8026,7 @@
       <c r="BL45" s="15" t="n"/>
       <c r="BM45" s="15" t="n"/>
       <c r="BN45" s="15" t="n"/>
+      <c r="BO45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -8116,6 +8226,9 @@
       </c>
       <c r="BN46" s="15" t="n">
         <v>59.12</v>
+      </c>
+      <c r="BO46" s="15" t="n">
+        <v>61.11</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -8268,6 +8381,9 @@
       </c>
       <c r="BN47" s="15" t="n">
         <v>7033.51</v>
+      </c>
+      <c r="BO47" s="15" t="n">
+        <v>6954.12</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -8385,6 +8501,7 @@
       <c r="BL48" s="15" t="n"/>
       <c r="BM48" s="15" t="n"/>
       <c r="BN48" s="15" t="n"/>
+      <c r="BO48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -8584,6 +8701,9 @@
       </c>
       <c r="BN49" s="15" t="n">
         <v>25.33</v>
+      </c>
+      <c r="BO49" s="15" t="n">
+        <v>23.69</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -8736,6 +8856,9 @@
       </c>
       <c r="BN50" s="15" t="n">
         <v>33541.54</v>
+      </c>
+      <c r="BO50" s="15" t="n">
+        <v>34087.79</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -8853,6 +8976,7 @@
       <c r="BL51" s="15" t="n"/>
       <c r="BM51" s="15" t="n"/>
       <c r="BN51" s="15" t="n"/>
+      <c r="BO51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -9052,6 +9176,9 @@
       </c>
       <c r="BN52" s="15" t="n">
         <v>42.98</v>
+      </c>
+      <c r="BO52" s="15" t="n">
+        <v>40.28</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -9204,6 +9331,9 @@
       </c>
       <c r="BN53" s="15" t="n">
         <v>3634.34</v>
+      </c>
+      <c r="BO53" s="15" t="n">
+        <v>3588.13</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -9321,6 +9451,7 @@
       <c r="BL54" s="15" t="n"/>
       <c r="BM54" s="15" t="n"/>
       <c r="BN54" s="15" t="n"/>
+      <c r="BO54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -9520,6 +9651,9 @@
       </c>
       <c r="BN55" s="15" t="n">
         <v>49.17</v>
+      </c>
+      <c r="BO55" s="15" t="n">
+        <v>47.98</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -9672,6 +9806,9 @@
       </c>
       <c r="BN56" s="15" t="n">
         <v>3473.35</v>
+      </c>
+      <c r="BO56" s="15" t="n">
+        <v>3438.68</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -9789,6 +9926,7 @@
       <c r="BL57" s="15" t="n"/>
       <c r="BM57" s="15" t="n"/>
       <c r="BN57" s="15" t="n"/>
+      <c r="BO57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -9988,6 +10126,9 @@
       </c>
       <c r="BN58" s="15" t="n">
         <v>15</v>
+      </c>
+      <c r="BO58" s="15" t="n">
+        <v>15.29</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -10140,6 +10281,9 @@
       </c>
       <c r="BN59" s="15" t="n">
         <v>6842.42</v>
+      </c>
+      <c r="BO59" s="15" t="n">
+        <v>6719.7</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -10257,6 +10401,7 @@
       <c r="BL60" s="15" t="n"/>
       <c r="BM60" s="15" t="n"/>
       <c r="BN60" s="15" t="n"/>
+      <c r="BO60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -10456,6 +10601,9 @@
       </c>
       <c r="BN61" s="15" t="n">
         <v>31.95</v>
+      </c>
+      <c r="BO61" s="15" t="n">
+        <v>35.3</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -10608,6 +10756,9 @@
       </c>
       <c r="BN62" s="15" t="n">
         <v>8289.290000000001</v>
+      </c>
+      <c r="BO62" s="15" t="n">
+        <v>8095.99</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -10725,6 +10876,7 @@
       <c r="BL63" s="15" t="n"/>
       <c r="BM63" s="15" t="n"/>
       <c r="BN63" s="15" t="n"/>
+      <c r="BO63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -10924,6 +11076,9 @@
       </c>
       <c r="BN64" s="15" t="n">
         <v>8.710000000000001</v>
+      </c>
+      <c r="BO64" s="15" t="n">
+        <v>9.91</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -11076,6 +11231,9 @@
       </c>
       <c r="BN65" s="15" t="n">
         <v>10752.99</v>
+      </c>
+      <c r="BO65" s="15" t="n">
+        <v>10784.55</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -11193,6 +11351,7 @@
       <c r="BL66" s="15" t="n"/>
       <c r="BM66" s="15" t="n"/>
       <c r="BN66" s="15" t="n"/>
+      <c r="BO66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -11392,6 +11551,9 @@
       </c>
       <c r="BN67" s="15" t="n">
         <v>20.38</v>
+      </c>
+      <c r="BO67" s="15" t="n">
+        <v>24.34</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -11544,6 +11706,9 @@
       </c>
       <c r="BN68" s="15" t="n">
         <v>11413.66</v>
+      </c>
+      <c r="BO68" s="15" t="n">
+        <v>11479.92</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -11661,6 +11826,7 @@
       <c r="BL69" s="15" t="n"/>
       <c r="BM69" s="15" t="n"/>
       <c r="BN69" s="15" t="n"/>
+      <c r="BO69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -11860,6 +12026,9 @@
       </c>
       <c r="BN70" s="15" t="n">
         <v>16.7</v>
+      </c>
+      <c r="BO70" s="15" t="n">
+        <v>18.1</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -12012,6 +12181,9 @@
       </c>
       <c r="BN71" s="15" t="n">
         <v>6460.01</v>
+      </c>
+      <c r="BO71" s="15" t="n">
+        <v>6405.39</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -12129,6 +12301,7 @@
       <c r="BL72" s="15" t="n"/>
       <c r="BM72" s="15" t="n"/>
       <c r="BN72" s="15" t="n"/>
+      <c r="BO72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -12328,6 +12501,9 @@
       </c>
       <c r="BN73" s="15" t="n">
         <v>17.53</v>
+      </c>
+      <c r="BO73" s="15" t="n">
+        <v>19.93</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -12480,6 +12656,9 @@
       </c>
       <c r="BN74" s="15" t="n">
         <v>12489.39</v>
+      </c>
+      <c r="BO74" s="15" t="n">
+        <v>12480.96</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -12597,6 +12776,7 @@
       <c r="BL75" s="15" t="n"/>
       <c r="BM75" s="15" t="n"/>
       <c r="BN75" s="15" t="n"/>
+      <c r="BO75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -12796,6 +12976,9 @@
       </c>
       <c r="BN76" s="15" t="n">
         <v>51.33</v>
+      </c>
+      <c r="BO76" s="15" t="n">
+        <v>51.39</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -12948,6 +13131,9 @@
       </c>
       <c r="BN77" s="15" t="n">
         <v>16268.73</v>
+      </c>
+      <c r="BO77" s="15" t="n">
+        <v>15569.82</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
@@ -13065,6 +13251,7 @@
       <c r="BL78" s="15" t="n"/>
       <c r="BM78" s="15" t="n"/>
       <c r="BN78" s="15" t="n"/>
+      <c r="BO78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -13264,6 +13451,9 @@
       </c>
       <c r="BN79" s="15" t="n">
         <v>5.49</v>
+      </c>
+      <c r="BO79" s="15" t="n">
+        <v>6.1</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -13416,6 +13606,9 @@
       </c>
       <c r="BN80" s="15" t="n">
         <v>6955.02</v>
+      </c>
+      <c r="BO80" s="15" t="n">
+        <v>6930.11</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -13533,6 +13726,7 @@
       <c r="BL81" s="15" t="n"/>
       <c r="BM81" s="15" t="n"/>
       <c r="BN81" s="15" t="n"/>
+      <c r="BO81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -13732,6 +13926,9 @@
       </c>
       <c r="BN82" s="15" t="n">
         <v>5.04</v>
+      </c>
+      <c r="BO82" s="15" t="n">
+        <v>4.88</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -13884,6 +14081,9 @@
       </c>
       <c r="BN83" s="15" t="n">
         <v>8661.26</v>
+      </c>
+      <c r="BO83" s="15" t="n">
+        <v>8507.450000000001</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -14001,6 +14201,7 @@
       <c r="BL84" s="15" t="n"/>
       <c r="BM84" s="15" t="n"/>
       <c r="BN84" s="15" t="n"/>
+      <c r="BO84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -14200,6 +14401,9 @@
       </c>
       <c r="BN85" s="15" t="n">
         <v>17.02</v>
+      </c>
+      <c r="BO85" s="15" t="n">
+        <v>17.16</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -14352,6 +14556,9 @@
       </c>
       <c r="BN86" s="15" t="n">
         <v>2631.9</v>
+      </c>
+      <c r="BO86" s="15" t="n">
+        <v>2217.09</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -14469,6 +14676,7 @@
       <c r="BL87" s="15" t="n"/>
       <c r="BM87" s="15" t="n"/>
       <c r="BN87" s="15" t="n"/>
+      <c r="BO87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -14668,6 +14876,9 @@
       </c>
       <c r="BN88" s="15" t="n">
         <v>33.41</v>
+      </c>
+      <c r="BO88" s="15" t="n">
+        <v>33.44</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -14820,6 +15031,9 @@
       </c>
       <c r="BN89" s="15" t="n">
         <v>5075.31</v>
+      </c>
+      <c r="BO89" s="15" t="n">
+        <v>4619.87</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -14937,6 +15151,7 @@
       <c r="BL90" s="15" t="n"/>
       <c r="BM90" s="15" t="n"/>
       <c r="BN90" s="15" t="n"/>
+      <c r="BO90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -15136,6 +15351,9 @@
       </c>
       <c r="BN91" s="15" t="n">
         <v>19.14</v>
+      </c>
+      <c r="BO91" s="15" t="n">
+        <v>18.88</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -15288,6 +15506,9 @@
       </c>
       <c r="BN92" s="15" t="n">
         <v>8723.85</v>
+      </c>
+      <c r="BO92" s="15" t="n">
+        <v>8522.209999999999</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -15405,6 +15626,7 @@
       <c r="BL93" s="15" t="n"/>
       <c r="BM93" s="15" t="n"/>
       <c r="BN93" s="15" t="n"/>
+      <c r="BO93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -15604,6 +15826,9 @@
       </c>
       <c r="BN94" s="15" t="n">
         <v>7.73</v>
+      </c>
+      <c r="BO94" s="15" t="n">
+        <v>6.98</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -15756,6 +15981,9 @@
       </c>
       <c r="BN95" s="15" t="n">
         <v>1230.57</v>
+      </c>
+      <c r="BO95" s="15" t="n">
+        <v>1222.61</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -15873,6 +16101,7 @@
       <c r="BL96" s="15" t="n"/>
       <c r="BM96" s="15" t="n"/>
       <c r="BN96" s="15" t="n"/>
+      <c r="BO96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -16072,6 +16301,9 @@
       </c>
       <c r="BN97" s="15" t="n">
         <v>6.77</v>
+      </c>
+      <c r="BO97" s="15" t="n">
+        <v>7.04</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -16224,6 +16456,9 @@
       </c>
       <c r="BN98" s="15" t="n">
         <v>13943.49</v>
+      </c>
+      <c r="BO98" s="15" t="n">
+        <v>13945.5</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -16341,6 +16576,7 @@
       <c r="BL99" s="15" t="n"/>
       <c r="BM99" s="15" t="n"/>
       <c r="BN99" s="15" t="n"/>
+      <c r="BO99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -16540,6 +16776,9 @@
       </c>
       <c r="BN100" s="15" t="n">
         <v>39.95</v>
+      </c>
+      <c r="BO100" s="15" t="n">
+        <v>38.18</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -16692,6 +16931,9 @@
       </c>
       <c r="BN101" s="15" t="n">
         <v>3318.54</v>
+      </c>
+      <c r="BO101" s="15" t="n">
+        <v>3283.79</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -16809,6 +17051,7 @@
       <c r="BL102" s="15" t="n"/>
       <c r="BM102" s="15" t="n"/>
       <c r="BN102" s="15" t="n"/>
+      <c r="BO102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -17008,6 +17251,9 @@
       </c>
       <c r="BN103" s="15" t="n">
         <v>33.67</v>
+      </c>
+      <c r="BO103" s="15" t="n">
+        <v>33.38</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -17160,6 +17406,9 @@
       </c>
       <c r="BN104" s="15" t="n">
         <v>2424.25</v>
+      </c>
+      <c r="BO104" s="15" t="n">
+        <v>2387.17</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -17277,6 +17526,7 @@
       <c r="BL105" s="15" t="n"/>
       <c r="BM105" s="15" t="n"/>
       <c r="BN105" s="15" t="n"/>
+      <c r="BO105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -17476,6 +17726,9 @@
       </c>
       <c r="BN106" s="15" t="n">
         <v>16.21</v>
+      </c>
+      <c r="BO106" s="15" t="n">
+        <v>16.55</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -17628,6 +17881,9 @@
       </c>
       <c r="BN107" s="15" t="n">
         <v>2494.19</v>
+      </c>
+      <c r="BO107" s="15" t="n">
+        <v>2491.47</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -17745,6 +18001,7 @@
       <c r="BL108" s="15" t="n"/>
       <c r="BM108" s="15" t="n"/>
       <c r="BN108" s="15" t="n"/>
+      <c r="BO108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -17944,6 +18201,9 @@
       </c>
       <c r="BN109" s="15" t="n">
         <v>35.69</v>
+      </c>
+      <c r="BO109" s="15" t="n">
+        <v>34.3</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -18096,6 +18356,9 @@
       </c>
       <c r="BN110" s="15" t="n">
         <v>2602.09</v>
+      </c>
+      <c r="BO110" s="15" t="n">
+        <v>2602.89</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -18213,6 +18476,7 @@
       <c r="BL111" s="15" t="n"/>
       <c r="BM111" s="15" t="n"/>
       <c r="BN111" s="15" t="n"/>
+      <c r="BO111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -18412,6 +18676,9 @@
       </c>
       <c r="BN112" s="15" t="n">
         <v>54.26</v>
+      </c>
+      <c r="BO112" s="15" t="n">
+        <v>51.32</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -18562,6 +18829,9 @@
       </c>
       <c r="BN113" s="15" t="n">
         <v>1971.87</v>
+      </c>
+      <c r="BO113" s="15" t="n">
+        <v>1912.23</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -18679,6 +18949,7 @@
       <c r="BL114" s="15" t="n"/>
       <c r="BM114" s="15" t="n"/>
       <c r="BN114" s="15" t="n"/>
+      <c r="BO114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -18878,6 +19149,9 @@
       </c>
       <c r="BN115" s="15" t="n">
         <v>17.88</v>
+      </c>
+      <c r="BO115" s="15" t="n">
+        <v>17.62</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -19015,6 +19289,9 @@
       </c>
       <c r="BN116" s="15" t="n">
         <v>8915.129999999999</v>
+      </c>
+      <c r="BO116" s="15" t="n">
+        <v>8836.23</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -19087,6 +19364,7 @@
       <c r="BL117" s="15" t="n"/>
       <c r="BM117" s="15" t="n"/>
       <c r="BN117" s="15" t="n"/>
+      <c r="BO117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -19242,6 +19520,9 @@
       <c r="BN118" s="15" t="n">
         <v>83.54000000000001</v>
       </c>
+      <c r="BO118" s="15" t="n">
+        <v>75.51000000000001</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -19369,6 +19650,9 @@
       </c>
       <c r="BN119" s="15" t="n">
         <v>13386.38</v>
+      </c>
+      <c r="BO119" s="15" t="n">
+        <v>12866.99</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -19390,6 +19674,7 @@
       <c r="BL120" s="15" t="n"/>
       <c r="BM120" s="15" t="n"/>
       <c r="BN120" s="15" t="n"/>
+      <c r="BO120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -19446,6 +19731,9 @@
       <c r="BN121" s="15" t="n">
         <v>23.67</v>
       </c>
+      <c r="BO121" s="15" t="n">
+        <v>22.05</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -19501,6 +19789,9 @@
       </c>
       <c r="BN122" s="15" t="n">
         <v>1191.9</v>
+      </c>
+      <c r="BO122" s="15" t="n">
+        <v>1193.66</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -19522,6 +19813,7 @@
       <c r="BL123" s="15" t="n"/>
       <c r="BM123" s="15" t="n"/>
       <c r="BN123" s="15" t="n"/>
+      <c r="BO123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -19578,6 +19870,9 @@
       <c r="BN124" s="15" t="n">
         <v>41.8</v>
       </c>
+      <c r="BO124" s="15" t="n">
+        <v>46.13</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -19633,6 +19928,9 @@
       </c>
       <c r="BN125" s="15" t="n">
         <v>11350.16</v>
+      </c>
+      <c r="BO125" s="15" t="n">
+        <v>11558.72</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -19654,6 +19952,7 @@
       <c r="BL126" s="15" t="n"/>
       <c r="BM126" s="15" t="n"/>
       <c r="BN126" s="15" t="n"/>
+      <c r="BO126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -19710,6 +20009,9 @@
       <c r="BN127" s="15" t="n">
         <v>3.4</v>
       </c>
+      <c r="BO127" s="15" t="n">
+        <v>5.93</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -19765,6 +20067,9 @@
       </c>
       <c r="BN128" s="15" t="n">
         <v>1861.56</v>
+      </c>
+      <c r="BO128" s="15" t="n">
+        <v>1905.4</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -19786,6 +20091,7 @@
       <c r="BL129" s="15" t="n"/>
       <c r="BM129" s="15" t="n"/>
       <c r="BN129" s="15" t="n"/>
+      <c r="BO129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -19842,6 +20148,9 @@
       <c r="BN130" s="15" t="n">
         <v>12.63</v>
       </c>
+      <c r="BO130" s="15" t="n">
+        <v>13.34</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -19897,6 +20206,9 @@
       </c>
       <c r="BN131" s="15" t="n">
         <v>769.36</v>
+      </c>
+      <c r="BO131" s="15" t="n">
+        <v>769.05</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -19918,6 +20230,7 @@
       <c r="BL132" s="15" t="n"/>
       <c r="BM132" s="15" t="n"/>
       <c r="BN132" s="15" t="n"/>
+      <c r="BO132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -19974,6 +20287,9 @@
       <c r="BN133" s="15" t="n">
         <v>68.69</v>
       </c>
+      <c r="BO133" s="15" t="n">
+        <v>68.03</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -20029,6 +20345,9 @@
       </c>
       <c r="BN134" s="15" t="n">
         <v>3112.31</v>
+      </c>
+      <c r="BO134" s="15" t="n">
+        <v>3094.52</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -20050,6 +20369,7 @@
       <c r="BL135" s="15" t="n"/>
       <c r="BM135" s="15" t="n"/>
       <c r="BN135" s="15" t="n"/>
+      <c r="BO135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -20106,6 +20426,9 @@
       <c r="BN136" s="15" t="n">
         <v>21.01</v>
       </c>
+      <c r="BO136" s="15" t="n">
+        <v>22.47</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -20161,6 +20484,9 @@
       </c>
       <c r="BN137" s="15" t="n">
         <v>3608.61</v>
+      </c>
+      <c r="BO137" s="15" t="n">
+        <v>3599.35</v>
       </c>
     </row>
     <row r="138">
@@ -20174,6 +20500,7 @@
       <c r="BL138" s="15" t="n"/>
       <c r="BM138" s="15" t="n"/>
       <c r="BN138" s="15" t="n"/>
+      <c r="BO138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -20206,6 +20533,9 @@
       <c r="BN139" s="15" t="n">
         <v>3.72</v>
       </c>
+      <c r="BO139" s="15" t="n">
+        <v>4.17</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -20237,6 +20567,9 @@
       </c>
       <c r="BN140" s="15" t="n">
         <v>2443.4</v>
+      </c>
+      <c r="BO140" s="15" t="n">
+        <v>2430.11</v>
       </c>
     </row>
     <row r="141">
@@ -20250,6 +20583,7 @@
       <c r="BL141" s="15" t="n"/>
       <c r="BM141" s="15" t="n"/>
       <c r="BN141" s="15" t="n"/>
+      <c r="BO141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -20282,6 +20616,9 @@
       <c r="BN142" s="15" t="n">
         <v>12.27</v>
       </c>
+      <c r="BO142" s="15" t="n">
+        <v>16.87</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -20313,6 +20650,9 @@
       </c>
       <c r="BN143" s="15" t="n">
         <v>5446.1</v>
+      </c>
+      <c r="BO143" s="15" t="n">
+        <v>5572.31</v>
       </c>
     </row>
     <row r="144">
@@ -20321,6 +20661,7 @@
       <c r="BL144" s="15" t="n"/>
       <c r="BM144" s="15" t="n"/>
       <c r="BN144" s="15" t="n"/>
+      <c r="BO144" s="15" t="n"/>
     </row>
     <row r="145">
       <c r="BJ145" s="15" t="n">
@@ -20338,6 +20679,9 @@
       <c r="BN145" s="15" t="n">
         <v>25.55</v>
       </c>
+      <c r="BO145" s="15" t="n">
+        <v>27.7</v>
+      </c>
     </row>
     <row r="146">
       <c r="BJ146" s="15" t="n">
@@ -20354,6 +20698,9 @@
       </c>
       <c r="BN146" s="15" t="n">
         <v>2305.74</v>
+      </c>
+      <c r="BO146" s="15" t="n">
+        <v>2319.23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-09-03 08:20:23]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BO146"/>
+  <dimension ref="A1:BP146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -601,6 +601,7 @@
     <col width="15" customWidth="1" min="65" max="65"/>
     <col width="15" customWidth="1" min="66" max="66"/>
     <col width="15" customWidth="1" min="67" max="67"/>
+    <col width="15" customWidth="1" min="68" max="68"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -939,6 +940,11 @@
           <t>2026/08/31</t>
         </is>
       </c>
+      <c r="BP1" s="15" t="inlineStr">
+        <is>
+          <t>2026/09/03</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1276,6 +1282,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BP2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1479,6 +1490,9 @@
       <c r="BO3" s="15" t="n">
         <v>65.77</v>
       </c>
+      <c r="BP3" s="15" t="n">
+        <v>60.14</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1681,6 +1695,9 @@
       </c>
       <c r="BO4" s="15" t="n">
         <v>3986.3</v>
+      </c>
+      <c r="BP4" s="15" t="n">
+        <v>3942.09</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1751,6 +1768,7 @@
       <c r="BM5" s="15" t="n"/>
       <c r="BN5" s="15" t="n"/>
       <c r="BO5" s="15" t="n"/>
+      <c r="BP5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1868,6 +1886,7 @@
       <c r="BM6" s="15" t="n"/>
       <c r="BN6" s="15" t="n"/>
       <c r="BO6" s="15" t="n"/>
+      <c r="BP6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -2070,6 +2089,9 @@
       </c>
       <c r="BO7" s="15" t="n">
         <v>56.39</v>
+      </c>
+      <c r="BP7" s="15" t="n">
+        <v>54.76</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -2225,6 +2247,9 @@
       </c>
       <c r="BO8" s="15" t="n">
         <v>5729.95</v>
+      </c>
+      <c r="BP8" s="15" t="n">
+        <v>5623.55</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2343,6 +2368,7 @@
       <c r="BM9" s="15" t="n"/>
       <c r="BN9" s="15" t="n"/>
       <c r="BO9" s="15" t="n"/>
+      <c r="BP9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2545,6 +2571,9 @@
       </c>
       <c r="BO10" s="15" t="n">
         <v>50.78</v>
+      </c>
+      <c r="BP10" s="15" t="n">
+        <v>50.47</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2700,6 +2729,9 @@
       </c>
       <c r="BO11" s="15" t="n">
         <v>4625.09</v>
+      </c>
+      <c r="BP11" s="15" t="n">
+        <v>4552.58</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -2818,6 +2850,7 @@
       <c r="BM12" s="15" t="n"/>
       <c r="BN12" s="15" t="n"/>
       <c r="BO12" s="15" t="n"/>
+      <c r="BP12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -3020,6 +3053,9 @@
       </c>
       <c r="BO13" s="15" t="n">
         <v>62.03</v>
+      </c>
+      <c r="BP13" s="15" t="n">
+        <v>59.8</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -3175,6 +3211,9 @@
       </c>
       <c r="BO14" s="15" t="n">
         <v>7952.1</v>
+      </c>
+      <c r="BP14" s="15" t="n">
+        <v>7755.36</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -3293,6 +3332,7 @@
       <c r="BM15" s="15" t="n"/>
       <c r="BN15" s="15" t="n"/>
       <c r="BO15" s="15" t="n"/>
+      <c r="BP15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -3495,6 +3535,9 @@
       </c>
       <c r="BO16" s="15" t="n">
         <v>31.55</v>
+      </c>
+      <c r="BP16" s="15" t="n">
+        <v>30.57</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -3650,6 +3693,9 @@
       </c>
       <c r="BO17" s="15" t="n">
         <v>2562.04</v>
+      </c>
+      <c r="BP17" s="15" t="n">
+        <v>2571.45</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -3768,6 +3814,7 @@
       <c r="BM18" s="15" t="n"/>
       <c r="BN18" s="15" t="n"/>
       <c r="BO18" s="15" t="n"/>
+      <c r="BP18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -3970,6 +4017,9 @@
       </c>
       <c r="BO19" s="15" t="n">
         <v>80.75</v>
+      </c>
+      <c r="BP19" s="15" t="n">
+        <v>79.98</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -4125,6 +4175,9 @@
       </c>
       <c r="BO20" s="15" t="n">
         <v>7711.76</v>
+      </c>
+      <c r="BP20" s="15" t="n">
+        <v>7666.6</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -4243,6 +4296,7 @@
       <c r="BM21" s="15" t="n"/>
       <c r="BN21" s="15" t="n"/>
       <c r="BO21" s="15" t="n"/>
+      <c r="BP21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -4442,6 +4496,9 @@
         <v>36.34</v>
       </c>
       <c r="BO22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BP22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -4598,6 +4655,9 @@
       </c>
       <c r="BO23" s="15" t="n">
         <v>76924.92999999999</v>
+      </c>
+      <c r="BP23" s="15" t="n">
+        <v>76593.75</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -4716,6 +4776,7 @@
       <c r="BM24" s="15" t="n"/>
       <c r="BN24" s="15" t="n"/>
       <c r="BO24" s="15" t="n"/>
+      <c r="BP24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -4917,6 +4978,9 @@
         <v>49.88</v>
       </c>
       <c r="BO25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BP25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -5059,6 +5123,9 @@
       </c>
       <c r="BO26" s="15" t="n">
         <v>26400.58</v>
+      </c>
+      <c r="BP26" s="15" t="n">
+        <v>25847.99</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -5177,6 +5244,7 @@
       <c r="BM27" s="15" t="n"/>
       <c r="BN27" s="15" t="n"/>
       <c r="BO27" s="15" t="n"/>
+      <c r="BP27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -5378,6 +5446,9 @@
         <v>92.09</v>
       </c>
       <c r="BO28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BP28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -5534,6 +5605,9 @@
       </c>
       <c r="BO29" s="15" t="n">
         <v>66311.92999999999</v>
+      </c>
+      <c r="BP29" s="15" t="n">
+        <v>64214.48</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -5652,6 +5726,7 @@
       <c r="BM30" s="15" t="n"/>
       <c r="BN30" s="15" t="n"/>
       <c r="BO30" s="15" t="n"/>
+      <c r="BP30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -5853,6 +5928,9 @@
         <v>97.44</v>
       </c>
       <c r="BO31" s="15" t="n">
+        <v>97.44</v>
+      </c>
+      <c r="BP31" s="15" t="n">
         <v>97.44</v>
       </c>
     </row>
@@ -6009,6 +6087,9 @@
       </c>
       <c r="BO32" s="15" t="n">
         <v>6820.02</v>
+      </c>
+      <c r="BP32" s="15" t="n">
+        <v>6579.48</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -6127,6 +6208,7 @@
       <c r="BM33" s="15" t="n"/>
       <c r="BN33" s="15" t="n"/>
       <c r="BO33" s="15" t="n"/>
+      <c r="BP33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -6329,6 +6411,9 @@
       </c>
       <c r="BO34" s="15" t="n">
         <v>45.48</v>
+      </c>
+      <c r="BP34" s="15" t="n">
+        <v>45.86</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -6484,6 +6569,9 @@
       </c>
       <c r="BO35" s="15" t="n">
         <v>5718.42</v>
+      </c>
+      <c r="BP35" s="15" t="n">
+        <v>5635.06</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -6602,6 +6690,7 @@
       <c r="BM36" s="15" t="n"/>
       <c r="BN36" s="15" t="n"/>
       <c r="BO36" s="15" t="n"/>
+      <c r="BP36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -6804,6 +6893,9 @@
       </c>
       <c r="BO37" s="15" t="n">
         <v>59.29</v>
+      </c>
+      <c r="BP37" s="15" t="n">
+        <v>52.57</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -6959,6 +7051,9 @@
       </c>
       <c r="BO38" s="15" t="n">
         <v>11317.65</v>
+      </c>
+      <c r="BP38" s="15" t="n">
+        <v>11353.77</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -7077,6 +7172,7 @@
       <c r="BM39" s="15" t="n"/>
       <c r="BN39" s="15" t="n"/>
       <c r="BO39" s="15" t="n"/>
+      <c r="BP39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -7279,6 +7375,9 @@
       </c>
       <c r="BO40" s="15" t="n">
         <v>50.7</v>
+      </c>
+      <c r="BP40" s="15" t="n">
+        <v>47.49</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -7434,6 +7533,9 @@
       </c>
       <c r="BO41" s="15" t="n">
         <v>10941.54</v>
+      </c>
+      <c r="BP41" s="15" t="n">
+        <v>11083.48</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -7552,6 +7654,7 @@
       <c r="BM42" s="15" t="n"/>
       <c r="BN42" s="15" t="n"/>
       <c r="BO42" s="15" t="n"/>
+      <c r="BP42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -7754,6 +7857,9 @@
       </c>
       <c r="BO43" s="15" t="n">
         <v>49.33</v>
+      </c>
+      <c r="BP43" s="15" t="n">
+        <v>48.81</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -7909,6 +8015,9 @@
       </c>
       <c r="BO44" s="15" t="n">
         <v>3372</v>
+      </c>
+      <c r="BP44" s="15" t="n">
+        <v>3345.83</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -8027,6 +8136,7 @@
       <c r="BM45" s="15" t="n"/>
       <c r="BN45" s="15" t="n"/>
       <c r="BO45" s="15" t="n"/>
+      <c r="BP45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -8229,6 +8339,9 @@
       </c>
       <c r="BO46" s="15" t="n">
         <v>61.11</v>
+      </c>
+      <c r="BP46" s="15" t="n">
+        <v>52.5</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -8384,6 +8497,9 @@
       </c>
       <c r="BO47" s="15" t="n">
         <v>6954.12</v>
+      </c>
+      <c r="BP47" s="15" t="n">
+        <v>7050.7</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -8502,6 +8618,7 @@
       <c r="BM48" s="15" t="n"/>
       <c r="BN48" s="15" t="n"/>
       <c r="BO48" s="15" t="n"/>
+      <c r="BP48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -8704,6 +8821,9 @@
       </c>
       <c r="BO49" s="15" t="n">
         <v>23.69</v>
+      </c>
+      <c r="BP49" s="15" t="n">
+        <v>21.94</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -8859,6 +8979,9 @@
       </c>
       <c r="BO50" s="15" t="n">
         <v>34087.79</v>
+      </c>
+      <c r="BP50" s="15" t="n">
+        <v>33673.16</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -8977,6 +9100,7 @@
       <c r="BM51" s="15" t="n"/>
       <c r="BN51" s="15" t="n"/>
       <c r="BO51" s="15" t="n"/>
+      <c r="BP51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -9179,6 +9303,9 @@
       </c>
       <c r="BO52" s="15" t="n">
         <v>40.28</v>
+      </c>
+      <c r="BP52" s="15" t="n">
+        <v>36.89</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -9334,6 +9461,9 @@
       </c>
       <c r="BO53" s="15" t="n">
         <v>3588.13</v>
+      </c>
+      <c r="BP53" s="15" t="n">
+        <v>3449.92</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -9452,6 +9582,7 @@
       <c r="BM54" s="15" t="n"/>
       <c r="BN54" s="15" t="n"/>
       <c r="BO54" s="15" t="n"/>
+      <c r="BP54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -9654,6 +9785,9 @@
       </c>
       <c r="BO55" s="15" t="n">
         <v>47.98</v>
+      </c>
+      <c r="BP55" s="15" t="n">
+        <v>44.16</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -9809,6 +9943,9 @@
       </c>
       <c r="BO56" s="15" t="n">
         <v>3438.68</v>
+      </c>
+      <c r="BP56" s="15" t="n">
+        <v>3312.54</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -9927,6 +10064,7 @@
       <c r="BM57" s="15" t="n"/>
       <c r="BN57" s="15" t="n"/>
       <c r="BO57" s="15" t="n"/>
+      <c r="BP57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -10129,6 +10267,9 @@
       </c>
       <c r="BO58" s="15" t="n">
         <v>15.29</v>
+      </c>
+      <c r="BP58" s="15" t="n">
+        <v>13.94</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -10284,6 +10425,9 @@
       </c>
       <c r="BO59" s="15" t="n">
         <v>6719.7</v>
+      </c>
+      <c r="BP59" s="15" t="n">
+        <v>6690.39</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -10402,6 +10546,7 @@
       <c r="BM60" s="15" t="n"/>
       <c r="BN60" s="15" t="n"/>
       <c r="BO60" s="15" t="n"/>
+      <c r="BP60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -10604,6 +10749,9 @@
       </c>
       <c r="BO61" s="15" t="n">
         <v>35.3</v>
+      </c>
+      <c r="BP61" s="15" t="n">
+        <v>32.61</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -10759,6 +10907,9 @@
       </c>
       <c r="BO62" s="15" t="n">
         <v>8095.99</v>
+      </c>
+      <c r="BP62" s="15" t="n">
+        <v>8149.53</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -10877,6 +11028,7 @@
       <c r="BM63" s="15" t="n"/>
       <c r="BN63" s="15" t="n"/>
       <c r="BO63" s="15" t="n"/>
+      <c r="BP63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -11079,6 +11231,9 @@
       </c>
       <c r="BO64" s="15" t="n">
         <v>9.91</v>
+      </c>
+      <c r="BP64" s="15" t="n">
+        <v>9.82</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -11234,6 +11389,9 @@
       </c>
       <c r="BO65" s="15" t="n">
         <v>10784.55</v>
+      </c>
+      <c r="BP65" s="15" t="n">
+        <v>10831.21</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -11352,6 +11510,7 @@
       <c r="BM66" s="15" t="n"/>
       <c r="BN66" s="15" t="n"/>
       <c r="BO66" s="15" t="n"/>
+      <c r="BP66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -11554,6 +11713,9 @@
       </c>
       <c r="BO67" s="15" t="n">
         <v>24.34</v>
+      </c>
+      <c r="BP67" s="15" t="n">
+        <v>24.09</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -11709,6 +11871,9 @@
       </c>
       <c r="BO68" s="15" t="n">
         <v>11479.92</v>
+      </c>
+      <c r="BP68" s="15" t="n">
+        <v>11352.7</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -11827,6 +11992,7 @@
       <c r="BM69" s="15" t="n"/>
       <c r="BN69" s="15" t="n"/>
       <c r="BO69" s="15" t="n"/>
+      <c r="BP69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -12029,6 +12195,9 @@
       </c>
       <c r="BO70" s="15" t="n">
         <v>18.1</v>
+      </c>
+      <c r="BP70" s="15" t="n">
+        <v>18.81</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -12184,6 +12353,9 @@
       </c>
       <c r="BO71" s="15" t="n">
         <v>6405.39</v>
+      </c>
+      <c r="BP71" s="15" t="n">
+        <v>6436.71</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -12302,6 +12474,7 @@
       <c r="BM72" s="15" t="n"/>
       <c r="BN72" s="15" t="n"/>
       <c r="BO72" s="15" t="n"/>
+      <c r="BP72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -12504,6 +12677,9 @@
       </c>
       <c r="BO73" s="15" t="n">
         <v>19.93</v>
+      </c>
+      <c r="BP73" s="15" t="n">
+        <v>19.37</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -12659,6 +12835,9 @@
       </c>
       <c r="BO74" s="15" t="n">
         <v>12480.96</v>
+      </c>
+      <c r="BP74" s="15" t="n">
+        <v>12478.59</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -12777,6 +12956,7 @@
       <c r="BM75" s="15" t="n"/>
       <c r="BN75" s="15" t="n"/>
       <c r="BO75" s="15" t="n"/>
+      <c r="BP75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -12979,6 +13159,9 @@
       </c>
       <c r="BO76" s="15" t="n">
         <v>51.39</v>
+      </c>
+      <c r="BP76" s="15" t="n">
+        <v>50.91</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -13133,6 +13316,9 @@
         <v>16268.73</v>
       </c>
       <c r="BO77" s="15" t="n">
+        <v>15569.82</v>
+      </c>
+      <c r="BP77" s="15" t="n">
         <v>15569.82</v>
       </c>
     </row>
@@ -13252,6 +13438,7 @@
       <c r="BM78" s="15" t="n"/>
       <c r="BN78" s="15" t="n"/>
       <c r="BO78" s="15" t="n"/>
+      <c r="BP78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -13454,6 +13641,9 @@
       </c>
       <c r="BO79" s="15" t="n">
         <v>6.1</v>
+      </c>
+      <c r="BP79" s="15" t="n">
+        <v>3.56</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -13609,6 +13799,9 @@
       </c>
       <c r="BO80" s="15" t="n">
         <v>6930.11</v>
+      </c>
+      <c r="BP80" s="15" t="n">
+        <v>6753.16</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -13727,6 +13920,7 @@
       <c r="BM81" s="15" t="n"/>
       <c r="BN81" s="15" t="n"/>
       <c r="BO81" s="15" t="n"/>
+      <c r="BP81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -13929,6 +14123,9 @@
       </c>
       <c r="BO82" s="15" t="n">
         <v>4.88</v>
+      </c>
+      <c r="BP82" s="15" t="n">
+        <v>4.21</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -14084,6 +14281,9 @@
       </c>
       <c r="BO83" s="15" t="n">
         <v>8507.450000000001</v>
+      </c>
+      <c r="BP83" s="15" t="n">
+        <v>8473</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -14202,6 +14402,7 @@
       <c r="BM84" s="15" t="n"/>
       <c r="BN84" s="15" t="n"/>
       <c r="BO84" s="15" t="n"/>
+      <c r="BP84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -14404,6 +14605,9 @@
       </c>
       <c r="BO85" s="15" t="n">
         <v>17.16</v>
+      </c>
+      <c r="BP85" s="15" t="n">
+        <v>14.53</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -14559,6 +14763,9 @@
       </c>
       <c r="BO86" s="15" t="n">
         <v>2217.09</v>
+      </c>
+      <c r="BP86" s="15" t="n">
+        <v>2126.97</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -14677,6 +14884,7 @@
       <c r="BM87" s="15" t="n"/>
       <c r="BN87" s="15" t="n"/>
       <c r="BO87" s="15" t="n"/>
+      <c r="BP87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -14879,6 +15087,9 @@
       </c>
       <c r="BO88" s="15" t="n">
         <v>33.44</v>
+      </c>
+      <c r="BP88" s="15" t="n">
+        <v>30.27</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -15034,6 +15245,9 @@
       </c>
       <c r="BO89" s="15" t="n">
         <v>4619.87</v>
+      </c>
+      <c r="BP89" s="15" t="n">
+        <v>4459.72</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -15152,6 +15366,7 @@
       <c r="BM90" s="15" t="n"/>
       <c r="BN90" s="15" t="n"/>
       <c r="BO90" s="15" t="n"/>
+      <c r="BP90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -15354,6 +15569,9 @@
       </c>
       <c r="BO91" s="15" t="n">
         <v>18.88</v>
+      </c>
+      <c r="BP91" s="15" t="n">
+        <v>16.21</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -15509,6 +15727,9 @@
       </c>
       <c r="BO92" s="15" t="n">
         <v>8522.209999999999</v>
+      </c>
+      <c r="BP92" s="15" t="n">
+        <v>8528.389999999999</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -15627,6 +15848,7 @@
       <c r="BM93" s="15" t="n"/>
       <c r="BN93" s="15" t="n"/>
       <c r="BO93" s="15" t="n"/>
+      <c r="BP93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -15829,6 +16051,9 @@
       </c>
       <c r="BO94" s="15" t="n">
         <v>6.98</v>
+      </c>
+      <c r="BP94" s="15" t="n">
+        <v>6.59</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -15984,6 +16209,9 @@
       </c>
       <c r="BO95" s="15" t="n">
         <v>1222.61</v>
+      </c>
+      <c r="BP95" s="15" t="n">
+        <v>1243.68</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -16102,6 +16330,7 @@
       <c r="BM96" s="15" t="n"/>
       <c r="BN96" s="15" t="n"/>
       <c r="BO96" s="15" t="n"/>
+      <c r="BP96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -16304,6 +16533,9 @@
       </c>
       <c r="BO97" s="15" t="n">
         <v>7.04</v>
+      </c>
+      <c r="BP97" s="15" t="n">
+        <v>10.13</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -16459,6 +16691,9 @@
       </c>
       <c r="BO98" s="15" t="n">
         <v>13945.5</v>
+      </c>
+      <c r="BP98" s="15" t="n">
+        <v>13880.34</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -16577,6 +16812,7 @@
       <c r="BM99" s="15" t="n"/>
       <c r="BN99" s="15" t="n"/>
       <c r="BO99" s="15" t="n"/>
+      <c r="BP99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -16779,6 +17015,9 @@
       </c>
       <c r="BO100" s="15" t="n">
         <v>38.18</v>
+      </c>
+      <c r="BP100" s="15" t="n">
+        <v>33.41</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -16934,6 +17173,9 @@
       </c>
       <c r="BO101" s="15" t="n">
         <v>3283.79</v>
+      </c>
+      <c r="BP101" s="15" t="n">
+        <v>3215.2</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -17052,6 +17294,7 @@
       <c r="BM102" s="15" t="n"/>
       <c r="BN102" s="15" t="n"/>
       <c r="BO102" s="15" t="n"/>
+      <c r="BP102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -17254,6 +17497,9 @@
       </c>
       <c r="BO103" s="15" t="n">
         <v>33.38</v>
+      </c>
+      <c r="BP103" s="15" t="n">
+        <v>30.48</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -17409,6 +17655,9 @@
       </c>
       <c r="BO104" s="15" t="n">
         <v>2387.17</v>
+      </c>
+      <c r="BP104" s="15" t="n">
+        <v>2305.71</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -17527,6 +17776,7 @@
       <c r="BM105" s="15" t="n"/>
       <c r="BN105" s="15" t="n"/>
       <c r="BO105" s="15" t="n"/>
+      <c r="BP105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -17729,6 +17979,9 @@
       </c>
       <c r="BO106" s="15" t="n">
         <v>16.55</v>
+      </c>
+      <c r="BP106" s="15" t="n">
+        <v>13.55</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -17883,6 +18136,9 @@
         <v>2494.19</v>
       </c>
       <c r="BO107" s="15" t="n">
+        <v>2491.47</v>
+      </c>
+      <c r="BP107" s="15" t="n">
         <v>2491.47</v>
       </c>
     </row>
@@ -18002,6 +18258,7 @@
       <c r="BM108" s="15" t="n"/>
       <c r="BN108" s="15" t="n"/>
       <c r="BO108" s="15" t="n"/>
+      <c r="BP108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -18204,6 +18461,9 @@
       </c>
       <c r="BO109" s="15" t="n">
         <v>34.3</v>
+      </c>
+      <c r="BP109" s="15" t="n">
+        <v>30.62</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -18359,6 +18619,9 @@
       </c>
       <c r="BO110" s="15" t="n">
         <v>2602.89</v>
+      </c>
+      <c r="BP110" s="15" t="n">
+        <v>2499.93</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -18477,6 +18740,7 @@
       <c r="BM111" s="15" t="n"/>
       <c r="BN111" s="15" t="n"/>
       <c r="BO111" s="15" t="n"/>
+      <c r="BP111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -18679,6 +18943,9 @@
       </c>
       <c r="BO112" s="15" t="n">
         <v>51.32</v>
+      </c>
+      <c r="BP112" s="15" t="n">
+        <v>48.1</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -18832,6 +19099,9 @@
       </c>
       <c r="BO113" s="15" t="n">
         <v>1912.23</v>
+      </c>
+      <c r="BP113" s="15" t="n">
+        <v>1898.76</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -18950,6 +19220,7 @@
       <c r="BM114" s="15" t="n"/>
       <c r="BN114" s="15" t="n"/>
       <c r="BO114" s="15" t="n"/>
+      <c r="BP114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -19152,6 +19423,9 @@
       </c>
       <c r="BO115" s="15" t="n">
         <v>17.62</v>
+      </c>
+      <c r="BP115" s="15" t="n">
+        <v>17.14</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -19292,6 +19566,9 @@
       </c>
       <c r="BO116" s="15" t="n">
         <v>8836.23</v>
+      </c>
+      <c r="BP116" s="15" t="n">
+        <v>8769.57</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -19365,6 +19642,7 @@
       <c r="BM117" s="15" t="n"/>
       <c r="BN117" s="15" t="n"/>
       <c r="BO117" s="15" t="n"/>
+      <c r="BP117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -19523,6 +19801,9 @@
       <c r="BO118" s="15" t="n">
         <v>75.51000000000001</v>
       </c>
+      <c r="BP118" s="15" t="n">
+        <v>74.13</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -19653,6 +19934,9 @@
       </c>
       <c r="BO119" s="15" t="n">
         <v>12866.99</v>
+      </c>
+      <c r="BP119" s="15" t="n">
+        <v>12659.95</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -19675,6 +19959,7 @@
       <c r="BM120" s="15" t="n"/>
       <c r="BN120" s="15" t="n"/>
       <c r="BO120" s="15" t="n"/>
+      <c r="BP120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -19734,6 +20019,9 @@
       <c r="BO121" s="15" t="n">
         <v>22.05</v>
       </c>
+      <c r="BP121" s="15" t="n">
+        <v>25.34</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -19792,6 +20080,9 @@
       </c>
       <c r="BO122" s="15" t="n">
         <v>1193.66</v>
+      </c>
+      <c r="BP122" s="15" t="n">
+        <v>1221.87</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -19814,6 +20105,7 @@
       <c r="BM123" s="15" t="n"/>
       <c r="BN123" s="15" t="n"/>
       <c r="BO123" s="15" t="n"/>
+      <c r="BP123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -19873,6 +20165,9 @@
       <c r="BO124" s="15" t="n">
         <v>46.13</v>
       </c>
+      <c r="BP124" s="15" t="n">
+        <v>46.52</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -19931,6 +20226,9 @@
       </c>
       <c r="BO125" s="15" t="n">
         <v>11558.72</v>
+      </c>
+      <c r="BP125" s="15" t="n">
+        <v>11534.72</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -19953,6 +20251,7 @@
       <c r="BM126" s="15" t="n"/>
       <c r="BN126" s="15" t="n"/>
       <c r="BO126" s="15" t="n"/>
+      <c r="BP126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -20012,6 +20311,9 @@
       <c r="BO127" s="15" t="n">
         <v>5.93</v>
       </c>
+      <c r="BP127" s="15" t="n">
+        <v>5.42</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -20070,6 +20372,9 @@
       </c>
       <c r="BO128" s="15" t="n">
         <v>1905.4</v>
+      </c>
+      <c r="BP128" s="15" t="n">
+        <v>1882.19</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -20092,6 +20397,7 @@
       <c r="BM129" s="15" t="n"/>
       <c r="BN129" s="15" t="n"/>
       <c r="BO129" s="15" t="n"/>
+      <c r="BP129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -20151,6 +20457,9 @@
       <c r="BO130" s="15" t="n">
         <v>13.34</v>
       </c>
+      <c r="BP130" s="15" t="n">
+        <v>10.98</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -20209,6 +20518,9 @@
       </c>
       <c r="BO131" s="15" t="n">
         <v>769.05</v>
+      </c>
+      <c r="BP131" s="15" t="n">
+        <v>764.0700000000001</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -20231,6 +20543,7 @@
       <c r="BM132" s="15" t="n"/>
       <c r="BN132" s="15" t="n"/>
       <c r="BO132" s="15" t="n"/>
+      <c r="BP132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -20290,6 +20603,9 @@
       <c r="BO133" s="15" t="n">
         <v>68.03</v>
       </c>
+      <c r="BP133" s="15" t="n">
+        <v>63.29</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -20347,6 +20663,9 @@
         <v>3112.31</v>
       </c>
       <c r="BO134" s="15" t="n">
+        <v>3094.52</v>
+      </c>
+      <c r="BP134" s="15" t="n">
         <v>3094.52</v>
       </c>
     </row>
@@ -20370,6 +20689,7 @@
       <c r="BM135" s="15" t="n"/>
       <c r="BN135" s="15" t="n"/>
       <c r="BO135" s="15" t="n"/>
+      <c r="BP135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -20429,6 +20749,9 @@
       <c r="BO136" s="15" t="n">
         <v>22.47</v>
       </c>
+      <c r="BP136" s="15" t="n">
+        <v>21.88</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -20487,6 +20810,9 @@
       </c>
       <c r="BO137" s="15" t="n">
         <v>3599.35</v>
+      </c>
+      <c r="BP137" s="15" t="n">
+        <v>3565.52</v>
       </c>
     </row>
     <row r="138">
@@ -20501,6 +20827,7 @@
       <c r="BM138" s="15" t="n"/>
       <c r="BN138" s="15" t="n"/>
       <c r="BO138" s="15" t="n"/>
+      <c r="BP138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -20536,6 +20863,9 @@
       <c r="BO139" s="15" t="n">
         <v>4.17</v>
       </c>
+      <c r="BP139" s="15" t="n">
+        <v>4.04</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -20570,6 +20900,9 @@
       </c>
       <c r="BO140" s="15" t="n">
         <v>2430.11</v>
+      </c>
+      <c r="BP140" s="15" t="n">
+        <v>2412.96</v>
       </c>
     </row>
     <row r="141">
@@ -20584,6 +20917,7 @@
       <c r="BM141" s="15" t="n"/>
       <c r="BN141" s="15" t="n"/>
       <c r="BO141" s="15" t="n"/>
+      <c r="BP141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -20619,6 +20953,9 @@
       <c r="BO142" s="15" t="n">
         <v>16.87</v>
       </c>
+      <c r="BP142" s="15" t="n">
+        <v>19.78</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -20653,6 +20990,9 @@
       </c>
       <c r="BO143" s="15" t="n">
         <v>5572.31</v>
+      </c>
+      <c r="BP143" s="15" t="n">
+        <v>5665.88</v>
       </c>
     </row>
     <row r="144">
@@ -20662,6 +21002,7 @@
       <c r="BM144" s="15" t="n"/>
       <c r="BN144" s="15" t="n"/>
       <c r="BO144" s="15" t="n"/>
+      <c r="BP144" s="15" t="n"/>
     </row>
     <row r="145">
       <c r="BJ145" s="15" t="n">
@@ -20682,6 +21023,9 @@
       <c r="BO145" s="15" t="n">
         <v>27.7</v>
       </c>
+      <c r="BP145" s="15" t="n">
+        <v>2.34</v>
+      </c>
     </row>
     <row r="146">
       <c r="BJ146" s="15" t="n">
@@ -20701,6 +21045,9 @@
       </c>
       <c r="BO146" s="15" t="n">
         <v>2319.23</v>
+      </c>
+      <c r="BP146" s="15" t="n">
+        <v>2309.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-09-07 08:41:06]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BP146"/>
+  <dimension ref="A1:BQ146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -602,6 +602,7 @@
     <col width="15" customWidth="1" min="66" max="66"/>
     <col width="15" customWidth="1" min="67" max="67"/>
     <col width="15" customWidth="1" min="68" max="68"/>
+    <col width="15" customWidth="1" min="69" max="69"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -945,6 +946,11 @@
           <t>2026/09/03</t>
         </is>
       </c>
+      <c r="BQ1" s="15" t="inlineStr">
+        <is>
+          <t>2026/09/07</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1287,6 +1293,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BQ2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1493,6 +1504,9 @@
       <c r="BP3" s="15" t="n">
         <v>60.14</v>
       </c>
+      <c r="BQ3" s="15" t="n">
+        <v>59.89</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1698,6 +1712,9 @@
       </c>
       <c r="BP4" s="15" t="n">
         <v>3942.09</v>
+      </c>
+      <c r="BQ4" s="15" t="n">
+        <v>3932.7</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1769,6 +1786,7 @@
       <c r="BN5" s="15" t="n"/>
       <c r="BO5" s="15" t="n"/>
       <c r="BP5" s="15" t="n"/>
+      <c r="BQ5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1887,6 +1905,7 @@
       <c r="BN6" s="15" t="n"/>
       <c r="BO6" s="15" t="n"/>
       <c r="BP6" s="15" t="n"/>
+      <c r="BQ6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -2092,6 +2111,9 @@
       </c>
       <c r="BP7" s="15" t="n">
         <v>54.76</v>
+      </c>
+      <c r="BQ7" s="15" t="n">
+        <v>54.47</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -2250,6 +2272,9 @@
       </c>
       <c r="BP8" s="15" t="n">
         <v>5623.55</v>
+      </c>
+      <c r="BQ8" s="15" t="n">
+        <v>5644.97</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2369,6 +2394,7 @@
       <c r="BN9" s="15" t="n"/>
       <c r="BO9" s="15" t="n"/>
       <c r="BP9" s="15" t="n"/>
+      <c r="BQ9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2574,6 +2600,9 @@
       </c>
       <c r="BP10" s="15" t="n">
         <v>50.47</v>
+      </c>
+      <c r="BQ10" s="15" t="n">
+        <v>50.57</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2732,6 +2761,9 @@
       </c>
       <c r="BP11" s="15" t="n">
         <v>4552.58</v>
+      </c>
+      <c r="BQ11" s="15" t="n">
+        <v>4575.02</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -2851,6 +2883,7 @@
       <c r="BN12" s="15" t="n"/>
       <c r="BO12" s="15" t="n"/>
       <c r="BP12" s="15" t="n"/>
+      <c r="BQ12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -3056,6 +3089,9 @@
       </c>
       <c r="BP13" s="15" t="n">
         <v>59.8</v>
+      </c>
+      <c r="BQ13" s="15" t="n">
+        <v>58.69</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -3214,6 +3250,9 @@
       </c>
       <c r="BP14" s="15" t="n">
         <v>7755.36</v>
+      </c>
+      <c r="BQ14" s="15" t="n">
+        <v>7759.37</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -3333,6 +3372,7 @@
       <c r="BN15" s="15" t="n"/>
       <c r="BO15" s="15" t="n"/>
       <c r="BP15" s="15" t="n"/>
+      <c r="BQ15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -3538,6 +3578,9 @@
       </c>
       <c r="BP16" s="15" t="n">
         <v>30.57</v>
+      </c>
+      <c r="BQ16" s="15" t="n">
+        <v>30.79</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -3696,6 +3739,9 @@
       </c>
       <c r="BP17" s="15" t="n">
         <v>2571.45</v>
+      </c>
+      <c r="BQ17" s="15" t="n">
+        <v>2594.35</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -3815,6 +3861,7 @@
       <c r="BN18" s="15" t="n"/>
       <c r="BO18" s="15" t="n"/>
       <c r="BP18" s="15" t="n"/>
+      <c r="BQ18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -4020,6 +4067,9 @@
       </c>
       <c r="BP19" s="15" t="n">
         <v>79.98</v>
+      </c>
+      <c r="BQ19" s="15" t="n">
+        <v>80.69</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -4178,6 +4228,9 @@
       </c>
       <c r="BP20" s="15" t="n">
         <v>7666.6</v>
+      </c>
+      <c r="BQ20" s="15" t="n">
+        <v>7718.6</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -4297,6 +4350,7 @@
       <c r="BN21" s="15" t="n"/>
       <c r="BO21" s="15" t="n"/>
       <c r="BP21" s="15" t="n"/>
+      <c r="BQ21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -4499,6 +4553,9 @@
         <v>36.34</v>
       </c>
       <c r="BP22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BQ22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -4658,6 +4715,9 @@
       </c>
       <c r="BP23" s="15" t="n">
         <v>76593.75</v>
+      </c>
+      <c r="BQ23" s="15" t="n">
+        <v>76060.39999999999</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -4777,6 +4837,7 @@
       <c r="BN24" s="15" t="n"/>
       <c r="BO24" s="15" t="n"/>
       <c r="BP24" s="15" t="n"/>
+      <c r="BQ24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -4981,6 +5042,9 @@
         <v>49.88</v>
       </c>
       <c r="BP25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BQ25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -5126,6 +5190,9 @@
       </c>
       <c r="BP26" s="15" t="n">
         <v>25847.99</v>
+      </c>
+      <c r="BQ26" s="15" t="n">
+        <v>25996.7</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -5245,6 +5312,7 @@
       <c r="BN27" s="15" t="n"/>
       <c r="BO27" s="15" t="n"/>
       <c r="BP27" s="15" t="n"/>
+      <c r="BQ27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -5449,6 +5517,9 @@
         <v>92.09</v>
       </c>
       <c r="BP28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BQ28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -5608,6 +5679,9 @@
       </c>
       <c r="BP29" s="15" t="n">
         <v>64214.48</v>
+      </c>
+      <c r="BQ29" s="15" t="n">
+        <v>66399.84</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -5727,6 +5801,7 @@
       <c r="BN30" s="15" t="n"/>
       <c r="BO30" s="15" t="n"/>
       <c r="BP30" s="15" t="n"/>
+      <c r="BQ30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -5931,6 +6006,9 @@
         <v>97.44</v>
       </c>
       <c r="BP31" s="15" t="n">
+        <v>97.44</v>
+      </c>
+      <c r="BQ31" s="15" t="n">
         <v>97.44</v>
       </c>
     </row>
@@ -6090,6 +6168,9 @@
       </c>
       <c r="BP32" s="15" t="n">
         <v>6579.48</v>
+      </c>
+      <c r="BQ32" s="15" t="n">
+        <v>6995.39</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -6209,6 +6290,7 @@
       <c r="BN33" s="15" t="n"/>
       <c r="BO33" s="15" t="n"/>
       <c r="BP33" s="15" t="n"/>
+      <c r="BQ33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -6414,6 +6496,9 @@
       </c>
       <c r="BP34" s="15" t="n">
         <v>45.86</v>
+      </c>
+      <c r="BQ34" s="15" t="n">
+        <v>45.19</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -6572,6 +6657,9 @@
       </c>
       <c r="BP35" s="15" t="n">
         <v>5635.06</v>
+      </c>
+      <c r="BQ35" s="15" t="n">
+        <v>5580.21</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -6691,6 +6779,7 @@
       <c r="BN36" s="15" t="n"/>
       <c r="BO36" s="15" t="n"/>
       <c r="BP36" s="15" t="n"/>
+      <c r="BQ36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -6896,6 +6985,9 @@
       </c>
       <c r="BP37" s="15" t="n">
         <v>52.57</v>
+      </c>
+      <c r="BQ37" s="15" t="n">
+        <v>52.63</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -7053,6 +7145,9 @@
         <v>11317.65</v>
       </c>
       <c r="BP38" s="15" t="n">
+        <v>11353.77</v>
+      </c>
+      <c r="BQ38" s="15" t="n">
         <v>11353.77</v>
       </c>
     </row>
@@ -7173,6 +7268,7 @@
       <c r="BN39" s="15" t="n"/>
       <c r="BO39" s="15" t="n"/>
       <c r="BP39" s="15" t="n"/>
+      <c r="BQ39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -7378,6 +7474,9 @@
       </c>
       <c r="BP40" s="15" t="n">
         <v>47.49</v>
+      </c>
+      <c r="BQ40" s="15" t="n">
+        <v>47.57</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -7536,6 +7635,9 @@
       </c>
       <c r="BP41" s="15" t="n">
         <v>11083.48</v>
+      </c>
+      <c r="BQ41" s="15" t="n">
+        <v>11122.86</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -7655,6 +7757,7 @@
       <c r="BN42" s="15" t="n"/>
       <c r="BO42" s="15" t="n"/>
       <c r="BP42" s="15" t="n"/>
+      <c r="BQ42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -7860,6 +7963,9 @@
       </c>
       <c r="BP43" s="15" t="n">
         <v>48.81</v>
+      </c>
+      <c r="BQ43" s="15" t="n">
+        <v>48.67</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -8018,6 +8124,9 @@
       </c>
       <c r="BP44" s="15" t="n">
         <v>3345.83</v>
+      </c>
+      <c r="BQ44" s="15" t="n">
+        <v>3351.34</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -8137,6 +8246,7 @@
       <c r="BN45" s="15" t="n"/>
       <c r="BO45" s="15" t="n"/>
       <c r="BP45" s="15" t="n"/>
+      <c r="BQ45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -8342,6 +8452,9 @@
       </c>
       <c r="BP46" s="15" t="n">
         <v>52.5</v>
+      </c>
+      <c r="BQ46" s="15" t="n">
+        <v>52.53</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -8500,6 +8613,9 @@
       </c>
       <c r="BP47" s="15" t="n">
         <v>7050.7</v>
+      </c>
+      <c r="BQ47" s="15" t="n">
+        <v>7083.61</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -8619,6 +8735,7 @@
       <c r="BN48" s="15" t="n"/>
       <c r="BO48" s="15" t="n"/>
       <c r="BP48" s="15" t="n"/>
+      <c r="BQ48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -8824,6 +8941,9 @@
       </c>
       <c r="BP49" s="15" t="n">
         <v>21.94</v>
+      </c>
+      <c r="BQ49" s="15" t="n">
+        <v>21.06</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -8982,6 +9102,9 @@
       </c>
       <c r="BP50" s="15" t="n">
         <v>33673.16</v>
+      </c>
+      <c r="BQ50" s="15" t="n">
+        <v>33528.53</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -9101,6 +9224,7 @@
       <c r="BN51" s="15" t="n"/>
       <c r="BO51" s="15" t="n"/>
       <c r="BP51" s="15" t="n"/>
+      <c r="BQ51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -9306,6 +9430,9 @@
       </c>
       <c r="BP52" s="15" t="n">
         <v>36.89</v>
+      </c>
+      <c r="BQ52" s="15" t="n">
+        <v>36.3</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -9464,6 +9591,9 @@
       </c>
       <c r="BP53" s="15" t="n">
         <v>3449.92</v>
+      </c>
+      <c r="BQ53" s="15" t="n">
+        <v>3559.19</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -9583,6 +9713,7 @@
       <c r="BN54" s="15" t="n"/>
       <c r="BO54" s="15" t="n"/>
       <c r="BP54" s="15" t="n"/>
+      <c r="BQ54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -9788,6 +9919,9 @@
       </c>
       <c r="BP55" s="15" t="n">
         <v>44.16</v>
+      </c>
+      <c r="BQ55" s="15" t="n">
+        <v>43.02</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -9946,6 +10080,9 @@
       </c>
       <c r="BP56" s="15" t="n">
         <v>3312.54</v>
+      </c>
+      <c r="BQ56" s="15" t="n">
+        <v>3398.68</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -10065,6 +10202,7 @@
       <c r="BN57" s="15" t="n"/>
       <c r="BO57" s="15" t="n"/>
       <c r="BP57" s="15" t="n"/>
+      <c r="BQ57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -10270,6 +10408,9 @@
       </c>
       <c r="BP58" s="15" t="n">
         <v>13.94</v>
+      </c>
+      <c r="BQ58" s="15" t="n">
+        <v>14.05</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -10428,6 +10569,9 @@
       </c>
       <c r="BP59" s="15" t="n">
         <v>6690.39</v>
+      </c>
+      <c r="BQ59" s="15" t="n">
+        <v>6648.2</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -10547,6 +10691,7 @@
       <c r="BN60" s="15" t="n"/>
       <c r="BO60" s="15" t="n"/>
       <c r="BP60" s="15" t="n"/>
+      <c r="BQ60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -10752,6 +10897,9 @@
       </c>
       <c r="BP61" s="15" t="n">
         <v>32.61</v>
+      </c>
+      <c r="BQ61" s="15" t="n">
+        <v>34.34</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -10910,6 +11058,9 @@
       </c>
       <c r="BP62" s="15" t="n">
         <v>8149.53</v>
+      </c>
+      <c r="BQ62" s="15" t="n">
+        <v>8102.26</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -11029,6 +11180,7 @@
       <c r="BN63" s="15" t="n"/>
       <c r="BO63" s="15" t="n"/>
       <c r="BP63" s="15" t="n"/>
+      <c r="BQ63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -11234,6 +11386,9 @@
       </c>
       <c r="BP64" s="15" t="n">
         <v>9.82</v>
+      </c>
+      <c r="BQ64" s="15" t="n">
+        <v>11.77</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -11392,6 +11547,9 @@
       </c>
       <c r="BP65" s="15" t="n">
         <v>10831.21</v>
+      </c>
+      <c r="BQ65" s="15" t="n">
+        <v>10949.77</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -11511,6 +11669,7 @@
       <c r="BN66" s="15" t="n"/>
       <c r="BO66" s="15" t="n"/>
       <c r="BP66" s="15" t="n"/>
+      <c r="BQ66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -11716,6 +11875,9 @@
       </c>
       <c r="BP67" s="15" t="n">
         <v>24.09</v>
+      </c>
+      <c r="BQ67" s="15" t="n">
+        <v>26.04</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -11874,6 +12036,9 @@
       </c>
       <c r="BP68" s="15" t="n">
         <v>11352.7</v>
+      </c>
+      <c r="BQ68" s="15" t="n">
+        <v>11489.08</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -11993,6 +12158,7 @@
       <c r="BN69" s="15" t="n"/>
       <c r="BO69" s="15" t="n"/>
       <c r="BP69" s="15" t="n"/>
+      <c r="BQ69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -12198,6 +12364,9 @@
       </c>
       <c r="BP70" s="15" t="n">
         <v>18.81</v>
+      </c>
+      <c r="BQ70" s="15" t="n">
+        <v>21.46</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -12356,6 +12525,9 @@
       </c>
       <c r="BP71" s="15" t="n">
         <v>6436.71</v>
+      </c>
+      <c r="BQ71" s="15" t="n">
+        <v>6624.29</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -12475,6 +12647,7 @@
       <c r="BN72" s="15" t="n"/>
       <c r="BO72" s="15" t="n"/>
       <c r="BP72" s="15" t="n"/>
+      <c r="BQ72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -12680,6 +12853,9 @@
       </c>
       <c r="BP73" s="15" t="n">
         <v>19.37</v>
+      </c>
+      <c r="BQ73" s="15" t="n">
+        <v>21.75</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -12838,6 +13014,9 @@
       </c>
       <c r="BP74" s="15" t="n">
         <v>12478.59</v>
+      </c>
+      <c r="BQ74" s="15" t="n">
+        <v>12775.54</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -12957,6 +13136,7 @@
       <c r="BN75" s="15" t="n"/>
       <c r="BO75" s="15" t="n"/>
       <c r="BP75" s="15" t="n"/>
+      <c r="BQ75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -13162,6 +13342,9 @@
       </c>
       <c r="BP76" s="15" t="n">
         <v>50.91</v>
+      </c>
+      <c r="BQ76" s="15" t="n">
+        <v>51.21</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -13319,6 +13502,9 @@
         <v>15569.82</v>
       </c>
       <c r="BP77" s="15" t="n">
+        <v>15569.82</v>
+      </c>
+      <c r="BQ77" s="15" t="n">
         <v>15569.82</v>
       </c>
     </row>
@@ -13439,6 +13625,7 @@
       <c r="BN78" s="15" t="n"/>
       <c r="BO78" s="15" t="n"/>
       <c r="BP78" s="15" t="n"/>
+      <c r="BQ78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -13644,6 +13831,9 @@
       </c>
       <c r="BP79" s="15" t="n">
         <v>3.56</v>
+      </c>
+      <c r="BQ79" s="15" t="n">
+        <v>4.36</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -13802,6 +13992,9 @@
       </c>
       <c r="BP80" s="15" t="n">
         <v>6753.16</v>
+      </c>
+      <c r="BQ80" s="15" t="n">
+        <v>6783.29</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -13921,6 +14114,7 @@
       <c r="BN81" s="15" t="n"/>
       <c r="BO81" s="15" t="n"/>
       <c r="BP81" s="15" t="n"/>
+      <c r="BQ81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -14126,6 +14320,9 @@
       </c>
       <c r="BP82" s="15" t="n">
         <v>4.21</v>
+      </c>
+      <c r="BQ82" s="15" t="n">
+        <v>4.51</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -14284,6 +14481,9 @@
       </c>
       <c r="BP83" s="15" t="n">
         <v>8473</v>
+      </c>
+      <c r="BQ83" s="15" t="n">
+        <v>8501.110000000001</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -14403,6 +14603,7 @@
       <c r="BN84" s="15" t="n"/>
       <c r="BO84" s="15" t="n"/>
       <c r="BP84" s="15" t="n"/>
+      <c r="BQ84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -14608,6 +14809,9 @@
       </c>
       <c r="BP85" s="15" t="n">
         <v>14.53</v>
+      </c>
+      <c r="BQ85" s="15" t="n">
+        <v>15.22</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -14766,6 +14970,9 @@
       </c>
       <c r="BP86" s="15" t="n">
         <v>2126.97</v>
+      </c>
+      <c r="BQ86" s="15" t="n">
+        <v>2171.98</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -14885,6 +15092,7 @@
       <c r="BN87" s="15" t="n"/>
       <c r="BO87" s="15" t="n"/>
       <c r="BP87" s="15" t="n"/>
+      <c r="BQ87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -15090,6 +15298,9 @@
       </c>
       <c r="BP88" s="15" t="n">
         <v>30.27</v>
+      </c>
+      <c r="BQ88" s="15" t="n">
+        <v>30.02</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -15248,6 +15459,9 @@
       </c>
       <c r="BP89" s="15" t="n">
         <v>4459.72</v>
+      </c>
+      <c r="BQ89" s="15" t="n">
+        <v>4527.71</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -15367,6 +15581,7 @@
       <c r="BN90" s="15" t="n"/>
       <c r="BO90" s="15" t="n"/>
       <c r="BP90" s="15" t="n"/>
+      <c r="BQ90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -15572,6 +15787,9 @@
       </c>
       <c r="BP91" s="15" t="n">
         <v>16.21</v>
+      </c>
+      <c r="BQ91" s="15" t="n">
+        <v>17.09</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -15730,6 +15948,9 @@
       </c>
       <c r="BP92" s="15" t="n">
         <v>8528.389999999999</v>
+      </c>
+      <c r="BQ92" s="15" t="n">
+        <v>8469.49</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -15849,6 +16070,7 @@
       <c r="BN93" s="15" t="n"/>
       <c r="BO93" s="15" t="n"/>
       <c r="BP93" s="15" t="n"/>
+      <c r="BQ93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -16054,6 +16276,9 @@
       </c>
       <c r="BP94" s="15" t="n">
         <v>6.59</v>
+      </c>
+      <c r="BQ94" s="15" t="n">
+        <v>7.26</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -16212,6 +16437,9 @@
       </c>
       <c r="BP95" s="15" t="n">
         <v>1243.68</v>
+      </c>
+      <c r="BQ95" s="15" t="n">
+        <v>1280.28</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -16331,6 +16559,7 @@
       <c r="BN96" s="15" t="n"/>
       <c r="BO96" s="15" t="n"/>
       <c r="BP96" s="15" t="n"/>
+      <c r="BQ96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -16536,6 +16765,9 @@
       </c>
       <c r="BP97" s="15" t="n">
         <v>10.13</v>
+      </c>
+      <c r="BQ97" s="15" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -16694,6 +16926,9 @@
       </c>
       <c r="BP98" s="15" t="n">
         <v>13880.34</v>
+      </c>
+      <c r="BQ98" s="15" t="n">
+        <v>14151.03</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -16813,6 +17048,7 @@
       <c r="BN99" s="15" t="n"/>
       <c r="BO99" s="15" t="n"/>
       <c r="BP99" s="15" t="n"/>
+      <c r="BQ99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -17018,6 +17254,9 @@
       </c>
       <c r="BP100" s="15" t="n">
         <v>33.41</v>
+      </c>
+      <c r="BQ100" s="15" t="n">
+        <v>34.12</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -17176,6 +17415,9 @@
       </c>
       <c r="BP101" s="15" t="n">
         <v>3215.2</v>
+      </c>
+      <c r="BQ101" s="15" t="n">
+        <v>3215.13</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -17295,6 +17537,7 @@
       <c r="BN102" s="15" t="n"/>
       <c r="BO102" s="15" t="n"/>
       <c r="BP102" s="15" t="n"/>
+      <c r="BQ102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -17500,6 +17743,9 @@
       </c>
       <c r="BP103" s="15" t="n">
         <v>30.48</v>
+      </c>
+      <c r="BQ103" s="15" t="n">
+        <v>30.23</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -17658,6 +17904,9 @@
       </c>
       <c r="BP104" s="15" t="n">
         <v>2305.71</v>
+      </c>
+      <c r="BQ104" s="15" t="n">
+        <v>2305.86</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -17777,6 +18026,7 @@
       <c r="BN105" s="15" t="n"/>
       <c r="BO105" s="15" t="n"/>
       <c r="BP105" s="15" t="n"/>
+      <c r="BQ105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -17982,6 +18232,9 @@
       </c>
       <c r="BP106" s="15" t="n">
         <v>13.55</v>
+      </c>
+      <c r="BQ106" s="15" t="n">
+        <v>13.1</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -18140,6 +18393,9 @@
       </c>
       <c r="BP107" s="15" t="n">
         <v>2491.47</v>
+      </c>
+      <c r="BQ107" s="15" t="n">
+        <v>2412.23</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -18259,6 +18515,7 @@
       <c r="BN108" s="15" t="n"/>
       <c r="BO108" s="15" t="n"/>
       <c r="BP108" s="15" t="n"/>
+      <c r="BQ108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -18464,6 +18721,9 @@
       </c>
       <c r="BP109" s="15" t="n">
         <v>30.62</v>
+      </c>
+      <c r="BQ109" s="15" t="n">
+        <v>30.64</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -18622,6 +18882,9 @@
       </c>
       <c r="BP110" s="15" t="n">
         <v>2499.93</v>
+      </c>
+      <c r="BQ110" s="15" t="n">
+        <v>2502.43</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -18741,6 +19004,7 @@
       <c r="BN111" s="15" t="n"/>
       <c r="BO111" s="15" t="n"/>
       <c r="BP111" s="15" t="n"/>
+      <c r="BQ111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -18946,6 +19210,9 @@
       </c>
       <c r="BP112" s="15" t="n">
         <v>48.1</v>
+      </c>
+      <c r="BQ112" s="15" t="n">
+        <v>48.77</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -19102,6 +19369,9 @@
       </c>
       <c r="BP113" s="15" t="n">
         <v>1898.76</v>
+      </c>
+      <c r="BQ113" s="15" t="n">
+        <v>1898.47</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -19221,6 +19491,7 @@
       <c r="BN114" s="15" t="n"/>
       <c r="BO114" s="15" t="n"/>
       <c r="BP114" s="15" t="n"/>
+      <c r="BQ114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -19426,6 +19697,9 @@
       </c>
       <c r="BP115" s="15" t="n">
         <v>17.14</v>
+      </c>
+      <c r="BQ115" s="15" t="n">
+        <v>17.34</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -19569,6 +19843,9 @@
       </c>
       <c r="BP116" s="15" t="n">
         <v>8769.57</v>
+      </c>
+      <c r="BQ116" s="15" t="n">
+        <v>8794.76</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -19643,6 +19920,7 @@
       <c r="BN117" s="15" t="n"/>
       <c r="BO117" s="15" t="n"/>
       <c r="BP117" s="15" t="n"/>
+      <c r="BQ117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -19804,6 +20082,9 @@
       <c r="BP118" s="15" t="n">
         <v>74.13</v>
       </c>
+      <c r="BQ118" s="15" t="n">
+        <v>71.87</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -19937,6 +20218,9 @@
       </c>
       <c r="BP119" s="15" t="n">
         <v>12659.95</v>
+      </c>
+      <c r="BQ119" s="15" t="n">
+        <v>12639.56</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -19960,6 +20244,7 @@
       <c r="BN120" s="15" t="n"/>
       <c r="BO120" s="15" t="n"/>
       <c r="BP120" s="15" t="n"/>
+      <c r="BQ120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -20022,6 +20307,9 @@
       <c r="BP121" s="15" t="n">
         <v>25.34</v>
       </c>
+      <c r="BQ121" s="15" t="n">
+        <v>28.69</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -20083,6 +20371,9 @@
       </c>
       <c r="BP122" s="15" t="n">
         <v>1221.87</v>
+      </c>
+      <c r="BQ122" s="15" t="n">
+        <v>1258.61</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -20106,6 +20397,7 @@
       <c r="BN123" s="15" t="n"/>
       <c r="BO123" s="15" t="n"/>
       <c r="BP123" s="15" t="n"/>
+      <c r="BQ123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -20168,6 +20460,9 @@
       <c r="BP124" s="15" t="n">
         <v>46.52</v>
       </c>
+      <c r="BQ124" s="15" t="n">
+        <v>48.08</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -20229,6 +20524,9 @@
       </c>
       <c r="BP125" s="15" t="n">
         <v>11534.72</v>
+      </c>
+      <c r="BQ125" s="15" t="n">
+        <v>11645.88</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -20252,6 +20550,7 @@
       <c r="BN126" s="15" t="n"/>
       <c r="BO126" s="15" t="n"/>
       <c r="BP126" s="15" t="n"/>
+      <c r="BQ126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -20314,6 +20613,9 @@
       <c r="BP127" s="15" t="n">
         <v>5.42</v>
       </c>
+      <c r="BQ127" s="15" t="n">
+        <v>8.470000000000001</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -20375,6 +20677,9 @@
       </c>
       <c r="BP128" s="15" t="n">
         <v>1882.19</v>
+      </c>
+      <c r="BQ128" s="15" t="n">
+        <v>1984.08</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -20398,6 +20703,7 @@
       <c r="BN129" s="15" t="n"/>
       <c r="BO129" s="15" t="n"/>
       <c r="BP129" s="15" t="n"/>
+      <c r="BQ129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -20460,6 +20766,9 @@
       <c r="BP130" s="15" t="n">
         <v>10.98</v>
       </c>
+      <c r="BQ130" s="15" t="n">
+        <v>12.73</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -20521,6 +20830,9 @@
       </c>
       <c r="BP131" s="15" t="n">
         <v>764.0700000000001</v>
+      </c>
+      <c r="BQ131" s="15" t="n">
+        <v>758.4</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -20544,6 +20856,7 @@
       <c r="BN132" s="15" t="n"/>
       <c r="BO132" s="15" t="n"/>
       <c r="BP132" s="15" t="n"/>
+      <c r="BQ132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -20606,6 +20919,9 @@
       <c r="BP133" s="15" t="n">
         <v>63.29</v>
       </c>
+      <c r="BQ133" s="15" t="n">
+        <v>62.87</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -20667,6 +20983,9 @@
       </c>
       <c r="BP134" s="15" t="n">
         <v>3094.52</v>
+      </c>
+      <c r="BQ134" s="15" t="n">
+        <v>2960.13</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -20690,6 +21009,7 @@
       <c r="BN135" s="15" t="n"/>
       <c r="BO135" s="15" t="n"/>
       <c r="BP135" s="15" t="n"/>
+      <c r="BQ135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -20752,6 +21072,9 @@
       <c r="BP136" s="15" t="n">
         <v>21.88</v>
       </c>
+      <c r="BQ136" s="15" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -20813,6 +21136,9 @@
       </c>
       <c r="BP137" s="15" t="n">
         <v>3565.52</v>
+      </c>
+      <c r="BQ137" s="15" t="n">
+        <v>3573.26</v>
       </c>
     </row>
     <row r="138">
@@ -20828,6 +21154,7 @@
       <c r="BN138" s="15" t="n"/>
       <c r="BO138" s="15" t="n"/>
       <c r="BP138" s="15" t="n"/>
+      <c r="BQ138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -20866,6 +21193,9 @@
       <c r="BP139" s="15" t="n">
         <v>4.04</v>
       </c>
+      <c r="BQ139" s="15" t="n">
+        <v>4.25</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -20902,6 +21232,9 @@
         <v>2430.11</v>
       </c>
       <c r="BP140" s="15" t="n">
+        <v>2412.96</v>
+      </c>
+      <c r="BQ140" s="15" t="n">
         <v>2412.96</v>
       </c>
     </row>
@@ -20918,6 +21251,7 @@
       <c r="BN141" s="15" t="n"/>
       <c r="BO141" s="15" t="n"/>
       <c r="BP141" s="15" t="n"/>
+      <c r="BQ141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -20956,6 +21290,9 @@
       <c r="BP142" s="15" t="n">
         <v>19.78</v>
       </c>
+      <c r="BQ142" s="15" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -20993,6 +21330,9 @@
       </c>
       <c r="BP143" s="15" t="n">
         <v>5665.88</v>
+      </c>
+      <c r="BQ143" s="15" t="n">
+        <v>5754.63</v>
       </c>
     </row>
     <row r="144">
@@ -21003,6 +21343,7 @@
       <c r="BN144" s="15" t="n"/>
       <c r="BO144" s="15" t="n"/>
       <c r="BP144" s="15" t="n"/>
+      <c r="BQ144" s="15" t="n"/>
     </row>
     <row r="145">
       <c r="BJ145" s="15" t="n">
@@ -21026,6 +21367,9 @@
       <c r="BP145" s="15" t="n">
         <v>2.34</v>
       </c>
+      <c r="BQ145" s="15" t="n">
+        <v>2.79</v>
+      </c>
     </row>
     <row r="146">
       <c r="BJ146" s="15" t="n">
@@ -21048,6 +21392,9 @@
       </c>
       <c r="BP146" s="15" t="n">
         <v>2309.6</v>
+      </c>
+      <c r="BQ146" s="15" t="n">
+        <v>2338.32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update stocks_data.xlsx [2026-09-10 08:26:18]
</commit_message>
<xml_diff>
--- a/stocks_data.xlsx
+++ b/stocks_data.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BQ146"/>
+  <dimension ref="A1:BR146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="51"/>
@@ -603,6 +603,7 @@
     <col width="15" customWidth="1" min="67" max="67"/>
     <col width="15" customWidth="1" min="68" max="68"/>
     <col width="15" customWidth="1" min="69" max="69"/>
+    <col width="15" customWidth="1" min="70" max="70"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -951,6 +952,11 @@
           <t>2026/09/07</t>
         </is>
       </c>
+      <c r="BR1" s="15" t="inlineStr">
+        <is>
+          <t>2026/09/10</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1298,6 +1304,11 @@
           <t>上证</t>
         </is>
       </c>
+      <c r="BR2" s="16" t="inlineStr">
+        <is>
+          <t>上证</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1507,6 +1518,9 @@
       <c r="BQ3" s="15" t="n">
         <v>59.89</v>
       </c>
+      <c r="BR3" s="15" t="n">
+        <v>60.57</v>
+      </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -1715,6 +1729,9 @@
       </c>
       <c r="BQ4" s="15" t="n">
         <v>3932.7</v>
+      </c>
+      <c r="BR4" s="15" t="n">
+        <v>3934.4</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -1787,6 +1804,7 @@
       <c r="BO5" s="15" t="n"/>
       <c r="BP5" s="15" t="n"/>
       <c r="BQ5" s="15" t="n"/>
+      <c r="BR5" s="15" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1906,6 +1924,7 @@
       <c r="BO6" s="15" t="n"/>
       <c r="BP6" s="15" t="n"/>
       <c r="BQ6" s="15" t="n"/>
+      <c r="BR6" s="15" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -2114,6 +2133,9 @@
       </c>
       <c r="BQ7" s="15" t="n">
         <v>54.47</v>
+      </c>
+      <c r="BR7" s="15" t="n">
+        <v>54.29</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
@@ -2275,6 +2297,9 @@
       </c>
       <c r="BQ8" s="15" t="n">
         <v>5644.97</v>
+      </c>
+      <c r="BR8" s="15" t="n">
+        <v>5606.98</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
@@ -2395,6 +2420,7 @@
       <c r="BO9" s="15" t="n"/>
       <c r="BP9" s="15" t="n"/>
       <c r="BQ9" s="15" t="n"/>
+      <c r="BR9" s="15" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -2603,6 +2629,9 @@
       </c>
       <c r="BQ10" s="15" t="n">
         <v>50.57</v>
+      </c>
+      <c r="BR10" s="15" t="n">
+        <v>49.39</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
@@ -2764,6 +2793,9 @@
       </c>
       <c r="BQ11" s="15" t="n">
         <v>4575.02</v>
+      </c>
+      <c r="BR11" s="15" t="n">
+        <v>4548.39</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
@@ -2884,6 +2916,7 @@
       <c r="BO12" s="15" t="n"/>
       <c r="BP12" s="15" t="n"/>
       <c r="BQ12" s="15" t="n"/>
+      <c r="BR12" s="15" t="n"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -3092,6 +3125,9 @@
       </c>
       <c r="BQ13" s="15" t="n">
         <v>58.69</v>
+      </c>
+      <c r="BR13" s="15" t="n">
+        <v>60.09</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
@@ -3253,6 +3289,9 @@
       </c>
       <c r="BQ14" s="15" t="n">
         <v>7759.37</v>
+      </c>
+      <c r="BR14" s="15" t="n">
+        <v>7717.8</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -3373,6 +3412,7 @@
       <c r="BO15" s="15" t="n"/>
       <c r="BP15" s="15" t="n"/>
       <c r="BQ15" s="15" t="n"/>
+      <c r="BR15" s="15" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -3581,6 +3621,9 @@
       </c>
       <c r="BQ16" s="15" t="n">
         <v>30.79</v>
+      </c>
+      <c r="BR16" s="15" t="n">
+        <v>30.5</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -3742,6 +3785,9 @@
       </c>
       <c r="BQ17" s="15" t="n">
         <v>2594.35</v>
+      </c>
+      <c r="BR17" s="15" t="n">
+        <v>2538.76</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -3862,6 +3908,7 @@
       <c r="BO18" s="15" t="n"/>
       <c r="BP18" s="15" t="n"/>
       <c r="BQ18" s="15" t="n"/>
+      <c r="BR18" s="15" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -4070,6 +4117,9 @@
       </c>
       <c r="BQ19" s="15" t="n">
         <v>80.69</v>
+      </c>
+      <c r="BR19" s="15" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -4231,6 +4281,9 @@
       </c>
       <c r="BQ20" s="15" t="n">
         <v>7718.6</v>
+      </c>
+      <c r="BR20" s="15" t="n">
+        <v>7636.36</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
@@ -4351,6 +4404,7 @@
       <c r="BO21" s="15" t="n"/>
       <c r="BP21" s="15" t="n"/>
       <c r="BQ21" s="15" t="n"/>
+      <c r="BR21" s="15" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -4556,6 +4610,9 @@
         <v>36.34</v>
       </c>
       <c r="BQ22" s="15" t="n">
+        <v>36.34</v>
+      </c>
+      <c r="BR22" s="15" t="n">
         <v>36.34</v>
       </c>
     </row>
@@ -4718,6 +4775,9 @@
       </c>
       <c r="BQ23" s="15" t="n">
         <v>76060.39999999999</v>
+      </c>
+      <c r="BR23" s="15" t="n">
+        <v>74764.7</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -4838,6 +4898,7 @@
       <c r="BO24" s="15" t="n"/>
       <c r="BP24" s="15" t="n"/>
       <c r="BQ24" s="15" t="n"/>
+      <c r="BR24" s="15" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -5045,6 +5106,9 @@
         <v>49.88</v>
       </c>
       <c r="BQ25" s="15" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="BR25" s="15" t="n">
         <v>49.88</v>
       </c>
     </row>
@@ -5193,6 +5257,9 @@
       </c>
       <c r="BQ26" s="15" t="n">
         <v>25996.7</v>
+      </c>
+      <c r="BR26" s="15" t="n">
+        <v>25550.9</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -5313,6 +5380,7 @@
       <c r="BO27" s="15" t="n"/>
       <c r="BP27" s="15" t="n"/>
       <c r="BQ27" s="15" t="n"/>
+      <c r="BR27" s="15" t="n"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -5520,6 +5588,9 @@
         <v>92.09</v>
       </c>
       <c r="BQ28" s="15" t="n">
+        <v>92.09</v>
+      </c>
+      <c r="BR28" s="15" t="n">
         <v>92.09</v>
       </c>
     </row>
@@ -5682,6 +5753,9 @@
       </c>
       <c r="BQ29" s="15" t="n">
         <v>66399.84</v>
+      </c>
+      <c r="BR29" s="15" t="n">
+        <v>65270.95</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
@@ -5802,6 +5876,7 @@
       <c r="BO30" s="15" t="n"/>
       <c r="BP30" s="15" t="n"/>
       <c r="BQ30" s="15" t="n"/>
+      <c r="BR30" s="15" t="n"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -6009,6 +6084,9 @@
         <v>97.44</v>
       </c>
       <c r="BQ31" s="15" t="n">
+        <v>97.44</v>
+      </c>
+      <c r="BR31" s="15" t="n">
         <v>97.44</v>
       </c>
     </row>
@@ -6171,6 +6249,9 @@
       </c>
       <c r="BQ32" s="15" t="n">
         <v>6995.39</v>
+      </c>
+      <c r="BR32" s="15" t="n">
+        <v>7033.92</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1">
@@ -6291,6 +6372,7 @@
       <c r="BO33" s="15" t="n"/>
       <c r="BP33" s="15" t="n"/>
       <c r="BQ33" s="15" t="n"/>
+      <c r="BR33" s="15" t="n"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -6499,6 +6581,9 @@
       </c>
       <c r="BQ34" s="15" t="n">
         <v>45.19</v>
+      </c>
+      <c r="BR34" s="15" t="n">
+        <v>45.3</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
@@ -6660,6 +6745,9 @@
       </c>
       <c r="BQ35" s="15" t="n">
         <v>5580.21</v>
+      </c>
+      <c r="BR35" s="15" t="n">
+        <v>5677.09</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
@@ -6780,6 +6868,7 @@
       <c r="BO36" s="15" t="n"/>
       <c r="BP36" s="15" t="n"/>
       <c r="BQ36" s="15" t="n"/>
+      <c r="BR36" s="15" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -6988,6 +7077,9 @@
       </c>
       <c r="BQ37" s="15" t="n">
         <v>52.63</v>
+      </c>
+      <c r="BR37" s="15" t="n">
+        <v>51.76</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
@@ -7149,6 +7241,9 @@
       </c>
       <c r="BQ38" s="15" t="n">
         <v>11353.77</v>
+      </c>
+      <c r="BR38" s="15" t="n">
+        <v>11346.49</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
@@ -7269,6 +7364,7 @@
       <c r="BO39" s="15" t="n"/>
       <c r="BP39" s="15" t="n"/>
       <c r="BQ39" s="15" t="n"/>
+      <c r="BR39" s="15" t="n"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -7477,6 +7573,9 @@
       </c>
       <c r="BQ40" s="15" t="n">
         <v>47.57</v>
+      </c>
+      <c r="BR40" s="15" t="n">
+        <v>47.31</v>
       </c>
     </row>
     <row r="41" ht="14.25" customHeight="1">
@@ -7638,6 +7737,9 @@
       </c>
       <c r="BQ41" s="15" t="n">
         <v>11122.86</v>
+      </c>
+      <c r="BR41" s="15" t="n">
+        <v>11161.29</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
@@ -7758,6 +7860,7 @@
       <c r="BO42" s="15" t="n"/>
       <c r="BP42" s="15" t="n"/>
       <c r="BQ42" s="15" t="n"/>
+      <c r="BR42" s="15" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="3" t="n">
@@ -7966,6 +8069,9 @@
       </c>
       <c r="BQ43" s="15" t="n">
         <v>48.67</v>
+      </c>
+      <c r="BR43" s="15" t="n">
+        <v>48.92</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1">
@@ -8127,6 +8233,9 @@
       </c>
       <c r="BQ44" s="15" t="n">
         <v>3351.34</v>
+      </c>
+      <c r="BR44" s="15" t="n">
+        <v>3407.41</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1">
@@ -8247,6 +8356,7 @@
       <c r="BO45" s="15" t="n"/>
       <c r="BP45" s="15" t="n"/>
       <c r="BQ45" s="15" t="n"/>
+      <c r="BR45" s="15" t="n"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -8455,6 +8565,9 @@
       </c>
       <c r="BQ46" s="15" t="n">
         <v>52.53</v>
+      </c>
+      <c r="BR46" s="15" t="n">
+        <v>48.28</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1">
@@ -8616,6 +8729,9 @@
       </c>
       <c r="BQ47" s="15" t="n">
         <v>7083.61</v>
+      </c>
+      <c r="BR47" s="15" t="n">
+        <v>7038.44</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1">
@@ -8736,6 +8852,7 @@
       <c r="BO48" s="15" t="n"/>
       <c r="BP48" s="15" t="n"/>
       <c r="BQ48" s="15" t="n"/>
+      <c r="BR48" s="15" t="n"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -8944,6 +9061,9 @@
       </c>
       <c r="BQ49" s="15" t="n">
         <v>21.06</v>
+      </c>
+      <c r="BR49" s="15" t="n">
+        <v>23.4</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1">
@@ -9105,6 +9225,9 @@
       </c>
       <c r="BQ50" s="15" t="n">
         <v>33528.53</v>
+      </c>
+      <c r="BR50" s="15" t="n">
+        <v>33145.69</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
@@ -9225,6 +9348,7 @@
       <c r="BO51" s="15" t="n"/>
       <c r="BP51" s="15" t="n"/>
       <c r="BQ51" s="15" t="n"/>
+      <c r="BR51" s="15" t="n"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -9433,6 +9557,9 @@
       </c>
       <c r="BQ52" s="15" t="n">
         <v>36.3</v>
+      </c>
+      <c r="BR52" s="15" t="n">
+        <v>38.38</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
@@ -9594,6 +9721,9 @@
       </c>
       <c r="BQ53" s="15" t="n">
         <v>3559.19</v>
+      </c>
+      <c r="BR53" s="15" t="n">
+        <v>3495.93</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
@@ -9714,6 +9844,7 @@
       <c r="BO54" s="15" t="n"/>
       <c r="BP54" s="15" t="n"/>
       <c r="BQ54" s="15" t="n"/>
+      <c r="BR54" s="15" t="n"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="3" t="n">
@@ -9922,6 +10053,9 @@
       </c>
       <c r="BQ55" s="15" t="n">
         <v>43.02</v>
+      </c>
+      <c r="BR55" s="15" t="n">
+        <v>45.15</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1">
@@ -10083,6 +10217,9 @@
       </c>
       <c r="BQ56" s="15" t="n">
         <v>3398.68</v>
+      </c>
+      <c r="BR56" s="15" t="n">
+        <v>3338.42</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
@@ -10203,6 +10340,7 @@
       <c r="BO57" s="15" t="n"/>
       <c r="BP57" s="15" t="n"/>
       <c r="BQ57" s="15" t="n"/>
+      <c r="BR57" s="15" t="n"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -10411,6 +10549,9 @@
       </c>
       <c r="BQ58" s="15" t="n">
         <v>14.05</v>
+      </c>
+      <c r="BR58" s="15" t="n">
+        <v>13.95</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
@@ -10572,6 +10713,9 @@
       </c>
       <c r="BQ59" s="15" t="n">
         <v>6648.2</v>
+      </c>
+      <c r="BR59" s="15" t="n">
+        <v>6582.88</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1">
@@ -10692,6 +10836,7 @@
       <c r="BO60" s="15" t="n"/>
       <c r="BP60" s="15" t="n"/>
       <c r="BQ60" s="15" t="n"/>
+      <c r="BR60" s="15" t="n"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -10900,6 +11045,9 @@
       </c>
       <c r="BQ61" s="15" t="n">
         <v>34.34</v>
+      </c>
+      <c r="BR61" s="15" t="n">
+        <v>31.41</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
@@ -11061,6 +11209,9 @@
       </c>
       <c r="BQ62" s="15" t="n">
         <v>8102.26</v>
+      </c>
+      <c r="BR62" s="15" t="n">
+        <v>7931.58</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
@@ -11181,6 +11332,7 @@
       <c r="BO63" s="15" t="n"/>
       <c r="BP63" s="15" t="n"/>
       <c r="BQ63" s="15" t="n"/>
+      <c r="BR63" s="15" t="n"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -11389,6 +11541,9 @@
       </c>
       <c r="BQ64" s="15" t="n">
         <v>11.77</v>
+      </c>
+      <c r="BR64" s="15" t="n">
+        <v>9.74</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
@@ -11550,6 +11705,9 @@
       </c>
       <c r="BQ65" s="15" t="n">
         <v>10949.77</v>
+      </c>
+      <c r="BR65" s="15" t="n">
+        <v>10652.53</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
@@ -11670,6 +11828,7 @@
       <c r="BO66" s="15" t="n"/>
       <c r="BP66" s="15" t="n"/>
       <c r="BQ66" s="15" t="n"/>
+      <c r="BR66" s="15" t="n"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -11878,6 +12037,9 @@
       </c>
       <c r="BQ67" s="15" t="n">
         <v>26.04</v>
+      </c>
+      <c r="BR67" s="15" t="n">
+        <v>24.24</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
@@ -12039,6 +12201,9 @@
       </c>
       <c r="BQ68" s="15" t="n">
         <v>11489.08</v>
+      </c>
+      <c r="BR68" s="15" t="n">
+        <v>11392.59</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
@@ -12159,6 +12324,7 @@
       <c r="BO69" s="15" t="n"/>
       <c r="BP69" s="15" t="n"/>
       <c r="BQ69" s="15" t="n"/>
+      <c r="BR69" s="15" t="n"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -12367,6 +12533,9 @@
       </c>
       <c r="BQ70" s="15" t="n">
         <v>21.46</v>
+      </c>
+      <c r="BR70" s="15" t="n">
+        <v>18.46</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1">
@@ -12528,6 +12697,9 @@
       </c>
       <c r="BQ71" s="15" t="n">
         <v>6624.29</v>
+      </c>
+      <c r="BR71" s="15" t="n">
+        <v>6361.07</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1">
@@ -12648,6 +12820,7 @@
       <c r="BO72" s="15" t="n"/>
       <c r="BP72" s="15" t="n"/>
       <c r="BQ72" s="15" t="n"/>
+      <c r="BR72" s="15" t="n"/>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -12856,6 +13029,9 @@
       </c>
       <c r="BQ73" s="15" t="n">
         <v>21.75</v>
+      </c>
+      <c r="BR73" s="15" t="n">
+        <v>20.41</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
@@ -13017,6 +13193,9 @@
       </c>
       <c r="BQ74" s="15" t="n">
         <v>12775.54</v>
+      </c>
+      <c r="BR74" s="15" t="n">
+        <v>12475.28</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1">
@@ -13137,6 +13316,7 @@
       <c r="BO75" s="15" t="n"/>
       <c r="BP75" s="15" t="n"/>
       <c r="BQ75" s="15" t="n"/>
+      <c r="BR75" s="15" t="n"/>
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -13345,6 +13525,9 @@
       </c>
       <c r="BQ76" s="15" t="n">
         <v>51.21</v>
+      </c>
+      <c r="BR76" s="15" t="n">
+        <v>52.81</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1">
@@ -13506,6 +13689,9 @@
       </c>
       <c r="BQ77" s="15" t="n">
         <v>15569.82</v>
+      </c>
+      <c r="BR77" s="15" t="n">
+        <v>15061.96</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1">
@@ -13626,6 +13812,7 @@
       <c r="BO78" s="15" t="n"/>
       <c r="BP78" s="15" t="n"/>
       <c r="BQ78" s="15" t="n"/>
+      <c r="BR78" s="15" t="n"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -13834,6 +14021,9 @@
       </c>
       <c r="BQ79" s="15" t="n">
         <v>4.36</v>
+      </c>
+      <c r="BR79" s="15" t="n">
+        <v>2.48</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1">
@@ -13995,6 +14185,9 @@
       </c>
       <c r="BQ80" s="15" t="n">
         <v>6783.29</v>
+      </c>
+      <c r="BR80" s="15" t="n">
+        <v>6478.77</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
@@ -14115,6 +14308,7 @@
       <c r="BO81" s="15" t="n"/>
       <c r="BP81" s="15" t="n"/>
       <c r="BQ81" s="15" t="n"/>
+      <c r="BR81" s="15" t="n"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="3" t="n">
@@ -14323,6 +14517,9 @@
       </c>
       <c r="BQ82" s="15" t="n">
         <v>4.51</v>
+      </c>
+      <c r="BR82" s="15" t="n">
+        <v>4.34</v>
       </c>
     </row>
     <row r="83" ht="14.25" customHeight="1">
@@ -14484,6 +14681,9 @@
       </c>
       <c r="BQ83" s="15" t="n">
         <v>8501.110000000001</v>
+      </c>
+      <c r="BR83" s="15" t="n">
+        <v>8473</v>
       </c>
     </row>
     <row r="84" ht="14.25" customHeight="1">
@@ -14604,6 +14804,7 @@
       <c r="BO84" s="15" t="n"/>
       <c r="BP84" s="15" t="n"/>
       <c r="BQ84" s="15" t="n"/>
+      <c r="BR84" s="15" t="n"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -14812,6 +15013,9 @@
       </c>
       <c r="BQ85" s="15" t="n">
         <v>15.22</v>
+      </c>
+      <c r="BR85" s="15" t="n">
+        <v>18.04</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1">
@@ -14973,6 +15177,9 @@
       </c>
       <c r="BQ86" s="15" t="n">
         <v>2171.98</v>
+      </c>
+      <c r="BR86" s="15" t="n">
+        <v>2631.9</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
@@ -15093,6 +15300,7 @@
       <c r="BO87" s="15" t="n"/>
       <c r="BP87" s="15" t="n"/>
       <c r="BQ87" s="15" t="n"/>
+      <c r="BR87" s="15" t="n"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -15301,6 +15509,9 @@
       </c>
       <c r="BQ88" s="15" t="n">
         <v>30.02</v>
+      </c>
+      <c r="BR88" s="15" t="n">
+        <v>27.46</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
@@ -15462,6 +15673,9 @@
       </c>
       <c r="BQ89" s="15" t="n">
         <v>4527.71</v>
+      </c>
+      <c r="BR89" s="15" t="n">
+        <v>4333.4</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1">
@@ -15582,6 +15796,7 @@
       <c r="BO90" s="15" t="n"/>
       <c r="BP90" s="15" t="n"/>
       <c r="BQ90" s="15" t="n"/>
+      <c r="BR90" s="15" t="n"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="n">
@@ -15790,6 +16005,9 @@
       </c>
       <c r="BQ91" s="15" t="n">
         <v>17.09</v>
+      </c>
+      <c r="BR91" s="15" t="n">
+        <v>14.77</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1">
@@ -15951,6 +16169,9 @@
       </c>
       <c r="BQ92" s="15" t="n">
         <v>8469.49</v>
+      </c>
+      <c r="BR92" s="15" t="n">
+        <v>8312.059999999999</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1">
@@ -16071,6 +16292,7 @@
       <c r="BO93" s="15" t="n"/>
       <c r="BP93" s="15" t="n"/>
       <c r="BQ93" s="15" t="n"/>
+      <c r="BR93" s="15" t="n"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -16279,6 +16501,9 @@
       </c>
       <c r="BQ94" s="15" t="n">
         <v>7.26</v>
+      </c>
+      <c r="BR94" s="15" t="n">
+        <v>6.53</v>
       </c>
     </row>
     <row r="95" ht="14.25" customHeight="1">
@@ -16440,6 +16665,9 @@
       </c>
       <c r="BQ95" s="15" t="n">
         <v>1280.28</v>
+      </c>
+      <c r="BR95" s="15" t="n">
+        <v>1239.83</v>
       </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
@@ -16560,6 +16788,7 @@
       <c r="BO96" s="15" t="n"/>
       <c r="BP96" s="15" t="n"/>
       <c r="BQ96" s="15" t="n"/>
+      <c r="BR96" s="15" t="n"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -16768,6 +16997,9 @@
       </c>
       <c r="BQ97" s="15" t="n">
         <v>12</v>
+      </c>
+      <c r="BR97" s="15" t="n">
+        <v>10.36</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1">
@@ -16929,6 +17161,9 @@
       </c>
       <c r="BQ98" s="15" t="n">
         <v>14151.03</v>
+      </c>
+      <c r="BR98" s="15" t="n">
+        <v>13914.44</v>
       </c>
     </row>
     <row r="99" ht="14.25" customHeight="1">
@@ -17049,6 +17284,7 @@
       <c r="BO99" s="15" t="n"/>
       <c r="BP99" s="15" t="n"/>
       <c r="BQ99" s="15" t="n"/>
+      <c r="BR99" s="15" t="n"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="3" t="n">
@@ -17257,6 +17493,9 @@
       </c>
       <c r="BQ100" s="15" t="n">
         <v>34.12</v>
+      </c>
+      <c r="BR100" s="15" t="n">
+        <v>31.82</v>
       </c>
     </row>
     <row r="101" ht="14.25" customHeight="1">
@@ -17418,6 +17657,9 @@
       </c>
       <c r="BQ101" s="15" t="n">
         <v>3215.13</v>
+      </c>
+      <c r="BR101" s="15" t="n">
+        <v>3203.69</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
@@ -17538,6 +17780,7 @@
       <c r="BO102" s="15" t="n"/>
       <c r="BP102" s="15" t="n"/>
       <c r="BQ102" s="15" t="n"/>
+      <c r="BR102" s="15" t="n"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
       <c r="A103" s="3" t="n">
@@ -17746,6 +17989,9 @@
       </c>
       <c r="BQ103" s="15" t="n">
         <v>30.23</v>
+      </c>
+      <c r="BR103" s="15" t="n">
+        <v>29.75</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
@@ -17907,6 +18153,9 @@
       </c>
       <c r="BQ104" s="15" t="n">
         <v>2305.86</v>
+      </c>
+      <c r="BR104" s="15" t="n">
+        <v>2281.11</v>
       </c>
     </row>
     <row r="105" ht="14.25" customHeight="1">
@@ -18027,6 +18276,7 @@
       <c r="BO105" s="15" t="n"/>
       <c r="BP105" s="15" t="n"/>
       <c r="BQ105" s="15" t="n"/>
+      <c r="BR105" s="15" t="n"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
       <c r="A106" s="3" t="n">
@@ -18235,6 +18485,9 @@
       </c>
       <c r="BQ106" s="15" t="n">
         <v>13.1</v>
+      </c>
+      <c r="BR106" s="15" t="n">
+        <v>14.18</v>
       </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
@@ -18396,6 +18649,9 @@
       </c>
       <c r="BQ107" s="15" t="n">
         <v>2412.23</v>
+      </c>
+      <c r="BR107" s="15" t="n">
+        <v>2413.21</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
@@ -18516,6 +18772,7 @@
       <c r="BO108" s="15" t="n"/>
       <c r="BP108" s="15" t="n"/>
       <c r="BQ108" s="15" t="n"/>
+      <c r="BR108" s="15" t="n"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
       <c r="A109" s="3" t="n">
@@ -18724,6 +18981,9 @@
       </c>
       <c r="BQ109" s="15" t="n">
         <v>30.64</v>
+      </c>
+      <c r="BR109" s="15" t="n">
+        <v>30.04</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1">
@@ -18885,6 +19145,9 @@
       </c>
       <c r="BQ110" s="15" t="n">
         <v>2502.43</v>
+      </c>
+      <c r="BR110" s="15" t="n">
+        <v>2419.39</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
@@ -19005,6 +19268,7 @@
       <c r="BO111" s="15" t="n"/>
       <c r="BP111" s="15" t="n"/>
       <c r="BQ111" s="15" t="n"/>
+      <c r="BR111" s="15" t="n"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -19213,6 +19477,9 @@
       </c>
       <c r="BQ112" s="15" t="n">
         <v>48.77</v>
+      </c>
+      <c r="BR112" s="15" t="n">
+        <v>45.48</v>
       </c>
     </row>
     <row r="113" ht="14.25" customHeight="1">
@@ -19372,6 +19639,9 @@
       </c>
       <c r="BQ113" s="15" t="n">
         <v>1898.47</v>
+      </c>
+      <c r="BR113" s="15" t="n">
+        <v>1883.01</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1">
@@ -19492,6 +19762,7 @@
       <c r="BO114" s="15" t="n"/>
       <c r="BP114" s="15" t="n"/>
       <c r="BQ114" s="15" t="n"/>
+      <c r="BR114" s="15" t="n"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -19700,6 +19971,9 @@
       </c>
       <c r="BQ115" s="15" t="n">
         <v>17.34</v>
+      </c>
+      <c r="BR115" s="15" t="n">
+        <v>16.45</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1">
@@ -19846,6 +20120,9 @@
       </c>
       <c r="BQ116" s="15" t="n">
         <v>8794.76</v>
+      </c>
+      <c r="BR116" s="15" t="n">
+        <v>8587.74</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1">
@@ -19921,6 +20198,7 @@
       <c r="BO117" s="15" t="n"/>
       <c r="BP117" s="15" t="n"/>
       <c r="BQ117" s="15" t="n"/>
+      <c r="BR117" s="15" t="n"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="P118" s="13" t="n">
@@ -20085,6 +20363,9 @@
       <c r="BQ118" s="15" t="n">
         <v>71.87</v>
       </c>
+      <c r="BR118" s="15" t="n">
+        <v>72.06999999999999</v>
+      </c>
     </row>
     <row r="119" ht="14.25" customHeight="1">
       <c r="Y119" s="13" t="n">
@@ -20221,6 +20502,9 @@
       </c>
       <c r="BQ119" s="15" t="n">
         <v>12639.56</v>
+      </c>
+      <c r="BR119" s="15" t="n">
+        <v>12348.16</v>
       </c>
     </row>
     <row r="120" ht="14.25" customHeight="1">
@@ -20245,6 +20529,7 @@
       <c r="BO120" s="15" t="n"/>
       <c r="BP120" s="15" t="n"/>
       <c r="BQ120" s="15" t="n"/>
+      <c r="BR120" s="15" t="n"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
       <c r="AW121" s="13" t="n">
@@ -20310,6 +20595,9 @@
       <c r="BQ121" s="15" t="n">
         <v>28.69</v>
       </c>
+      <c r="BR121" s="15" t="n">
+        <v>27.45</v>
+      </c>
     </row>
     <row r="122" ht="14.25" customHeight="1">
       <c r="AW122" s="13" t="n">
@@ -20374,6 +20662,9 @@
       </c>
       <c r="BQ122" s="15" t="n">
         <v>1258.61</v>
+      </c>
+      <c r="BR122" s="15" t="n">
+        <v>1242.48</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1">
@@ -20398,6 +20689,7 @@
       <c r="BO123" s="15" t="n"/>
       <c r="BP123" s="15" t="n"/>
       <c r="BQ123" s="15" t="n"/>
+      <c r="BR123" s="15" t="n"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
       <c r="AW124" s="13" t="n">
@@ -20463,6 +20755,9 @@
       <c r="BQ124" s="15" t="n">
         <v>48.08</v>
       </c>
+      <c r="BR124" s="15" t="n">
+        <v>52.69</v>
+      </c>
     </row>
     <row r="125" ht="14.25" customHeight="1">
       <c r="AW125" s="13" t="n">
@@ -20527,6 +20822,9 @@
       </c>
       <c r="BQ125" s="15" t="n">
         <v>11645.88</v>
+      </c>
+      <c r="BR125" s="15" t="n">
+        <v>11914.41</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1">
@@ -20551,6 +20849,7 @@
       <c r="BO126" s="15" t="n"/>
       <c r="BP126" s="15" t="n"/>
       <c r="BQ126" s="15" t="n"/>
+      <c r="BR126" s="15" t="n"/>
     </row>
     <row r="127" ht="14.25" customHeight="1">
       <c r="AW127" s="13" t="n">
@@ -20616,6 +20915,9 @@
       <c r="BQ127" s="15" t="n">
         <v>8.470000000000001</v>
       </c>
+      <c r="BR127" s="15" t="n">
+        <v>8.48</v>
+      </c>
     </row>
     <row r="128" ht="14.25" customHeight="1">
       <c r="AW128" s="13" t="n">
@@ -20680,6 +20982,9 @@
       </c>
       <c r="BQ128" s="15" t="n">
         <v>1984.08</v>
+      </c>
+      <c r="BR128" s="15" t="n">
+        <v>1943.68</v>
       </c>
     </row>
     <row r="129" ht="14.25" customHeight="1">
@@ -20704,6 +21009,7 @@
       <c r="BO129" s="15" t="n"/>
       <c r="BP129" s="15" t="n"/>
       <c r="BQ129" s="15" t="n"/>
+      <c r="BR129" s="15" t="n"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="AW130" s="13" t="n">
@@ -20769,6 +21075,9 @@
       <c r="BQ130" s="15" t="n">
         <v>12.73</v>
       </c>
+      <c r="BR130" s="15" t="n">
+        <v>10.29</v>
+      </c>
     </row>
     <row r="131" ht="14.25" customHeight="1">
       <c r="AW131" s="13" t="n">
@@ -20833,6 +21142,9 @@
       </c>
       <c r="BQ131" s="15" t="n">
         <v>758.4</v>
+      </c>
+      <c r="BR131" s="15" t="n">
+        <v>759.02</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1">
@@ -20857,6 +21169,7 @@
       <c r="BO132" s="15" t="n"/>
       <c r="BP132" s="15" t="n"/>
       <c r="BQ132" s="15" t="n"/>
+      <c r="BR132" s="15" t="n"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
       <c r="AW133" s="13" t="n">
@@ -20922,6 +21235,9 @@
       <c r="BQ133" s="15" t="n">
         <v>62.87</v>
       </c>
+      <c r="BR133" s="15" t="n">
+        <v>65.87</v>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="AW134" s="13" t="n">
@@ -20986,6 +21302,9 @@
       </c>
       <c r="BQ134" s="15" t="n">
         <v>2960.13</v>
+      </c>
+      <c r="BR134" s="15" t="n">
+        <v>3015.83</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1">
@@ -21010,6 +21329,7 @@
       <c r="BO135" s="15" t="n"/>
       <c r="BP135" s="15" t="n"/>
       <c r="BQ135" s="15" t="n"/>
+      <c r="BR135" s="15" t="n"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
       <c r="AW136" s="13" t="n">
@@ -21075,6 +21395,9 @@
       <c r="BQ136" s="15" t="n">
         <v>21.99</v>
       </c>
+      <c r="BR136" s="15" t="n">
+        <v>22.65</v>
+      </c>
     </row>
     <row r="137" ht="14.25" customHeight="1">
       <c r="AW137" s="13" t="n">
@@ -21139,6 +21462,9 @@
       </c>
       <c r="BQ137" s="15" t="n">
         <v>3573.26</v>
+      </c>
+      <c r="BR137" s="15" t="n">
+        <v>3616.98</v>
       </c>
     </row>
     <row r="138">
@@ -21155,6 +21481,7 @@
       <c r="BO138" s="15" t="n"/>
       <c r="BP138" s="15" t="n"/>
       <c r="BQ138" s="15" t="n"/>
+      <c r="BR138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="BE139" s="15" t="n">
@@ -21196,6 +21523,9 @@
       <c r="BQ139" s="15" t="n">
         <v>4.25</v>
       </c>
+      <c r="BR139" s="15" t="n">
+        <v>4.25</v>
+      </c>
     </row>
     <row r="140">
       <c r="BE140" s="15" t="n">
@@ -21236,6 +21566,9 @@
       </c>
       <c r="BQ140" s="15" t="n">
         <v>2412.96</v>
+      </c>
+      <c r="BR140" s="15" t="n">
+        <v>2431.48</v>
       </c>
     </row>
     <row r="141">
@@ -21252,6 +21585,7 @@
       <c r="BO141" s="15" t="n"/>
       <c r="BP141" s="15" t="n"/>
       <c r="BQ141" s="15" t="n"/>
+      <c r="BR141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="BE142" s="15" t="n">
@@ -21293,6 +21627,9 @@
       <c r="BQ142" s="15" t="n">
         <v>20.49</v>
       </c>
+      <c r="BR142" s="15" t="n">
+        <v>23.64</v>
+      </c>
     </row>
     <row r="143">
       <c r="BE143" s="15" t="n">
@@ -21333,6 +21670,9 @@
       </c>
       <c r="BQ143" s="15" t="n">
         <v>5754.63</v>
+      </c>
+      <c r="BR143" s="15" t="n">
+        <v>5803.28</v>
       </c>
     </row>
     <row r="144">
@@ -21344,6 +21684,7 @@
       <c r="BO144" s="15" t="n"/>
       <c r="BP144" s="15" t="n"/>
       <c r="BQ144" s="15" t="n"/>
+      <c r="BR144" s="15" t="n"/>
     </row>
     <row r="145">
       <c r="BJ145" s="15" t="n">
@@ -21370,6 +21711,9 @@
       <c r="BQ145" s="15" t="n">
         <v>2.79</v>
       </c>
+      <c r="BR145" s="15" t="n">
+        <v>3.22</v>
+      </c>
     </row>
     <row r="146">
       <c r="BJ146" s="15" t="n">
@@ -21395,6 +21739,9 @@
       </c>
       <c r="BQ146" s="15" t="n">
         <v>2338.32</v>
+      </c>
+      <c r="BR146" s="15" t="n">
+        <v>2354.67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>